<commit_message>
Add the grants-keyword primitive: Naval/Magistrate/Kensai + Elite-effect fix (issue #179)
GrantKeyword is now idempotent. Wires Scourge of the Sea (Follower wave 5) and
the first ability-bearing Item cards, Justice of the Crane and Unparalleled
Sword (Item wave 1), all using AttachGrantsKeyword plus a new Battle Dishonor
action. Corrects Follower Wave 3's Seppun Heavy Elite: it was wrongly granting
the real Elite keyword instead of just Elite's effect (new
AttachGrantsEliteEffect + EliteEffect()).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -533,14 +533,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>39.3%</t>
+          <t>40.2%</t>
         </is>
       </c>
     </row>
@@ -551,14 +551,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
         <v>127</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.6%</t>
+          <t>3.1%</t>
         </is>
       </c>
     </row>
@@ -695,14 +695,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
@@ -27603,14 +27603,10 @@
       </c>
       <c r="E952" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="F952" t="inlineStr">
-        <is>
-          <t>Not blocked; trivial AttachGrantsKeyword grant (same shape as Commander's Steed/Seppun Heavy Elite), deferred for scope.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="F952" t="inlineStr"/>
     </row>
     <row r="953">
       <c r="A953" t="inlineStr">
@@ -27814,11 +27810,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="F959" t="inlineStr">
-        <is>
-          <t>Needs a passive attack-defense modifier plus a new Reaction trigger (another card's own entry).</t>
-        </is>
-      </c>
+      <c r="F959" t="inlineStr"/>
     </row>
     <row r="960">
       <c r="A960" t="inlineStr">
@@ -29867,7 +29859,7 @@
       </c>
       <c r="E1030" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1030" t="inlineStr"/>
@@ -31967,7 +31959,7 @@
       </c>
       <c r="E1105" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1105" t="inlineStr"/>

</xml_diff>

<commit_message>
Add the grants-keyword primitive: Naval/Magistrate/Kensai + Elite-effect fix (issue #179) (#180)
GrantKeyword is now idempotent. Wires Scourge of the Sea (Follower wave 5) and
the first ability-bearing Item cards, Justice of the Crane and Unparalleled
Sword (Item wave 1), all using AttachGrantsKeyword plus a new Battle Dishonor
action. Corrects Follower Wave 3's Seppun Heavy Elite: it was wrongly granting
the real Elite keyword instead of just Elite's effect (new
AttachGrantsEliteEffect + EliteEffect()).

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -533,14 +533,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>39.3%</t>
+          <t>40.2%</t>
         </is>
       </c>
     </row>
@@ -551,14 +551,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
         <v>127</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.6%</t>
+          <t>3.1%</t>
         </is>
       </c>
     </row>
@@ -695,14 +695,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
@@ -27603,14 +27603,10 @@
       </c>
       <c r="E952" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="F952" t="inlineStr">
-        <is>
-          <t>Not blocked; trivial AttachGrantsKeyword grant (same shape as Commander's Steed/Seppun Heavy Elite), deferred for scope.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="F952" t="inlineStr"/>
     </row>
     <row r="953">
       <c r="A953" t="inlineStr">
@@ -27814,11 +27810,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="F959" t="inlineStr">
-        <is>
-          <t>Needs a passive attack-defense modifier plus a new Reaction trigger (another card's own entry).</t>
-        </is>
-      </c>
+      <c r="F959" t="inlineStr"/>
     </row>
     <row r="960">
       <c r="A960" t="inlineStr">
@@ -29867,7 +29859,7 @@
       </c>
       <c r="E1030" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1030" t="inlineStr"/>
@@ -31967,7 +31959,7 @@
       </c>
       <c r="E1105" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1105" t="inlineStr"/>

</xml_diff>

<commit_message>
Add the Additional Action primitive: Again!, Two Hands, Effortless Counterattack (issue #181)
A Battle action a player may take out of the normal back-and-forth alternation
without ceding priority first. NextAction's stay-or-flip decision now lives in
ExecuteAbilityEffects' own tail (a by-reference before/after grant snapshot, so
an unrelated action forfeits dangling grants rather than letting them linger),
and a new additionalActionReaction window lets Effortless Counterattack negate
one before it resolves. Reframes Equip (Battle)'s bespoke spellFollowUp window
as a genuine scoped grant, and wires Justice of the Crane's own deferred
printed-Magistrate bonus now that the primitive it needed exists.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -587,14 +587,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.2%</t>
+          <t>2.7%</t>
         </is>
       </c>
     </row>
@@ -695,14 +695,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
@@ -26728,7 +26728,7 @@
       </c>
       <c r="F923" t="inlineStr">
         <is>
-          <t>Needs Dishonor-as-an-action (known gap) plus a "may not attack" restriction flag.</t>
+          <t>Needs a "may not attack" restriction flag (Dishonor-as-an-action is now built -- Justice of the Crane -- and directly reusable here).</t>
         </is>
       </c>
     </row>
@@ -36691,7 +36691,7 @@
       </c>
       <c r="E1274" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1274" t="inlineStr"/>
@@ -39827,7 +39827,7 @@
       </c>
       <c r="E1386" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1386" t="inlineStr"/>
@@ -51195,7 +51195,7 @@
       </c>
       <c r="E1792" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1792" t="inlineStr"/>

</xml_diff>

<commit_message>
Add the Additional Action primitive: Again!, Two Hands, Effortless Counterattack (issue #181) (#182)
A Battle action a player may take out of the normal back-and-forth alternation
without ceding priority first. NextAction's stay-or-flip decision now lives in
ExecuteAbilityEffects' own tail (a by-reference before/after grant snapshot, so
an unrelated action forfeits dangling grants rather than letting them linger),
and a new additionalActionReaction window lets Effortless Counterattack negate
one before it resolves. Reframes Equip (Battle)'s bespoke spellFollowUp window
as a genuine scoped grant, and wires Justice of the Crane's own deferred
printed-Magistrate bonus now that the primitive it needed exists.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -587,14 +587,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.2%</t>
+          <t>2.7%</t>
         </is>
       </c>
     </row>
@@ -695,14 +695,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
@@ -26728,7 +26728,7 @@
       </c>
       <c r="F923" t="inlineStr">
         <is>
-          <t>Needs Dishonor-as-an-action (known gap) plus a "may not attack" restriction flag.</t>
+          <t>Needs a "may not attack" restriction flag (Dishonor-as-an-action is now built -- Justice of the Crane -- and directly reusable here).</t>
         </is>
       </c>
     </row>
@@ -36691,7 +36691,7 @@
       </c>
       <c r="E1274" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1274" t="inlineStr"/>
@@ -39827,7 +39827,7 @@
       </c>
       <c r="E1386" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1386" t="inlineStr"/>
@@ -51195,7 +51195,7 @@
       </c>
       <c r="E1792" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1792" t="inlineStr"/>

</xml_diff>

<commit_message>
Add Reserve, Stalwart, Discipline keywords and a Removed-from-Game zone (issue #184)
New terminal Zone.RemovedFromGame + PlayerView.RemovedFromGame, visible like
the existing discard piles. Discipline: a new Timing playable from a discard
pile, paying the card's own printed Gold cost, then removed from the game.
Stalwart: negates the first enemy-caused bow each turn, retrofitted onto
every existing bow-dealing ability. Reserve: a new absent-battle-action
recruit straight to the battlefield (Dynasty side), and equip-battle
generalized from Spell-only to any Reserve-keyword attachment, withholding
the bonus Additional Action grant for non-Spells (Fate side). Wires the
first four real cards for these keywords (Personality Wave 6, Follower
Wave 6), all pure reminder text.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -515,14 +515,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C6" t="n">
         <v>810</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
@@ -533,14 +533,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>40.2%</t>
+          <t>41.0%</t>
         </is>
       </c>
     </row>
@@ -695,14 +695,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.4%</t>
         </is>
       </c>
     </row>
@@ -5518,7 +5518,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr"/>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Needs an "Absent Interrupt" mechanic (Bayushi Wateru's own printed ability, on top of Reserve).</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -6554,7 +6558,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F208" t="inlineStr"/>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Needs a Follower-Equip Battle ability with no Shugenja/opposed requirement (Daigotsu Chiboshi's own "Equip a Follower to Chiboshi"), plus tying its own Additional Action grant to a Reserve recruitment specifically.</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -8959,7 +8967,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F294" t="inlineStr"/>
@@ -10474,7 +10482,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F348" t="inlineStr"/>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>Needs a "count of Spells in this unit" Attack-strength axis (Isawa Ikariya's own Ranged Attack).</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -12406,7 +12418,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F417" t="inlineStr"/>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Needs conditional Gold-cost reduction (Kakita Ujirou's own "enters play for N less Gold if...").</t>
+        </is>
+      </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -14699,7 +14715,7 @@
       </c>
       <c r="E499" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F499" t="inlineStr"/>
@@ -15654,7 +15670,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F533" t="inlineStr"/>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>Needs clarification on "Fire Battle:" (a Ring-gated Timing, unclear whether it depends on the not-yet-built Rings primitive) before wiring Moshi Ikako's own Ranged Attack.</t>
+        </is>
+      </c>
     </row>
     <row r="534">
       <c r="A534" t="inlineStr">
@@ -17947,7 +17967,7 @@
       </c>
       <c r="E615" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F615" t="inlineStr"/>
@@ -20638,7 +20658,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F711" t="inlineStr"/>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>Needs conditional Gold-cost reduction (Tamori Shinji's own "enters play for 4 less Gold if you are the Defender").</t>
+        </is>
+      </c>
     </row>
     <row r="712">
       <c r="A712" t="inlineStr">
@@ -22962,7 +22986,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F794" t="inlineStr"/>
+      <c r="F794" t="inlineStr">
+        <is>
+          <t>Needs an "Absent Engage" mechanic (Utaku Sakiko's own printed ability, on top of Destined/Reserve).</t>
+        </is>
+      </c>
     </row>
     <row r="795">
       <c r="A795" t="inlineStr">
@@ -24418,7 +24446,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F846" t="inlineStr"/>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>Needs an "actions must target this card if legal" redirect mechanic (Yoritomo Naoto's own Battle ability), on top of its own Additional Action grant.</t>
+        </is>
+      </c>
     </row>
     <row r="847">
       <c r="A847" t="inlineStr">
@@ -26043,14 +26075,10 @@
       </c>
       <c r="E901" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="F901" t="inlineStr">
-        <is>
-          <t>Needs "Equip this Follower as a Battle action" (Reserve keyword's own reminder).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr"/>
     </row>
     <row r="902">
       <c r="A902" t="inlineStr">
@@ -26600,7 +26628,7 @@
       </c>
       <c r="F919" t="inlineStr">
         <is>
-          <t>Needs a "removed from game" zone plus discard-pile keyword search.</t>
+          <t>Needs discard-pile keyword search (the "removed from game" zone it also needs is now built, issue #184).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Reserve, Stalwart, Discipline keywords and a Removed-from-Game zone (issue #184) (#185)
New terminal Zone.RemovedFromGame + PlayerView.RemovedFromGame, visible like
the existing discard piles. Discipline: a new Timing playable from a discard
pile, paying the card's own printed Gold cost, then removed from the game.
Stalwart: negates the first enemy-caused bow each turn, retrofitted onto
every existing bow-dealing ability. Reserve: a new absent-battle-action
recruit straight to the battlefield (Dynasty side), and equip-battle
generalized from Spell-only to any Reserve-keyword attachment, withholding
the bonus Additional Action grant for non-Spells (Fate side). Wires the
first four real cards for these keywords (Personality Wave 6, Follower
Wave 6), all pure reminder text.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -515,14 +515,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C6" t="n">
         <v>810</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
@@ -533,14 +533,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>40.2%</t>
+          <t>41.0%</t>
         </is>
       </c>
     </row>
@@ -695,14 +695,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.4%</t>
         </is>
       </c>
     </row>
@@ -5518,7 +5518,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr"/>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Needs an "Absent Interrupt" mechanic (Bayushi Wateru's own printed ability, on top of Reserve).</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -6554,7 +6558,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F208" t="inlineStr"/>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Needs a Follower-Equip Battle ability with no Shugenja/opposed requirement (Daigotsu Chiboshi's own "Equip a Follower to Chiboshi"), plus tying its own Additional Action grant to a Reserve recruitment specifically.</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -8959,7 +8967,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F294" t="inlineStr"/>
@@ -10474,7 +10482,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F348" t="inlineStr"/>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>Needs a "count of Spells in this unit" Attack-strength axis (Isawa Ikariya's own Ranged Attack).</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -12406,7 +12418,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F417" t="inlineStr"/>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Needs conditional Gold-cost reduction (Kakita Ujirou's own "enters play for N less Gold if...").</t>
+        </is>
+      </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -14699,7 +14715,7 @@
       </c>
       <c r="E499" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F499" t="inlineStr"/>
@@ -15654,7 +15670,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F533" t="inlineStr"/>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>Needs clarification on "Fire Battle:" (a Ring-gated Timing, unclear whether it depends on the not-yet-built Rings primitive) before wiring Moshi Ikako's own Ranged Attack.</t>
+        </is>
+      </c>
     </row>
     <row r="534">
       <c r="A534" t="inlineStr">
@@ -17947,7 +17967,7 @@
       </c>
       <c r="E615" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F615" t="inlineStr"/>
@@ -20638,7 +20658,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F711" t="inlineStr"/>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>Needs conditional Gold-cost reduction (Tamori Shinji's own "enters play for 4 less Gold if you are the Defender").</t>
+        </is>
+      </c>
     </row>
     <row r="712">
       <c r="A712" t="inlineStr">
@@ -22962,7 +22986,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F794" t="inlineStr"/>
+      <c r="F794" t="inlineStr">
+        <is>
+          <t>Needs an "Absent Engage" mechanic (Utaku Sakiko's own printed ability, on top of Destined/Reserve).</t>
+        </is>
+      </c>
     </row>
     <row r="795">
       <c r="A795" t="inlineStr">
@@ -24418,7 +24446,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F846" t="inlineStr"/>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>Needs an "actions must target this card if legal" redirect mechanic (Yoritomo Naoto's own Battle ability), on top of its own Additional Action grant.</t>
+        </is>
+      </c>
     </row>
     <row r="847">
       <c r="A847" t="inlineStr">
@@ -26043,14 +26075,10 @@
       </c>
       <c r="E901" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="F901" t="inlineStr">
-        <is>
-          <t>Needs "Equip this Follower as a Battle action" (Reserve keyword's own reminder).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr"/>
     </row>
     <row r="902">
       <c r="A902" t="inlineStr">
@@ -26600,7 +26628,7 @@
       </c>
       <c r="F919" t="inlineStr">
         <is>
-          <t>Needs a "removed from game" zone plus discard-pile keyword search.</t>
+          <t>Needs discard-pile keyword search (the "removed from game" zone it also needs is now built, issue #184).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Formalize Dishonor/Rehonor, wire Justice of the Crane and Utaku Chikako (issue #186)
Named Dishonor(card)/Rehonor(card) pair, replacing ad hoc .Dishonorable
assignments. CardPersonalHonor gets an override hook for Utaku Chikako's own
passive (dishonorable Battle Maidens keep their printed Personal Honor). New
GainHonorFromPerformer negates an Honor gain and rehonors a dishonorable
performer instead; battle resolution now rehonors a dishonorable winner/tier
and negates the full victory Honor gain, with a tie rehonoring before its own
mutual destruction to avoid a double penalty. Confirms Justice of the Crane's
PrintedKeyword check was already correct. Wires Utaku Chikako (Personality
Wave 7): the Personal-Honor override plus her Limited ability, backed by a
new per-turn "may not declare an attack" player flag. Documents the Recon
keyword's classification rule without speculative code.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -515,14 +515,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C6" t="n">
         <v>810</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
@@ -22731,7 +22731,7 @@
       </c>
       <c r="E785" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F785" t="inlineStr"/>
@@ -26756,7 +26756,7 @@
       </c>
       <c r="F923" t="inlineStr">
         <is>
-          <t>Needs a "may not attack" restriction flag (Dishonor-as-an-action is now built -- Justice of the Crane -- and directly reusable here).</t>
+          <t>Needs a per-card, permanent "this Personality may not attack" attachment flag (Utaku Chikako's own restriction, issue #186, is a player-and-turn-scoped flag, not directly reusable here) plus a self-destroying Limited ability. Dishonor-as-an-action is now built (Justice of the Crane) and directly reusable for its own Dishonor half.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Formalize Dishonor/Rehonor, wire Justice of the Crane and Utaku Chikako (issue #186) (#187)
Named Dishonor(card)/Rehonor(card) pair, replacing ad hoc .Dishonorable
assignments. CardPersonalHonor gets an override hook for Utaku Chikako's own
passive (dishonorable Battle Maidens keep their printed Personal Honor). New
GainHonorFromPerformer negates an Honor gain and rehonors a dishonorable
performer instead; battle resolution now rehonors a dishonorable winner/tier
and negates the full victory Honor gain, with a tie rehonoring before its own
mutual destruction to avoid a double penalty. Confirms Justice of the Crane's
PrintedKeyword check was already correct. Wires Utaku Chikako (Personality
Wave 7): the Personal-Honor override plus her Limited ability, backed by a
new per-turn "may not declare an attack" player flag. Documents the Recon
keyword's classification rule without speculative code.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -515,14 +515,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C6" t="n">
         <v>810</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
@@ -22731,7 +22731,7 @@
       </c>
       <c r="E785" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F785" t="inlineStr"/>
@@ -26756,7 +26756,7 @@
       </c>
       <c r="F923" t="inlineStr">
         <is>
-          <t>Needs a "may not attack" restriction flag (Dishonor-as-an-action is now built -- Justice of the Crane -- and directly reusable here).</t>
+          <t>Needs a per-card, permanent "this Personality may not attack" attachment flag (Utaku Chikako's own restriction, issue #186, is a player-and-turn-scoped flag, not directly reusable here) plus a self-destroying Limited ability. Dishonor-as-an-action is now built (Justice of the Crane) and directly reusable for its own Dishonor half.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kiho keyword, discard-to-hand primitive; wire Hunter of Harmony and Volcano Tattoo (issue #190)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -533,14 +533,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>41.0%</t>
+          <t>41.8%</t>
         </is>
       </c>
     </row>
@@ -587,14 +587,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.7%</t>
+          <t>2.8%</t>
         </is>
       </c>
     </row>
@@ -695,14 +695,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>8.4%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
@@ -26623,14 +26623,10 @@
       </c>
       <c r="E919" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="F919" t="inlineStr">
-        <is>
-          <t>Needs discard-pile keyword search (the "removed from game" zone it also needs is now built, issue #184).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="F919" t="inlineStr"/>
     </row>
     <row r="920">
       <c r="A920" t="inlineStr">
@@ -52175,7 +52171,7 @@
       </c>
       <c r="E1826" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1826" t="inlineStr"/>

</xml_diff>

<commit_message>
Deck-return and top-of-Fate-deck-discard primitives; wire Goju House Guard, Aberrations, and a Focus-1 Battle-action wave (issue #192)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -533,14 +533,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>41.0%</t>
+          <t>42.6%</t>
         </is>
       </c>
     </row>
@@ -551,14 +551,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C8" t="n">
         <v>127</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.1%</t>
+          <t>4.7%</t>
         </is>
       </c>
     </row>
@@ -587,14 +587,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.7%</t>
+          <t>2.8%</t>
         </is>
       </c>
     </row>
@@ -695,14 +695,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>8.4%</t>
+          <t>8.7%</t>
         </is>
       </c>
     </row>
@@ -24923,14 +24923,10 @@
       </c>
       <c r="E863" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="F863" t="inlineStr">
-        <is>
-          <t>No "discard top of Fate deck" mechanic.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr"/>
     </row>
     <row r="864">
       <c r="A864" t="inlineStr">
@@ -26291,14 +26287,10 @@
       </c>
       <c r="E908" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="F908" t="inlineStr">
-        <is>
-          <t>Needs "put on top/bottom of own Fate deck as a cost" plus a mass bottom-of-deck effect.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="F908" t="inlineStr"/>
     </row>
     <row r="909">
       <c r="A909" t="inlineStr">
@@ -26628,7 +26620,7 @@
       </c>
       <c r="F919" t="inlineStr">
         <is>
-          <t>Needs discard-pile keyword search (the "removed from game" zone it also needs is now built, issue #184).</t>
+          <t>Needs a top-of-hand "freshly drawn" return-from-discard mechanic (in flight on a sibling PR, issue #190 -- not yet merged as of this wave).</t>
         </is>
       </c>
     </row>
@@ -27036,7 +27028,7 @@
       </c>
       <c r="F932" t="inlineStr">
         <is>
-          <t>No "discard top of Fate deck" mechanic.</t>
+          <t>Focus 4, not 1 -- outside the #192 wave's own scope. The top-of-Fate-deck discard primitive now exists (Aberrations, issue #192), but this needs a "whose deck" target choice ("any Fate deck", not just your own) plus a variable-strength Melee Attack keyed off the discarded card's Focus Value, not a Force modifier.</t>
         </is>
       </c>
     </row>
@@ -29414,7 +29406,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1013" t="inlineStr"/>
+      <c r="F1013" t="inlineStr">
+        <is>
+          <t>Needs Chi as a repeatable payable cost resource (distinct from a Force/Stat modifier), interacting correctly with the existing Chi&lt;=0 death rule.</t>
+        </is>
+      </c>
     </row>
     <row r="1014">
       <c r="A1014" t="inlineStr">
@@ -30783,7 +30779,7 @@
       </c>
       <c r="E1062" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1062" t="inlineStr"/>
@@ -31035,7 +31031,7 @@
       </c>
       <c r="E1071" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1071" t="inlineStr"/>
@@ -31150,7 +31146,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1075" t="inlineStr"/>
+      <c r="F1075" t="inlineStr">
+        <is>
+          <t>Needs Dueling/Focus Effects (the Battle half, a plain Force debuff, is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1076">
       <c r="A1076" t="inlineStr">
@@ -31290,7 +31290,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1080" t="inlineStr"/>
+      <c r="F1080" t="inlineStr">
+        <is>
+          <t>Needs Dueling/Focus Effects (the Battle half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1081">
       <c r="A1081" t="inlineStr">
@@ -33194,7 +33198,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1148" t="inlineStr"/>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>Needs Rings (not built).</t>
+        </is>
+      </c>
     </row>
     <row r="1149">
       <c r="A1149" t="inlineStr">
@@ -33838,7 +33846,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1171" t="inlineStr"/>
+      <c r="F1171" t="inlineStr">
+        <is>
+          <t>Needs a keyword-conditional cost EXEMPTION (bow the performer unless it has a given keyword) -- distinct from every existing keyword-conditional EFFECT.</t>
+        </is>
+      </c>
     </row>
     <row r="1172">
       <c r="A1172" t="inlineStr">
@@ -34314,7 +34326,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1188" t="inlineStr"/>
+      <c r="F1188" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (similar shape to the existing move-to-battlefield-if-opposed patterns).</t>
+        </is>
+      </c>
     </row>
     <row r="1189">
       <c r="A1189" t="inlineStr">
@@ -34678,7 +34694,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1201" t="inlineStr"/>
+      <c r="F1201" t="inlineStr">
+        <is>
+          <t>Needs a delayed, multi-step revival mechanic ("before this turn ends, put a removed unit into play ignoring costs") -- not built.</t>
+        </is>
+      </c>
     </row>
     <row r="1202">
       <c r="A1202" t="inlineStr">
@@ -34902,7 +34922,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1209" t="inlineStr"/>
+      <c r="F1209" t="inlineStr">
+        <is>
+          <t>Needs an "after being targeted, negate" Reaction trigger (same gap as oracle-l5r-1292/10107).</t>
+        </is>
+      </c>
     </row>
     <row r="1210">
       <c r="A1210" t="inlineStr">
@@ -35294,7 +35318,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1223" t="inlineStr"/>
+      <c r="F1223" t="inlineStr">
+        <is>
+          <t>Needs an ability-copying mechanism (novel meta-effect; not built).</t>
+        </is>
+      </c>
     </row>
     <row r="1224">
       <c r="A1224" t="inlineStr">
@@ -35994,7 +36022,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1248" t="inlineStr"/>
+      <c r="F1248" t="inlineStr">
+        <is>
+          <t>Needs an "after being targeted" Reaction trigger (the Battle half, a plain Force boost, is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1249">
       <c r="A1249" t="inlineStr">
@@ -36078,7 +36110,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1251" t="inlineStr"/>
+      <c r="F1251" t="inlineStr">
+        <is>
+          <t>Needs a Gold-Cost comparison Target category plus a Gold-Cost-reduction effect (both novel).</t>
+        </is>
+      </c>
     </row>
     <row r="1252">
       <c r="A1252" t="inlineStr">
@@ -37058,7 +37094,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1286" t="inlineStr"/>
+      <c r="F1286" t="inlineStr">
+        <is>
+          <t>Needs a Retainer mechanic, movement to any location (not just home), and a province-card discard (three separate gaps).</t>
+        </is>
+      </c>
     </row>
     <row r="1287">
       <c r="A1287" t="inlineStr">
@@ -37310,7 +37350,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1295" t="inlineStr"/>
+      <c r="F1295" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (Discipline is already built; needs only a new "own opposed Personality" Target category).</t>
+        </is>
+      </c>
     </row>
     <row r="1296">
       <c r="A1296" t="inlineStr">
@@ -37730,7 +37774,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1310" t="inlineStr"/>
+      <c r="F1310" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (CardInstance.StraightenBlockedTurn already exists for the negate-next-straightening half; needs a new Paragon Performer category and an enemy-unit-card Target).</t>
+        </is>
+      </c>
     </row>
     <row r="1311">
       <c r="A1311" t="inlineStr">
@@ -37758,7 +37806,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1311" t="inlineStr"/>
+      <c r="F1311" t="inlineStr">
+        <is>
+          <t>Needs Regions (not built).</t>
+        </is>
+      </c>
     </row>
     <row r="1312">
       <c r="A1312" t="inlineStr">
@@ -37870,7 +37922,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1315" t="inlineStr"/>
+      <c r="F1315" t="inlineStr">
+        <is>
+          <t>Needs Dueling/Focus Effects (not started at all).</t>
+        </is>
+      </c>
     </row>
     <row r="1316">
       <c r="A1316" t="inlineStr">
@@ -38178,7 +38234,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1326" t="inlineStr"/>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (similar shape to the existing move-to-battlefield patterns, e.g. Journey's End).</t>
+        </is>
+      </c>
     </row>
     <row r="1327">
       <c r="A1327" t="inlineStr">
@@ -38374,7 +38434,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1333" t="inlineStr"/>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (RemoveFromGame and the discarded-personality Target already exist; needs a Shadowlands/Undead-conditional bonus amount).</t>
+        </is>
+      </c>
     </row>
     <row r="1334">
       <c r="A1334" t="inlineStr">
@@ -38486,7 +38550,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1337" t="inlineStr"/>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>Needs an ability-lock mechanism ("abilities on other cards in its unit may not be used") -- not built.</t>
+        </is>
+      </c>
     </row>
     <row r="1338">
       <c r="A1338" t="inlineStr">
@@ -38654,7 +38722,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1343" t="inlineStr"/>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>Needs a new Reaction trigger: "after an action resolves that a Personality performed" (the Terrain-play and additional-Battle-action halves are separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1344">
       <c r="A1344" t="inlineStr">
@@ -39522,7 +39594,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1374" t="inlineStr"/>
+      <c r="F1374" t="inlineStr">
+        <is>
+          <t>Needs an opponent-chooses-or-random discard mechanic (Reconnaissance-conditional).</t>
+        </is>
+      </c>
     </row>
     <row r="1375">
       <c r="A1375" t="inlineStr">
@@ -39998,7 +40074,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1391" t="inlineStr"/>
+      <c r="F1391" t="inlineStr">
+        <is>
+          <t>Needs a "before this battle resolves" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1392">
       <c r="A1392" t="inlineStr">
@@ -40026,7 +40106,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1392" t="inlineStr"/>
+      <c r="F1392" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (Monk Performer, attachment-destroy Target, and Fire-token-conditional Attack strength are all existing patterns, just not yet combined on one card).</t>
+        </is>
+      </c>
     </row>
     <row r="1393">
       <c r="A1393" t="inlineStr">
@@ -40222,7 +40306,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1399" t="inlineStr"/>
+      <c r="F1399" t="inlineStr">
+        <is>
+          <t>Needs a "before this battle resolves" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1400">
       <c r="A1400" t="inlineStr">
@@ -40530,7 +40618,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1410" t="inlineStr"/>
+      <c r="F1410" t="inlineStr">
+        <is>
+          <t>Needs a "before a card effect destroys a Personality, negate" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1411">
       <c r="A1411" t="inlineStr">
@@ -40642,7 +40734,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1414" t="inlineStr"/>
+      <c r="F1414" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (DiscardTopOfFateDeck, the Madness token, and an unattached-unit-card Target all now exist; needs resolving "a Fate deck"'s ownership the same way Aberrations did).</t>
+        </is>
+      </c>
     </row>
     <row r="1415">
       <c r="A1415" t="inlineStr">
@@ -40698,7 +40794,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1416" t="inlineStr"/>
+      <c r="F1416" t="inlineStr">
+        <is>
+          <t>Needs an Absent-Battle-timed Terrain-play variant (the existing one is Battle-timed only) plus a province-strength passive.</t>
+        </is>
+      </c>
     </row>
     <row r="1417">
       <c r="A1417" t="inlineStr">
@@ -41062,7 +41162,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1429" t="inlineStr"/>
+      <c r="F1429" t="inlineStr">
+        <is>
+          <t>Needs a two-performer selection (existing abilities support only one Performer) plus an army-unit-count comparison (both novel).</t>
+        </is>
+      </c>
     </row>
     <row r="1430">
       <c r="A1430" t="inlineStr">
@@ -41286,7 +41390,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1437" t="inlineStr"/>
+      <c r="F1437" t="inlineStr">
+        <is>
+          <t>Needs an "after being targeted" Reaction trigger (the additional-Battle-action half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1438">
       <c r="A1438" t="inlineStr">
@@ -41398,7 +41506,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1441" t="inlineStr"/>
+      <c r="F1441" t="inlineStr">
+        <is>
+          <t>Needs a unit-Force-total comparison Target (existing categories only compare individual card Force).</t>
+        </is>
+      </c>
     </row>
     <row r="1442">
       <c r="A1442" t="inlineStr">
@@ -41482,7 +41594,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1444" t="inlineStr"/>
+      <c r="F1444" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (an army-scoped keyword-conditional Force boost mirrors Utaku Elite Guard's existing pattern).</t>
+        </is>
+      </c>
     </row>
     <row r="1445">
       <c r="A1445" t="inlineStr">
@@ -41538,7 +41654,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1446" t="inlineStr"/>
+      <c r="F1446" t="inlineStr">
+        <is>
+          <t>Needs a movement-negation passive for a Terrain (the Terrain-play and additional-Battle-action halves are separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1447">
       <c r="A1447" t="inlineStr">
@@ -41566,7 +41686,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1447" t="inlineStr"/>
+      <c r="F1447" t="inlineStr">
+        <is>
+          <t>Needs a "before this battle's resolution" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1448">
       <c r="A1448" t="inlineStr">
@@ -41622,7 +41746,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1449" t="inlineStr"/>
+      <c r="F1449" t="inlineStr">
+        <is>
+          <t>Needs Equip from the discard pile (explicitly known gap, oracle-l5r-10681) plus a "before this battle resolves" destruction trigger.</t>
+        </is>
+      </c>
     </row>
     <row r="1450">
       <c r="A1450" t="inlineStr">
@@ -41706,7 +41834,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1452" t="inlineStr"/>
+      <c r="F1452" t="inlineStr">
+        <is>
+          <t>Needs a new tracked EnteredPlayTurn field on CardInstance (same gap as oracle-l5r-10335).</t>
+        </is>
+      </c>
     </row>
     <row r="1453">
       <c r="A1453" t="inlineStr">
@@ -41762,7 +41894,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1454" t="inlineStr"/>
+      <c r="F1454" t="inlineStr">
+        <is>
+          <t>Needs a "before this battle resolves" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1455">
       <c r="A1455" t="inlineStr">
@@ -41930,7 +42066,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1460" t="inlineStr"/>
+      <c r="F1460" t="inlineStr">
+        <is>
+          <t>Needs a self-replacing Terrain variant ("destroy a Terrain if able, then play this one") plus an ongoing army-wide Force passive tied to being in play as Terrain.</t>
+        </is>
+      </c>
     </row>
     <row r="1461">
       <c r="A1461" t="inlineStr">
@@ -42630,7 +42770,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1485" t="inlineStr"/>
+      <c r="F1485" t="inlineStr">
+        <is>
+          <t>Needs Equip from the discard pile (explicitly known gap, oracle-l5r-10681).</t>
+        </is>
+      </c>
     </row>
     <row r="1486">
       <c r="A1486" t="inlineStr">
@@ -42770,7 +42914,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1490" t="inlineStr"/>
+      <c r="F1490" t="inlineStr">
+        <is>
+          <t>Needs a "move an enemy Personality into the current battlefield" mechanic -- every existing move primitive moves the acting player's own cards, or moves a card home, never an opponent's card into battle.</t>
+        </is>
+      </c>
     </row>
     <row r="1491">
       <c r="A1491" t="inlineStr">
@@ -43190,7 +43338,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1505" t="inlineStr"/>
+      <c r="F1505" t="inlineStr">
+        <is>
+          <t>Needs a "before this battle resolves" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1506">
       <c r="A1506" t="inlineStr">
@@ -43330,7 +43482,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1510" t="inlineStr"/>
+      <c r="F1510" t="inlineStr">
+        <is>
+          <t>Needs a self-replacing Terrain variant plus an ongoing army-wide Force passive tied to being in play as Terrain (same two gaps as oracle-l5r-10941).</t>
+        </is>
+      </c>
     </row>
     <row r="1511">
       <c r="A1511" t="inlineStr">
@@ -43358,7 +43514,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1511" t="inlineStr"/>
+      <c r="F1511" t="inlineStr">
+        <is>
+          <t>Needs a unit-Force-total comparison Target (same gap as oracle-l5r-2900/4118).</t>
+        </is>
+      </c>
     </row>
     <row r="1512">
       <c r="A1512" t="inlineStr">
@@ -43386,7 +43546,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1512" t="inlineStr"/>
+      <c r="F1512" t="inlineStr">
+        <is>
+          <t>Needs an "after this battle resolves" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1513">
       <c r="A1513" t="inlineStr">
@@ -43470,7 +43634,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1515" t="inlineStr"/>
+      <c r="F1515" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (Discipline is already built; needs a standalone "attachment" Target category, a subset of the existing attachment-or-dishonorable-personality shape).</t>
+        </is>
+      </c>
     </row>
     <row r="1516">
       <c r="A1516" t="inlineStr">
@@ -43554,7 +43722,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1518" t="inlineStr"/>
+      <c r="F1518" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (own-personality Target, CardPersonalHonor, and dual Force/Chi modifiers all already exist; needs a new "unopposed" condition check).</t>
+        </is>
+      </c>
     </row>
     <row r="1519">
       <c r="A1519" t="inlineStr">
@@ -43974,7 +44146,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1533" t="inlineStr"/>
+      <c r="F1533" t="inlineStr">
+        <is>
+          <t>Needs a "count this card's own keywords, excluding a named pattern" mechanism (novel).</t>
+        </is>
+      </c>
     </row>
     <row r="1534">
       <c r="A1534" t="inlineStr">
@@ -44254,7 +44430,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1543" t="inlineStr"/>
+      <c r="F1543" t="inlineStr">
+        <is>
+          <t>Needs an exemption from the generic Battle-timing army-presence requirement (the adjacent-battlefield Performer shape itself, Moto Gunso's own, already exists).</t>
+        </is>
+      </c>
     </row>
     <row r="1544">
       <c r="A1544" t="inlineStr">
@@ -44282,7 +44462,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1544" t="inlineStr"/>
+      <c r="F1544" t="inlineStr">
+        <is>
+          <t>Needs the discard-to-hand "freshly drawn" primitive (in flight on a sibling PR, issue #190) plus an "after this battle ends" trigger for the optional return.</t>
+        </is>
+      </c>
     </row>
     <row r="1545">
       <c r="A1545" t="inlineStr">
@@ -44506,7 +44690,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1552" t="inlineStr"/>
+      <c r="F1552" t="inlineStr">
+        <is>
+          <t>Needs a dual-target selection with a relational constraint ("not sharing a Clan alignment") -- every existing multi-target category compares against a fixed performer/self, not between two chosen targets.</t>
+        </is>
+      </c>
     </row>
     <row r="1553">
       <c r="A1553" t="inlineStr">
@@ -44618,7 +44806,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1556" t="inlineStr"/>
+      <c r="F1556" t="inlineStr">
+        <is>
+          <t>Needs a general "attach any attachment from hand, at a Gold discount" Battle action, distinct from a Reserve/Spell-specific Equip variant.</t>
+        </is>
+      </c>
     </row>
     <row r="1557">
       <c r="A1557" t="inlineStr">
@@ -44646,7 +44838,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1557" t="inlineStr"/>
+      <c r="F1557" t="inlineStr">
+        <is>
+          <t>Needs a tracked "has the enemy leader taken a Battle action this battle" flag (novel state; the additional-Battle-actions half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1558">
       <c r="A1558" t="inlineStr">
@@ -44786,7 +44982,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1562" t="inlineStr"/>
+      <c r="F1562" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (an army-scoped Follower-presence-conditional Force passive mirrors Utaku Elite Guard's existing pattern).</t>
+        </is>
+      </c>
     </row>
     <row r="1563">
       <c r="A1563" t="inlineStr">
@@ -44954,7 +45154,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1568" t="inlineStr"/>
+      <c r="F1568" t="inlineStr">
+        <is>
+          <t>Needs Dueling/Focus Effects (not started at all).</t>
+        </is>
+      </c>
     </row>
     <row r="1569">
       <c r="A1569" t="inlineStr">
@@ -45066,7 +45270,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1572" t="inlineStr"/>
+      <c r="F1572" t="inlineStr">
+        <is>
+          <t>Needs an "after being targeted" Reaction trigger plus card creation (a temporary token Personality) -- both known gaps.</t>
+        </is>
+      </c>
     </row>
     <row r="1573">
       <c r="A1573" t="inlineStr">
@@ -45122,7 +45330,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1574" t="inlineStr"/>
+      <c r="F1574" t="inlineStr">
+        <is>
+          <t>Needs a non-AtBattle-gated compound Performer category for BattleOrOpen abilities (every existing keyword-Performer category requires the current battlefield).</t>
+        </is>
+      </c>
     </row>
     <row r="1575">
       <c r="A1575" t="inlineStr">
@@ -45150,7 +45362,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1575" t="inlineStr"/>
+      <c r="F1575" t="inlineStr">
+        <is>
+          <t>Needs a "count copies of this same card played this battle" mechanism (novel; the additional-Battle-action half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1576">
       <c r="A1576" t="inlineStr">
@@ -45262,7 +45478,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1579" t="inlineStr"/>
+      <c r="F1579" t="inlineStr">
+        <is>
+          <t>Needs a Gold-Cost comparison Target category (same gap as oracle-l5r-24).</t>
+        </is>
+      </c>
     </row>
     <row r="1580">
       <c r="A1580" t="inlineStr">
@@ -45486,7 +45706,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1587" t="inlineStr"/>
+      <c r="F1587" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (the opponent-chooses-effect shape, shinden-choice's own, already exists; needs a "was this negated" detection hook feeding a fallback effect).</t>
+        </is>
+      </c>
     </row>
     <row r="1588">
       <c r="A1588" t="inlineStr">
@@ -45626,7 +45850,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1592" t="inlineStr"/>
+      <c r="F1592" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (needs the same new "own opposed Personality" Target category noted for oracle-l5r-10929).</t>
+        </is>
+      </c>
     </row>
     <row r="1593">
       <c r="A1593" t="inlineStr">
@@ -46379,7 +46607,7 @@
       </c>
       <c r="E1619" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1619" t="inlineStr"/>
@@ -46494,7 +46722,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1623" t="inlineStr"/>
+      <c r="F1623" t="inlineStr">
+        <is>
+          <t>Needs an "actions must target this card if legal" redirect mechanic (same gap as oracle-l5r-10300).</t>
+        </is>
+      </c>
     </row>
     <row r="1624">
       <c r="A1624" t="inlineStr">
@@ -46690,7 +46922,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1630" t="inlineStr"/>
+      <c r="F1630" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (mirrors the existing Chi&lt;=0-after-modifier check pattern, applied to Force instead).</t>
+        </is>
+      </c>
     </row>
     <row r="1631">
       <c r="A1631" t="inlineStr">
@@ -47110,7 +47346,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1645" t="inlineStr"/>
+      <c r="F1645" t="inlineStr">
+        <is>
+          <t>Needs a non-AtBattle-gated Performer category ("at any location", same gap as oracle-l5r-5941).</t>
+        </is>
+      </c>
     </row>
     <row r="1646">
       <c r="A1646" t="inlineStr">
@@ -47250,7 +47490,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1650" t="inlineStr"/>
+      <c r="F1650" t="inlineStr">
+        <is>
+          <t>Needs an ongoing army-wide Force passive tied to being in play as Terrain (same gap as oracle-l5r-10941; the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1651">
       <c r="A1651" t="inlineStr">
@@ -47334,7 +47578,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1653" t="inlineStr"/>
+      <c r="F1653" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (Ninja Performer and Bow already exist; needs a province-card discard similar to Kharmic-discard's own).</t>
+        </is>
+      </c>
     </row>
     <row r="1654">
       <c r="A1654" t="inlineStr">
@@ -48398,7 +48646,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1691" t="inlineStr"/>
+      <c r="F1691" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (a dynamic Force-reduction-by-another-card's-Force and a sub-choice of which attachment to destroy are both close to existing patterns).</t>
+        </is>
+      </c>
     </row>
     <row r="1692">
       <c r="A1692" t="inlineStr">
@@ -48454,7 +48706,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1693" t="inlineStr"/>
+      <c r="F1693" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (a numeric-threshold Performer condition mirrors existing Force-threshold conditions elsewhere).</t>
+        </is>
+      </c>
     </row>
     <row r="1694">
       <c r="A1694" t="inlineStr">
@@ -48482,7 +48738,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1694" t="inlineStr"/>
+      <c r="F1694" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (single-card Force comparisons and a printed-Force threshold both already exist elsewhere).</t>
+        </is>
+      </c>
     </row>
     <row r="1695">
       <c r="A1695" t="inlineStr">
@@ -48510,7 +48770,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1695" t="inlineStr"/>
+      <c r="F1695" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (a dual-choice pattern sharing one UsageKey, Horibe's own shape, already exists).</t>
+        </is>
+      </c>
     </row>
     <row r="1696">
       <c r="A1696" t="inlineStr">
@@ -48622,7 +48886,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1699" t="inlineStr"/>
+      <c r="F1699" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (the Reaction half mirrors Khol Regulars' own -3 exactly; the Battle half needs a "defending Personality" Performer filter plus a before-battle-resolves straighten).</t>
+        </is>
+      </c>
     </row>
     <row r="1700">
       <c r="A1700" t="inlineStr">
@@ -48958,7 +49226,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1711" t="inlineStr"/>
+      <c r="F1711" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (the lower-or-equal-honor-than-performer Target already exists).</t>
+        </is>
+      </c>
     </row>
     <row r="1712">
       <c r="A1712" t="inlineStr">
@@ -49182,7 +49454,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1719" t="inlineStr"/>
+      <c r="F1719" t="inlineStr">
+        <is>
+          <t>Needs a "Political" Reaction timing (not built; the Battle half, a plain straighten, is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1720">
       <c r="A1720" t="inlineStr">
@@ -49406,7 +49682,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1727" t="inlineStr"/>
+      <c r="F1727" t="inlineStr">
+        <is>
+          <t>Needs Dueling/Focus Effects (the Battle half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1728">
       <c r="A1728" t="inlineStr">
@@ -49462,7 +49742,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1729" t="inlineStr"/>
+      <c r="F1729" t="inlineStr">
+        <is>
+          <t>Needs a self-replacing Terrain variant plus a delayed post-destruction straighten (two gaps, same self-replace gap as oracle-l5r-10941).</t>
+        </is>
+      </c>
     </row>
     <row r="1730">
       <c r="A1730" t="inlineStr">
@@ -49882,7 +50166,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1744" t="inlineStr"/>
+      <c r="F1744" t="inlineStr">
+        <is>
+          <t>Needs a new trigger keyed to passing instead of a Battle action (novel; the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1745">
       <c r="A1745" t="inlineStr">
@@ -49966,7 +50254,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1747" t="inlineStr"/>
+      <c r="F1747" t="inlineStr">
+        <is>
+          <t>Needs a "Political" Reaction timing (not built; the plain Ranged 1 Attack half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1748">
       <c r="A1748" t="inlineStr">
@@ -50274,7 +50566,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1758" t="inlineStr"/>
+      <c r="F1758" t="inlineStr">
+        <is>
+          <t>Needs a unit-Force-total comparison Target (same gap as oracle-l5r-2900) plus a per-card override of "a bowed card contributes no Force."</t>
+        </is>
+      </c>
     </row>
     <row r="1759">
       <c r="A1759" t="inlineStr">
@@ -50470,7 +50766,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1765" t="inlineStr"/>
+      <c r="F1765" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (a Spider-Clan-keyword Performer, dynamic Force reduction, and a conditional bow-if-Force-now-0 are each close to existing patterns).</t>
+        </is>
+      </c>
     </row>
     <row r="1766">
       <c r="A1766" t="inlineStr">
@@ -50722,7 +51022,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1774" t="inlineStr"/>
+      <c r="F1774" t="inlineStr">
+        <is>
+          <t>Needs a unit-Force-total comparison Target (same gap as oracle-l5r-2900).</t>
+        </is>
+      </c>
     </row>
     <row r="1775">
       <c r="A1775" t="inlineStr">
@@ -50834,7 +51138,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1778" t="inlineStr"/>
+      <c r="F1778" t="inlineStr">
+        <is>
+          <t>Needs an ongoing "negate all current and new Force penalties" effect (novel; the plain-straighten half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1779">
       <c r="A1779" t="inlineStr">
@@ -51058,7 +51366,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1786" t="inlineStr"/>
+      <c r="F1786" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (the Reaction half mirrors Khol Regulars' own -2; the Battle half is a move-to-an-opposed-battlefield variant of existing move mechanics).</t>
+        </is>
+      </c>
     </row>
     <row r="1787">
       <c r="A1787" t="inlineStr">
@@ -51282,7 +51594,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1794" t="inlineStr"/>
+      <c r="F1794" t="inlineStr">
+        <is>
+          <t>Needs a discard-pile-usable variant distinct from Discipline (its own printed ability, not a Discipline-keyword card).</t>
+        </is>
+      </c>
     </row>
     <row r="1795">
       <c r="A1795" t="inlineStr">
@@ -51450,7 +51766,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1800" t="inlineStr"/>
+      <c r="F1800" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (an optional bow-then-draw needs a small player choice, otherwise all existing patterns).</t>
+        </is>
+      </c>
     </row>
     <row r="1801">
       <c r="A1801" t="inlineStr">
@@ -51590,7 +51910,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1805" t="inlineStr"/>
+      <c r="F1805" t="inlineStr">
+        <is>
+          <t>Needs an "Interrupt" timing (not built; the plain Melee 2 Attack half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1806">
       <c r="A1806" t="inlineStr">
@@ -51618,7 +51942,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1806" t="inlineStr"/>
+      <c r="F1806" t="inlineStr">
+        <is>
+          <t>Needs a broad "before another player's action" Reaction trigger (existing triggers are narrow -- before an Attack, before an additional action -- not any action).</t>
+        </is>
+      </c>
     </row>
     <row r="1807">
       <c r="A1807" t="inlineStr">
@@ -52066,7 +52394,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1822" t="inlineStr"/>
+      <c r="F1822" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (the Set-Force pattern already exists, per oracle-l5r-543's own note).</t>
+        </is>
+      </c>
     </row>
     <row r="1823">
       <c r="A1823" t="inlineStr">
@@ -52122,7 +52454,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1824" t="inlineStr"/>
+      <c r="F1824" t="inlineStr">
+        <is>
+          <t>Needs an "after this battlefield's province is destroyed" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1825">
       <c r="A1825" t="inlineStr">
@@ -52402,7 +52738,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1834" t="inlineStr"/>
+      <c r="F1834" t="inlineStr">
+        <is>
+          <t>Needs a "before an action's effect destroys a card, negate" Reaction trigger (same gap as oracle-l5r-2530; the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1835">
       <c r="A1835" t="inlineStr">
@@ -52514,7 +52854,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1838" t="inlineStr"/>
+      <c r="F1838" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (Spirit-keyword Performer and MoveHome already exist; the 'will not be negated' clause just means never opening the reaction window for this specific move).</t>
+        </is>
+      </c>
     </row>
     <row r="1839">
       <c r="A1839" t="inlineStr">

</xml_diff>

<commit_message>
Rings concept: recruitment as a granted Additional Battle Action, Enlightenment victory; wire 6 Rings plus Moshi Ikako and Scholarly Hermit (issue #194)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -15672,7 +15672,7 @@
       </c>
       <c r="F533" t="inlineStr">
         <is>
-          <t>Needs clarification on "Fire Battle:" (a Ring-gated Timing, unclear whether it depends on the not-yet-built Rings primitive) before wiring Moshi Ikako's own Ranged Attack.</t>
+          <t>Wired (issue #194) -- "Fire Battle" was confirmed to be a plain classification, not a Ring-gated Timing. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
         </is>
       </c>
     </row>
@@ -25320,7 +25320,7 @@
       </c>
       <c r="F876" t="inlineStr">
         <is>
-          <t>Needs an "after being targeted" Reaction trigger, plus Rings (not built).</t>
+          <t>Needs a retroactive partial-negation Reaction trigger ("after another player's action targets a card, negate just its bowing" -- existing triggers fully negate, or fire before resolution, never after with a partial effect). Rings themselves are now built (issue #194); "if you control any Rings" is trivial.</t>
         </is>
       </c>
     </row>
@@ -27604,7 +27604,7 @@
       </c>
       <c r="F951" t="inlineStr">
         <is>
-          <t>Needs Rings (not built).</t>
+          <t>Wired (issue #194) -- needed only a Ring-type check in a discard pile, now trivial. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
         </is>
       </c>
     </row>
@@ -60830,7 +60830,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2135" t="inlineStr"/>
+      <c r="F2135" t="inlineStr">
+        <is>
+          <t>Wired (issue #194) -- False Ring of Air. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
+        </is>
+      </c>
     </row>
     <row r="2136">
       <c r="A2136" t="inlineStr">
@@ -60858,7 +60862,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2136" t="inlineStr"/>
+      <c r="F2136" t="inlineStr">
+        <is>
+          <t>Needs Dueling/Focus Effects (not started at all) for False Ring of Earth's own recruitment condition.</t>
+        </is>
+      </c>
     </row>
     <row r="2137">
       <c r="A2137" t="inlineStr">
@@ -60886,7 +60894,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2137" t="inlineStr"/>
+      <c r="F2137" t="inlineStr">
+        <is>
+          <t>Needs an Interrupt timing (not built) for its own printed action, plus an adjustable maximum-hand-size mechanism (not built) for its own recruitment condition.</t>
+        </is>
+      </c>
     </row>
     <row r="2138">
       <c r="A2138" t="inlineStr">
@@ -60914,7 +60926,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2138" t="inlineStr"/>
+      <c r="F2138" t="inlineStr">
+        <is>
+          <t>Wired (issue #194) -- False Ring of Water. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
+        </is>
+      </c>
     </row>
     <row r="2139">
       <c r="A2139" t="inlineStr">
@@ -60942,7 +60958,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2139" t="inlineStr"/>
+      <c r="F2139" t="inlineStr">
+        <is>
+          <t>Needs an Engage timing (explicitly not started, #15) for its own printed action; its recruitment condition is otherwise wirable.</t>
+        </is>
+      </c>
     </row>
     <row r="2140">
       <c r="A2140" t="inlineStr">
@@ -60970,7 +60990,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2140" t="inlineStr"/>
+      <c r="F2140" t="inlineStr">
+        <is>
+          <t>Wired (issue #194) -- Ring of Air. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
+        </is>
+      </c>
     </row>
     <row r="2141">
       <c r="A2141" t="inlineStr">
@@ -60998,7 +61022,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2141" t="inlineStr"/>
+      <c r="F2141" t="inlineStr">
+        <is>
+          <t>Needs an Interrupt timing (not built) for Ring of Earth's own printed action; its recruitment condition is otherwise wirable.</t>
+        </is>
+      </c>
     </row>
     <row r="2142">
       <c r="A2142" t="inlineStr">
@@ -61026,7 +61054,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2142" t="inlineStr"/>
+      <c r="F2142" t="inlineStr">
+        <is>
+          <t>Set aside (issue #195) -- the local oracle data's own selected printing/text for this Emperor Edition card is uncertain; a user-supplied photo did not match either candidate text found.</t>
+        </is>
+      </c>
     </row>
     <row r="2143">
       <c r="A2143" t="inlineStr">
@@ -61054,7 +61086,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2143" t="inlineStr"/>
+      <c r="F2143" t="inlineStr">
+        <is>
+          <t>Wired (issue #194) -- Ring of Water. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
+        </is>
+      </c>
     </row>
     <row r="2144">
       <c r="A2144" t="inlineStr">
@@ -61082,7 +61118,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2144" t="inlineStr"/>
+      <c r="F2144" t="inlineStr">
+        <is>
+          <t>Wired (issue #194) -- Ring of the Void. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Wire 17 Lion Clan Personalities, audit and log blockers for the other 49 (issue #198)
Reviews all 79 catalogue Lion Clan Personalities (66 previously unwired) and
wires the clearest, most confidently-buildable 17 using only primitives
already built through issue #194: five small new Target categories, a
token-gated Additional Action grant (Akodo Kano), and two passive Force
modifiers (Matsu Yoshito, Pride of the Hand). The other 49 each get a
specific, accurate blocker note in docs/CARD_INVENTORY.xlsx instead of a
generic "not wired".

Also discovers the local scan-image cache is missing repo-wide (a deliberate
.gitignore policy, not a bug), and recovers 2,485 of 2,952 scans locally from
the "Catalogue artwork - WebP 85 - v1" GitHub Release via a new reusable tool
(tools/content/audit_and_install_scans.py). Per explicit instruction, the
rewritten receipt JSON files stay local/uncommitted.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -515,14 +515,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="C6" t="n">
         <v>810</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>13.6%</t>
         </is>
       </c>
     </row>
@@ -695,14 +695,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>181</v>
+        <v>198</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>8.4%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Needs a Battle-timed Recruit-from-province mechanic (distinct from ordinary Dynasty purchase) plus a unit-count comparison between sides.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2354,7 +2358,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Not blocked; the Melee 4 Attack is directly wirable with the existing attack primitive. Deferred for scope this pass: a cross-player Honor-Requirement-waiver-for-recruitment clause (Crab Clan players may ignore her Honor Requirement).</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2410,7 +2418,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Needs a 'battle resolution does not bow winning cards' modifier flag, triggered by a before-resolution Reaction (not built). The Melee 8 Attack itself is trivial but incomplete without it.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2435,7 +2447,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -2463,7 +2475,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2494,7 +2506,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Needs a modifiable Personal Honor stat (current PersonalHonor is a fixed printed value with no StatModifier equivalent), a 'Dark Virtue' action classification, and an Honor-Victory-threshold modifier -- none built.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2522,7 +2538,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Needs a broad 'after another player's action targets this card' Reaction trigger (the single largest recurring gap across multiple waves).</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2547,7 +2567,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
@@ -2575,7 +2595,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
@@ -2603,7 +2623,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -2634,7 +2654,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Needs a modifier hook into the existing Tactical Advantage rulebook action's own Force-bonus amount (a generic action-amount-modifier mechanism doesn't exist yet).</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2690,7 +2714,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Needs a 'Tactical action resolved' classification-dispatch trigger, a broad 'after an enemy Battle action destroys your card' Reaction trigger, and a cost/Honor-Requirement-ignoring Recruit -- none built.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2718,7 +2746,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Needs card creation (a new Follower instance). 'Tactical Limited' itself maps onto the existing Limited Timing per the established Political/Tactical precedent, so is not itself a blocker.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2743,7 +2775,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
@@ -2771,7 +2803,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -2802,7 +2834,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Needs a broad, repeatable 'before another player's action resolves' Reaction trigger (a before-resolution window keyed to enemy actions, not built).</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2858,7 +2894,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Needs a 'discard all your other Sensei Personalities' entry effect (recurs on Ikoma Aimi's base printing) and an action-classification-dispatch Reaction trigger spanning Tactical/Bushido Virtue/Terrain actions (a three-way version of the still-unbuilt 'action resolved' classification gap).</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2886,7 +2926,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Needs Bushido Virtue as a targetable/filterable Strategy sub-classification (Discipline's own 'play from discard, remove from game after' mechanism is built and partly reusable, but gated here behind an Additional Action and a Bushido-Virtue-specific discard-pile filter).</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2911,7 +2955,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -2939,7 +2983,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -2970,7 +3014,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>The Phoenix-opposition Force bonus is directly wirable (reuses this wave's own clan-conditional attacking-vs-dragon-bonus pattern); blocked only by its Limited ability -- 'look at the top Fate card and choose to leave/discard/bottom it' (no look-then-choose deck-top primitive exists; DiscardTopOfFateDeck is one-way only).</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2998,7 +3046,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Needs a 'retrieve a specific card from your discard pile into hand' primitive (distinct from deck search; not built).</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -9754,7 +9806,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F322" t="inlineStr"/>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Needs a 'discard all your other Sensei Personalities' entry effect (recurs on Akodo Tamisu) and a keyword-suppression mechanism (grant Courtier while stripping six named keywords from every Lion Clan Personality you control) -- keyword suppression not built.</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -9779,7 +9835,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F323" t="inlineStr"/>
@@ -9807,7 +9863,7 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F324" t="inlineStr"/>
@@ -9838,7 +9894,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F325" t="inlineStr"/>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Needs the 'Tactical action' classification-trigger gap -- specifically a Reaction firing when a Tactical action is announced, not merely after it resolves.</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -9866,7 +9926,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F326" t="inlineStr"/>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>Needs a 'will not gain [keyword]' immunity flag, and a per-performer Timing override on the shared Tactical Advantage rulebook action -- neither built.</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -9894,7 +9958,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F327" t="inlineStr"/>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>Needs generalization of the existing move-home primitives (Incapacitated/Block are battle-resolution-specific, tied to attacker/defender roles) into a standalone 'move this targeted Personality home' Battle-ability effect, usable as one branch of a dual choice alongside a Force bonus.</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -9922,7 +9990,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F328" t="inlineStr"/>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Invest itself is built, but this variant needs 'refill the specific province this card entered from, face-up' -- a targeted, face-up province refill tied to entry-provenance (existing refills are face-down and untargeted).</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -9947,7 +10019,7 @@
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F329" t="inlineStr"/>
@@ -10006,7 +10078,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F331" t="inlineStr"/>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>The Open Cavalry-grant is directly wirable (reuses the existing generic GrantKeyword primitive); blocked only by 'will not join a Unicorn Clan player' -- a recruitment clan-exclusion rule, not built.</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -10034,7 +10110,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F332" t="inlineStr"/>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>Needs a reveal-a-hand-card-and-offer-to-another-player mechanism with an opponent's accept/reject choice, plus a Home-targeted Attack (existing Attacks only target the current battlefield).</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -10090,7 +10170,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F334" t="inlineStr"/>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Needs an optional-discard-for-attack-bonus primitive (a Ranged Attack whose strength depends on an optional cost paid at the same time, plus a card-type-conditional follow-up draw) -- not built.</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -10118,7 +10202,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F335" t="inlineStr"/>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>Needs a dual-independent-target primitive (choosing a Terrain AND a separate enemy card in one ability) -- no existing shape supports two independently-chosen targets.</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -10146,7 +10234,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F336" t="inlineStr"/>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Needs both a dual-independent-target primitive (a Follower in hand plus a separate Personality target) and 'Equip this Follower as a Battle action' (not yet a general capability) -- two established gaps compounding on the same card.</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -10174,7 +10266,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F337" t="inlineStr"/>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Needs deck search (pull a specific card out of a shuffled deck) and Regions (neither built).</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -10199,7 +10295,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F338" t="inlineStr"/>
@@ -10311,7 +10407,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F342" t="inlineStr"/>
@@ -10342,7 +10438,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F343" t="inlineStr"/>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>The Battle Ranged 4 Attack is directly wirable; blocked by its own passive -- a global 'all your Ranged Attacks get +1 strength while you control a Terrain' scope, distinct from a single card's own conditional Attack strength (existing kamina-exp-attack/shuji-attack-style bonuses only affect their own card's attack, not every Attack the controller makes).</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -11494,7 +11594,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F384" t="inlineStr"/>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Needs the Engage-timing Reaction window (explicitly not started, #15), plus a 'first Battle-action opportunity, restricted to Terrain actions' priority override.</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -11550,7 +11654,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F386" t="inlineStr"/>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Needs the Ring of Earth (not yet wired as a real published card) and clarification on 'Earth Battle' as a Ring-gated Timing (same open question already flagged for Moshi Ikako, oracle-l5r-10857) before wiring Jikoji's own army-wide Force bonus, plus a conditional Gold-Cost waiver tied to Ring control.</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -12702,7 +12810,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F427" t="inlineStr"/>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>Needs card creation (a new Personality instance) -- Kitsu Akai's own Limited half creates the only Ancestors his Battle half can use as a Performer.</t>
+        </is>
+      </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -12730,7 +12842,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F428" t="inlineStr"/>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>Needs a 'bow OR destroy the performer' cost-choice (not yet built), and is functionally contingent on card creation existing elsewhere (every other Ancestor-Personality source for this deck is itself blocked on 'Needs card creation').</t>
+        </is>
+      </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -12758,7 +12874,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F429" t="inlineStr"/>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Needs card creation (a new Personality instance) as an entry Reaction effect.</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -12842,7 +12962,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F432" t="inlineStr"/>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>Needs card creation (a new Personality instance created directly at a battlefield, then removed from the game when the battle ends) and a 'Home Battle' Timing (performable from Home, unlike ordinary Battle actions which require AtBattle) -- neither built.</t>
+        </is>
+      </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
@@ -12870,7 +12994,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F433" t="inlineStr"/>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>Needs deck search (pull a specific card, filtered by Clan/Type/Unique-status, out of a shuffled Dynasty deck) -- not built.</t>
+        </is>
+      </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -12898,7 +13026,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F434" t="inlineStr"/>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>Not blocked; the Destined half is already built (KeywordMechanics), and a controller-clan-conditional Honor-Requirement waiver has direct precedent (Allegiance/clan-discount mechanics) -- deferred for scope this pass, not a genuine gap.</t>
+        </is>
+      </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -12954,7 +13086,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F436" t="inlineStr"/>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>Needs card creation (two new Personality instances) as an entry/overlay Reaction effect; 'overlays' as an alternate entry-trigger condition (distinct from ordinary Purchase) is not yet verified as built.</t>
+        </is>
+      </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -12982,7 +13118,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F437" t="inlineStr"/>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>Needs a per-player 'controls an Ancestor' Honor-gain/loss sweep referencing each player's own starting Family Honor baseline (not tracked as a stat) plus an imposed choice against another player's own card state.</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -13010,7 +13150,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F438" t="inlineStr"/>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Needs Interrupt timing (not started) and card creation (a new Personality instance).</t>
+        </is>
+      </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
@@ -13038,7 +13182,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F439" t="inlineStr"/>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Needs card creation (a new Personality instance) plus a turn-spanning 'lost Honor from another player's action since your last turn began' tracked condition, and a variable one-to-four multi-target selection -- none built.</t>
+        </is>
+      </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
@@ -14435,7 +14583,7 @@
       </c>
       <c r="E489" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F489" t="inlineStr"/>
@@ -14494,7 +14642,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F491" t="inlineStr"/>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Needs a unit-scoped 'bow every card in the target unit meeting a Force comparison' primitive (existing unit/army-scoped primitives only apply static Force modifiers, none perform a bow across a filtered set of cards); the per-card Honor gain has direct precedent (BattleHonor).</t>
+        </is>
+      </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
@@ -14522,7 +14674,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F492" t="inlineStr"/>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Not blocked; both halves have direct precedent (a plain 'while attacking' Force bonus, and a Force-penalty-equal-to-current-Force pattern matching Mirumoto Reiyu) -- deferred for scope this pass. 'Fear Battle' Timing-prefix meaning not yet confirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
@@ -14550,7 +14706,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F493" t="inlineStr"/>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>The +2F while attacking is free (reuses the existing attacking-two Effect verbatim); the Battle half needs a general 'move a target Personality home' action (existing move-home mechanics -- Incapacitated/Block -- are battle-resolution-specific, not a standalone targeted ability).</t>
+        </is>
+      </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
@@ -14578,7 +14738,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F494" t="inlineStr"/>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Needs an activated (not passive/static) 'apply a Force penalty to every card in the target unit, then bow any now at 0' primitive -- the existing unit-scoped Force primitives (UnitForceBoostPrimitive, ArmyBattleMaidenBoostPrimitive) are passive/continuous, not one-shot activated effects across a filtered unit.</t>
+        </is>
+      </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
@@ -14606,7 +14770,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F495" t="inlineStr"/>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Needs an army-wide activated Force bonus where the amount varies per target (each card's own Personal Honor) -- existing army/unit-boost primitives only grant a flat, identical bonus to every qualifying card.</t>
+        </is>
+      </c>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
@@ -14634,7 +14802,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F496" t="inlineStr"/>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Not blocked; identical in shape to Matsu Arata's own arata-force-penalty ability wired in Personality wave 8 (a Force penalty on a target equal to the performer's own Personal Honor) -- deferred for scope this pass, a trivial follow-up wire-up.</t>
+        </is>
+      </c>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
@@ -14662,7 +14834,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F497" t="inlineStr"/>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Needs card creation (a new Personality copying this card's own printed Force/Chi/Personal Honor/keywords) and a 'this card's own ability will not be copied' flag -- no card-copying mechanism exists yet at all.</t>
+        </is>
+      </c>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
@@ -14690,7 +14866,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F498" t="inlineStr"/>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Needs the 'Bushido Virtue action resolved' classification-dispatch Reaction trigger (same unbuilt family as 'Tactical action resolved'), and a three-times-per-turn usage counter (existing dedupe is strictly once-per-turn).</t>
+        </is>
+      </c>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
@@ -14746,7 +14926,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F500" t="inlineStr"/>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Needs a 'this card's Force counts twice during battle resolution' hook (no existing mechanism double-counts one specific card in a resolution total), and a personality-level 'will not attach Items' restriction (the existing 'Will only/not attach to X' restriction gates the ATTACHMENT side, not a blanket type-level refusal from the host).</t>
+        </is>
+      </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
@@ -14771,7 +14955,7 @@
       </c>
       <c r="E501" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F501" t="inlineStr"/>
@@ -14802,7 +14986,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F502" t="inlineStr"/>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Needs a targeting-immunity flag against a specific Attack kind (Ranged) scoped to a whole unit -- distinct from the existing passive Attack-strength defense (Destrier/Singh Remnants), which reduces effective strength rather than making the target illegal outright.</t>
+        </is>
+      </c>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
@@ -15642,7 +15830,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F532" t="inlineStr"/>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>Needs a control-transfer mechanic (explicitly deferred since Loyal, #142) -- specifically a temporary, Gold-production-only control grant over another player's Holding, without a full ownership change.</t>
+        </is>
+      </c>
     </row>
     <row r="533">
       <c r="A533" t="inlineStr">
@@ -17351,7 +17543,7 @@
       </c>
       <c r="E593" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F593" t="inlineStr"/>
@@ -24898,7 +25090,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F862" t="inlineStr"/>
+      <c r="F862" t="inlineStr">
+        <is>
+          <t>Needs a payment-time interrupt -- an alternate Gold source triggered DURING an in-progress Gold payment (destroying a Mine/Farm mid-payment), not built.</t>
+        </is>
+      </c>
     </row>
     <row r="863">
       <c r="A863" t="inlineStr">

</xml_diff>

<commit_message>
Wire 17 Lion Clan Personalities, audit and log blockers for the other 49 (issue #198) (#199)
Reviews all 79 catalogue Lion Clan Personalities (66 previously unwired) and
wires the clearest, most confidently-buildable 17 using only primitives
already built through issue #194: five small new Target categories, a
token-gated Additional Action grant (Akodo Kano), and two passive Force
modifiers (Matsu Yoshito, Pride of the Hand). The other 49 each get a
specific, accurate blocker note in docs/CARD_INVENTORY.xlsx instead of a
generic "not wired".

Also discovers the local scan-image cache is missing repo-wide (a deliberate
.gitignore policy, not a bug), and recovers 2,485 of 2,952 scans locally from
the "Catalogue artwork - WebP 85 - v1" GitHub Release via a new reusable tool
(tools/content/audit_and_install_scans.py). Per explicit instruction, the
rewritten receipt JSON files stay local/uncommitted.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -515,14 +515,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="C6" t="n">
         <v>810</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>13.6%</t>
         </is>
       </c>
     </row>
@@ -695,14 +695,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>181</v>
+        <v>198</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>8.4%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Needs a Battle-timed Recruit-from-province mechanic (distinct from ordinary Dynasty purchase) plus a unit-count comparison between sides.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2354,7 +2358,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Not blocked; the Melee 4 Attack is directly wirable with the existing attack primitive. Deferred for scope this pass: a cross-player Honor-Requirement-waiver-for-recruitment clause (Crab Clan players may ignore her Honor Requirement).</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2410,7 +2418,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Needs a 'battle resolution does not bow winning cards' modifier flag, triggered by a before-resolution Reaction (not built). The Melee 8 Attack itself is trivial but incomplete without it.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2435,7 +2447,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -2463,7 +2475,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2494,7 +2506,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Needs a modifiable Personal Honor stat (current PersonalHonor is a fixed printed value with no StatModifier equivalent), a 'Dark Virtue' action classification, and an Honor-Victory-threshold modifier -- none built.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2522,7 +2538,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Needs a broad 'after another player's action targets this card' Reaction trigger (the single largest recurring gap across multiple waves).</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2547,7 +2567,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
@@ -2575,7 +2595,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
@@ -2603,7 +2623,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -2634,7 +2654,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Needs a modifier hook into the existing Tactical Advantage rulebook action's own Force-bonus amount (a generic action-amount-modifier mechanism doesn't exist yet).</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2690,7 +2714,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Needs a 'Tactical action resolved' classification-dispatch trigger, a broad 'after an enemy Battle action destroys your card' Reaction trigger, and a cost/Honor-Requirement-ignoring Recruit -- none built.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2718,7 +2746,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Needs card creation (a new Follower instance). 'Tactical Limited' itself maps onto the existing Limited Timing per the established Political/Tactical precedent, so is not itself a blocker.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2743,7 +2775,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
@@ -2771,7 +2803,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -2802,7 +2834,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Needs a broad, repeatable 'before another player's action resolves' Reaction trigger (a before-resolution window keyed to enemy actions, not built).</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2858,7 +2894,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Needs a 'discard all your other Sensei Personalities' entry effect (recurs on Ikoma Aimi's base printing) and an action-classification-dispatch Reaction trigger spanning Tactical/Bushido Virtue/Terrain actions (a three-way version of the still-unbuilt 'action resolved' classification gap).</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2886,7 +2926,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Needs Bushido Virtue as a targetable/filterable Strategy sub-classification (Discipline's own 'play from discard, remove from game after' mechanism is built and partly reusable, but gated here behind an Additional Action and a Bushido-Virtue-specific discard-pile filter).</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2911,7 +2955,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -2939,7 +2983,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -2970,7 +3014,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>The Phoenix-opposition Force bonus is directly wirable (reuses this wave's own clan-conditional attacking-vs-dragon-bonus pattern); blocked only by its Limited ability -- 'look at the top Fate card and choose to leave/discard/bottom it' (no look-then-choose deck-top primitive exists; DiscardTopOfFateDeck is one-way only).</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2998,7 +3046,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Needs a 'retrieve a specific card from your discard pile into hand' primitive (distinct from deck search; not built).</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -9754,7 +9806,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F322" t="inlineStr"/>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Needs a 'discard all your other Sensei Personalities' entry effect (recurs on Akodo Tamisu) and a keyword-suppression mechanism (grant Courtier while stripping six named keywords from every Lion Clan Personality you control) -- keyword suppression not built.</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -9779,7 +9835,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F323" t="inlineStr"/>
@@ -9807,7 +9863,7 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F324" t="inlineStr"/>
@@ -9838,7 +9894,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F325" t="inlineStr"/>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Needs the 'Tactical action' classification-trigger gap -- specifically a Reaction firing when a Tactical action is announced, not merely after it resolves.</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -9866,7 +9926,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F326" t="inlineStr"/>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>Needs a 'will not gain [keyword]' immunity flag, and a per-performer Timing override on the shared Tactical Advantage rulebook action -- neither built.</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -9894,7 +9958,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F327" t="inlineStr"/>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>Needs generalization of the existing move-home primitives (Incapacitated/Block are battle-resolution-specific, tied to attacker/defender roles) into a standalone 'move this targeted Personality home' Battle-ability effect, usable as one branch of a dual choice alongside a Force bonus.</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -9922,7 +9990,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F328" t="inlineStr"/>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Invest itself is built, but this variant needs 'refill the specific province this card entered from, face-up' -- a targeted, face-up province refill tied to entry-provenance (existing refills are face-down and untargeted).</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -9947,7 +10019,7 @@
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F329" t="inlineStr"/>
@@ -10006,7 +10078,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F331" t="inlineStr"/>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>The Open Cavalry-grant is directly wirable (reuses the existing generic GrantKeyword primitive); blocked only by 'will not join a Unicorn Clan player' -- a recruitment clan-exclusion rule, not built.</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -10034,7 +10110,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F332" t="inlineStr"/>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>Needs a reveal-a-hand-card-and-offer-to-another-player mechanism with an opponent's accept/reject choice, plus a Home-targeted Attack (existing Attacks only target the current battlefield).</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -10090,7 +10170,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F334" t="inlineStr"/>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Needs an optional-discard-for-attack-bonus primitive (a Ranged Attack whose strength depends on an optional cost paid at the same time, plus a card-type-conditional follow-up draw) -- not built.</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -10118,7 +10202,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F335" t="inlineStr"/>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>Needs a dual-independent-target primitive (choosing a Terrain AND a separate enemy card in one ability) -- no existing shape supports two independently-chosen targets.</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -10146,7 +10234,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F336" t="inlineStr"/>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Needs both a dual-independent-target primitive (a Follower in hand plus a separate Personality target) and 'Equip this Follower as a Battle action' (not yet a general capability) -- two established gaps compounding on the same card.</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -10174,7 +10266,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F337" t="inlineStr"/>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Needs deck search (pull a specific card out of a shuffled deck) and Regions (neither built).</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -10199,7 +10295,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F338" t="inlineStr"/>
@@ -10311,7 +10407,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F342" t="inlineStr"/>
@@ -10342,7 +10438,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F343" t="inlineStr"/>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>The Battle Ranged 4 Attack is directly wirable; blocked by its own passive -- a global 'all your Ranged Attacks get +1 strength while you control a Terrain' scope, distinct from a single card's own conditional Attack strength (existing kamina-exp-attack/shuji-attack-style bonuses only affect their own card's attack, not every Attack the controller makes).</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -11494,7 +11594,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F384" t="inlineStr"/>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Needs the Engage-timing Reaction window (explicitly not started, #15), plus a 'first Battle-action opportunity, restricted to Terrain actions' priority override.</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -11550,7 +11654,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F386" t="inlineStr"/>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Needs the Ring of Earth (not yet wired as a real published card) and clarification on 'Earth Battle' as a Ring-gated Timing (same open question already flagged for Moshi Ikako, oracle-l5r-10857) before wiring Jikoji's own army-wide Force bonus, plus a conditional Gold-Cost waiver tied to Ring control.</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -12702,7 +12810,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F427" t="inlineStr"/>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>Needs card creation (a new Personality instance) -- Kitsu Akai's own Limited half creates the only Ancestors his Battle half can use as a Performer.</t>
+        </is>
+      </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -12730,7 +12842,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F428" t="inlineStr"/>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>Needs a 'bow OR destroy the performer' cost-choice (not yet built), and is functionally contingent on card creation existing elsewhere (every other Ancestor-Personality source for this deck is itself blocked on 'Needs card creation').</t>
+        </is>
+      </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -12758,7 +12874,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F429" t="inlineStr"/>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Needs card creation (a new Personality instance) as an entry Reaction effect.</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -12842,7 +12962,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F432" t="inlineStr"/>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>Needs card creation (a new Personality instance created directly at a battlefield, then removed from the game when the battle ends) and a 'Home Battle' Timing (performable from Home, unlike ordinary Battle actions which require AtBattle) -- neither built.</t>
+        </is>
+      </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
@@ -12870,7 +12994,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F433" t="inlineStr"/>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>Needs deck search (pull a specific card, filtered by Clan/Type/Unique-status, out of a shuffled Dynasty deck) -- not built.</t>
+        </is>
+      </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -12898,7 +13026,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F434" t="inlineStr"/>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>Not blocked; the Destined half is already built (KeywordMechanics), and a controller-clan-conditional Honor-Requirement waiver has direct precedent (Allegiance/clan-discount mechanics) -- deferred for scope this pass, not a genuine gap.</t>
+        </is>
+      </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -12954,7 +13086,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F436" t="inlineStr"/>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>Needs card creation (two new Personality instances) as an entry/overlay Reaction effect; 'overlays' as an alternate entry-trigger condition (distinct from ordinary Purchase) is not yet verified as built.</t>
+        </is>
+      </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -12982,7 +13118,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F437" t="inlineStr"/>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>Needs a per-player 'controls an Ancestor' Honor-gain/loss sweep referencing each player's own starting Family Honor baseline (not tracked as a stat) plus an imposed choice against another player's own card state.</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -13010,7 +13150,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F438" t="inlineStr"/>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Needs Interrupt timing (not started) and card creation (a new Personality instance).</t>
+        </is>
+      </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
@@ -13038,7 +13182,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F439" t="inlineStr"/>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Needs card creation (a new Personality instance) plus a turn-spanning 'lost Honor from another player's action since your last turn began' tracked condition, and a variable one-to-four multi-target selection -- none built.</t>
+        </is>
+      </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
@@ -14435,7 +14583,7 @@
       </c>
       <c r="E489" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F489" t="inlineStr"/>
@@ -14494,7 +14642,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F491" t="inlineStr"/>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Needs a unit-scoped 'bow every card in the target unit meeting a Force comparison' primitive (existing unit/army-scoped primitives only apply static Force modifiers, none perform a bow across a filtered set of cards); the per-card Honor gain has direct precedent (BattleHonor).</t>
+        </is>
+      </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
@@ -14522,7 +14674,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F492" t="inlineStr"/>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Not blocked; both halves have direct precedent (a plain 'while attacking' Force bonus, and a Force-penalty-equal-to-current-Force pattern matching Mirumoto Reiyu) -- deferred for scope this pass. 'Fear Battle' Timing-prefix meaning not yet confirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
@@ -14550,7 +14706,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F493" t="inlineStr"/>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>The +2F while attacking is free (reuses the existing attacking-two Effect verbatim); the Battle half needs a general 'move a target Personality home' action (existing move-home mechanics -- Incapacitated/Block -- are battle-resolution-specific, not a standalone targeted ability).</t>
+        </is>
+      </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
@@ -14578,7 +14738,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F494" t="inlineStr"/>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Needs an activated (not passive/static) 'apply a Force penalty to every card in the target unit, then bow any now at 0' primitive -- the existing unit-scoped Force primitives (UnitForceBoostPrimitive, ArmyBattleMaidenBoostPrimitive) are passive/continuous, not one-shot activated effects across a filtered unit.</t>
+        </is>
+      </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
@@ -14606,7 +14770,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F495" t="inlineStr"/>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Needs an army-wide activated Force bonus where the amount varies per target (each card's own Personal Honor) -- existing army/unit-boost primitives only grant a flat, identical bonus to every qualifying card.</t>
+        </is>
+      </c>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
@@ -14634,7 +14802,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F496" t="inlineStr"/>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Not blocked; identical in shape to Matsu Arata's own arata-force-penalty ability wired in Personality wave 8 (a Force penalty on a target equal to the performer's own Personal Honor) -- deferred for scope this pass, a trivial follow-up wire-up.</t>
+        </is>
+      </c>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
@@ -14662,7 +14834,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F497" t="inlineStr"/>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Needs card creation (a new Personality copying this card's own printed Force/Chi/Personal Honor/keywords) and a 'this card's own ability will not be copied' flag -- no card-copying mechanism exists yet at all.</t>
+        </is>
+      </c>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
@@ -14690,7 +14866,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F498" t="inlineStr"/>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Needs the 'Bushido Virtue action resolved' classification-dispatch Reaction trigger (same unbuilt family as 'Tactical action resolved'), and a three-times-per-turn usage counter (existing dedupe is strictly once-per-turn).</t>
+        </is>
+      </c>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
@@ -14746,7 +14926,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F500" t="inlineStr"/>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Needs a 'this card's Force counts twice during battle resolution' hook (no existing mechanism double-counts one specific card in a resolution total), and a personality-level 'will not attach Items' restriction (the existing 'Will only/not attach to X' restriction gates the ATTACHMENT side, not a blanket type-level refusal from the host).</t>
+        </is>
+      </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
@@ -14771,7 +14955,7 @@
       </c>
       <c r="E501" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F501" t="inlineStr"/>
@@ -14802,7 +14986,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F502" t="inlineStr"/>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Needs a targeting-immunity flag against a specific Attack kind (Ranged) scoped to a whole unit -- distinct from the existing passive Attack-strength defense (Destrier/Singh Remnants), which reduces effective strength rather than making the target illegal outright.</t>
+        </is>
+      </c>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
@@ -15642,7 +15830,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F532" t="inlineStr"/>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>Needs a control-transfer mechanic (explicitly deferred since Loyal, #142) -- specifically a temporary, Gold-production-only control grant over another player's Holding, without a full ownership change.</t>
+        </is>
+      </c>
     </row>
     <row r="533">
       <c r="A533" t="inlineStr">
@@ -17351,7 +17543,7 @@
       </c>
       <c r="E593" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F593" t="inlineStr"/>
@@ -24898,7 +25090,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F862" t="inlineStr"/>
+      <c r="F862" t="inlineStr">
+        <is>
+          <t>Needs a payment-time interrupt -- an alternate Gold source triggered DURING an in-progress Gold payment (destroying a Mine/Farm mid-payment), not built.</t>
+        </is>
+      </c>
     </row>
     <row r="863">
       <c r="A863" t="inlineStr">

</xml_diff>

<commit_message>
Add Dueling (issue #204) and the Duelist keyword
A paused sub-state-machine (MatchState.PendingDuel) mirroring the
existing PendingAttack/additional-action deferral pattern: an ability
flagged AbilityDefinition.IssuesDuel resolves generically, then defers
its effect to IssueChallenge until the whole duel -- accept/refuse,
reaction window, alternating focus/strike (new Zone.Focused, hidden
from the opponent until Struck), Duelist re-focus, Focus-Effect
ordering (new Timing:FocusEffect), and resolution -- finishes, at
which point play resumes exactly where the challenge was issued.

Wires Strategy Wave 5 (Steel on Steel, The Courtesy of the Crane) as
the first real cards, reproducing the user's own worked example
(Doji Tatsuki 8 vs. Matsu Hachiro 7) as a test. Files issue #205
asking Alfredo to illustrate the special duel battlefield.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -587,14 +587,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.7%</t>
+          <t>3.0%</t>
         </is>
       </c>
     </row>
@@ -695,14 +695,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
@@ -48423,7 +48423,7 @@
       </c>
       <c r="E1685" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1685" t="inlineStr"/>
@@ -49627,7 +49627,7 @@
       </c>
       <c r="E1728" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1728" t="inlineStr"/>

</xml_diff>

<commit_message>
Kiho keyword, discard-to-hand primitive; wire Hunter of Harmony and Volcano Tattoo (#191)
* Kiho keyword, discard-to-hand primitive; wire Hunter of Harmony and Volcano Tattoo (issue #190)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Generalize RequiredKeyword into a multi-keyword requirement primitive (issue #190)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Add handoff for the main-merge conflict resolution (issue #190)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -533,14 +533,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>41.0%</t>
+          <t>41.8%</t>
         </is>
       </c>
     </row>
@@ -587,14 +587,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.7%</t>
+          <t>2.8%</t>
         </is>
       </c>
     </row>
@@ -695,14 +695,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
@@ -26819,14 +26819,10 @@
       </c>
       <c r="E919" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="F919" t="inlineStr">
-        <is>
-          <t>Needs discard-pile keyword search (the "removed from game" zone it also needs is now built, issue #184).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="F919" t="inlineStr"/>
     </row>
     <row r="920">
       <c r="A920" t="inlineStr">
@@ -52371,7 +52367,7 @@
       </c>
       <c r="E1826" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1826" t="inlineStr"/>

</xml_diff>

<commit_message>
Deck-return/top-of-Fate-deck primitives; Goju House Guard, Aberrations, Focus-1 wave (#193)
* Deck-return and top-of-Fate-deck-discard primitives; wire Goju House Guard, Aberrations, and a Focus-1 Battle-action wave (issue #192)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Add handoff for the main-merge conflict resolution (issue #192)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Add handoff for the main-merge conflict resolution (issue #192)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -533,14 +533,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>41.8%</t>
+          <t>43.4%</t>
         </is>
       </c>
     </row>
@@ -551,14 +551,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C8" t="n">
         <v>127</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.1%</t>
+          <t>4.7%</t>
         </is>
       </c>
     </row>
@@ -587,14 +587,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.8%</t>
+          <t>3.0%</t>
         </is>
       </c>
     </row>
@@ -695,14 +695,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="C16" t="n">
         <v>2143</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
@@ -25119,14 +25119,10 @@
       </c>
       <c r="E863" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="F863" t="inlineStr">
-        <is>
-          <t>No "discard top of Fate deck" mechanic.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr"/>
     </row>
     <row r="864">
       <c r="A864" t="inlineStr">
@@ -26487,14 +26483,10 @@
       </c>
       <c r="E908" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="F908" t="inlineStr">
-        <is>
-          <t>Needs "put on top/bottom of own Fate deck as a cost" plus a mass bottom-of-deck effect.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="F908" t="inlineStr"/>
     </row>
     <row r="909">
       <c r="A909" t="inlineStr">
@@ -27228,7 +27220,7 @@
       </c>
       <c r="F932" t="inlineStr">
         <is>
-          <t>No "discard top of Fate deck" mechanic.</t>
+          <t>Focus 4, not 1 -- outside the #192 wave's own scope. The top-of-Fate-deck discard primitive now exists (Aberrations, issue #192), but this needs a "whose deck" target choice ("any Fate deck", not just your own) plus a variable-strength Melee Attack keyed off the discarded card's Focus Value, not a Force modifier.</t>
         </is>
       </c>
     </row>
@@ -29606,7 +29598,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1013" t="inlineStr"/>
+      <c r="F1013" t="inlineStr">
+        <is>
+          <t>Needs Chi as a repeatable payable cost resource (distinct from a Force/Stat modifier), interacting correctly with the existing Chi&lt;=0 death rule.</t>
+        </is>
+      </c>
     </row>
     <row r="1014">
       <c r="A1014" t="inlineStr">
@@ -30975,7 +30971,7 @@
       </c>
       <c r="E1062" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1062" t="inlineStr"/>
@@ -31227,7 +31223,7 @@
       </c>
       <c r="E1071" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1071" t="inlineStr"/>
@@ -31342,7 +31338,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1075" t="inlineStr"/>
+      <c r="F1075" t="inlineStr">
+        <is>
+          <t>Needs Dueling/Focus Effects (the Battle half, a plain Force debuff, is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1076">
       <c r="A1076" t="inlineStr">
@@ -31482,7 +31482,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1080" t="inlineStr"/>
+      <c r="F1080" t="inlineStr">
+        <is>
+          <t>Needs Dueling/Focus Effects (the Battle half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1081">
       <c r="A1081" t="inlineStr">
@@ -33386,7 +33390,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1148" t="inlineStr"/>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>Needs Rings (not built).</t>
+        </is>
+      </c>
     </row>
     <row r="1149">
       <c r="A1149" t="inlineStr">
@@ -34030,7 +34038,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1171" t="inlineStr"/>
+      <c r="F1171" t="inlineStr">
+        <is>
+          <t>Needs a keyword-conditional cost EXEMPTION (bow the performer unless it has a given keyword) -- distinct from every existing keyword-conditional EFFECT.</t>
+        </is>
+      </c>
     </row>
     <row r="1172">
       <c r="A1172" t="inlineStr">
@@ -34506,7 +34518,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1188" t="inlineStr"/>
+      <c r="F1188" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (similar shape to the existing move-to-battlefield-if-opposed patterns).</t>
+        </is>
+      </c>
     </row>
     <row r="1189">
       <c r="A1189" t="inlineStr">
@@ -34870,7 +34886,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1201" t="inlineStr"/>
+      <c r="F1201" t="inlineStr">
+        <is>
+          <t>Needs a delayed, multi-step revival mechanic ("before this turn ends, put a removed unit into play ignoring costs") -- not built.</t>
+        </is>
+      </c>
     </row>
     <row r="1202">
       <c r="A1202" t="inlineStr">
@@ -35094,7 +35114,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1209" t="inlineStr"/>
+      <c r="F1209" t="inlineStr">
+        <is>
+          <t>Needs an "after being targeted, negate" Reaction trigger (same gap as oracle-l5r-1292/10107).</t>
+        </is>
+      </c>
     </row>
     <row r="1210">
       <c r="A1210" t="inlineStr">
@@ -35486,7 +35510,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1223" t="inlineStr"/>
+      <c r="F1223" t="inlineStr">
+        <is>
+          <t>Needs an ability-copying mechanism (novel meta-effect; not built).</t>
+        </is>
+      </c>
     </row>
     <row r="1224">
       <c r="A1224" t="inlineStr">
@@ -36186,7 +36214,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1248" t="inlineStr"/>
+      <c r="F1248" t="inlineStr">
+        <is>
+          <t>Needs an "after being targeted" Reaction trigger (the Battle half, a plain Force boost, is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1249">
       <c r="A1249" t="inlineStr">
@@ -36270,7 +36302,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1251" t="inlineStr"/>
+      <c r="F1251" t="inlineStr">
+        <is>
+          <t>Needs a Gold-Cost comparison Target category plus a Gold-Cost-reduction effect (both novel).</t>
+        </is>
+      </c>
     </row>
     <row r="1252">
       <c r="A1252" t="inlineStr">
@@ -37250,7 +37286,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1286" t="inlineStr"/>
+      <c r="F1286" t="inlineStr">
+        <is>
+          <t>Needs a Retainer mechanic, movement to any location (not just home), and a province-card discard (three separate gaps).</t>
+        </is>
+      </c>
     </row>
     <row r="1287">
       <c r="A1287" t="inlineStr">
@@ -37502,7 +37542,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1295" t="inlineStr"/>
+      <c r="F1295" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (Discipline is already built; needs only a new "own opposed Personality" Target category).</t>
+        </is>
+      </c>
     </row>
     <row r="1296">
       <c r="A1296" t="inlineStr">
@@ -37922,7 +37966,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1310" t="inlineStr"/>
+      <c r="F1310" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (CardInstance.StraightenBlockedTurn already exists for the negate-next-straightening half; needs a new Paragon Performer category and an enemy-unit-card Target).</t>
+        </is>
+      </c>
     </row>
     <row r="1311">
       <c r="A1311" t="inlineStr">
@@ -37950,7 +37998,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1311" t="inlineStr"/>
+      <c r="F1311" t="inlineStr">
+        <is>
+          <t>Needs Regions (not built).</t>
+        </is>
+      </c>
     </row>
     <row r="1312">
       <c r="A1312" t="inlineStr">
@@ -38062,7 +38114,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1315" t="inlineStr"/>
+      <c r="F1315" t="inlineStr">
+        <is>
+          <t>Needs Dueling/Focus Effects (not started at all).</t>
+        </is>
+      </c>
     </row>
     <row r="1316">
       <c r="A1316" t="inlineStr">
@@ -38370,7 +38426,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1326" t="inlineStr"/>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (similar shape to the existing move-to-battlefield patterns, e.g. Journey's End).</t>
+        </is>
+      </c>
     </row>
     <row r="1327">
       <c r="A1327" t="inlineStr">
@@ -38566,7 +38626,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1333" t="inlineStr"/>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (RemoveFromGame and the discarded-personality Target already exist; needs a Shadowlands/Undead-conditional bonus amount).</t>
+        </is>
+      </c>
     </row>
     <row r="1334">
       <c r="A1334" t="inlineStr">
@@ -38678,7 +38742,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1337" t="inlineStr"/>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>Needs an ability-lock mechanism ("abilities on other cards in its unit may not be used") -- not built.</t>
+        </is>
+      </c>
     </row>
     <row r="1338">
       <c r="A1338" t="inlineStr">
@@ -38846,7 +38914,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1343" t="inlineStr"/>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>Needs a new Reaction trigger: "after an action resolves that a Personality performed" (the Terrain-play and additional-Battle-action halves are separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1344">
       <c r="A1344" t="inlineStr">
@@ -39714,7 +39786,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1374" t="inlineStr"/>
+      <c r="F1374" t="inlineStr">
+        <is>
+          <t>Needs an opponent-chooses-or-random discard mechanic (Reconnaissance-conditional).</t>
+        </is>
+      </c>
     </row>
     <row r="1375">
       <c r="A1375" t="inlineStr">
@@ -40190,7 +40266,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1391" t="inlineStr"/>
+      <c r="F1391" t="inlineStr">
+        <is>
+          <t>Needs a "before this battle resolves" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1392">
       <c r="A1392" t="inlineStr">
@@ -40218,7 +40298,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1392" t="inlineStr"/>
+      <c r="F1392" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (Monk Performer, attachment-destroy Target, and Fire-token-conditional Attack strength are all existing patterns, just not yet combined on one card).</t>
+        </is>
+      </c>
     </row>
     <row r="1393">
       <c r="A1393" t="inlineStr">
@@ -40414,7 +40498,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1399" t="inlineStr"/>
+      <c r="F1399" t="inlineStr">
+        <is>
+          <t>Needs a "before this battle resolves" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1400">
       <c r="A1400" t="inlineStr">
@@ -40722,7 +40810,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1410" t="inlineStr"/>
+      <c r="F1410" t="inlineStr">
+        <is>
+          <t>Needs a "before a card effect destroys a Personality, negate" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1411">
       <c r="A1411" t="inlineStr">
@@ -40834,7 +40926,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1414" t="inlineStr"/>
+      <c r="F1414" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (DiscardTopOfFateDeck, the Madness token, and an unattached-unit-card Target all now exist; needs resolving "a Fate deck"'s ownership the same way Aberrations did).</t>
+        </is>
+      </c>
     </row>
     <row r="1415">
       <c r="A1415" t="inlineStr">
@@ -40890,7 +40986,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1416" t="inlineStr"/>
+      <c r="F1416" t="inlineStr">
+        <is>
+          <t>Needs an Absent-Battle-timed Terrain-play variant (the existing one is Battle-timed only) plus a province-strength passive.</t>
+        </is>
+      </c>
     </row>
     <row r="1417">
       <c r="A1417" t="inlineStr">
@@ -41254,7 +41354,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1429" t="inlineStr"/>
+      <c r="F1429" t="inlineStr">
+        <is>
+          <t>Needs a two-performer selection (existing abilities support only one Performer) plus an army-unit-count comparison (both novel).</t>
+        </is>
+      </c>
     </row>
     <row r="1430">
       <c r="A1430" t="inlineStr">
@@ -41478,7 +41582,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1437" t="inlineStr"/>
+      <c r="F1437" t="inlineStr">
+        <is>
+          <t>Needs an "after being targeted" Reaction trigger (the additional-Battle-action half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1438">
       <c r="A1438" t="inlineStr">
@@ -41590,7 +41698,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1441" t="inlineStr"/>
+      <c r="F1441" t="inlineStr">
+        <is>
+          <t>Needs a unit-Force-total comparison Target (existing categories only compare individual card Force).</t>
+        </is>
+      </c>
     </row>
     <row r="1442">
       <c r="A1442" t="inlineStr">
@@ -41674,7 +41786,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1444" t="inlineStr"/>
+      <c r="F1444" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (an army-scoped keyword-conditional Force boost mirrors Utaku Elite Guard's existing pattern).</t>
+        </is>
+      </c>
     </row>
     <row r="1445">
       <c r="A1445" t="inlineStr">
@@ -41730,7 +41846,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1446" t="inlineStr"/>
+      <c r="F1446" t="inlineStr">
+        <is>
+          <t>Needs a movement-negation passive for a Terrain (the Terrain-play and additional-Battle-action halves are separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1447">
       <c r="A1447" t="inlineStr">
@@ -41758,7 +41878,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1447" t="inlineStr"/>
+      <c r="F1447" t="inlineStr">
+        <is>
+          <t>Needs a "before this battle's resolution" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1448">
       <c r="A1448" t="inlineStr">
@@ -41814,7 +41938,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1449" t="inlineStr"/>
+      <c r="F1449" t="inlineStr">
+        <is>
+          <t>Needs Equip from the discard pile (explicitly known gap, oracle-l5r-10681) plus a "before this battle resolves" destruction trigger.</t>
+        </is>
+      </c>
     </row>
     <row r="1450">
       <c r="A1450" t="inlineStr">
@@ -41898,7 +42026,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1452" t="inlineStr"/>
+      <c r="F1452" t="inlineStr">
+        <is>
+          <t>Needs a new tracked EnteredPlayTurn field on CardInstance (same gap as oracle-l5r-10335).</t>
+        </is>
+      </c>
     </row>
     <row r="1453">
       <c r="A1453" t="inlineStr">
@@ -41954,7 +42086,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1454" t="inlineStr"/>
+      <c r="F1454" t="inlineStr">
+        <is>
+          <t>Needs a "before this battle resolves" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1455">
       <c r="A1455" t="inlineStr">
@@ -42122,7 +42258,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1460" t="inlineStr"/>
+      <c r="F1460" t="inlineStr">
+        <is>
+          <t>Needs a self-replacing Terrain variant ("destroy a Terrain if able, then play this one") plus an ongoing army-wide Force passive tied to being in play as Terrain.</t>
+        </is>
+      </c>
     </row>
     <row r="1461">
       <c r="A1461" t="inlineStr">
@@ -42822,7 +42962,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1485" t="inlineStr"/>
+      <c r="F1485" t="inlineStr">
+        <is>
+          <t>Needs Equip from the discard pile (explicitly known gap, oracle-l5r-10681).</t>
+        </is>
+      </c>
     </row>
     <row r="1486">
       <c r="A1486" t="inlineStr">
@@ -42962,7 +43106,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1490" t="inlineStr"/>
+      <c r="F1490" t="inlineStr">
+        <is>
+          <t>Needs a "move an enemy Personality into the current battlefield" mechanic -- every existing move primitive moves the acting player's own cards, or moves a card home, never an opponent's card into battle.</t>
+        </is>
+      </c>
     </row>
     <row r="1491">
       <c r="A1491" t="inlineStr">
@@ -43382,7 +43530,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1505" t="inlineStr"/>
+      <c r="F1505" t="inlineStr">
+        <is>
+          <t>Needs a "before this battle resolves" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1506">
       <c r="A1506" t="inlineStr">
@@ -43522,7 +43674,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1510" t="inlineStr"/>
+      <c r="F1510" t="inlineStr">
+        <is>
+          <t>Needs a self-replacing Terrain variant plus an ongoing army-wide Force passive tied to being in play as Terrain (same two gaps as oracle-l5r-10941).</t>
+        </is>
+      </c>
     </row>
     <row r="1511">
       <c r="A1511" t="inlineStr">
@@ -43550,7 +43706,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1511" t="inlineStr"/>
+      <c r="F1511" t="inlineStr">
+        <is>
+          <t>Needs a unit-Force-total comparison Target (same gap as oracle-l5r-2900/4118).</t>
+        </is>
+      </c>
     </row>
     <row r="1512">
       <c r="A1512" t="inlineStr">
@@ -43578,7 +43738,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1512" t="inlineStr"/>
+      <c r="F1512" t="inlineStr">
+        <is>
+          <t>Needs an "after this battle resolves" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1513">
       <c r="A1513" t="inlineStr">
@@ -43662,7 +43826,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1515" t="inlineStr"/>
+      <c r="F1515" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (Discipline is already built; needs a standalone "attachment" Target category, a subset of the existing attachment-or-dishonorable-personality shape).</t>
+        </is>
+      </c>
     </row>
     <row r="1516">
       <c r="A1516" t="inlineStr">
@@ -43746,7 +43914,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1518" t="inlineStr"/>
+      <c r="F1518" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (own-personality Target, CardPersonalHonor, and dual Force/Chi modifiers all already exist; needs a new "unopposed" condition check).</t>
+        </is>
+      </c>
     </row>
     <row r="1519">
       <c r="A1519" t="inlineStr">
@@ -44166,7 +44338,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1533" t="inlineStr"/>
+      <c r="F1533" t="inlineStr">
+        <is>
+          <t>Needs a "count this card's own keywords, excluding a named pattern" mechanism (novel).</t>
+        </is>
+      </c>
     </row>
     <row r="1534">
       <c r="A1534" t="inlineStr">
@@ -44446,7 +44622,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1543" t="inlineStr"/>
+      <c r="F1543" t="inlineStr">
+        <is>
+          <t>Needs an exemption from the generic Battle-timing army-presence requirement (the adjacent-battlefield Performer shape itself, Moto Gunso's own, already exists).</t>
+        </is>
+      </c>
     </row>
     <row r="1544">
       <c r="A1544" t="inlineStr">
@@ -44474,7 +44654,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1544" t="inlineStr"/>
+      <c r="F1544" t="inlineStr">
+        <is>
+          <t>Needs the discard-to-hand "freshly drawn" primitive (in flight on a sibling PR, issue #190) plus an "after this battle ends" trigger for the optional return.</t>
+        </is>
+      </c>
     </row>
     <row r="1545">
       <c r="A1545" t="inlineStr">
@@ -44698,7 +44882,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1552" t="inlineStr"/>
+      <c r="F1552" t="inlineStr">
+        <is>
+          <t>Needs a dual-target selection with a relational constraint ("not sharing a Clan alignment") -- every existing multi-target category compares against a fixed performer/self, not between two chosen targets.</t>
+        </is>
+      </c>
     </row>
     <row r="1553">
       <c r="A1553" t="inlineStr">
@@ -44810,7 +44998,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1556" t="inlineStr"/>
+      <c r="F1556" t="inlineStr">
+        <is>
+          <t>Needs a general "attach any attachment from hand, at a Gold discount" Battle action, distinct from a Reserve/Spell-specific Equip variant.</t>
+        </is>
+      </c>
     </row>
     <row r="1557">
       <c r="A1557" t="inlineStr">
@@ -44838,7 +45030,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1557" t="inlineStr"/>
+      <c r="F1557" t="inlineStr">
+        <is>
+          <t>Needs a tracked "has the enemy leader taken a Battle action this battle" flag (novel state; the additional-Battle-actions half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1558">
       <c r="A1558" t="inlineStr">
@@ -44978,7 +45174,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1562" t="inlineStr"/>
+      <c r="F1562" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (an army-scoped Follower-presence-conditional Force passive mirrors Utaku Elite Guard's existing pattern).</t>
+        </is>
+      </c>
     </row>
     <row r="1563">
       <c r="A1563" t="inlineStr">
@@ -45146,7 +45346,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1568" t="inlineStr"/>
+      <c r="F1568" t="inlineStr">
+        <is>
+          <t>Needs Dueling/Focus Effects (not started at all).</t>
+        </is>
+      </c>
     </row>
     <row r="1569">
       <c r="A1569" t="inlineStr">
@@ -45258,7 +45462,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1572" t="inlineStr"/>
+      <c r="F1572" t="inlineStr">
+        <is>
+          <t>Needs an "after being targeted" Reaction trigger plus card creation (a temporary token Personality) -- both known gaps.</t>
+        </is>
+      </c>
     </row>
     <row r="1573">
       <c r="A1573" t="inlineStr">
@@ -45314,7 +45522,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1574" t="inlineStr"/>
+      <c r="F1574" t="inlineStr">
+        <is>
+          <t>Needs a non-AtBattle-gated compound Performer category for BattleOrOpen abilities (every existing keyword-Performer category requires the current battlefield).</t>
+        </is>
+      </c>
     </row>
     <row r="1575">
       <c r="A1575" t="inlineStr">
@@ -45342,7 +45554,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1575" t="inlineStr"/>
+      <c r="F1575" t="inlineStr">
+        <is>
+          <t>Needs a "count copies of this same card played this battle" mechanism (novel; the additional-Battle-action half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1576">
       <c r="A1576" t="inlineStr">
@@ -45454,7 +45670,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1579" t="inlineStr"/>
+      <c r="F1579" t="inlineStr">
+        <is>
+          <t>Needs a Gold-Cost comparison Target category (same gap as oracle-l5r-24).</t>
+        </is>
+      </c>
     </row>
     <row r="1580">
       <c r="A1580" t="inlineStr">
@@ -45678,7 +45898,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1587" t="inlineStr"/>
+      <c r="F1587" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (the opponent-chooses-effect shape, shinden-choice's own, already exists; needs a "was this negated" detection hook feeding a fallback effect).</t>
+        </is>
+      </c>
     </row>
     <row r="1588">
       <c r="A1588" t="inlineStr">
@@ -45818,7 +46042,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1592" t="inlineStr"/>
+      <c r="F1592" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (needs the same new "own opposed Personality" Target category noted for oracle-l5r-10929).</t>
+        </is>
+      </c>
     </row>
     <row r="1593">
       <c r="A1593" t="inlineStr">
@@ -46571,7 +46799,7 @@
       </c>
       <c r="E1619" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="F1619" t="inlineStr"/>
@@ -46686,7 +46914,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1623" t="inlineStr"/>
+      <c r="F1623" t="inlineStr">
+        <is>
+          <t>Needs an "actions must target this card if legal" redirect mechanic (same gap as oracle-l5r-10300).</t>
+        </is>
+      </c>
     </row>
     <row r="1624">
       <c r="A1624" t="inlineStr">
@@ -46882,7 +47114,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1630" t="inlineStr"/>
+      <c r="F1630" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (mirrors the existing Chi&lt;=0-after-modifier check pattern, applied to Force instead).</t>
+        </is>
+      </c>
     </row>
     <row r="1631">
       <c r="A1631" t="inlineStr">
@@ -47302,7 +47538,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1645" t="inlineStr"/>
+      <c r="F1645" t="inlineStr">
+        <is>
+          <t>Needs a non-AtBattle-gated Performer category ("at any location", same gap as oracle-l5r-5941).</t>
+        </is>
+      </c>
     </row>
     <row r="1646">
       <c r="A1646" t="inlineStr">
@@ -47442,7 +47682,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1650" t="inlineStr"/>
+      <c r="F1650" t="inlineStr">
+        <is>
+          <t>Needs an ongoing army-wide Force passive tied to being in play as Terrain (same gap as oracle-l5r-10941; the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1651">
       <c r="A1651" t="inlineStr">
@@ -47526,7 +47770,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1653" t="inlineStr"/>
+      <c r="F1653" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (Ninja Performer and Bow already exist; needs a province-card discard similar to Kharmic-discard's own).</t>
+        </is>
+      </c>
     </row>
     <row r="1654">
       <c r="A1654" t="inlineStr">
@@ -48590,7 +48838,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1691" t="inlineStr"/>
+      <c r="F1691" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (a dynamic Force-reduction-by-another-card's-Force and a sub-choice of which attachment to destroy are both close to existing patterns).</t>
+        </is>
+      </c>
     </row>
     <row r="1692">
       <c r="A1692" t="inlineStr">
@@ -48646,7 +48898,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1693" t="inlineStr"/>
+      <c r="F1693" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (a numeric-threshold Performer condition mirrors existing Force-threshold conditions elsewhere).</t>
+        </is>
+      </c>
     </row>
     <row r="1694">
       <c r="A1694" t="inlineStr">
@@ -48674,7 +48930,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1694" t="inlineStr"/>
+      <c r="F1694" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (single-card Force comparisons and a printed-Force threshold both already exist elsewhere).</t>
+        </is>
+      </c>
     </row>
     <row r="1695">
       <c r="A1695" t="inlineStr">
@@ -48702,7 +48962,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1695" t="inlineStr"/>
+      <c r="F1695" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (a dual-choice pattern sharing one UsageKey, Horibe's own shape, already exists).</t>
+        </is>
+      </c>
     </row>
     <row r="1696">
       <c r="A1696" t="inlineStr">
@@ -48814,7 +49078,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1699" t="inlineStr"/>
+      <c r="F1699" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (the Reaction half mirrors Khol Regulars' own -3 exactly; the Battle half needs a "defending Personality" Performer filter plus a before-battle-resolves straighten).</t>
+        </is>
+      </c>
     </row>
     <row r="1700">
       <c r="A1700" t="inlineStr">
@@ -49150,7 +49418,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1711" t="inlineStr"/>
+      <c r="F1711" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (the lower-or-equal-honor-than-performer Target already exists).</t>
+        </is>
+      </c>
     </row>
     <row r="1712">
       <c r="A1712" t="inlineStr">
@@ -49374,7 +49646,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1719" t="inlineStr"/>
+      <c r="F1719" t="inlineStr">
+        <is>
+          <t>Needs a "Political" Reaction timing (not built; the Battle half, a plain straighten, is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1720">
       <c r="A1720" t="inlineStr">
@@ -49598,7 +49874,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1727" t="inlineStr"/>
+      <c r="F1727" t="inlineStr">
+        <is>
+          <t>Needs Dueling/Focus Effects (the Battle half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1728">
       <c r="A1728" t="inlineStr">
@@ -49654,7 +49934,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1729" t="inlineStr"/>
+      <c r="F1729" t="inlineStr">
+        <is>
+          <t>Needs a self-replacing Terrain variant plus a delayed post-destruction straighten (two gaps, same self-replace gap as oracle-l5r-10941).</t>
+        </is>
+      </c>
     </row>
     <row r="1730">
       <c r="A1730" t="inlineStr">
@@ -50074,7 +50358,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1744" t="inlineStr"/>
+      <c r="F1744" t="inlineStr">
+        <is>
+          <t>Needs a new trigger keyed to passing instead of a Battle action (novel; the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1745">
       <c r="A1745" t="inlineStr">
@@ -50158,7 +50446,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1747" t="inlineStr"/>
+      <c r="F1747" t="inlineStr">
+        <is>
+          <t>Needs a "Political" Reaction timing (not built; the plain Ranged 1 Attack half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1748">
       <c r="A1748" t="inlineStr">
@@ -50466,7 +50758,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1758" t="inlineStr"/>
+      <c r="F1758" t="inlineStr">
+        <is>
+          <t>Needs a unit-Force-total comparison Target (same gap as oracle-l5r-2900) plus a per-card override of "a bowed card contributes no Force."</t>
+        </is>
+      </c>
     </row>
     <row r="1759">
       <c r="A1759" t="inlineStr">
@@ -50662,7 +50958,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1765" t="inlineStr"/>
+      <c r="F1765" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (a Spider-Clan-keyword Performer, dynamic Force reduction, and a conditional bow-if-Force-now-0 are each close to existing patterns).</t>
+        </is>
+      </c>
     </row>
     <row r="1766">
       <c r="A1766" t="inlineStr">
@@ -50914,7 +51214,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1774" t="inlineStr"/>
+      <c r="F1774" t="inlineStr">
+        <is>
+          <t>Needs a unit-Force-total comparison Target (same gap as oracle-l5r-2900).</t>
+        </is>
+      </c>
     </row>
     <row r="1775">
       <c r="A1775" t="inlineStr">
@@ -51026,7 +51330,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1778" t="inlineStr"/>
+      <c r="F1778" t="inlineStr">
+        <is>
+          <t>Needs an ongoing "negate all current and new Force penalties" effect (novel; the plain-straighten half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1779">
       <c r="A1779" t="inlineStr">
@@ -51250,7 +51558,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1786" t="inlineStr"/>
+      <c r="F1786" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (the Reaction half mirrors Khol Regulars' own -2; the Battle half is a move-to-an-opposed-battlefield variant of existing move mechanics).</t>
+        </is>
+      </c>
     </row>
     <row r="1787">
       <c r="A1787" t="inlineStr">
@@ -51474,7 +51786,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1794" t="inlineStr"/>
+      <c r="F1794" t="inlineStr">
+        <is>
+          <t>Needs a discard-pile-usable variant distinct from Discipline (its own printed ability, not a Discipline-keyword card).</t>
+        </is>
+      </c>
     </row>
     <row r="1795">
       <c r="A1795" t="inlineStr">
@@ -51642,7 +51958,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1800" t="inlineStr"/>
+      <c r="F1800" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (an optional bow-then-draw needs a small player choice, otherwise all existing patterns).</t>
+        </is>
+      </c>
     </row>
     <row r="1801">
       <c r="A1801" t="inlineStr">
@@ -51782,7 +52102,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1805" t="inlineStr"/>
+      <c r="F1805" t="inlineStr">
+        <is>
+          <t>Needs an "Interrupt" timing (not built; the plain Melee 2 Attack half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1806">
       <c r="A1806" t="inlineStr">
@@ -51810,7 +52134,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1806" t="inlineStr"/>
+      <c r="F1806" t="inlineStr">
+        <is>
+          <t>Needs a broad "before another player's action" Reaction trigger (existing triggers are narrow -- before an Attack, before an additional action -- not any action).</t>
+        </is>
+      </c>
     </row>
     <row r="1807">
       <c r="A1807" t="inlineStr">
@@ -52258,7 +52586,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1822" t="inlineStr"/>
+      <c r="F1822" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (the Set-Force pattern already exists, per oracle-l5r-543's own note).</t>
+        </is>
+      </c>
     </row>
     <row r="1823">
       <c r="A1823" t="inlineStr">
@@ -52314,7 +52646,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1824" t="inlineStr"/>
+      <c r="F1824" t="inlineStr">
+        <is>
+          <t>Needs an "after this battlefield's province is destroyed" Reaction trigger (the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1825">
       <c r="A1825" t="inlineStr">
@@ -52594,7 +52930,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1834" t="inlineStr"/>
+      <c r="F1834" t="inlineStr">
+        <is>
+          <t>Needs a "before an action's effect destroys a card, negate" Reaction trigger (same gap as oracle-l5r-2530; the Terrain-play half is separately wirable).</t>
+        </is>
+      </c>
     </row>
     <row r="1835">
       <c r="A1835" t="inlineStr">
@@ -52706,7 +53046,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F1838" t="inlineStr"/>
+      <c r="F1838" t="inlineStr">
+        <is>
+          <t>Not blocked; deferred for scope (Spirit-keyword Performer and MoveHome already exist; the 'will not be negated' clause just means never opening the reaction window for this specific move).</t>
+        </is>
+      </c>
     </row>
     <row r="1839">
       <c r="A1839" t="inlineStr">

</xml_diff>

<commit_message>
Rings concept: recruitment as an Additional Battle Action, Enlightenment victory (#197)
* Rings concept: recruitment as a granted Additional Battle Action, Enlightenment victory; wire 6 Rings plus Moshi Ikako and Scholarly Hermit (issue #194)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Add handoff for the main-merge conflict resolution (issue #194)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Add handoff for the main-merge conflict resolution (issue #194)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Add handoff for the main-merge conflict resolution round 2 (issue #194)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -15864,7 +15864,7 @@
       </c>
       <c r="F533" t="inlineStr">
         <is>
-          <t>Needs clarification on "Fire Battle:" (a Ring-gated Timing, unclear whether it depends on the not-yet-built Rings primitive) before wiring Moshi Ikako's own Ranged Attack.</t>
+          <t>Wired (issue #194) -- "Fire Battle" was confirmed to be a plain classification, not a Ring-gated Timing. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
         </is>
       </c>
     </row>
@@ -25512,7 +25512,7 @@
       </c>
       <c r="F876" t="inlineStr">
         <is>
-          <t>Needs an "after being targeted" Reaction trigger, plus Rings (not built).</t>
+          <t>Needs a retroactive partial-negation Reaction trigger ("after another player's action targets a card, negate just its bowing" -- existing triggers fully negate, or fire before resolution, never after with a partial effect). Rings themselves are now built (issue #194); "if you control any Rings" is trivial.</t>
         </is>
       </c>
     </row>
@@ -27788,7 +27788,7 @@
       </c>
       <c r="F951" t="inlineStr">
         <is>
-          <t>Needs Rings (not built).</t>
+          <t>Wired (issue #194) -- needed only a Ring-type check in a discard pile, now trivial. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
         </is>
       </c>
     </row>
@@ -61366,7 +61366,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2135" t="inlineStr"/>
+      <c r="F2135" t="inlineStr">
+        <is>
+          <t>Wired (issue #194) -- False Ring of Air. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
+        </is>
+      </c>
     </row>
     <row r="2136">
       <c r="A2136" t="inlineStr">
@@ -61394,7 +61398,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2136" t="inlineStr"/>
+      <c r="F2136" t="inlineStr">
+        <is>
+          <t>Needs Dueling/Focus Effects (not started at all) for False Ring of Earth's own recruitment condition.</t>
+        </is>
+      </c>
     </row>
     <row r="2137">
       <c r="A2137" t="inlineStr">
@@ -61422,7 +61430,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2137" t="inlineStr"/>
+      <c r="F2137" t="inlineStr">
+        <is>
+          <t>Needs an Interrupt timing (not built) for its own printed action, plus an adjustable maximum-hand-size mechanism (not built) for its own recruitment condition.</t>
+        </is>
+      </c>
     </row>
     <row r="2138">
       <c r="A2138" t="inlineStr">
@@ -61450,7 +61462,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2138" t="inlineStr"/>
+      <c r="F2138" t="inlineStr">
+        <is>
+          <t>Wired (issue #194) -- False Ring of Water. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
+        </is>
+      </c>
     </row>
     <row r="2139">
       <c r="A2139" t="inlineStr">
@@ -61478,7 +61494,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2139" t="inlineStr"/>
+      <c r="F2139" t="inlineStr">
+        <is>
+          <t>Needs an Engage timing (explicitly not started, #15) for its own printed action; its recruitment condition is otherwise wirable.</t>
+        </is>
+      </c>
     </row>
     <row r="2140">
       <c r="A2140" t="inlineStr">
@@ -61506,7 +61526,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2140" t="inlineStr"/>
+      <c r="F2140" t="inlineStr">
+        <is>
+          <t>Wired (issue #194) -- Ring of Air. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
+        </is>
+      </c>
     </row>
     <row r="2141">
       <c r="A2141" t="inlineStr">
@@ -61534,7 +61558,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2141" t="inlineStr"/>
+      <c r="F2141" t="inlineStr">
+        <is>
+          <t>Needs an Interrupt timing (not built) for Ring of Earth's own printed action; its recruitment condition is otherwise wirable.</t>
+        </is>
+      </c>
     </row>
     <row r="2142">
       <c r="A2142" t="inlineStr">
@@ -61562,7 +61590,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2142" t="inlineStr"/>
+      <c r="F2142" t="inlineStr">
+        <is>
+          <t>Set aside (issue #195) -- the local oracle data's own selected printing/text for this Emperor Edition card is uncertain; a user-supplied photo did not match either candidate text found.</t>
+        </is>
+      </c>
     </row>
     <row r="2143">
       <c r="A2143" t="inlineStr">
@@ -61590,7 +61622,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2143" t="inlineStr"/>
+      <c r="F2143" t="inlineStr">
+        <is>
+          <t>Wired (issue #194) -- Ring of Water. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
+        </is>
+      </c>
     </row>
     <row r="2144">
       <c r="A2144" t="inlineStr">
@@ -61618,7 +61654,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="F2144" t="inlineStr"/>
+      <c r="F2144" t="inlineStr">
+        <is>
+          <t>Wired (issue #194) -- Ring of the Void. Blocked only on its own scan image, not yet downloaded locally (issue #196).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Wire Front Rank Troops and Fudo's Fiends (issue #271)
Both cards' BLOCKERS notes claimed they needed a new Reaction trigger, but
MatchEngine.ExpendableDraw already exists and is already generically
correct for any card carrying the Expendable keyword -- checked at every
real destroy path (DestroyAttachment, DestroyUnits/MarkDead). Both cards'
only printed text is the keyword's own reminder text, so zero AbilityCatalog
wiring is needed. Adds the first direct regression test for ExpendableDraw,
which previously had none despite being live code.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -534,14 +534,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>44.3%</t>
+          <t>45.9%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C16" t="n">
         <v>2144</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.9%</t>
         </is>
       </c>
     </row>
@@ -31032,14 +31032,10 @@
       </c>
       <c r="F903" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G903" t="inlineStr">
-        <is>
-          <t>Needs an "after a card with this keyword dies" Reaction trigger (Expendable's own reminder).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G903" t="inlineStr"/>
     </row>
     <row r="904">
       <c r="A904" t="inlineStr">
@@ -31143,14 +31139,10 @@
       </c>
       <c r="F906" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G906" t="inlineStr">
-        <is>
-          <t>Needs an "after a card with this keyword dies" Reaction trigger (Expendable's own reminder).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G906" t="inlineStr"/>
     </row>
     <row r="907">
       <c r="A907" t="inlineStr">

</xml_diff>

<commit_message>
Wire Front Rank Troops and Fudo's Fiends (issue #271) (#272)
Both cards' BLOCKERS notes claimed they needed a new Reaction trigger, but
MatchEngine.ExpendableDraw already exists and is already generically
correct for any card carrying the Expendable keyword -- checked at every
real destroy path (DestroyAttachment, DestroyUnits/MarkDead). Both cards'
only printed text is the keyword's own reminder text, so zero AbilityCatalog
wiring is needed. Adds the first direct regression test for ExpendableDraw,
which previously had none despite being live code.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -534,14 +534,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>44.3%</t>
+          <t>45.9%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C16" t="n">
         <v>2144</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.9%</t>
         </is>
       </c>
     </row>
@@ -31032,14 +31032,10 @@
       </c>
       <c r="F903" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G903" t="inlineStr">
-        <is>
-          <t>Needs an "after a card with this keyword dies" Reaction trigger (Expendable's own reminder).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G903" t="inlineStr"/>
     </row>
     <row r="904">
       <c r="A904" t="inlineStr">
@@ -31143,14 +31139,10 @@
       </c>
       <c r="F906" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G906" t="inlineStr">
-        <is>
-          <t>Needs an "after a card with this keyword dies" Reaction trigger (Expendable's own reminder).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G906" t="inlineStr"/>
     </row>
     <row r="907">
       <c r="A907" t="inlineStr">

</xml_diff>

<commit_message>
Regenerate CARD_INVENTORY.xlsx after rebasing onto origin/main
Picks up Front Rank Troops/Fudo's Fiends (Follower wave 10, merged
concurrently) alongside this branch's own 3 cards: 322 wired total.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -534,14 +534,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>45.9%</t>
+          <t>47.5%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C16" t="n">
         <v>2144</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
@@ -31024,14 +31024,10 @@
       </c>
       <c r="F903" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G903" t="inlineStr">
-        <is>
-          <t>Needs an "after a card with this keyword dies" Reaction trigger (Expendable's own reminder).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G903" t="inlineStr"/>
     </row>
     <row r="904">
       <c r="A904" t="inlineStr">
@@ -31135,14 +31131,10 @@
       </c>
       <c r="F906" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G906" t="inlineStr">
-        <is>
-          <t>Needs an "after a card with this keyword dies" Reaction trigger (Expendable's own reminder).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G906" t="inlineStr"/>
     </row>
     <row r="907">
       <c r="A907" t="inlineStr">

</xml_diff>

<commit_message>
Complete Follower wave 14: engine primitives, publication, tests, inventory, handoff
Follow-up to 074a4b6 (which only committed the six new card-art copies due to a
pathspec mistake) -- the same logical change, completing it: CardAbilities.cs/
MatchEngine.cs/Models.cs/PublishedContent.cs/CardCatalog.cs primitives,
content/published/follower-wave-14.json(-sources.json), the packaging script,
regression tests, the regenerated card inventory, the six-entry BLOCKERS cleanup,
and the task handoff. See 074a4b6's own message for the full description.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -534,14 +534,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>51.6%</t>
+          <t>56.6%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="C16" t="n">
         <v>2144</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.9%</t>
         </is>
       </c>
     </row>
@@ -29785,14 +29785,10 @@
       </c>
       <c r="F868" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G868" t="inlineStr">
-        <is>
-          <t>Not blocked; deferred for scope (dual-choice Set-Force pattern already exists).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G868" t="inlineStr"/>
     </row>
     <row r="869">
       <c r="A869" t="inlineStr">
@@ -31922,14 +31918,10 @@
       </c>
       <c r="F929" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G929" t="inlineStr">
-        <is>
-          <t>Not fully blocked; entry Honor loss and a self-Force-keyed Attack strength both reuse existing patterns, but needs verification that AttackStrength can read its own source's Force at validation time.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G929" t="inlineStr"/>
     </row>
     <row r="930">
       <c r="A930" t="inlineStr">
@@ -33660,14 +33652,10 @@
       </c>
       <c r="F979" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G979" t="inlineStr">
-        <is>
-          <t>Not blocked; deferred for scope (existing entry-Reaction plus a simple province-destruction count).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G979" t="inlineStr"/>
     </row>
     <row r="980">
       <c r="A980" t="inlineStr">
@@ -33697,14 +33685,10 @@
       </c>
       <c r="F980" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G980" t="inlineStr">
-        <is>
-          <t>Not blocked; deferred for scope (existing entry-Honor-loss, Conqueror-grant, and Attack patterns).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G980" t="inlineStr"/>
     </row>
     <row r="981">
       <c r="A981" t="inlineStr">
@@ -33771,14 +33755,10 @@
       </c>
       <c r="F982" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G982" t="inlineStr">
-        <is>
-          <t>Not blocked; pure attach restriction with no ability text, deferred for scope.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G982" t="inlineStr"/>
     </row>
     <row r="983">
       <c r="A983" t="inlineStr">
@@ -33841,14 +33821,10 @@
       </c>
       <c r="F984" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G984" t="inlineStr">
-        <is>
-          <t>Not blocked; deferred for scope (existing entry-Honor-loss pattern; carries the Legionnaire keyword Aulus's boost needs).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G984" t="inlineStr"/>
     </row>
     <row r="985">
       <c r="A985" t="inlineStr">

</xml_diff>

<commit_message>
Wire Brawl (oracle-l5r-1127) as strategy-wave-16
Its "Needs Regions (not built)" blocker was stale: Regions and Terrains
already existed. Adds the region-or-terrain Target (exempt from the
Battle-timing at-battlefield Require, since a Region sits in Zone.Region),
a DestroyRegion helper mirroring province-destruction's Region discard,
and the paired brawl-bow / brawl-destroy abilities. Client FindCard now
searches ProvinceView.Region so a Region target resolves in the picker.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
@@ -44715,14 +44715,10 @@
       </c>
       <c r="F1314" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1314" t="inlineStr">
-        <is>
-          <t>Needs Regions (not built).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1314" t="inlineStr"/>
     </row>
     <row r="1315">
       <c r="A1315" t="inlineStr">

</xml_diff>

<commit_message>
Wire Brawl (oracle-l5r-1127) as strategy-wave-16 (#306)
Its "Needs Regions (not built)" blocker was stale: Regions and Terrains
already existed. Adds the region-or-terrain Target (exempt from the
Battle-timing at-battlefield Require, since a Region sits in Zone.Region),
a DestroyRegion helper mirroring province-destruction's Region discard,
and the paired brawl-bow / brawl-destroy abilities. Client FindCard now
searches ProvinceView.Region so a Region target resolves in the picker.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
@@ -44715,14 +44715,10 @@
       </c>
       <c r="F1314" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1314" t="inlineStr">
-        <is>
-          <t>Needs Regions (not built).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1314" t="inlineStr"/>
     </row>
     <row r="1315">
       <c r="A1315" t="inlineStr">

</xml_diff>

<commit_message>
Wire Akodo Kakihara (personality-wave-23): react when another player's action or Attack targets him (#305)
Reaction: after another player's action targets Kakihara, give him a Force
bonus equal to his (current) Personal Honor. His BLOCKERS note was stale: the
general in-play targeting Reaction primitive (#278) already existed.

Non-Attack actions reach him through a new KakiharaWatcher branch of the
existing beforeActionReaction window; Ranged/Melee Attacks through the existing
attackReaction window, so the bonus lands before the strength comparison and
changes the outcome. One printed ability, two catalog entries sharing one
UsageKey. Dishonored (PH 0) opens no window; own-controller actions, Reactions,
bowed, spent and not-in-play cases never trigger it. QueryActions now lists the
beforeActionReaction window's own reactions and validates the attackReaction
ones. Scan-verified; text follows the scan (colon, not comma).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>25.2%</t>
+          <t>25.3%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
@@ -2853,14 +2853,10 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>Needs a broad 'after another player's action targets this card' Reaction trigger (the single largest recurring gap across multiple waves).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">

</xml_diff>

<commit_message>
Wire Daidoji Ebizo (personality-wave-26) and Master Scouts (follower-wave-15): the Recon-action classification and the "after the resolution of your [keyword] action" trait (#321, #309)
- ActionCarriesKeyword: an action carries a keyword when its ability prints it (AbilityDefinition.ActionKeywords) or its card has it.
- AfterOwnActionTraits / FireAfterOwnActionTraits: a mandatory, repeatable trait fired from the ability funnel and from deferred Attack and duel resolution; Ebizo's +1F is an ApplyModifier (until end of turn).
- ebizo-attack: Ranged Attack with strength equal to his live Force. Master Scouts is the same Effect on a Follower.

Decision doc: docs/decisions/2026-09-18-recon-action-tag-and-daidoji-ebizo.md

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>25.5%</t>
+          <t>25.6%</t>
         </is>
       </c>
     </row>
@@ -534,14 +534,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>56.6%</t>
+          <t>57.4%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
@@ -6886,14 +6886,10 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G185" t="inlineStr">
-        <is>
-          <t>Needs a new Reaction trigger: "after the resolution of your Recon action" (the same gap as oracle-l5r-4867); the Ranged Attack strength equal to Ebizo's own Force is separately wirable (AttackStrength already takes a sourceId parameter, and CardForce is a generic helper).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -32061,14 +32057,10 @@
       </c>
       <c r="F936" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G936" t="inlineStr">
-        <is>
-          <t>Needs a new Reaction trigger: "after a Recon action resolves."</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G936" t="inlineStr"/>
     </row>
     <row r="937">
       <c r="A937" t="inlineStr">

</xml_diff>

<commit_message>
Add the look-at-the-top-N-cards primitive; wire Public Records, Isawa Tamaki, Banish All Doubt, Bayushi Kahoku exp2 and Signs and Portents (#322)
A private, engine-authoritative arrangement of the top N cards of a chosen deck (own or the opponent's): one arrangeTopCards command, per-card legal dispositions with min/max enforced, no shuffle, and a shared deferred-action tail with the deck search.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>25.5%</t>
+          <t>25.7%</t>
         </is>
       </c>
     </row>
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
@@ -606,14 +606,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" t="n">
         <v>149</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>8.7%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
@@ -624,14 +624,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
@@ -3410,7 +3410,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>The Phoenix-opposition Force bonus is directly wirable (reuses this wave's own clan-conditional attacking-vs-dragon-bonus pattern); blocked only by its Limited ability -- 'look at the top Fate card and choose to leave/discard/bottom it' (no look-then-choose deck-top primitive exists; DiscardTopOfFateDeck is one-way only).</t>
+          <t>The Phoenix-opposition Force bonus is directly wirable (reuses this wave's own clan-conditional attacking-vs-dragon-bonus pattern). Its Limited ability is now expressible: the look-at-the-top-N-cards primitive (issue #322, DeckLook.cs) covers 'look at the top Fate card; leave it, discard it, or put it at the bottom' as a LookSpec (N=1, own Fate, discard 0-1, bottom 0-1) -- unblocked, deliberately not wired in that PR.</t>
         </is>
       </c>
     </row>
@@ -5529,7 +5529,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G144" t="inlineStr"/>
@@ -12947,7 +12947,7 @@
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G366" t="inlineStr"/>
@@ -15508,7 +15508,7 @@
       </c>
       <c r="G442" t="inlineStr">
         <is>
-          <t>Needs a deck-search primitive (look at the top three cards of a Fate deck, conditionally take one matching a printed criterion, put the rest back in chosen order) -- an established, still-unbuilt gap (deck search).</t>
+          <t>The look-at-the-top-N-cards primitive (issue #322) covers 'look at the top three cards of your Fate deck, show an Iaijutsu Strategy and put it into your hand, put the remaining cards back in any order' (a show disposition with criteria, exactly Bayushi Kahoku exp2's shape). Still needs the follow-up 'then discard a card' (the same after-effect step Ikoma Shizuka's Terrain half has in the deck search) and an Iaijutsu Strategy criteria check -- not wired in that PR.</t>
         </is>
       </c>
     </row>
@@ -38898,7 +38898,7 @@
       </c>
       <c r="G1140" t="inlineStr">
         <is>
-          <t>Needs a look-then-reorder deck-top primitive ('look at the top three cards of your Fate or Dynasty deck, put one or two on the bottom, the rest on top in any order') -- the same still-unbuilt gap noted at oracle-l5r-305, here compounded by a choice of WHICH deck (Fate or Dynasty) to look at, itself unprecedented.</t>
+          <t>The look-at-the-top-N-cards primitive (issue #322) covers the look itself: N=3, a choice of own Fate or own Dynasty deck, one or two cards may go to the bottom, the rest back on top in any order (LookCatalog.TrainingAny is the same shape). Still needs its cost 'Bow this Shugenja unless he is Void' and its Spell attachment plumbing (a Limited ability on an attached Spell whose performer is its wielder) -- not wired in that PR.</t>
         </is>
       </c>
     </row>
@@ -44134,7 +44134,7 @@
       </c>
       <c r="F1297" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1297" t="inlineStr"/>
@@ -64985,7 +64985,7 @@
       </c>
       <c r="F1920" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1920" t="inlineStr"/>
@@ -69180,7 +69180,7 @@
       </c>
       <c r="F2047" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2047" t="inlineStr"/>
@@ -70707,7 +70707,7 @@
       </c>
       <c r="G2093" t="inlineStr">
         <is>
-          <t>Needs a look-then-optional-discard primitive for its own Limited half ('look at the top card of your Fate deck, you may discard it') -- the same still-unbuilt gap noted at oracle-l5r-305 (DiscardTopOfFateDeck only ever discards unconditionally, one-way). Its own Open half (retrieve a non-Unique Strategy from your Fate discard pile to hand) directly reuses hunter-of-harmony-return/scholarly-hermit-search's shape and is separately wirable.</t>
+          <t>Its Limited half ('look at the top card of your Fate deck; you may discard it') is now expressible with the look-at-the-top-N-cards primitive (issue #322: N=1, own Fate, discard 0-1) -- unblocked, deliberately not wired in that PR. Its own Open half (retrieve a non-Unique Strategy from your Fate discard pile to hand) directly reuses hunter-of-harmony-return/scholarly-hermit-search's shape and is separately wirable.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire Daidoji Ebizo (personality-wave-26) and Master Scouts (follower-wave-15): the Recon-action classification and the "after the resolution of your [keyword] action" trait (#321, #309) (#326)
- ActionCarriesKeyword: an action carries a keyword when its ability prints it (AbilityDefinition.ActionKeywords) or its card has it.
- AfterOwnActionTraits / FireAfterOwnActionTraits: a mandatory, repeatable trait fired from the ability funnel and from deferred Attack and duel resolution; Ebizo's +1F is an ApplyModifier (until end of turn).
- ebizo-attack: Ranged Attack with strength equal to his live Force. Master Scouts is the same Effect on a Follower.

Decision doc: docs/decisions/2026-09-18-recon-action-tag-and-daidoji-ebizo.md

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>25.5%</t>
+          <t>25.6%</t>
         </is>
       </c>
     </row>
@@ -534,14 +534,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>56.6%</t>
+          <t>57.4%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
@@ -6886,14 +6886,10 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G185" t="inlineStr">
-        <is>
-          <t>Needs a new Reaction trigger: "after the resolution of your Recon action" (the same gap as oracle-l5r-4867); the Ranged Attack strength equal to Ebizo's own Force is separately wirable (AttackStrength already takes a sourceId parameter, and CardForce is a generic helper).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -32061,14 +32057,10 @@
       </c>
       <c r="F936" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G936" t="inlineStr">
-        <is>
-          <t>Needs a new Reaction trigger: "after a Recon action resolves."</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G936" t="inlineStr"/>
     </row>
     <row r="937">
       <c r="A937" t="inlineStr">

</xml_diff>

<commit_message>
Add the look-at-the-top-N-cards primitive; wire Public Records, Isawa Tamaki, Banish All Doubt, Bayushi Kahoku exp2 and Signs and Portents (#322) (#329)
A private, engine-authoritative arrangement of the top N cards of a chosen deck (own or the opponent's): one arrangeTopCards command, per-card legal dispositions with min/max enforced, no shuffle, and a shared deferred-action tail with the deck search.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>25.5%</t>
+          <t>25.7%</t>
         </is>
       </c>
     </row>
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
@@ -606,14 +606,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" t="n">
         <v>149</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>8.7%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
@@ -624,14 +624,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
@@ -3410,7 +3410,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>The Phoenix-opposition Force bonus is directly wirable (reuses this wave's own clan-conditional attacking-vs-dragon-bonus pattern); blocked only by its Limited ability -- 'look at the top Fate card and choose to leave/discard/bottom it' (no look-then-choose deck-top primitive exists; DiscardTopOfFateDeck is one-way only).</t>
+          <t>The Phoenix-opposition Force bonus is directly wirable (reuses this wave's own clan-conditional attacking-vs-dragon-bonus pattern). Its Limited ability is now expressible: the look-at-the-top-N-cards primitive (issue #322, DeckLook.cs) covers 'look at the top Fate card; leave it, discard it, or put it at the bottom' as a LookSpec (N=1, own Fate, discard 0-1, bottom 0-1) -- unblocked, deliberately not wired in that PR.</t>
         </is>
       </c>
     </row>
@@ -5529,7 +5529,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G144" t="inlineStr"/>
@@ -12947,7 +12947,7 @@
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G366" t="inlineStr"/>
@@ -15508,7 +15508,7 @@
       </c>
       <c r="G442" t="inlineStr">
         <is>
-          <t>Needs a deck-search primitive (look at the top three cards of a Fate deck, conditionally take one matching a printed criterion, put the rest back in chosen order) -- an established, still-unbuilt gap (deck search).</t>
+          <t>The look-at-the-top-N-cards primitive (issue #322) covers 'look at the top three cards of your Fate deck, show an Iaijutsu Strategy and put it into your hand, put the remaining cards back in any order' (a show disposition with criteria, exactly Bayushi Kahoku exp2's shape). Still needs the follow-up 'then discard a card' (the same after-effect step Ikoma Shizuka's Terrain half has in the deck search) and an Iaijutsu Strategy criteria check -- not wired in that PR.</t>
         </is>
       </c>
     </row>
@@ -38898,7 +38898,7 @@
       </c>
       <c r="G1140" t="inlineStr">
         <is>
-          <t>Needs a look-then-reorder deck-top primitive ('look at the top three cards of your Fate or Dynasty deck, put one or two on the bottom, the rest on top in any order') -- the same still-unbuilt gap noted at oracle-l5r-305, here compounded by a choice of WHICH deck (Fate or Dynasty) to look at, itself unprecedented.</t>
+          <t>The look-at-the-top-N-cards primitive (issue #322) covers the look itself: N=3, a choice of own Fate or own Dynasty deck, one or two cards may go to the bottom, the rest back on top in any order (LookCatalog.TrainingAny is the same shape). Still needs its cost 'Bow this Shugenja unless he is Void' and its Spell attachment plumbing (a Limited ability on an attached Spell whose performer is its wielder) -- not wired in that PR.</t>
         </is>
       </c>
     </row>
@@ -44134,7 +44134,7 @@
       </c>
       <c r="F1297" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1297" t="inlineStr"/>
@@ -64985,7 +64985,7 @@
       </c>
       <c r="F1920" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1920" t="inlineStr"/>
@@ -69180,7 +69180,7 @@
       </c>
       <c r="F2047" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2047" t="inlineStr"/>
@@ -70707,7 +70707,7 @@
       </c>
       <c r="G2093" t="inlineStr">
         <is>
-          <t>Needs a look-then-optional-discard primitive for its own Limited half ('look at the top card of your Fate deck, you may discard it') -- the same still-unbuilt gap noted at oracle-l5r-305 (DiscardTopOfFateDeck only ever discards unconditionally, one-way). Its own Open half (retrieve a non-Unique Strategy from your Fate discard pile to hand) directly reuses hunter-of-harmony-return/scholarly-hermit-search's shape and is separately wirable.</t>
+          <t>Its Limited half ('look at the top card of your Fate deck; you may discard it') is now expressible with the look-at-the-top-N-cards primitive (issue #322: N=1, own Fate, discard 0-1) -- unblocked, deliberately not wired in that PR. Its own Open half (retrieve a non-Unique Strategy from your Fate discard pile to hand) directly reuses hunter-of-harmony-return/scholarly-hermit-search's shape and is separately wirable.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daidoji Yuki grants Reconnaissance to his controller as Attacker or Defender
Rules lead's ruling: the all-Scouts condition alone decides the grant, on either
side. A Defender's grant sits at their own province; the opponent gains nothing.
Every Reconnaissance reader (Hiruma Sniper, Keppo, the training strike) now asks
"does this player have it at the current battlefield" instead of addressing the
province owner as 1 - player, which only ever answered for an Attacker.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -32536,7 +32536,7 @@
       </c>
       <c r="G950" t="inlineStr">
         <is>
-          <t>The Engage window and first-action claim now exist (issue #310; a Follower's 'Engage:' is a Reaction to trigger after-engaging, claim: MatchEngine.ClaimFirstOpportunity, conditional on being the Attacker). Still needs: a Follower-sourced Engage action scoped to 'this battlefield' (the Follower's own unit) and its optional 'you may target ... -3F' effect target; Reconnaissance is only ever held by the Attacker at present (a defending Follower's grant is a no-op, see docs/decisions/2026-09-18-battle-timing-primitives.md).</t>
+          <t>The Engage window and first-action claim now exist (issue #310; a Follower's 'Engage:' is a Reaction to trigger after-engaging, claim: MatchEngine.ClaimFirstOpportunity, conditional on being the Attacker). Still needs: a Follower-sourced Engage action scoped to 'this battlefield' (the Follower's own unit) and its optional 'you may target ... -3F' effect target; Reconnaissance for the acting side is settled (MatchEngine.GrantReconnaissanceAtCurrentBattlefield serves an Attacker at the enemy's province and a Defender at their own, see docs/decisions/2026-09-18-battle-timing-primitives.md decision 5).</t>
         </is>
       </c>
     </row>
@@ -33681,7 +33681,7 @@
       </c>
       <c r="G983" t="inlineStr">
         <is>
-          <t>The Engage window now exists (issue #310); its 'Recon Reaction: After engaging at this card's battlefield' is Trigger after-engaging-at-own-battlefield (a Follower's own battlefield is its host's) with ActionKeywords ["Recon"]. Still needs: 'give your other Followers there +1F' (a per-Follower ApplyModifier sweep over the unit's siblings and the army's other Followers) and the Reconnaissance grant (Attacker only at present, see docs/decisions/2026-09-18-battle-timing-primitives.md).</t>
+          <t>The Engage window now exists (issue #310); its 'Recon Reaction: After engaging at this card's battlefield' is Trigger after-engaging-at-own-battlefield (a Follower's own battlefield is its host's) with ActionKeywords ["Recon"]. Still needs: 'give your other Followers there +1F' (a per-Follower ApplyModifier sweep over the unit's siblings and the army's other Followers) and the Reconnaissance grant (already built for either side: MatchEngine.GrantReconnaissanceAtCurrentBattlefield, see docs/decisions/2026-09-18-battle-timing-primitives.md decision 5).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WIP: Daigotsu Bofana (base and exp): once-per-phase limit, generalized forced discard, discard-pile additional action (issue #333)
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>26.9%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>19.1%</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Needs Bushido Virtue as a targetable/filterable Strategy sub-classification (Discipline's own 'play from discard, remove from game after' mechanism is built and partly reusable, but gated here behind an Additional Action and a Bushido-Virtue-specific discard-pile filter).</t>
+          <t>Needs Bushido Virtue as a targetable/filterable Strategy sub-classification (the general "take an additional action to play a discard-pile card, then remove it from the game" is built for Daigotsu Bofana - exp's Dark Virtue: AdditionalActionGrant.FromDiscard, own-dark-virtue-in-discard), his "discard a card" cost, and Battle, Limited or Open "as appropriate to the current phase" -- that grant is only ever consumed by a Battle action.</t>
         </is>
       </c>
     </row>
@@ -7546,14 +7546,10 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G205" t="inlineStr">
-        <is>
-          <t>Needs a broad "after another player's action targets this card" Reaction trigger (the same gap as oracle-l5r-223, the single largest recurring gap across multiple waves), plus a once-per-PHASE usage dedupe distinct from the engine's existing once-per-TURN AbilityUses stamp -- a second, independent gap.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -7583,7 +7579,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G206" t="inlineStr"/>
@@ -32396,7 +32392,7 @@
       </c>
       <c r="G946" t="inlineStr">
         <is>
-          <t>Needs a "negate the first Political action against this card each phase" mechanism (the flat +1PH half is separately wirable).</t>
+          <t>Needs a way for a TRAIT to negate the announced Political action's remaining effects, plus a Political-action classification (the flat +1PH half is separately wirable). The "first time each phase" half now exists: the once-per-phase limit (PhaseLimits.cs) and the announce-time targeting trait hook (Daigotsu Bofana, MatchEngine.OpenForcedDiscardForTargetedTrait).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire Daigotsu Bofana and Bofana - exp (personality-wave-29): once-per-phase limit, forced discard, discard-pile play (#334)
* WIP: Daigotsu Bofana (base and exp): once-per-phase limit, generalized forced discard, discard-pile additional action (issue #333)

* Daigotsu Bofana decision note, handoff, direct-command Dark Virtue target check (issue #333)

* WIP: per-action same-turn rule, Proclaim-first ordering, tests (issue #333)

* Bofana: per-action same-turn rule, Proclaim gain before entering effects, decision note records Mendon's rulings (issue #333)
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>26.9%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>19.1%</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Needs Bushido Virtue as a targetable/filterable Strategy sub-classification (Discipline's own 'play from discard, remove from game after' mechanism is built and partly reusable, but gated here behind an Additional Action and a Bushido-Virtue-specific discard-pile filter).</t>
+          <t>Needs Bushido Virtue as a targetable/filterable Strategy sub-classification (the general "take an additional action to play a discard-pile card, then remove it from the game" is built for Daigotsu Bofana - exp's Dark Virtue: AdditionalActionGrant.FromDiscard, own-dark-virtue-in-discard), his "discard a card" cost, and Battle, Limited or Open "as appropriate to the current phase" -- that grant is only ever consumed by a Battle action.</t>
         </is>
       </c>
     </row>
@@ -7546,14 +7546,10 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G205" t="inlineStr">
-        <is>
-          <t>Needs a broad "after another player's action targets this card" Reaction trigger (the same gap as oracle-l5r-223, the single largest recurring gap across multiple waves), plus a once-per-PHASE usage dedupe distinct from the engine's existing once-per-TURN AbilityUses stamp -- a second, independent gap.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -7583,7 +7579,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G206" t="inlineStr"/>
@@ -32396,7 +32392,7 @@
       </c>
       <c r="G946" t="inlineStr">
         <is>
-          <t>Needs a "negate the first Political action against this card each phase" mechanism (the flat +1PH half is separately wirable).</t>
+          <t>Needs a way for a TRAIT to negate the announced Political action's remaining effects, plus a Political-action classification (the flat +1PH half is separately wirable). The "first time each phase" half now exists: the once-per-phase limit (PhaseLimits.cs) and the announce-time targeting trait hook (Daigotsu Bofana, MatchEngine.OpenForcedDiscardForTargetedTrait).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WIP: decision note, BLOCKERS, inventory, AI test, Blade own-cards test, Strategy-attack redirect test (issue #335)
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>26.9%</t>
+          <t>27.4%</t>
         </is>
       </c>
     </row>
@@ -552,14 +552,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C8" t="n">
         <v>127</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.7%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>19.3%</t>
         </is>
       </c>
     </row>
@@ -9872,14 +9872,10 @@
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G275" t="inlineStr">
-        <is>
-          <t>Needs an "after being targeted" Reaction trigger (the same gap as oracle-l5r-1292/10107/7767) to react to another player's Battle action targeting Yurishi, plus a conditional negation keyed on whether the moved card is still a legal target for the original action -- a second novel piece on top of the trigger itself.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -10569,14 +10565,10 @@
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G296" t="inlineStr">
-        <is>
-          <t>Needs an "after being targeted" Reaction trigger (the same gap as oracle-l5r-1292/10107/7767), a twice-per-turn usage counter (the existing dedupe is strictly once-per-turn -- the same still-unbuilt gap noted for oracle-l5r-9827's three-times-per-turn case), and negating TWO named effects (bowing AND destruction) from one action at once -- NegatedEffectKind is a single string field, only ever one effect kind at a time (Rokai's destroy, Tamoko's move-or-straighten) -- three compounding gaps.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -17614,14 +17606,10 @@
       </c>
       <c r="F505" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G505" t="inlineStr">
-        <is>
-          <t>Needs a target-redirection mechanism (another player's action, once targeted, is redirected to a different card instead) -- an established gap, the same family already deferred for Yoritomo Naoto (see the Reserve primitive row).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr"/>
     </row>
     <row r="506">
       <c r="A506" t="inlineStr">
@@ -27904,14 +27892,10 @@
       </c>
       <c r="F815" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G815" t="inlineStr">
-        <is>
-          <t>Needs a generic "after another player's action targets one of your cards, negate its effects unless the acting player pays a cost" Reaction mechanism for its Political Reaction half -- distinct from the existing before-action-resolves negation (Rokai/Tamoko), which is a curated classification that only ever negates destruction OR movement/straightening specifically, never a blanket "negate the action's effects," and is never conditioned on the AFFECTED player's own optional payment; its Political Open half (straighten a Holding or Stronghold) is separately wirable: the any-holding Target it needs already exists (Yasuki Tsujiken's own -- personality-wave-22, issue #301, wired oracle-l5r-142/3866 through it, contrary to those two cards' own old notes claiming a new Holding Target was needed), so only the Stronghold half of the union would be new.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G815" t="inlineStr"/>
     </row>
     <row r="816">
       <c r="A816" t="inlineStr">
@@ -29039,7 +29023,7 @@
       </c>
       <c r="G849" t="inlineStr">
         <is>
-          <t>Needs an "actions must target this card if legal" redirect mechanic (Yoritomo Naoto's own Battle ability), on top of its own Additional Action grant.</t>
+          <t>Needs an "actions must target this card if legal" forced-redirection rule (Yoritomo Naoto's own Battle ability), on top of its own Additional Action grant. The legality half now exists (ActionAcceptsTarget, issue #335 -- "if legal" is that check); the standing hook that applies it to every action is the gap.</t>
         </is>
       </c>
     </row>
@@ -32355,7 +32339,7 @@
       </c>
       <c r="G945" t="inlineStr">
         <is>
-          <t>Needs an "after being targeted, negate" Reaction trigger.</t>
+          <t>The in-play "after another player's action targets a card in this unit: negate the action's effects on this card" Reaction exists (Champion of Thunder's champion-of-thunder-negate, own-unit-member target, the blanket "all" negation; issue #278) and so does the trigger family it now shares (issue #335, TargetedActionReactions.cs). Directly wirable as a second carrier of champion-of-thunder-negate; not yet wired.</t>
         </is>
       </c>
     </row>
@@ -33570,7 +33554,7 @@
       </c>
       <c r="G980" t="inlineStr">
         <is>
-          <t>Needs two new Reaction triggers (after its own bow; after being targeted, negate destruction).</t>
+          <t>Needs an "after this card bows" Reaction trigger plus negating its own future straightening (the second trait); the first ("After another player's action targets a card in this unit: Negate this card's destruction") is now expressible through the targeted-by-action trigger and NegateEffects(card, "destroy") (issue #335).</t>
         </is>
       </c>
     </row>
@@ -34105,14 +34089,10 @@
       </c>
       <c r="F996" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G996" t="inlineStr">
-        <is>
-          <t>Needs a target-redirection mechanism ('a Battle action that would target a card in this unit instead targets a different one of your own cards') -- the same still-unbuilt gap already noted for oracle-l5r-5086 (Yoritomo Naoto's own deferred case).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G996" t="inlineStr"/>
     </row>
     <row r="997">
       <c r="A997" t="inlineStr">
@@ -41294,7 +41274,7 @@
       </c>
       <c r="G1212" t="inlineStr">
         <is>
-          <t>Needs an "after being targeted, negate" Reaction trigger (same gap as oracle-l5r-1292/10107).</t>
+          <t>Its Reaction half is now expressible: the targeted-by-action trigger (issue #335) plus NegateEffects(card, "destroy") ("another player's action targets your defending Personality, if this Shugenja is Earth, destroy this card: negate the Personality's destruction" -- Rokai's shape, with a Spell as the reactor and a defending-Personality condition). Its Battle/Open half ("even if this unit is not at the current battlefield, bow this Shugenja and target your Nonhuman: Straighten it") keeps its own gap (a non-AtBattle keyword target); not re-audited here.</t>
         </is>
       </c>
     </row>
@@ -48902,7 +48882,7 @@
       </c>
       <c r="G1440" t="inlineStr">
         <is>
-          <t>Needs an "after being targeted" Reaction trigger (the additional-Battle-action half is separately wirable).</t>
+          <t>Its "after the next time (this turn) an action targets him" is a standing watch set up by the Battle action (not a printed in-play Reaction), then a choice between negating the action's effects on the Monk (NegateAllEffectsOn exists, issue #335) or bowing the unit of a performer after the action resolves; the additional-Battle-action half is separately wirable. The standing-watch shape and the either/or choice are the gaps.</t>
         </is>
       </c>
     </row>
@@ -49594,7 +49574,7 @@
       </c>
       <c r="G1460" t="inlineStr">
         <is>
-          <t>Needs an 'after being targeted, negate' Reaction trigger (the same established gap as oracle-l5r-1292/10107/7767/8500) for its own delayed negation half, and its own Nonhuman Performer choice hits the same non-AtBattle keyword-Performer gap as oracle-l5r-5941/6727 (Open has no battlefield for a keyword/type-filtered Performer category to validate against). Its own negate-straightening-until-next-turn half directly reuses the existing StraightenBlockedTurn field.</t>
+          <t>Its delayed negation is a standing watch ("after the next time this game another player's Battle action targets it, negate the action's effects") set by an Open action -- NegateAllEffectsOn (issue #335) is the negation, the standing watch is the gap -- and its Nonhuman Performer choice hits the same non-AtBattle keyword-Performer gap as oracle-l5r-5941/6727 (Open has no battlefield for a keyword/type-filtered Performer category to validate against). Its own negate-straightening-until-next-turn half directly reuses the existing StraightenBlockedTurn field.</t>
         </is>
       </c>
     </row>
@@ -51066,7 +51046,7 @@
       </c>
       <c r="G1504" t="inlineStr">
         <is>
-          <t>Its own first Reaction ('after another player's action targets your performing Samurai, negate his bowing and movement') is exactly the broad, still-unbuilt 'after another player's action targets this card' Reaction trigger (the single largest recurring gap across multiple waves, per oracle-l5r-223). Its second Reaction needs a 'Fear action' classification-dispatch trigger on top of that -- the same still-unbuilt family as the Tactical/Bushido-Virtue/Kiho/Recon 'was this an [X] action' gap noted elsewhere ('Fear Battle' itself is only confirmed as a Timing-prefix, per oracle-l5r-4934's own note, not as a detectable trigger classification).</t>
+          <t>Its first Reaction ("after another player's action targets your performing Samurai, negate his bowing and movement", from hand) is the targeted-by-action shape (issue #335) with two kinds negated at once (NegateEffects(card, "bow", "move")); it needs the trigger offered from a hand and a "performing Samurai" performer for a Reaction. Its second ("after a Fear action targets your performing Samurai: negate its effects") also needs a Fear-action classification.</t>
         </is>
       </c>
     </row>
@@ -53461,7 +53441,7 @@
       </c>
       <c r="G1575" t="inlineStr">
         <is>
-          <t>Needs an "after being targeted" Reaction trigger plus card creation (a temporary token Personality) -- both known gaps.</t>
+          <t>Its Reaction ("after another player's action targets your Personality: Discard him") is now expressible through the targeted-by-action trigger (issue #335, played from hand: see the decision note's Known limits); the Battle half needs card creation (a temporary token Personality) -- a known gap.</t>
         </is>
       </c>
     </row>
@@ -55164,7 +55144,7 @@
       </c>
       <c r="G1626" t="inlineStr">
         <is>
-          <t>Needs an "actions must target this card if legal" redirect mechanic (same gap as oracle-l5r-10300).</t>
+          <t>Needs an "actions must target this card if legal" forced-redirection rule (same gap as oracle-l5r-10300): a standing effect that rewrites every other player's Battle action for the rest of the battle. The legality half now exists (ActionAcceptsTarget, issue #335 -- "if legal" is that check); the standing hook that applies it to every action is the gap.</t>
         </is>
       </c>
     </row>
@@ -60400,7 +60380,7 @@
       </c>
       <c r="G1782" t="inlineStr">
         <is>
-          <t>Its own FocusEffect half (negate destruction for losing; winner's controller gains 2 Honor) is directly wirable. Its own Reaction half needs an 'after being targeted, negate' trigger -- the same still-unbuilt gap as oracle-l5r-1292/10107/7767, here scoped to Iaijutsu actions specifically.</t>
+          <t>Its own FocusEffect half (negate destruction for losing; winner's controller gains 2 Honor) is directly wirable. Its Reaction half ("after another player's Iaijutsu action targets your Personality: negate his destruction", played from hand) needs the targeted-by-action trigger offered from a hand (issue #335 offers it for in-play cards only) and an Iaijutsu classification (a hardcoded id list today; ActionKeywords could carry it).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire Fukui, Jun-Ni, Yumaru, Tensin (personality-wave-31) and Fading Shadows (follower-wave-17): alternative costs, attach from a discard pile, conditional effect choice, Follower performer (#337)
Four general primitives (CostOptions, AttachSpec with cost modes through the Gold quote path, Branch read at resolution, a Follower Performer category) and a per-card deck copy limit. The four older bow-or-bow cost choices are expressed on the alternative-cost primitive. Foothills Keep is left: its Equip-of-Weapons timing passive is not built.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>26.9%</t>
+          <t>27.4%</t>
         </is>
       </c>
     </row>
@@ -534,14 +534,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>57.4%</t>
+          <t>58.2%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>19.3%</t>
         </is>
       </c>
     </row>
@@ -963,7 +963,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Its Battle/Open Equip half is built (issue #337: an AttachSpec with the performing Kensai as wielder, your own pile, Weapons only, Cost AttachCost() -- proved as the training-attach-weapon-performer fixture). Left unwired because a card is published whole: its first line, "Equipping Weapons is a Battle/Open action for you", changes the timing of the ORDINARY Equip command (a Limited action from hand, Action phase, active player, hardcoded in MatchEngine.Equip and QueryActions) for Weapons only. What remains is an Effect-keyed timing override on Equip for Weapons -- Open in the Action phase for whoever holds priority, and as a Battle action presence and a wielder at the battlefield -- plus its QueryActions listing; and an open rules question for Mendon (does it add to or replace the Limited timing; must the wielder be at the battlefield).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7650,7 +7654,7 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>Needs a Follower-Equip Battle ability with no Shugenja/opposed requirement (Daigotsu Chiboshi's own "Equip a Follower to Chiboshi"), plus tying its own Additional Action grant to a Reserve recruitment specifically.</t>
+          <t>Needs a Follower-Equip Battle ability with no Shugenja/opposed requirement (Daigotsu Chiboshi's own "Equip a Follower to Chiboshi"; the attach primitive of issue #337 needs a hand pile for it), plus tying its own Additional Action grant to a Reserve recruitment specifically.</t>
         </is>
       </c>
     </row>
@@ -11233,14 +11237,10 @@
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G316" t="inlineStr">
-        <is>
-          <t>Needs a Follower-eligible Performer category (the same gap as oracle-l5r-1992; existing Performer categories are Personality-only) for bowing "your performing Follower in Tensin's unit" as a cost; his first ability ("If you have Reconnaissance: Ranged 4 Attack") is already an exact match for the published Hiruma Sniper's own hiruma-sniper-attack shape and is separately, trivially wirable.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="G336" t="inlineStr">
         <is>
-          <t>Needs both a dual-independent-target primitive (a Follower in hand plus a separate Personality target) and 'Equip this Follower as a Battle action' (not yet a general capability) -- two established gaps compounding on the same card.</t>
+          <t>Needs a dual-independent-target primitive (a Follower in hand plus a separate Personality target). The attach half now has its primitive (issue #337: attach a card to a Personality, paying all costs) but for a card in a discard pile or the source itself, not a hand card chosen as a target.</t>
         </is>
       </c>
     </row>
@@ -14997,14 +14997,10 @@
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G428" t="inlineStr">
-        <is>
-          <t>Card creation itself is now built (issue #257), but this card still needs a 'bow OR destroy the performer' cost-choice, distinct from the existing bow-or-bow cost choices (own-wielder-or-source-with-wielder-keyword, own-source-or-unbowed-holding-with-keyword) -- not yet built.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr"/>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -17961,7 +17957,7 @@
       </c>
       <c r="G515" t="inlineStr">
         <is>
-          <t>Needs Equip from a discard pile -- an established gap (no mechanism returns a card to play from a discard pile yet, the same one blocking Bayushi Wateru's own 'Absent Interrupt').</t>
+          <t>Unblocked by the attach-from-a-discard-pile primitive (issue #337): "Battle, [Gold]: Equip a target non-Unique Weapon in your discard pile to Katagi" is one ability definition -- Attach: AttachSpec(Target, Own pile, Wielder Source, [Item], Keywords [Weapon], Excluded [Unique]) with Cost: GoldCostRule.AttachCost(), exactly the training-attach-weapon-discount shape at full cost (his from-hand discount does not apply to a discard-pile attach). Deferred for scope, not wired in #337.</t>
         </is>
       </c>
     </row>
@@ -18496,14 +18492,10 @@
       </c>
       <c r="F531" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G531" t="inlineStr">
-        <is>
-          <t>Needs an independent, per-target optional move-home choice (two cards, each optionally moved) where the two printed branches differ only in mandatory-vs-optional -- this project treats a dropped 'may' sub-choice cautiously (see Nishimura's own deferred precedent) rather than guessing at a simplification.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr"/>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
@@ -19197,14 +19189,10 @@
       </c>
       <c r="F552" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G552" t="inlineStr">
-        <is>
-          <t>Needs Equip from the discard pile (the same gap as oracle-l5r-10681/10631/3767 -- no mechanism returns a card to play from a discard pile yet) for his own Limited ability; the passive "Followers in this unit have Cavalry" is separately wirable as a live-conditional-keyword grant on the attached-to relationship, the same shape as Isawa Kojiro's own Naval-while-has-Spell (a live check in Keyword() itself, published in personality-wave-22, issue #301).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G552" t="inlineStr"/>
     </row>
     <row r="553">
       <c r="A553" t="inlineStr">
@@ -28507,7 +28495,7 @@
       </c>
       <c r="G833" t="inlineStr">
         <is>
-          <t>Needs a Follower-eligible Performer category (the same gap as oracle-l5r-1992/3332) for bowing "your performing Follower" as a cost.</t>
+          <t>The Follower Performer category and the bow cost option now exist (issue #337: a single 'bow' CostOption on the performing Follower), but Emoto's performer is ANY unbowed Follower of yours at the current battlefield, not one in his own unit -- one more category (own-unbowed-follower-at-battle) -- plus 'Destroy it' on an enemy card without attachments (the existing elite-sentry-destroy shape). Deferred for scope, not wired in #337.</t>
         </is>
       </c>
     </row>
@@ -30535,7 +30523,7 @@
       </c>
       <c r="G893" t="inlineStr">
         <is>
-          <t>Needs a Follower-eligible Performer category (existing categories are Personality-only).</t>
+          <t>The Follower Performer category now exists (own-unbowed-follower-in-source-unit, issue #337: Hiruma Tensin), but this card's performer is "one of your Followers or Personalities in this army" (any unit card of either type, bowed as the cost) and its target is "a Follower or Personality in this army": neither category is built.</t>
         </is>
       </c>
     </row>
@@ -30781,14 +30769,10 @@
       </c>
       <c r="F900" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G900" t="inlineStr">
-        <is>
-          <t>Needs "Equip this Follower as a Battle action" (not yet a general capability).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G900" t="inlineStr"/>
     </row>
     <row r="901">
       <c r="A901" t="inlineStr">
@@ -30996,7 +30980,7 @@
       </c>
       <c r="G906" t="inlineStr">
         <is>
-          <t>Needs Equip from the discard pile (explicitly known gap -- no mechanism returns a card to play from a discard pile yet).</t>
+          <t>Its ordinary Equip is allowed from YOUR discard pile ("You may Equip this Follower from your discard pile"). The attach-from-a-discard-pile primitive exists (AttachAction.cs, issue #337) for an ability that TARGETS a card in a pile, but here the SOURCE card in the pile is the attachment (AttachSource.Self is hand-only) and the action is the ordinary Limited Equip command, not an ability -- not built.</t>
         </is>
       </c>
     </row>
@@ -32907,7 +32891,7 @@
       </c>
       <c r="G961" t="inlineStr">
         <is>
-          <t>Needs "Equip this Follower as a Battle action" (not yet a general capability).</t>
+          <t>"You may Equip this Follower as a Battle action" is now a general capability (AttachSource.Self, issue #337: Fading Shadows attaches itself from hand to a performing Ninja). Shinobi Vassal differs in that the wielder is any Ninja Personality chosen as a target, and its own Battle action destroys a target enemy card without attachments and then the Follower itself -- deferred, not wired in #337.</t>
         </is>
       </c>
     </row>
@@ -49314,7 +49298,7 @@
       </c>
       <c r="G1452" t="inlineStr">
         <is>
-          <t>Needs Equip from the discard pile (explicitly known gap, oracle-l5r-10681) plus a DELAYED "before this battle resolves" destruction registered by an action (the general before-resolution window, issue #310, applies traits of cards in play at the battlefield; an action-registered delayed effect queue is not built).</t>
+          <t>The attach-from-a-discard-pile primitive exists now (issue #337; ignoring costs is no Cost rule), but this card's Follower may come from hand OR a discard pile (AttachPile has discard values only), and it needs a DELAYED "destroy it before this battle resolves" registered by an action (the general before-resolution window, issue #310, applies traits of cards in play at the battlefield; an action-registered delayed effect queue is not built).</t>
         </is>
       </c>
     </row>
@@ -50526,7 +50510,7 @@
       </c>
       <c r="G1488" t="inlineStr">
         <is>
-          <t>Needs Equip from the discard pile (explicitly known gap, oracle-l5r-10681).</t>
+          <t>Its Follower may come from your hand OR a discard pile, paying 1 less Gold. The attach-from-a-discard-pile primitive (issue #337) covers the discard half (AttachCost(-1, 0)); a hand-or-discard pile choice (AttachPile has discard values only) is the piece left.</t>
         </is>
       </c>
     </row>
@@ -52921,7 +52905,7 @@
       </c>
       <c r="G1559" t="inlineStr">
         <is>
-          <t>Needs a general "attach any attachment from hand, at a Gold discount" Battle action, distinct from a Reserve/Spell-specific Equip variant.</t>
+          <t>Needs a general "attach any attachment from hand, at a Gold discount" Battle action. The attach primitive (issue #337) prices it (AttachCost(-4)) but its pile choices are discard piles and the source itself, not the acting player's hand: one AttachPile value away, plus its separate Open half.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire Fukuzo, Yoritomo Sakuma and Unfortunate Hesitation: keyword/ability copy primitives and the opposing player's Either/Or choice (#338)
Two independent copy primitives (copy one keyword, copy one ability) over a new GrantedAbility model; a general opposing-player Either/Or
decision; a payment-time alternate Gold source; a minimal whole-action negation; a per-player forced pass. personality-wave-33 (Fukuzo,
Sakuma) and strategy-wave-22 (Unfortunate Hesitation); published count 412.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>26.9%</t>
+          <t>27.2%</t>
         </is>
       </c>
     </row>
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>19.2%</t>
         </is>
       </c>
     </row>
@@ -9472,14 +9472,10 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G263" t="inlineStr">
-        <is>
-          <t>Needs an ability-copying mechanism (the same gap as oracle-l5r-10699; novel meta-effect, not built).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -17372,7 +17368,7 @@
       </c>
       <c r="G498" t="inlineStr">
         <is>
-          <t>Needs card creation (a new Personality copying this card's own printed Force/Chi/Personal Honor/keywords) and a 'this card's own ability will not be copied' flag -- no card-copying mechanism exists yet at all.</t>
+          <t>Needs card creation (a new Personality copying this card's own printed Force/Chi/Personal Honor/keywords) and a per-card "this card's own ability will not be copied" flag; the keyword/ability copy primitives now exist (CardCopy.cs, issue #338) and CopyableAbility is the one place such a flag would be honored.</t>
         </is>
       </c>
     </row>
@@ -29104,14 +29100,10 @@
       </c>
       <c r="F851" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G851" t="inlineStr">
-        <is>
-          <t>Needs a payment-time interrupt (the same gap as oracle-l5r-9828 -- an alternate Gold source triggered DURING an in-progress Gold payment, not built) for its first ability, plus the same generic "negate unless the affected player pays a cost" Political Reaction mechanism noted for oracle-l5r-9445 for its second -- two independent, compounding gaps.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G851" t="inlineStr"/>
     </row>
     <row r="852">
       <c r="A852" t="inlineStr">
@@ -29575,7 +29567,7 @@
       </c>
       <c r="G865" t="inlineStr">
         <is>
-          <t>Needs a payment-time interrupt -- an alternate Gold source triggered DURING an in-progress Gold payment (destroying a Mine/Farm mid-payment), not built.</t>
+          <t>The payment-time alternate Gold source now exists (AlternateGoldSource in GoldQuotes.cs, issue #338: "bow this card: produce N Gold" chosen inside the payment, as Yoritomo Sakuma does). Zlkyt needs it extended with a sacrifice chosen inside the payment: "destroy your target Mine or Farm: Produce Gold equal to its base Gold Cost" (a target selected as part of the payment, destroyed as the cost, its cost read as the amount).</t>
         </is>
       </c>
     </row>
@@ -39987,7 +39979,7 @@
       </c>
       <c r="G1173" t="inlineStr">
         <is>
-          <t>Needs an ability/card-copying mechanism -- the same still-unbuilt gap as oracle-l5r-10699/10463, neither of which is built either.</t>
+          <t>The copy primitives now exist (CardCopy.cs, issue #338) but each copies ONE chosen keyword or ability; this card copies ALL of a Spell's keywords, traits and base abilities that do not copy abilities, permanently, so it needs a copy-all variant (Duration "Permanent", no choice), the trait/ability distinction (traits are Effect strings, not abilities), and its once-per-game Reaction paying Gold equal to the target Spell's base cost.</t>
         </is>
       </c>
     </row>
@@ -41760,7 +41752,7 @@
       </c>
       <c r="G1226" t="inlineStr">
         <is>
-          <t>Needs an ability-copying mechanism (novel meta-effect; not built).</t>
+          <t>The ability-copying primitive now exists (CardCopy.cs, issue #338: copy one ability that does not itself copy abilities, with Duration "Turn" for a copy "this turn"). What is still missing is this Spell's own target category (a Spell at this battlefield or a Thunder Spell at any location) and copying onto a Spell receiver during a Thunder Battle action.</t>
         </is>
       </c>
     </row>
@@ -61228,7 +61220,7 @@
       </c>
       <c r="F1807" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1807" t="inlineStr"/>

</xml_diff>

<commit_message>
Wire Fukui, Jun-Ni, Yumaru, Tensin (personality-wave-31) and Fading Shadows (follower-wave-17): alternative costs, attach from a discard pile, conditional effect choice, Follower performer (#337) (#340)
Four general primitives (CostOptions, AttachSpec with cost modes through the Gold quote path, Branch read at resolution, a Follower Performer category) and a per-card deck copy limit. The four older bow-or-bow cost choices are expressed on the alternative-cost primitive. Foothills Keep is left: its Equip-of-Weapons timing passive is not built.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>26.9%</t>
+          <t>27.4%</t>
         </is>
       </c>
     </row>
@@ -534,14 +534,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C7" t="n">
         <v>122</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>57.4%</t>
+          <t>58.2%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>19.3%</t>
         </is>
       </c>
     </row>
@@ -963,7 +963,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Its Battle/Open Equip half is built (issue #337: an AttachSpec with the performing Kensai as wielder, your own pile, Weapons only, Cost AttachCost() -- proved as the training-attach-weapon-performer fixture). Left unwired because a card is published whole: its first line, "Equipping Weapons is a Battle/Open action for you", changes the timing of the ORDINARY Equip command (a Limited action from hand, Action phase, active player, hardcoded in MatchEngine.Equip and QueryActions) for Weapons only. What remains is an Effect-keyed timing override on Equip for Weapons -- Open in the Action phase for whoever holds priority, and as a Battle action presence and a wielder at the battlefield -- plus its QueryActions listing; and an open rules question for Mendon (does it add to or replace the Limited timing; must the wielder be at the battlefield).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7650,7 +7654,7 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>Needs a Follower-Equip Battle ability with no Shugenja/opposed requirement (Daigotsu Chiboshi's own "Equip a Follower to Chiboshi"), plus tying its own Additional Action grant to a Reserve recruitment specifically.</t>
+          <t>Needs a Follower-Equip Battle ability with no Shugenja/opposed requirement (Daigotsu Chiboshi's own "Equip a Follower to Chiboshi"; the attach primitive of issue #337 needs a hand pile for it), plus tying its own Additional Action grant to a Reserve recruitment specifically.</t>
         </is>
       </c>
     </row>
@@ -11233,14 +11237,10 @@
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G316" t="inlineStr">
-        <is>
-          <t>Needs a Follower-eligible Performer category (the same gap as oracle-l5r-1992; existing Performer categories are Personality-only) for bowing "your performing Follower in Tensin's unit" as a cost; his first ability ("If you have Reconnaissance: Ranged 4 Attack") is already an exact match for the published Hiruma Sniper's own hiruma-sniper-attack shape and is separately, trivially wirable.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="G336" t="inlineStr">
         <is>
-          <t>Needs both a dual-independent-target primitive (a Follower in hand plus a separate Personality target) and 'Equip this Follower as a Battle action' (not yet a general capability) -- two established gaps compounding on the same card.</t>
+          <t>Needs a dual-independent-target primitive (a Follower in hand plus a separate Personality target). The attach half now has its primitive (issue #337: attach a card to a Personality, paying all costs) but for a card in a discard pile or the source itself, not a hand card chosen as a target.</t>
         </is>
       </c>
     </row>
@@ -14997,14 +14997,10 @@
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G428" t="inlineStr">
-        <is>
-          <t>Card creation itself is now built (issue #257), but this card still needs a 'bow OR destroy the performer' cost-choice, distinct from the existing bow-or-bow cost choices (own-wielder-or-source-with-wielder-keyword, own-source-or-unbowed-holding-with-keyword) -- not yet built.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr"/>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -17961,7 +17957,7 @@
       </c>
       <c r="G515" t="inlineStr">
         <is>
-          <t>Needs Equip from a discard pile -- an established gap (no mechanism returns a card to play from a discard pile yet, the same one blocking Bayushi Wateru's own 'Absent Interrupt').</t>
+          <t>Unblocked by the attach-from-a-discard-pile primitive (issue #337): "Battle, [Gold]: Equip a target non-Unique Weapon in your discard pile to Katagi" is one ability definition -- Attach: AttachSpec(Target, Own pile, Wielder Source, [Item], Keywords [Weapon], Excluded [Unique]) with Cost: GoldCostRule.AttachCost(), exactly the training-attach-weapon-discount shape at full cost (his from-hand discount does not apply to a discard-pile attach). Deferred for scope, not wired in #337.</t>
         </is>
       </c>
     </row>
@@ -18496,14 +18492,10 @@
       </c>
       <c r="F531" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G531" t="inlineStr">
-        <is>
-          <t>Needs an independent, per-target optional move-home choice (two cards, each optionally moved) where the two printed branches differ only in mandatory-vs-optional -- this project treats a dropped 'may' sub-choice cautiously (see Nishimura's own deferred precedent) rather than guessing at a simplification.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr"/>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
@@ -19197,14 +19189,10 @@
       </c>
       <c r="F552" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G552" t="inlineStr">
-        <is>
-          <t>Needs Equip from the discard pile (the same gap as oracle-l5r-10681/10631/3767 -- no mechanism returns a card to play from a discard pile yet) for his own Limited ability; the passive "Followers in this unit have Cavalry" is separately wirable as a live-conditional-keyword grant on the attached-to relationship, the same shape as Isawa Kojiro's own Naval-while-has-Spell (a live check in Keyword() itself, published in personality-wave-22, issue #301).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G552" t="inlineStr"/>
     </row>
     <row r="553">
       <c r="A553" t="inlineStr">
@@ -28507,7 +28495,7 @@
       </c>
       <c r="G833" t="inlineStr">
         <is>
-          <t>Needs a Follower-eligible Performer category (the same gap as oracle-l5r-1992/3332) for bowing "your performing Follower" as a cost.</t>
+          <t>The Follower Performer category and the bow cost option now exist (issue #337: a single 'bow' CostOption on the performing Follower), but Emoto's performer is ANY unbowed Follower of yours at the current battlefield, not one in his own unit -- one more category (own-unbowed-follower-at-battle) -- plus 'Destroy it' on an enemy card without attachments (the existing elite-sentry-destroy shape). Deferred for scope, not wired in #337.</t>
         </is>
       </c>
     </row>
@@ -30535,7 +30523,7 @@
       </c>
       <c r="G893" t="inlineStr">
         <is>
-          <t>Needs a Follower-eligible Performer category (existing categories are Personality-only).</t>
+          <t>The Follower Performer category now exists (own-unbowed-follower-in-source-unit, issue #337: Hiruma Tensin), but this card's performer is "one of your Followers or Personalities in this army" (any unit card of either type, bowed as the cost) and its target is "a Follower or Personality in this army": neither category is built.</t>
         </is>
       </c>
     </row>
@@ -30781,14 +30769,10 @@
       </c>
       <c r="F900" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G900" t="inlineStr">
-        <is>
-          <t>Needs "Equip this Follower as a Battle action" (not yet a general capability).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G900" t="inlineStr"/>
     </row>
     <row r="901">
       <c r="A901" t="inlineStr">
@@ -30996,7 +30980,7 @@
       </c>
       <c r="G906" t="inlineStr">
         <is>
-          <t>Needs Equip from the discard pile (explicitly known gap -- no mechanism returns a card to play from a discard pile yet).</t>
+          <t>Its ordinary Equip is allowed from YOUR discard pile ("You may Equip this Follower from your discard pile"). The attach-from-a-discard-pile primitive exists (AttachAction.cs, issue #337) for an ability that TARGETS a card in a pile, but here the SOURCE card in the pile is the attachment (AttachSource.Self is hand-only) and the action is the ordinary Limited Equip command, not an ability -- not built.</t>
         </is>
       </c>
     </row>
@@ -32907,7 +32891,7 @@
       </c>
       <c r="G961" t="inlineStr">
         <is>
-          <t>Needs "Equip this Follower as a Battle action" (not yet a general capability).</t>
+          <t>"You may Equip this Follower as a Battle action" is now a general capability (AttachSource.Self, issue #337: Fading Shadows attaches itself from hand to a performing Ninja). Shinobi Vassal differs in that the wielder is any Ninja Personality chosen as a target, and its own Battle action destroys a target enemy card without attachments and then the Follower itself -- deferred, not wired in #337.</t>
         </is>
       </c>
     </row>
@@ -49314,7 +49298,7 @@
       </c>
       <c r="G1452" t="inlineStr">
         <is>
-          <t>Needs Equip from the discard pile (explicitly known gap, oracle-l5r-10681) plus a DELAYED "before this battle resolves" destruction registered by an action (the general before-resolution window, issue #310, applies traits of cards in play at the battlefield; an action-registered delayed effect queue is not built).</t>
+          <t>The attach-from-a-discard-pile primitive exists now (issue #337; ignoring costs is no Cost rule), but this card's Follower may come from hand OR a discard pile (AttachPile has discard values only), and it needs a DELAYED "destroy it before this battle resolves" registered by an action (the general before-resolution window, issue #310, applies traits of cards in play at the battlefield; an action-registered delayed effect queue is not built).</t>
         </is>
       </c>
     </row>
@@ -50526,7 +50510,7 @@
       </c>
       <c r="G1488" t="inlineStr">
         <is>
-          <t>Needs Equip from the discard pile (explicitly known gap, oracle-l5r-10681).</t>
+          <t>Its Follower may come from your hand OR a discard pile, paying 1 less Gold. The attach-from-a-discard-pile primitive (issue #337) covers the discard half (AttachCost(-1, 0)); a hand-or-discard pile choice (AttachPile has discard values only) is the piece left.</t>
         </is>
       </c>
     </row>
@@ -52921,7 +52905,7 @@
       </c>
       <c r="G1559" t="inlineStr">
         <is>
-          <t>Needs a general "attach any attachment from hand, at a Gold discount" Battle action, distinct from a Reserve/Spell-specific Equip variant.</t>
+          <t>Needs a general "attach any attachment from hand, at a Gold discount" Battle action. The attach primitive (issue #337) prices it (AttachCost(-4)) but its pile choices are discard piles and the source itself, not the acting player's hand: one AttachPile value away, plus its separate Open half.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hotako exp3, Yoshitada, Sea Troll Predator, Liu-Xeung exp, Bonds of Coin, Gold and Steel, Fear Me!: decision doc, inventory, handoff (issue #336)
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>26.9%</t>
+          <t>27.4%</t>
         </is>
       </c>
     </row>
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>10.2%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>19.4%</t>
         </is>
       </c>
     </row>
@@ -7186,7 +7186,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G194" t="inlineStr"/>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Not blocked since issue #336: its Battle action is Sea Troll Predator's verbatim (predator-move, MoveSpec source-and-target to an adjacent unresolved battlefield); not yet wired.</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -7880,14 +7884,10 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G215" t="inlineStr">
-        <is>
-          <t>Needs an action-lock ("may not perform actions") status for its Fear Open ability (the same gap as oracle-l5r-7776); the Lion-Clan-conditional entry discount and the entry Honor loss are both separately wirable (lion-clan-discount already exists as a conditional Effect term, just on Equip's cost formula rather than QuotePurchase's; own-enters-play already covers the Honor loss).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -9270,14 +9270,10 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G257" t="inlineStr">
-        <is>
-          <t>Needs a compound two-independently-chosen-target ability shape (bow a targeted enemy Personality, AND separately choose a player who gains or loses Honor) -- AbilityDefinition carries only one Target category per ability, and ValidateAbility's own Target switch treats the "player" category and every card-Target category as mutually exclusive branches, so a single ability cannot select both a card and a player today (the same class of gap as oracle-l5r-3638/2738 -- no existing shape supports two independently-chosen targets). The bow itself is trivial, and "choose a player who gains or loses N Honor" is fully built (issue #210, Kitsuki Horume) -- but only as an ability's own single Target, not layered onto a second, already-chosen card target.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -11005,7 +11001,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G309" t="inlineStr"/>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>Not blocked since issue #336: "Bow him. He may not perform actions." is a bow plus the action-lock (ActionLock.cs); not yet wired.</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="G335" t="inlineStr">
         <is>
-          <t>Needs a dual-independent-target primitive (choosing a Terrain AND a separate enemy card in one ability) -- no existing shape supports two independently-chosen targets.</t>
+          <t>Now expressible on the multi-target shape (TargetSlots.cs, issue #336): two slots, terrain-at-battle and enemy-card-without-attachments, both existing categories; not yet wired.</t>
         </is>
       </c>
     </row>
@@ -14431,7 +14431,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G411" t="inlineStr"/>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>The action-lock exists (issue #336) with a turn duration; this one lasts "until the current phase ends" -- it needs a phase-scoped duration on ActionLock (PrintedPhases.Instance, the stamp the once-per-phase limit already uses).</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -15393,7 +15397,7 @@
       </c>
       <c r="G439" t="inlineStr">
         <is>
-          <t>Needs card creation (a new Personality instance) plus a turn-spanning 'lost Honor from another player's action since your last turn began' tracked condition, and a variable one-to-four multi-target selection -- none built.</t>
+          <t>Needs card creation (a new Personality instance) plus a turn-spanning "lost Honor from another player's action since your last turn began" tracked condition, and a one-to-four selection whose MAXIMUM depends on that condition (the multi-target slots, issue #336, have a fixed Min..Max per slot; a condition-dependent Max is the remaining gap).</t>
         </is>
       </c>
     </row>
@@ -20946,14 +20950,10 @@
       </c>
       <c r="F605" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G605" t="inlineStr">
-        <is>
-          <t>Needs a "move an enemy Personality to a battlefield other than home" mechanic -- every existing move primitive moves the acting player's own cards, or moves an enemy card home (the same gap noted for oracle-l5r-3790, generalized further here to jointly move the source there too and to an adjacent, specifically unresolved, battlefield); the entry Honor loss is separately wirable.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" t="inlineStr">
@@ -27203,14 +27203,10 @@
       </c>
       <c r="F794" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G794" t="inlineStr">
-        <is>
-          <t>Needs a new Reaction trigger classifying "an action that gave a Force penalty to an enemy card" (the same broad after-resolution-classification family as oracle-l5r-9900/3083, still unbuilt); the Battle half (move an enemy Personality with lower Personal Honor home, gain Honor) is already an exact match for shamate-move's own shape, using the existing enemy-personality-lower-honor-than-self Target, and is separately, trivially wirable.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G794" t="inlineStr"/>
     </row>
     <row r="795">
       <c r="A795" t="inlineStr">
@@ -33146,7 +33142,7 @@
       </c>
       <c r="G968" t="inlineStr">
         <is>
-          <t>Needs an action-lock ("may not perform actions") status.</t>
+          <t>The action-lock it needed now exists (ActionLock.cs, issue #336): "may not perform actions" for the rest of the turn, blocking every action the card or its attachments perform, still targetable. Nothing else is known to block it (the Dragon-only attach is AttachRequiresKeyword, -4F is ApplyModifier, its target is the existing enemy-force category); not yet wired.</t>
         </is>
       </c>
     </row>
@@ -33976,7 +33972,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G992" t="inlineStr"/>
+      <c r="G992" t="inlineStr">
+        <is>
+          <t>The multi-target slots exist (issue #336: one or two target enemy cards, a Min 1 / Max 2 slot); still needs the printed Fallen/maximum-Personal-Honor static and the bow cost; not yet wired.</t>
+        </is>
+      </c>
     </row>
     <row r="993">
       <c r="A993" t="inlineStr">
@@ -44588,14 +44588,10 @@
       </c>
       <c r="F1311" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1311" t="inlineStr">
-        <is>
-          <t>Needs a variable one-to-three multi-target selection (the same still-unbuilt gap as oracle-l5r-4397's own one-to-four) for its own Political Open half; its Favor Political Limited half is a smaller, separately wirable draw-for-Favor variant of the existing favor-cycle shape.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1311" t="inlineStr"/>
     </row>
     <row r="1312">
       <c r="A1312" t="inlineStr">
@@ -45160,7 +45156,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1328" t="inlineStr"/>
+      <c r="G1328" t="inlineStr">
+        <is>
+          <t>The multi-target slots exist (issue #336: one or two target opposed Personalities); still needs the count of different Clan alignments at the battlefield; not yet wired.</t>
+        </is>
+      </c>
     </row>
     <row r="1329">
       <c r="A1329" t="inlineStr">
@@ -46158,7 +46158,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1358" t="inlineStr"/>
+      <c r="G1358" t="inlineStr">
+        <is>
+          <t>Not blocked since issue #336: one to three of your target defending Personalities, +2F -- a Min 1 / Max 3 slot; not yet wired.</t>
+        </is>
+      </c>
     </row>
     <row r="1359">
       <c r="A1359" t="inlineStr">
@@ -46488,7 +46492,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1368" t="inlineStr"/>
+      <c r="G1368" t="inlineStr">
+        <is>
+          <t>Not blocked since issue #336: two independent targets (your unbowed attacking Personality; an enemy Personality at any location) and the move of the second to the current battlefield (MoveSpec target/current-battlefield), plus the straighten; not yet wired.</t>
+        </is>
+      </c>
     </row>
     <row r="1369">
       <c r="A1369" t="inlineStr">
@@ -46659,7 +46667,7 @@
       </c>
       <c r="G1373" t="inlineStr">
         <is>
-          <t>Needs a variable one-or-more multi-target selection (same gap as oracle-l5r-4397/1092) for its own performing-Tacticians choice, compounded by those targets all having to share one specific non-current battlefield -- a novel constraint no existing multi-target shape expresses.</t>
+          <t>The multi-target slots exist (issue #336) but its "one or more of your performing Tacticians" are performers, not targets -- it needs a multi-performer selection (the same gap as oracle-l5r-2738), compounded by those performers all having to share one specific non-current battlefield. Moving them to the current battlefield is now a MoveSpec.</t>
         </is>
       </c>
     </row>
@@ -47895,7 +47903,7 @@
       </c>
       <c r="F1410" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1410" t="inlineStr"/>
@@ -48831,7 +48839,7 @@
       </c>
       <c r="F1438" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1438" t="inlineStr"/>
@@ -50699,7 +50707,7 @@
       </c>
       <c r="G1493" t="inlineStr">
         <is>
-          <t>Needs a "move an enemy Personality into the current battlefield" mechanic -- every existing move primitive moves the acting player's own cards, or moves a card home, never an opponent's card into battle.</t>
+          <t>The move to a destination the ability's own rule defines (MoveSpec, issue #336) now moves an enemy Personality to the current battlefield and can move the chosen performer with it (Movers performer-and-target). Still needs a target category for "another player's Personality not at the current battlefield" and the "straighten each unit that this moved" follow-up.</t>
         </is>
       </c>
     </row>
@@ -51171,7 +51179,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1507" t="inlineStr"/>
+      <c r="G1507" t="inlineStr">
+        <is>
+          <t>The action-lock exists (issue #336) for its "He may not perform actions"; not yet wired (Battle/Open with a base-Force performer condition, +3F, straighten, an optional bow of a card at his location).</t>
+        </is>
+      </c>
     </row>
     <row r="1508">
       <c r="A1508" t="inlineStr">
@@ -52412,7 +52424,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1544" t="inlineStr"/>
+      <c r="G1544" t="inlineStr">
+        <is>
+          <t>The action-lock exists (issue #336); this one lasts "until this battle ends" -- it needs a battle-scoped duration on ActionLock, plus reducing a unit's Force to 0.</t>
+        </is>
+      </c>
     </row>
     <row r="1545">
       <c r="A1545" t="inlineStr">
@@ -52785,7 +52801,7 @@
       </c>
       <c r="G1555" t="inlineStr">
         <is>
-          <t>Needs a dual-target selection with a relational constraint ("not sharing a Clan alignment") -- every existing multi-target category compares against a fixed performer/self, not between two chosen targets.</t>
+          <t>Needs a dual-target selection with a relational constraint ("not sharing a Clan alignment"). The multi-target shape (issue #336) makes the two targets independent slots, each judged on its own; a constraint BETWEEN the two chosen targets is still not expressible.</t>
         </is>
       </c>
     </row>
@@ -54069,7 +54085,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1593" t="inlineStr"/>
+      <c r="G1593" t="inlineStr">
+        <is>
+          <t>The move of an enemy Personality to the current battlefield exists (MoveSpec target/current-battlefield, issue #336); still needs its Magistrate performer and the status-conditional straighten; not yet wired.</t>
+        </is>
+      </c>
     </row>
     <row r="1594">
       <c r="A1594" t="inlineStr">
@@ -54434,7 +54454,7 @@
       </c>
       <c r="G1604" t="inlineStr">
         <is>
-          <t>Needs a new Reaction trigger: 'after a battle's resolution ends' (the same still-unbuilt gap as oracle-l5r-683), plus a variable one-or-two multi-target selection (same gap as oracle-l5r-4397).</t>
+          <t>Needs a new Reaction trigger: 'after a battle's resolution ends' (the same still-unbuilt gap as oracle-l5r-683), plus a variable one-or-two "performing Personalities" selection -- performers, not targets, so the multi-target slots (issue #336) do not cover it.</t>
         </is>
       </c>
     </row>
@@ -57656,7 +57676,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1700" t="inlineStr"/>
+      <c r="G1700" t="inlineStr">
+        <is>
+          <t>The multi-target slots exist (issue #336: one to three Personalities controlled by other players) and the command keeps the order they were chosen in, which is what its -1F, -2F, -3F assignment reads; not yet wired.</t>
+        </is>
+      </c>
     </row>
     <row r="1701">
       <c r="A1701" t="inlineStr">
@@ -59363,7 +59387,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1751" t="inlineStr"/>
+      <c r="G1751" t="inlineStr">
+        <is>
+          <t>The move of another player's Personality to the current battlefield exists (MoveSpec target/current-battlefield, issue #336); still needs its Monk performer and the Earth-conditional straighten; not yet wired.</t>
+        </is>
+      </c>
     </row>
     <row r="1752">
       <c r="A1752" t="inlineStr">
@@ -59594,7 +59622,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1758" t="inlineStr"/>
+      <c r="G1758" t="inlineStr">
+        <is>
+          <t>Its Battle half (one to three enemy dishonorable Personalities moved home) is a multi-target slot now (issue #336); its Reaction half is the still-unbuilt "negate unless the affected player pays a cost" mechanism.</t>
+        </is>
+      </c>
     </row>
     <row r="1759">
       <c r="A1759" t="inlineStr">
@@ -64213,7 +64245,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1897" t="inlineStr"/>
+      <c r="G1897" t="inlineStr">
+        <is>
+          <t>The lock (Card.ActionLocks) and every modifier (with IsStatPenalty classifying the current Force penalties) are data that can be removed now (issue #336); the negating action itself is not written.</t>
+        </is>
+      </c>
     </row>
     <row r="1898">
       <c r="A1898" t="inlineStr">
@@ -72017,7 +72053,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2133" t="inlineStr"/>
+      <c r="G2133" t="inlineStr">
+        <is>
+          <t>The multi-target slots exist (issue #336: one or two target attachments); a Region Open action with a bow cost; not yet wired.</t>
+        </is>
+      </c>
     </row>
     <row r="2134">
       <c r="A2134" t="inlineStr">

</xml_diff>

<commit_message>
Wire Fukuzo, Yoritomo Sakuma and Unfortunate Hesitation: keyword/ability copy primitives and the opposing player's Either/Or choice (#338) (#344)
Two independent copy primitives (copy one keyword, copy one ability) over a new GrantedAbility model; a general opposing-player Either/Or
decision; a payment-time alternate Gold source; a minimal whole-action negation; a per-player forced pass. personality-wave-33 (Fukuzo,
Sakuma) and strategy-wave-22 (Unfortunate Hesitation); published count 412.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>27.4%</t>
+          <t>27.7%</t>
         </is>
       </c>
     </row>
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>19.3%</t>
+          <t>19.4%</t>
         </is>
       </c>
     </row>
@@ -9476,14 +9476,10 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G263" t="inlineStr">
-        <is>
-          <t>Needs an ability-copying mechanism (the same gap as oracle-l5r-10699; novel meta-effect, not built).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -17368,7 +17364,7 @@
       </c>
       <c r="G498" t="inlineStr">
         <is>
-          <t>Needs card creation (a new Personality copying this card's own printed Force/Chi/Personal Honor/keywords) and a 'this card's own ability will not be copied' flag -- no card-copying mechanism exists yet at all.</t>
+          <t>Needs card creation (a new Personality copying this card's own printed Force/Chi/Personal Honor/keywords) and a per-card "this card's own ability will not be copied" flag; the keyword/ability copy primitives now exist (CardCopy.cs, issue #338) and CopyableAbility is the one place such a flag would be honored.</t>
         </is>
       </c>
     </row>
@@ -29092,14 +29088,10 @@
       </c>
       <c r="F851" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G851" t="inlineStr">
-        <is>
-          <t>Needs a payment-time interrupt (the same gap as oracle-l5r-9828 -- an alternate Gold source triggered DURING an in-progress Gold payment, not built) for its first ability, plus the same generic "negate unless the affected player pays a cost" Political Reaction mechanism noted for oracle-l5r-9445 for its second -- two independent, compounding gaps.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G851" t="inlineStr"/>
     </row>
     <row r="852">
       <c r="A852" t="inlineStr">
@@ -29563,7 +29555,7 @@
       </c>
       <c r="G865" t="inlineStr">
         <is>
-          <t>Needs a payment-time interrupt -- an alternate Gold source triggered DURING an in-progress Gold payment (destroying a Mine/Farm mid-payment), not built.</t>
+          <t>The payment-time alternate Gold source now exists (AlternateGoldSource in GoldQuotes.cs, issue #338: "bow this card: produce N Gold" chosen inside the payment, as Yoritomo Sakuma does). Zlkyt needs it extended with a sacrifice chosen inside the payment: "destroy your target Mine or Farm: Produce Gold equal to its base Gold Cost" (a target selected as part of the payment, destroyed as the cost, its cost read as the amount).</t>
         </is>
       </c>
     </row>
@@ -39971,7 +39963,7 @@
       </c>
       <c r="G1173" t="inlineStr">
         <is>
-          <t>Needs an ability/card-copying mechanism -- the same still-unbuilt gap as oracle-l5r-10699/10463, neither of which is built either.</t>
+          <t>The copy primitives now exist (CardCopy.cs, issue #338) but each copies ONE chosen keyword or ability; this card copies ALL of a Spell's keywords, traits and base abilities that do not copy abilities, permanently, so it needs a copy-all variant (Duration "Permanent", no choice), the trait/ability distinction (traits are Effect strings, not abilities), and its once-per-game Reaction paying Gold equal to the target Spell's base cost.</t>
         </is>
       </c>
     </row>
@@ -41744,7 +41736,7 @@
       </c>
       <c r="G1226" t="inlineStr">
         <is>
-          <t>Needs an ability-copying mechanism (novel meta-effect; not built).</t>
+          <t>The ability-copying primitive now exists (CardCopy.cs, issue #338: copy one ability that does not itself copy abilities, with Duration "Turn" for a copy "this turn"). What is still missing is this Spell's own target category (a Spell at this battlefield or a Thunder Spell at any location) and copying onto a Spell receiver during a Thunder Battle action.</t>
         </is>
       </c>
     </row>
@@ -61212,7 +61204,7 @@
       </c>
       <c r="F1807" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1807" t="inlineStr"/>

</xml_diff>

<commit_message>
Rulings on #340: negated destroy-as-cost negates the action, control follows Jun-Ni, wire Foothills Keep with a player-level timing grant (#352)
A blocked cost (Fields of Mercy etc.) is checked before anything is paid and negates the whole action (seam CostPaymentBlockedByNegation). A card taken from an enemy pile is controlled by its taker (OriginalOwnerId) and returns to its owner on any exit. Foothills Keep (stronghold-wave-5): a Battle/Open attach from your own pile and the first player-level timing grant, which adds Battle/Open equips of Weapons without replacing Equip (Limited).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -498,14 +498,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C5" t="n">
         <v>51</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>19.6%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>19.5%</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,10 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Its Battle/Open Equip half is built (issue #337: an AttachSpec with the performing Kensai as wielder, your own pile, Weapons only, Cost AttachCost() -- proved as the training-attach-weapon-performer fixture). Left unwired because a card is published whole: its first line, "Equipping Weapons is a Battle/Open action for you", changes the timing of the ORDINARY Equip command (a Limited action from hand, Action phase, active player, hardcoded in MatchEngine.Equip and QueryActions) for Weapons only. What remains is an Effect-keyed timing override on Equip for Weapons -- Open in the Action phase for whoever holds priority, and as a Battle action presence and a wielder at the battlefield -- plus its QueryActions listing; and an open rules question for Mendon (does it add to or replace the Limited timing; must the wielder be at the battlefield).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">

</xml_diff>

<commit_message>
Discipline rulings: additive Discipline cost, Lost in Transit modes, False Ring of Air bow cost; wire strategy-wave-23 (#353)
Mendon's rulings on #332's open questions. A Discipline play from a discard
pile now pays the Discipline cost first and then the action's own cost as one
combined Gold quote (two payments, Gold does not carry over, offered only when
both parts are payable); from hand only the action's own cost. That unblocks
Expensive Achievement, Knowledge and Power and Two Steady Breaths, wired as
strategy-wave-23 (Mercantile Conflict stays blocked on an Honor-loss-increase
primitive). Lost in Transit's two modes (no presence as an Open action in the
Action phase, presence only as a Battle action) are pinned by tests, no
behavior change needed. False Ring of Air: bowing the Ring is a cost, so it
has no free hand play.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>19.6%</t>
         </is>
       </c>
     </row>
@@ -47537,7 +47537,7 @@
       </c>
       <c r="F1400" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1400" t="inlineStr"/>
@@ -51111,7 +51111,7 @@
       </c>
       <c r="F1506" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1506" t="inlineStr"/>
@@ -51819,7 +51819,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1527" t="inlineStr"/>
+      <c r="G1527" t="inlineStr">
+        <is>
+          <t>Mercantile Conflict (Discipline, issue #353): the Discipline flag and the additive Discipline cost exist, and its first effect (bow your target unbowed Courtier, Political Open) is wirable, but "the next two Honor losses from your cards (this turn) are increased by 1 each" needs an Honor-loss-increase primitive -- a per-player, per-turn counter consulted at every Honor loss (GainHonor with a negative amount) that raises the first two by 1; nothing like it exists. Left unwired until that primitive is built.</t>
+        </is>
+      </c>
     </row>
     <row r="1528">
       <c r="A1528" t="inlineStr">
@@ -60837,7 +60841,7 @@
       </c>
       <c r="F1796" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1796" t="inlineStr"/>

</xml_diff>

<commit_message>
Battle rulings round 2 (#354): docs, inventory, test hardening
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -2722,7 +2722,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Needs a 'battle resolution does not bow winning cards' modifier flag, triggered by a before-resolution Reaction (not built). The Melee 8 Attack itself is trivial but incomplete without it.</t>
+          <t>The Tireless Reaction is built (issue #354: ability dairuko-rally on the general "Reaction: Before a battle resolves" window and the per-battle 'resolution will not bow your army' flag, proven through a training Personality carrying it). Still needs: its Battle: Melee 8 Attack (ability id, strength and AttackKind entries) and packaging (a personality wave: scan, art, published JSON).</t>
         </is>
       </c>
     </row>
@@ -41804,7 +41804,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1228" t="inlineStr"/>
+      <c r="G1228" t="inlineStr">
+        <is>
+          <t>The general before-resolution machinery exists (issue #354) but this Spell's delayed effect is a MOVE ("move the target home, and if he moved, move this Shugenja to the current battlefield"): a delayed-effect kind 'move home' with a dependent second move is not built (kinds today: bow, straighten, destroy, modifier). Also a Spell package.</t>
+        </is>
+      </c>
     </row>
     <row r="1229">
       <c r="A1229" t="inlineStr">
@@ -49290,7 +49294,7 @@
       </c>
       <c r="G1452" t="inlineStr">
         <is>
-          <t>The attach-from-a-discard-pile primitive exists now (issue #337; ignoring costs is no Cost rule), but this card's Follower may come from hand OR a discard pile (AttachPile has discard values only), and it needs a DELAYED "destroy it before this battle resolves" registered by an action (the general before-resolution window, issue #310, applies traits of cards in play at the battlefield; an action-registered delayed effect queue is not built).</t>
+          <t>The attach-from-a-discard-pile primitive exists now (issue #337; ignoring costs is no Cost rule) and so does the DELAYED "destroy it before this battle resolves" (issue #354: RegisterDelayedBattleEffect, kind destroy, joins the one ordered before-resolution set). Still needs: this card's Follower may come from hand OR a discard pile (AttachPile has discard values only), and its additional Battle action.</t>
         </is>
       </c>
     </row>
@@ -49708,7 +49712,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1464" t="inlineStr"/>
+      <c r="G1464" t="inlineStr">
+        <is>
+          <t>The DELAYED "before this battle resolves, bow him" exists now (issue #354: RegisterDelayedBattleEffect, kind bow). Still needs: the Kolat keyword tag, its 4 Gold cost, the immediate "Lose 1 Honor" and the Strategy package.</t>
+        </is>
+      </c>
     </row>
     <row r="1465">
       <c r="A1465" t="inlineStr">
@@ -53715,7 +53723,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1583" t="inlineStr"/>
+      <c r="G1583" t="inlineStr">
+        <is>
+          <t>The DELAYED "before this battle resolves, give him -3C" exists now (issue #354: RegisterDelayedBattleEffect, kind modifier; a lethal Chi penalty destroys through ApplyModifier). Still needs: the performing unbowed Ninja Personality cost ("bow him if he is not Shadowlands") and the Strategy package.</t>
+        </is>
+      </c>
     </row>
     <row r="1584">
       <c r="A1584" t="inlineStr">
@@ -54144,7 +54156,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1596" t="inlineStr"/>
+      <c r="G1596" t="inlineStr">
+        <is>
+          <t>The DELAYED "before this battle's resolution, straighten the targeted card" exists now (issue #354: RegisterDelayedBattleEffect, kind straighten). Still needs: the target category 'a bowed card in the performer's unit (which may be him)' and the Strategy package.</t>
+        </is>
+      </c>
     </row>
     <row r="1597">
       <c r="A1597" t="inlineStr">
@@ -54309,7 +54325,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1601" t="inlineStr"/>
+      <c r="G1601" t="inlineStr">
+        <is>
+          <t>The DELAYED "before this battle's resolution, straighten your Personality" exists now (issue #354: kind straighten). Still needs: the immediate half (bow the performer as a cost; bow the enemy card; destroy it if an attachment or base Gold Cost 0), the 'enemy card without attachments' target and the Strategy package.</t>
+        </is>
+      </c>
     </row>
     <row r="1602">
       <c r="A1602" t="inlineStr">
@@ -57170,7 +57190,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1686" t="inlineStr"/>
+      <c r="G1686" t="inlineStr">
+        <is>
+          <t>Engine effect built (issue #354: ability steady-resolve-boost on the general "Reaction: Before a battle resolves" window, performer category own-personality-with-keyword-opposed-at-battle, proven through a training Strategy carrying it). Only packaging remains: a strategy wave (scan, art, published JSON).</t>
+        </is>
+      </c>
     </row>
     <row r="1687">
       <c r="A1687" t="inlineStr">
@@ -59937,7 +59961,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1769" t="inlineStr"/>
+      <c r="G1769" t="inlineStr">
+        <is>
+          <t>The DELAYED conditional "straighten him before this battle resolves" exists now (issue #354: kind straighten). Still needs: two targets in one action (a Personality of yours and an enemy card), the Fallen/Magistrate condition and the Strategy package.</t>
+        </is>
+      </c>
     </row>
     <row r="1770">
       <c r="A1770" t="inlineStr">

</xml_diff>

<commit_message>
Battle rulings round 2: Declaration Segment, one ordered before-resolution set, Reactions are actions, Kyuden Hida pinned, deferred Attack source (#354) (#359)
* WIP battle rulings round 2 (#354): declaration segment, Reactions are actions, before-resolution set, deferred Attack source

* WIP battle rulings round 2 (#354): tests, fixtures, AI and transport updates

* WIP battle rulings round 2 (#354): deferred Reaction fixture and expiry test

* Battle rulings round 2 (#354): docs, inventory, test hardening

* Battle rulings round 2 (#354): duel source test, merge follow-ups

* Battle rulings round 2 (#354): handoff and docs
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -2722,7 +2722,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Needs a 'battle resolution does not bow winning cards' modifier flag, triggered by a before-resolution Reaction (not built). The Melee 8 Attack itself is trivial but incomplete without it.</t>
+          <t>The Tireless Reaction is built (issue #354: ability dairuko-rally on the general "Reaction: Before a battle resolves" window and the per-battle 'resolution will not bow your army' flag, proven through a training Personality carrying it). Still needs: its Battle: Melee 8 Attack (ability id, strength and AttackKind entries) and packaging (a personality wave: scan, art, published JSON).</t>
         </is>
       </c>
     </row>
@@ -41784,7 +41784,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1228" t="inlineStr"/>
+      <c r="G1228" t="inlineStr">
+        <is>
+          <t>The general before-resolution machinery exists (issue #354) but this Spell's delayed effect is a MOVE ("move the target home, and if he moved, move this Shugenja to the current battlefield"): a delayed-effect kind 'move home' with a dependent second move is not built (kinds today: bow, straighten, destroy, modifier). Also a Spell package.</t>
+        </is>
+      </c>
     </row>
     <row r="1229">
       <c r="A1229" t="inlineStr">
@@ -49270,7 +49274,7 @@
       </c>
       <c r="G1452" t="inlineStr">
         <is>
-          <t>The attach-from-a-discard-pile primitive exists now (issue #337; ignoring costs is no Cost rule), but this card's Follower may come from hand OR a discard pile (AttachPile has discard values only), and it needs a DELAYED "destroy it before this battle resolves" registered by an action (the general before-resolution window, issue #310, applies traits of cards in play at the battlefield; an action-registered delayed effect queue is not built).</t>
+          <t>The attach-from-a-discard-pile primitive exists now (issue #337; ignoring costs is no Cost rule) and so does the DELAYED "destroy it before this battle resolves" (issue #354: RegisterDelayedBattleEffect, kind destroy, joins the one ordered before-resolution set). Still needs: this card's Follower may come from hand OR a discard pile (AttachPile has discard values only), and its additional Battle action.</t>
         </is>
       </c>
     </row>
@@ -49688,7 +49692,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1464" t="inlineStr"/>
+      <c r="G1464" t="inlineStr">
+        <is>
+          <t>The DELAYED "before this battle resolves, bow him" exists now (issue #354: RegisterDelayedBattleEffect, kind bow). Still needs: the Kolat keyword tag, its 4 Gold cost, the immediate "Lose 1 Honor" and the Strategy package.</t>
+        </is>
+      </c>
     </row>
     <row r="1465">
       <c r="A1465" t="inlineStr">
@@ -53695,7 +53703,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1583" t="inlineStr"/>
+      <c r="G1583" t="inlineStr">
+        <is>
+          <t>The DELAYED "before this battle resolves, give him -3C" exists now (issue #354: RegisterDelayedBattleEffect, kind modifier; a lethal Chi penalty destroys through ApplyModifier). Still needs: the performing unbowed Ninja Personality cost ("bow him if he is not Shadowlands") and the Strategy package.</t>
+        </is>
+      </c>
     </row>
     <row r="1584">
       <c r="A1584" t="inlineStr">
@@ -54124,7 +54136,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1596" t="inlineStr"/>
+      <c r="G1596" t="inlineStr">
+        <is>
+          <t>The DELAYED "before this battle's resolution, straighten the targeted card" exists now (issue #354: RegisterDelayedBattleEffect, kind straighten). Still needs: the target category 'a bowed card in the performer's unit (which may be him)' and the Strategy package.</t>
+        </is>
+      </c>
     </row>
     <row r="1597">
       <c r="A1597" t="inlineStr">
@@ -54289,7 +54305,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1601" t="inlineStr"/>
+      <c r="G1601" t="inlineStr">
+        <is>
+          <t>The DELAYED "before this battle's resolution, straighten your Personality" exists now (issue #354: kind straighten). Still needs: the immediate half (bow the performer as a cost; bow the enemy card; destroy it if an attachment or base Gold Cost 0), the 'enemy card without attachments' target and the Strategy package.</t>
+        </is>
+      </c>
     </row>
     <row r="1602">
       <c r="A1602" t="inlineStr">
@@ -57150,7 +57170,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1686" t="inlineStr"/>
+      <c r="G1686" t="inlineStr">
+        <is>
+          <t>Engine effect built (issue #354: ability steady-resolve-boost on the general "Reaction: Before a battle resolves" window, performer category own-personality-with-keyword-opposed-at-battle, proven through a training Strategy carrying it). Only packaging remains: a strategy wave (scan, art, published JSON).</t>
+        </is>
+      </c>
     </row>
     <row r="1687">
       <c r="A1687" t="inlineStr">
@@ -59917,7 +59941,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1769" t="inlineStr"/>
+      <c r="G1769" t="inlineStr">
+        <is>
+          <t>The DELAYED conditional "straighten him before this battle resolves" exists now (issue #354: kind straighten). Still needs: two targets in one action (a Personality of yours and an enemy card), the Fallen/Magistrate condition and the Strategy package.</t>
+        </is>
+      </c>
     </row>
     <row r="1770">
       <c r="A1770" t="inlineStr">

</xml_diff>

<commit_message>
Delayed move-home and the cards it completes: The Wave Persists, six Strategies, Akodo Dairuko, Kyuden Hida - exp (#364)
The delayed before-resolution effect gains a moveHome kind with one dependent second move ("if he moved, move this Shugenja to the current battlefield"), which wires The Wave Persists (spell-wave-9). The delayed effects of #354 now complete Holding Cells, Power of the Night, Quick Recovery, Reckless Rush and Harsh Taskmaster, published with the already-built Steady Resolve in strategy-wave-27; Akodo Dairuko (personality-wave-38) gains her Melee 8 Attack; Kyuden Hida - exp (stronghold-wave-8) creates Scout Followers removed from the game when the battle ends. The Tale of the Disgraced stays unwired: two targets in one action need the multi-target selection.

All nine scans came from the local reference cache after sha256 verification against the committed receipts; nothing was downloaded.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -498,14 +498,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C5" t="n">
         <v>51</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>19.6%</t>
         </is>
       </c>
     </row>
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C6" t="n">
         <v>813</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>28.3%</t>
         </is>
       </c>
     </row>
@@ -570,14 +570,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>6.8%</t>
         </is>
       </c>
     </row>
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>10.9%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>422</v>
+        <v>431</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>19.7%</t>
+          <t>20.1%</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -2717,14 +2717,10 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>The Tireless Reaction is built (issue #354: ability dairuko-rally on the general "Reaction: Before a battle resolves" window and the per-battle 'resolution will not bow your army' flag, proven through a training Personality carrying it). Still needs: its Battle: Melee 8 Attack (ability id, strength and AttackKind entries) and packaging (a personality wave: scan, art, published JSON).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -41781,14 +41777,10 @@
       </c>
       <c r="F1228" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1228" t="inlineStr">
-        <is>
-          <t>The general before-resolution machinery exists (issue #354) but this Spell's delayed effect is a MOVE ("move the target home, and if he moved, move this Shugenja to the current battlefield"): a delayed-effect kind 'move home' with a dependent second move is not built (kinds today: bow, straighten, destroy, modifier). Also a Spell package.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1228" t="inlineStr"/>
     </row>
     <row r="1229">
       <c r="A1229" t="inlineStr">
@@ -49269,14 +49261,10 @@
       </c>
       <c r="F1452" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1452" t="inlineStr">
-        <is>
-          <t>The attach-from-a-discard-pile primitive exists now (issue #337; ignoring costs is no Cost rule) and so does the DELAYED "destroy it before this battle resolves" (issue #354: RegisterDelayedBattleEffect, kind destroy, joins the one ordered before-resolution set). Still needs: this card's Follower may come from hand OR a discard pile (AttachPile has discard values only), and its additional Battle action.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1452" t="inlineStr"/>
     </row>
     <row r="1453">
       <c r="A1453" t="inlineStr">
@@ -49689,14 +49677,10 @@
       </c>
       <c r="F1464" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1464" t="inlineStr">
-        <is>
-          <t>The DELAYED "before this battle resolves, bow him" exists now (issue #354: RegisterDelayedBattleEffect, kind bow). Still needs: the Kolat keyword tag, its 4 Gold cost, the immediate "Lose 1 Honor" and the Strategy package.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1464" t="inlineStr"/>
     </row>
     <row r="1465">
       <c r="A1465" t="inlineStr">
@@ -53700,14 +53684,10 @@
       </c>
       <c r="F1583" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1583" t="inlineStr">
-        <is>
-          <t>The DELAYED "before this battle resolves, give him -3C" exists now (issue #354: RegisterDelayedBattleEffect, kind modifier; a lethal Chi penalty destroys through ApplyModifier). Still needs: the performing unbowed Ninja Personality cost ("bow him if he is not Shadowlands") and the Strategy package.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1583" t="inlineStr"/>
     </row>
     <row r="1584">
       <c r="A1584" t="inlineStr">
@@ -54133,14 +54113,10 @@
       </c>
       <c r="F1596" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1596" t="inlineStr">
-        <is>
-          <t>The DELAYED "before this battle's resolution, straighten the targeted card" exists now (issue #354: RegisterDelayedBattleEffect, kind straighten). Still needs: the target category 'a bowed card in the performer's unit (which may be him)' and the Strategy package.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1596" t="inlineStr"/>
     </row>
     <row r="1597">
       <c r="A1597" t="inlineStr">
@@ -54302,14 +54278,10 @@
       </c>
       <c r="F1601" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1601" t="inlineStr">
-        <is>
-          <t>The DELAYED "before this battle's resolution, straighten your Personality" exists now (issue #354: kind straighten). Still needs: the immediate half (bow the performer as a cost; bow the enemy card; destroy it if an attachment or base Gold Cost 0), the 'enemy card without attachments' target and the Strategy package.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1601" t="inlineStr"/>
     </row>
     <row r="1602">
       <c r="A1602" t="inlineStr">
@@ -57167,14 +57139,10 @@
       </c>
       <c r="F1686" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1686" t="inlineStr">
-        <is>
-          <t>Engine effect built (issue #354: ability steady-resolve-boost on the general "Reaction: Before a battle resolves" window, performer category own-personality-with-keyword-opposed-at-battle, proven through a training Strategy carrying it). Only packaging remains: a strategy wave (scan, art, published JSON).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1686" t="inlineStr"/>
     </row>
     <row r="1687">
       <c r="A1687" t="inlineStr">
@@ -59943,7 +59911,7 @@
       </c>
       <c r="G1769" t="inlineStr">
         <is>
-          <t>The DELAYED conditional "straighten him before this battle resolves" exists now (issue #354: kind straighten). Still needs: two targets in one action (a Personality of yours and an enemy card), the Fallen/Magistrate condition and the Strategy package.</t>
+          <t>The DELAYED conditional "straighten him before this battle resolves" exists (issue #354) and Fallen/Magistrate are readable keywords, but the action names TWO targets (your unbowed Personality and an enemy card) and the engine offers one: an action option lists the legal targets of a single choice. Needs the general multi-target selection (PR #348: action-lock, multi-target, move destinations) and the Strategy package (scan on hand, no download needed).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rulings on #340: negated destroy-as-cost, control follows Jun-Ni, Foothills Keep and the player-level timing grant (#357)
* Rulings on #340: negated destroy-as-cost negates the action, control follows Jun-Ni, wire Foothills Keep with a player-level timing grant (#352)

A blocked cost (Fields of Mercy etc.) is checked before anything is paid and negates the whole action (seam CostPaymentBlockedByNegation). A card taken from an enemy pile is controlled by its taker (OriginalOwnerId) and returns to its owner on any exit. Foothills Keep (stronghold-wave-5): a Battle/Open attach from your own pile and the first player-level timing grant, which adds Battle/Open equips of Weapons without replacing Equip (Limited).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Document the single cost-block predicate and re-run the mutation table

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -498,14 +498,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" t="n">
         <v>51</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>21.6%</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
@@ -960,14 +960,10 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Its Battle/Open Equip half is built (issue #337: an AttachSpec with the performing Kensai as wielder, your own pile, Weapons only, Cost AttachCost() -- proved as the training-attach-weapon-performer fixture). Left unwired because a card is published whole: its first line, "Equipping Weapons is a Battle/Open action for you", changes the timing of the ORDINARY Equip command (a Limited action from hand, Action phase, active player, hardcoded in MatchEngine.Equip and QueryActions) for Weapons only. What remains is an Effect-keyed timing override on Equip for Weapons -- Open in the Action phase for whoever holds priority, and as a Battle action presence and a wielder at the battlefield -- plus its QueryActions listing; and an open rules question for Mendon (does it add to or replace the Limited timing; must the wielder be at the battlefield).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">

</xml_diff>

<commit_message>
Discipline rulings: additive Discipline cost, Lost in Transit modes, False Ring of Air bow cost; wire strategy-wave-23 (#353) (#358)
Mendon's rulings on #332's open questions. A Discipline play from a discard
pile now pays the Discipline cost first and then the action's own cost as one
combined Gold quote (two payments, Gold does not carry over, offered only when
both parts are payable); from hand only the action's own cost. That unblocks
Expensive Achievement, Knowledge and Power and Two Steady Breaths, wired as
strategy-wave-23 (Mercantile Conflict stays blocked on an Honor-loss-increase
primitive). Lost in Transit's two modes (no presence as an Open action in the
Action phase, presence only as a Battle action) are pinned by tests, no
behavior change needed. False Ring of Air: bowing the Ring is a cost, so it
has no free hand play.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>20.1%</t>
+          <t>20.3%</t>
         </is>
       </c>
     </row>
@@ -47509,7 +47509,7 @@
       </c>
       <c r="F1400" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1400" t="inlineStr"/>
@@ -51079,7 +51079,7 @@
       </c>
       <c r="F1506" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1506" t="inlineStr"/>
@@ -51787,7 +51787,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1527" t="inlineStr"/>
+      <c r="G1527" t="inlineStr">
+        <is>
+          <t>Mercantile Conflict (Discipline, issue #353): the Discipline flag and the additive Discipline cost exist, and its first effect (bow your target unbowed Courtier, Political Open) is wirable, but "the next two Honor losses from your cards (this turn) are increased by 1 each" needs an Honor-loss-increase primitive -- a per-player, per-turn counter consulted at every Honor loss (GainHonor with a negative amount) that raises the first two by 1; nothing like it exists. Left unwired until that primitive is built.</t>
+        </is>
+      </c>
     </row>
     <row r="1528">
       <c r="A1528" t="inlineStr">
@@ -60809,7 +60813,7 @@
       </c>
       <c r="F1796" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1796" t="inlineStr"/>

</xml_diff>

<commit_message>
Refresh CARD_INVENTORY.xlsx (442 wired) and drop stale Matsu Kasei blocker (issue #371)
The checked-in workbook predated many waves. Regenerated from origin/main;
removed the oracle-l5r-4937 BLOCKERS entry, which #265 wired but left
annotated as blocked (same defect class as #225).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -17206,11 +17206,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G494" t="inlineStr">
-        <is>
-          <t>The +2F while attacking is free (reuses the existing attacking-two Effect verbatim); the Battle half needs a general 'move a target Personality home' action (existing move-home mechanics -- Incapacitated/Block -- are battle-resolution-specific, not a standalone targeted ability).</t>
-        </is>
-      </c>
+      <c r="G494" t="inlineStr"/>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">

</xml_diff>

<commit_message>
Refresh CARD_INVENTORY.xlsx (442 wired) and drop stale Matsu Kasei blocker (issue #371) (#372)
The checked-in workbook predated many waves. Regenerated from origin/main;
removed the oracle-l5r-4937 BLOCKERS entry, which #265 wired but left
annotated as blocked (same defect class as #225).

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -17206,11 +17206,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G494" t="inlineStr">
-        <is>
-          <t>The +2F while attacking is free (reuses the existing attacking-two Effect verbatim); the Battle half needs a general 'move a target Personality home' action (existing move-home mechanics -- Incapacitated/Block -- are battle-resolution-specific, not a standalone targeted ability).</t>
-        </is>
-      </c>
+      <c r="G494" t="inlineStr"/>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">

</xml_diff>

<commit_message>
Wire The Tale of the Disgraced (oracle-l5r-10553, strategy-wave-28) on the multi-target primitive (#369)
Two up-front slots (your unbowed Personality, a new own-unbowed-personality category; an enemy card) and the existing delayed straighten, per Mendon: the first bow is an effect, so the two bows and the straighten are independent effects. Fallen and Magistrate are keywords; the condition is read when the action resolves. Strategy package with the art's sha256 checked against the receipt, wave manifest, BLOCKERS removed, inventory regenerated.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.1%</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
@@ -59938,14 +59938,10 @@
       </c>
       <c r="F1769" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1769" t="inlineStr">
-        <is>
-          <t>The DELAYED conditional "straighten him before this battle resolves" exists (issue #354) and Fallen/Magistrate are readable keywords, but the action names TWO targets (your unbowed Personality and an enemy card) and the engine offers one: an action option lists the legal targets of a single choice. The multi-target selection it needs exists since PR #348 (TargetSlots.cs: two up-front slots, an own unbowed Personality and an enemy card; one before-action window per target; the delayed straighten is RegisterDelayedBattleEffect "straighten"), so wiring it is now an ability with two slots, one effect case and the Strategy package (scan on hand, no download needed).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1769" t="inlineStr"/>
     </row>
     <row r="1770">
       <c r="A1770" t="inlineStr">

</xml_diff>

<commit_message>
Gold payment rulings: opponent's variable payment (Virtuous Charity), dead-pile recruit (At Any Cost), current-cost totals (Disgraceful Conduct, A Stain Cleansed) (#373)
Mendon's answers to the generalized Gold payment's open questions. The second
player is shown the first player's Virtuous Charity amount and pays any amount
from 0 to what they can produce through the ordinary payment path (a general
primitive: OpponentPayment.cs, MatchView.PendingOpponentPayment, the
chooseOpponentPayment command). At Any Cost recruits a dead Samurai through
QuotePurchase itself (Unique/Singular, Sensei, Honor Requirement, Loyal, never
proclaimed). Disgraceful Conduct and A Stain Cleansed are priced from a unit's
current total Gold cost. Wired as strategy-wave-29; decision docs, tests with
mutation checks, and a scripted showcase scenario for the UI issue (#377).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.6%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>20.8%</t>
         </is>
       </c>
     </row>
@@ -43002,7 +43002,7 @@
       </c>
       <c r="F1265" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1265" t="inlineStr"/>
@@ -43868,7 +43868,7 @@
       </c>
       <c r="F1291" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1291" t="inlineStr"/>
@@ -46577,7 +46577,7 @@
       </c>
       <c r="F1372" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1372" t="inlineStr"/>
@@ -61777,7 +61777,7 @@
       </c>
       <c r="F1824" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1824" t="inlineStr"/>

</xml_diff>

<commit_message>
Wire The Tale of the Disgraced (oracle-l5r-10553, strategy-wave-28) on the multi-target primitive (#369) (#376)
Two up-front slots (your unbowed Personality, a new own-unbowed-personality category; an enemy card) and the existing delayed straighten, per Mendon: the first bow is an effect, so the two bows and the straighten are independent effects. Fallen and Magistrate are keywords; the condition is read when the action resolves. Strategy package with the art's sha256 checked against the receipt, wave manifest, BLOCKERS removed, inventory regenerated.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.1%</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
@@ -59934,14 +59934,10 @@
       </c>
       <c r="F1769" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1769" t="inlineStr">
-        <is>
-          <t>The DELAYED conditional "straighten him before this battle resolves" exists (issue #354) and Fallen/Magistrate are readable keywords, but the action names TWO targets (your unbowed Personality and an enemy card) and the engine offers one: an action option lists the legal targets of a single choice. The multi-target selection it needs exists since PR #348 (TargetSlots.cs: two up-front slots, an own unbowed Personality and an enemy card; one before-action window per target; the delayed straighten is RegisterDelayedBattleEffect "straighten"), so wiring it is now an ability with two slots, one effect case and the Strategy package (scan on hand, no download needed).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1769" t="inlineStr"/>
     </row>
     <row r="1770">
       <c r="A1770" t="inlineStr">

</xml_diff>

<commit_message>
Gold payment rulings: opponent's variable payment (Virtuous Charity), dead-pile recruit (At Any Cost), current-cost totals (Disgraceful Conduct, A Stain Cleansed) (#373) (#378)
Mendon's answers to the generalized Gold payment's open questions. The second
player is shown the first player's Virtuous Charity amount and pays any amount
from 0 to what they can produce through the ordinary payment path (a general
primitive: OpponentPayment.cs, MatchView.PendingOpponentPayment, the
chooseOpponentPayment command). At Any Cost recruits a dead Samurai through
QuotePurchase itself (Unique/Singular, Sensei, Honor Requirement, Loyal, never
proclaimed). Disgraceful Conduct and A Stain Cleansed are priced from a unit's
current total Gold cost. Wired as strategy-wave-29; decision docs, tests with
mutation checks, and a scripted showcase scenario for the UI issue (#377).

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>20.8%</t>
         </is>
       </c>
     </row>
@@ -42998,7 +42998,7 @@
       </c>
       <c r="F1265" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1265" t="inlineStr"/>
@@ -43864,7 +43864,7 @@
       </c>
       <c r="F1291" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1291" t="inlineStr"/>
@@ -46573,7 +46573,7 @@
       </c>
       <c r="F1372" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1372" t="inlineStr"/>
@@ -61769,7 +61769,7 @@
       </c>
       <c r="F1824" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1824" t="inlineStr"/>

</xml_diff>

<commit_message>
Created copies: a real copy of the target with a per-instance created marker; Gates of Chikushudo
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -570,14 +570,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C16" t="n">
         <v>2147</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>21.0%</t>
         </is>
       </c>
     </row>
@@ -37203,7 +37203,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1091" t="inlineStr"/>
+      <c r="G1091" t="inlineStr">
+        <is>
+          <t>Created copies exist now (issue #398: a real copy of the target, marked as created; Gates of Chikushudo is the first user). Still needs a second target (bow one of your unbowed Personalities, copy another), the Item removing itself from the game as a cost, 'will not straighten, attack, or defend until after your next turn begins' on the second target, and removing the copy after your next turn begins.</t>
+        </is>
+      </c>
     </row>
     <row r="1092">
       <c r="A1092" t="inlineStr">
@@ -39386,7 +39390,7 @@
       </c>
       <c r="F1157" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1157" t="inlineStr"/>
@@ -43488,7 +43492,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1280" t="inlineStr"/>
+      <c r="G1280" t="inlineStr">
+        <is>
+          <t>Created copies exist now (issue #398) but this is a PARTIAL copy: the created Personality has the target's printed Force, Chi, Personal Honor and keywords and copies all its abilities except those that copy abilities, and no other text; it needs a per-instance printed definition (planned with the per-instance created values), a target restriction (non-Unique) and a Battle-less Limited action performed by an Artisan, plus removal when your next turn begins.</t>
+        </is>
+      </c>
     </row>
     <row r="1281">
       <c r="A1281" t="inlineStr">
@@ -60935,7 +60943,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1799" t="inlineStr"/>
+      <c r="G1799" t="inlineStr">
+        <is>
+          <t>Created copies exist now (issue #398) but this is a partial copy with computed Force: the same base Chi, Personal Honor and keywords as the target Paragon and a base Force equal to the target's Personal Honor, removed after the battle; needs the per-instance printed definition planned with the per-instance created values.</t>
+        </is>
+      </c>
     </row>
     <row r="1800">
       <c r="A1800" t="inlineStr">

</xml_diff>

<commit_message>
Ability grants (#386): attachment cleanup, attack-Reaction usage check, public showcase, native probe, decision record
Resumed after pause: preserves the local work after 5881cc19 before integrating main.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.9%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C16" t="n">
         <v>2146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>20.8%</t>
+          <t>20.9%</t>
         </is>
       </c>
     </row>
@@ -38360,7 +38360,7 @@
       </c>
       <c r="G1126" t="inlineStr">
         <is>
-          <t>Needs a created Item instance carrying its own brand-new, ad-hoc printed ability ('Battle: Bow a target enemy card without attachments') -- CreatePersonality's own doc comment explicitly scopes a created attachment as accepted future scope, not built, and even that would only cover instantiating a fixed pre-existing CardDefinition, not minting one with novel ability text at runtime (the same underlying gap as oracle-l5r-7420's own runtime ability grant).</t>
+          <t>Predefined per-card ability grants exist (#386); generating novel ability text at runtime is unnecessary. Not yet wired: create the Item with its predefined enemy-card-without-attachments bow ability and implement the creating card's remaining text.</t>
         </is>
       </c>
     </row>
@@ -56608,7 +56608,7 @@
       </c>
       <c r="G1670" t="inlineStr">
         <is>
-          <t>Needs a genuinely new primitive: granting a brand-new, ad-hoc, printed-on-this-card ability (with its own Target/Timing) to an arbitrary target CardInstance at runtime, permanently. GrantedKeywords already covers granting a KEYWORD this way; nothing grants a whole new ABILITY id this way -- CardDefinition.Abilities is fixed per definition, never per-instance.</t>
+          <t>Permanent per-card ability grants exist (#338/#386). Not yet wired: still needs the granted Reaction that delays destruction from the targeting action until before turn end, plus permanent +2F.</t>
         </is>
       </c>
     </row>
@@ -56678,7 +56678,7 @@
       </c>
       <c r="G1672" t="inlineStr">
         <is>
-          <t>Same gap as oracle-l5r-7420 (Spirit of the Berserker): needs a runtime per-instance ability grant, not just a keyword grant.</t>
+          <t>Permanent per-card ability grants exist (#386). Not yet wired: define its Iaijutsu Battle duel with move-home stakes and the Duelist keyword alternative; the grant mechanism is no longer a blocker.</t>
         </is>
       </c>
     </row>
@@ -56710,14 +56710,10 @@
       </c>
       <c r="F1673" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1673" t="inlineStr">
-        <is>
-          <t>Same gap as oracle-l5r-7420 (Spirit of the Berserker): needs a runtime per-instance ability grant, not just a keyword grant.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1673" t="inlineStr"/>
     </row>
     <row r="1674">
       <c r="A1674" t="inlineStr">
@@ -56752,7 +56748,7 @@
       </c>
       <c r="G1674" t="inlineStr">
         <is>
-          <t>Same gap as oracle-l5r-7420 (Spirit of the Berserker): needs a runtime per-instance ability grant, not just a keyword grant.</t>
+          <t>Permanent per-card ability grants exist (#386). Not yet wired: define its enemy Force-or-Personal-Honor comparison bow action and Paragon keyword alternative; the grant mechanism is no longer a blocker.</t>
         </is>
       </c>
     </row>
@@ -56789,7 +56785,7 @@
       </c>
       <c r="G1675" t="inlineStr">
         <is>
-          <t>Same gap as oracle-l5r-7420 (Spirit of the Berserker): needs a runtime per-instance ability grant, not just a keyword grant.</t>
+          <t>Permanent per-card ability grants exist (#386). Not yet wired: define the granted Ranged 4 Attack with its conditional bow cost unless Reconnaissance, and the Scout keyword alternative.</t>
         </is>
       </c>
     </row>
@@ -56925,7 +56921,7 @@
       </c>
       <c r="G1679" t="inlineStr">
         <is>
-          <t>Same gap as oracle-l5r-7420 (Spirit of the Berserker): needs a runtime per-instance ability grant, not just a keyword grant.</t>
+          <t>Permanent per-card ability grants exist (#386). Not yet wired: define the granted same-location target-redirection Reaction, reusing TargetedActionReactions where applicable, and the Yojimbo keyword alternative.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grant permanent abilities to individual cards; wire Spirit of the Monk (#388)
* Build permanent per-card ability grants with Spirit of the Monk (#386)

* Ability grants (#386): attachment cleanup, attack-Reaction usage check, public showcase, native probe, decision record

Resumed after pause: preserves the local work after 5881cc19 before integrating main.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Ability grants (#386): record native verification and update the handoff

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.9%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C16" t="n">
         <v>2152</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>21.3%</t>
         </is>
       </c>
     </row>
@@ -56774,7 +56774,7 @@
       </c>
       <c r="G1676" t="inlineStr">
         <is>
-          <t>Needs a genuinely new primitive: granting a brand-new, ad-hoc, printed-on-this-card ability (with its own Target/Timing) to an arbitrary target CardInstance at runtime, permanently. GrantedKeywords already covers granting a KEYWORD this way; nothing grants a whole new ABILITY id this way -- CardDefinition.Abilities is fixed per definition, never per-instance.</t>
+          <t>Permanent per-card ability grants exist (#338/#386). Not yet wired: still needs the granted Reaction that delays destruction from the targeting action until before turn end, plus permanent +2F.</t>
         </is>
       </c>
     </row>
@@ -56844,7 +56844,7 @@
       </c>
       <c r="G1678" t="inlineStr">
         <is>
-          <t>Same gap as oracle-l5r-7420 (Spirit of the Berserker): needs a runtime per-instance ability grant, not just a keyword grant.</t>
+          <t>Permanent per-card ability grants exist (#386). Not yet wired: define its Iaijutsu Battle duel with move-home stakes and the Duelist keyword alternative; the grant mechanism is no longer a blocker.</t>
         </is>
       </c>
     </row>
@@ -56876,14 +56876,10 @@
       </c>
       <c r="F1679" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1679" t="inlineStr">
-        <is>
-          <t>Same gap as oracle-l5r-7420 (Spirit of the Berserker): needs a runtime per-instance ability grant, not just a keyword grant.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1679" t="inlineStr"/>
     </row>
     <row r="1680">
       <c r="A1680" t="inlineStr">
@@ -56918,7 +56914,7 @@
       </c>
       <c r="G1680" t="inlineStr">
         <is>
-          <t>Same gap as oracle-l5r-7420 (Spirit of the Berserker): needs a runtime per-instance ability grant, not just a keyword grant.</t>
+          <t>Permanent per-card ability grants exist (#386). Not yet wired: define its enemy Force-or-Personal-Honor comparison bow action and Paragon keyword alternative; the grant mechanism is no longer a blocker.</t>
         </is>
       </c>
     </row>
@@ -56955,7 +56951,7 @@
       </c>
       <c r="G1681" t="inlineStr">
         <is>
-          <t>Same gap as oracle-l5r-7420 (Spirit of the Berserker): needs a runtime per-instance ability grant, not just a keyword grant.</t>
+          <t>Permanent per-card ability grants exist (#386). Not yet wired: define the granted Ranged 4 Attack with its conditional bow cost unless Reconnaissance, and the Scout keyword alternative.</t>
         </is>
       </c>
     </row>
@@ -57091,7 +57087,7 @@
       </c>
       <c r="G1685" t="inlineStr">
         <is>
-          <t>Same gap as oracle-l5r-7420 (Spirit of the Berserker): needs a runtime per-instance ability grant, not just a keyword grant.</t>
+          <t>Permanent per-card ability grants exist (#386). Not yet wired: define the granted same-location target-redirection Reaction, reusing TargetedActionReactions where applicable, and the Yojimbo keyword alternative.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Created copies: a real copy of the target with a per-instance created marker; Gates of Chikushudo (#399)
Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -570,14 +570,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C16" t="n">
         <v>2152</v>
@@ -37315,7 +37315,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1095" t="inlineStr"/>
+      <c r="G1095" t="inlineStr">
+        <is>
+          <t>Created copies exist now (issue #398: a real copy of the target, marked as created; Gates of Chikushudo is the first user). Still needs a second target (bow one of your unbowed Personalities, copy another), the Item removing itself from the game as a cost, 'will not straighten, attack, or defend until after your next turn begins' on the second target, and removing the copy after your next turn begins.</t>
+        </is>
+      </c>
     </row>
     <row r="1096">
       <c r="A1096" t="inlineStr">
@@ -39527,7 +39531,7 @@
       </c>
       <c r="F1162" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1162" t="inlineStr"/>
@@ -43629,7 +43633,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1285" t="inlineStr"/>
+      <c r="G1285" t="inlineStr">
+        <is>
+          <t>Created copies exist now (issue #398) but this is a PARTIAL copy: the created Personality has the target's printed Force, Chi, Personal Honor and keywords and copies all its abilities except those that copy abilities, and no other text; it needs a per-instance printed definition (planned with the per-instance created values), a target restriction (non-Unique) and a Battle-less Limited action performed by an Artisan, plus removal when your next turn begins.</t>
+        </is>
+      </c>
     </row>
     <row r="1286">
       <c r="A1286" t="inlineStr">
@@ -61072,7 +61080,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1804" t="inlineStr"/>
+      <c r="G1804" t="inlineStr">
+        <is>
+          <t>Created copies exist now (issue #398) but this is a partial copy with computed Force: the same base Chi, Personal Honor and keywords as the target Paragon and a base Force equal to the target's Personal Honor, removed after the battle; needs the per-instance printed definition planned with the per-instance created values.</t>
+        </is>
+      </c>
     </row>
     <row r="1805">
       <c r="A1805" t="inlineStr">

</xml_diff>

<commit_message>
Second City pass (#264): blockers and decision doc for the five rulings cards, workbook, art imports, stronger Dislodge test
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -498,14 +498,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" t="n">
         <v>51</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>23.5%</t>
         </is>
       </c>
     </row>
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="C16" t="n">
         <v>2159</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>22.8%</t>
+          <t>23.1%</t>
         </is>
       </c>
     </row>
@@ -1294,14 +1294,10 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Two gaps: 'Negate the first movement each battle into attacking armies at your provinces' battlefields from other players' actions' is a per-battle counter hooked into every action-driven movement to a battlefield (there is no such hook), and 'Your forests are maddening' prints no mechanical text (a ruling on whether it is flavor). Its Limited half, 'Bow your target Forest to gain 1 Honor', is easy (Forest is a keyword on Holdings, Regions and Spells).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -42926,14 +42922,10 @@
       </c>
       <c r="F1265" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1265" t="inlineStr">
-        <is>
-          <t>Blocked on a ruling, not a primitive. The Gold-cost pieces exist (a Gold Cost stat modifier, tokens and 'reduce its Gold Cost to 0' from #336, and 'target your performing X' is a Performer, as Strength of the Bear does). What the printed text leaves open: whether 'If your Personality is a Magistrate, you may target an enemy card and reduce its Gold Cost to 0' is a second, independent, optional target (bow one card that has a lower Gold Cost AND separately zero another's), or the Magistrate's way round the restriction (zero a card's Gold Cost so that it counts as 'lower', then bow it, even with attachments); whether 'lower Gold Cost' is the performer's current or printed Gold Cost; and how long the reduction lasts.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1265" t="inlineStr"/>
     </row>
     <row r="1266">
       <c r="A1266" t="inlineStr">
@@ -46893,14 +46885,10 @@
       </c>
       <c r="F1384" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1384" t="inlineStr">
-        <is>
-          <t>'One or more of your performing Tacticians' are performers, and an ability has one Performer; modelling them as a 1-to-N target slot (multi-target slots exist, #336) would make them targets of reactions, which the printed 'performing' does not say -- a modelling ruling for Mendon. Also needs them all at one non-current battlefield with the enemy Personality opposing them there, and 'move the targets to the current battlefield' for every chosen card (MoveSpec has PerformerAndTarget and SourceAndTarget, no 'each chosen card').</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1384" t="inlineStr"/>
     </row>
     <row r="1385">
       <c r="A1385" t="inlineStr">
@@ -51284,14 +51272,10 @@
       </c>
       <c r="F1515" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1515" t="inlineStr">
-        <is>
-          <t>Its Reactions are played FROM A HAND when another player's action targets your Samurai (the second, 'after a Fear action', also needs the Fear classification, which exists: ActionKeywords ["Fear"]). The targeted-by-action window is offered from in-play cards only (TargetedActionReactionCandidates). Offering it from a hand means the window opens only when its reactor holds a matching card, which shows the opponent that he does (Unimpeachable Name accepts that for its own window) -- a hidden-information ruling for Mendon first.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1515" t="inlineStr"/>
     </row>
     <row r="1516">
       <c r="A1516" t="inlineStr">
@@ -60606,14 +60590,10 @@
       </c>
       <c r="F1793" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1793" t="inlineStr">
-        <is>
-          <t>Its Focus Effect is close: winner's controller gains 2 Honor is direct, but 'negate any destruction for losing this duel' must apply BEFORE the duel's own outcome (ApplyDuelOutcome runs first, the focus effects after). Its Reaction, 'after another player's Iaijutsu action targets your Personality: negate his destruction', is played from a hand: the Iaijutsu classification exists now (ActionKeywords), but a targeted-by-action window offered from a hand is the same hidden-information ruling as oracle-l5r-4481.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1793" t="inlineStr"/>
     </row>
     <row r="1794">
       <c r="A1794" t="inlineStr">

</xml_diff>

<commit_message>
Second City pass (#264): wire the five cards Mendon's rulings unblocked (#414)
* Second City pass (#264): wire the four cards Mendon's rulings unblocked (Know No Fear, To First Blood, A Fugitive Apprehended, Dislodge the Foe) and Kyuden Kitsune

* Second City pass (#264): blockers and decision doc for the five rulings cards, workbook, art imports, stronger Dislodge test

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Second City pass (#264): handoff for the rulings follow-up

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -498,14 +498,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" t="n">
         <v>51</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>23.5%</t>
         </is>
       </c>
     </row>
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="C16" t="n">
         <v>2159</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>22.8%</t>
+          <t>23.1%</t>
         </is>
       </c>
     </row>
@@ -1294,14 +1294,10 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Two gaps: 'Negate the first movement each battle into attacking armies at your provinces' battlefields from other players' actions' is a per-battle counter hooked into every action-driven movement to a battlefield (there is no such hook), and 'Your forests are maddening' prints no mechanical text (a ruling on whether it is flavor). Its Limited half, 'Bow your target Forest to gain 1 Honor', is easy (Forest is a keyword on Holdings, Regions and Spells).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -42926,14 +42922,10 @@
       </c>
       <c r="F1265" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1265" t="inlineStr">
-        <is>
-          <t>Blocked on a ruling, not a primitive. The Gold-cost pieces exist (a Gold Cost stat modifier, tokens and 'reduce its Gold Cost to 0' from #336, and 'target your performing X' is a Performer, as Strength of the Bear does). What the printed text leaves open: whether 'If your Personality is a Magistrate, you may target an enemy card and reduce its Gold Cost to 0' is a second, independent, optional target (bow one card that has a lower Gold Cost AND separately zero another's), or the Magistrate's way round the restriction (zero a card's Gold Cost so that it counts as 'lower', then bow it, even with attachments); whether 'lower Gold Cost' is the performer's current or printed Gold Cost; and how long the reduction lasts.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1265" t="inlineStr"/>
     </row>
     <row r="1266">
       <c r="A1266" t="inlineStr">
@@ -46893,14 +46885,10 @@
       </c>
       <c r="F1384" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1384" t="inlineStr">
-        <is>
-          <t>'One or more of your performing Tacticians' are performers, and an ability has one Performer; modelling them as a 1-to-N target slot (multi-target slots exist, #336) would make them targets of reactions, which the printed 'performing' does not say -- a modelling ruling for Mendon. Also needs them all at one non-current battlefield with the enemy Personality opposing them there, and 'move the targets to the current battlefield' for every chosen card (MoveSpec has PerformerAndTarget and SourceAndTarget, no 'each chosen card').</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1384" t="inlineStr"/>
     </row>
     <row r="1385">
       <c r="A1385" t="inlineStr">
@@ -51284,14 +51272,10 @@
       </c>
       <c r="F1515" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1515" t="inlineStr">
-        <is>
-          <t>Its Reactions are played FROM A HAND when another player's action targets your Samurai (the second, 'after a Fear action', also needs the Fear classification, which exists: ActionKeywords ["Fear"]). The targeted-by-action window is offered from in-play cards only (TargetedActionReactionCandidates). Offering it from a hand means the window opens only when its reactor holds a matching card, which shows the opponent that he does (Unimpeachable Name accepts that for its own window) -- a hidden-information ruling for Mendon first.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1515" t="inlineStr"/>
     </row>
     <row r="1516">
       <c r="A1516" t="inlineStr">
@@ -60606,14 +60590,10 @@
       </c>
       <c r="F1793" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1793" t="inlineStr">
-        <is>
-          <t>Its Focus Effect is close: winner's controller gains 2 Honor is direct, but 'negate any destruction for losing this duel' must apply BEFORE the duel's own outcome (ApplyDuelOutcome runs first, the focus effects after). Its Reaction, 'after another player's Iaijutsu action targets your Personality: negate his destruction', is played from a hand: the Iaijutsu classification exists now (ActionKeywords), but a targeted-by-action window offered from a hand is the same hidden-information ruling as oracle-l5r-4481.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1793" t="inlineStr"/>
     </row>
     <row r="1794">
       <c r="A1794" t="inlineStr">

</xml_diff>

<commit_message>
Second City primitives 1/6 (#415): timed straighten holds, movement locks, Hibernation's shield; wire Hibernation, Visitation, Strength of the Tsunami
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -570,14 +570,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="C16" t="n">
         <v>2159</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>23.1%</t>
+          <t>23.2%</t>
         </is>
       </c>
     </row>
@@ -41330,14 +41330,10 @@
       </c>
       <c r="F1217" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1217" t="inlineStr">
-        <is>
-          <t>Its first Battle ability ('even if this card is bowed, if this Shugenja is Water: straighten him, and you may move him home') works through the per-ability 'Even if bowed' exemption, and '+6F' is a static wielder bonus. The second, 'target an enemy Personality: move him home; if he moved, negate his (future) movement', needs a ruling on how long the negation lasts (the parenthesis is unexplained) and a per-card movement-negation flag, parallel to StraightenBlockedTurn.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1217" t="inlineStr"/>
     </row>
     <row r="1218">
       <c r="A1218" t="inlineStr">
@@ -49804,14 +49800,10 @@
       </c>
       <c r="F1471" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1471" t="inlineStr">
-        <is>
-          <t>Needs (a) 'negate its straightening until your next turn begins' -- StraightenBlockedTurn is one turn number and StraightenLockedTurn (Basic Lesson) one whole turn, neither spans another player's turn; (b) a standing watch across turns, 'after the next time this game another player's Battle action targets it, negate the action's effects' (NegateAllEffectsOn is per held action); its Nonhuman performer for an Open action works now.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1471" t="inlineStr"/>
     </row>
     <row r="1472">
       <c r="A1472" t="inlineStr">
@@ -62054,14 +62046,10 @@
       </c>
       <c r="F1837" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1837" t="inlineStr">
-        <is>
-          <t>Its Limited half (if you control an Ancestor Personality gain 2 Honor; each player who does not loses 2) is direct. Its Open half needs 'negate his straightening until after you reveal cards in your Provinces at the start of your next turn' -- a straighten lock that spans the other player's turn and ends at a named step of yours (StraightenBlockedTurn is one turn number) -- and an Ancestor performer destroyed as its cost (both exist).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1837" t="inlineStr"/>
     </row>
     <row r="1838">
       <c r="A1838" t="inlineStr">

</xml_diff>

<commit_message>
Second City primitives 2/6 (#416): Gold cost from a printed number, conditional Holding production, temporary keyword removal; wire A Quiet Transaction, Red Crane Dojo, Bushi Dojo
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
@@ -606,14 +606,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C11" t="n">
         <v>151</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.3%</t>
+          <t>12.6%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C16" t="n">
         <v>2159</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>23.2%</t>
+          <t>23.3%</t>
         </is>
       </c>
     </row>
@@ -43215,14 +43215,10 @@
       </c>
       <c r="F1274" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1274" t="inlineStr">
-        <is>
-          <t>Its second Open half (two -2 Gold Cost tokens on a dishonorable Personality) is expressible now (CreateToken with the GoldCost stat, #336). The first half is not: it needs a Gold cost rule for 'Gold equal to his base Personal Honor plus one' (GoldCostBasis has no Personal Honor basis) and 'may not be assigned, and will not move, to battlefields this turn' -- no per-card flag blocks assignment or movement to a battlefield (compare StraightenBlockedTurn / StraightenLockedTurn).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1274" t="inlineStr"/>
     </row>
     <row r="1275">
       <c r="A1275" t="inlineStr">
@@ -63172,7 +63168,7 @@
       </c>
       <c r="F1871" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1871" t="inlineStr"/>
@@ -65412,14 +65408,10 @@
       </c>
       <c r="F1939" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1939" t="inlineStr">
-        <is>
-          <t>Two gaps. (a) '4 Gold when paying for a Ninja card, which may only pay for that card' -- every Gold-production bonus is unconditional (crane-gold/dragon-gold), none is restricted to a purchase. (b) Its Reaction ('after an action targets your Personality, remove Ninja and Shadowlands from him until the action ends') has its trigger now (targeted-by-action offers in-play cards, a Holding included), but RemovedKeywords has no duration: a keyword removal that ends with the action is unbuilt.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1939" t="inlineStr"/>
     </row>
     <row r="1940">
       <c r="A1940" t="inlineStr">

</xml_diff>

<commit_message>
Second City primitives 3/6 (#417): the after-resolution window; wire Never Safe, Redoubled Attack, Tales of Dishonor, Quagmire
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
@@ -660,14 +660,14 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C14" t="n">
         <v>26</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>19.2%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="C16" t="n">
         <v>2159</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>23.5%</t>
         </is>
       </c>
     </row>
@@ -52715,14 +52715,10 @@
       </c>
       <c r="F1558" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1558" t="inlineStr">
-        <is>
-          <t>-4F to an enemy Personality or Follower is a stat penalty and works now. 'After this battle ends, if this card is in your discard pile, you may put it into your hand' is a delayed effect of a played Strategy that outlives its action: DelayedBattleEffects run before resolution only, and no other 'after this battle ends' window exists (the Rings' recruit window is the only one).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1558" t="inlineStr"/>
     </row>
     <row r="1559">
       <c r="A1559" t="inlineStr">
@@ -54632,14 +54628,10 @@
       </c>
       <c r="F1615" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1615" t="inlineStr">
-        <is>
-          <t>Needs an 'after a battle's resolution ends' Reaction window (the Rings' recruit window is the only one after resolution) and a ruling on 'They will not bow from the battle's resolution', which reads as a statement about a resolution that has already ended. The one-or-two 'performing Personalities' are performers (an ability has one Performer).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1615" t="inlineStr"/>
     </row>
     <row r="1616">
       <c r="A1616" t="inlineStr">
@@ -58562,14 +58554,10 @@
       </c>
       <c r="F1733" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1733" t="inlineStr">
-        <is>
-          <t>Its Battle half (straighten a Magistrate performer) is trivial. Its Political Reaction, 'after the resolution of a battle at a province, if you destroyed any enemy units or a province in that resolution: the battle's loser loses 4 Honor', needs an after-resolution window that knows what the resolution destroyed (the Rings' recruit window is the only one after resolution, and it records recruits, not casualties).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1733" t="inlineStr"/>
     </row>
     <row r="1734">
       <c r="A1734" t="inlineStr">
@@ -71946,14 +71934,10 @@
       </c>
       <c r="F2137" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2137" t="inlineStr">
-        <is>
-          <t>OpenBowReactionWindow (the shared bowed-personality-at-own-battlefield Reaction watcher Hizumi/Ruya both already use) hardcodes AtBattle(c) for the watching card and same-province-only matching for its own trigger condition -- both structurally exclude a Region source (never AtBattle-eligible) and its own "at this province or an adjacent province" text. Reusable only by loosening that SHARED function (adding an AdjacentProvinces branch and waiving its own AtBattle check), which is genuine shared-infrastructure surgery, not a routine per-card wiring addition, and risks regressing Hizumi/Ruya's own already-published behavior.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2137" t="inlineStr"/>
     </row>
     <row r="2138">
       <c r="A2138" t="inlineStr">

</xml_diff>

<commit_message>
Second City primitives 1/6 (#415): timed straighten holds, movement locks, Hibernation's shield; wire Hibernation, Visitation, Strength of the Tsunami (#421)
Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -570,14 +570,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="C16" t="n">
         <v>2159</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>23.1%</t>
+          <t>23.2%</t>
         </is>
       </c>
     </row>
@@ -41330,14 +41330,10 @@
       </c>
       <c r="F1217" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1217" t="inlineStr">
-        <is>
-          <t>Its first Battle ability ('even if this card is bowed, if this Shugenja is Water: straighten him, and you may move him home') works through the per-ability 'Even if bowed' exemption, and '+6F' is a static wielder bonus. The second, 'target an enemy Personality: move him home; if he moved, negate his (future) movement', needs a ruling on how long the negation lasts (the parenthesis is unexplained) and a per-card movement-negation flag, parallel to StraightenBlockedTurn.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1217" t="inlineStr"/>
     </row>
     <row r="1218">
       <c r="A1218" t="inlineStr">
@@ -49804,14 +49800,10 @@
       </c>
       <c r="F1471" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1471" t="inlineStr">
-        <is>
-          <t>Needs (a) 'negate its straightening until your next turn begins' -- StraightenBlockedTurn is one turn number and StraightenLockedTurn (Basic Lesson) one whole turn, neither spans another player's turn; (b) a standing watch across turns, 'after the next time this game another player's Battle action targets it, negate the action's effects' (NegateAllEffectsOn is per held action); its Nonhuman performer for an Open action works now.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1471" t="inlineStr"/>
     </row>
     <row r="1472">
       <c r="A1472" t="inlineStr">
@@ -62054,14 +62046,10 @@
       </c>
       <c r="F1837" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1837" t="inlineStr">
-        <is>
-          <t>Its Limited half (if you control an Ancestor Personality gain 2 Honor; each player who does not loses 2) is direct. Its Open half needs 'negate his straightening until after you reveal cards in your Provinces at the start of your next turn' -- a straighten lock that spans the other player's turn and ends at a named step of yours (StraightenBlockedTurn is one turn number) -- and an Ancestor performer destroyed as its cost (both exist).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1837" t="inlineStr"/>
     </row>
     <row r="1838">
       <c r="A1838" t="inlineStr">

</xml_diff>

<commit_message>
Second City primitives 4/6 (#418): province strength maximum and Terrain statics; wire Ancient Feud, Hasty Fortifications, Shiotome Plains
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="C16" t="n">
         <v>2159</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>23.7%</t>
         </is>
       </c>
     </row>
@@ -43912,14 +43912,10 @@
       </c>
       <c r="F1295" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1295" t="inlineStr">
-        <is>
-          <t>Terrain Strategies are playable (Looting the Ruins is the 'destroy a Terrain, then put this one into play' precedent, strategy-wave-10), so its Battle half is the routine shape. Its passive is not: 'this battlefield's province has a maximum strength equal to its base strength' caps a value that every province-strength change in the engine (Improved Defenses, Ring of Earth, Yogo Adi, Dueling) raises permanently on ProvinceState.Strength -- a cap needs an effective-strength read wherever strength is used (battle resolution and Attacks on the province).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1295" t="inlineStr"/>
     </row>
     <row r="1296">
       <c r="A1296" t="inlineStr">
@@ -49553,14 +49549,10 @@
       </c>
       <c r="F1464" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1464" t="inlineStr">
-        <is>
-          <t>Needs (a) the trait 'after each resolution of one of your own Battle actions (including this card's)' -- mandatory, repeatable and not tied to one effect kind (the nearest, Stormless Fury's after-battle-action-resolves, is an optional Reaction offered to a card in a hand, a discard pile or in play); and (b) '+1 strength until this card leaves play' stacking on a province and ending when the card leaves: ProvinceState.Strength is one integer, so a removable, per-source province modifier does not exist.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1464" t="inlineStr"/>
     </row>
     <row r="1465">
       <c r="A1465" t="inlineStr">
@@ -56261,14 +56253,10 @@
       </c>
       <c r="F1664" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1664" t="inlineStr">
-        <is>
-          <t>Terrain Strategies are playable (strategy-wave-10). The gap is its passive, 'While at this battlefield, Cavalry cards have +1F and Infantry cards have -1F': a Force change from a Terrain to cards there, read in PersonalityForce/FollowerForce. Cavalry is a printed keyword (144 cards, Personalities and Followers) but 'Infantry' has no keyword: the engine knows an Infantry UNIT as one without Cavalry (IsCavalryUnit's complement, Horseback Warriors). A ruling is needed on whether 'Infantry cards' are the Personality and Follower cards without Cavalry, and whether either side's cards are affected.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1664" t="inlineStr"/>
     </row>
     <row r="1665">
       <c r="A1665" t="inlineStr">

</xml_diff>

<commit_message>
Second City primitives 2/6 (#416): Gold cost from a printed number; conditional production; A Quiet Transaction, Red Crane Dojo, Bushi Dojo (#422)
* Second City primitives 1/6 (#415): timed straighten holds, movement locks, Hibernation's shield; wire Hibernation, Visitation, Strength of the Tsunami

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Second City primitives 2/6 (#416): Gold cost from a printed number, conditional Holding production, temporary keyword removal; wire A Quiet Transaction, Red Crane Dojo, Bushi Dojo

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
@@ -606,14 +606,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C11" t="n">
         <v>151</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.3%</t>
+          <t>12.6%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C16" t="n">
         <v>2159</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>23.2%</t>
+          <t>23.3%</t>
         </is>
       </c>
     </row>
@@ -43215,14 +43215,10 @@
       </c>
       <c r="F1274" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1274" t="inlineStr">
-        <is>
-          <t>Its second Open half (two -2 Gold Cost tokens on a dishonorable Personality) is expressible now (CreateToken with the GoldCost stat, #336). The first half is not: it needs a Gold cost rule for 'Gold equal to his base Personal Honor plus one' (GoldCostBasis has no Personal Honor basis) and 'may not be assigned, and will not move, to battlefields this turn' -- no per-card flag blocks assignment or movement to a battlefield (compare StraightenBlockedTurn / StraightenLockedTurn).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1274" t="inlineStr"/>
     </row>
     <row r="1275">
       <c r="A1275" t="inlineStr">
@@ -63172,7 +63168,7 @@
       </c>
       <c r="F1871" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1871" t="inlineStr"/>
@@ -65412,14 +65408,10 @@
       </c>
       <c r="F1939" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1939" t="inlineStr">
-        <is>
-          <t>Two gaps. (a) '4 Gold when paying for a Ninja card, which may only pay for that card' -- every Gold-production bonus is unconditional (crane-gold/dragon-gold), none is restricted to a purchase. (b) Its Reaction ('after an action targets your Personality, remove Ninja and Shadowlands from him until the action ends') has its trigger now (targeted-by-action offers in-play cards, a Holding included), but RemovedKeywords has no duration: a keyword removal that ends with the action is unbuilt.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1939" t="inlineStr"/>
     </row>
     <row r="1940">
       <c r="A1940" t="inlineStr">

</xml_diff>

<commit_message>
Second City primitives 5/6: other-player decisions, a paused Focus Effect, sequenced targets
Know Their Minds, Scandalous Rumors, Dragon's Breath Castle, Disreputable Deal
and Engulfing Flames, built on three general primitives (issue #419).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -498,14 +498,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5" t="n">
         <v>51</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>25.5%</t>
         </is>
       </c>
     </row>
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>18.6%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="C16" t="n">
         <v>2159</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>23.7%</t>
+          <t>23.9%</t>
         </is>
       </c>
     </row>
@@ -894,14 +894,10 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Two halves, both unbuilt. (a) 'After another player's Dynasty Phase begins, if he controls any Personalities and he assigned none of them to an attacking army this turn: gain 2 Honor' is a mandatory start-of-phase trait: SetPhase(Dynasty) is the hook (Wave Man's straighten uses it) and AssignedToAttackTurn records assignment, so it is buildable. (b) 'Reaction: Even if bowed, after engaging at one of your provinces: The Attacker targets and bows one of his Personalities there' needs the OTHER player to make a targeting decision inside your Reaction (Either/Or offers fixed options only); the card cannot be half-wired.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -46972,14 +46968,10 @@
       </c>
       <c r="F1387" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1387" t="inlineStr">
-        <is>
-          <t>Its Political Open half is buildable now (a Courtier performer for an Open action works, actingAsBattle; -3F is a stat penalty; the Honor loss reads a printed Personal Honor). The Focus Effect is the gap: 'you may put a non-Unique Strategy with a Political ability in your discard pile into your hand' is a CHOICE made while the duel's Focus Effects resolve, and ApplyDuelFocusEffect applies fixed outcomes only -- no decision hook.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1387" t="inlineStr"/>
     </row>
     <row r="1388">
       <c r="A1388" t="inlineStr">
@@ -47607,14 +47599,10 @@
       </c>
       <c r="F1406" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1406" t="inlineStr">
-        <is>
-          <t>'You may target and destroy an enemy attachment' is an OPTIONAL target (a slot with Min 0) and 'if your Monk has any Fire tokens, Ranged 4 Attack' a conditional Attack in the same action. Slots exist (#336) but a multi-target ability never runs the Attack pipeline (ResolveOrDeferAttack takes one target; Kahoku exp carries an Attack's own target beside a primary one in CardIds) -- the combination is unbuilt.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1406" t="inlineStr"/>
     </row>
     <row r="1407">
       <c r="A1407" t="inlineStr">
@@ -51285,14 +51273,10 @@
       </c>
       <c r="F1516" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1516" t="inlineStr">
-        <is>
-          <t>Needs the OTHER player to choose which of his own face-up province Personalities is affected (Either/Or offers fixed options only) and a 'turn a face-up Personality back face-down' primitive that does not exist (every FaceUp transition in the engine is one-directional). Its Samurai Performer for an Open action works now.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1516" t="inlineStr"/>
     </row>
     <row r="1517">
       <c r="A1517" t="inlineStr">
@@ -55482,14 +55466,10 @@
       </c>
       <c r="F1641" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1641" t="inlineStr">
-        <is>
-          <t>Needs the ATTACKER (the other player, when you defend) to choose which of his own Personalities at the battlefield move home -- 'may target any of his Personalities' -- then lose 1 Honor for each that did not, and be dishonored: an opponent-made, variable selection inside your action (Either/Or offers fixed options). Its 'Courtier at any location' Performer (own-unbowed-personality-with-keyword-at-any-location) exists.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1641" t="inlineStr"/>
     </row>
     <row r="1642">
       <c r="A1642" t="inlineStr">

</xml_diff>

<commit_message>
Second City primitives 3/6 (#417): the after-resolution window; Never Safe, Redoubled Attack, Tales of Dishonor, Quagmire (#423)
* Second City primitives 1/6 (#415): timed straighten holds, movement locks, Hibernation's shield; wire Hibernation, Visitation, Strength of the Tsunami

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Second City primitives 2/6 (#416): Gold cost from a printed number, conditional Holding production, temporary keyword removal; wire A Quiet Transaction, Red Crane Dojo, Bushi Dojo

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Second City primitives 3/6 (#417): the after-resolution window; wire Never Safe, Redoubled Attack, Tales of Dishonor, Quagmire

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
@@ -660,14 +660,14 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C14" t="n">
         <v>26</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>19.2%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="C16" t="n">
         <v>2159</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>23.5%</t>
         </is>
       </c>
     </row>
@@ -52715,14 +52715,10 @@
       </c>
       <c r="F1558" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1558" t="inlineStr">
-        <is>
-          <t>-4F to an enemy Personality or Follower is a stat penalty and works now. 'After this battle ends, if this card is in your discard pile, you may put it into your hand' is a delayed effect of a played Strategy that outlives its action: DelayedBattleEffects run before resolution only, and no other 'after this battle ends' window exists (the Rings' recruit window is the only one).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1558" t="inlineStr"/>
     </row>
     <row r="1559">
       <c r="A1559" t="inlineStr">
@@ -54632,14 +54628,10 @@
       </c>
       <c r="F1615" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1615" t="inlineStr">
-        <is>
-          <t>Needs an 'after a battle's resolution ends' Reaction window (the Rings' recruit window is the only one after resolution) and a ruling on 'They will not bow from the battle's resolution', which reads as a statement about a resolution that has already ended. The one-or-two 'performing Personalities' are performers (an ability has one Performer).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1615" t="inlineStr"/>
     </row>
     <row r="1616">
       <c r="A1616" t="inlineStr">
@@ -58562,14 +58554,10 @@
       </c>
       <c r="F1733" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1733" t="inlineStr">
-        <is>
-          <t>Its Battle half (straighten a Magistrate performer) is trivial. Its Political Reaction, 'after the resolution of a battle at a province, if you destroyed any enemy units or a province in that resolution: the battle's loser loses 4 Honor', needs an after-resolution window that knows what the resolution destroyed (the Rings' recruit window is the only one after resolution, and it records recruits, not casualties).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1733" t="inlineStr"/>
     </row>
     <row r="1734">
       <c r="A1734" t="inlineStr">
@@ -71946,14 +71934,10 @@
       </c>
       <c r="F2137" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2137" t="inlineStr">
-        <is>
-          <t>OpenBowReactionWindow (the shared bowed-personality-at-own-battlefield Reaction watcher Hizumi/Ruya both already use) hardcodes AtBattle(c) for the watching card and same-province-only matching for its own trigger condition -- both structurally exclude a Region source (never AtBattle-eligible) and its own "at this province or an adjacent province" text. Reusable only by loosening that SHARED function (adding an AdjacentProvinces branch and waiving its own AtBattle check), which is genuine shared-infrastructure surgery, not a routine per-card wiring addition, and risks regressing Hizumi/Ruya's own already-published behavior.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2137" t="inlineStr"/>
     </row>
     <row r="2138">
       <c r="A2138" t="inlineStr">

</xml_diff>

<commit_message>
Second City primitives 6/6: permanent copy, Kata, target bars, dead Personalities as discarded
Mastering the Elements, Skipping the Puddle, Superior Reach and Scavenging Party
(issue #420).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -570,14 +570,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>19.1%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="C16" t="n">
         <v>2159</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>23.9%</t>
+          <t>24.1%</t>
         </is>
       </c>
     </row>
@@ -40225,14 +40225,10 @@
       </c>
       <c r="F1184" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1184" t="inlineStr">
-        <is>
-          <t>The copy primitives (CardCopy.cs, #338) copy ONE chosen keyword or ability from a discarded Personality. This Reaction 'permanently copies the Spell's keywords, traits, and its base abilities that do not themselves copy abilities' -- all of them, from a Spell in play, once per game, paying that Spell's base Gold Cost after this card enters play (the own-enters-play trigger exists). A permanent copy-all variant with the trait (Effect) / ability distinction, on a per-instance printed-values override (CardInstance.Printed, #399), is unbuilt.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1184" t="inlineStr"/>
     </row>
     <row r="1185">
       <c r="A1185" t="inlineStr">
@@ -55532,14 +55528,10 @@
       </c>
       <c r="F1643" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1643" t="inlineStr">
-        <is>
-          <t>Its Focus Effect (-3F to the duel's winner) and Open half (each of your provinces +2 strength) are buildable now. Its Limited half is not: 'Target your discarded Personality: Discard a card from one of your provinces and refill it face-up with the Personality' needs the Personality placed face-up into a province the player chooses in the command (Your Clan Needs You!'s province choice belongs to its end-of-battle flow, chooseYourClanNeedsYouProvince) and 'discarded' fixed as the Dynasty discard pile rather than the dead pile.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1643" t="inlineStr"/>
     </row>
     <row r="1644">
       <c r="A1644" t="inlineStr">
@@ -56398,14 +56390,10 @@
       </c>
       <c r="F1669" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1669" t="inlineStr">
-        <is>
-          <t>Needs a standing, unattached Strategy-in-play lifecycle distinct from every existing 'stays in play' shape (Terrain is battlefield-bound; Rings and Regions have their own Zones; an Event uses Zone.EventInPlay) for a Kata that gives its controller a repeatable, keyword-filtered Battle action while it sits in play; the entry effect ('discard all your other Kata') is routine.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1669" t="inlineStr"/>
     </row>
     <row r="1670">
       <c r="A1670" t="inlineStr">
@@ -58221,14 +58209,10 @@
       </c>
       <c r="F1724" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1724" t="inlineStr">
-        <is>
-          <t>Needs a targeting restriction between two cards -- 'actions the Personality performs may not target your performer', while the performer holds a Weapon, and for a duration the text does not give: the targeting-immunity family (oracle-l5r-4699/5010) is unbuilt, and this one is keyed to the acting Personality and a live condition on the performer. Its Force-to-0 half reuses the existing Set-Force pattern.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1724" t="inlineStr"/>
     </row>
     <row r="1725">
       <c r="A1725" t="inlineStr">

</xml_diff>

<commit_message>
Dueling/Focus Effect reevaluation: wire 3 of 8 Before the Dawn blockers, refresh the rest (#435)
Dueling (#204) and Focus Effects (#419) now exist, making the "Dueling/Focus
Effects (not started at all)" note on 8 Before the Dawn cards stale. Reevaluated
all eight: Hiromi's Vassals and Shamsir share a "attach this card to one of your
Personalities, ignoring Gold cost" Focus Effect, generalized as a third choice
kind on FocusEffectChoice.cs; Home Guard's mandatory +3F Focus Effect,
+3F-while-defending static and Battle bow-and-Honor-gain each reuse an existing
shape. The other five (Flanking Unit, Broken Cipher, Paralyzing Touch,
Splintered Weapon, The Courage of the Mantis) stay blocked, now on their real
gap (an attachment Transfer mechanic, a delayed negation of a future action, or
a delayed duel-loss-consequence mechanism) instead of the stale blanket note.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -534,14 +534,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C7" t="n">
         <v>127</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>62.2%</t>
+          <t>63.8%</t>
         </is>
       </c>
     </row>
@@ -552,14 +552,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C8" t="n">
         <v>131</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.7%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="C16" t="n">
         <v>2164</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>27.4%</t>
+          <t>27.5%</t>
         </is>
       </c>
     </row>
@@ -31138,7 +31138,7 @@
       </c>
       <c r="G912" t="inlineStr">
         <is>
-          <t>Needs Dueling/Focus Effects (not started at all).</t>
+          <t>Needs an attachment Transfer mechanic (same gap as oracle-l5r-2520/10900): its Focus Effect is "you may transfer a Follower from your Personality in this duel to another of your Personalities." The Battle half (move a target Personality at the current battlefield home or to an adjacent battlefield) is separately wirable.</t>
         </is>
       </c>
     </row>
@@ -31611,14 +31611,10 @@
       </c>
       <c r="F926" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G926" t="inlineStr">
-        <is>
-          <t>Needs Dueling/Focus Effects (not started at all).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G926" t="inlineStr"/>
     </row>
     <row r="927">
       <c r="A927" t="inlineStr">
@@ -31681,14 +31677,10 @@
       </c>
       <c r="F928" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G928" t="inlineStr">
-        <is>
-          <t>Needs Dueling/Focus Effects (not started at all).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G928" t="inlineStr"/>
     </row>
     <row r="929">
       <c r="A929" t="inlineStr">
@@ -37205,14 +37197,10 @@
       </c>
       <c r="F1092" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1092" t="inlineStr">
-        <is>
-          <t>Needs Dueling/Focus Effects (the Battle half, a plain Force debuff, is separately wirable).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1092" t="inlineStr"/>
     </row>
     <row r="1093">
       <c r="A1093" t="inlineStr">
@@ -37379,7 +37367,7 @@
       </c>
       <c r="G1097" t="inlineStr">
         <is>
-          <t>Needs Dueling/Focus Effects (the Battle half is separately wirable).</t>
+          <t>Needs an attachment Transfer mechanic (issue #435 reevaluation; same gap as oracle-l5r-2520/10900/2598/1151): its Focus Effect is "you may transfer an attachment from your Personality in this duel to another of your Personalities." The Battle half (an enemy card without attachments, bow it, destroy it if this Personality is a Berserker) is separately wirable.</t>
         </is>
       </c>
     </row>
@@ -45256,7 +45244,7 @@
       </c>
       <c r="G1334" t="inlineStr">
         <is>
-          <t>Needs Dueling/Focus Effects (not started at all).</t>
+          <t>Needs an attachment Transfer mechanic (issue #435 reevaluation; same gap as oracle-l5r-2520/10900/2598): its Focus Effect is "you may transfer a Spell from your Personality in this duel to another of your Shugenja at the same location." Its Battle half also needs two live-tracked conditions not built anywhere else: "you have not put cards into your hand this phase" and "you have attached a Spell this turn."</t>
         </is>
       </c>
     </row>
@@ -53741,7 +53729,7 @@
       </c>
       <c r="G1587" t="inlineStr">
         <is>
-          <t>Needs Dueling/Focus Effects (not started at all).</t>
+          <t>Needs a delayed negation of a FUTURE action (issue #435 reevaluation; same gap as oracle-l5r-2580): its Focus Effect is "after this duel ends, negate the effects of the next action performed by its winner" -- every negation the engine has applies to an action already being held in a reaction window, none waits on a card until it next acts. The Battle half (a Monk performer, move an enemy Personality to a different battlefield, conditional bow) is separately wirable.</t>
         </is>
       </c>
     </row>
@@ -59044,7 +59032,7 @@
       </c>
       <c r="G1746" t="inlineStr">
         <is>
-          <t>Needs Dueling/Focus Effects (the Battle half is separately wirable).</t>
+          <t>Needs a delayed duel-loss-consequence mechanism (issue #435 reevaluation): its Focus Effect is "you may choose (now) to delay the effects of losing this duel until after the next Dynasty Phase begins" -- genuinely novel duel-resolution-timing plumbing (Strength of the Spider, oracle-l5r-8362, is blocked on the identical clause and deliberately deferred rather than invented for one card; see CardAbilities.cs). The Battle half (a Mantis Clan performer, move to the current battlefield, an additional Battle action) is separately wirable.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire Akodo Ashiko: a Reserve recruit without the Reserve keyword (#440)
Her "Battle, [Gold]: If Ashiko is face-up in one of your Provinces,
Recruit her reducing her Gold Cost by 2 if there are more units on the
enemy side..." is exactly the Reserve keyword's own shape (RecruitReserve:
an absent battle action, no presence of her own side required, only enemy
presence), on a card that carries no printed Reserve keyword.
IsReserveRecruitable admits her by her own Effect string instead of adding
a keyword she does not have. The unit-count comparison reuses Army(playerId,
province) -- already the engine's live, always-current unit-count primitive
(e.g. barred-passage-bow) -- so no new primitive was needed; it is read
fresh at the moment she is recruited, reflecting any Battle action that
changed either side's presence since the battle began.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C6" t="n">
         <v>821</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>34.2%</t>
+          <t>34.3%</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C16" t="n">
         <v>2165</v>
@@ -2610,14 +2610,10 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>Needs a Battle-timed Recruit of the card itself from a Province. Recruit is a Dynasty-phase purchase (QuotePurchase); the only Battle-timed ways into play bring a dead Personality (At Any Cost, Goju Plot) or a Ring (Ring of Fire) into play, and nothing lets a face-up Province card act as a Battle action. The discount also reads a comparison of the unit counts on the two sides of the current battle.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">

</xml_diff>

<commit_message>
Wire the Emperor Edition Gempukku pass: all 17 unwired cards (#461)
holding-wave-10: the nine Market Holdings (produce 2 Gold; Limited bow draw
for a player of the printed Clan with four or fewer cards in hand).
personality-wave-65: Hida Yamadera, Doji Dainagon, Jade's Roar, Moshi Madoka,
Kunji, Shosuro Hawado (exp 2), Daigotsu Negishi, Shinjo Byung.

New primitives: abilities taken from the dead pile (FromDead), a
keyword-limited first Battle action (Jade's Roar's Terrain-only opportunity),
PlayerState.AttachedFromHandThisTurn, Negishi's conditional destruction
negation by unit Gold Cost, and a card-in-province target with face-up
refill. Removed the stale Jade's Roar blocker; no new blockers.

docs/CARD_INVENTORY.xlsx: 2172 cards, 803 wired (+17). Catalogue art pack
pinned to catalogue-art-pr461-20260924-r1 (3250 scans).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="C6" t="n">
         <v>826</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>44.4%</t>
         </is>
       </c>
     </row>
@@ -606,14 +606,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C11" t="n">
         <v>151</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>25.8%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>786</v>
+        <v>803</v>
       </c>
       <c r="C16" t="n">
         <v>2172</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>36.2%</t>
+          <t>37.0%</t>
         </is>
       </c>
     </row>
@@ -8304,7 +8304,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G227" t="inlineStr"/>
@@ -8807,7 +8807,7 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G242" t="inlineStr"/>
@@ -11001,7 +11001,7 @@
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G308" t="inlineStr"/>
@@ -13775,14 +13775,10 @@
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G390" t="inlineStr">
-        <is>
-          <t>The Engage window and first-action claim now exist (issue #310; Recon Reaction, Trigger after-engaging-at-own-battlefield, claim via ClaimFirstOpportunity). Still needs: the claim's printed restriction 'which must be a Terrain action' -- FirstActionRestriction already binds a first action to a performer (Naval Invasion) or to passing (Rebuilding Kyuden Hida); a required-keyword variant (an action from a Terrain-keyword card, including the playStrategy Terrain path) is the one new field.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -16920,7 +16916,7 @@
       </c>
       <c r="F483" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G483" t="inlineStr"/>
@@ -19006,7 +19002,7 @@
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G545" t="inlineStr"/>
@@ -22285,7 +22281,7 @@
       </c>
       <c r="F644" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G644" t="inlineStr"/>
@@ -23250,7 +23246,7 @@
       </c>
       <c r="F673" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G673" t="inlineStr"/>
@@ -63804,7 +63800,7 @@
       </c>
       <c r="F1883" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1883" t="inlineStr"/>
@@ -65912,7 +65908,7 @@
       </c>
       <c r="F1947" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1947" t="inlineStr"/>
@@ -67009,7 +67005,7 @@
       </c>
       <c r="F1980" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1980" t="inlineStr"/>
@@ -67409,7 +67405,7 @@
       </c>
       <c r="F1992" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1992" t="inlineStr"/>
@@ -67508,7 +67504,7 @@
       </c>
       <c r="F1995" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1995" t="inlineStr"/>
@@ -67640,7 +67636,7 @@
       </c>
       <c r="F1999" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1999" t="inlineStr"/>
@@ -67673,7 +67669,7 @@
       </c>
       <c r="F2000" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2000" t="inlineStr"/>
@@ -67772,7 +67768,7 @@
       </c>
       <c r="F2003" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2003" t="inlineStr"/>
@@ -68003,7 +67999,7 @@
       </c>
       <c r="F2010" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2010" t="inlineStr"/>

</xml_diff>

<commit_message>
Forgotten Legacy pass: decision doc, card inventory and handoff (#467)
64 of the set's 81 unwired cards are wired across five batches; the other
17 carry specific blocker notes. docs/CARD_INVENTORY.xlsx regenerated: 2172
cards, 850 wired (786 before). The catalogue art pack republish is the one
remaining step: release creation is not permitted from this session.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNrBVZ4tAzMKc9NrCTm41Z
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -498,14 +498,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5" t="n">
         <v>51</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>33.3%</t>
+          <t>35.3%</t>
         </is>
       </c>
     </row>
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>359</v>
+        <v>386</v>
       </c>
       <c r="C6" t="n">
         <v>826</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>46.7%</t>
         </is>
       </c>
     </row>
@@ -534,14 +534,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C7" t="n">
         <v>128</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>68.8%</t>
+          <t>69.5%</t>
         </is>
       </c>
     </row>
@@ -552,14 +552,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C8" t="n">
         <v>132</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>27.3%</t>
         </is>
       </c>
     </row>
@@ -570,14 +570,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>24.8%</t>
+          <t>27.8%</t>
         </is>
       </c>
     </row>
@@ -588,14 +588,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>194</v>
+        <v>214</v>
       </c>
       <c r="C10" t="n">
         <v>597</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>32.5%</t>
+          <t>35.8%</t>
         </is>
       </c>
     </row>
@@ -606,14 +606,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C11" t="n">
         <v>151</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>22.5%</t>
         </is>
       </c>
     </row>
@@ -624,14 +624,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
@@ -642,14 +642,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" t="n">
         <v>37</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
@@ -660,14 +660,14 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C14" t="n">
         <v>26</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>30.8%</t>
+          <t>34.6%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>786</v>
+        <v>850</v>
       </c>
       <c r="C16" t="n">
         <v>2172</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>36.2%</t>
+          <t>39.1%</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -3896,7 +3896,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G95" t="inlineStr"/>
@@ -4064,7 +4064,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Asako Chukage (Forgotten Legacy printing; the Seeds of Decay pass's own oracle-l5r-10072 Chukage is a different, experienced printing with different text, so none of its ability ids apply). Three separate gaps: (1) "search your discard pile, then hand, then deck, for a Ring of Water. Put it into play or in your hand" -- DeckSearch.cs's SearchSpec/SearchDeck only searches the Dynasty or Fate DECK; there is no ordered fallback across discard pile, hand and deck, and no search effect that puts a Ring into play (a Ring enters play only through its own printed recruit ability, e.g. ring-of-water-recruit from the hand); (2) "If this put it into play, while it remains in play, it does not count towards an Enlightenment Victory" -- StartTurn's Enlightenment check counts every in-play real Ring by keyword (excluding only Fudo False Rings) and has no per-card exclusion flag; (3) "Water Tireless Reaction: After the resolution of an action that moved your Personality, move Chukage to the Personality's location. After this moves him, straighten Chukage's unit" -- no Reaction trigger reads LastResolvedAction's MovedKind for an OWN moved Personality to follow him to any location (home or a battlefield). Each is a new primitive; not wired whole.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4391,7 +4395,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G110" t="inlineStr"/>
@@ -5290,7 +5294,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G137" t="inlineStr"/>
@@ -6263,7 +6267,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G166" t="inlineStr"/>
@@ -7199,14 +7203,10 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G194" t="inlineStr">
-        <is>
-          <t>Not blocked since issue #336: its Battle action is Sea Troll Predator's verbatim (predator-move, MoveSpec source-and-target to an adjacent unresolved battlefield); not yet wired.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -7768,7 +7768,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G211" t="inlineStr"/>
@@ -8238,7 +8238,7 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G225" t="inlineStr"/>
@@ -8873,7 +8873,7 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G244" t="inlineStr"/>
@@ -9170,7 +9170,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G253" t="inlineStr"/>
@@ -11228,14 +11228,10 @@
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G315" t="inlineStr">
-        <is>
-          <t>Not blocked since issue #336: "Bow him. He may not perform actions." is a bow plus the action-lock (ActionLock.cs); not yet wired.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -13379,7 +13375,7 @@
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G378" t="inlineStr"/>
@@ -15296,14 +15292,10 @@
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G435" t="inlineStr">
-        <is>
-          <t>Now unblocked (issue #387, not wired there): its Reaction is a Creates ability (the Lion Ancestor scan is published) plus gaining 1 Honor. See docs/decisions/2026-09-20-created-cards-from-proxy-scans.md.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr"/>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
@@ -16263,7 +16255,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G463" t="inlineStr"/>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>Kitsune Hisano: its only printed ability is "Reaction: Once per game, after Hisano enters play: Create a 2F/2C/3PH Mantis Clan - Nonhuman - Fox - Spirit - Unique Personality with the ability, 'Battle: Target an enemy attacking Personality: Move him home.'" Mechanically this is Kitsune Ohsuki's own entering-play Creates Reaction plus AbilityDefinition.OncePerGame, and the created Guide's ability is favor-battle's own target and move without the Favor discard (target "enemy-attacking", MoveHome). Blocked only because the created card has no scan: CreatedCards.Resolve needs a published CreatedOnly Proxy scan that fits the spec, and Hisano's Guide (oracle-l5r-10020) has none available (see its own note). Wire both together once that scan is fetched.</t>
+        </is>
+      </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
@@ -17522,14 +17518,10 @@
       </c>
       <c r="F501" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G501" t="inlineStr">
-        <is>
-          <t>Needs an activated (not passive/static) 'apply a Force penalty to every card in the target unit, then bow any now at 0' primitive -- the existing unit-scoped Force primitives (UnitForceBoostPrimitive, ArmyBattleMaidenBoostPrimitive) are passive/continuous, not one-shot activated effects across a filtered unit.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr"/>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
@@ -19105,7 +19097,7 @@
       </c>
       <c r="F548" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G548" t="inlineStr"/>
@@ -20004,7 +19996,7 @@
       </c>
       <c r="F575" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G575" t="inlineStr"/>
@@ -20429,7 +20421,7 @@
       </c>
       <c r="F588" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G588" t="inlineStr"/>
@@ -21955,7 +21947,7 @@
       </c>
       <c r="F634" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G634" t="inlineStr"/>
@@ -22520,7 +22512,7 @@
       </c>
       <c r="F651" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G651" t="inlineStr"/>
@@ -23088,7 +23080,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G668" t="inlineStr"/>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>Shosuro Aroru. Three independent gaps, so the card cannot be wired whole: (1) "Will not attach non-Ninja Followers" is a HOST-side attach refusal -- CardDefinition's AttachRequiresKeyword/AttachExcludesKeyword/AttachRequiresName gate only the ATTACHMENT's own text, so a Personality refusing a class of attachments needs a new field read at every attach funnel (MatchEngine.Equip's AttachmentLegalTarget, AttachAction.ValidateAttach, the spell-in-hand/equip-battle Requires in CardAbilities.cs). (2) "Reaction: When an action would target a Ninja at Aroru's location: Choose another of your cards. The action targets it instead, if legal." is the existing redirect (RedirectAction with Blade of Champions' redirect-target-own-card, Castle of Order's Ninja-at-location check), but its tail "After the action's resolution, you may move Aroru to a different location" needs a Reaction to register a DEFERRED optional effect that fires when the held action finishes resolving (CompleteAbilityResolution / ResolveAttack's tails carry no per-reaction deferred effect) and then asks for a destination (home or another unresolved battlefield) at that later moment. (3) "Battle: Other players may not take Reactions until this action ends. Ranged 5 Attack." -- the Attack is trivial, but nothing forbids Reactions: every window (before-action, targeted-by-action, attackReaction, OpenAlternatingReactionWindow) would need a per-action lockout of the other player until the action ends.</t>
+        </is>
+      </c>
     </row>
     <row r="669">
       <c r="A669" t="inlineStr">
@@ -23485,7 +23481,7 @@
       </c>
       <c r="F680" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G680" t="inlineStr"/>
@@ -25286,7 +25282,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G734" t="inlineStr"/>
+      <c r="G734" t="inlineStr">
+        <is>
+          <t>The Dark Naga. "After The Dark Naga enters play: Lose 3 Honor" is EntryHonorLoss 3, and "Reaction: After another player targets The Dark Naga with an action: You may bow one of your Forests. If you did, negate The Dark Naga's destruction from the action's effects" is buildable (a targeted-by-action Reaction with an optional Forest bow and Mirumoto Rokai's destruction negation). The blocker is the Battle action: "If he is Nonhuman, take control of him (he joins your army)" is an in-play control change of an enemy Personality and his unit -- TakeControl (AttachAction.cs) only covers a card brought into play from another player's discard pile; moving a controlled unit to the taker's side of the battlefield, Loyal, and the unit-wide Unique/Singular control check required by docs/decisions/2026-09-12-unique-singular-control-transfer.md are all unbuilt. ("Destroy him before this turn ends" has a model in DelayedDestruction.cs's end-of-turn destruction.)</t>
+        </is>
+      </c>
     </row>
     <row r="735">
       <c r="A735" t="inlineStr">
@@ -25477,7 +25477,7 @@
       </c>
       <c r="F740" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G740" t="inlineStr"/>
@@ -25543,7 +25543,7 @@
       </c>
       <c r="F742" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G742" t="inlineStr"/>
@@ -26170,14 +26170,10 @@
       </c>
       <c r="F761" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G761" t="inlineStr">
-        <is>
-          <t>Needs a 'same location as source' targeting axis for a non-battle-restricted (BattleOrOpen) ability -- every existing 'at the same battlefield' check assumes Battle timing's own blanket AtBattle requirement, which BattleOrOpen deliberately carries none of.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G761" t="inlineStr"/>
     </row>
     <row r="762">
       <c r="A762" t="inlineStr">
@@ -26471,7 +26467,7 @@
       </c>
       <c r="F770" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G770" t="inlineStr"/>
@@ -26969,7 +26965,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G785" t="inlineStr"/>
+      <c r="G785" t="inlineStr">
+        <is>
+          <t>Tsuruchi Nobukatsu (the inexperienced printing; unrelated to Nobukatsu - exp's text). "Battle: Ranged 4 Attack. If the Ranged Attack destroyed a card, you may target and straighten a Holding." The Attack and the destroyed-a-card check are built (Sticks and Stones' AfterSticksAndStonesAttack reads targetInPlayBefore). The gap is the optional Holding TARGET chosen after the Attack resolves: an Attack can resolve inline or later in ResolveAttack after its reaction window, and neither pausing primitive fits -- SequencedTarget.cs pauses BEFORE a sequenced Attack, DeciderChoice.cs pauses inside the ordinary effect switch and resumes with CompleteAbilityResolution, but nothing pauses AFTER a deferred ResolveAttack (whose own tail finishes the action). Shiba Iaimiko's up-front optional slot (TargetSlots.cs) would pick the Holding before the Attack, but an ability with Target "attack" cannot also carry Slots, and choosing it up front would target the Holding even when the Attack destroys nothing.</t>
+        </is>
+      </c>
     </row>
     <row r="786">
       <c r="A786" t="inlineStr">
@@ -27535,7 +27535,7 @@
       </c>
       <c r="F802" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G802" t="inlineStr"/>
@@ -28071,7 +28071,7 @@
       </c>
       <c r="F818" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G818" t="inlineStr"/>
@@ -28170,7 +28170,7 @@
       </c>
       <c r="F821" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G821" t="inlineStr"/>
@@ -29028,7 +29028,7 @@
       </c>
       <c r="F847" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G847" t="inlineStr"/>
@@ -33867,14 +33867,10 @@
       </c>
       <c r="F990" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G990" t="inlineStr">
-        <is>
-          <t>Needs a "usable even while bowed" exception on a second ability (already a known gap elsewhere).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G990" t="inlineStr"/>
     </row>
     <row r="991">
       <c r="A991" t="inlineStr">
@@ -34695,7 +34691,7 @@
       </c>
       <c r="F1014" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1014" t="inlineStr"/>
@@ -35392,14 +35388,10 @@
       </c>
       <c r="F1035" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1035" t="inlineStr">
-        <is>
-          <t>Needs Chi as a repeatable payable cost resource (distinct from a Force/Stat modifier), interacting correctly with the existing Chi&lt;=0 death rule.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1035" t="inlineStr"/>
     </row>
     <row r="1036">
       <c r="A1036" t="inlineStr">
@@ -41149,7 +41141,7 @@
       </c>
       <c r="F1208" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1208" t="inlineStr"/>
@@ -42382,7 +42374,7 @@
       </c>
       <c r="F1245" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1245" t="inlineStr"/>
@@ -42753,7 +42745,7 @@
       </c>
       <c r="F1256" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1256" t="inlineStr"/>
@@ -43050,7 +43042,7 @@
       </c>
       <c r="F1265" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1265" t="inlineStr"/>
@@ -43516,7 +43508,7 @@
       </c>
       <c r="F1279" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1279" t="inlineStr"/>
@@ -44077,7 +44069,7 @@
       </c>
       <c r="F1296" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1296" t="inlineStr"/>
@@ -44143,7 +44135,7 @@
       </c>
       <c r="F1298" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1298" t="inlineStr"/>
@@ -44651,7 +44643,7 @@
       </c>
       <c r="G1313" t="inlineStr">
         <is>
-          <t>Needs a Retainer mechanic, movement to any location (not just home), and a province-card discard (three separate gaps).</t>
+          <t>Asset Denial (re-verified; the old note's "Retainer mechanic" is stale -- Retainer is a plain keyword on Holdings, e.g. Recruitment Officer/Slanderer, so the Open half "Bow your performing Ninja Personality and target a Retainer: Destroy it" is an ordinary BowPerformer cost plus a keyword-gated Holding target and would wire on its own). Blocked on its Battle half, "Choose your performing Ninja Personality with no non-Ninja Followers at the current battlefield: Move him to a different location. If he moved, straighten his unit. Discard a card in a province.": (1) "a different location" is home OR another battlefield, the player's choice -- Hawado's own split into two ability ids sharing a UsageKey, the battlefield one naming its destination in GameCommand.Province (MoveDestinations.cs); (2) "Discard a card in a province" is a second, independent choice of ANY player's province card (face down included). GameCommand carries one Province (already taken by the battlefield destination) and one TargetPlayerId; a Slots selection cannot carry it instead, because SlotCandidateCards (TargetSlots.cs) never lists a card in Zone.Province and a Slots ability is listed through SlotAbilityOption, which never enumerates a chosen battlefield destination (AbilityActions skips the destination loop for it). Both halves are kept together rather than splitting one card.</t>
         </is>
       </c>
     </row>
@@ -45582,7 +45574,7 @@
       </c>
       <c r="F1341" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1341" t="inlineStr"/>
@@ -45854,7 +45846,7 @@
       </c>
       <c r="F1349" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1349" t="inlineStr"/>
@@ -46188,7 +46180,7 @@
       </c>
       <c r="F1359" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1359" t="inlineStr"/>
@@ -46485,7 +46477,7 @@
       </c>
       <c r="F1368" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1368" t="inlineStr"/>
@@ -47730,7 +47722,7 @@
       </c>
       <c r="F1405" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1405" t="inlineStr"/>
@@ -47964,7 +47956,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1412" t="inlineStr"/>
+      <c r="G1412" t="inlineStr">
+        <is>
+          <t>Economic Repercussions. "Limited: Put this card into play" is Kata's own EnterPlayAsKata shape (KataCards.cs, Zone.Home) and "Other players' Personalities and Followers in play have -2 Gold Cost" is a one-term addition to CardGoldCost (StatPenalties.cs). Blocked on the granted ability: "all players have the ability, 'Political Limited: Discard the Imperial Favor or pay 6 Gold: Discard a card titled Economic Repercussions from play'" -- the card's OPPONENT must be able to take an action granted by a card he does not control. A PlayerAbility (AbilityDefinition.PlayerAbility) is unconditional and listed in every match's QueryActions (AbilityActions adds every PlayerAbility whenever the Stronghold is not ScenarioOnly), so it would add two permanently-disabled actions to every published game; the only conditional grant, StaticGrantedAbilityIds (HonorAndTreacheryPass.cs), grants to a player's own Personalities, whose abilities are refused while the source is bowed. A conditional player-ability grant (listed and legal only while a named card is in play) is the missing primitive.</t>
+        </is>
+      </c>
     </row>
     <row r="1413">
       <c r="A1413" t="inlineStr">
@@ -48225,7 +48221,7 @@
       </c>
       <c r="F1420" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1420" t="inlineStr"/>
@@ -48757,7 +48753,7 @@
       </c>
       <c r="F1436" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1436" t="inlineStr"/>
@@ -49399,7 +49395,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1455" t="inlineStr"/>
+      <c r="G1455" t="inlineStr">
+        <is>
+          <t>Fruitless Search: mechanically wirable, scan unavailable for its token. "Reaction: After engaging, if any enemy units are at the current battlefield: Create a 4F/4C/3PH Imperial Samurai Duelist Magistrate Personality on your side there. Remove him from the game after this battle ends" is Kyuden Hida - exp's own after-engaging Creates shape with CreatedCardSpec.AtBattlefield + UntilBattleEnds (Kitsu Miro's Ancestor) and a by-id enemy-presence Require. The Proxy it creates is Emerald Magistrate (oracle-l5r-9996, Embers of War: 4F/4C/3PH, Duelist/Imperial/Magistrate/Samurai, same artist), which is not published: its receipt names only the master scan (no working_copy), the Oracle image host is refused by this sandbox's network policy, and it is not in the local art pack. CreatedCards.Resolve/Verify need a published CreatedOnly scan, so the creator cannot be wired until the Proxy is published (package it the way package_personality_wave_64.py published Guest/Haruki's Deer once its scan can be fetched).</t>
+        </is>
+      </c>
     </row>
     <row r="1456">
       <c r="A1456" t="inlineStr">
@@ -49770,7 +49770,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1466" t="inlineStr"/>
+      <c r="G1466" t="inlineStr">
+        <is>
+          <t>Grateful Reward: mechanically wirable, scan unavailable for its token. "Reaction: After engaging, choose your performing Samurai at the current battlefield: Create a 1F Ashigaru Cavalry Follower and attach it to him. If he is a Paragon, gain 2 Honor and draw a card" is Nakanu Technique's own after-engaging Creates shape (HostIsPerformer, an at-battle Samurai Performer) plus a Paragon-conditional GainHonor/Draw in its case. The Proxy it creates is Mounted Ashigaru (oracle-l5r-10010, Emperor Edition: 1F, Cavalry/Ashigaru), which is not published: its receipt names only the master scan (no working_copy), the Oracle image host is refused by this sandbox's network policy, and it is not in the local art pack. CreatedCards.Resolve/Verify need a published CreatedOnly scan, so the creator cannot be wired until the Proxy is published.</t>
+        </is>
+      </c>
     </row>
     <row r="1467">
       <c r="A1467" t="inlineStr">
@@ -50245,7 +50249,7 @@
       </c>
       <c r="F1480" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1480" t="inlineStr"/>
@@ -50590,7 +50594,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1490" t="inlineStr"/>
+      <c r="G1490" t="inlineStr">
+        <is>
+          <t>Honor Never Falls. Its Focus Effect, "Delay all consequences of losing this duel (from any source) until the end of the turn", has no primitive: Dueling.cs applies a duel's outcome as one indivisible case per duel-issuing ability (ApplyDuelOutcome, winner and loser effects interleaved) plus each focused card's own ApplyDuelFocusEffect and loss-keyed traits, and the only deferral the engine has is DelayedDestruction.cs's delay-destroy kind (Spirit of the Berserker), which puts off one DESTRUCTION until EndTurn -- not the bows, moves home, Honor/Gold losses, penalties and tokens that are also consequences of losing, from every source at once. It needs a per-duel queue of the loser's consequences drained at the end of the turn. The Battle half's "you may take an additional Battle action to use one of his base abilities" also has no exact shape: AdditionalActionGrant.ScopeCardIds scopes a grant to a source CARD, so an ability granted to him (CardInstance.GrantedAbilities, sourced from the same card) could consume it too; a scope limited to his printed (base) abilities does not exist. Its straighten of a bowed performer (own-personality-with-keyword-at-battle-style, Unique read off his keywords) is ordinary; the card is kept whole.</t>
+        </is>
+      </c>
     </row>
     <row r="1491">
       <c r="A1491" t="inlineStr">
@@ -51494,14 +51502,10 @@
       </c>
       <c r="F1517" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1517" t="inlineStr">
-        <is>
-          <t>The move to a destination the ability's own rule defines (MoveSpec, issue #336) now moves an enemy Personality to the current battlefield and can move the chosen performer with it (Movers performer-and-target). Still needs a target category for "another player's Personality not at the current battlefield" and the "straighten each unit that this moved" follow-up.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1517" t="inlineStr"/>
     </row>
     <row r="1518">
       <c r="A1518" t="inlineStr">
@@ -53287,14 +53291,10 @@
       </c>
       <c r="F1570" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1570" t="inlineStr">
-        <is>
-          <t>Needs an exemption from the generic Battle-timing army-presence requirement (the adjacent-battlefield Performer shape itself, Moto Gunso's own, already exists).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1570" t="inlineStr"/>
     </row>
     <row r="1571">
       <c r="A1571" t="inlineStr">
@@ -54202,7 +54202,7 @@
       </c>
       <c r="F1597" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1597" t="inlineStr"/>
@@ -54312,7 +54312,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1600" t="inlineStr"/>
+      <c r="G1600" t="inlineStr">
+        <is>
+          <t>Petty Squabbles. Its Limited half, "Target one or two face-down cards in provinces: Turn them face-up", cannot be offered without leaking hidden information: every target/slot names a card by CardInstance.Id, and those ids are assigned sequentially in deck-list order at setup (MatchEngine/PublishedMatch "card-NNNN"), so listing a face-down province card's real id in QueryActions would reveal which card it is -- MatchQueries.ViewCard deliberately shows a face-down province card as "hidden-p{owner}-province{n}" instead. The province-addressed alternative (Target any-province: TargetPlayerId + Province) names ONE province, and SlotSelection carries only CardIds or a PlayerId, so "one or two" provinces of any player is not expressible; SlotCandidateCards never lists province cards either. (Turning a Celestial face-up would also have to enter it into play through ResolveCelestial.) Its Battle/Open half, "Target an attachment owned by another player: He may pay 4 Gold. If he did not, return it to its owner's hand", is wirable as an EitherOr spec (Yasuki Makoto's owner-decides pay-4-Gold shape); the card is kept whole.</t>
+        </is>
+      </c>
     </row>
     <row r="1601">
       <c r="A1601" t="inlineStr">
@@ -55653,7 +55657,7 @@
       </c>
       <c r="F1640" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1640" t="inlineStr"/>
@@ -55826,7 +55830,7 @@
       </c>
       <c r="F1645" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1645" t="inlineStr"/>
@@ -56407,7 +56411,7 @@
       </c>
       <c r="F1662" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1662" t="inlineStr"/>
@@ -56972,7 +56976,7 @@
       </c>
       <c r="F1679" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1679" t="inlineStr"/>
@@ -57966,7 +57970,7 @@
       </c>
       <c r="F1709" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1709" t="inlineStr"/>
@@ -58832,7 +58836,7 @@
       </c>
       <c r="F1735" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1735" t="inlineStr"/>
@@ -59037,7 +59041,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1741" t="inlineStr"/>
+      <c r="G1741" t="inlineStr">
+        <is>
+          <t>Sword for Hire. "Create a 0F/3C/0PH Assassin • Duelist Personality" is the Embers of War Proxy oracle-l5r-9995 (the orphan Proxy recorded there -- this is its creator), and CreatedCards.Resolve needs that Proxy published as a CreatedOnly scan: its scan is not in this sandbox (assets/reference/oracle/embers-of-war holds receipts only), so neither card can be packaged here. Once the Proxy is published the rest is buildable: Creates (a Personality at home), IssueChallenge (Dueling.cs) with the created card as the challenger and DuelRefusable false, a "destroy the duel's loser" outcome, and a new small hook removing the created challenger from the game when its duel ends (CreatedUntilBattleEndsIds is battle-scoped; this is duel-scoped).</t>
+        </is>
+      </c>
     </row>
     <row r="1742">
       <c r="A1742" t="inlineStr">
@@ -60356,7 +60364,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1780" t="inlineStr"/>
+      <c r="G1780" t="inlineStr">
+        <is>
+          <t>The Perfect Moment. Needs an additional Attack Phase created by a Reaction (same gap as oracle-l5r-10184, Aramasu's Legacy: the turn's phase sequence is fixed and nothing inserts a second Attack Phase), here with the previous Attacker as the new Defender (the Attack Phase is always the active player's own), plus restrictions scoped to that one phase instance: the acting player "will not destroy more than one of the Defender's provinces" (a cap on DestroyProvince across the phase's battles) and his Personalities "may not assign and will not move unless they are Paragons or Battle Maidens" (an assignment-and-movement lock by keyword). No part of this exists.</t>
+        </is>
+      </c>
     </row>
     <row r="1781">
       <c r="A1781" t="inlineStr">
@@ -62879,7 +62891,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1855" t="inlineStr"/>
+      <c r="G1855" t="inlineStr">
+        <is>
+          <t>Wanted for Questioning. "Your Magistrate takes him into custody" is a mechanic docs/rules/EMPEROR_EDITION_CORE_RULES.md does not define (no Glossary entry for custody; grep finds none) and the engine has no representation of (no custody state, zone or link in Models.cs) -- what custody does, how long it lasts and how it ends has no rules source here, so it cannot be wired consistently with the core rules. The rest is ordinary (an unbowed Magistrate Performer, own-unbowed-personality-at-battle-with-keyword; "if he is dishonorable, destroy his attachments"; MoveHome); the card is kept whole.</t>
+        </is>
+      </c>
     </row>
     <row r="1856">
       <c r="A1856" t="inlineStr">
@@ -63375,7 +63391,7 @@
       </c>
       <c r="F1870" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1870" t="inlineStr"/>
@@ -63507,7 +63523,7 @@
       </c>
       <c r="F1874" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1874" t="inlineStr"/>
@@ -63705,7 +63721,7 @@
       </c>
       <c r="F1880" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1880" t="inlineStr"/>
@@ -64031,7 +64047,7 @@
       </c>
       <c r="F1890" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1890" t="inlineStr"/>
@@ -68564,7 +68580,7 @@
       </c>
       <c r="F2027" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2027" t="inlineStr"/>
@@ -68663,7 +68679,7 @@
       </c>
       <c r="F2030" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2030" t="inlineStr"/>
@@ -70947,7 +70963,7 @@
       </c>
       <c r="F2098" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2098" t="inlineStr"/>
@@ -71879,7 +71895,7 @@
       </c>
       <c r="F2126" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2126" t="inlineStr"/>
@@ -73038,7 +73054,7 @@
       </c>
       <c r="F2161" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2161" t="inlineStr"/>

</xml_diff>

<commit_message>
Card inventory: unwired cards by Set and Type summary table
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="3">
@@ -60,10 +64,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -446,13 +451,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -705,6 +719,667 @@
         <is>
           <t>39.9%</t>
         </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Unwired cards by Set and Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Set</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Stronghold</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Personality</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Follower</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Spell</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Holding</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Celestial</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Emperor Edition</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>24</v>
+      </c>
+      <c r="C20" t="n">
+        <v>78</v>
+      </c>
+      <c r="D20" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" t="n">
+        <v>11</v>
+      </c>
+      <c r="F20" t="n">
+        <v>13</v>
+      </c>
+      <c r="G20" t="n">
+        <v>94</v>
+      </c>
+      <c r="H20" t="n">
+        <v>11</v>
+      </c>
+      <c r="I20" t="n">
+        <v>12</v>
+      </c>
+      <c r="J20" t="n">
+        <v>9</v>
+      </c>
+      <c r="K20" t="n">
+        <v>5</v>
+      </c>
+      <c r="M20" t="n">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Promotional–Emperor</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>18</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>30</v>
+      </c>
+      <c r="F21" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" t="n">
+        <v>22</v>
+      </c>
+      <c r="H21" t="n">
+        <v>24</v>
+      </c>
+      <c r="I21" t="n">
+        <v>20</v>
+      </c>
+      <c r="J21" t="n">
+        <v>5</v>
+      </c>
+      <c r="K21" t="n">
+        <v>6</v>
+      </c>
+      <c r="M21" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Coils of Madness</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="n">
+        <v>67</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" t="n">
+        <v>7</v>
+      </c>
+      <c r="G22" t="n">
+        <v>13</v>
+      </c>
+      <c r="H22" t="n">
+        <v>9</v>
+      </c>
+      <c r="I22" t="n">
+        <v>8</v>
+      </c>
+      <c r="J22" t="n">
+        <v>3</v>
+      </c>
+      <c r="L22" t="n">
+        <v>2</v>
+      </c>
+      <c r="M22" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Torn Asunder</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="n">
+        <v>45</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" t="n">
+        <v>6</v>
+      </c>
+      <c r="F23" t="n">
+        <v>12</v>
+      </c>
+      <c r="G23" t="n">
+        <v>41</v>
+      </c>
+      <c r="H23" t="n">
+        <v>6</v>
+      </c>
+      <c r="I23" t="n">
+        <v>5</v>
+      </c>
+      <c r="J23" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>The Shadow's Embrace</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="n">
+        <v>45</v>
+      </c>
+      <c r="D24" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" t="n">
+        <v>8</v>
+      </c>
+      <c r="F24" t="n">
+        <v>8</v>
+      </c>
+      <c r="G24" t="n">
+        <v>39</v>
+      </c>
+      <c r="H24" t="n">
+        <v>5</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5</v>
+      </c>
+      <c r="J24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Gates of Chaos</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>44</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" t="n">
+        <v>7</v>
+      </c>
+      <c r="F25" t="n">
+        <v>8</v>
+      </c>
+      <c r="G25" t="n">
+        <v>32</v>
+      </c>
+      <c r="H25" t="n">
+        <v>7</v>
+      </c>
+      <c r="I25" t="n">
+        <v>3</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Aftermath</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>43</v>
+      </c>
+      <c r="D26" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" t="n">
+        <v>10</v>
+      </c>
+      <c r="G26" t="n">
+        <v>24</v>
+      </c>
+      <c r="H26" t="n">
+        <v>4</v>
+      </c>
+      <c r="I26" t="n">
+        <v>3</v>
+      </c>
+      <c r="J26" t="n">
+        <v>3</v>
+      </c>
+      <c r="M26" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Embers of War</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="n">
+        <v>34</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>8</v>
+      </c>
+      <c r="G27" t="n">
+        <v>29</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" t="n">
+        <v>4</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1</v>
+      </c>
+      <c r="M27" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Twenty Festivals</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>15</v>
+      </c>
+      <c r="D28" t="n">
+        <v>4</v>
+      </c>
+      <c r="E28" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" t="n">
+        <v>7</v>
+      </c>
+      <c r="G28" t="n">
+        <v>21</v>
+      </c>
+      <c r="H28" t="n">
+        <v>13</v>
+      </c>
+      <c r="M28" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ivory Edition</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="n">
+        <v>7</v>
+      </c>
+      <c r="G29" t="n">
+        <v>17</v>
+      </c>
+      <c r="H29" t="n">
+        <v>18</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1</v>
+      </c>
+      <c r="M29" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Before the Dawn</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>17</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" t="n">
+        <v>19</v>
+      </c>
+      <c r="H30" t="n">
+        <v>2</v>
+      </c>
+      <c r="I30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1</v>
+      </c>
+      <c r="M30" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Promotional–Celestial</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>8</v>
+      </c>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" t="n">
+        <v>7</v>
+      </c>
+      <c r="H31" t="n">
+        <v>6</v>
+      </c>
+      <c r="I31" t="n">
+        <v>2</v>
+      </c>
+      <c r="J31" t="n">
+        <v>3</v>
+      </c>
+      <c r="K31" t="n">
+        <v>3</v>
+      </c>
+      <c r="M31" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Seeds of Decay</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>5</v>
+      </c>
+      <c r="I32" t="n">
+        <v>3</v>
+      </c>
+      <c r="M32" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Forgotten Legacy</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>5</v>
+      </c>
+      <c r="G33" t="n">
+        <v>9</v>
+      </c>
+      <c r="M33" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>War of Honor</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" t="n">
+        <v>10</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1</v>
+      </c>
+      <c r="M34" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Celestial Edition</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Honor and Treachery</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="M36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Second City</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>1</v>
+      </c>
+      <c r="M37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Words and Deeds</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>1</v>
+      </c>
+      <c r="M38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>383</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="J39" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="L39" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>1305</v>
       </c>
     </row>
   </sheetData>
@@ -731,37 +1406,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Id</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Set</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Clan</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Blocker</t>
         </is>

</xml_diff>

<commit_message>
Emperor Edition Personality pass: blockers for the seven unwired cards; regenerate inventory
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -516,14 +516,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>394</v>
+        <v>465</v>
       </c>
       <c r="C6" t="n">
         <v>826</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>47.7%</t>
+          <t>56.3%</t>
         </is>
       </c>
     </row>
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>867</v>
+        <v>938</v>
       </c>
       <c r="C16" t="n">
         <v>2172</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>39.9%</t>
+          <t>43.2%</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Card creation is built (issue #387): the 2F Follower it creates is the Infantry Follower scan (oracle-l5r-9738), not yet published as a created-only Follower wave. Remaining: that wave and this card's Creates ability. 'Tactical Limited' itself maps onto the existing Limited Timing per the established Political/Tactical precedent, so is not itself a blocker.</t>
+          <t>Akodo Makotai (Tactical Limited: Create a 2F Follower and attach it to Makotai). The engine side exists (Creates: new(CardType.Follower, Force: 2, ProxyId: "oracle-l5r-9738") { HostIsSource = true } on a Limited ability with ActionKeywords ["Tactical"], the Tactician performer/once-per-turn Tactical rule already reads the keyword), but the created card must be the plain 2F Follower Proxy, the Emperor Edition 'Infantry Follower' (oracle-l5r-9738, printing 4, #11: Force 2, no keywords, no text). No published created-only Follower fits: the only 2F one is the Ronin Follower (oracle-l5r-10203), whose Ronin keyword would be a wrong extra keyword on a plain 'Follower', and the Infantry Follower is not published. Publishing it needs a created-only follower wave (follower-wave-24's shape: Type Follower, CreatedOnly true, Effect none) built from its scan, but the scan is not among the local assets (only its receipt JSON exists under assets/reference/oracle/emperor-edition/receipts; the jpg/webp was never downloaded). Once that scan is fetched (source_url in the receipt) and packaged, wiring Makotai is one catalogue entry plus the Creates spec and a case in RunEmperorPersonalityBatch2Effect (CreatedCardEntry already attaches to command.CardId for HostIsSource).</t>
         </is>
       </c>
     </row>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G86" t="inlineStr"/>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G88" t="inlineStr"/>
@@ -3764,7 +3764,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
@@ -4733,7 +4733,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G120" t="inlineStr"/>
@@ -4898,7 +4898,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G125" t="inlineStr"/>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G128" t="inlineStr"/>
@@ -5327,7 +5327,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G138" t="inlineStr"/>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G153" t="inlineStr"/>
@@ -5892,7 +5892,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G155" t="inlineStr"/>
@@ -6065,7 +6065,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G160" t="inlineStr"/>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G169" t="inlineStr"/>
@@ -6733,7 +6733,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G180" t="inlineStr"/>
@@ -7533,7 +7533,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G204" t="inlineStr"/>
@@ -7735,7 +7735,7 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G210" t="inlineStr"/>
@@ -7933,7 +7933,7 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G216" t="inlineStr"/>
@@ -7966,7 +7966,7 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G217" t="inlineStr"/>
@@ -8135,7 +8135,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G222" t="inlineStr"/>
@@ -8205,7 +8205,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G224" t="inlineStr"/>
@@ -8271,7 +8271,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G226" t="inlineStr"/>
@@ -9071,7 +9071,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G250" t="inlineStr"/>
@@ -9434,7 +9434,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G261" t="inlineStr"/>
@@ -9702,7 +9702,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G269" t="inlineStr"/>
@@ -9870,7 +9870,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G274" t="inlineStr"/>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Goju Kobashi: "Battle: Target an enemy attachment: Kobashi consumes it. Destroy it. You may target one of your Ninja, create a 1F Shadowlands . Ninja Follower, and attach it to him." Two blockers. (1) The created Follower is the Proxy scan Kobashi's Spawn (oracle-l5r-10008, decision 2026-09-20-created-cards-from-proxy-scans.md pairs it with this card), but its scan is not in the local scan set: assets/reference/oracle/emperor-edition/receipts/oracle-l5r-10008-printing-1-image-1.json has no working_copy block, the original master under assets/reference/oracle/emperor-edition/images/ does not exist in a worktree, and no L5R-Catalogue-WebP85.zip on this machine contains the file (looked up by the receipt's sha256 c4db3440...), so the Proxy cannot be packaged (tools/content/package_vanilla_wave.py needs the image) and CreatedCards.Resolve would fail. Once the webp is restored, publish it as a CreatedOnly Follower (Force 1, keywords Shadowlands and Ninja) and the rest is data: an enemy-attachment target ("any-attachment" filtered to enemy cards), DestroyAttachment, and an optional second slot (0..1) on "own-ninja-personality" carrying Creates: new(CardType.Follower, Force: 1, Keywords: ["Shadowlands", "Ninja"]) -- the shape of Makubesu's/Iaimiko's optional slot. (2) "Kobashi consumes it" is not defined anywhere in docs/rules/EMPEROR_EDITION_CORE_RULES.md (Consumer is a printed keyword with no rules text; this card is the only user of the verb). Reading it as flavor for the destroy would be the smallest faithful reading, but it is a ruling for Mendon, not an inference to bake in.</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -9933,7 +9937,7 @@
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G276" t="inlineStr"/>
@@ -10498,7 +10502,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G293" t="inlineStr"/>
@@ -10630,7 +10634,7 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G297" t="inlineStr"/>
@@ -10663,7 +10667,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G298" t="inlineStr"/>
@@ -10898,7 +10902,7 @@
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G305" t="inlineStr"/>
@@ -10931,7 +10935,7 @@
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G306" t="inlineStr"/>
@@ -12114,7 +12118,7 @@
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
@@ -12625,7 +12629,7 @@
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G356" t="inlineStr"/>
@@ -12934,7 +12938,7 @@
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G365" t="inlineStr"/>
@@ -13540,7 +13544,7 @@
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G383" t="inlineStr"/>
@@ -13874,7 +13878,7 @@
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G393" t="inlineStr"/>
@@ -14006,7 +14010,7 @@
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G397" t="inlineStr"/>
@@ -14340,7 +14344,7 @@
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G407" t="inlineStr"/>
@@ -14785,7 +14789,7 @@
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G420" t="inlineStr"/>
@@ -14818,7 +14822,7 @@
       </c>
       <c r="F421" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G421" t="inlineStr"/>
@@ -15634,7 +15638,7 @@
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G445" t="inlineStr">
@@ -16071,7 +16075,7 @@
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G458" t="inlineStr">
@@ -16148,7 +16152,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G460" t="inlineStr"/>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>Kitsune Denhei: "Reaction: After Denhei enters play: Create a 2F/2C/3PH Mantis Clan - Nonhuman - Snake - Spirit Personality with the ability, 'Open: Target a Personality: He is bitten. His base abilities may not be used.'" The creation shape exists (Kagako's own-enters-play Create), but the created card is the Proxy "Denhei's Snake" (oracle-l5r-10002) and its scan is not in the local scan pack, so it cannot be published as a CreatedOnly Personality. Its ability also needs a primitive that does not exist: "his base abilities may not be used" (every PRINTED ability of the target, not granted ones, locked -- DisabledAbilities locks one usage key per turn and BattleAbilityLocks locks a card whole until a battle ends) with an unstated duration ("He is bitten" reads as a status; the core-rules default is until the end of the turn). Unblock: the 10002 scan, and a ruling on how long "bitten" lasts; then a printed-abilities-only lock keyed by card, expiring per that ruling.</t>
+        </is>
+      </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -16181,7 +16189,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G461" t="inlineStr"/>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>Kitsune Gina: "Reaction: After Gina enters play: Create a 2F/2C/3PH Mantis Clan - Nonhuman - Fox - Spirit Personality with the trait, 'Enemy attacking Personalities and Followers at this card's battlefield have -1F'." The creation shape exists (Kagako's), and the static Force term is small (TerrainForceAdjustment / Shiotome Plains' battlefield-scoped Force adjustment, read for the created card's own battlefield, on the attacking enemy side), but the created card is the Proxy "Gina's Fox" (oracle-l5r-10005) whose scan is not in the local scan pack, so the created Personality cannot be published. Unblock: add the 10005 scan, package it CreatedOnly with an Effect for the trait, add the -1F term to PersonalityForce/FollowerForce, then wire the Reaction.</t>
+        </is>
+      </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
@@ -16813,7 +16825,7 @@
       </c>
       <c r="F480" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G480" t="inlineStr"/>
@@ -17411,7 +17423,7 @@
       </c>
       <c r="F498" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G498" t="inlineStr">
@@ -17782,7 +17794,7 @@
       </c>
       <c r="F509" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G509" t="inlineStr">
@@ -19621,7 +19633,7 @@
       </c>
       <c r="F564" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G564" t="inlineStr"/>
@@ -19790,7 +19802,7 @@
       </c>
       <c r="F569" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G569" t="inlineStr"/>
@@ -19959,7 +19971,7 @@
       </c>
       <c r="F574" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G574" t="inlineStr"/>
@@ -20351,7 +20363,7 @@
       </c>
       <c r="F586" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G586" t="inlineStr"/>
@@ -20516,7 +20528,7 @@
       </c>
       <c r="F591" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G591" t="inlineStr"/>
@@ -20615,7 +20627,7 @@
       </c>
       <c r="F594" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G594" t="inlineStr"/>
@@ -20974,7 +20986,7 @@
       </c>
       <c r="F605" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G605" t="inlineStr"/>
@@ -21506,7 +21518,7 @@
       </c>
       <c r="F621" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G621" t="inlineStr"/>
@@ -21745,7 +21757,7 @@
       </c>
       <c r="F628" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G628" t="inlineStr"/>
@@ -21910,7 +21922,7 @@
       </c>
       <c r="F633" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G633" t="inlineStr"/>
@@ -22108,7 +22120,7 @@
       </c>
       <c r="F639" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G639" t="inlineStr"/>
@@ -22442,7 +22454,7 @@
       </c>
       <c r="F649" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G649" t="inlineStr"/>
@@ -22610,7 +22622,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G654" t="inlineStr"/>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>Shinjo Ki-Chang - exp: "Reaction: After your target Personality enters play: Create a 1F Cavalry Follower and attach it to him." The engine side is small (Singh Remnants' any-personality-enters-play watcher, CreatedCardSpec Follower Force 1 Keywords [Cavalry] attached to the entering Personality, plus one new target category for "the Personality that just entered play"), but the created card is the Proxy "Dutiful Cavalry" (oracle-l5r-10003: Follower, 1F, keyword Cavalry only) and its scan is not in the local Emperor Edition scan pack (assets/reference/oracle/emperor-edition/webp holds only the real cards) and no published wave carries it, so CreatedCards.Resolve cannot find a scan and an unresolvable creator must not be published. Unblock: add the oracle-l5r-10003 scan, package it CreatedOnly in a follower wave, then wire the Reaction. Also to confirm: "attach it to him" is read as the entering (target) Personality, not Ki-Chang.</t>
+        </is>
+      </c>
     </row>
     <row r="655">
       <c r="A655" t="inlineStr">
@@ -23312,7 +23328,7 @@
       </c>
       <c r="F675" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G675" t="inlineStr"/>
@@ -23678,7 +23694,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G686" t="inlineStr"/>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>Shosuro Rokuta -- "Reaction: After the resolution of a battle, or an action or trait from a card that another player owns, if the resolution or card destroyed Rokuta: Create a 0F/2C/1PH Scorpion Clan - Courtier - Apprentice Personality (in your home). Choose a player, who loses 3 Honor." Blocked on ONE missing asset, not on the rules structure: every 'create' ability must resolve to a published CreatedOnly Proxy scan (CreatedCards.Verify / CreatedCardSpec), and the Proxy this text creates -- "Rokuta's Apprentice", oracle-l5r-10013 (Scorpion Clan - Courtier - Apprentice, 0F/2C/1PH, 'May not be included in decks') -- has no scan in this working tree (no webp working copy under assets/reference/oracle/emperor-edition/webp, no images/ master, and its receipt sha256 0be21a50... is not in the Catalogue WebP 85 art pack), so it cannot be published and no Creates entry can resolve. To build it: fetch the master from the receipt's source_url (verify the sha256), publish the Proxy CreatedOnly with Type=Personality, Clan=Scorpion, Force 0, Chi 2, PersonalHonor 1, Keywords [Apprentice, Courtier, Scorpion Clan] (package_personality_wave_64.py's Guest / Haruki's Deer are the precedent), then wire two FromDead Reactions sharing one use: (1) the action half is Hida Yamadera - exp's shape (Trigger after-action-resolved, AfterActionResolvedApplies reading LastResolvedAction: another player's action -- any timing, not only Battle -- whose Affected list holds Rokuta as destroyed, facts.PlayerId != his controller) with Creates = new(CardType.Personality, Force: 0, Chi: 2, PersonalHonor: 1, Keywords: ["Scorpion Clan", "Courtier", "Apprentice"]) via ExecuteCreate and a 'player' Target for the 3-Honor loss (Kitsu Kagako's create plus Kitsuki Horume's chosen player); (2) the battle half needs PendingAfterResolution (AfterResolution.cs) to carry the ids of the cards the resolution destroyed (today it carries only counts per player) so an after-battle-resolution Reaction can test 'the resolution destroyed Rokuta' -- MatchEngine.cs's two DestroyUnits(d)/DestroyUnits(a) results are where to collect them. Reading to confirm with Mendon: 'a trait from a card that another player owns' -- no published trait destroys a Personality apart from the rulebook's own 0-Chi destruction (attributed to the last Chi-penalty effect), so only actions and battle resolution would be recorded.</t>
+        </is>
+      </c>
     </row>
     <row r="687">
       <c r="A687" t="inlineStr">
@@ -23840,7 +23860,7 @@
       </c>
       <c r="F691" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G691" t="inlineStr"/>
@@ -24145,7 +24165,7 @@
       </c>
       <c r="F700" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G700" t="inlineStr"/>
@@ -24247,7 +24267,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G703" t="inlineStr"/>
+      <c r="G703" t="inlineStr">
+        <is>
+          <t>Suiteiru no Oni: "Open: Destroy your target unbowed Personality: Create a number of 1F Shadowlands . Nonhuman . Oni Followers equal to his Chi. Attach them to one or more of your Personalities. Lose Honor equal to the number of Followers this created." Blockers: (1) the created Follower is the Proxy scan Suiteiru's Podling (oracle-l5r-10021), whose scan is not in the local scan set (receipt oracle-l5r-10021-printing-1-image-1.json has no working_copy block; the original master is absent from a worktree and not in any local L5R-Catalogue-WebP85.zip, sha256 65c50653...), so it cannot be packaged as a CreatedOnly Follower. (2) A created COUNT computed from the destroyed Personality's Chi does not exist: CreatedCardSpec.Count is a constant. It could be built as a CountFrom (Target Chi, read before the destroy cost removes him, like Abodan's _abodanChoseDead capture) beside CreatedValue. (3) "Attach them to one or more of your Personalities" needs a variable number of hosts (1..N, N up to the count), where Makubesu's slot is fixed at one or two; the hosts would be a slot with Max = the count, dealt in turn (CreatedCardSpec's non-PerHost distribution already deals Count cards across the chosen hosts). (4) "Lose Honor equal to the number of Followers this created" needs the created count read back after creation (a created card that is refused, e.g. by Unique/Honor Requirement attach legality, is not counted). A destroyed target that is not in play again (unbowed check as a cost) and a Chi of 0 (creates nothing, lose 0) are the edge cases to pin.</t>
+        </is>
+      </c>
     </row>
     <row r="704">
       <c r="A704" t="inlineStr">
@@ -24739,7 +24763,7 @@
       </c>
       <c r="F718" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G718" t="inlineStr">
@@ -26562,7 +26586,7 @@
       </c>
       <c r="F773" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G773" t="inlineStr"/>
@@ -27028,7 +27052,7 @@
       </c>
       <c r="F787" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G787" t="inlineStr"/>
@@ -27164,7 +27188,7 @@
       </c>
       <c r="F791" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G791" t="inlineStr"/>
@@ -27296,7 +27320,7 @@
       </c>
       <c r="F795" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G795" t="inlineStr"/>
@@ -27329,7 +27353,7 @@
       </c>
       <c r="F796" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G796" t="inlineStr"/>
@@ -27700,7 +27724,7 @@
       </c>
       <c r="F807" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G807" t="inlineStr"/>
@@ -28331,7 +28355,7 @@
       </c>
       <c r="F826" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G826" t="inlineStr"/>
@@ -28463,7 +28487,7 @@
       </c>
       <c r="F830" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G830" t="inlineStr"/>
@@ -28991,7 +29015,7 @@
       </c>
       <c r="F846" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G846" t="inlineStr"/>
@@ -29090,7 +29114,7 @@
       </c>
       <c r="F849" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G849" t="inlineStr"/>
@@ -29453,7 +29477,7 @@
       </c>
       <c r="F860" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G860" t="inlineStr"/>
@@ -29923,7 +29947,7 @@
       </c>
       <c r="F874" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G874" t="inlineStr"/>

</xml_diff>

<commit_message>
Card inventory: unwired cards by Set and Type summary table (#475)
* Card inventory: unwired cards by Set and Type summary table

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Handoff: shared lane

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Regenerate the card inventory after merging main

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="3">
@@ -60,10 +64,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -446,13 +451,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -705,6 +719,667 @@
         <is>
           <t>39.9%</t>
         </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Unwired cards by Set and Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Set</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Stronghold</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Personality</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Follower</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Spell</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Holding</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Celestial</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Emperor Edition</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>24</v>
+      </c>
+      <c r="C20" t="n">
+        <v>78</v>
+      </c>
+      <c r="D20" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" t="n">
+        <v>11</v>
+      </c>
+      <c r="F20" t="n">
+        <v>13</v>
+      </c>
+      <c r="G20" t="n">
+        <v>94</v>
+      </c>
+      <c r="H20" t="n">
+        <v>11</v>
+      </c>
+      <c r="I20" t="n">
+        <v>12</v>
+      </c>
+      <c r="J20" t="n">
+        <v>9</v>
+      </c>
+      <c r="K20" t="n">
+        <v>5</v>
+      </c>
+      <c r="M20" t="n">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Promotional–Emperor</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>18</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>30</v>
+      </c>
+      <c r="F21" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" t="n">
+        <v>22</v>
+      </c>
+      <c r="H21" t="n">
+        <v>24</v>
+      </c>
+      <c r="I21" t="n">
+        <v>20</v>
+      </c>
+      <c r="J21" t="n">
+        <v>5</v>
+      </c>
+      <c r="K21" t="n">
+        <v>6</v>
+      </c>
+      <c r="M21" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Coils of Madness</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="n">
+        <v>67</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" t="n">
+        <v>7</v>
+      </c>
+      <c r="G22" t="n">
+        <v>13</v>
+      </c>
+      <c r="H22" t="n">
+        <v>9</v>
+      </c>
+      <c r="I22" t="n">
+        <v>8</v>
+      </c>
+      <c r="J22" t="n">
+        <v>3</v>
+      </c>
+      <c r="L22" t="n">
+        <v>2</v>
+      </c>
+      <c r="M22" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Torn Asunder</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="n">
+        <v>45</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" t="n">
+        <v>6</v>
+      </c>
+      <c r="F23" t="n">
+        <v>12</v>
+      </c>
+      <c r="G23" t="n">
+        <v>41</v>
+      </c>
+      <c r="H23" t="n">
+        <v>6</v>
+      </c>
+      <c r="I23" t="n">
+        <v>5</v>
+      </c>
+      <c r="J23" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>The Shadow's Embrace</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="n">
+        <v>45</v>
+      </c>
+      <c r="D24" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" t="n">
+        <v>8</v>
+      </c>
+      <c r="F24" t="n">
+        <v>8</v>
+      </c>
+      <c r="G24" t="n">
+        <v>39</v>
+      </c>
+      <c r="H24" t="n">
+        <v>5</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5</v>
+      </c>
+      <c r="J24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Gates of Chaos</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>44</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" t="n">
+        <v>7</v>
+      </c>
+      <c r="F25" t="n">
+        <v>8</v>
+      </c>
+      <c r="G25" t="n">
+        <v>32</v>
+      </c>
+      <c r="H25" t="n">
+        <v>7</v>
+      </c>
+      <c r="I25" t="n">
+        <v>3</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Aftermath</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>43</v>
+      </c>
+      <c r="D26" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" t="n">
+        <v>10</v>
+      </c>
+      <c r="G26" t="n">
+        <v>24</v>
+      </c>
+      <c r="H26" t="n">
+        <v>4</v>
+      </c>
+      <c r="I26" t="n">
+        <v>3</v>
+      </c>
+      <c r="J26" t="n">
+        <v>3</v>
+      </c>
+      <c r="M26" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Embers of War</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="n">
+        <v>34</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>8</v>
+      </c>
+      <c r="G27" t="n">
+        <v>29</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" t="n">
+        <v>4</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1</v>
+      </c>
+      <c r="M27" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Twenty Festivals</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>15</v>
+      </c>
+      <c r="D28" t="n">
+        <v>4</v>
+      </c>
+      <c r="E28" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" t="n">
+        <v>7</v>
+      </c>
+      <c r="G28" t="n">
+        <v>21</v>
+      </c>
+      <c r="H28" t="n">
+        <v>13</v>
+      </c>
+      <c r="M28" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ivory Edition</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="n">
+        <v>7</v>
+      </c>
+      <c r="G29" t="n">
+        <v>17</v>
+      </c>
+      <c r="H29" t="n">
+        <v>18</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1</v>
+      </c>
+      <c r="M29" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Before the Dawn</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>17</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" t="n">
+        <v>19</v>
+      </c>
+      <c r="H30" t="n">
+        <v>2</v>
+      </c>
+      <c r="I30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1</v>
+      </c>
+      <c r="M30" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Promotional–Celestial</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>8</v>
+      </c>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" t="n">
+        <v>7</v>
+      </c>
+      <c r="H31" t="n">
+        <v>6</v>
+      </c>
+      <c r="I31" t="n">
+        <v>2</v>
+      </c>
+      <c r="J31" t="n">
+        <v>3</v>
+      </c>
+      <c r="K31" t="n">
+        <v>3</v>
+      </c>
+      <c r="M31" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Seeds of Decay</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>5</v>
+      </c>
+      <c r="I32" t="n">
+        <v>3</v>
+      </c>
+      <c r="M32" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Forgotten Legacy</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>5</v>
+      </c>
+      <c r="G33" t="n">
+        <v>9</v>
+      </c>
+      <c r="M33" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>War of Honor</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" t="n">
+        <v>10</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1</v>
+      </c>
+      <c r="M34" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Celestial Edition</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Honor and Treachery</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="M36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Second City</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>1</v>
+      </c>
+      <c r="M37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Words and Deeds</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>1</v>
+      </c>
+      <c r="M38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>383</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="J39" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="L39" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>1305</v>
       </c>
     </row>
   </sheetData>
@@ -731,37 +1406,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Id</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Set</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Clan</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Blocker</t>
         </is>

</xml_diff>

<commit_message>
Emperor Edition remaining-cards pass: inventory, art pack pin, decision doc, handoff (#492)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -548,14 +548,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="C7" t="n">
         <v>128</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>72.7%</t>
+          <t>78.9%</t>
         </is>
       </c>
     </row>
@@ -566,14 +566,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="C8" t="n">
         <v>132</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>32.6%</t>
+          <t>40.9%</t>
         </is>
       </c>
     </row>
@@ -584,14 +584,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>33.8%</t>
+          <t>42.1%</t>
         </is>
       </c>
     </row>
@@ -602,14 +602,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>251</v>
+        <v>337</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>42.0%</t>
+          <t>56.4%</t>
         </is>
       </c>
     </row>
@@ -620,14 +620,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="C11" t="n">
         <v>151</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>32.5%</t>
+          <t>39.7%</t>
         </is>
       </c>
     </row>
@@ -638,14 +638,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>34.6%</t>
         </is>
       </c>
     </row>
@@ -656,14 +656,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C13" t="n">
         <v>37</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>24.3%</t>
+          <t>48.6%</t>
         </is>
       </c>
     </row>
@@ -674,14 +674,14 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C14" t="n">
         <v>26</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>34.6%</t>
+          <t>46.2%</t>
         </is>
       </c>
     </row>
@@ -710,14 +710,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1072</v>
+        <v>1223</v>
       </c>
       <c r="C16" t="n">
         <v>2174</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>49.3%</t>
+          <t>56.3%</t>
         </is>
       </c>
     </row>
@@ -798,115 +798,115 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Emperor Edition</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1</v>
+          <t>Promotional–Emperor</t>
+        </is>
       </c>
       <c r="C20" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="D20" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F20" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="G20" t="n">
-        <v>94</v>
+        <v>22</v>
       </c>
       <c r="H20" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="I20" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="J20" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M20" t="n">
-        <v>171</v>
+        <v>134</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Promotional–Emperor</t>
-        </is>
+          <t>Coils of Madness</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
       </c>
       <c r="C21" t="n">
-        <v>18</v>
+        <v>67</v>
       </c>
       <c r="D21" t="n">
         <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="F21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G21" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="H21" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="I21" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="J21" t="n">
-        <v>5</v>
-      </c>
-      <c r="K21" t="n">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2</v>
       </c>
       <c r="M21" t="n">
-        <v>134</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Coils of Madness</t>
+          <t>Torn Asunder</t>
         </is>
       </c>
       <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>45</v>
+      </c>
+      <c r="D22" t="n">
+        <v>4</v>
+      </c>
+      <c r="E22" t="n">
+        <v>6</v>
+      </c>
+      <c r="F22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G22" t="n">
+        <v>41</v>
+      </c>
+      <c r="H22" t="n">
+        <v>6</v>
+      </c>
+      <c r="I22" t="n">
+        <v>5</v>
+      </c>
+      <c r="J22" t="n">
         <v>2</v>
       </c>
-      <c r="C22" t="n">
-        <v>67</v>
-      </c>
-      <c r="D22" t="n">
-        <v>3</v>
-      </c>
-      <c r="E22" t="n">
-        <v>9</v>
-      </c>
-      <c r="F22" t="n">
-        <v>7</v>
-      </c>
-      <c r="G22" t="n">
-        <v>13</v>
-      </c>
-      <c r="H22" t="n">
-        <v>9</v>
-      </c>
-      <c r="I22" t="n">
-        <v>8</v>
-      </c>
-      <c r="J22" t="n">
-        <v>3</v>
-      </c>
-      <c r="L22" t="n">
-        <v>2</v>
+      <c r="K22" t="n">
+        <v>1</v>
       </c>
       <c r="M22" t="n">
         <v>123</v>
@@ -915,51 +915,45 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Torn Asunder</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>1</v>
+          <t>Gates of Chaos</t>
+        </is>
       </c>
       <c r="C23" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D23" t="n">
         <v>4</v>
       </c>
       <c r="E23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F23" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G23" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="H23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J23" t="n">
-        <v>2</v>
-      </c>
-      <c r="K23" t="n">
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>123</v>
+        <v>106</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Gates of Chaos</t>
+          <t>Aftermath</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D24" t="n">
         <v>4</v>
@@ -968,220 +962,211 @@
         <v>7</v>
       </c>
       <c r="F24" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G24" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="H24" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
         <v>3</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M24" t="n">
-        <v>106</v>
+        <v>98</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aftermath</t>
-        </is>
+          <t>Embers of War</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2</v>
       </c>
       <c r="C25" t="n">
-        <v>43</v>
-      </c>
-      <c r="D25" t="n">
+        <v>34</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="n">
+        <v>8</v>
+      </c>
+      <c r="G25" t="n">
+        <v>29</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" t="n">
         <v>4</v>
       </c>
-      <c r="E25" t="n">
-        <v>7</v>
-      </c>
-      <c r="F25" t="n">
-        <v>10</v>
-      </c>
-      <c r="G25" t="n">
-        <v>24</v>
-      </c>
-      <c r="H25" t="n">
-        <v>4</v>
-      </c>
-      <c r="I25" t="n">
-        <v>3</v>
-      </c>
       <c r="J25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>98</v>
+        <v>81</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Embers of War</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>2</v>
+          <t>Twenty Festivals</t>
+        </is>
       </c>
       <c r="C26" t="n">
-        <v>34</v>
+        <v>15</v>
+      </c>
+      <c r="D26" t="n">
+        <v>4</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F26" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G26" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="H26" t="n">
-        <v>1</v>
-      </c>
-      <c r="I26" t="n">
-        <v>4</v>
-      </c>
-      <c r="J26" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="M26" t="n">
-        <v>81</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Twenty Festivals</t>
+          <t>Before the Dawn</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="n">
         <v>4</v>
       </c>
-      <c r="E27" t="n">
-        <v>6</v>
-      </c>
-      <c r="F27" t="n">
-        <v>7</v>
-      </c>
       <c r="G27" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H27" t="n">
-        <v>12</v>
+        <v>2</v>
+      </c>
+      <c r="I27" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" t="n">
+        <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Before the Dawn</t>
+          <t>Ivory Edition</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="D28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E28" t="n">
         <v>2</v>
       </c>
       <c r="F28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G28" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="H28" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I28" t="n">
-        <v>3</v>
-      </c>
-      <c r="K28" t="n">
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ivory Edition</t>
+          <t>Promotional–Celestial</t>
         </is>
       </c>
       <c r="C29" t="n">
+        <v>8</v>
+      </c>
+      <c r="D29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" t="n">
+        <v>4</v>
+      </c>
+      <c r="F29" t="n">
+        <v>3</v>
+      </c>
+      <c r="G29" t="n">
+        <v>7</v>
+      </c>
+      <c r="H29" t="n">
         <v>6</v>
       </c>
-      <c r="D29" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" t="n">
+      <c r="I29" t="n">
         <v>2</v>
       </c>
-      <c r="F29" t="n">
-        <v>5</v>
-      </c>
-      <c r="G29" t="n">
-        <v>15</v>
-      </c>
-      <c r="H29" t="n">
-        <v>17</v>
-      </c>
-      <c r="I29" t="n">
-        <v>1</v>
+      <c r="J29" t="n">
+        <v>3</v>
+      </c>
+      <c r="K29" t="n">
+        <v>3</v>
       </c>
       <c r="M29" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Promotional–Celestial</t>
-        </is>
+          <t>Emperor Edition</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
       </c>
       <c r="C30" t="n">
+        <v>7</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" t="n">
         <v>8</v>
       </c>
-      <c r="D30" t="n">
+      <c r="K30" t="n">
         <v>2</v>
       </c>
-      <c r="E30" t="n">
-        <v>4</v>
-      </c>
-      <c r="F30" t="n">
-        <v>3</v>
-      </c>
-      <c r="G30" t="n">
-        <v>7</v>
-      </c>
-      <c r="H30" t="n">
-        <v>6</v>
-      </c>
-      <c r="I30" t="n">
-        <v>2</v>
-      </c>
-      <c r="J30" t="n">
-        <v>3</v>
-      </c>
-      <c r="K30" t="n">
-        <v>3</v>
-      </c>
       <c r="M30" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31">
@@ -1346,34 +1331,34 @@
         <v>321</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>347</v>
+        <v>261</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="L39" s="2" t="n">
         <v>2</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>1102</v>
+        <v>951</v>
       </c>
     </row>
   </sheetData>
@@ -3871,11 +3856,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>Needs a broad, repeatable 'before another player's action resolves' Reaction trigger (a before-resolution window keyed to enemy actions, not built).</t>
-        </is>
-      </c>
+      <c r="G74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -12798,11 +12779,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G341" t="inlineStr">
-        <is>
-          <t>Now expressible on the multi-target shape (TargetSlots.cs, issue #336): two slots, terrain-at-battle and enemy-card-without-attachments, both existing categories; not yet wired.</t>
-        </is>
-      </c>
+      <c r="G341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -16318,11 +16295,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G445" t="inlineStr">
-        <is>
-          <t>Card creation is built (issue #387); still needs a turn-spanning "lost Honor from another player's action since your last turn began" tracked condition, and a one-to-four selection whose MAXIMUM depends on that condition (the multi-target slots, issue #336, have a fixed Min..Max per slot; a condition-dependent Max is the remaining gap).</t>
-        </is>
-      </c>
+      <c r="G445" t="inlineStr"/>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -16755,11 +16728,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G458" t="inlineStr">
-        <is>
-          <t>Needs a new Reaction trigger for 'after an action targets a Samurai' (a card-targeted, not action-classified, trigger -- a different shape from every existing Reaction window) and a duel-refusal override tied to a specific pending challenge -- both novel.</t>
-        </is>
-      </c>
+      <c r="G458" t="inlineStr"/>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
@@ -17720,11 +17689,7 @@
           <t>Lion Ancestor</t>
         </is>
       </c>
-      <c r="C487" t="inlineStr">
-        <is>
-          <t>Second City</t>
-        </is>
-      </c>
+      <c r="C487" t="inlineStr"/>
       <c r="D487" t="inlineStr">
         <is>
           <t>Personality</t>
@@ -18107,11 +18072,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G498" t="inlineStr">
-        <is>
-          <t>Needs a unit-scoped 'bow every card in the target unit meeting a Force comparison' primitive (existing unit/army-scoped primitives only apply static Force modifiers, none perform a bow across a filtered set of cards); the per-card Honor gain has direct precedent (BattleHonor).</t>
-        </is>
-      </c>
+      <c r="G498" t="inlineStr"/>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
@@ -18478,11 +18439,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G509" t="inlineStr">
-        <is>
-          <t>Needs a targeting-immunity flag against a specific Attack kind (Ranged) scoped to a whole unit -- distinct from the existing passive Attack-strength defense (Destrier/Singh Remnants), which reduces effective strength rather than making the target illegal outright.</t>
-        </is>
-      </c>
+      <c r="G509" t="inlineStr"/>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
@@ -25476,11 +25433,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G719" t="inlineStr">
-        <is>
-          <t>Needs an exception to the shared Battle-timing AtBattle requirement (bowing itself 'even if not at the current battlefield') -- buildable as a one-off id exception, the same shape Mirumoto Michi/Togashi Rikyou use in wave 9, but deferred this pass to limit how many such exceptions land in one wave; its own province-Strength raise-or-lower effect directly reuses The Courtesy of the Crane's own precedent and is not itself blocked.</t>
-        </is>
-      </c>
+      <c r="G719" t="inlineStr"/>
     </row>
     <row r="720">
       <c r="A720" t="inlineStr">
@@ -31160,14 +31113,10 @@
       </c>
       <c r="F890" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G890" t="inlineStr">
-        <is>
-          <t>Needs a new Reaction trigger: "after a battle resolution ends."</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G890" t="inlineStr"/>
     </row>
     <row r="891">
       <c r="A891" t="inlineStr">
@@ -32846,14 +32795,10 @@
       </c>
       <c r="F940" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G940" t="inlineStr">
-        <is>
-          <t>The Attack-vs-attachments override now exists (AttackFollowerException, personality-wave-24: an unconditional printed exception is one FollowerException: new("Ranged")). Still needs "last attached to" tracking after detachment (the strength is that Personality's Chi, and the Honor loss and dishonor act on him).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G940" t="inlineStr"/>
     </row>
     <row r="941">
       <c r="A941" t="inlineStr">
@@ -32883,14 +32828,10 @@
       </c>
       <c r="F941" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G941" t="inlineStr">
-        <is>
-          <t>Needs a performer/wielder-keyed Attack-strength axis (already a known gap elsewhere).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G941" t="inlineStr"/>
     </row>
     <row r="942">
       <c r="A942" t="inlineStr">
@@ -32920,14 +32861,10 @@
       </c>
       <c r="F942" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G942" t="inlineStr">
-        <is>
-          <t>Needs a unit-Force-total comparison target (existing categories only compare individual card Force).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G942" t="inlineStr"/>
     </row>
     <row r="943">
       <c r="A943" t="inlineStr">
@@ -33056,14 +32993,10 @@
       </c>
       <c r="F946" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G946" t="inlineStr">
-        <is>
-          <t>Needs a targeting immunity keyed off the acting Personality's own Gold Cost.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G946" t="inlineStr"/>
     </row>
     <row r="947">
       <c r="A947" t="inlineStr">
@@ -33439,14 +33372,10 @@
       </c>
       <c r="F957" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G957" t="inlineStr">
-        <is>
-          <t>Needs an ad hoc "move this Personality into battle" mechanic, distinct from normal Maneuvers assignment.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G957" t="inlineStr"/>
     </row>
     <row r="958">
       <c r="A958" t="inlineStr">
@@ -34478,14 +34407,10 @@
       </c>
       <c r="F988" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G988" t="inlineStr">
-        <is>
-          <t>The action-lock it needed now exists (ActionLock.cs, issue #336): "may not perform actions" for the rest of the turn, blocking every action the card or its attachments perform, still targetable. Nothing else is known to block it (the Dragon-only attach is AttachRequiresKeyword, -4F is ApplyModifier, its target is the existing enemy-force category); not yet wired.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G988" t="inlineStr"/>
     </row>
     <row r="989">
       <c r="A989" t="inlineStr">
@@ -34688,14 +34613,10 @@
       </c>
       <c r="F994" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G994" t="inlineStr">
-        <is>
-          <t>Needs an alternate Attack comparison axis against Gold Cost instead of Force.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G994" t="inlineStr"/>
     </row>
     <row r="995">
       <c r="A995" t="inlineStr">
@@ -35265,7 +35186,7 @@
       </c>
       <c r="F1011" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1011" t="inlineStr"/>
@@ -35471,7 +35392,7 @@
       </c>
       <c r="F1017" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1017" t="inlineStr"/>
@@ -35937,7 +35858,7 @@
       </c>
       <c r="F1031" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1031" t="inlineStr"/>
@@ -35970,7 +35891,7 @@
       </c>
       <c r="F1032" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1032" t="inlineStr"/>
@@ -36461,7 +36382,7 @@
       </c>
       <c r="F1047" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1047" t="inlineStr"/>
@@ -36824,7 +36745,7 @@
       </c>
       <c r="F1058" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1058" t="inlineStr"/>
@@ -37253,7 +37174,7 @@
       </c>
       <c r="F1071" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1071" t="inlineStr"/>
@@ -37484,7 +37405,7 @@
       </c>
       <c r="F1078" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1078" t="inlineStr"/>
@@ -38016,7 +37937,7 @@
       </c>
       <c r="F1094" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1094" t="inlineStr"/>
@@ -38148,7 +38069,7 @@
       </c>
       <c r="F1098" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1098" t="inlineStr"/>
@@ -38415,11 +38336,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1106" t="inlineStr">
-        <is>
-          <t>Needs an attachment Transfer mechanic (issue #435 reevaluation; same gap as oracle-l5r-2520/10900/2598/1151): its Focus Effect is "you may transfer an attachment from your Personality in this duel to another of your Personalities." The Battle half (an enemy card without attachments, bow it, destroy it if this Personality is a Berserker) is separately wirable.</t>
-        </is>
-      </c>
+      <c r="G1106" t="inlineStr"/>
     </row>
     <row r="1107">
       <c r="A1107" t="inlineStr">
@@ -39216,7 +39133,7 @@
       </c>
       <c r="F1130" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1130" t="inlineStr"/>
@@ -39938,7 +39855,7 @@
       </c>
       <c r="F1152" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1152" t="inlineStr"/>
@@ -40143,7 +40060,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1158" t="inlineStr"/>
+      <c r="G1158" t="inlineStr">
+        <is>
+          <t>Chikushudo's Trickery (Open, destroy this Spell, bow its Shugenja, one or two performing unbowed Nonhuman Spirit Personalities and another player's unbowed Personality: "Create a battlefield. Negate all movement to it. Assign the target to attack there; he will not be destroyed during the battle's Combat Segment. Assign the performing Spirits to defend there. Fight a battle there."). A battle outside an Attack Phase at a battlefield that belongs to no province: the same unbuilt structure as Shinobi Assault (oracle-l5r-9927) and The Perfect Moment. Every battle in the engine is keyed by the Defender's province index (MatchState.CurrentBattleProvince / UnresolvedBattlefields, Army(), EffectiveProvinceStrength, the province-destruction step of ResolveBattle, Reconnaissance on ProvinceState) and is reached only through the Attack Phase's SelectBattle and its phase sequence (Battle -&gt; BattleSelection -&gt; Dynasty). It needs (1) a created province-less battlefield that Army()/AtBattle/the resolution step accept (no province to destroy, no Honor from a province), (2) a battle fought from and returning to the Action Phase (with the first-opportunity, Combat Segment and Resolution Segment machinery re-entered), (3) direct assignment of chosen units to the attacking and defending sides with no Maneuvers Segment, (4) a battlefield-scoped 'negate all movement to it' and (5) a Combat-Segment-only 'will not be destroyed' shield on one card. Best built once, jointly with Shinobi Assault and The Perfect Moment (the shared 'create a battle' primitive); the rest of the card (the Nonhuman Spirit performers slot, the unbowed target of another player's, the Spell destroyed and the Shugenja bowed as costs) uses existing primitives.</t>
+        </is>
+      </c>
     </row>
     <row r="1159">
       <c r="A1159" t="inlineStr">
@@ -40173,7 +40094,7 @@
       </c>
       <c r="F1159" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1159" t="inlineStr"/>
@@ -40272,7 +40193,7 @@
       </c>
       <c r="F1162" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1162" t="inlineStr"/>
@@ -40338,7 +40259,7 @@
       </c>
       <c r="F1164" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1164" t="inlineStr"/>
@@ -40952,7 +40873,7 @@
       </c>
       <c r="F1182" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1182" t="inlineStr"/>
@@ -41084,7 +41005,7 @@
       </c>
       <c r="F1186" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1186" t="inlineStr"/>
@@ -41657,7 +41578,7 @@
       </c>
       <c r="F1203" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1203" t="inlineStr"/>
@@ -42765,7 +42686,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1236" t="inlineStr"/>
+      <c r="G1236" t="inlineStr">
+        <is>
+          <t>Summon Swamp Spirits (Limited, bow this Shugenja and target your Personality: "Create a 1F Shadowlands - Nonhuman - Spirit - Swamp Spirit Follower and attach it to him."). Its created card, the Swamp Spirit Follower Proxy (oracle-l5r-10014), has no scan available locally: only its receipt (assets/reference/oracle/emperor-edition/receipts/oracle-l5r-10014-printing-1-image-1.json) is present -- the master image is not on disk and there is no webp working copy -- so the Proxy cannot be published (a created card resolves to a published CreatedOnly scan, CreatedCards.Resolve) and the Spell must not be published without it. The wiring itself is a plain create-and-attach: Limited, Costs ActionCost.BowWielder, Target own-personality, Creates new(CardType.Follower, Force: 1, Keywords: ["Shadowlands", "Nonhuman", "Spirit", "Swamp Spirit"], ProxyId: "oracle-l5r-10014") attached to the target (Merihiko's Swarm / Measure of Devotion shape); it needs no new primitive once the scan is fetched, converted to WebP and published as a CreatedOnly Follower Proxy.</t>
+        </is>
+      </c>
     </row>
     <row r="1237">
       <c r="A1237" t="inlineStr">
@@ -43026,7 +42951,7 @@
       </c>
       <c r="F1244" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1244" t="inlineStr"/>
@@ -43401,7 +43326,7 @@
       </c>
       <c r="F1255" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1255" t="inlineStr"/>
@@ -43632,7 +43557,7 @@
       </c>
       <c r="F1262" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1262" t="inlineStr"/>
@@ -43731,7 +43656,7 @@
       </c>
       <c r="F1265" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1265" t="inlineStr"/>
@@ -44168,7 +44093,7 @@
       </c>
       <c r="F1278" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1278" t="inlineStr"/>
@@ -44432,7 +44357,7 @@
       </c>
       <c r="F1286" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1286" t="inlineStr"/>
@@ -44465,7 +44390,7 @@
       </c>
       <c r="F1287" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1287" t="inlineStr"/>
@@ -44630,7 +44555,7 @@
       </c>
       <c r="F1292" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1292" t="inlineStr"/>
@@ -45162,7 +45087,7 @@
       </c>
       <c r="F1308" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1308" t="inlineStr"/>
@@ -45261,7 +45186,7 @@
       </c>
       <c r="F1311" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1311" t="inlineStr"/>
@@ -45566,7 +45491,7 @@
       </c>
       <c r="F1320" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1320" t="inlineStr"/>
@@ -45830,7 +45755,7 @@
       </c>
       <c r="F1328" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1328" t="inlineStr"/>
@@ -45896,7 +45821,7 @@
       </c>
       <c r="F1330" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1330" t="inlineStr"/>
@@ -46267,7 +46192,7 @@
       </c>
       <c r="F1341" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1341" t="inlineStr"/>
@@ -46440,7 +46365,7 @@
       </c>
       <c r="F1346" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1346" t="inlineStr"/>
@@ -46605,7 +46530,7 @@
       </c>
       <c r="F1351" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1351" t="inlineStr"/>
@@ -47005,7 +46930,7 @@
       </c>
       <c r="F1363" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1363" t="inlineStr"/>
@@ -47339,7 +47264,7 @@
       </c>
       <c r="F1373" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1373" t="inlineStr"/>
@@ -47405,7 +47330,7 @@
       </c>
       <c r="F1375" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1375" t="inlineStr"/>
@@ -47504,7 +47429,7 @@
       </c>
       <c r="F1378" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1378" t="inlineStr"/>
@@ -48481,7 +48406,7 @@
       </c>
       <c r="F1407" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1407" t="inlineStr"/>
@@ -49149,14 +49074,10 @@
       </c>
       <c r="F1427" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1427" t="inlineStr">
-        <is>
-          <t>The general "before this battle resolves" window now exists (issue #310: a Terrain's trait is an AbilityCatalog entry of Timing BeforeResolution, applied once both players pass, ordered by the turn player). Still needs its own effect: TWO independent optional choices ('you may choose and straighten a Samurai ... and you may choose and bow a non-Samurai') -- the optional window (beforeBattleOptional) names one target today; the Terrain-play half is separately wirable.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1427" t="inlineStr"/>
     </row>
     <row r="1428">
       <c r="A1428" t="inlineStr">
@@ -49219,7 +49140,7 @@
       </c>
       <c r="F1429" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1429" t="inlineStr"/>
@@ -49351,7 +49272,7 @@
       </c>
       <c r="F1433" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1433" t="inlineStr"/>
@@ -49582,7 +49503,7 @@
       </c>
       <c r="F1440" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1440" t="inlineStr"/>
@@ -49718,14 +49639,10 @@
       </c>
       <c r="F1444" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1444" t="inlineStr">
-        <is>
-          <t>Needs an Absent-Battle-timed Terrain-play variant (the existing one is Battle-timed only) plus a province-strength passive.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1444" t="inlineStr"/>
     </row>
     <row r="1445">
       <c r="A1445" t="inlineStr">
@@ -49821,7 +49738,7 @@
       </c>
       <c r="F1447" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1447" t="inlineStr"/>
@@ -50056,7 +49973,7 @@
       </c>
       <c r="F1454" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1454" t="inlineStr"/>
@@ -50703,7 +50620,7 @@
       </c>
       <c r="F1473" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1473" t="inlineStr"/>
@@ -50773,14 +50690,10 @@
       </c>
       <c r="F1475" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1475" t="inlineStr">
-        <is>
-          <t>The general "before this battle's resolution" window now exists (issue #310). Still needs its own effect: the controller chooses one unit at the current battlefield to move home, and may then bow it (a mandatory unit-choice window followed by an optional bow); the Terrain-play half is separately wirable.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1475" t="inlineStr"/>
     </row>
     <row r="1476">
       <c r="A1476" t="inlineStr">
@@ -50909,7 +50822,7 @@
       </c>
       <c r="F1479" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1479" t="inlineStr"/>
@@ -51012,14 +50925,10 @@
       </c>
       <c r="F1482" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1482" t="inlineStr">
-        <is>
-          <t>The general "before this battle resolves" window now exists (issue #310); this Terrain's trait is a mandatory sweep (+1F each of your Human Personalities and Followers at the battlefield, -1F each Nonhuman one there) -- the shape training-before-resolution-boost already proves -- so it is nearly unblocked (Human = no Nonhuman keyword); the Terrain-play half is separately wirable.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1482" t="inlineStr"/>
     </row>
     <row r="1483">
       <c r="A1483" t="inlineStr">
@@ -51049,7 +50958,7 @@
       </c>
       <c r="F1483" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1483" t="inlineStr"/>
@@ -51148,7 +51057,7 @@
       </c>
       <c r="F1486" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1486" t="inlineStr"/>
@@ -51391,7 +51300,7 @@
       </c>
       <c r="F1493" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1493" t="inlineStr"/>
@@ -51754,7 +51663,7 @@
       </c>
       <c r="F1504" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1504" t="inlineStr"/>
@@ -52265,7 +52174,7 @@
       </c>
       <c r="F1519" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1519" t="inlineStr"/>
@@ -53213,7 +53122,7 @@
       </c>
       <c r="F1547" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1547" t="inlineStr"/>
@@ -53345,7 +53254,7 @@
       </c>
       <c r="F1551" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1551" t="inlineStr"/>
@@ -53679,14 +53588,10 @@
       </c>
       <c r="F1561" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1561" t="inlineStr">
-        <is>
-          <t>Needs a "count this card's own keywords, excluding a named pattern" mechanism (novel).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1561" t="inlineStr"/>
     </row>
     <row r="1562">
       <c r="A1562" t="inlineStr">
@@ -53749,7 +53654,7 @@
       </c>
       <c r="F1563" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1563" t="inlineStr"/>
@@ -53815,7 +53720,7 @@
       </c>
       <c r="F1565" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1565" t="inlineStr"/>
@@ -53947,14 +53852,10 @@
       </c>
       <c r="F1569" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1569" t="inlineStr">
-        <is>
-          <t>The action-lock exists (issue #336); this one lasts "until this battle ends" -- it needs a battle-scoped duration on ActionLock, plus reducing a unit's Force to 0.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1569" t="inlineStr"/>
     </row>
     <row r="1570">
       <c r="A1570" t="inlineStr">
@@ -54149,7 +54050,7 @@
       </c>
       <c r="F1575" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1575" t="inlineStr"/>
@@ -54185,7 +54086,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1576" t="inlineStr"/>
+      <c r="G1576" t="inlineStr">
+        <is>
+          <t>No Hiding Place: "Reaction: After you announce an action with a Ranged Attack: Give one Ranged Attack from the action -1 strength. That Ranged Attack may target a card in the Defender's home (if otherwise legal)." Still blocked, for the reason AttackTargeting.cs (GrantAttackFollowerException) already records: an Attack's target is chosen and validated ONCE, in the announcing useAbility command (ValidateAbility / RequireLegalAttackTarget), and PendingAttack.TargetId is fixed from then on; the announce window (FindAnnounceWatcher / the announceReaction window Tsuruchi Yakusho uses) opens AFTER that validation, so a Reaction there can neither legalise a target the announcement rejected (a card in the Defender's home is never a legal Attack target today: Attack targets must be at the current battlefield) nor re-select the target. To build it: (1) a target re-selection step in the announce window (the Attack's target, or its province, chosen after the Reaction, with the declaring command carrying no target, or carrying a provisional one); (2) a per-announced-action record (like RangedAttackStrengthReductionImmune, MatchState) holding the -1 strength delta and a 'may target a card in the Defender's home' permission consumed by the first Ranged Attack the action produces; (3) RequireLegalAttackTarget and the Attack reaction windows accepting a Defender's-home card under that permission (its 'location' being the Defender's home, so location-keyed reactions such as Ezuno/Yojimbo redirects read it correctly). 'One Ranged Attack from the action' also needs the action's Attacks counted (only single-Attack actions exist today).</t>
+        </is>
+      </c>
     </row>
     <row r="1577">
       <c r="A1577" t="inlineStr">
@@ -54421,7 +54326,7 @@
       </c>
       <c r="F1583" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1583" t="inlineStr"/>
@@ -54594,7 +54499,7 @@
       </c>
       <c r="F1588" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1588" t="inlineStr"/>
@@ -54792,7 +54697,7 @@
       </c>
       <c r="F1594" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1594" t="inlineStr"/>
@@ -55204,7 +55109,7 @@
       </c>
       <c r="F1606" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1606" t="inlineStr"/>
@@ -56078,7 +55983,7 @@
       </c>
       <c r="F1632" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1632" t="inlineStr"/>
@@ -56111,7 +56016,7 @@
       </c>
       <c r="F1633" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1633" t="inlineStr"/>
@@ -56147,7 +56052,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1634" t="inlineStr"/>
+      <c r="G1634" t="inlineStr">
+        <is>
+          <t>Rend the Soul: two halves, neither expressible with today's primitives. (1) "As a Focus Effect: Raise this card's Focus Value to 5. If your Personality wins this duel, he loses instead (the other Personality still also loses)." Dueling.cs totals a focused card's PRINTED Focus (+ the Duel to First Blood +1 per-card bonus); there is no 'raise this card's Focus Value to N' Focus Effect (a per-focused-card override read by the duel totals) and no outcome rewrite that makes the winner take the loser's consequences as well as the loser (ApplyDuelOutcome / winnerId,loserIds are computed once from the totals; a tie has no winner, so 'both lose' is not a state of the resolution). (2) "Battle: Choose your performing opposed Personality: Give him +5F. If the army he is in during this battle's resolution wins, this battle is tied instead. You will not destroy the province in this battle's resolution." The +5F is an ordinary modifier, but MatchEngine.ContinueResolveBattle has no hook that (a) reads which army a marked Personality is in when the battle resolves and, if that army would win, resolves the battle as the existing tie (each side destroys the other army, tie Honor rules) instead, or (b) carries a per-battle 'this player will not destroy the province' flag consulted where the margin over province strength is judged. To build it: a MatchState record of marked Personalities + 'no province destruction for player P' for the current battle (cleared with the battle, like Nerve Strike's ActionLockUntilBattleEnd), read in ContinueResolveBattle right after the totals are compared; and, for the Focus Effect, a FocusEffect kind 'raise-focus-to' plus a duel-outcome kind 'winner-also-loses' in ApplyDuelFocusEffect. Both halves must ship together (an unwired half is a partially working card).</t>
+        </is>
+      </c>
     </row>
     <row r="1635">
       <c r="A1635" t="inlineStr">
@@ -56346,7 +56255,7 @@
       </c>
       <c r="F1640" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1640" t="inlineStr"/>
@@ -56478,7 +56387,7 @@
       </c>
       <c r="F1644" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1644" t="inlineStr"/>
@@ -56651,7 +56560,7 @@
       </c>
       <c r="F1649" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1649" t="inlineStr"/>
@@ -56684,7 +56593,7 @@
       </c>
       <c r="F1650" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1650" t="inlineStr"/>
@@ -56783,7 +56692,7 @@
       </c>
       <c r="F1653" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1653" t="inlineStr"/>
@@ -57199,7 +57108,7 @@
       </c>
       <c r="F1665" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1665" t="inlineStr"/>
@@ -57331,7 +57240,7 @@
       </c>
       <c r="F1669" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1669" t="inlineStr"/>
@@ -57397,7 +57306,7 @@
       </c>
       <c r="F1671" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1671" t="inlineStr"/>
@@ -57933,7 +57842,7 @@
       </c>
       <c r="F1687" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1687" t="inlineStr"/>
@@ -57999,7 +57908,7 @@
       </c>
       <c r="F1689" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1689" t="inlineStr"/>
@@ -58065,7 +57974,7 @@
       </c>
       <c r="F1691" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1691" t="inlineStr"/>
@@ -58197,7 +58106,7 @@
       </c>
       <c r="F1695" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1695" t="inlineStr"/>
@@ -58696,7 +58605,7 @@
       </c>
       <c r="F1710" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1710" t="inlineStr"/>
@@ -58960,7 +58869,7 @@
       </c>
       <c r="F1718" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1718" t="inlineStr"/>
@@ -59562,7 +59471,7 @@
       </c>
       <c r="F1736" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1736" t="inlineStr"/>
@@ -59628,7 +59537,7 @@
       </c>
       <c r="F1738" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1738" t="inlineStr"/>
@@ -59730,7 +59639,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1741" t="inlineStr"/>
+      <c r="G1741" t="inlineStr">
+        <is>
+          <t>Surprise Attack: "Battle: Choose one or more of your performing Nonhuman Personalities at the current battlefield and target one of the enemy leader's Personalities there or at home: Create a battlefield (not associated with any province). Move all the performers and targets there." Blocked on the battlefield model: every battlefield in the engine IS one of the Defender's provinces (an index 0..3 -- UnresolvedBattlefields, CurrentBattleProvince (over 150 uses), Province.Reconnaissance, Province Strength and province destruction in ContinueResolveBattle, AdjacentProvinces, the Terrain and Region placement, the attack-assignment and battle-selection commands, and the client's per-province battle board via MatchView). A battlefield associated with no province needs a new battlefield concept (an id that is not a province index, with its own Terrain slot, Reconnaissance state, adjacency -- the printed text does not say whether it counts as adjacent to anything -- a resolution with no Province Strength and nothing to destroy, and a slot in the Attacker's battle order, since the core rules say every battlefield is fought exactly once), threaded through all of those readers and the client view. It could be built as a synthetic Province entry appended to the Defender's list flagged Phantom (Destroyed never set, Strength 0, excluded from Hidden Falls Dojo's and the maneuver assignment listings), but that touches every Provinces enumeration (the attack/defense assignment lists, DestroyProvince, victory checks) and the shared MatchView shape, and it is a larger change than one card justifies without Mendon's ruling on the open questions above (is the created battlefield fought as an extra battle this Attack Phase? which cards may be assigned or moved there? does it disappear when its battle ends?).</t>
+        </is>
+      </c>
     </row>
     <row r="1742">
       <c r="A1742" t="inlineStr">
@@ -60032,7 +59945,7 @@
       </c>
       <c r="F1750" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1750" t="inlineStr"/>
@@ -60204,7 +60117,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1755" t="inlineStr"/>
+      <c r="G1755" t="inlineStr">
+        <is>
+          <t>The Compassion of the Unicorn: "As a Focus Effect: You may choose (now) to delay the effects of losing this duel until after the next Dynasty Phase begins. // Battle/Open: Choose your performing unbowed Unicorn Clan Personality and target another unit: Straighten it. Gain 1 Honor, or 2 Honor if you do not control the target." Unwired because of the Focus Effect only: it needs the shared delay mechanism Mendon and the coordinator are designing together ("delay effects / actions / a phase" -- Halls of the Forgotten, Strength of the Spider oracle-l5r-8362 and The Courage of the Mantis, oracle-l5r-7995, are blocked on the same clause). What is missing is a duel-loss consequence that is not applied when the duel resolves (Dueling.cs ApplyDuelOutcome applies the loser's consequences immediately) but is held, per duel and per loser, as a persisted pending consequence and released when the next Dynasty Phase begins (SetPhase(Phase.Dynasty) is the one place that phase starts), plus the "(now)" yes/no choice at Focus Effect resolution (FocusEffectChoice.cs is the place: a choice among {delay, do not delay}). The Battle/Open half is separately buildable from existing pieces: a performer category "own-unbowed-personality-with-keyword-at-battle" over the Unicorn Clan (a Clan check, HasClanAffiliation, like own-unbowed-spider-personality-at-battle), the "other-unit" target category, StraightenUnit, and GainHonor(1 or 2) read from whether the target is the player's own. It was not published half-built.</t>
+        </is>
+      </c>
     </row>
     <row r="1756">
       <c r="A1756" t="inlineStr">
@@ -60239,7 +60156,7 @@
       </c>
       <c r="G1756" t="inlineStr">
         <is>
-          <t>Needs a delayed duel-loss-consequence mechanism (issue #435 reevaluation): its Focus Effect is "you may choose (now) to delay the effects of losing this duel until after the next Dynasty Phase begins" -- genuinely novel duel-resolution-timing plumbing (Strength of the Spider, oracle-l5r-8362, is blocked on the identical clause and deliberately deferred rather than invented for one card; see CardAbilities.cs). The Battle half (a Mantis Clan performer, move to the current battlefield, an additional Battle action) is separately wirable.</t>
+          <t>The Courage of the Mantis: "As a Focus Effect: You may choose (now) to delay the effects of losing this duel until after the next Dynasty Phase begins. // Battle: If any enemy units are at the current battlefield, choose your performing unbowed Mantis Clan Personality: Move him there. You may take an additional Battle action." Unwired because of the Focus Effect only -- the same missing shared delay mechanism as The Compassion of the Unicorn (oracle-l5r-7991; see its note for what the mechanism must do). The Battle half is Broken Alliance's shape (Move: new(MoveSpec.Performer, MoveSpec.CurrentBattlefield), MovesToBattle, the enemy-units-at-the-battlefield Require) with a Mantis Clan performer (a Clan check) and GrantAdditionalAction(player.Id, null), and is buildable now. Not published half-built.</t>
         </is>
       </c>
     </row>
@@ -60407,7 +60324,7 @@
       </c>
       <c r="F1761" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1761" t="inlineStr"/>
@@ -60539,7 +60456,7 @@
       </c>
       <c r="F1765" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1765" t="inlineStr"/>
@@ -60638,7 +60555,7 @@
       </c>
       <c r="F1768" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1768" t="inlineStr"/>
@@ -60711,7 +60628,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1770" t="inlineStr"/>
+      <c r="G1770" t="inlineStr">
+        <is>
+          <t>The Honesty of the Phoenix: "As a Focus Effect: You may choose (now) to delay the effects of losing this duel until after the next Dynasty Phase begins. // Battle/Open: If you are a Phoenix Clan player, choose your performing unbowed Phoenix Clan Personality: Name a card. After the next resolution this turn of your action from another Strategy or Ring with that title, draw a card, and choose a player, who discards a card. Remove this card from the game." Three missing pieces: (1) the shared delay mechanism for the Focus Effect (see The Compassion of the Unicorn, oracle-l5r-7991); (2) NAMING a card title: there is no command or choice in the engine that names a title (a free-text or catalogue-list title choice on the acting player's command, validated against the catalogue), and (3) a standing per-turn watch keyed on the named title -- "after the next resolution this turn of your action from another Strategy or Ring with that title" -- which would read MatchState.LastResolvedAction (ActionEffectTracking.cs already records the resolved action's AbilityId/SourceId/PlayerId) once, then run a draw and a chosen player's discard (DeciderChoice.cs / ForcedDiscard cover the discard), and finally the cost "remove this card from the game" (CostVerbs.Remove exists and RemoveSource is declared). Only (1) and (2) are genuinely new structure; the watch is an AfterActionResolved-style watch like Fair Warning's.</t>
+        </is>
+      </c>
     </row>
     <row r="1771">
       <c r="A1771" t="inlineStr">
@@ -60744,7 +60665,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1771" t="inlineStr"/>
+      <c r="G1771" t="inlineStr">
+        <is>
+          <t>The Honor of the Lion (Strategy): its Focus Effect, "You may choose (now) to delay the effects of losing this duel until after the next Dynasty Phase begins", needs the shared delay mechanism (Mendon 2026-09-24: cards that delay effects, actions or a phase are to be built together by Mendon and the coordinator, not card by card): Dueling.cs applies a duel's outcome as one indivisible case per duel-issuing ability (ApplyDuelOutcome) plus each focused card's own loss-keyed traits, and the only deferral the engine has is DelayedDestruction.cs's delay-destroy kind (one destruction put off until the turn ends), not the bows, moves home, Honor/Gold losses, penalties and tokens that are also consequences of losing. It needs a per-duel queue of the loser's consequences, drained when the next Dynasty Phase begins (SetPhase(Phase.Dynasty) is the hook). The Battle/Open half is separately wirable with what exists and was checked: "Choose your performing unbowed honorable Lion Clan Personality: Permanently give him a bonus raising his PH to 4 and the ability, 'Battle: Target an enemy Personality with equal or lower Personal Honor: Bow him. Gain 2 Honor.'" is a permanent PersonalHonor modifier (AddPermanentModifier, set to 4 from his current value), a permanent granted ability (GrantAbility, GrantDuration.Permanent) with a small new Target category (an enemy Personality with equal or lower Personal Honor than the source, the holder; enemy-personality-honor-lt-source is the strictly-lower sibling), and the honorable/unbowed Lion Clan performer category (HasClanAffiliation + MatchesTargetStatus(IsHonorable)) -- so the card would be wired whole the moment the delay mechanism exists.</t>
+        </is>
+      </c>
     </row>
     <row r="1772">
       <c r="A1772" t="inlineStr">
@@ -60811,14 +60736,10 @@
       </c>
       <c r="F1773" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1773" t="inlineStr">
-        <is>
-          <t>Needs a new trigger keyed to passing instead of a Battle action (novel; the Terrain-play half is separately wirable).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1773" t="inlineStr"/>
     </row>
     <row r="1774">
       <c r="A1774" t="inlineStr">
@@ -60881,7 +60802,7 @@
       </c>
       <c r="F1775" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1775" t="inlineStr"/>
@@ -60984,7 +60905,7 @@
       </c>
       <c r="F1778" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1778" t="inlineStr"/>
@@ -61053,7 +60974,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1780" t="inlineStr"/>
+      <c r="G1780" t="inlineStr">
+        <is>
+          <t>The Loyalty of the Scorpion (Strategy): its Focus Effect, "You may choose (now) to delay the effects of losing this duel until after the next Dynasty Phase begins", needs the shared delay mechanism (see oracle-l5r-8138: a per-duel queue of the loser's consequences drained when the next Dynasty Phase begins; Mendon's instruction of 2026-09-24 is that delay cards are built together, not invented card by card). The Reaction half is otherwise wirable with what exists and was checked: "After an action targets your Scorpion Clan Personality, destroy your performing Scorpion Clan Personality: Negate either the bowing, movement, or destruction of the target from the action's effects" is a targeted-by-action Reaction (TargetedActionReactions.cs; TargetedActionReactionApplies would need a case: the action, any player's, targets a Scorpion Clan Personality of the reactor's, and the reactor has another Scorpion Clan Personality to destroy), whose cost is a declared CostVerbs.Sacrifice of a chosen performing Personality (Performer category own-personality of Clan Scorpion), and whose effect is NegateEffects(target, kind) for one kind the player names among bow / move / destroy -- the choice of kind is three sibling ability ids sharing one use (the Hama/Isul bow-or-straighten pair shape), each offered only against an action that could cause that kind (BowsTarget / MoveOrStraightenKind / DestroysTarget). Only the delayed Focus Effect is missing.</t>
+        </is>
+      </c>
     </row>
     <row r="1781">
       <c r="A1781" t="inlineStr">
@@ -61153,7 +61078,7 @@
       </c>
       <c r="F1783" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1783" t="inlineStr"/>
@@ -61186,14 +61111,10 @@
       </c>
       <c r="F1784" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1784" t="inlineStr">
-        <is>
-          <t>Its Battle half (one to three enemy dishonorable Personalities moved home) is a multi-target slot now (issue #336); its Reaction half is the still-unbuilt "negate unless the affected player pays a cost" mechanism.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1784" t="inlineStr"/>
     </row>
     <row r="1785">
       <c r="A1785" t="inlineStr">
@@ -61293,14 +61214,10 @@
       </c>
       <c r="F1787" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1787" t="inlineStr">
-        <is>
-          <t>Needs a unit-Force-total comparison Target (same gap as oracle-l5r-2900) plus a per-card override of "a bowed card contributes no Force."</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1787" t="inlineStr"/>
     </row>
     <row r="1788">
       <c r="A1788" t="inlineStr">
@@ -61330,7 +61247,7 @@
       </c>
       <c r="F1788" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1788" t="inlineStr"/>
@@ -61363,7 +61280,7 @@
       </c>
       <c r="F1789" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1789" t="inlineStr"/>
@@ -61396,7 +61313,7 @@
       </c>
       <c r="F1790" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1790" t="inlineStr"/>
@@ -61631,7 +61548,7 @@
       </c>
       <c r="F1797" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1797" t="inlineStr"/>
@@ -62068,7 +61985,7 @@
       </c>
       <c r="F1810" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1810" t="inlineStr"/>
@@ -62369,7 +62286,7 @@
       </c>
       <c r="F1819" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1819" t="inlineStr"/>
@@ -62674,7 +62591,7 @@
       </c>
       <c r="F1828" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1828" t="inlineStr"/>
@@ -63078,7 +62995,7 @@
       </c>
       <c r="F1840" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1840" t="inlineStr"/>
@@ -63280,7 +63197,7 @@
       </c>
       <c r="F1846" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1846" t="inlineStr"/>
@@ -63313,7 +63230,7 @@
       </c>
       <c r="F1847" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1847" t="inlineStr"/>
@@ -63610,7 +63527,7 @@
       </c>
       <c r="F1856" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1856" t="inlineStr"/>
@@ -63746,7 +63663,7 @@
       </c>
       <c r="F1860" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1860" t="inlineStr"/>
@@ -63812,7 +63729,7 @@
       </c>
       <c r="F1862" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1862" t="inlineStr"/>
@@ -63944,7 +63861,7 @@
       </c>
       <c r="F1866" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1866" t="inlineStr"/>
@@ -64179,7 +64096,7 @@
       </c>
       <c r="F1873" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1873" t="inlineStr"/>
@@ -64670,7 +64587,7 @@
       </c>
       <c r="F1888" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1888" t="inlineStr"/>
@@ -65132,7 +65049,7 @@
       </c>
       <c r="F1902" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1902" t="inlineStr"/>
@@ -65297,7 +65214,7 @@
       </c>
       <c r="F1907" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1907" t="inlineStr"/>
@@ -65561,7 +65478,7 @@
       </c>
       <c r="F1915" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1915" t="inlineStr"/>
@@ -66159,7 +66076,7 @@
       </c>
       <c r="F1933" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1933" t="inlineStr"/>
@@ -66357,7 +66274,7 @@
       </c>
       <c r="F1939" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1939" t="inlineStr"/>
@@ -66980,7 +66897,7 @@
       </c>
       <c r="F1958" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1958" t="inlineStr"/>
@@ -67318,7 +67235,7 @@
       </c>
       <c r="F1968" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1968" t="inlineStr"/>
@@ -68052,7 +67969,7 @@
       </c>
       <c r="F1990" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1990" t="inlineStr"/>
@@ -68877,7 +68794,7 @@
       </c>
       <c r="F2015" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2015" t="inlineStr"/>
@@ -69207,7 +69124,7 @@
       </c>
       <c r="F2025" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2025" t="inlineStr"/>
@@ -69240,7 +69157,7 @@
       </c>
       <c r="F2026" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2026" t="inlineStr"/>
@@ -69372,7 +69289,7 @@
       </c>
       <c r="F2030" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2030" t="inlineStr"/>
@@ -69405,7 +69322,7 @@
       </c>
       <c r="F2031" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2031" t="inlineStr"/>
@@ -69504,7 +69421,7 @@
       </c>
       <c r="F2034" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2034" t="inlineStr"/>
@@ -69607,7 +69524,7 @@
       </c>
       <c r="F2037" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2037" t="inlineStr"/>
@@ -69706,7 +69623,7 @@
       </c>
       <c r="F2040" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2040" t="inlineStr"/>
@@ -69945,7 +69862,7 @@
       </c>
       <c r="F2047" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2047" t="inlineStr"/>
@@ -70386,7 +70303,7 @@
       </c>
       <c r="F2060" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2060" t="inlineStr"/>
@@ -70419,7 +70336,7 @@
       </c>
       <c r="F2061" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2061" t="inlineStr"/>
@@ -70687,7 +70604,7 @@
       </c>
       <c r="F2069" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2069" t="inlineStr"/>
@@ -70988,7 +70905,7 @@
       </c>
       <c r="F2078" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2078" t="inlineStr"/>
@@ -71825,7 +71742,7 @@
       </c>
       <c r="F2103" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2103" t="inlineStr"/>
@@ -71891,7 +71808,7 @@
       </c>
       <c r="F2105" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2105" t="inlineStr"/>
@@ -72060,7 +71977,7 @@
       </c>
       <c r="F2110" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2110" t="inlineStr"/>
@@ -72093,7 +72010,7 @@
       </c>
       <c r="F2111" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2111" t="inlineStr"/>
@@ -72291,7 +72208,7 @@
       </c>
       <c r="F2117" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2117" t="inlineStr"/>
@@ -72757,7 +72674,7 @@
       </c>
       <c r="F2131" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2131" t="inlineStr"/>
@@ -72790,7 +72707,7 @@
       </c>
       <c r="F2132" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2132" t="inlineStr"/>
@@ -72988,7 +72905,7 @@
       </c>
       <c r="F2138" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2138" t="inlineStr"/>
@@ -73021,7 +72938,7 @@
       </c>
       <c r="F2139" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2139" t="inlineStr"/>
@@ -73087,7 +73004,7 @@
       </c>
       <c r="F2141" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2141" t="inlineStr"/>
@@ -73255,7 +73172,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2146" t="inlineStr"/>
+      <c r="G2146" t="inlineStr">
+        <is>
+          <t>Kaiu Village (Region, group F): both Reactions create an Item and attach it to the entering Personality. The Armor half is buildable (Kaiu Armor, oracle-l5r-10007, is a published +1F Armor proxy), but the Weapon half needs a created "+1F/+1C Weapon Item" and no such Proxy scan exists locally: the only created Weapons are Yasunori's Gift (+1F/+0C, oracle-l5r-10019), Water Bo (+2F/+0C, oracle-l5r-10026), Flame Katana (+3F/+1C, oracle-l5r-10022) and Masayoshi's Blade (4F/1C, oracle-l5r-10204). CreatedCards.Resolve fits a created card to a published CreatedOnly scan by Force, Chi and keywords, so it cannot invent one. The rest is existing machinery: an own-personality-enters-play window (The Spider's Web's trigger) and Create-and-attach with a Fixed(2) Gold cost. Wire both halves as soon as a +1F/+1C Weapon Proxy scan (Kaiu Weapon) is fetched; a card with only one working Reaction is not published.</t>
+        </is>
+      </c>
     </row>
     <row r="2147">
       <c r="A2147" t="inlineStr">
@@ -73424,7 +73345,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2151" t="inlineStr"/>
+      <c r="G2151" t="inlineStr">
+        <is>
+          <t>Plains of Otosan Uchi (Region, group F): "This province holds two Dynasty cards; do not reveal the second card in the Events Phase this card enters play. You decide each time which card slot is revealed, resolved, or refilled first. Before this province is destroyed: Lose 10 Honor." Every province is modelled as exactly one card slot (ProvinceState.CardId): the Events Phase reveal loop, Purchase and Reserve recruits from a province, Refill, DestroyProvince's discard, Border Keep's and the Kharmic cycles, the private province looks, MatchView.ProvinceView and the client's province stacks all assume one card, so a second slot (a SecondCardId with its own reveal, refill, purchase and destruction paths, the controller's choice of which slot goes first, and a view/client field for it) is a structural change across the engine, the wire view and the client rather than a card-sized primitive. The 10-Honor trait ("before this province is destroyed", a cost-like loss that DestroyProvince would have to make first) is buildable once the province has both slots. Not published.</t>
+        </is>
+      </c>
     </row>
     <row r="2152">
       <c r="A2152" t="inlineStr">
@@ -73520,7 +73445,7 @@
       </c>
       <c r="F2154" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2154" t="inlineStr"/>
@@ -73689,7 +73614,7 @@
       </c>
       <c r="F2159" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2159" t="inlineStr"/>

</xml_diff>

<commit_message>
Rulings pass: inventory, art pack r2 pin, decision doc and handoff after the Shinobi Assault, Two Fronts, Perfect Moment and Honesty scans (#494)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -602,14 +602,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>57.4%</t>
+          <t>57.9%</t>
         </is>
       </c>
     </row>
@@ -710,14 +710,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1249</v>
+        <v>1252</v>
       </c>
       <c r="C16" t="n">
         <v>2183</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>57.2%</t>
+          <t>57.4%</t>
         </is>
       </c>
     </row>
@@ -999,7 +999,7 @@
         <v>8</v>
       </c>
       <c r="G25" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H25" t="n">
         <v>1</v>
@@ -1011,7 +1011,7 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26">
@@ -1191,7 +1191,7 @@
         <v>2</v>
       </c>
       <c r="G31" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H31" t="n">
         <v>1</v>
@@ -1203,7 +1203,7 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="32">
@@ -1216,10 +1216,10 @@
         <v>5</v>
       </c>
       <c r="G32" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M32" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33">
@@ -1331,7 +1331,7 @@
         <v>75</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="H39" s="2" t="n">
         <v>91</v>
@@ -1349,7 +1349,7 @@
         <v>2</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>934</v>
+        <v>931</v>
       </c>
     </row>
   </sheetData>
@@ -57749,14 +57749,10 @@
       </c>
       <c r="F1687" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1687" t="inlineStr">
-        <is>
-          <t>Shinobi Assault (The Shadow's Embrace, Limited, Ninja). WIRED and tested (ability shinobi-assault-battle, EmperorRulingR1Cards.cs; EmperorRulingR1Tests.ShinobiAssault, through a Strategy that carries its own printed definition) on the battle-without-a-province model (Mendon's ruling): a battlefield created at no province, the performing unbowed Ninja assigned to attack, the target assigned to defend even if bowed, the battle fought inside the Action Phase with the player of Shinobi Assault as its Attacker and holding the first opportunity (a first-opportunity claim), then Lose 5 Honor, then the Action Phase resumes. NOT PUBLISHED: the scan is not in the repository (only assets/reference/oracle/the-shadow-s-embrace/receipts/oracle-l5r-9927-printing-1-image-1.json; there is no images/ or webp/ folder, and the catalogue art pack holds only hashed art), so the printed text could not be read by eye and tools/content/package_vanilla_wave.build_definition_fields cannot copy the art. The Oracle text used for the wiring is 'Limited: Choose your performing unbowed Ninja Personality and target another player's Personality: Create a battlefield (not at any province). Assign your Personality to attack there. Assign the target to defend there, even if he is bowed. Fight a battle there, in which you have the first opportunity to take a Battle action or pass. Lose 5 Honor.' (cost 4, focus 1, Ninja). To publish: supply the scan (webp working copy plus receipt), read it against that text, add a strategy-wave-63 packager with Abilities ["shinobi-assault-battle"], and register the wave (csproj, PublishedContent, CardCatalog, manifest).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1687" t="inlineStr"/>
     </row>
     <row r="1688">
       <c r="A1688" t="inlineStr">
@@ -61229,14 +61225,10 @@
       </c>
       <c r="F1791" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1791" t="inlineStr">
-        <is>
-          <t>The Perfect Moment (Forgotten Legacy, Reaction). WIRED and tested (ability perfect-moment-declare; EmperorRulingR1Tests.PerfectMoment): Retribution's window and additional Attack Phase (shared now as DeclareAdditionalAttackPhase): its player, the Defender of the phase that ended, declares the additional Attack Phase and is its Attacker (Mendon's ruling); during it (RulingR1State.PerfectMoment) he destroys at most one of the previous Attacker's provinces (the second victory destroys none), and his Personalities may not be assigned and will not move (assignment, movement to a battlefield and moving home are all refused through MovementLocked) unless they are Paragons or Battle Maidens; Retribution's one-Personality limit and +1F do not apply to it. NOT PUBLISHED: the scan is not in the repository (receipt only: assets/reference/oracle/forgotten-legacy/receipts/oracle-l5r-8257-printing-1-image-1.json). Oracle text used: 'Reaction: After the end of an Attack Phase in which you were the Defender: Create an additional Attack Phase with the previous phase's Attacker as the Defender. During this Attack Phase, you will not destroy more than one of the Defender's provinces and your Personalities may not assign and will not move unless they are Paragons or Battle Maidens.' (cost 0, focus 4). Reading to confirm against the scan: 'will not move' covers every movement of his Personalities during the phase, not only movement to battlefields; a Personality's return home after a battle is the rules' own and is not a movement. To publish: supply the scan, read it, add the packager with Abilities ["perfect-moment-declare"] and register the wave.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1791" t="inlineStr"/>
     </row>
     <row r="1792">
       <c r="A1792" t="inlineStr">
@@ -62507,14 +62499,10 @@
       </c>
       <c r="F1829" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1829" t="inlineStr">
-        <is>
-          <t>Two Fronts (Embers of War, Limited). WIRED and tested (ability two-fronts-mark; the primitive is MatchEngine.MarkTwoFronts / CreateTwoFrontsBattlefields, EmperorRulingR1.cs; EmperorRulingR1Tests.TwoFrontsSecondBattle and TwoFrontsCard): 'During your next normal Attack Phase (this turn), create two battlefields associated with it instead of one' makes the declaration of the player's next NORMAL Attack Phase (an additional one does not count) create a second, additional battlefield associated with the marked province; it destroys the province like the first, and when the first battle destroys the province the second is fought at a battlefield without one (both orders tested). Requires the province's player to have two or more provinces. NOT PUBLISHED: the scan is not in the repository (receipt only: assets/reference/oracle/embers-of-war/receipts/oracle-l5r-8922-printing-1-image-1.json). Oracle text used: 'Limited: Target a province whose player has two or more provinces: During your next normal Attack Phase (this turn), create two battlefields associated with it instead of one.' (cost 0, focus 2). The client's attack-assignment picker can name an additional battlefield (BattlefieldName) but has no province mat to click for it; the assignment goes through the sidebar picker. To publish: supply the scan, read it, add the packager with Abilities ["two-fronts-mark"] and register the wave.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1829" t="inlineStr"/>
     </row>
     <row r="1830">
       <c r="A1830" t="inlineStr">

</xml_diff>

<commit_message>
Honor Never Falls, Kurohito's Perfection and Makito: inventory, art pack pin, decision doc, handoff (#496)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -530,14 +530,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C6" t="n">
         <v>830</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>62.2%</t>
+          <t>62.3%</t>
         </is>
       </c>
     </row>
@@ -602,14 +602,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>57.9%</t>
+          <t>58.0%</t>
         </is>
       </c>
     </row>
@@ -656,14 +656,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C13" t="n">
         <v>37</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>48.6%</t>
+          <t>51.4%</t>
         </is>
       </c>
     </row>
@@ -710,14 +710,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1252</v>
+        <v>1255</v>
       </c>
       <c r="C16" t="n">
         <v>2183</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>57.4%</t>
+          <t>57.5%</t>
         </is>
       </c>
     </row>
@@ -903,13 +903,13 @@
         <v>5</v>
       </c>
       <c r="J22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K22" t="n">
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="23">
@@ -990,7 +990,7 @@
         <v>2</v>
       </c>
       <c r="C25" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E25" t="n">
         <v>2</v>
@@ -1011,7 +1011,7 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26">
@@ -1209,14 +1209,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Forgotten Legacy</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>5</v>
+          <t>War of Honor</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>2</v>
       </c>
       <c r="G32" t="n">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1</v>
       </c>
       <c r="M32" t="n">
         <v>13</v>
@@ -1225,20 +1228,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>War of Honor</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>2</v>
+          <t>Forgotten Legacy</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>5</v>
       </c>
       <c r="G33" t="n">
-        <v>10</v>
-      </c>
-      <c r="H33" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="M33" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34">
@@ -1319,7 +1319,7 @@
         <v>7</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D39" s="2" t="n">
         <v>27</v>
@@ -1331,7 +1331,7 @@
         <v>75</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H39" s="2" t="n">
         <v>91</v>
@@ -1340,7 +1340,7 @@
         <v>53</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K39" s="2" t="n">
         <v>13</v>
@@ -1349,7 +1349,7 @@
         <v>2</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>931</v>
+        <v>928</v>
       </c>
     </row>
   </sheetData>
@@ -17896,14 +17896,10 @@
       </c>
       <c r="F494" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G494" t="inlineStr">
-        <is>
-          <t>Makito - experienced (Embers of War): "Maho Battle: Target an enemy Personality with equal or lower Chi: Destroy a card without attachments in his unit; this destruction will not be negated or delayed". NO LOCAL SCAN, so not wired. The DELAY half is supported by the new layer as a per-effect exemption (Delay() asks CannotBeDelayed(kind), the one place a "will not be delayed" promise is added, as Yoritomo Hiromi's, The Shadow's Lair's, Suitengu's Torch's and Journey's End Keep's are); the NEGATION half is still the per-EFFECT unnegatable-destruction flag the existing blocker describes (Protection protects an action, not one destruction of a card the acting player does not own).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr"/>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
@@ -51442,14 +51438,10 @@
       </c>
       <c r="F1500" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1500" t="inlineStr">
-        <is>
-          <t>Honor Never Falls (Forgotten Legacy). Its Focus Effect "Delay all consequences of losing this duel (from any source) until the end of the turn" is now BUILDABLE on the shared delay mechanism (src/L5R.Core/EmperorRulingR2.cs): DelayUntil.EndOfTurn is the trigger, and the duel's delay (EmperorRulingR2Cards.cs, WithDuelLossDelays) records every effect the duel's outcome applies to the loser's unit; "from any source" additionally needs the same scope wrapped around the OTHER Focus Effects that hit the loser (ContinueDuelFocusEffects/ResolveFocusEffectChoiceCommand call ApplyDuelFocusEffect outside the scope today) -- one wrapper per call. NOT wired, for two other reasons: (1) NO LOCAL SCAN (assets/reference/oracle/forgotten-legacy has receipts only, no webp), so the printed text could not be verified and the card cannot be packaged (build_definition_fields needs the scan and its receipt); (2) its Battle half "you may take an additional Battle action to use one of his base abilities" has no exact shape: AdditionalActionGrant.ScopeCardIds scopes a grant to a source CARD, so an ability granted to him could consume it; a scope limited to his printed (base) abilities does not exist.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1500" t="inlineStr"/>
     </row>
     <row r="1501">
       <c r="A1501" t="inlineStr">
@@ -72586,14 +72578,10 @@
       </c>
       <c r="F2132" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2132" t="inlineStr">
-        <is>
-          <t>Kurohito's Perfection (Torn Asunder): "When paying the cost of the rulebook Favor Political Limited action: You may ignore the cost of discarding a card; if you did, delay its effects until your End Phase begins." NO LOCAL SCAN (assets/reference/oracle/torn-asunder has receipts only), so it is not wired or published. The trigger point exists (DelayUntil.EndPhaseBegins, applied by SetPhase(Phase.End)) but this delays a WHOLE action's effects -- the Favor action's Honor, Gold, draw and Imperial Favor changes as well as card effects -- and the recording layer captures only effects on a card (bow, straighten, dishonor, destroy, move, modifiers, tokens, keyword and ability grants). It needs a whole-action capture (every effect the rulebook Favor action applies, on cards AND players, recorded as closures and replayed in order), plus the alternative cost (ignore the discard) tied to the choice; the rulebook Favor action has no AbilityDefinition, so its effects would have to be recorded where the universal command runs.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2132" t="inlineStr"/>
     </row>
     <row r="2133">
       <c r="A2133" t="inlineStr">

</xml_diff>

<commit_message>
Mechanics batch: inventory, art pack, decision doc and handoff for #501
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -514,14 +514,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C5" t="n">
         <v>51</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>86.3%</t>
+          <t>90.2%</t>
         </is>
       </c>
     </row>
@@ -532,14 +532,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>518</v>
+        <v>534</v>
       </c>
       <c r="C6" t="n">
         <v>830</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>62.4%</t>
+          <t>64.3%</t>
         </is>
       </c>
     </row>
@@ -604,14 +604,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>349</v>
+        <v>362</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>58.4%</t>
+          <t>60.5%</t>
         </is>
       </c>
     </row>
@@ -622,14 +622,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C11" t="n">
         <v>151</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>39.7%</t>
+          <t>40.4%</t>
         </is>
       </c>
     </row>
@@ -676,14 +676,14 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C14" t="n">
         <v>26</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>53.8%</t>
         </is>
       </c>
     </row>
@@ -712,14 +712,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1260</v>
+        <v>1293</v>
       </c>
       <c r="C16" t="n">
         <v>2183</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>57.7%</t>
+          <t>59.2%</t>
         </is>
       </c>
     </row>
@@ -989,10 +989,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E25" t="n">
         <v>2</v>
@@ -1001,7 +1001,7 @@
         <v>8</v>
       </c>
       <c r="G25" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="H25" t="n">
         <v>1</v>
@@ -1013,7 +1013,7 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>79</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26">
@@ -1047,184 +1047,178 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Before the Dawn</t>
+          <t>Ivory Edition</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="D27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27" t="n">
         <v>2</v>
       </c>
       <c r="F27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G27" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="H27" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I27" t="n">
-        <v>3</v>
-      </c>
-      <c r="K27" t="n">
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ivory Edition</t>
+          <t>Promotional–Celestial</t>
         </is>
       </c>
       <c r="C28" t="n">
+        <v>8</v>
+      </c>
+      <c r="D28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" t="n">
+        <v>3</v>
+      </c>
+      <c r="G28" t="n">
+        <v>7</v>
+      </c>
+      <c r="H28" t="n">
         <v>6</v>
       </c>
-      <c r="D28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" t="n">
+      <c r="I28" t="n">
         <v>2</v>
       </c>
-      <c r="F28" t="n">
-        <v>5</v>
-      </c>
-      <c r="G28" t="n">
-        <v>15</v>
-      </c>
-      <c r="H28" t="n">
-        <v>17</v>
-      </c>
-      <c r="I28" t="n">
-        <v>1</v>
+      <c r="J28" t="n">
+        <v>3</v>
+      </c>
+      <c r="K28" t="n">
+        <v>3</v>
       </c>
       <c r="M28" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Promotional–Celestial</t>
+          <t>Before the Dawn</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D29" t="n">
         <v>2</v>
       </c>
       <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="n">
         <v>4</v>
       </c>
-      <c r="F29" t="n">
+      <c r="G29" t="n">
+        <v>13</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" t="n">
         <v>3</v>
       </c>
-      <c r="G29" t="n">
-        <v>7</v>
-      </c>
-      <c r="H29" t="n">
-        <v>6</v>
-      </c>
-      <c r="I29" t="n">
-        <v>2</v>
-      </c>
-      <c r="J29" t="n">
-        <v>3</v>
-      </c>
-      <c r="K29" t="n">
-        <v>3</v>
-      </c>
       <c r="M29" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Seeds of Decay</t>
+          <t>The Shadow's Embrace</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E30" t="n">
         <v>1</v>
       </c>
       <c r="F30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" t="n">
+        <v>4</v>
+      </c>
+      <c r="H30" t="n">
         <v>1</v>
       </c>
-      <c r="G30" t="n">
-        <v>5</v>
-      </c>
       <c r="I30" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>The Shadow's Embrace</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" t="n">
-        <v>5</v>
-      </c>
-      <c r="E31" t="n">
-        <v>1</v>
+          <t>War of Honor</t>
+        </is>
       </c>
       <c r="F31" t="n">
         <v>2</v>
       </c>
       <c r="G31" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H31" t="n">
         <v>1</v>
       </c>
-      <c r="I31" t="n">
-        <v>1</v>
-      </c>
-      <c r="K31" t="n">
-        <v>1</v>
-      </c>
       <c r="M31" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>War of Honor</t>
-        </is>
+          <t>Seeds of Decay</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>10</v>
-      </c>
-      <c r="H32" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="I32" t="n">
+        <v>3</v>
       </c>
       <c r="M32" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="33">
@@ -1234,13 +1228,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G33" t="n">
         <v>7</v>
       </c>
       <c r="M33" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34">
@@ -1315,10 +1309,10 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>312</v>
+        <v>296</v>
       </c>
       <c r="D39" s="2" t="n">
         <v>26</v>
@@ -1330,10 +1324,10 @@
         <v>75</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>249</v>
+        <v>236</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I39" s="2" t="n">
         <v>53</v>
@@ -1342,13 +1336,13 @@
         <v>18</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L39" s="2" t="n">
         <v>2</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>923</v>
+        <v>890</v>
       </c>
     </row>
   </sheetData>
@@ -1445,19 +1439,11 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Aramasu's Legacy (Seeds of Decay Mantis Stronghold, Limited). STILL UNWIRED; this pass built part of what it needed. Its text creates an additional Attack Phase from a Limited action, so inside the Action Phase, during which 'battle resolution does not destroy defending armies or Provinces and does not bow your Mantis Clan Magistrates or your attachments', and afterwards 'if you won any of its battles (even against no units at resolution), you may target a Personality or Holding, bow it, and negate its straightening until after your next turn begins'. Available now: an additional Attack Phase declared by a reaction window (DeclareAdditionalAttackPhase, whose declarer is its Attacker by Mendon's ruling) and a battle fought inside the Action Phase that returns to it with the action's own tail (AsideBattle / FinishAsideBattle). Still missing: (1) a WHOLE Attack Phase (Declaration, Infantry and Cavalry Maneuvers, every battle) entered from and returning to the Action Phase, i.e. AsideBattle generalised to a phase sequence that restores the Action Phase's priority and windows afterwards (the aside battle handles one battlefield); (2) resolution-time exemptions scoped to that one phase instance (no army destroyed, no province destroyed, no bow for the player's Mantis Clan Magistrates or their attachments), which would sit beside RulingR1State.PerfectMoment's phase-scoped restrictions; (3) 'if you won any of its battles' (a per-phase win record, even with no units) driving a delayed optional bow of a Personality or Holding with a straighten hold (StraightenHolds can express 'until after your next turn begins'). NOT PUBLISHABLE either way: no scan in the repository (receipt only: assets/reference/oracle/seeds-of-decay/receipts/oracle-l5r-10184-printing-1-image-1.json); Aramasu's Legacy is a Pre-Game Stronghold, so it is not covered by Mendon's battles-without-a-province explanation and was not built speculatively.</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2745,19 +2731,11 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>The Marshalling Fields: "Once per battle, you may ignore any of a Terrain action's restrictions based on another Terrain being in play" needs a conditional override of the one existing restriction that shape actually describes (CreatedCardEntry.cs's "this battlefield already has a Terrain in play" Require), offered as a real choice at the moment the Terrain action is announced -- no primitive bypasses a specific Require conditionally and optionally yet. "After the first time each turn one of your Terrain actions resolves: Draw a card" is buildable now (an ordinary once-per-turn Reaction keyed on ActionCarriesKeyword "Terrain", Draw). Left unwired whole rather than half-wiring one clause of two.</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7979,19 +7957,11 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G191" t="inlineStr">
-        <is>
-          <t>Daidoji Narizane. "Battle: Target an enemy Personality: Bow zero or more different cards in his unit up to the number of Recon actions you have taken this turn" needs a live per-turn Recon-action counter (no card in the published catalogue currently reads "Recon actions taken this turn" as a number; Akeha's own Reaction above only needs a boolean "did the last Recon action come from a Strategy", not a running count) plus a 0..N-of-a-unit bow selection sized by that live count (TargetSlots' own slot-count field is fixed at authoring time, not read from engine state at offer time). Two gaps, not built.</t>
-        </is>
-      </c>
-      <c r="H191" t="inlineStr">
-        <is>
-          <t>COUNTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr"/>
+      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -8943,19 +8913,11 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G219" t="inlineStr">
-        <is>
-          <t>Daigotsu Kazuko. Her entry Honor loss is EntryHonorLoss 1 (built). "Fear Battle: You may destroy one of Kazuko's Followers: Melee 3 Attack, or Melee 6 Attack if you destroyed a Follower" needs an OPTIONAL cost (destroying her own attached Follower) that changes the Attack's own strength formula depending on whether it was paid -- every optional-cost-then-bonus shape built so far (Unexpected's "may bow performer; if you did, draw a card", Sticks and Stones' "if it destroyed a card, draw a card") reads the RESULT of the action to grant a side effect, never feeds back into the Attack's own strength at declare time. Needs a cost-conditional Attack-strength selection.</t>
-        </is>
-      </c>
-      <c r="H219" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr"/>
+      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -9519,19 +9481,11 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G235" t="inlineStr">
-        <is>
-          <t>Needs the removal "when the turn ends" of a card brought into play: bringing a dead Personality out of any player's dead pile under the acting player's control exists (BringDeadPersonalityIntoPlay, Goju Plot; TakeControl and OriginalOwnerId for a card taken from an enemy pile), but nothing removes a card from the game at the end of the turn (created cards leave with the battle, CreatedUntilBattleEndsIds; Events expire on ExpiresAtTurnsTaken). Also ignores the Honor Requirement, and "After Yajinden enters play: Lose 4 Honor" is EntryHonorLoss.</t>
-        </is>
-      </c>
-      <c r="H235" t="inlineStr">
-        <is>
-          <t>CREATE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr"/>
+      <c r="H235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -10475,19 +10429,11 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G263" t="inlineStr">
-        <is>
-          <t>Needs an additional cost of entering play: "either remove a card in your hand from the game or destroy one of your Sake tokens" is paid as part of the Recruit, with a choice between two costs, and the entry path (QuotePurchase, Purchase) knows Gold, Honor Requirements and discounts only. Sake tokens exist (Togashi Sakata).</t>
-        </is>
-      </c>
-      <c r="H263" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr"/>
+      <c r="H263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -10785,19 +10731,11 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G272" t="inlineStr">
-        <is>
-          <t>Needs giving control of an in-play Personality to another player ("After Asuka enters play: You may give control of her to another player"): control transfer of a Personality in play is deliberately not built (docs/decisions/2026-09-12-unique-singular-control-transfer.md; TakeControl covers attachments and cards brought from a discard or dead pile). The other two halves are buildable: "may not assign, and will not move, into a defending army" is an assignment/movement restriction keyed on her Effect (a check in AssignDefense plus a MovementLock kind for moves to a defending side), and "After a Straighten Phase begins: Choose your bowed non-Spider Clan Personality. Negate his straightening this phase" is a StraightenHold (StraightenPoint.StraightenPhaseEnds, the Unseasonable Weather shape already listed in StraightenHolds.cs) on a Personality her controller chooses at the Straighten phase -- a decision at that phase, which no card opens yet.</t>
-        </is>
-      </c>
-      <c r="H272" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr"/>
+      <c r="H272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -13229,19 +13167,11 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G342" t="inlineStr">
-        <is>
-          <t>Ikoma Shika - Experienced (re-verified; the Honor and Treachery pass's own note stands). "Battle: You may discard a card: Ranged 4 Attack, with +2 strength if you discarded a card; if that card was a Terrain, draw a card" still needs an optional-discard-paid-at-declare-time cost whose payment changes the Attack's own strength formula (the same cost-conditional-strength gap oracle-l5r-1734 above needs, plus a card-type check on the specific card discarded and a follow-up draw) -- not built.</t>
-        </is>
-      </c>
-      <c r="H342" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr"/>
+      <c r="H342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -14055,19 +13985,11 @@
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G365" t="inlineStr">
-        <is>
-          <t>Needs "You may take an additional action" for the Open half: an Additional Action grant is only ever consumed by a Battle action (ContinueUseAbility), so in the Action Phase nothing can take the granted action (the gap oracle-l5r-7588 names). The standing watch ("after the next time this turn you announce an action on one of Momoko's Spells, ignore the action's bowing costs" -- the scan prints "non-destruction costs"; the catalogue text carries the October 5th erratum) is buildable as a per-card turn stamp read by CostExempt (AbilityCosts.cs) for a Bow cost whose source is a Spell attached to her, and the Battle half's additional action is the ordinary grant.</t>
-        </is>
-      </c>
-      <c r="H365" t="inlineStr">
-        <is>
-          <t>ADDACT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr"/>
+      <c r="H365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -14233,19 +14155,11 @@
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G370" t="inlineStr">
-        <is>
-          <t>Needs a Reaction to an action targeting one of your OTHER Personalities at Sakonoko's location, with the cost "bow Sakonoko or one of his Spells". The targeted-by-action family fits the trigger (Kota, Taishuu, Rokai), but the reaction window lists one option per reacting card and target: it carries no choice of which card pays the cost (a Performer or CostOption choice is offered for actions, not inside a reaction window).</t>
-        </is>
-      </c>
-      <c r="H370" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr"/>
+      <c r="H370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -15807,19 +15721,11 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G415" t="inlineStr">
-        <is>
-          <t>Kakita Kae: "After a Battle action targets Kae, you may discard the Imperial Favor to negate Kae's destruction, bowing, and movement from the action's effects" needs a targeted-action Reaction whose COST is discarding the Imperial Favor specifically (every existing negation Reaction with a Favor-adjacent cost -- Yoritomo Sakuma's own EitherOr -- pays Gold, never the Favor itself) that negates a bundle of THREE effect kinds (destroy/bow/move) on the reacting card alone, the same three-kind bundle Jinn-Kuen's own blanket negation already proves buildable, but keyed to a brand new cost verb the ActionCost/CostVerbs enums do not carry (Favor discard is currently only ever a printed ability COST via ActionNegation.cs's own hardcoded path, not offered as a Reaction's own payable option). Her plain "Battle: Move Kae home" is trivial in isolation.</t>
-        </is>
-      </c>
-      <c r="H415" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr"/>
+      <c r="H415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -19495,19 +19401,11 @@
       </c>
       <c r="F521" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G521" t="inlineStr">
-        <is>
-          <t>Needs Additional-Action grants scoped by required ability classification (Iaijutsu) and by a specific performer rather than by source card id (AdditionalActionGrant.ScopeCardIds cannot express the first), and "If you don't, bow him": a consequence when the additional action is not taken (a burst that is passed or forfeited).</t>
-        </is>
-      </c>
-      <c r="H521" t="inlineStr">
-        <is>
-          <t>ADDACT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr"/>
+      <c r="H521" t="inlineStr"/>
     </row>
     <row r="522">
       <c r="A522" t="inlineStr">
@@ -21189,19 +21087,11 @@
       </c>
       <c r="F570" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G570" t="inlineStr">
-        <is>
-          <t>Moto Rani - experienced: "Water Reaction: When paying for a Spell Equipping to Rani, remove a dead Personality in your discard pile from the game to reduce the Spell's Gold Cost by the Personality's Chi" needs a brand new hook into the Equip Gold-cost pipeline (EquipGoldCost/QuoteEquipGold, GoldQuotes.cs) that lets a Reaction played AT PAYMENT TIME apply a discount sized by a card removed from the game as its own cost -- every existing Equip discount (Katagi's wielder-dependent term, ClanEntryDiscount) is a fixed or static-condition term computed automatically, never a player-chosen action taken mid-quote. Her own "Water Tireless Battle: Straighten Rani. You may move her home" is trivial in isolation (Tireless/Absent plus an optional MoveHome), but is not wired alone.</t>
-        </is>
-      </c>
-      <c r="H570" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr"/>
+      <c r="H570" t="inlineStr"/>
     </row>
     <row r="571">
       <c r="A571" t="inlineStr">
@@ -23105,19 +22995,11 @@
       </c>
       <c r="F626" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G626" t="inlineStr">
-        <is>
-          <t>Unchanged: control transfer of an in-play Personality (deliberately not built) and a reversion 'after the next time this game this ability is announced' (a watch on a future announcement). NO LOCAL SCAN.</t>
-        </is>
-      </c>
-      <c r="H626" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr"/>
+      <c r="H626" t="inlineStr"/>
     </row>
     <row r="627">
       <c r="A627" t="inlineStr">
@@ -26981,19 +26863,11 @@
       </c>
       <c r="F738" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G738" t="inlineStr">
-        <is>
-          <t>Refreshed: "Destroy him before this turn ends" is now a scheduled delayed destruction (ScheduleDelayedEffect at DelayUntil.EndOfTurn); the blocker is still the in-play control change of an enemy Personality and his unit (TakeControl covers only cards brought from a discard pile) and the unit-wide Unique/Singular check. NO LOCAL SCAN.</t>
-        </is>
-      </c>
-      <c r="H738" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G738" t="inlineStr"/>
+      <c r="H738" t="inlineStr"/>
     </row>
     <row r="739">
       <c r="A739" t="inlineStr">
@@ -31385,19 +31259,11 @@
       </c>
       <c r="F866" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G866" t="inlineStr">
-        <is>
-          <t>Unchanged: control of another player's in-play Personality, and giving him back 'after the next time this game Sachina leaves play' (a watch on a card leaving play). NO LOCAL SCAN.</t>
-        </is>
-      </c>
-      <c r="H866" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G866" t="inlineStr"/>
+      <c r="H866" t="inlineStr"/>
     </row>
     <row r="867">
       <c r="A867" t="inlineStr">
@@ -31461,19 +31327,11 @@
       </c>
       <c r="F868" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G868" t="inlineStr">
-        <is>
-          <t>Needs an alternate Gold source that does not bow: "Reaction: When paying an action's Gold cost: Produce 3 Gold" (AlternateGoldSource and ConditionalProduction both bow the card when chosen as a source, and Singh's Reaction has no bow cost), limited to actions. His Battle half (pay Gold equal to an enemy card's Gold Cost: destroy it, the card without attachments) is TargetCurrent.</t>
-        </is>
-      </c>
-      <c r="H868" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G868" t="inlineStr"/>
+      <c r="H868" t="inlineStr"/>
     </row>
     <row r="869">
       <c r="A869" t="inlineStr">
@@ -31941,19 +31799,11 @@
       </c>
       <c r="F882" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G882" t="inlineStr">
-        <is>
-          <t>Zlkyt (re-verified). "Reaction: When paying a Gold cost, destroy your target Mine or Farm: Produce Gold equal to its base Gold Cost" does not fit the payment model: a payment is GameCommand.SourceIds, a flat list of card ids each producing GoldProduced(id) and then bowed (MatchEngine.Pay/ValidatePayment/PaymentOptionsExcluding, Producers() -- unbowed cards only). A Mine or Farm would need two different ways to be a source -- bowed for its printed production, or destroyed through Zlkyt for its base Gold Cost (legal even while it is bowed) -- and the use would be spent on Zlkyt, not on the source. AlternateGoldSource (GoldQuotes.cs, Yoritomo Sakuma) is only "bow THIS card: produce N"; Zlkyt needs a per-source payment mode carried by PaymentOption and the command, validated, quoted and paid (destroy, not bow) -- not a small extension.</t>
-        </is>
-      </c>
-      <c r="H882" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G882" t="inlineStr"/>
+      <c r="H882" t="inlineStr"/>
     </row>
     <row r="883">
       <c r="A883" t="inlineStr">
@@ -46839,19 +46689,11 @@
       </c>
       <c r="F1313" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1313" t="inlineStr">
-        <is>
-          <t>A copy: the created-copy primitive exists (CreatedCardSpec.CopyOfTarget, Mendon's ruling that a copy is a created copy of the target card), but this card copies all the abilities except those that copy abilities, and the created Personality is removed "when your next turn begins" (created cards leave with the battle or never; Events expire on ExpiresAtTurnsTaken). The Artisan performer bowed as its cost and the non-Unique target are ordinary categories.</t>
-        </is>
-      </c>
-      <c r="H1313" t="inlineStr">
-        <is>
-          <t>CREATE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1313" t="inlineStr"/>
+      <c r="H1313" t="inlineStr"/>
     </row>
     <row r="1314">
       <c r="A1314" t="inlineStr">
@@ -47119,19 +46961,11 @@
       </c>
       <c r="F1321" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1321" t="inlineStr">
-        <is>
-          <t>Ambiguous, and needs a cost that depends on the phase: "bow him unless this is the Attack Phase" is an exemption from the cost by phase (CostExempt knows a keyword, not a phase), together with "lose 3 Honor" and a target with lower Force than the performer. The reading of "to bow a target Personality" is Mendon's to confirm.</t>
-        </is>
-      </c>
-      <c r="H1321" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1321" t="inlineStr"/>
+      <c r="H1321" t="inlineStr"/>
     </row>
     <row r="1322">
       <c r="A1322" t="inlineStr">
@@ -47781,19 +47615,11 @@
       </c>
       <c r="F1340" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1340" t="inlineStr">
-        <is>
-          <t>Needs an additional Battle action scoped by ability classification ("a Limited or Open Recon ability" used as a Battle action) that must target the current battlefield's Province, with a draw after its resolution: AdditionalActionGrant is scoped by card ids, not classification.</t>
-        </is>
-      </c>
-      <c r="H1340" t="inlineStr">
-        <is>
-          <t>ADDACT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1340" t="inlineStr"/>
+      <c r="H1340" t="inlineStr"/>
     </row>
     <row r="1341">
       <c r="A1341" t="inlineStr">
@@ -47823,19 +47649,11 @@
       </c>
       <c r="F1341" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1341" t="inlineStr">
-        <is>
-          <t>Needs control of another player's Personality who is IN PLAY ("Take control of him"), deliberately not built (docs/decisions/2026-09-12-unique-singular-control-transfer.md: TakeControl exists for attachments and for cards taken from a discard or dead pile only), and "give control of him to his owner before the turn ends" (a timed return of control). Buildable now: the target ("enemy Personality whose unit's total Gold cost is 10 or lower" is TargetUnitTotal's shape), the dishonor, and destroying his Followers whose Honor Requirement he then fails (CardPersonalHonor against Follower.HonorRequirement).</t>
-        </is>
-      </c>
-      <c r="H1341" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1341" t="inlineStr"/>
+      <c r="H1341" t="inlineStr"/>
     </row>
     <row r="1342">
       <c r="A1342" t="inlineStr">
@@ -48205,19 +48023,11 @@
       </c>
       <c r="F1352" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1352" t="inlineStr">
-        <is>
-          <t>Re-evaluated for the Embers of War pass (issue #460): the attachment Transfer mechanic it was blocked on (AttachmentTransfers.cs, CanTransferTo/TransferAttachment) now exists (issue #458's Communion with Earth), so its Focus Effect ("you may transfer a Spell from your Personality in this duel to another of your Shugenja at the same location") is wirable on its own. Its Battle half is still blocked: "If you have not put cards into your hand this phase and you have attached a Spell this turn: Draw two cards" needs two live-tracked per-turn conditions neither built anywhere else -- a per-phase "cards put into hand" counter distinct from the existing per-action Draw effects, and a per-turn "attached a Spell" stamp (distinct from AttachGrantsKeyword's one-time entry effect) -- and the card's single printed ability id would need splitting to wire only the Focus Effect half, which the pass's own convention (a whole card, or none) avoids for a two-sentence ability like this.</t>
-        </is>
-      </c>
-      <c r="H1352" t="inlineStr">
-        <is>
-          <t>COUNTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1352" t="inlineStr"/>
+      <c r="H1352" t="inlineStr"/>
     </row>
     <row r="1353">
       <c r="A1353" t="inlineStr">
@@ -52181,19 +51991,11 @@
       </c>
       <c r="F1466" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1466" t="inlineStr">
-        <is>
-          <t>Needs "bow your two performing Nonhumans" as a cost: Slots with Performing exist, but a cost cannot name the cards of a performing slot (CostSubject knows the single performer), and "if your current army has more units than the current enemy army" is a comparison of unit counts.</t>
-        </is>
-      </c>
-      <c r="H1466" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1466" t="inlineStr"/>
+      <c r="H1466" t="inlineStr"/>
     </row>
     <row r="1467">
       <c r="A1467" t="inlineStr">
@@ -52579,19 +52381,11 @@
       </c>
       <c r="F1477" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1477" t="inlineStr">
-        <is>
-          <t>Needs two new pieces: a Focus Effect that lowers a DUEL WINNER's Gold Cost to 0 (Sandalwood Incense's own effect-key Focus Effect choice, issue #453 batch 5, only ever names a fixed set of EFFECTS, not a live Gold Cost override keyed to whichever card wins), and a "pay Gold equal to a unit's total Gold Cost minus 6, or straighten the unit instead" branch -- GoldCostRule.TargetUnitTotal(-2, floor: 0) (A Stain Cleansed) prices an action's own COST from a unit total, not a conditional in-effect choice between paying that amount for one outcome or taking a different outcome for free.</t>
-        </is>
-      </c>
-      <c r="H1477" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1477" t="inlineStr"/>
+      <c r="H1477" t="inlineStr"/>
     </row>
     <row r="1478">
       <c r="A1478" t="inlineStr">
@@ -54013,19 +53807,11 @@
       </c>
       <c r="F1518" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1518" t="inlineStr">
-        <is>
-          <t>Needs a per-phase "resolved two or more actions that put cards into his hand" counter read by a Reaction ("after an action resolves, if its player has resolved two or more actions which put cards into his hand this phase: he discards two cards") -- no existing primitive counts a PLAYER's own qualifying actions across a phase and re-checks the running total after each one (Advanced Intelligence's ReconStrategyActionsThisBattle, issue #453 batch 1, is the closest shape but counts a keyword-tagged action, not "put cards into hand" as a category of effect). The Battle half (move a performing Personality to an opposed current battlefield and straighten his unit) is Skipping the Puddle's own ordinary shape and separately wirable.</t>
-        </is>
-      </c>
-      <c r="H1518" t="inlineStr">
-        <is>
-          <t>COUNTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1518" t="inlineStr"/>
+      <c r="H1518" t="inlineStr"/>
     </row>
     <row r="1519">
       <c r="A1519" t="inlineStr">
@@ -56669,19 +56455,11 @@
       </c>
       <c r="F1594" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1594" t="inlineStr">
-        <is>
-          <t>Needs a tracked "has the enemy leader taken a Battle action during this battle" (novel state) and additional Battle actions granted "after this one" with "you will not take any other additional Battle actions this battle".</t>
-        </is>
-      </c>
-      <c r="H1594" t="inlineStr">
-        <is>
-          <t>ADDACT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1594" t="inlineStr"/>
+      <c r="H1594" t="inlineStr"/>
     </row>
     <row r="1595">
       <c r="A1595" t="inlineStr">
@@ -56745,19 +56523,11 @@
       </c>
       <c r="F1596" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1596" t="inlineStr">
-        <is>
-          <t>Needs control of your own Personality given to another player while he stays in play ("Give control of him to another player"), deliberately not built (docs/decisions/2026-09-12-unique-singular-control-transfer.md), and a granted TRAIT with its own Straighten-Phase decision ("After a Straighten Phase begins: Choose your bowed non-Ninja Personality. Negate his straightening this phase" -- a trait is not an ability, and GrantAbility grants abilities only; the straighten hold itself is StraightenHolds' StraightenPhaseEnds shape). The performer ("your performing unbowed Personality with the base Ninja keyword") is an ordinary keyword performer read from the printed keywords.</t>
-        </is>
-      </c>
-      <c r="H1596" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1596" t="inlineStr"/>
+      <c r="H1596" t="inlineStr"/>
     </row>
     <row r="1597">
       <c r="A1597" t="inlineStr">
@@ -61657,19 +61427,11 @@
       </c>
       <c r="F1736" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1736" t="inlineStr">
-        <is>
-          <t>Needs "an additional action appropriate to this phase": an additional action is only ever a Battle action, and this is also an Open one in the Action Phase. Straightening all your Rings and taking a Ring from the discard pile are ordinary effects.</t>
-        </is>
-      </c>
-      <c r="H1736" t="inlineStr">
-        <is>
-          <t>ADDACT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1736" t="inlineStr"/>
+      <c r="H1736" t="inlineStr"/>
     </row>
     <row r="1737">
       <c r="A1737" t="inlineStr">
@@ -63121,19 +62883,11 @@
       </c>
       <c r="F1778" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1778" t="inlineStr">
-        <is>
-          <t>Needs a Gold-Cost comparison Target category (same gap as oracle-l5r-24/6034): "destroy another player's target Personality whose unit has a total Gold Cost equal to or less than what you paid for this action" compares the chosen target's whole unit's printed Gold Cost total against the variable amount the acting player actually paid (a gold-star/variable cost, issue #416) -- no existing Target category reads a paid amount back against a unit's cost total. Also needs the Imperial Favor discard modeled as a first-class alternative COST (issue #337's CostOption family) rather than the ad hoc, hardcoded-ability-id shape every existing "discard the Imperial Favor" card uses today, since here it is one of two alternative ways to pay alongside "bow a Personality with 5+ Force."</t>
-        </is>
-      </c>
-      <c r="H1778" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1778" t="inlineStr"/>
+      <c r="H1778" t="inlineStr"/>
     </row>
     <row r="1779">
       <c r="A1779" t="inlineStr">
@@ -63231,19 +62985,11 @@
       </c>
       <c r="F1781" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1781" t="inlineStr">
-        <is>
-          <t>Needs the Imperial Favor discard as a first-class alternative COST (same modeling gap as oracle-l5r-8127): both of its abilities offer "discard the Imperial Favor" as an alternative to an ordinary cost (bowing the Stronghold, or bowing the performing Courtier) on the SAME action, which the engine's alternative-cost primitive (CostOption, issue #337) could express generically but which every existing "discard the Imperial Favor" card instead hardcodes as its own single fixed cost, never offered as a choice against another cost on the same ability. The enemy-Personality-bow half would otherwise be immediately wirable with the new enemy-personality-at-any-location Target category this pass added.</t>
-        </is>
-      </c>
-      <c r="H1781" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1781" t="inlineStr"/>
+      <c r="H1781" t="inlineStr"/>
     </row>
     <row r="1782">
       <c r="A1782" t="inlineStr">
@@ -69711,19 +69457,11 @@
       </c>
       <c r="F1969" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1969" t="inlineStr">
-        <is>
-          <t>Needs an alternate Gold source that does not bow: "Reaction: When paying a Gold Cost, produce 1 Gold (this can be used together with bowing this card to produce Gold)" while its printed ":bow: Produce 2 Gold" is an ordinary production (AlternateGoldSource bows the card).</t>
-        </is>
-      </c>
-      <c r="H1969" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1969" t="inlineStr"/>
+      <c r="H1969" t="inlineStr"/>
     </row>
     <row r="1970">
       <c r="A1970" t="inlineStr">
@@ -76591,19 +76329,11 @@
       </c>
       <c r="F2167" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2167" t="inlineStr">
-        <is>
-          <t>Needs two performing Personalities with different Clan alignments and a cost of bowing ONE of them (a chosen one of two performers): Slots with Performing exist, but a cost cannot name a chosen card of a performing slot. "Give your provinces +2 strength" is buildable (Genji).</t>
-        </is>
-      </c>
-      <c r="H2167" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2167" t="inlineStr"/>
+      <c r="H2167" t="inlineStr"/>
     </row>
     <row r="2168">
       <c r="A2168" t="inlineStr">
@@ -77328,7 +77058,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -77488,7 +77218,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -77508,7 +77238,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -77608,7 +77338,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -77708,7 +77438,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -77728,7 +77458,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Remaining-cards pass: inventory, art pack, decision doc and handoff for #503
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -514,14 +514,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C5" t="n">
         <v>51</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>90.2%</t>
+          <t>94.1%</t>
         </is>
       </c>
     </row>
@@ -532,14 +532,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>534</v>
+        <v>580</v>
       </c>
       <c r="C6" t="n">
         <v>830</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>64.3%</t>
+          <t>69.9%</t>
         </is>
       </c>
     </row>
@@ -550,14 +550,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C7" t="n">
         <v>133</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>80.5%</t>
+          <t>82.0%</t>
         </is>
       </c>
     </row>
@@ -568,14 +568,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C8" t="n">
         <v>133</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>42.1%</t>
+          <t>45.9%</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>43.6%</t>
+          <t>53.4%</t>
         </is>
       </c>
     </row>
@@ -604,14 +604,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>362</v>
+        <v>405</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>60.5%</t>
+          <t>67.7%</t>
         </is>
       </c>
     </row>
@@ -622,14 +622,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C11" t="n">
         <v>151</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>40.4%</t>
+          <t>41.7%</t>
         </is>
       </c>
     </row>
@@ -640,14 +640,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>34.6%</t>
+          <t>48.1%</t>
         </is>
       </c>
     </row>
@@ -658,14 +658,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C13" t="n">
         <v>37</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>51.4%</t>
+          <t>56.8%</t>
         </is>
       </c>
     </row>
@@ -712,14 +712,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1293</v>
+        <v>1419</v>
       </c>
       <c r="C16" t="n">
         <v>2183</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>59.2%</t>
+          <t>65.0%</t>
         </is>
       </c>
     </row>
@@ -985,265 +985,208 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Embers of War</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1</v>
+          <t>Twenty Festivals</t>
+        </is>
       </c>
       <c r="C25" t="n">
-        <v>27</v>
+        <v>15</v>
+      </c>
+      <c r="D25" t="n">
+        <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G25" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H25" t="n">
-        <v>1</v>
-      </c>
-      <c r="I25" t="n">
-        <v>4</v>
-      </c>
-      <c r="J25" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="M25" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Twenty Festivals</t>
+          <t>Ivory Edition</t>
         </is>
       </c>
       <c r="C26" t="n">
+        <v>6</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" t="n">
+        <v>5</v>
+      </c>
+      <c r="G26" t="n">
         <v>15</v>
       </c>
-      <c r="D26" t="n">
-        <v>3</v>
-      </c>
-      <c r="E26" t="n">
-        <v>6</v>
-      </c>
-      <c r="F26" t="n">
-        <v>7</v>
-      </c>
-      <c r="G26" t="n">
-        <v>21</v>
-      </c>
       <c r="H26" t="n">
-        <v>12</v>
+        <v>17</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>64</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Ivory Edition</t>
+          <t>Promotional–Celestial</t>
         </is>
       </c>
       <c r="C27" t="n">
+        <v>8</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" t="n">
+        <v>4</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" t="n">
+        <v>7</v>
+      </c>
+      <c r="H27" t="n">
         <v>6</v>
       </c>
-      <c r="D27" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" t="n">
+      <c r="I27" t="n">
         <v>2</v>
       </c>
-      <c r="F27" t="n">
-        <v>5</v>
-      </c>
-      <c r="G27" t="n">
-        <v>15</v>
-      </c>
-      <c r="H27" t="n">
-        <v>17</v>
-      </c>
-      <c r="I27" t="n">
-        <v>1</v>
+      <c r="J27" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" t="n">
+        <v>3</v>
       </c>
       <c r="M27" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Promotional–Celestial</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>8</v>
-      </c>
-      <c r="D28" t="n">
+          <t>War of Honor</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
         <v>2</v>
       </c>
-      <c r="E28" t="n">
-        <v>4</v>
-      </c>
-      <c r="F28" t="n">
-        <v>3</v>
-      </c>
       <c r="G28" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H28" t="n">
-        <v>6</v>
-      </c>
-      <c r="I28" t="n">
-        <v>2</v>
-      </c>
-      <c r="J28" t="n">
-        <v>3</v>
-      </c>
-      <c r="K28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Before the Dawn</t>
+          <t>The Shadow's Embrace</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>11</v>
-      </c>
-      <c r="D29" t="n">
         <v>2</v>
       </c>
       <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="n">
         <v>2</v>
       </c>
-      <c r="F29" t="n">
-        <v>4</v>
-      </c>
       <c r="G29" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="H29" t="n">
         <v>1</v>
       </c>
-      <c r="I29" t="n">
-        <v>3</v>
+      <c r="K29" t="n">
+        <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>36</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>The Shadow's Embrace</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
+          <t>Forgotten Legacy</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
         <v>1</v>
-      </c>
-      <c r="C30" t="n">
-        <v>4</v>
-      </c>
-      <c r="E30" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" t="n">
-        <v>2</v>
       </c>
       <c r="G30" t="n">
         <v>4</v>
       </c>
-      <c r="H30" t="n">
-        <v>1</v>
-      </c>
-      <c r="I30" t="n">
-        <v>1</v>
-      </c>
-      <c r="K30" t="n">
-        <v>1</v>
-      </c>
       <c r="M30" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>War of Honor</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>2</v>
-      </c>
-      <c r="G31" t="n">
-        <v>10</v>
+          <t>Celestial Edition</t>
+        </is>
       </c>
       <c r="H31" t="n">
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Seeds of Decay</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>4</v>
-      </c>
-      <c r="E32" t="n">
+          <t>Embers of War</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
         <v>1</v>
       </c>
-      <c r="F32" t="n">
+      <c r="M32" t="n">
         <v>1</v>
-      </c>
-      <c r="G32" t="n">
-        <v>3</v>
-      </c>
-      <c r="I32" t="n">
-        <v>3</v>
-      </c>
-      <c r="M32" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Forgotten Legacy</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>3</v>
-      </c>
-      <c r="G33" t="n">
-        <v>7</v>
+          <t>Emperor Edition</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Celestial Edition</t>
-        </is>
-      </c>
-      <c r="H34" t="n">
+          <t>Honor and Treachery</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
@@ -1253,10 +1196,10 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Emperor Edition</t>
-        </is>
-      </c>
-      <c r="K35" t="n">
+          <t>Words and Deeds</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
@@ -1264,85 +1207,46 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Honor and Treachery</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
-      <c r="M36" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Second City</t>
-        </is>
-      </c>
-      <c r="J37" t="n">
-        <v>1</v>
-      </c>
-      <c r="M37" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Words and Deeds</t>
-        </is>
-      </c>
-      <c r="G38" t="n">
-        <v>1</v>
-      </c>
-      <c r="M38" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>296</v>
-      </c>
-      <c r="D39" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="E39" s="2" t="n">
-        <v>77</v>
-      </c>
-      <c r="F39" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="G39" s="2" t="n">
-        <v>236</v>
-      </c>
-      <c r="H39" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="I39" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="J39" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="K39" s="2" t="n">
+      <c r="B36" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>193</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="J36" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="K36" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="L39" s="2" t="n">
+      <c r="L36" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M39" s="2" t="n">
-        <v>890</v>
+      <c r="M36" s="2" t="n">
+        <v>764</v>
       </c>
     </row>
   </sheetData>
@@ -2765,19 +2669,11 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>The New Foundries (Phoenix Stronghold): "Limited: Put a Spell from your hand face-up underneath this card" needs cards kept UNDER another card, which the engine has no zone for (Zone has no 'under a card' value; every card is in a deck, hand, discard pile, province, play or removed from the game), and the Battle action "discard a Spell from under this card: Either straighten one to three Shugenja at the current battlefield if the Spell is Air or Water, or Ranged 4 Attack if it is Earth or Fire, or draw a card if it is Void" pays with such a card and branches on its element. A new zone touches every view (MatchQueries.ViewCard, the client's card layout) and the other cards that read it (Agasha Kurou, oracle-l5r-9835: 'a target non-Unique Spell in your discard pile or under your Stronghold'); not wired whole.</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>ZONE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2841,19 +2737,11 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>The Plain of Glass: three separate gaps. (1) "You do not lose Honor from Spider Clan and Fate cards you own" is a two-condition (clan-OR-card-type) Honor-loss immunity, broader than any existing single-condition one (The Castle of Order's own keyword-keyed immunity is the closest shape, narrower). (2) "You may use the rulebook Conquest ability twice per turn during the same battle" needs the engine's own Conquest resolution (MatchState.PendingConqueror) restructured from a single per-battle choice slot into a per-player use counter, since nothing today enforces or could raise a per-turn Conquest cap. (3) "Equipping Followers is a Battle/Limited ability for you" changes WHEN an entire category of action (Equip) may be taken for this player, not merely who or what it targets -- no primitive grants a new timing to an existing global action type. Left unwired whole; the first two are individually small, the third is the disproportionate one.</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>RULEBOOK</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3975,19 +3863,11 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>Akodo Tamisu (re-verified, note otherwise unchanged from the Lion Clan Personality review): her entry trait -- "discard all your other Sensei Personalities" -- is now a bare data flag (discard-other-sensei/HasSenseiEntryEffect, built since that review) and no longer any part of her blocker. What remains is her second sentence, "After your Tactical, Bushido Virtue, or Terrain action resolves: Give a Lion Clan Personality +1F": the after-action-resolved Reaction window (issue #437) and ActionCarriesKeyword's own source-card-keyword fallback (issue #321) together read the three-way action-keyword check (Matsu Rika's own self-buff precedent), but Rika's own case is a mandatory SELF bonus with no target choice at all -- Tamisu's own wording is a mandatory Reaction that still asks its controller to CHOOSE a target Lion Clan Personality (which need not be Tamisu). No mandatory (non-"may") Reaction with its own target choice exists yet; every mandatory Reaction built so far (EntryHonorLoss, Destined's draw, DiscardOtherSensei) targets nothing, and every targeted Reaction built so far is optional. Needs that one shape.</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>SMALL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5279,19 +5159,11 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>Asako Kikugoro. "Reaction: After your Ring or Henshin (including Kikugoro) enters play or overlays: Look at the top two cards of your Dynasty deck. You may put one of them at the bottom of the deck" -- the LOOK itself is already a built spec verbatim (LookCatalog.TrainingDynasty, a fixture built ahead of a published card needing it: own Dynasty deck, two cards, one may go to the bottom). What's missing is the TRIGGER: no Reaction window opens on "a Ring or Henshin entering play or overlaying" specifically (Ring recruitment is its own -recruit ability path, not a general entry event other cards' Reactions can watch; "overlays" -- an Experienced Henshin replacing its own base printing -- has no watched event either). Needs a Ring/Henshin entry-or-overlay Reaction trigger; the look that follows it is otherwise ready to wire the moment that trigger exists.</t>
-        </is>
-      </c>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5355,19 +5227,11 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>Asako Megu. "Battle: Target an enemy Personality: Bow him. You may target and straighten a Personality. If the enemy Personality is Kolat, Ninja, or Shadowlands, gain 2 Honor" is two independent target choices (a required enemy bow, an optional second straighten of anyone) on one action -- the Slots shape (Akodo Tezuka/Utoro's own two-slot pattern) covers exactly this, with the second slot's count 0-1 for the "You may" wording. The conditional Honor gain reads the bowed target's own Clan alignment or printed keyword (TargetStatus, Bayushi Tenzan's own IfTarget-adjacent Kolat/Ninja/Shadowlands set already exists as a term elsewhere in this batch). Not wired this pass for lack of remaining implementation time, not a genuine engine gap.</t>
-        </is>
-      </c>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -6383,19 +6247,11 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G146" t="inlineStr">
-        <is>
-          <t>Bayushi Kazutoshi - Experienced. His Sensei entry trait is a bare discard-other-sensei flag now (built). The card's actual identity is its always-on static clause: "Other players' Personalities in and out of play have their Honor Requirements increased by 10, and they may pay 2 additional Gold when paying for Personalities with their Clan Alignment to ignore their Honor Requirements." QuotePurchase already supports a FLAT, unconditional Honor Requirement waiver keyed to one Clan (ignoreHonorRequirementIfPersonalityClan, Shinden Shorai's own shape) but nothing (a) raises the effective HonorRequirement value read everywhere a card's requirement matters (in play AND in a province/hand/deck, per the printed "in and out of play"), or (b) makes that waiver a PAID option (2 extra Gold) rather than free, or (c) scopes it to "cards sharing the affected player's own Clan Alignment" rather than one fixed clan. All three are new, and together are a controller-wide purchase-pricing system out of proportion for one card.</t>
-        </is>
-      </c>
-      <c r="H146" t="inlineStr">
-        <is>
-          <t>STAT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -6770,7 +6626,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Needs a "peek the top card of a deck, branch on its type, and either attach it in place (paying costs) or grant an additional action to play it, else leave it on top" primitive -- LookSpec only covers look-then-discard/keep/reorder shapes, not a type-conditional attach-or-grant off a peeked (not drawn) card.</t>
+          <t>Bayushi Nitoshi - inexperienced (Honor and Treachery; the scan: "Battle/Limited: Look at the top card of your Fate deck. If it is an attachment, you may attach it to one of your Personalities at Nitoshi's location, paying all costs. If it is a Strategy, you may take an additional action to play it (if legal)."). Re-verified after issue #503: the look (DeckLook), the Battle/Limited split (two ids sharing one use, Kakita Tadanobu's shape) and a card-scoped additional-action grant exist, and the attach half is buildable as a mid-resolution attach with payment (Versatile Farm's ChoosePayment stage, AttachAction's RequireAttachable). Still missing: PLAYING A CARD FROM THE TOP OF THE FATE DECK. Every play path assumes the source Strategy is in the hand or (Discipline, Bofana/Tezuka grants) a discard pile: AbilitySourceZoneAllows' Strategy branch and QueryActions' source list (FateDeck cards are never candidates), the Terrain "playStrategy" command (hand only), SpendHandPlayedCard / the CompleteAbilityResolution and CompleteNegatedAction tails (they discard from the hand; a card left in PlayerState.FateDeck would be duplicated), PaymentSubjectFor (Play vs Action), and the grant would have to be RESTRICTED to that card (a Tag rule in RequireRestrictedBurstAllows / PerformerGrantMatches, which today ignore ScopeCardIds). The client view also has no way to show an action on a card that sits face-down in a deck. Suggested build: a FromDeckTop grant (AdditionalActionGrant flag) mirroring DiscardPlayGrant through those five places, the card leaving the deck list as the action is announced.</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -6807,19 +6663,11 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>Bayushi Nomen - Experienced 2. "Political Battle: Even if Nomen is not at the current battlefield, bow her and target a Personality: Move him home" is very likely wirable now: SourceUnitMayBeAway ("even if this unit is not at the current battlefield", Taming the Beast/Rage of the Spirits' own shape) plus MoveHome (now a fully generic helper, read live by IrezuMove/gold-and-steel-bow-move/fear-me-move/dispensing-justice-destroy's own "else" branch, not only Incapacitated/Block's battle-resolution-specific case) and ActionCost.BowPerformer for her own bow. "Political" is a plain ActionKeywords tag (Favor's own "Political Battle" precedent). Not wired this pass for lack of remaining implementation time, not a genuine engine gap.</t>
-        </is>
-      </c>
-      <c r="H158" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -7053,19 +6901,11 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G165" t="inlineStr">
-        <is>
-          <t>Bayushi Tenzan. "Battle/Limited: Target a Personality, or one or two Personalities if you control a Courtier ... Give each target -3F. If this is the Combat Segment, dishonor them" needs a target COUNT that is itself conditional on board state (whether the controller has a Courtier) -- TargetSlots.cs's own multi-slot shape (issue #336) gives every slot a fixed count set at authoring time, not one chosen per-resolution off a live keyword check. "If this is the Combat Segment" (distinguishing the card's own Battle-timing use from its Limited-timing use, both printed on one line) is a live phase-and-timing read at resolution, not built as a per-ability branch. "You may target a Shadowlands Personality" (an exemption from an otherwise-implied own-side-only target, letting an enemy Shadowlands card be chosen too) layers a third gap on top. Needs a conditional slot-count primitive before this is wirable at all.</t>
-        </is>
-      </c>
-      <c r="H165" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr"/>
+      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -7711,19 +7551,11 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G184" t="inlineStr">
-        <is>
-          <t>Daidoji Akeha. "Reaction: After your Recon action from a Strategy resolves: Draw a card" reads the same Recon-action-from-Strategy watch Narizane's own "Recon actions you have taken this turn" counter already tracks in this same batch (Daidoji Narizane, oracle-l5r-1663, below) -- a live per-turn count exists, so "the Recon action just resolved and it came from a Strategy" only needs the AfterResolution facts to also record the resolved action's own Strategy-or-not provenance, which they do not yet (AfterResolution tracks destruction/province facts, not a resolved action's own card-type source). "Recon Limited: Discard a card: Search your Fate deck for a non-Unique card with a Recon ability, show it, put it in your hand" is directly wirable now (DeckSearch.cs's SearchCriteria already supports a keyword/ability-tag search with a Unique exclusion, Daidoji Yuki's own precedent). Not wired this pass for the Reaction half's one remaining provenance gap.</t>
-        </is>
-      </c>
-      <c r="H184" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -9049,19 +8881,11 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G223" t="inlineStr">
-        <is>
-          <t>Needs a start-of-turn trait for a card in play: after the Provinces are revealed and their triggered traits have resolved, its controller may remove a Dark Virtue in their hand or discard pile from the game, and if none is removed Miki is destroyed. The Events Phase reveal (ContinueEventsReveal) resolves the Events and Regions in Provinces and the ongoing Events only; a card in play has no such trigger, and the optional-choice-else-destroy needs a decision in the middle of that reveal, as Harsh Choices does.</t>
-        </is>
-      </c>
-      <c r="H223" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr"/>
+      <c r="H223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -9363,19 +9187,11 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G232" t="inlineStr">
-        <is>
-          <t>Daigotsu Susaiken. His Sensei entry trait is a bare discard-other-sensei flag now (built; his Effect field is otherwise free, so "discard-other-sensei" itself, not a HasSenseiEntryEffect addition). "Once per turn, you may refill one of your provinces face-up" is close to built but not quite: the catalogue's only face-up refill is entry-provenance-tied (a card's OWN province, refilled face-up because IT was the one destroyed/discarded from there -- the gap oracle-l5r-10639 names), where Susaiken's is untargeted-provenance -- the controller freely CHOOSES which of their own (already-empty) provinces to refill face-up, once a turn. Needs a plain "choose one of your own empty provinces; refill it face-up" action, distinct from both the existing face-down Invest-style refill and the entry-tied one.</t>
-        </is>
-      </c>
-      <c r="H232" t="inlineStr">
-        <is>
-          <t>PROVINCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr"/>
+      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -9439,19 +9255,11 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G234" t="inlineStr">
-        <is>
-          <t>Daigotsu Tenbatsu. "Reaction: After engaging at Tenbatsu's battlefield: Look at the top three cards of your Fate deck. Put them back in any order. You may discard a Dark Virtue; if you did, draw a card" -- the Engage window itself now exists (issue #310, Recon Reaction/ClaimFirstOpportunity), and the look-3-reorder half is PublicRecords' own LookSpec shape verbatim. What is missing is triggering a Reaction off "engaging at THIS card's own battlefield" as a general watched event (today's Engage consumers are all first-action CLAIMS made during the window, not a Reaction fired by the window opening) and a conditional discard-a-Dark-Virtue-then-draw appended after a look resolves (no look spec composes with a following conditional discard/draw of a different, keyword-filtered card from hand). Two gaps.</t>
-        </is>
-      </c>
-      <c r="H234" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr"/>
+      <c r="H234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -9549,19 +9357,11 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G237" t="inlineStr">
-        <is>
-          <t>Needs three things: (1) a Battle action taken by a DEAD card from the dead pile ("If Yutaka is dead ... Bring him into play at the current battlefield"): AbilityDefinition.FromDiscard admits a source in Zone.FateDiscard/DynastyDiscard only, never Zone.Dead, and no recruit cost basis prices the SOURCE's own recruit (GoldCostRule.TargetRecruit prices a target); (2) "paying 3 less Gold if you have taken a Dark Virtue action this phase": no per-player record of the action keywords taken this phase (AfterOwnActionTraits tracks per-card stat bonuses, not a phase flag); (3) "Yutaka may not perform Bushido Virtue actions" is a performer-side action-keyword ban -- a small check in RequireCanPerform (ActionLock.cs) on ActionCarriesKeyword(ability, source, "Bushido Virtue") keyed by his Effect, not built because the card cannot be wired whole. "If he would be opposed" is Army(1 - player, current battlefield).Any(). His entry Honor loss is EntryHonorLoss 1.</t>
-        </is>
-      </c>
-      <c r="H237" t="inlineStr">
-        <is>
-          <t>ZONE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr"/>
+      <c r="H237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -11067,19 +10867,11 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G282" t="inlineStr">
-        <is>
-          <t>Gozaru no Oni. His entry Honor loss is EntryHonorLoss 5 (built). "After Gozaru is destroyed: It becomes discarded (not dead)" needs a per-card destruction-outcome override (every DestroyUnits call sends a card to Zone.Dead unconditionally; nothing reroutes one card's own destruction to Zone.DynastyDiscard/FateDiscard instead) -- a small, plausible primitive, not attempted this pass. "Battle: Target one or two enemy cards: Bow them. If you only targeted one card, destroy it" needs a target-count-dependent EFFECT (not just a count-dependent bow, which TargetSlots already supports fine, but the destroy half firing only when exactly one of the two optional slots was actually used) -- no ability reads "how many of my own optional target slots were filled" today. Two gaps, neither large alone; not attempted this pass.</t>
-        </is>
-      </c>
-      <c r="H282" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr"/>
+      <c r="H282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -11305,19 +11097,11 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G289" t="inlineStr">
-        <is>
-          <t>Hida Bakishi. "Reaction: After an action resolves that Bakishi performed and that destroyed a card at the current battlefield: The next time (this turn) another player's action targets Bakishi, negate its effects on him" is very likely wirable now off the destruction shield generalized in the Seeds of Decay pass (CardInstance.DestructionShieldTurn, Megumi's Guidance's own "outlives one action" shield) combined with AfterResolution's own DestroyedEnemyUnits/performer facts to gate the grant on Bakishi himself having performed the destroying action. Not wired this pass for lack of remaining implementation time, not a genuine engine gap.</t>
-        </is>
-      </c>
-      <c r="H289" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr"/>
+      <c r="H289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -11449,19 +11233,11 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G293" t="inlineStr">
-        <is>
-          <t>Needs a before-action Reaction that is not tied to a target ("before the resolution of another player's action, if Fujita is at the current battlefield") that negates the destruction of every Follower of yours the action would destroy. NegatedEffects entries are per known card, and DestroyUnits discards a destroyed unit's attachments unconditionally, so whether a Follower lost with its destroyed host counts as "destroyed from the action's effects", and what negating it would leave attached to a dead host, is unsettled: a reading for Mendon.</t>
-        </is>
-      </c>
-      <c r="H293" t="inlineStr">
-        <is>
-          <t>TRIG-ANN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr"/>
+      <c r="H293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -11865,19 +11641,11 @@
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G305" t="inlineStr">
-        <is>
-          <t>Hida Osote. His Sensei entry trait needs a HasSenseiEntryEffect addition (his Effect field is taken by his own static trait below, the Zansho/Aimi/Nagi/Nobukatsu convention). "After the first time each turn another player's action targets your Crab Clan Personality at Osote's location, the player discards a card after the action ends" is very likely wirable now off the after-action-resolved Reaction window (issue #437, the same window Akodo Tamisu's own third clause above needs) plus a per-turn once-only stamp (the established once-per-turn-per-trigger convention, e.g. Hida Kaiji's own automatic negation). Not wired this pass for lack of remaining implementation time, not a genuine engine gap.</t>
-        </is>
-      </c>
-      <c r="H305" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr"/>
+      <c r="H305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -12009,19 +11777,11 @@
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G309" t="inlineStr">
-        <is>
-          <t>Needs the Province a card came from: "After Yamadera enters play from a province: Refill it face-up". A purchased card leaves its Province and the Province is refilled face-down at once (Refill), and nothing records where a card in play entered from. Her Battle action (an enemy card with lower Force: bow it) is buildable on its own.</t>
-        </is>
-      </c>
-      <c r="H309" t="inlineStr">
-        <is>
-          <t>PROVENANCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr"/>
+      <c r="H309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -12829,19 +12589,11 @@
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G333" t="inlineStr">
-        <is>
-          <t>Needs a Reaction fired when you announce a Tactical action (not after it resolves), even if Ayumu is bowed: reactions to an own action exist only after resolution (AfterOwnActionTraits, OpenBattleActionReactionWindow) or to another player's action (before-action, targeted-by-action).</t>
-        </is>
-      </c>
-      <c r="H333" t="inlineStr">
-        <is>
-          <t>TRIG-ANN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr"/>
+      <c r="H333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -12909,19 +12661,11 @@
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G335" t="inlineStr">
-        <is>
-          <t>Ikoma Hakige (re-verified; the Honor and Treachery pass's own note -- "needs generalization of the existing move-home primitives" -- is now STALE). MoveHome is a fully generic "move this targeted Personality home" helper since that pass (read directly by IrezuMove, gold-and-steel-bow-move, fear-me-move and dispensing-justice-destroy's own "else" branch, none of them battle-resolution-specific), and CardPersonalHonor is already read live for a Force-equal-to-Personal-Honor formula elsewhere (strength-of-the-divine-honor). "Target another Personality: Move him home or give him a Force bonus equal to his Personal Honor" is very likely wirable now as two abilities sharing one UsageKey (Bayushi Chikata's own bow-or-straighten toggle shape), targeting the existing "personality" category with a same-as-source Require rather than a new Performer/Target category. Not wired this pass for lack of remaining implementation time -- no genuine engine gap remains.</t>
-        </is>
-      </c>
-      <c r="H335" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr"/>
+      <c r="H335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -13235,19 +12979,11 @@
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G344" t="inlineStr">
-        <is>
-          <t>Needs two independent targets for an attach: a Follower in your hand and a Personality of yours to receive it. AttachSpec takes its wielder from the source or the chosen performer (AttachWielder) and its card from a single target; Slots (issue #336) give two targets but an ability cannot both carry Slots and read the attached card from one of them. The hand pile itself is built (AttachPile.OwnHand: Ebara, Hailung).</t>
-        </is>
-      </c>
-      <c r="H344" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr"/>
+      <c r="H344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -13481,19 +13217,11 @@
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G351" t="inlineStr">
-        <is>
-          <t>Ikoma Yamahatsu (re-verified; the Honor and Treachery pass's own note stands). "Battle: Ranged 4 Attack" is directly wirable (Akodo Chiyo's own fixed-strength shape, this batch's own takayasu-attack/onizuka-attack precedent); still blocked by its own passive, "While you control a Terrain, your Ranged Attacks have +1 strength" -- a global, controller-wide modifier reaching EVERY Ranged Attack the controller makes (not just this card's own), distinct from every existing conditional Attack-strength term (all keyed to the performing card's own abilityId in the AttackStrength switch, none scanning the controller's whole card pool for a passive add-on). Not built.</t>
-        </is>
-      </c>
-      <c r="H351" t="inlineStr">
-        <is>
-          <t>STAT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr"/>
+      <c r="H351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -13765,19 +13493,11 @@
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G359" t="inlineStr">
-        <is>
-          <t>Isawa Koiso. "Limited: Bow Koiso, destroy your Shugenja with the base Fire keyword, discard a card, and target a non-Unique card without attachments in a unit: Destroy it" is a four-part cost (bow self, destroy a specific own card, discard a hand card) gating a destroy effect with a Unique exclusion on the target -- individually ordinary pieces (BowSource, a DestroyToken-adjacent own-card-destruction cost, a hand discard cost, any-unit-card filtered by !Unique) that have not yet been combined into one ability's Costs array together with a Unique-excluding target filter. "Battle: Target a card without attachments in a unit: Destroy it" is directly wirable now (any-unit-card, filtered to !HasAttachments). Not wired this pass for lack of remaining implementation time on the Limited half's combined-cost shape.</t>
-        </is>
-      </c>
-      <c r="H359" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr"/>
+      <c r="H359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -13875,19 +13595,11 @@
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G362" t="inlineStr">
-        <is>
-          <t>Isawa Mina. "Battle: Target an attachment or token at the current battlefield: Destroy it. If this destroyed a card or token, give Mina two +1F Fire tokens" needs a target category spanning BOTH attachments (ordinary CardInstance targets) and TOKENS (a different, non-CardInstance kind of game object with no Target category of its own today -- every existing token interaction, e.g. mitsu-fire-attack's own token destruction, is a COST the performer pays on their own card, never a Battle ability's TARGET choice on an opponent's or any card's token). The token-grant half (CreateToken, called twice) is already built and used elsewhere (meiyu-fire-tokens). Needs a target-a-token primitive.</t>
-        </is>
-      </c>
-      <c r="H362" t="inlineStr">
-        <is>
-          <t>TOKEN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr"/>
+      <c r="H362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -14189,19 +13901,11 @@
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G371" t="inlineStr">
-        <is>
-          <t>Isawa Sanetomo. His Sensei entry trait needs a HasSenseiEntryEffect addition (his Effect field is taken by his own static trait below). "Once per battle, one of your Phoenix Clan Shugenja may perform the Equip Battle action even if bowed and even if unopposed" is very likely wirable now: "even if bowed" is the established hardcoded bowed-source exemption list (CardAbilities.cs) an ability id is simply added to, and "even if unopposed" is a printed-text exemption from the ordinary Battle-presence-of-an-opposing-army check already read elsewhere per-ability. The remaining piece is scoping BOTH exemptions to a once-per-battle CHOICE of performer (any of the controller's Phoenix Shugenja) rather than the card's own source, which the Equip Battle action does not currently expose as a chooseable performer at all. Not wired this pass for lack of remaining implementation time.</t>
-        </is>
-      </c>
-      <c r="H371" t="inlineStr">
-        <is>
-          <t>SMALL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr"/>
+      <c r="H371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -14469,19 +14173,11 @@
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G379" t="inlineStr">
-        <is>
-          <t>Itoku - Experienced. "Itoku has +1F while a Lion Clan player controls him" is directly wirable (Player(card.OwnerId).Clan == "Lion", a one-line CardForce term). "Reaction: After an action resolves which bowed your non-Void Ring: Straighten it. You may use each of its abilities an additional time this turn" is very likely wirable now off RefreshBattleAbilities (Shiba Tsukimi's own "may use its abilities a second time this turn" refresh, Honor and Treachery pass, already generalized past one card) applied to a Ring instead of a unit card, triggered off an after-action-resolved bow watch on the controller's own Ring. Not wired this pass for lack of remaining implementation time, not a genuine engine gap.</t>
-        </is>
-      </c>
-      <c r="H379" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr"/>
+      <c r="H379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -15297,19 +14993,11 @@
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G403" t="inlineStr">
-        <is>
-          <t>Needs a Force bonus that lasts "while he is in an army and while all Personalities in that army are Siege": a conditional duration re-judged from the army's composition. Force bonuses from actions are fixed amounts for the turn, and static conditional ones are Effect-keyed to their own card.</t>
-        </is>
-      </c>
-      <c r="H403" t="inlineStr">
-        <is>
-          <t>STAT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr"/>
+      <c r="H403" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -15543,19 +15231,11 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G410" t="inlineStr">
-        <is>
-          <t>Kakita Gonji: "Before you focus: Once per duel, instead of focusing that time, you may give your Crane Clan Personality in the duel +4 to his duel stat until the duel ends" needs a REPLACEMENT for the Focus decision itself, inside the duel's own Focusing stage (Dueling.cs's ResolveDuelCommand only ever accepts "focus" or "strike" from the turn player; there is no alternative-to-focusing effect a card can offer there, unlike a Focus EFFECT, which applies only after the duel already ends). His Sensei-entry trait (discard-other-sensei) is trivial and could ship alone, but this pass follows the established convention of wiring a card whole or not at all.</t>
-        </is>
-      </c>
-      <c r="H410" t="inlineStr">
-        <is>
-          <t>DUEL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr"/>
+      <c r="H410" t="inlineStr"/>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -15789,19 +15469,11 @@
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G417" t="inlineStr">
-        <is>
-          <t>Kakita Kenta: "Iaijutsu Reaction: After an action resolves during which Kenta won a duel, target a dishonorable enemy Personality at the current battlefield: Move him home" is the first own-won-duel Reaction with a real Target. DuelPresentation.cs's QueryDuelActions -- the SEPARATE listing path every duelWonReaction/duelReaction window uses instead of the ordinary QueryActions/AddReaction machinery -- is hardcoded to untargeted commands only ("All currently supported duel reactions are untargeted", its own comment; every existing own-won-duel/own-personality-won-duel card, Daisuke/Horume/Jakuei/Maratai, prints Target "none"). Extending that listing to enumerate legal targets for a targeted duel-won Reaction is the one piece needed; not attempted here given how heavily the live duel system is already tested.</t>
-        </is>
-      </c>
-      <c r="H417" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr"/>
+      <c r="H417" t="inlineStr"/>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -15899,19 +15571,11 @@
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G420" t="inlineStr">
-        <is>
-          <t>Needs "Your Stronghold's abilities have Tireless": Tireless (usable while bowed) is a hard-coded list of ability ids (Tsudoken, Dairuko, Red Crane Dojo), so it cannot be granted to another card's abilities. Its Favor half (discard the Imperial Favor: give each of your Provinces +2 strength) is a Favor ability like Shunya's.</t>
-        </is>
-      </c>
-      <c r="H420" t="inlineStr">
-        <is>
-          <t>GRANT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr"/>
+      <c r="H420" t="inlineStr"/>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -15946,7 +15610,7 @@
       </c>
       <c r="G421" t="inlineStr">
         <is>
-          <t>Kakita Saki: SCAN UNAVAILABLE for the card she creates. "Limited: Target your Personality: Create a +2F Armor Item with the trait, 'Melee and Ranged Attacks targeting this Personality have -3 strength' and attach it to him." Mechanically wirable: an AbilityDefinition.Creates spec (CardType.Item, Force 2, Chi 0, Keywords ["Armor"], the trait as AbilityText) attached to the targeted own Personality (the Creates/host shape of Kaiu Armor's creator), plus one static Attack-strength term keyed on the created Item's Effect (EffectiveAttackStrength: -3 against its wielder for a Melee or Ranged Attack, the Destrier/Singh Remnants defensive-strength shape). Blocked only because CreatedCards.Resolve needs a published CreatedOnly Proxy scan that fits the spec, and none exists: no Oracle record or art-pack scan is a +2F Armor with that trait (Kaiu Armor, oracle-l5r-10007, is +1F with no text). Wire it once a verified Proxy scan is available.</t>
+          <t>Kakita Saki (issue #503, pass group P6, re-checked): her own scan is now local (catalogue WebP working copy, sha256-verified), so the card itself could be packaged; still blocked only by the card she CREATES. "Limited: Target your Personality: Create a +2F Armor Item with the trait, 'Melee and Ranged Attacks targeting this Personality have -3 strength' and attach it to him." is buildable (a CreatedCardSpec(Item, Force 2, Chi 0, [Armor], AbilityText) attached to the target, plus a -3 Attack-strength term keyed on the created Item for a Melee or Ranged Attack targeting its wielder), but CreatedCards.Resolve needs a published CreatedOnly Proxy scan that fits, and none exists anywhere local (not in the repository, l5r-s3, l5r-emperor or either catalogue WebP pack; Kaiu Armor oracle-l5r-10007 is +1F with no text). docs/requests/created-card-scans-needed.md row B4 (assets/requested-scans/saki-armor.jpg) is still unticked.</t>
         </is>
       </c>
       <c r="H421" t="inlineStr">
@@ -17435,19 +17099,11 @@
       </c>
       <c r="F464" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G464" t="inlineStr">
-        <is>
-          <t>Kitsune Haruki: "Reaction: After Haruki enters play: Create a 2F/2C/3PH Mantis Clan · Nonhuman · Deer · Spirit Personality with the ability, 'Limited: If another player has higher Family Honor than you: Gain 2 Honor'" needs its own token PUBLISHED as a CreatedOnly scan first -- CreatedCards.Resolve only ever matches against CardDefinition.CreatedOnly cards already in the catalogue (Kitsu Akai's own Lion Ancestor, oracle-l5r-9785, is the precedent), and no such Deer token exists yet. Its own real printed proxy card, "Haruki's Deer" (oracle-l5r-9999, same set, type Proxy, text verified to match verbatim), has a receipt but no downloaded scan; publishing it as a CreatedOnly Personality (overriding its oracle "Proxy" type field, which the CardType enum does not carry) is a small follow-up, not attempted in this batch to avoid mis-publishing a new card under time pressure.</t>
-        </is>
-      </c>
-      <c r="H464" t="inlineStr">
-        <is>
-          <t>SCAN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr"/>
+      <c r="H464" t="inlineStr"/>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -17482,7 +17138,7 @@
       </c>
       <c r="G465" t="inlineStr">
         <is>
-          <t>Kitsune Hisano: its only printed ability is "Reaction: Once per game, after Hisano enters play: Create a 2F/2C/3PH Mantis Clan - Nonhuman - Fox - Spirit - Unique Personality with the ability, 'Battle: Target an enemy attacking Personality: Move him home.'" Mechanically this is Kitsune Ohsuki's own entering-play Creates Reaction plus AbilityDefinition.OncePerGame, and the created Guide's ability is favor-battle's own target and move without the Favor discard (target "enemy-attacking", MoveHome). Blocked only because the created card has no scan: CreatedCards.Resolve needs a published CreatedOnly Proxy scan that fits the spec, and Hisano's Guide (oracle-l5r-10020) has none available (see its own note). Wire both together once that scan is fetched.</t>
+          <t>Kitsune Hisano - exp (issue #503, P6, re-checked): her own scan is local; blocked only by her created card. The Reaction is Kitsune Ohsuki's entering-play Creates shape with OncePerGame, and the created Guide's 'Battle: Target an enemy attacking Personality: Move him home.' is a plain target-and-move-home; but the Proxy Hisano's Guide (oracle-l5r-10020: 2F/2C/3PH Unique Mantis Clan Nonhuman Fox Spirit) has only a receipt (no working_copy, not in either catalogue WebP pack, not in l5r-s3 or l5r-emperor), and downloading is not allowed in this pass. Gina's Fox (oracle-l5r-10005) fits the stats but is not Unique and prints a different ability, so it may not stand in (Mendon's near-miss ruling). Wire both together once the Guide's scan is fetched and published CreatedOnly.</t>
         </is>
       </c>
       <c r="H465" t="inlineStr">
@@ -17524,7 +17180,7 @@
       </c>
       <c r="G466" t="inlineStr">
         <is>
-          <t>Kitsune Kichi. NO SCAN FOR ITS CREATED CARD: "Reaction: After Kichi enters play: Create a 3F/2C/3PH Mantis Clan • Nonhuman • Badger • Spirit Personality with the ability, 'Battle: Target an enemy Personality: Reduce his Force to 0.'" -- CreatedCards.Resolve (CreatedCards.cs) instantiates a published created-only Proxy scan, and no Badger Proxy exists (the published created Personalities are the Lion Ancestor, Ohsuki's Sparrow, Tokoru's Bear, Haruki's Deer, Merihiko's Swarm and the rest listed by CreatedCards.Scans; no catalogue under content/oracle carries a Proxy for Kichi's Badger either), so neither Kichi nor his Badger can be published. Mechanically wirable once the Proxy scan is supplied: Kitsune Tokoru's own shape (an own-enters-play Reaction with Creates: Personality 3F/2C/3PH [Mantis Clan, Nonhuman, Badger, Spirit]) and, on the Proxy, Weak Poison's reduce-to-0 (a -CardForce Force penalty) on an enemy-personality target.</t>
+          <t>Kitsune Kichi (issue #503, P6, re-checked): his own scan is local; blocked only by the Badger he creates (3F/2C/3PH Mantis Clan Nonhuman Badger Spirit, 'Battle: Target an enemy Personality: Reduce his Force to 0.'). No Proxy scan exists for it in any local source (no Oracle Proxy record either); docs/requests/created-card-scans-needed.md row B5 (kichi-badger-a.jpg) is still unticked. Mechanically Kitsune Tokoru's entering-play Creates Reaction plus A Weak Poison's Force-to-0 on the created card.</t>
         </is>
       </c>
       <c r="H466" t="inlineStr">
@@ -17969,19 +17625,11 @@
       </c>
       <c r="F479" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G479" t="inlineStr">
-        <is>
-          <t>Kuni Renyu. "...If he did not choose this, create a province with a base strength of 4 to the left of your leftmost province" has no primitive: nothing creates a province at all, and one to the LEFT of the leftmost would renumber the whole row -- ProvinceState.Index is positional (MatchEngine.AdjacentProvinces reads Provinces[i] by index; CardInstance.ProvinceIndex, CurrentBattleProvince, UnresolvedBattlefields, Regions and attack assignments are all keyed by it), and a created province would also need its own face-down refill from the Dynasty deck. The rest is buildable: "After an action targets Renyu: Reduce any Honor losses from its effects to 0" is a triggered trait over the targeted-by-action window with Unimpeachable Name's per-command HonorLossReductionPlayerId (reduced to 0 rather than by 3), and the controller's choice to bow the unit and destroy its Shadowlands cards is an Either/Or (EitherOr.cs, Extend the Soul's shape). The card is wired whole or not at all, so it stays unwired.</t>
-        </is>
-      </c>
-      <c r="H479" t="inlineStr">
-        <is>
-          <t>PROVINCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr"/>
+      <c r="H479" t="inlineStr"/>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -21223,19 +20871,11 @@
       </c>
       <c r="F574" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G574" t="inlineStr">
-        <is>
-          <t>Needs the per-Tactician cap the Glossary states ("each individual Tactician may perform at most one Tactical action per turn"), which the engine does not enforce (Program.cs's own Tactical Advantage test lets one Tactician perform it twice in a turn), so "Taigo may perform up to three Tactical actions per turn" has no cap to raise. His Tactical Battle action (bow a target enemy Personality; if he is Infantry, you may target and destroy a card without attachments in his unit) is buildable: Kaiji/Iaimiko's optional collateral slot with a not-Cavalry condition, ActionKeywords Tactical.</t>
-        </is>
-      </c>
-      <c r="H574" t="inlineStr">
-        <is>
-          <t>SMALL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr"/>
+      <c r="H574" t="inlineStr"/>
     </row>
     <row r="575">
       <c r="A575" t="inlineStr">
@@ -22205,19 +21845,11 @@
       </c>
       <c r="F603" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G603" t="inlineStr">
-        <is>
-          <t>Needs a province GAINED ("gain a province to the left of your leftmost province": a player's Provinces list is fixed at setup and only ever destroyed, never extended -- Mining Apparatus' shape, not built) and its later destruction "after the next time this game Suikihime leaves play" (a leaves-play watch for the game). Buildable now: "may not assign, and will not move, to battlefields" (a standing MovementLock of Assign|ToBattlefield, today turn-scoped only), "will not become dishonorable" (a Dishonor() immunity keyed on the Effect), "other players' Political actions may not target Suikihime" (a TargetBar by action keyword and acting player) and the once-per-game, no-other-player-controls-The-Forgotten-Temple condition on the Reaction.</t>
-        </is>
-      </c>
-      <c r="H603" t="inlineStr">
-        <is>
-          <t>PROVINCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G603" t="inlineStr"/>
+      <c r="H603" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
@@ -22413,19 +22045,11 @@
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G609" t="inlineStr">
-        <is>
-          <t>Two static rules with no representation: "Will only enter play from a province" (an entry restriction by where the card comes from: Equip, Recruit and created entries are separate paths and nothing records the origin) and "may not perform Battle actions while your current army has higher total Force than the current enemy army" (a live army-Force comparison as a restriction on actions). "After Raido enters play: Lose 6 Honor" is EntryHonorLoss.</t>
-        </is>
-      </c>
-      <c r="H609" t="inlineStr">
-        <is>
-          <t>PROVENANCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G609" t="inlineStr"/>
+      <c r="H609" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" t="inlineStr">
@@ -23165,19 +22789,11 @@
       </c>
       <c r="F631" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G631" t="inlineStr">
-        <is>
-          <t>Needs an ability usable from the dead pile ("Even if Jouta is dead": FromDiscard covers a card in a discard pile, not a Personality in Zone.Dead) whose Ranged Attack is made by a chosen Shugenja who "may be at any location unless Jouta is dead": a location rule that depends on the source's own state.</t>
-        </is>
-      </c>
-      <c r="H631" t="inlineStr">
-        <is>
-          <t>ZONE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr"/>
+      <c r="H631" t="inlineStr"/>
     </row>
     <row r="632">
       <c r="A632" t="inlineStr">
@@ -23853,19 +23469,11 @@
       </c>
       <c r="F651" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G651" t="inlineStr">
-        <is>
-          <t>Shinjo Hayan: "After engaging: Once per turn, you may assign your (unbowed) Unicorn Clan Personality in your home to the current battlefield" needs a player-triggered ASSIGNMENT outside the normal Attack-phase Assign command: every existing Assign path (AssignAttackers/AssignDefense) runs once, at battle declaration, choosing every unit for every battlefield at once -- there is no primitive for a single Reaction-timed effect to assign one more Personality from home to an already-engaged battlefield afterward (MovesToBattle moves a card there directly, bypassing "assignment" as a rules concept entirely, which is not the same thing an Assign-based card like this one needs). His Sensei-entry trait is trivial in isolation but not wired alone.</t>
-        </is>
-      </c>
-      <c r="H651" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr"/>
+      <c r="H651" t="inlineStr"/>
     </row>
     <row r="652">
       <c r="A652" t="inlineStr">
@@ -24303,19 +23911,11 @@
       </c>
       <c r="F664" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G664" t="inlineStr">
-        <is>
-          <t>Shinjo Sarang: "Battle: Choose your performing Personality, and target your Follower at any location: Transfer it to the Personality. Straighten the Follower if the Personality is opposed or Spider Clan" needs a new own-follower-any-location Target category (every existing Follower target category location-restricts to the source's own unit, the current battlefield, or a specific named relationship -- Daigotsu Yamato's own-follower-at-any-location is the closest precedent but still requires CanTransferTo AND an AtAnyLocation exemption keyed to acting-as-Battle, both already narrower than "any location, unconditionally") plus a conditional straighten keyed on the CHOSEN PERFORMER's own state (opposed, or Spider Clan) rather than the target's, a combination not yet proven together.</t>
-        </is>
-      </c>
-      <c r="H664" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr"/>
+      <c r="H664" t="inlineStr"/>
     </row>
     <row r="665">
       <c r="A665" t="inlineStr">
@@ -24583,19 +24183,11 @@
       </c>
       <c r="F672" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G672" t="inlineStr">
-        <is>
-          <t>Shosuro Aroru. Three independent gaps, so the card cannot be wired whole: (1) "Will not attach non-Ninja Followers" is a HOST-side attach refusal -- CardDefinition's AttachRequiresKeyword/AttachExcludesKeyword/AttachRequiresName gate only the ATTACHMENT's own text, so a Personality refusing a class of attachments needs a new field read at every attach funnel (MatchEngine.Equip's AttachmentLegalTarget, AttachAction.ValidateAttach, the spell-in-hand/equip-battle Requires in CardAbilities.cs). (2) "Reaction: When an action would target a Ninja at Aroru's location: Choose another of your cards. The action targets it instead, if legal." is the existing redirect (RedirectAction with Blade of Champions' redirect-target-own-card, Castle of Order's Ninja-at-location check), but its tail "After the action's resolution, you may move Aroru to a different location" needs a Reaction to register a DEFERRED optional effect that fires when the held action finishes resolving (CompleteAbilityResolution / ResolveAttack's tails carry no per-reaction deferred effect) and then asks for a destination (home or another unresolved battlefield) at that later moment. (3) "Battle: Other players may not take Reactions until this action ends. Ranged 5 Attack." -- the Attack is trivial, but nothing forbids Reactions: every window (before-action, targeted-by-action, attackReaction, OpenAlternatingReactionWindow) would need a per-action lockout of the other player until the action ends.</t>
-        </is>
-      </c>
-      <c r="H672" t="inlineStr">
-        <is>
-          <t>TRIG-ANN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr"/>
+      <c r="H672" t="inlineStr"/>
     </row>
     <row r="673">
       <c r="A673" t="inlineStr">
@@ -24795,19 +24387,11 @@
       </c>
       <c r="F678" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G678" t="inlineStr">
-        <is>
-          <t>Shosuro Ietsuno: "After a card from a deck refills Ietsuno's battlefield's province: Look at it. You may switch it with a card owned by the same player in another province" needs a brand new province-refill hook -- DeckLook.cs's own Look primitive only ever looks at the top N cards of a deck as part of an ability's own effect, never as a standing watch that fires automatically whenever a SPECIFIC province (his own battlefield's) refills from a reveal, and "switch it with a card owned by the same player in another province" (a face-down province-to-province swap, same owner, either Dynasty or Fate) has no existing primitive at all. Her plain "Battle: Target an enemy card without attachments: Bow it" is trivial in isolation but not wired alone.</t>
-        </is>
-      </c>
-      <c r="H678" t="inlineStr">
-        <is>
-          <t>PROVINCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr"/>
+      <c r="H678" t="inlineStr"/>
     </row>
     <row r="679">
       <c r="A679" t="inlineStr">
@@ -24905,19 +24489,11 @@
       </c>
       <c r="F681" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G681" t="inlineStr">
-        <is>
-          <t>Shosuro Keirei. Three gaps: (1) "two -1F/-1C Poison tokens" -- CardToken (Models.cs) carries ONE Stat/Amount, and every token reader (StatModifier, CreateToken's Tireless Efforts/Creating Order/Aka-beko negations, SeedsOfDecayBatch4's removal of negative Force tokens, TokenCount) reads that one stat; splitting each Poison token into a Force token and a Chi token would double every count of Poison tokens and let a Force-only negation strip half a token. (2) "Move Keirei from the current battlefield to a different battlefield" -- MoveSpec (MoveDestinations.cs) offers only UNRESOLVED battlefields (AnyUnresolved/AdjacentUnresolved), while the text allows any other battlefield of the Attack Phase, resolved ones included. (3) "You may target ... a Personality at Keirei's new or previous location" is an optional target chosen after the move, possibly at a battlefield other than the current one: the Battle target Require in ValidateAbility demands AtBattle, and TargetSlots' at-resolution follow-ups offer fixed options (ConditionalChoice), not card targets.</t>
-        </is>
-      </c>
-      <c r="H681" t="inlineStr">
-        <is>
-          <t>TOKEN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr"/>
+      <c r="H681" t="inlineStr"/>
     </row>
     <row r="682">
       <c r="A682" t="inlineStr">
@@ -25423,19 +24999,11 @@
       </c>
       <c r="F696" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G696" t="inlineStr">
-        <is>
-          <t>Needs "you have the first opportunity to take a Battle action in this battle, which must be performed by Toson": a priority override for the first Battle action after an engage, with a forced performer for that one action. The Reaction after engaging exists (Detained), and so does discarding a card of the Province, but neither gives the opportunity or restricts who takes it.</t>
-        </is>
-      </c>
-      <c r="H696" t="inlineStr">
-        <is>
-          <t>PRIORITY</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G696" t="inlineStr"/>
+      <c r="H696" t="inlineStr"/>
     </row>
     <row r="697">
       <c r="A697" t="inlineStr">
@@ -27229,19 +26797,11 @@
       </c>
       <c r="F749" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G749" t="inlineStr">
-        <is>
-          <t>Needs a Reaction lockout: "After Thunder Dragon performs an action: Other players may not take Reactions until it ends" -- no primitive closes the other player's side of a reaction window (the before-action, attack, bow, move, after-battle-action and entry windows all offer either player their Reactions) for the duration of one pending action. The two statics ARE buildable now: "Your Mantis Clan Personalities have +1F" is one more controller-scoped static term of PersonalityForce (Zansho's zansho-follower-force shape, StaticKeywordRules.cs), and "have the ability Battle: Target an enemy card without unbowed attachments: Bow it" is a controller-scoped static ability grant read where AbilityIdsOf joins granted abilities (the category is enemy-card-without-unbowed-attachments, already built).</t>
-        </is>
-      </c>
-      <c r="H749" t="inlineStr">
-        <is>
-          <t>PRIORITY</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G749" t="inlineStr"/>
+      <c r="H749" t="inlineStr"/>
     </row>
     <row r="750">
       <c r="A750" t="inlineStr">
@@ -27951,19 +27511,11 @@
       </c>
       <c r="F770" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G770" t="inlineStr">
-        <is>
-          <t>Tokiko - experienced: "Battle/Open: Destroy Tokiko and target your dead Personality: Bring him into play in your home or at the current battlefield, paying all costs but paying 7 less Gold" needs a player-CHOSEN recruit destination: every existing dead-Personality recruit (Essence of Undeath's own-dead-personality precedent, "at this Shugenja's location"; At Any Cost, "at the battlefield the action was played at") recruits at a location fixed by the source's OWN position, never a home-or-battlefield choice independent of where the destroyed source itself was. GoldCostRule.TargetRecruit(modifier: -7, floor: 0) already prices the discount exactly; only the destination choice is missing.</t>
-        </is>
-      </c>
-      <c r="H770" t="inlineStr">
-        <is>
-          <t>ZONE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G770" t="inlineStr"/>
+      <c r="H770" t="inlineStr"/>
     </row>
     <row r="771">
       <c r="A771" t="inlineStr">
@@ -28601,19 +28153,11 @@
       </c>
       <c r="F789" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G789" t="inlineStr">
-        <is>
-          <t>Tsuruchi Nobukatsu (the inexperienced printing; unrelated to Nobukatsu - exp's text). "Battle: Ranged 4 Attack. If the Ranged Attack destroyed a card, you may target and straighten a Holding." The Attack and the destroyed-a-card check are built (Sticks and Stones' AfterSticksAndStonesAttack reads targetInPlayBefore). The gap is the optional Holding TARGET chosen after the Attack resolves: an Attack can resolve inline or later in ResolveAttack after its reaction window, and neither pausing primitive fits -- SequencedTarget.cs pauses BEFORE a sequenced Attack, DeciderChoice.cs pauses inside the ordinary effect switch and resumes with CompleteAbilityResolution, but nothing pauses AFTER a deferred ResolveAttack (whose own tail finishes the action). Shiba Iaimiko's up-front optional slot (TargetSlots.cs) would pick the Holding before the Attack, but an ability with Target "attack" cannot also carry Slots, and choosing it up front would target the Holding even when the Attack destroys nothing.</t>
-        </is>
-      </c>
-      <c r="H789" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G789" t="inlineStr"/>
+      <c r="H789" t="inlineStr"/>
     </row>
     <row r="790">
       <c r="A790" t="inlineStr">
@@ -28711,19 +28255,11 @@
       </c>
       <c r="F792" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G792" t="inlineStr">
-        <is>
-          <t>Tsuruchi Shichiro: "After a Ranged Attack action resolves that your Mantis Clan Personality performed: Once per battle, you may move him home" needs AfterActionReactionTriggers.AfterActionResolved narrowed to (a) specifically a RANGED Attack (every existing AfterActionResolved reader checks what was DESTROYED, never the acting ability's own AttackKind) and (b) the ACTOR's own Mantis Clan keyword rather than a fixed card -- a combination not yet proven, though each half has a partial precedent (AttackKind(facts.AbilityId) reads the kind; ActionCarriesKeyword-style clan checks exist for other triggers). His Sensei-entry trait is trivial in isolation but not wired alone.</t>
-        </is>
-      </c>
-      <c r="H792" t="inlineStr">
-        <is>
-          <t>SMALL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G792" t="inlineStr"/>
+      <c r="H792" t="inlineStr"/>
     </row>
     <row r="793">
       <c r="A793" t="inlineStr">
@@ -29267,19 +28803,11 @@
       </c>
       <c r="F808" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G808" t="inlineStr">
-        <is>
-          <t>Utaku Lishan: "While Lishan is attacking, she has +1F and +1PH" is buildable now (PersonalityForce's own attacking-one Effect term, plus a matching StaticPersonalHonorBonus term). "Reaction: After you announce a Battle action, if Lishan is at the current battlefield, target a Personality or Follower opposing her: Give it a Force penalty equal to Lishan's Personal Honor" needs the announce-reaction window (ResolveOrDeferAnnounceReaction, CardAbilities.cs) generalized past its own hardcoded Ranged-only gate ("only ever offered when the about-to-execute ability is classified Ranged", its own doc comment; Tsuruchi Yakusho is its one existing user) to ANY Battle action, which the same comment says a future card could do but nothing has yet -- not attempted here given the window's shared, heavily-tested role in every Ranged Attack. The card is not wired for its static bonus alone, following this pass's whole-card convention.</t>
-        </is>
-      </c>
-      <c r="H808" t="inlineStr">
-        <is>
-          <t>TRIG-ANN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G808" t="inlineStr"/>
+      <c r="H808" t="inlineStr"/>
     </row>
     <row r="809">
       <c r="A809" t="inlineStr">
@@ -29585,19 +29113,11 @@
       </c>
       <c r="F817" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G817" t="inlineStr">
-        <is>
-          <t>Needs a Reaction to "a Personality assigns or moves, if he is now opposing Tairu": there is no trigger on assignment or on movement of any Personality (only the after-move window Legion of the Bat uses, for enemy Infantry moved to its own battlefield).</t>
-        </is>
-      </c>
-      <c r="H817" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G817" t="inlineStr"/>
+      <c r="H817" t="inlineStr"/>
     </row>
     <row r="818">
       <c r="A818" t="inlineStr">
@@ -33621,19 +33141,11 @@
       </c>
       <c r="F935" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G935" t="inlineStr">
-        <is>
-          <t>Needs a Reaction fired "after the resolution of your action that bowed, destroyed, or moved a Personality who has opposed this card at the current battlefield": the destroyed/moved half is now recorded (MatchState.LastResolvedAction, issue #437), but a bow is not -- unlike DestroyUnits/MoveHome, no single choke point narrates every one of the hundred-plus call sites that set CardInstance.Bowed directly, so the printed "bowed, destroyed, or moved" cannot be checked in full yet.</t>
-        </is>
-      </c>
-      <c r="H935" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G935" t="inlineStr"/>
+      <c r="H935" t="inlineStr"/>
     </row>
     <row r="936">
       <c r="A936" t="inlineStr">
@@ -36139,19 +35651,11 @@
       </c>
       <c r="F1008" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1008" t="inlineStr">
-        <is>
-          <t>Needs an "after this card bows" trigger that straightens it (a trait, not a Reaction): the after-bow windows are for Personalities (Hizumi, Ruya) and for a sibling Follower (Nikutai). The second ability (negate this card's destruction from an action that targets a card in this unit) is expressible with the targeted-by-action trigger and NegateEffects(card, "destroy").</t>
-        </is>
-      </c>
-      <c r="H1008" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1008" t="inlineStr"/>
+      <c r="H1008" t="inlineStr"/>
     </row>
     <row r="1009">
       <c r="A1009" t="inlineStr">
@@ -36597,19 +36101,11 @@
       </c>
       <c r="F1021" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1021" t="inlineStr">
-        <is>
-          <t>Needs an Attack-strength modifier keyed on the DEFENDING unit rather than the attacking source ("Melee Attacks targeting cards in this unit have -2 strength"): AttackFollowerException and every strengthOverride path adjust an Attack's strength from its OWN source card (or a paid amount), never from a static trait on the unit being targeted -- no hook reads the target's own side when an Attack's effective strength is computed. The Reaction half ("before another player's action resolves, negate this Personality's movement from the action's effects") is separately wirable: NegatesEffect plus the existing "before-any-action-resolves" trigger.</t>
-        </is>
-      </c>
-      <c r="H1021" t="inlineStr">
-        <is>
-          <t>STAT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1021" t="inlineStr"/>
+      <c r="H1021" t="inlineStr"/>
     </row>
     <row r="1022">
       <c r="A1022" t="inlineStr">
@@ -37893,19 +37389,11 @@
       </c>
       <c r="F1059" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1059" t="inlineStr">
-        <is>
-          <t>"You must declare an attack each turn and assign this Personality to attack if possible" is an obligation the rules have no place for: nothing forces an attack declaration or an assignment. Its Reaction (after an action targets this Personality: negate his movement) would be buildable like Kota's.</t>
-        </is>
-      </c>
-      <c r="H1059" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1059" t="inlineStr"/>
+      <c r="H1059" t="inlineStr"/>
     </row>
     <row r="1060">
       <c r="A1060" t="inlineStr">
@@ -38807,19 +38295,11 @@
       </c>
       <c r="F1086" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1086" t="inlineStr">
-        <is>
-          <t>Needs "Gain a province to the left of your leftmost province": provinces are a fixed list of four per player (ProvinceState.Index 0..3 is read everywhere as a position: battlefields, assignments, the view); adding a province at index -1 or reindexing is not built. The cost is buildable: "Remove this card and any number of Holdings you control with total base Gold Cost of 10 or higher from the game" is a 0..N slot of own Holdings with a total printed-cost condition on the selection (a slot-level aggregate condition, a small extension of TargetSlots) plus RemoveSource.</t>
-        </is>
-      </c>
-      <c r="H1086" t="inlineStr">
-        <is>
-          <t>PROVINCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1086" t="inlineStr"/>
+      <c r="H1086" t="inlineStr"/>
     </row>
     <row r="1087">
       <c r="A1087" t="inlineStr">
@@ -39223,19 +38703,11 @@
       </c>
       <c r="F1098" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1098" t="inlineStr">
-        <is>
-          <t>Needs a "which other players' cards' effects may not discard" hand-discard immunity, shared with oracle-l5r-8298 (The Scorpion Wall is Finished): DiscardFate (CardAbilities.cs) is one shared function with 14 call sites mixing the hand owner's own cost payments/choices (never to be blocked) with another player's card forcing the discard (which these two cards' printed text would block) -- it carries no "who caused this" parameter today, and retrofitting one correctly across every call site is a cross-cutting change out of proportion for two cards' one shared clause. The hand-size clauses alone ("your maximum hand size is increased by 1; other players' maximum hand sizes are reduced by 1, to a minimum of 7") are buildable off HandLimitFor's existing increase-other-hand-size/decrease-other-hand-size shape (MatchEngine.cs), but the card is blocked as a whole rather than partially wired.</t>
-        </is>
-      </c>
-      <c r="H1098" t="inlineStr">
-        <is>
-          <t>HONOR</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1098" t="inlineStr"/>
+      <c r="H1098" t="inlineStr"/>
     </row>
     <row r="1099">
       <c r="A1099" t="inlineStr">
@@ -40561,19 +40033,11 @@
       </c>
       <c r="F1137" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1137" t="inlineStr">
-        <is>
-          <t>"Choose your performing Ninja, and destroy this card or discard it from your hand: Ranged 3 Attack" is an Item used from a hand: ValidateAbility's source-zone rule lets only a Strategy or a Ring be the source of an action from a hand (an Item is in play or attached). "Will only attach to a Ninja" exists (AttachRequiresKeyword).</t>
-        </is>
-      </c>
-      <c r="H1137" t="inlineStr">
-        <is>
-          <t>ZONE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1137" t="inlineStr"/>
+      <c r="H1137" t="inlineStr"/>
     </row>
     <row r="1138">
       <c r="A1138" t="inlineStr">
@@ -40744,7 +40208,7 @@
       </c>
       <c r="G1142" t="inlineStr">
         <is>
-          <t>Vanquisher's Blades: mechanically wirable, scan unavailable for its created card. "Reaction: After this card enters play: Create a +2F/+1C Weapon Item and attach it to this Personality (if legal)" is an own-enters-play Reaction with a CreatedCardSpec(Item, +2F/+1C, [Weapon]) attached to the wielder (Bo of Water's created-Item attach; RequireAttachable already makes the second Weapon legal only for a Kensai or with a Kama, which is exactly "(if legal)"). The one fitting Proxy is Readied Blade (oracle-l5r-9749, Promotional-Celestial: +2F/+1C Weapon, paired in docs/decisions/2026-09-20-created-cards-from-proxy-scans.md), which is not published: only its receipt is local (assets/reference/oracle/promotional-celestial/receipts), the Oracle image host is refused by this sandbox's network policy, and it is not in the catalogue art pack. CreatedCards.Resolve/Verify need a published CreatedOnly scan, so Vanquisher's Blades cannot be wired until Readied Blade is packaged as a CreatedOnly Item.</t>
+          <t>Vanquisher's Blades (issue #503, P6, re-checked): its own scan is local; blocked only by its created Weapon. The +2F/+1C Weapon Proxy is Readied Blade (oracle-l5r-9749, Promotional-Celestial), which has only a receipt (no working_copy; not in either catalogue WebP pack, l5r-s3 or l5r-emperor) and may not be downloaded in this pass. Once Readied Blade is published CreatedOnly the card is Bo of Water's entering-play create-and-attach (RequireAttachable already reads '(if legal)').</t>
         </is>
       </c>
       <c r="H1142" t="inlineStr">
@@ -41453,19 +40917,11 @@
       </c>
       <c r="F1163" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1163" t="inlineStr">
-        <is>
-          <t>Centering the Soul: "After an action resolves, bow this card and target one of your Rings the action bowed: Straighten the Ring" needs a new Reaction-target-legality shape -- WHICH Ring(s) the just-resolved action itself bowed (as opposed to a card ability or a manual straighten check, no primitive correlates a resolved action's own cost/effects against a Ring's Bowed flag the way LastResolvedAction already does for destroys/moves). Its "if this Shugenja is Void, you may destroy this card; if you did, you may use the Ring's base abilities an additional time this turn" then needs the per-turn-use-clear primitive (RefreshBattleAbilities, Shiba Tsukimi's shape) generalized past Battle-timing abilities to a Ring's own (non-Battle) base ability. Two new pieces for one card; left unwired.</t>
-        </is>
-      </c>
-      <c r="H1163" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1163" t="inlineStr"/>
+      <c r="H1163" t="inlineStr"/>
     </row>
     <row r="1164">
       <c r="A1164" t="inlineStr">
@@ -41869,19 +41325,11 @@
       </c>
       <c r="F1175" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1175" t="inlineStr">
-        <is>
-          <t>Damning Ceremony: "Give this Personality a permanent Force bonus raising his Force to equal his base Gold Cost" is a straightforward delta-to-value AddPermanentModifier (Kaido's own "reduce Force to 0" shape, generalized to a positive target value read off GoldCost instead of 0); "permanently give him Shadowlands, Nonhuman, Oni" is three ordinary GrantKeyword(..., Permanent) calls; "lose 2 Honor" is GainHonor with a negative amount. All three pieces already exist individually -- left unwired this pass for lack of time to also confirm the reading of "this Personality" (the performer versus the wielder the Spell is attached to) against the scan.</t>
-        </is>
-      </c>
-      <c r="H1175" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1175" t="inlineStr"/>
+      <c r="H1175" t="inlineStr"/>
     </row>
     <row r="1176">
       <c r="A1176" t="inlineStr">
@@ -41979,19 +41427,11 @@
       </c>
       <c r="F1178" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1178" t="inlineStr">
-        <is>
-          <t>Delving into History: "Search your Fate deck for a non-Unique Spell that must share a keyword with the performer unless he is Void" needs a search criterion compared against the PERFORMER's own live keyword set, not a fixed list -- DeckSearch.cs's own comment already flags this exact category of extension ("a comparison against the performer's own stat ... is a natural extension and is not built yet") for a numeric stat; a keyword-set version threads a performer reference through SearchEligibility/SearchGroups, both shared by every other search on the catalogue. Left unwired to avoid touching that shared signature without room to re-verify every existing search this pass.</t>
-        </is>
-      </c>
-      <c r="H1178" t="inlineStr">
-        <is>
-          <t>SEARCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1178" t="inlineStr"/>
+      <c r="H1178" t="inlineStr"/>
     </row>
     <row r="1179">
       <c r="A1179" t="inlineStr">
@@ -42055,19 +41495,11 @@
       </c>
       <c r="F1180" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1180" t="inlineStr">
-        <is>
-          <t>Needs "Negate his next straightening this game": a one-shot negation that persists until it is used. The negations that exist last the turn (StraightenBlockedTurn) or hold every attempt until a named moment (StraightenHolds). Its static half ("While this Shugenja is Earth, your provinces have +1 strength") would be one more StaticProvinceBonuses entry.</t>
-        </is>
-      </c>
-      <c r="H1180" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1180" t="inlineStr"/>
+      <c r="H1180" t="inlineStr"/>
     </row>
     <row r="1181">
       <c r="A1181" t="inlineStr">
@@ -42165,19 +41597,11 @@
       </c>
       <c r="F1183" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1183" t="inlineStr">
-        <is>
-          <t>Needs a Reaction "after the resolution of an action that moved a Personality to the current battlefield" that names the Personality moved: the after-move window (OpenMoveReactionWindow) serves Legion of the Bat alone. Its static half ("While this Shugenja is Water, other players' provinces have -1 strength") would be one more StaticProvinceBonuses entry.</t>
-        </is>
-      </c>
-      <c r="H1183" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1183" t="inlineStr"/>
+      <c r="H1183" t="inlineStr"/>
     </row>
     <row r="1184">
       <c r="A1184" t="inlineStr">
@@ -42275,19 +41699,11 @@
       </c>
       <c r="F1186" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1186" t="inlineStr">
-        <is>
-          <t>Extending Influence: its Air-entry Honor loss ("Each other player loses 1 Honor") is ordinary (EntryHonorLoss, gated live on the wielder's own Air keyword the way Kojiro's Naval already is); "the performing Shugenja copies one of the target's abilities which does not copy abilities" is CardCopy.cs's existing ability-copy step (Fukuzo's own BeginCopy(steps: [CopyStep.Ability])), narrowed to one step instead of Fukuzo's two. Individually buildable; left unwired this pass for lack of time to wire and test the destroy-this-card-as-cost Open shape end to end.</t>
-        </is>
-      </c>
-      <c r="H1186" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1186" t="inlineStr"/>
+      <c r="H1186" t="inlineStr"/>
     </row>
     <row r="1187">
       <c r="A1187" t="inlineStr">
@@ -42623,19 +42039,11 @@
       </c>
       <c r="F1196" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1196" t="inlineStr">
-        <is>
-          <t>Illusory Defense: its static "Your Air Shugenja have +1C" is an ordinary controller-scoped Chi bonus (StaticKeywordRules.cs's own shape, generalized from Force/keyword to Chi). Its Limited half -- "Create a province to the left of your leftmost province which permanently does not hold Dynasty cards" -- needs a GAINED province: every player's Provinces list is a fixed, position-indexed array read everywhere (battlefields, assignments, the view), the same gap already recorded against Otomo Suikihime (oracle-l5r-10094) and Mining Apparatus (oracle-l5r-10120) in the Seeds of Decay pass. Not built; the card stays whole or not at all.</t>
-        </is>
-      </c>
-      <c r="H1196" t="inlineStr">
-        <is>
-          <t>PROVINCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1196" t="inlineStr"/>
+      <c r="H1196" t="inlineStr"/>
     </row>
     <row r="1197">
       <c r="A1197" t="inlineStr">
@@ -42937,19 +42345,11 @@
       </c>
       <c r="F1205" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1205" t="inlineStr">
-        <is>
-          <t>Mara's Touch: its static "+2F while Nonhuman" is Scouring Flood's own Spell-Effect-keyed Force bonus, conditioned live on the wielder's Nonhuman keyword (the same shape this pass used unconditionally for The Swell of Strength); its Open ("-2F: He changes shape, give him Cavalry") and Battle ("-2F: Ranged 6 Attack") halves are both ordinary (a Force penalty plus GrantKeyword(Cavalry, Permanent); a Ranged Attack at -2F cost, Genji's own attack shape). "He changes shape" reads as flavor with no defined rules term (core rules' own Reading the Cards convention). All three pieces individually exist; left unwired this pass for lack of time to wire and test all three on one card.</t>
-        </is>
-      </c>
-      <c r="H1205" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1205" t="inlineStr"/>
+      <c r="H1205" t="inlineStr"/>
     </row>
     <row r="1206">
       <c r="A1206" t="inlineStr">
@@ -43221,19 +42621,11 @@
       </c>
       <c r="F1213" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1213" t="inlineStr">
-        <is>
-          <t>Ochiai's Bravery: its static "has Duelist while Fire" needs a live wielder-keyword-conditional KEYWORD grant generalized past the one built shape (AttachGrantsEliteEffectWhileWielderHas only ever grants the Elite EFFECT, never an arbitrary keyword) -- Isawa Kojiro's own conditional Naval grant is the closer precedent, but it is hardcoded to Naval, not parameterized by keyword. Its Battle half ("if unbowed, bow this card and target an enemy Personality: duels him; destroy a card without attachments in the duel's loser's unit") is ordinary (IssuesDuel, plus a duel-loser-scoped destroy). Left unwired for the static grant's missing generalization.</t>
-        </is>
-      </c>
-      <c r="H1213" t="inlineStr">
-        <is>
-          <t>SMALL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1213" t="inlineStr"/>
+      <c r="H1213" t="inlineStr"/>
     </row>
     <row r="1214">
       <c r="A1214" t="inlineStr">
@@ -43302,7 +42694,7 @@
       </c>
       <c r="G1215" t="inlineStr">
         <is>
-          <t>Our Ancestor's Call: mechanically wirable, no scan exists for its created card. "Battle: If this Shugenja is opposed, destroy this card: Create a 2F/2C/3PH Samurai • Ancestor • Spirit Personality with your Clan alignment at the current battlefield. If this Shugenja is Water and defending, create two such Personalities instead" is the Celestial Sword of the Lion's created-Personality shape (CreatedCardSpec AtBattlefield) with ControllerClan (#405, Venerable Master) and a count of two behind a Water-and-defending check, plus an opposed-Shugenja Require and a Sacrifice cost. No Proxy scan prints a 2F/2C/3PH Samurai/Ancestor/Spirit with "your Clan alignment" (the Lion Ancestor, oracle-l5r-9785, is fixed to Lion Clan): docs/requests/created-card-scans-needed.md row B6 asks for it (assets/requested-scans/ancestor-clan.jpg, shared with Offering Reverence). CreatedCards.Resolve fails without it, so the card stays unpublished.</t>
+          <t>Our Ancestor's Call (issue #503, P6, re-checked): its own scan is local; blocked only by its created card, a 2F/2C/3PH Samurai Ancestor Spirit Personality 'with your Clan alignment'. The only Ancestor Proxy (Lion Ancestor, oracle-l5r-9785) is fixed to Lion Clan; no clan-alignment Ancestor scan exists locally (docs/requests/created-card-scans-needed.md row B6, ancestor-clan.jpg, unticked). The rest is the Celestial Sword of the Lion's AtBattlefield create with ControllerClan, a count of two behind a Water-and-defending check, an opposed-Shugenja requirement and a Sacrifice cost.</t>
         </is>
       </c>
       <c r="H1215" t="inlineStr">
@@ -43849,19 +43241,11 @@
       </c>
       <c r="F1231" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1231" t="inlineStr">
-        <is>
-          <t>Needs the first sentence, "You may attach this card from your discard pile to your Void Shugenja": a standing permission on the Equip rulebook action (Equip from a discard pile) rather than an action of its own, restricted to a Void Shugenja. The Open half (bow this card: give another player's Personality Kolat, Ninja or Shadowlands) is Izuna's three abilities sharing one use.</t>
-        </is>
-      </c>
-      <c r="H1231" t="inlineStr">
-        <is>
-          <t>RULEBOOK</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1231" t="inlineStr"/>
+      <c r="H1231" t="inlineStr"/>
     </row>
     <row r="1232">
       <c r="A1232" t="inlineStr">
@@ -44095,19 +43479,11 @@
       </c>
       <c r="F1238" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1238" t="inlineStr">
-        <is>
-          <t>Refreshed: the delayed half ("Before this turn ends, put his unit into play") can be scheduled through the shared store at DelayUntil.EndOfTurn (ScheduleDelayedEffect), but the store applies effects to a card that is IN PLAY (a card that left play is negated), and this card removes a Shugenja and his whole unit from the game and puts it back: a new "enter play" kind that returns a removed unit whole (host plus attachments, ignoring costs, entering-play effects and restrictions) is still missing, and RemoveFromGame detaching a host's attachments is still unbuilt. NO LOCAL SCAN.</t>
-        </is>
-      </c>
-      <c r="H1238" t="inlineStr">
-        <is>
-          <t>ZONE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1238" t="inlineStr"/>
+      <c r="H1238" t="inlineStr"/>
     </row>
     <row r="1239">
       <c r="A1239" t="inlineStr">
@@ -44647,19 +44023,11 @@
       </c>
       <c r="F1254" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1254" t="inlineStr">
-        <is>
-          <t>The Menacing Sky: "After the next time (this turn) he assigns or an action resolves which moved him to a battlefield, bow him" needs SeedsOfDecayBatch2.cs's own AssignmentWatch ("after the next time this turn he is assigned to attack") widened to an OR against a second trigger (an action moving him to a battlefield, MovesToBattle-flagged abilities), which the existing watch does not compose with. "Unless he is Thunder" performer-side bow-cost exemption is the ordinary UnlessKeyword cost shape. Left unwired for the assign-or-move OR composition.</t>
-        </is>
-      </c>
-      <c r="H1254" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1254" t="inlineStr"/>
+      <c r="H1254" t="inlineStr"/>
     </row>
     <row r="1255">
       <c r="A1255" t="inlineStr">
@@ -44825,19 +44193,11 @@
       </c>
       <c r="F1259" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1259" t="inlineStr">
-        <is>
-          <t>Needs "You may destroy this card; if you do, discard the card you looked at": a look (LookSpec, "any Fate deck") whose discard is conditional on destroying the Spell itself, a cost tied to a disposition. Its static half ("While this Shugenja is Void, your maximum hand size is increased by 1") would be an Effect read by MaxHandSize, as Taishuu's is.</t>
-        </is>
-      </c>
-      <c r="H1259" t="inlineStr">
-        <is>
-          <t>SEARCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1259" t="inlineStr"/>
+      <c r="H1259" t="inlineStr"/>
     </row>
     <row r="1260">
       <c r="A1260" t="inlineStr">
@@ -45522,7 +44882,7 @@
       </c>
       <c r="G1279" t="inlineStr">
         <is>
-          <t>Yari of Air: mechanically wirable, no scan exists for its created card. "After this card enters play, if this Shugenja is Air: Gain 1 Honor" is the mandatory entry trait (the Celestial Swords' entry Honor, gated on the wielder's Air keyword) and "Limited: Once per game: Create a +1F/+1C Air • Weapon Item with the ability, 'Battle: Give each Personality and Follower in the enemy army -1F' and attach it to one of your Personalities" is Bo of Water's OncePerGame created-Weapon shape (CreatedCardSpec with AbilityText) plus an army-wide -1F Battle ability on the created Item. The only near scan, Tsi Weapon (oracle-l5r-9715: +1F/+1C Weapon), has neither Air nor the ability, so CreatedCards.Resolve finds nothing: docs/requests/created-card-scans-needed.md row A5 asks for it (assets/requested-scans/yari-of-air.jpg). The card stays unpublished until that scan exists.</t>
+          <t>Yari of Air (issue #503, P6, re-checked): its own scan is local; blocked only by its created +1F/+1C Air Weapon with 'Battle: Give each Personality and Follower in the enemy army -1F'. Tsi Weapon (oracle-l5r-9715) is a near miss (no Air, no ability) and has no local scan anyway; docs/requests/created-card-scans-needed.md row A5 (yari-of-air.jpg) is unticked. The rest (the Air-gated entry Honor, Bo of Water's OncePerGame create-and-attach, an army-wide -1F) is buildable.</t>
         </is>
       </c>
       <c r="H1279" t="inlineStr">
@@ -45661,19 +45021,11 @@
       </c>
       <c r="F1283" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1283" t="inlineStr">
-        <is>
-          <t>Needs a Focus Effect that substitutes one of your Yojimbo Personalities for your Personality in the duel (the duel's participants are fixed when it is issued), and Revenge tokens (+1F tokens of a named kind, three at once) given after another player's action destroys one of your Courtiers or Shugenja.</t>
-        </is>
-      </c>
-      <c r="H1283" t="inlineStr">
-        <is>
-          <t>DUEL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1283" t="inlineStr"/>
+      <c r="H1283" t="inlineStr"/>
     </row>
     <row r="1284">
       <c r="A1284" t="inlineStr">
@@ -47029,19 +46381,11 @@
       </c>
       <c r="F1323" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1323" t="inlineStr">
-        <is>
-          <t>Asset Denial (re-verified; the old note's "Retainer mechanic" is stale -- Retainer is a plain keyword on Holdings, e.g. Recruitment Officer/Slanderer, so the Open half "Bow your performing Ninja Personality and target a Retainer: Destroy it" is an ordinary BowPerformer cost plus a keyword-gated Holding target and would wire on its own). Blocked on its Battle half, "Choose your performing Ninja Personality with no non-Ninja Followers at the current battlefield: Move him to a different location. If he moved, straighten his unit. Discard a card in a province.": (1) "a different location" is home OR another battlefield, the player's choice -- Hawado's own split into two ability ids sharing a UsageKey, the battlefield one naming its destination in GameCommand.Province (MoveDestinations.cs); (2) "Discard a card in a province" is a second, independent choice of ANY player's province card (face down included). GameCommand carries one Province (already taken by the battlefield destination) and one TargetPlayerId; a Slots selection cannot carry it instead, because SlotCandidateCards (TargetSlots.cs) never lists a card in Zone.Province and a Slots ability is listed through SlotAbilityOption, which never enumerates a chosen battlefield destination (AbilityActions skips the destination loop for it). Both halves are kept together rather than splitting one card.</t>
-        </is>
-      </c>
-      <c r="H1323" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1323" t="inlineStr"/>
+      <c r="H1323" t="inlineStr"/>
     </row>
     <row r="1324">
       <c r="A1324" t="inlineStr">
@@ -48091,19 +47435,11 @@
       </c>
       <c r="F1354" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1354" t="inlineStr">
-        <is>
-          <t>Needs "+1F and the ability 'Battle: Ranged 4 Attack' while in an army with one or more of the others": a bonus and a granted ability that last while a condition on the army holds, for two or three performing Samurai at once (a conditional duration re-judged live, as Kaiu Nakano's).</t>
-        </is>
-      </c>
-      <c r="H1354" t="inlineStr">
-        <is>
-          <t>STAT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1354" t="inlineStr"/>
+      <c r="H1354" t="inlineStr"/>
     </row>
     <row r="1355">
       <c r="A1355" t="inlineStr">
@@ -48958,7 +48294,7 @@
       </c>
       <c r="G1379" t="inlineStr">
         <is>
-          <t>Unchanged: the created Maimed Retainer Holding has no Proxy scan, and 'after one of your Personalities is destroyed' covers destructions the after-action window does not see (the delayed destruction now applied by the shared store is one more of them: it is applied at a trigger point, outside any action, so it would need its own after-destruction hook). NO LOCAL SCAN.</t>
+          <t>Crippled Sensei (issue #503, P6, re-checked): the card's OWN scan is now local (catalogue WebP working copy, sha256-verified; the SCAN2 gap is closed). Still blocked by (1) its created Maimed Retainer Holding ('Battle/Open: Destroy this card and target a Personality: Straighten him. Rehonor him.'), for which no Proxy scan exists (docs/requests/created-card-scans-needed.md row B7, crippled-sensei-holding.jpg, unticked), and (2) 'Reaction: After one of your Personalities is destroyed' needs a hand-Strategy Reaction window on every destruction of a Personality, including those outside an action (battle resolution, the delayed destructions the shared store applies at trigger points), which the after-action window does not see. Its Focus Effect ('After this duel ends, choose a player who loses 2 Honor') is buildable.</t>
         </is>
       </c>
       <c r="H1379" t="inlineStr">
@@ -49301,19 +48637,11 @@
       </c>
       <c r="F1389" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1389" t="inlineStr">
-        <is>
-          <t>Needs a Strategy that PLAYS ITSELF INTO PLAY as a Terrain from a Reaction ("after a Battle action resolves, if there are no Terrains in play at the current battlefield: Put this card into play there") -- every existing Terrain enters play through its own printed Battle/Open action (TerrainStatics.cs), never as the effect of an unrelated card's Reaction while sitting in hand/discard; and a standing "after an action resolves: bow any Personalities it moved" watch, which needs a per-action record of which Personalities an arbitrary action just moved (ActionEffectTracking.cs records Honor losses and the last resolved action, not a per-mover move log) -- two separate new primitives for one card.</t>
-        </is>
-      </c>
-      <c r="H1389" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1389" t="inlineStr"/>
+      <c r="H1389" t="inlineStr"/>
     </row>
     <row r="1390">
       <c r="A1390" t="inlineStr">
@@ -49687,19 +49015,11 @@
       </c>
       <c r="F1400" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1400" t="inlineStr">
-        <is>
-          <t>Needs a Kata that gives its controller a Reaction: "Before you gain Honor during your turn, bow your target performing Courtier to negate the gain and choose a player who loses 2 Honor". Kata exist (KataCards.cs) and a granted player ability does not; no Reaction fires before the acting player gains Honor (only the opponent-payment fixture negates an Honor gain).</t>
-        </is>
-      </c>
-      <c r="H1400" t="inlineStr">
-        <is>
-          <t>TRIG-ANN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1400" t="inlineStr"/>
+      <c r="H1400" t="inlineStr"/>
     </row>
     <row r="1401">
       <c r="A1401" t="inlineStr">
@@ -50073,19 +49393,11 @@
       </c>
       <c r="F1411" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1411" t="inlineStr">
-        <is>
-          <t>Needs an opponent-chooses-or-random discard: "the enemy leader discards a card of his choice, or a random card if you have Reconnaissance". The choice is a decider decision (DeciderChoice, Tarao); a random card from a hidden hand is not: nothing draws a random hidden card during a game.</t>
-        </is>
-      </c>
-      <c r="H1411" t="inlineStr">
-        <is>
-          <t>HIDDEN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1411" t="inlineStr"/>
+      <c r="H1411" t="inlineStr"/>
     </row>
     <row r="1412">
       <c r="A1412" t="inlineStr">
@@ -50387,19 +49699,11 @@
       </c>
       <c r="F1420" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1420" t="inlineStr">
-        <is>
-          <t>Easy Persuasion: two gaps in its Reaction. "Reaction: After a Personality enters play, if his controller paid less than his base Gold Cost for him, bow your performing Merchant: The Personality's controller loses Honor equal to his base Personal Honor, or 3, whichever is lower." (1) The entering-play window (OpenEntryReactionWindow, MatchQueries' entryReaction listing) is opened only for the ENTERING Personality's controller -- the any-personality-enters-play trigger requires command.PlayerId == PendingChoice.PlayerId -- so the other player (the usual holder of this card) is never offered a Reaction to an opponent's entry; opening it to both players changes every Purchase/Proclaim flow. (2) Nothing records what was actually PAID for an entry: QuotePurchase prices it and Purchase pays it, but no CardInstance or MatchState field keeps the amount (and created, free or discounted entries -- Your Clan Needs You!, Black Pearl, Clan discount, Kyuden Hida - exp -- take different paths), so "paid less than his base Gold Cost" cannot be judged. Its Battle half ("Pay Gold equal to a target unit's total Gold Cost minus 5: Move it home. Its controller loses 2 Honor.") would also need a unit-total Gold rule (GoldCostRule.TargetCurrent reads the one target card, not the Personality plus his attachments) -- small, but the card is kept whole.</t>
-        </is>
-      </c>
-      <c r="H1420" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1420" t="inlineStr"/>
+      <c r="H1420" t="inlineStr"/>
     </row>
     <row r="1421">
       <c r="A1421" t="inlineStr">
@@ -50463,19 +49767,11 @@
       </c>
       <c r="F1422" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1422" t="inlineStr">
-        <is>
-          <t>Economic Repercussions. "Limited: Put this card into play" is Kata's own EnterPlayAsKata shape (KataCards.cs, Zone.Home) and "Other players' Personalities and Followers in play have -2 Gold Cost" is a one-term addition to CardGoldCost (StatPenalties.cs). Blocked on the granted ability: "all players have the ability, 'Political Limited: Discard the Imperial Favor or pay 6 Gold: Discard a card titled Economic Repercussions from play'" -- the card's OPPONENT must be able to take an action granted by a card he does not control. A PlayerAbility (AbilityDefinition.PlayerAbility) is unconditional and listed in every match's QueryActions (AbilityActions adds every PlayerAbility whenever the Stronghold is not ScenarioOnly), so it would add two permanently-disabled actions to every published game; the only conditional grant, StaticGrantedAbilityIds (HonorAndTreacheryPass.cs), grants to a player's own Personalities, whose abilities are refused while the source is bowed. A conditional player-ability grant (listed and legal only while a named card is in play) is the missing primitive.</t>
-        </is>
-      </c>
-      <c r="H1422" t="inlineStr">
-        <is>
-          <t>GRANT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1422" t="inlineStr"/>
+      <c r="H1422" t="inlineStr"/>
     </row>
     <row r="1423">
       <c r="A1423" t="inlineStr">
@@ -51491,19 +50787,11 @@
       </c>
       <c r="F1452" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1452" t="inlineStr">
-        <is>
-          <t>Needs "negate the effects of the next action performed by the targeted card (this turn)": a negation of a FUTURE action, waiting on the card until it acts. The negations that exist apply to the action being held in a reaction window.</t>
-        </is>
-      </c>
-      <c r="H1452" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1452" t="inlineStr"/>
+      <c r="H1452" t="inlineStr"/>
     </row>
     <row r="1453">
       <c r="A1453" t="inlineStr">
@@ -51771,19 +51059,11 @@
       </c>
       <c r="F1460" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1460" t="inlineStr">
-        <is>
-          <t>Needs a Reaction "before an Event resolves: negate its effects": an Event resolves when it is revealed (ResolveEvent) with no window before it. Its Battle half (move him home, straighten his unit if he moved) is buildable.</t>
-        </is>
-      </c>
-      <c r="H1460" t="inlineStr">
-        <is>
-          <t>TRIG-ANN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1460" t="inlineStr"/>
+      <c r="H1460" t="inlineStr"/>
     </row>
     <row r="1461">
       <c r="A1461" t="inlineStr">
@@ -51954,7 +51234,7 @@
       </c>
       <c r="G1465" t="inlineStr">
         <is>
-          <t>Fruitless Search: mechanically wirable, scan unavailable for its token. "Reaction: After engaging, if any enemy units are at the current battlefield: Create a 4F/4C/3PH Imperial Samurai Duelist Magistrate Personality on your side there. Remove him from the game after this battle ends" is Kyuden Hida - exp's own after-engaging Creates shape with CreatedCardSpec.AtBattlefield + UntilBattleEnds (Kitsu Miro's Ancestor) and a by-id enemy-presence Require. The Proxy it creates is Emerald Magistrate (oracle-l5r-9996, Embers of War: 4F/4C/3PH, Duelist/Imperial/Magistrate/Samurai, same artist), which is not published: its receipt names only the master scan (no working_copy), the Oracle image host is refused by this sandbox's network policy, and it is not in the local art pack. CreatedCards.Resolve/Verify need a published CreatedOnly scan, so the creator cannot be wired until the Proxy is published (package it the way package_personality_wave_64.py published Guest/Haruki's Deer once its scan can be fetched).</t>
+          <t>Fruitless Search (issue #503, P6, re-checked): its own scan is local; blocked only by its created Emerald Magistrate (oracle-l5r-9996, 4F/4C/3PH Duelist Imperial Magistrate Samurai), which has only a receipt (no working_copy; not in either catalogue WebP pack, l5r-s3 or l5r-emperor) and may not be downloaded in this pass. The card is otherwise Kyuden Hida - exp's after-engaging Creates with AtBattlefield + UntilBattleEnds and an enemy-presence requirement.</t>
         </is>
       </c>
       <c r="H1465" t="inlineStr">
@@ -52093,19 +51373,11 @@
       </c>
       <c r="F1469" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1469" t="inlineStr">
-        <is>
-          <t>Needs a Gold-Cost comparison Target category (same gap as oracle-l5r-24/6034): "target an enemy card with lower Gold Cost" than the performer's own. Its second Battle ability (negate Force penalties and negate effects preventing Force contribution) is separately wirable now (Tireless Efforts' own ForcePenalties.cs shape, issue #453 batch 5) but the card's own two Battle abilities are left together rather than split.</t>
-        </is>
-      </c>
-      <c r="H1469" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1469" t="inlineStr"/>
+      <c r="H1469" t="inlineStr"/>
     </row>
     <row r="1470">
       <c r="A1470" t="inlineStr">
@@ -52344,7 +51616,7 @@
       </c>
       <c r="G1476" t="inlineStr">
         <is>
-          <t>Grateful Reward: mechanically wirable, scan unavailable for its token. "Reaction: After engaging, choose your performing Samurai at the current battlefield: Create a 1F Ashigaru Cavalry Follower and attach it to him. If he is a Paragon, gain 2 Honor and draw a card" is Nakanu Technique's own after-engaging Creates shape (HostIsPerformer, an at-battle Samurai Performer) plus a Paragon-conditional GainHonor/Draw in its case. The Proxy it creates is Mounted Ashigaru (oracle-l5r-10010, Emperor Edition: 1F, Cavalry/Ashigaru), which is not published: its receipt names only the master scan (no working_copy), the Oracle image host is refused by this sandbox's network policy, and it is not in the local art pack. CreatedCards.Resolve/Verify need a published CreatedOnly scan, so the creator cannot be wired until the Proxy is published.</t>
+          <t>Grateful Reward (issue #503, P6, re-checked): its own scan is local; blocked only by its created 1F Ashigaru Cavalry Follower, the Proxy Mounted Ashigaru (oracle-l5r-10010), which has only a receipt (no working_copy; not in either catalogue WebP pack, l5r-s3 or l5r-emperor) and may not be downloaded in this pass. Otherwise Nakanu Technique's after-engaging HostIsPerformer create plus a Paragon-conditional Honor gain and draw.</t>
         </is>
       </c>
       <c r="H1476" t="inlineStr">
@@ -52793,19 +52065,11 @@
       </c>
       <c r="F1489" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1489" t="inlineStr">
-        <is>
-          <t>Needs to know that a card "was not in play when this Combat Segment began": nothing records when a card entered play (the same gap as oracle-l5r-10335).</t>
-        </is>
-      </c>
-      <c r="H1489" t="inlineStr">
-        <is>
-          <t>PROVENANCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1489" t="inlineStr"/>
+      <c r="H1489" t="inlineStr"/>
     </row>
     <row r="1490">
       <c r="A1490" t="inlineStr">
@@ -53145,19 +52409,11 @@
       </c>
       <c r="F1499" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1499" t="inlineStr">
-        <is>
-          <t>Needs a Family Honor read ("gain 1 Honor, or 3 Honor if your Family Honor is 9 or less") -- every existing Honor-threshold card reads a PERSONALITY's Personal/Family Honor (CardPersonalHonor), never the acting PLAYER's own Family Honor total as a branch condition on the amount gained; PlayerState carries no such stat to compare (Honor and Family Honor are recorded as separate concepts in the core rules' Honor section, and only the card-level one is wired). The bow-and-Honor-comparison performer/target shape itself (an unbowed Samurai bows an enemy with equal-or-lower Personal Honor) is ordinary and ready once that read exists.</t>
-        </is>
-      </c>
-      <c r="H1499" t="inlineStr">
-        <is>
-          <t>HONOR</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1499" t="inlineStr"/>
+      <c r="H1499" t="inlineStr"/>
     </row>
     <row r="1500">
       <c r="A1500" t="inlineStr">
@@ -53731,19 +52987,11 @@
       </c>
       <c r="F1516" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1516" t="inlineStr">
-        <is>
-          <t>Needs "Show the card in the current battlefield's province" as a reactive reveal with a branch on its own type ("if it is a Personality, negate the Melee or Ranged Attack's effects") -- LookSpec (issue #322) peeks the top of a DECK, not a province, and no primitive reveals a province's own face-down card to branch a Reaction's own effect on what it is. The Battle half (discard a card from the current battlefield's province, draw a card) reuses Scavenging Party's own ChoosesOwnProvince shape (issue #420) and is separately wirable, but the two are left together rather than splitting one printed ability.</t>
-        </is>
-      </c>
-      <c r="H1516" t="inlineStr">
-        <is>
-          <t>HIDDEN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1516" t="inlineStr"/>
+      <c r="H1516" t="inlineStr"/>
     </row>
     <row r="1517">
       <c r="A1517" t="inlineStr">
@@ -53846,7 +53094,7 @@
       </c>
       <c r="G1519" t="inlineStr">
         <is>
-          <t>Needs a meta-effect that answers a REACTION with a standing modifier on every OTHER Reaction announced for the rest of the Combat Segment ("after another player announces a Reaction during the Combat Segment: its effects will not negate other effects") -- every existing negation-of-a-negation is a one-shot targeted response to a single held action (Yoritomo Sakuma's own whole-action negation, the redirect family); nothing generalizes to "every reaction from here on, this segment, loses its own negating power," a standing rule change to how negation itself works rather than an effect two cards' worth of primitives could compose.</t>
+          <t>Inexorable (Embers of War): "Reaction: After another player announces a Reaction during the Combat Segment: Its effects will not negate other effects." Re-checked after issue #503. The trigger is now reachable (group P3 built announce windows that ask more than one watcher per announcement, EmperorP3Priority.cs, and the window could be opened for the OTHER player's hand Strategy when the announced action is a Reaction in a Combat Segment), but the effect is not: "its effects will not negate other effects" needs one engine-wide notion of 'a negation made by this action's effects' that can be switched off for one resolving action. Negations live in a dozen unrelated places -- MatchState.NegatedEffects (per card and kind), the whole-action flags (DeferredActionNegated, PendingAttack.Negated, AnnouncedActionNegated, RemANegatesHeldAction, HeldProclaim.Negated, the P3 Event negation), standing card fields that negate later effects (StraightenHolds, MovementLocks, TargetShield, ForceModifiersNegatedTurn, Stalwart-style per-turn stamps), the R4 Honor marks (RemC.NegateLossesActionKey, HonorReducedActionKey, P3 NegatedHonorGains), Fujita's Follower shields and the delay store's negated entries -- and no action records which of them it set. A snapshot-and-revert of a hand-picked list would silently miss the rest, so the card would be partial. Needs: a single NegationLedger that every negation writes through (kind, target, source action key), so an action marked 'non-negating' (Inexorable) has its entries dropped as it resolves; then Inexorable is an announce-window Reaction of the other player that marks the announced Reaction's key.</t>
         </is>
       </c>
       <c r="H1519" t="inlineStr">
@@ -54227,19 +53475,11 @@
       </c>
       <c r="F1530" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1530" t="inlineStr">
-        <is>
-          <t>Needs a Reaction to a Battle action targeting your Paragon that ignores the action's costs and negates its effects retroactively, and gives "that player" an additional Battle action: costs already paid are not unpaid, and an additional action is granted to the acting player only.</t>
-        </is>
-      </c>
-      <c r="H1530" t="inlineStr">
-        <is>
-          <t>TRIG-ANN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1530" t="inlineStr"/>
+      <c r="H1530" t="inlineStr"/>
     </row>
     <row r="1531">
       <c r="A1531" t="inlineStr">
@@ -54371,19 +53611,11 @@
       </c>
       <c r="F1534" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1534" t="inlineStr">
-        <is>
-          <t>Needs a Focus Effect that lets a duel's own STAT SUBSTITUTION be chosen live at focus time ("you may choose now to use the base Force of your Personality in this duel as his duel stat if he is at a battlefield") -- AbilityDefinition.DuelStat is fixed per ability at catalog-definition time (Chi/Force/PersonalHonor), read once when the duel is issued; a Focus Effect that retroactively swaps which stat the SAME ongoing duel compares has no existing hook (Dueling.cs computes DuelStatValue from the duel's own fixed Stat field throughout ResolveDuel). Its Battle half (straighten a performing Personality, optionally move him home) is ordinary and separately wirable.</t>
-        </is>
-      </c>
-      <c r="H1534" t="inlineStr">
-        <is>
-          <t>DUEL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1534" t="inlineStr"/>
+      <c r="H1534" t="inlineStr"/>
     </row>
     <row r="1535">
       <c r="A1535" t="inlineStr">
@@ -54689,19 +53921,11 @@
       </c>
       <c r="F1543" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1543" t="inlineStr">
-        <is>
-          <t>Learning. Three gaps: (a) a Battle Strategy in ANOTHER player's discard pile played by its non-owner (the FromDiscard additional-action grant, AbilitySourceZoneAllows and AbilityIdsOf all read the source's own controller; nothing lets a player play an opponent's card from the opponent's pile, then remove it from the game); (b) "its abilities may be used an additional time this turn" -- a per-card raise of the per-turn use limit (AbilityDefinition.UsesPerTurn is data on the ability, and the once-per-turn stamp lives on the card; no per-instance override exists); (c) the keyword copy ("copies a keyword on an enemy Personality") is CardCopy.cs's copyKeyword step and IS buildable. The performer half is ordinary.</t>
-        </is>
-      </c>
-      <c r="H1543" t="inlineStr">
-        <is>
-          <t>ZONE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1543" t="inlineStr"/>
+      <c r="H1543" t="inlineStr"/>
     </row>
     <row r="1544">
       <c r="A1544" t="inlineStr">
@@ -56171,19 +55395,11 @@
       </c>
       <c r="F1586" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1586" t="inlineStr">
-        <is>
-          <t>Unchanged: a Reaction to an announced Battle action before the Defender's first opportunity, and 'after the next time you lose Honor from another player's card effect' (a watch on a future Honor loss, not a delayed effect on a card). NO LOCAL SCAN.</t>
-        </is>
-      </c>
-      <c r="H1586" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1586" t="inlineStr"/>
+      <c r="H1586" t="inlineStr"/>
     </row>
     <row r="1587">
       <c r="A1587" t="inlineStr">
@@ -56931,19 +56147,11 @@
       </c>
       <c r="F1608" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1608" t="inlineStr">
-        <is>
-          <t>Refreshed: "destroy this whole unit before the turn ends" is now one call (ScheduleDelayedEffect(card, DelayedKinds.Destroy, DelayUntil.EndOfTurn, ...), as In the Heart of Battle does); the remaining gap is the one-time Force bonus per card EQUAL TO ITS OWN CURRENT FORCE applied to every Personality and Follower of a unit at once. NO LOCAL SCAN.</t>
-        </is>
-      </c>
-      <c r="H1608" t="inlineStr">
-        <is>
-          <t>SCAN2</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1608" t="inlineStr"/>
+      <c r="H1608" t="inlineStr"/>
     </row>
     <row r="1609">
       <c r="A1609" t="inlineStr">
@@ -56973,19 +56181,11 @@
       </c>
       <c r="F1609" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1609" t="inlineStr">
-        <is>
-          <t>Re-verified for the Embers of War pass (issue #460): its Reaction ("after another player's action targets your Personality: Discard him") is expressible through the targeted-by-action trigger (issue #335, played from hand). Its Battle half is still blocked: "Create a 1F/1C/1PH Monk Personality on your side there. Remove him from the game when the turn ends" -- CreatedCardSpec's own token-removal shape (UntilBattleEnds, e.g. Meddling Mob's Scout) only removes a created card when its BATTLE ends, not at the end of the TURN; those differ whenever the created card's own battle resolves before the turn does (a later battle, or the Action Phase). No UntilTurnEnds variant exists yet, and adding one touches the turn-transition code path (FinishTurn) rather than a self-contained ability primitive, so it is left for a dedicated pass rather than bolted on for one card.</t>
-        </is>
-      </c>
-      <c r="H1609" t="inlineStr">
-        <is>
-          <t>CREATE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1609" t="inlineStr"/>
+      <c r="H1609" t="inlineStr"/>
     </row>
     <row r="1610">
       <c r="A1610" t="inlineStr">
@@ -57015,19 +56215,11 @@
       </c>
       <c r="F1610" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1610" t="inlineStr">
-        <is>
-          <t>Petty Squabbles. Its Limited half, "Target one or two face-down cards in provinces: Turn them face-up", cannot be offered without leaking hidden information: every target/slot names a card by CardInstance.Id, and those ids are assigned sequentially in deck-list order at setup (MatchEngine/PublishedMatch "card-NNNN"), so listing a face-down province card's real id in QueryActions would reveal which card it is -- MatchQueries.ViewCard deliberately shows a face-down province card as "hidden-p{owner}-province{n}" instead. The province-addressed alternative (Target any-province: TargetPlayerId + Province) names ONE province, and SlotSelection carries only CardIds or a PlayerId, so "one or two" provinces of any player is not expressible; SlotCandidateCards never lists province cards either. (Turning a Celestial face-up would also have to enter it into play through ResolveCelestial.) Its Battle/Open half, "Target an attachment owned by another player: He may pay 4 Gold. If he did not, return it to its owner's hand", is wirable as an EitherOr spec (Yasuki Makoto's owner-decides pay-4-Gold shape); the card is kept whole.</t>
-        </is>
-      </c>
-      <c r="H1610" t="inlineStr">
-        <is>
-          <t>HIDDEN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1610" t="inlineStr"/>
+      <c r="H1610" t="inlineStr"/>
     </row>
     <row r="1611">
       <c r="A1611" t="inlineStr">
@@ -57129,19 +56321,11 @@
       </c>
       <c r="F1613" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1613" t="inlineStr">
-        <is>
-          <t>Needs a conditional SECOND TARGET, chosen only when the first (its own performer) satisfies a status ("Give your target performing unbowed Tattooed Monk +3F. If he is Earth, you may target and bow an enemy card without attachments") -- TargetSlot's own conditional follow-up shape (Resolution/ConditionalChoice, issue #336-#337: Doji Yoshitada's "if dishonorable, a player gains/loses Honor," Fear Me!'s "if he moved") only offers a fixed EffectOption menu at resolution, never an open CARD selection; a follow-up slot that is itself a real Target category (picking any legal enemy card, not choosing among a few named effects) does not exist yet.</t>
-        </is>
-      </c>
-      <c r="H1613" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1613" t="inlineStr"/>
+      <c r="H1613" t="inlineStr"/>
     </row>
     <row r="1614">
       <c r="A1614" t="inlineStr">
@@ -57269,19 +56453,11 @@
       </c>
       <c r="F1617" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1617" t="inlineStr">
-        <is>
-          <t>Needs a Gold-Cost comparison Target category (same gap as oracle-l5r-24).</t>
-        </is>
-      </c>
-      <c r="H1617" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1617" t="inlineStr"/>
+      <c r="H1617" t="inlineStr"/>
     </row>
     <row r="1618">
       <c r="A1618" t="inlineStr">
@@ -57379,19 +56555,11 @@
       </c>
       <c r="F1620" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1620" t="inlineStr">
-        <is>
-          <t>Needs a keyword-COUNT comparison Target category, excluding a named pattern ("an enemy Personality with fewer keywords, ignoring 'Soul of' keywords" than the performer) -- every existing keyword check is membership (HasKeywords/Keyword: does a card carry keyword X), never a COUNT of a card's own total keywords compared against another card's count, and Yoritomo Emiko's own "count this card's own keywords" gap (oracle-l5r-5444, recorded above) is the same missing primitive with no exclusion pattern on top.</t>
-        </is>
-      </c>
-      <c r="H1620" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1620" t="inlineStr"/>
+      <c r="H1620" t="inlineStr"/>
     </row>
     <row r="1621">
       <c r="A1621" t="inlineStr">
@@ -58076,7 +57244,7 @@
       </c>
       <c r="G1640" t="inlineStr">
         <is>
-          <t>Regret. Its Focus Effect ("After this duel ends, its winner's controller loses 1 Honor for each card he focused") is wirable as an ApplyDuelFocusEffect arm (the winner's side's focused list is on PendingDuel), but its Open half is not: "Target one or more Followers or Items in your discard pile: Attach them to any of your Personalities, paying all costs" attaches SEVERAL cards, each to a Personality of the player's choice, each paying its own Gold Cost. AttachAction.cs (AttachSpec/ExecuteAttach, Moto Jun-Ni's shape) attaches exactly one card per command to one wielder fixed by the ability (source, performer or a PersonalitySlot), and the Gold is paid once, up front, for that one card (GoldCostRule.AttachCost). The multi-target slots (TargetSlots.cs) can name the one-or-more cards but carry no card-to-host pairing, and a host chosen at resolution cannot be priced up front: an equip's price depends on its host (EquipGoldCost's per-host discounts) while a resolution-time choice (EffectChoice.cs) carries no Gold payment of its own. Needs a per-card host choice with a per-card payment, which is the Ivory-era "Equip" sequence repeated N times; not built small.</t>
+          <t>Regret (re-verified in issue #503, group P4). Its Focus Effect ("After this duel ends, its winner's controller loses 1 Honor for each card he focused") is one ApplyDuelFocusEffect arm (the winner's side's focused list is on PendingDuel), and the target half is now expressible: an up-front slot of one or more Followers/Items in the acting player's discard pile plus a Repeatable "hosts" slot paired by position (Suiteiru no Oni's Repeatable slot), priced by a new GoldCostRule basis summing EquipGoldCost per (attachment, host) pair. What is still missing is SEVERAL CARDS ENTERING PLAY IN ONE RESOLUTION: ExecuteAttach puts one card into play and opens OpenEntryReactionWindow for it, which pauses the action and has no queue -- a second attachment would either skip its own entry Reactions (only ApplyMandatoryEntryEffects) or never be attached. Needs an entering-play queue (each attached card's entry window opened in turn, the action finishing after the last), plus a combined legality check across the pairs (two Weapons or Armors to one host, two copies of a Unique/Singular card). Not published: a partial card is never published.</t>
         </is>
       </c>
       <c r="H1640" t="inlineStr">
@@ -58249,19 +57417,11 @@
       </c>
       <c r="F1645" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1645" t="inlineStr">
-        <is>
-          <t>Its Battle half ("Bow your performing Courtier at any location and target a Personality: Move him home") is now wirable, the personality-at-any-location Target category (Tsuruchi Nobukatsu) plus own-unbowed-personality-with-keyword-at-any-location Performer already covering it. Its Reaction half needs a genuinely new timing: "Before another player's Battle action resolves, target a Personality: Negate his movement to the current battlefield from the action's effects" is a pre-resolution INTERRUPT that can target any Personality the action would move, not only the action's own target -- every existing negation Reaction (ReactionTriggers.TargetedByAction, AfterActionResolved) fires either after the action targets a specific card or after it has already resolved, never before an arbitrary action resolves against an untargeted card. Unsafe Passage (oracle-l5r-9008) needs the identical Interrupt primitive.</t>
-        </is>
-      </c>
-      <c r="H1645" t="inlineStr">
-        <is>
-          <t>TRIG-ANN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1645" t="inlineStr"/>
+      <c r="H1645" t="inlineStr"/>
     </row>
     <row r="1646">
       <c r="A1646" t="inlineStr">
@@ -58563,19 +57723,11 @@
       </c>
       <c r="F1654" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1654" t="inlineStr">
-        <is>
-          <t>Needs a "move a whole in-play unit's cards to the bottom of their owners' decks, in chosen order" primitive: "Put all cards in the target's unit at the bottom of his owner's appropriate decks in any order" moves the target Personality AND his attachments, splitting them by card type (Personality to the Dynasty deck, Fate cards to the Fate deck) and letting the acting player choose the order within each. The existing deck primitives (DeckSearch, DeckLook/LookSpec) only ever move a card FROM a deck the ability is already searching or peeking, never an in-play unit TO the bottom of a deck.</t>
-        </is>
-      </c>
-      <c r="H1654" t="inlineStr">
-        <is>
-          <t>ZONE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1654" t="inlineStr"/>
+      <c r="H1654" t="inlineStr"/>
     </row>
     <row r="1655">
       <c r="A1655" t="inlineStr">
@@ -58605,19 +57757,11 @@
       </c>
       <c r="F1655" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1655" t="inlineStr">
-        <is>
-          <t>Not a delay of an action's effects: "negate the Personality's (future) movement" is a standing negation of a FUTURE action, which the delay store does not model (it records effects that already happened in the running action). It is the same gap as before (a watch that negates a card's next movement), now with the shape of Paralyzing Touch's watch (MatchState.ParalyzingTouchWatches) as the closest precedent. NO LOCAL SCAN.</t>
-        </is>
-      </c>
-      <c r="H1655" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1655" t="inlineStr"/>
+      <c r="H1655" t="inlineStr"/>
     </row>
     <row r="1656">
       <c r="A1656" t="inlineStr">
@@ -58987,19 +58131,11 @@
       </c>
       <c r="F1666" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1666" t="inlineStr">
-        <is>
-          <t>Needs "until the game ends, after each time it bows or an ability on it resolves, its controller loses 1 Honor": the only such watch is Tsujiken's on a bow (TsujikenWatches, hard-wired), and it is not a general "after an ability on it resolves" trigger.</t>
-        </is>
-      </c>
-      <c r="H1666" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1666" t="inlineStr"/>
+      <c r="H1666" t="inlineStr"/>
     </row>
     <row r="1667">
       <c r="A1667" t="inlineStr">
@@ -59097,19 +58233,11 @@
       </c>
       <c r="F1669" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1669" t="inlineStr">
-        <is>
-          <t>Needs a "look at cards in another player's HAND" primitive: "Choose and look at two cards in the Defender's hand" exposes hidden information from an opponent's hand to the acting player, which nothing in the engine does today (LookSpec peeks a DECK; every other "look" reads an already-public zone). The Reconnaissance-grant-plus-first-Battle-action-priority half ("You have Reconnaissance there. You have the first chance to take a Battle action in this battle") already has a proven shape, Daidoji Yuki's yuki-engage-recon (issue #309), and is separately wirable.</t>
-        </is>
-      </c>
-      <c r="H1669" t="inlineStr">
-        <is>
-          <t>HIDDEN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1669" t="inlineStr"/>
+      <c r="H1669" t="inlineStr"/>
     </row>
     <row r="1670">
       <c r="A1670" t="inlineStr">
@@ -59139,19 +58267,11 @@
       </c>
       <c r="F1670" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1670" t="inlineStr">
-        <is>
-          <t>Needs a temporary Recruit that auto-discards when the current battle ends: "you may Recruit him, ignoring Gold cost... Discard him after the battle ends" combines the existing Absent-Battle timing (issue #362) and the ordinary Recruit action with a scheduled discard keyed to the battle's own resolution, which no existing primitive threads together (AfterBattleResolution reactions fire from a card already in play or a pile, not as a teardown of a card this same ability just recruited). Its Focus Effect ("if your Personality won it, gain 1 Honor") is a plain, unconditional post-duel Honor gain and would be trivial once the Absent-Battle half exists to give the card a reason to ship.</t>
-        </is>
-      </c>
-      <c r="H1670" t="inlineStr">
-        <is>
-          <t>CREATE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1670" t="inlineStr"/>
+      <c r="H1670" t="inlineStr"/>
     </row>
     <row r="1671">
       <c r="A1671" t="inlineStr">
@@ -59181,19 +58301,11 @@
       </c>
       <c r="F1671" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1671" t="inlineStr">
-        <is>
-          <t>Needs a per-item transfer-TARGET mapping when several attachments are chosen at once: "Target one or more of your Items: Straighten them. You may transfer them to other Personalities you control" lets each of several chosen Items move to a different, independently chosen new wielder in the same action. The existing Transfer primitive (AttachmentTransfers.cs, issues #435/#453) pairs exactly one attachment with exactly one destination slot; a Slots ability whose slot selections name a card-to-card mapping, not just a set, is not built. Its Focus Effect ("+1C to each Weapon attached to your Personality in this duel", unconditional, no choice) is separately wirable now.</t>
-        </is>
-      </c>
-      <c r="H1671" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1671" t="inlineStr"/>
+      <c r="H1671" t="inlineStr"/>
     </row>
     <row r="1672">
       <c r="A1672" t="inlineStr">
@@ -59223,19 +58335,11 @@
       </c>
       <c r="F1672" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1672" t="inlineStr">
-        <is>
-          <t>Needs a self-replacing same-KEYWORD-in-play primitive: "Put this card into play. Discard all your other Kata (in play)" discards every other card the controller has in play that carries the printed Kata keyword, not just one Terrain at the same battlefield (the engine's only self-replacing precedent, e.g. Ancient Feud) -- a broader, board-wide sweep by shared keyword rather than a single like-for-like swap at one location. Its other Limited ability ("If this card is in play: Look at the top card of any deck. You may put it at the bottom of that deck") is a plain LookSpec (issue #322) and is separately wirable.</t>
-        </is>
-      </c>
-      <c r="H1672" t="inlineStr">
-        <is>
-          <t>SMALL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1672" t="inlineStr"/>
+      <c r="H1672" t="inlineStr"/>
     </row>
     <row r="1673">
       <c r="A1673" t="inlineStr">
@@ -59809,19 +58913,11 @@
       </c>
       <c r="F1689" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1689" t="inlineStr">
-        <is>
-          <t>Half of it exists: negating current Force penalties is NegateForcePenalties (Tireless Efforts). Needs "if he has a Weapon, negate the next card effect that moves him home or bows him": a one-shot protection against a kind of effect that persists until used (Protections are all-or-nothing for the turn).</t>
-        </is>
-      </c>
-      <c r="H1689" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1689" t="inlineStr"/>
+      <c r="H1689" t="inlineStr"/>
     </row>
     <row r="1690">
       <c r="A1690" t="inlineStr">
@@ -60565,19 +59661,11 @@
       </c>
       <c r="F1711" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1711" t="inlineStr">
-        <is>
-          <t>Buildable as a Spirit (GrantSpirit) except its granted ability, "Ninja Battle: Target two Personalities controlled by the same player at different locations: Switch their locations": nothing swaps the locations of two Personalities.</t>
-        </is>
-      </c>
-      <c r="H1711" t="inlineStr">
-        <is>
-          <t>EFFECT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1711" t="inlineStr"/>
+      <c r="H1711" t="inlineStr"/>
     </row>
     <row r="1712">
       <c r="A1712" t="inlineStr">
@@ -61937,19 +61025,11 @@
       </c>
       <c r="F1751" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1751" t="inlineStr">
-        <is>
-          <t>Needs a battle-scoped Ranged Attack strength bonus: "Ranged Attacks from your card effects during this battle have +2 strength" is an ongoing modifier to every Ranged Attack the controller's cards make for the rest of the current battle, which no existing primitive tracks (Attack strength today is either the ability's own printed number or a per-card static bonus, never a battle-wide buff applying to attacks not yet announced). The Reconnaissance-grant half ("After engaging, choose your performing unbowed Scout at the current battlefield: You have Reconnaissance there") is Daidoji Yuki's own proven shape and is separately wirable.</t>
-        </is>
-      </c>
-      <c r="H1751" t="inlineStr">
-        <is>
-          <t>STAT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1751" t="inlineStr"/>
+      <c r="H1751" t="inlineStr"/>
     </row>
     <row r="1752">
       <c r="A1752" t="inlineStr">
@@ -61984,7 +61064,7 @@
       </c>
       <c r="G1752" t="inlineStr">
         <is>
-          <t>Sword for Hire. "Create a 0F/3C/0PH Assassin • Duelist Personality" is the Embers of War Proxy oracle-l5r-9995 (the orphan Proxy recorded there -- this is its creator), and CreatedCards.Resolve needs that Proxy published as a CreatedOnly scan: its scan is not in this sandbox (assets/reference/oracle/embers-of-war holds receipts only), so neither card can be packaged here. Once the Proxy is published the rest is buildable: Creates (a Personality at home), IssueChallenge (Dueling.cs) with the created card as the challenger and DuelRefusable false, a "destroy the duel's loser" outcome, and a new small hook removing the created challenger from the game when its duel ends (CreatedUntilBattleEndsIds is battle-scoped; this is duel-scoped).</t>
+          <t>Sword for Hire (issue #503, P6, re-checked): its own scan is local; blocked by its created 0F/3C/0PH Assassin Duelist Personality, the Proxy Assassin (oracle-l5r-9995), which has only a receipt (no working_copy; not in either catalogue WebP pack, l5r-s3 or l5r-emperor) and may not be downloaded in this pass. Once published, still needed: a duel-scoped removal of the created challenger when its duel ends (CreatedUntilBattleEndsIds is battle-scoped; MechDState.TimedRemovals covers turn end / next turn only) and the 'destroy the duel's loser' outcome (both small).</t>
         </is>
       </c>
       <c r="H1752" t="inlineStr">
@@ -62361,19 +61441,11 @@
       </c>
       <c r="F1763" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1763" t="inlineStr">
-        <is>
-          <t>Needs an ability granted to EVERY PLAYER at once, not one card's controller: "All players have the ability, 'Open: Bow your Stronghold: Discard a card titled The Bite of Winter from play'" -- GrantAbility (AbilityGrants.cs) and the static per-controller grant shape (StaticGrantedAbilityIds, The Towers of the Yogo) both reach only cards of ONE player; nothing reaches both players' Strongholds from a single in-play Strategy. The accompanying "Personalities and Followers have -1F" (both sides, board-wide, while this card is in play) is the ordinary static-modifier shape several other in-play Strategies already use and would be trivial once the shared-ability gap is closed.</t>
-        </is>
-      </c>
-      <c r="H1763" t="inlineStr">
-        <is>
-          <t>GRANT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1763" t="inlineStr"/>
+      <c r="H1763" t="inlineStr"/>
     </row>
     <row r="1764">
       <c r="A1764" t="inlineStr">
@@ -63431,19 +62503,11 @@
       </c>
       <c r="F1794" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1794" t="inlineStr">
-        <is>
-          <t>Needs the opposing player's offer to "show you his hand" (hidden information the acting player may ask for), a discard from it chosen by the acting player, and a lock on the rulebook seppuku action for that Personality.</t>
-        </is>
-      </c>
-      <c r="H1794" t="inlineStr">
-        <is>
-          <t>HIDDEN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1794" t="inlineStr"/>
+      <c r="H1794" t="inlineStr"/>
     </row>
     <row r="1795">
       <c r="A1795" t="inlineStr">
@@ -63643,19 +62707,11 @@
       </c>
       <c r="F1800" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1800" t="inlineStr">
-        <is>
-          <t>Not a delay of an action's effects: "negate the next effect that would move one of your Personalities from its battlefield" and "after the next time this battle a Terrain enters play, destroy it" are one-shot watches on FUTURE events within the battle, unchanged by the delay mechanism. NO LOCAL SCAN.</t>
-        </is>
-      </c>
-      <c r="H1800" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1800" t="inlineStr"/>
+      <c r="H1800" t="inlineStr"/>
     </row>
     <row r="1801">
       <c r="A1801" t="inlineStr">
@@ -64267,19 +63323,11 @@
       </c>
       <c r="F1818" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1818" t="inlineStr">
-        <is>
-          <t>Needs an unconditional acting-player choice between two DIFFERENT effect shapes on two different subjects: "Bow him or destroy one of his attachments" is a free choice (not a Yumaru-style conditional Branch, which only offers a choice when a board-state condition holds) between bowing the target Personality outright and destroying an attachment on him that must itself be chosen if he has more than one -- combining an unconditional either/or with a second, only-sometimes-needed target selection is not expressible with either EitherOr.cs (built for the OPPOSING player's decisions) or ConditionalChoice (built for board-state-gated branches).</t>
-        </is>
-      </c>
-      <c r="H1818" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1818" t="inlineStr"/>
+      <c r="H1818" t="inlineStr"/>
     </row>
     <row r="1819">
       <c r="A1819" t="inlineStr">
@@ -64547,19 +63595,11 @@
       </c>
       <c r="F1826" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1826" t="inlineStr">
-        <is>
-          <t>Turning Away. Its Battle half is buildable now (Absent, a Monk performer at any location -- own-unbowed-personality-with-keyword-at-any-location -- bowing a target Ring as the cost, and Ring of Earth's +3/-3 province-strength choice on the current battlefield's province), but its Focus Effect, "You may discard your Personality in this duel (ending the duel without resolution)", needs a duel that ends WITHOUT resolving: in this engine the Focus Effects of a duel are applied after ResolveDuel has already computed the winner and applied the outcome (Dueling.cs), so there is no point at which a Focus Effect can discard a duelist and stop the resolution. Left unwired until a pre-resolution Focus Effect stage exists.</t>
-        </is>
-      </c>
-      <c r="H1826" t="inlineStr">
-        <is>
-          <t>DUEL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1826" t="inlineStr"/>
+      <c r="H1826" t="inlineStr"/>
     </row>
     <row r="1827">
       <c r="A1827" t="inlineStr">
@@ -64793,19 +63833,11 @@
       </c>
       <c r="F1833" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1833" t="inlineStr">
-        <is>
-          <t>Two-Fold Virtue (re-verified). A partial copy with computed Force: "Create a Personality with the same base Chi, Personal Honor and keywords as the target, and whose base Force equals that target's Personal Honor. Remove the Personality from the game after the battle ends." Created per-instance values exist (CreatedCardSpec.Values / CreatedValue, issue #402) and removal after the battle exists (UntilBattleEnds, issue #394), but CreatedStat (CreatedCards.cs) covers Name, GoldCost, Force, Chi and PersonalHonor only -- copying a keyword SET is not built (CopyOfTarget copies the whole card, not these three values) -- and no generic created-Personality Proxy scan exists for CreatedCards.Resolve to fit (every created Personality names its own printed Proxy). Rulings needed from Mendon: where the Personality is created (home or the current battlefield; the Glossary's default is home) and which scan represents it.</t>
-        </is>
-      </c>
-      <c r="H1833" t="inlineStr">
-        <is>
-          <t>CREATE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1833" t="inlineStr"/>
+      <c r="H1833" t="inlineStr"/>
     </row>
     <row r="1834">
       <c r="A1834" t="inlineStr">
@@ -65387,19 +64419,11 @@
       </c>
       <c r="F1850" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1850" t="inlineStr">
-        <is>
-          <t>Its Open half needs two things: where a Ring's last entry into play came from ("a Ring which did not last enter play by its own text" -- the engine puts a Ring into play only through its own recruit ability, so no provenance is recorded and today no Ring could ever qualify), and a permanent removal of a card's abilities (ActionLock lasts a turn or a phase; nothing blanks a card's printed abilities for the game). Buildable now: its Limited half ("target one or more cards in your provinces: discard them" is the provinces Target; "refill the provinces face-up from the bottom of your deck" needs only a bottom-of-deck variant of Refill, which is top-of-deck today).</t>
-        </is>
-      </c>
-      <c r="H1850" t="inlineStr">
-        <is>
-          <t>PROVENANCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1850" t="inlineStr"/>
+      <c r="H1850" t="inlineStr"/>
     </row>
     <row r="1851">
       <c r="A1851" t="inlineStr">
@@ -65944,7 +64968,7 @@
       </c>
       <c r="G1866" t="inlineStr">
         <is>
-          <t>Wanted for Questioning. "Your Magistrate takes him into custody" is a mechanic docs/rules/EMPEROR_EDITION_CORE_RULES.md does not define (no Glossary entry for custody; grep finds none) and the engine has no representation of (no custody state, zone or link in Models.cs) -- what custody does, how long it lasts and how it ends has no rules source here, so it cannot be wired consistently with the core rules. The rest is ordinary (an unbowed Magistrate Performer, own-unbowed-personality-at-battle-with-keyword; "if he is dishonorable, destroy his attachments"; MoveHome); the card is kept whole.</t>
+          <t>Wanted for Questioning (issue #503, P6, re-checked against its scan): 'Battle: Choose your performing unbowed Magistrate and target an enemy Personality: Your Magistrate takes him into custody. If he is dishonorable, destroy his attachments. Move him home.' 'Custody' is still undefined: docs/rules/EMPEROR_EDITION_CORE_RULES.md has no entry for it (grep finds none) and the engine has no custody state. Rules-lane question for Mendon: is 'takes him into custody' flavour (then the card is buildable at once: an unbowed-Magistrate performer at the battle, an enemy-personality target, destroy his attachments if dishonorable, MoveHome), or a mechanic (what it does, how long it lasts, how it ends)?</t>
         </is>
       </c>
       <c r="H1866" t="inlineStr">
@@ -66321,19 +65345,11 @@
       </c>
       <c r="F1877" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1877" t="inlineStr">
-        <is>
-          <t>Needs a "highest Chi among all Shugenja and Courtiers you control" aggregate-stat lookup: "an enemy card with Force lower than your Yojimbo's Force plus the highest Chi among all Shugenja and Courtiers you control" computes a per-action comparison value from the single highest PersonalityChi() across two keyword groups board-wide, which no existing Target category does (every existing performer-relative comparison, e.g. enemy-personality-chi-lte-performer, reads only the CHOSEN PERFORMER's own stat, never an aggregate over other cards the player merely controls).</t>
-        </is>
-      </c>
-      <c r="H1877" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1877" t="inlineStr"/>
+      <c r="H1877" t="inlineStr"/>
     </row>
     <row r="1878">
       <c r="A1878" t="inlineStr">
@@ -68166,7 +67182,7 @@
       </c>
       <c r="G1931" t="inlineStr">
         <is>
-          <t>Humble Farm: mechanically wirable, scan unavailable for its token. "Bow this card: Produce 2 Gold" is GoldProduction 2 and "Battle/Open: Destroy this card and target your Personality: Create a 2F Ashigaru Follower and attach it to him" is Ashigaru Recruits' own create-and-attach shape (CreatedCardSpec(Follower, Force: 2, Keywords: [Ashigaru]) on a BattleOrOpen ability with Costs [CostVerbs.Sacrifice] and target own-personality). Blocked because CreatedCards.Resolve needs a published CreatedOnly Proxy scan that fits a plain 2F Ashigaru Follower, and none exists anywhere in this checkout (Fledgling Ashigaru oracle-l5r-9713 is 0F, Mounted Ashigaru oracle-l5r-10010 is 1F Cavalry and unpublished, Ronin Follower oracle-l5r-10203 is 2F Ronin); the Oracle image host is blocked by the sandbox's network policy. Wire it with its token once that Proxy's scan is fetched and published.</t>
+          <t>Humble Farm (issue #503, P6, re-checked): its own scan is local; blocked only by its created plain 2F Ashigaru Follower. No local Proxy fits (Fledgling Ashigaru is 0F, Mounted Ashigaru 1F Cavalry with no local scan, Ronin Follower 2F Ronin, Infantry Follower 2F with no keyword); docs/requests/created-card-scans-needed.md row B3 (ashigaru-2f.jpg) is unticked. Otherwise GoldProduction 2 plus Ashigaru Recruits' Battle/Open create-and-attach with a Sacrifice cost.</t>
         </is>
       </c>
       <c r="H1931" t="inlineStr">
@@ -69661,19 +68677,11 @@
       </c>
       <c r="F1975" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1975" t="inlineStr">
-        <is>
-          <t>Needs a "Set a Province's strength to 0" effect: ProvinceStrengthEffects/ProvinceState.Strength only ever ADD or subtract a timed/permanent bonus (Incriminating Testimony, Ancient Feud's cap, Times of Strife's ceiling); nothing sets a province's strength to an absolute value, which "lower a target Province's strength to 0" needs (a straight subtraction is wrong once other bonuses/penalties are stacked -- Set, per the core rules Glossary, means "give a stat a bonus/penalty sufficient to reach the stated value", not merely subtract). The conditional production half (":bow:: Produce 2 Gold, or 3 Gold if you control a Tactician") is buildable with ConditionalProduction.cs (a new ProductionCondition.ControllingKeyword case, distinct from PayingForKeyword: this checks the PLAYER's board state at production time, not what the Gold is being spent on).</t>
-        </is>
-      </c>
-      <c r="H1975" t="inlineStr">
-        <is>
-          <t>EFFECT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1975" t="inlineStr"/>
+      <c r="H1975" t="inlineStr"/>
     </row>
     <row r="1976">
       <c r="A1976" t="inlineStr">
@@ -70043,19 +69051,11 @@
       </c>
       <c r="F1986" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1986" t="inlineStr">
-        <is>
-          <t>Needs a Holding that copies another player's Holding: "copies one of its printed abilities that does not itself copy abilities, one of its Gold-producing traits, or its Gold Production stat". Permanent copying is built for Personalities and Spells (PermanentCopy.cs), not Holdings, and a Holding's stat is not copyable.</t>
-        </is>
-      </c>
-      <c r="H1986" t="inlineStr">
-        <is>
-          <t>CREATE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1986" t="inlineStr"/>
+      <c r="H1986" t="inlineStr"/>
     </row>
     <row r="1987">
       <c r="A1987" t="inlineStr">
@@ -72061,19 +71061,11 @@
       </c>
       <c r="F2045" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2045" t="inlineStr">
-        <is>
-          <t>Needs a permanent per-province mark ("choose a Province. Permanently give it -2 strength ... Until the game ends, after a Region attaches to it, destroy the Region, and after a Holding enters play from it, give the Holding a -1GP token"): a province-level state that survives the Event (ProvinceState has no such record), a choice of province at reveal (Harsh Choices' PendingChoice shape, now also used by Tested Land and Offering Reverence), a hook in AttachRegionToProvince and one where a Holding leaves a province to enter play, and a Gold-production token on a Holding (CardToken carries Force/Chi/Honor stats; GoldProduced reads no tokens). The immediate halves (-2 strength: province.Strength -= 2; destroy the attached Region: DestroyRegion) are ordinary.</t>
-        </is>
-      </c>
-      <c r="H2045" t="inlineStr">
-        <is>
-          <t>PROVINCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2045" t="inlineStr"/>
+      <c r="H2045" t="inlineStr"/>
     </row>
     <row r="2046">
       <c r="A2046" t="inlineStr">
@@ -72239,19 +71231,11 @@
       </c>
       <c r="F2050" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2050" t="inlineStr">
-        <is>
-          <t>Distant Expansion (Event): "Until your third turn from now ends, you have the trait, 'In your Dynasty Phase, one time for each of your provinces destroyed this game, you may refill one of your provinces face-up.'" Conflicts with the core rules' province model (Setting Up the Game, 8): a province holds one card and is refilled immediately, face down, whenever it has none; it is only ever empty when the Dynasty deck is, and then it cannot be refilled at all. So under Emperor rules the granted trait has no legal object: 'refill' an occupied province is undefined (the card assumes the later Ivory Edition rule that a province may hold several cards). Not wired: publishing it would either do nothing or invent an undefined 'refill an occupied province' rule.</t>
-        </is>
-      </c>
-      <c r="H2050" t="inlineStr">
-        <is>
-          <t>PROVINCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2050" t="inlineStr"/>
+      <c r="H2050" t="inlineStr"/>
     </row>
     <row r="2051">
       <c r="A2051" t="inlineStr">
@@ -72417,19 +71401,11 @@
       </c>
       <c r="F2055" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2055" t="inlineStr">
-        <is>
-          <t>Needs a "Strategy with a Political ability" search criterion: SearchCriteria filters by a card's own Type/Keywords/Clan, never by whether one of its printed Abilities carries a given ActionKeywords tag (Political is recorded per-ability, e.g. jakuei-favor's ActionKeywords: ["Political"], not per-card) -- "search your Fate deck for a non-Unique Strategy with a Political ability" needs a new criterion cross-referencing CardDefinition.Abilities against AbilityCatalog.All's ActionKeywords, which DeckSearch.cs's SearchCriteria has no case for.</t>
-        </is>
-      </c>
-      <c r="H2055" t="inlineStr">
-        <is>
-          <t>SEARCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2055" t="inlineStr"/>
+      <c r="H2055" t="inlineStr"/>
     </row>
     <row r="2056">
       <c r="A2056" t="inlineStr">
@@ -72493,19 +71469,11 @@
       </c>
       <c r="F2057" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2057" t="inlineStr">
-        <is>
-          <t>Needs a global Gold Cost FLOOR applied to every Holding in and out of play ("until the game ends, Holdings in and out of play have a minimum Gold Cost of 1"): CardGoldCost/Definition(card).GoldCost have no live-modifier pipeline at all today (unlike Force/Chi's StatModifier or a province's Strength effects) -- there is nowhere to hook a floor, and it must apply even to cards never in play (a Holding still in a deck or discard pile), which no existing per-card-instance mechanism reaches. The immediate destruction half ("destroy all non-Unique Holdings with a printed Gold Cost of 0") is ordinary and would need no new primitive on its own.</t>
-        </is>
-      </c>
-      <c r="H2057" t="inlineStr">
-        <is>
-          <t>STAT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2057" t="inlineStr"/>
+      <c r="H2057" t="inlineStr"/>
     </row>
     <row r="2058">
       <c r="A2058" t="inlineStr">
@@ -72637,19 +71605,11 @@
       </c>
       <c r="F2061" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2061" t="inlineStr">
-        <is>
-          <t>Needs a Dynasty-deck search that REFILLS THE REVEALING PROVINCE FACE-UP with the found card, rather than putting it into a hand/into play by DeckSearch's existing effect list (ToHand/ToHandThenDiscard/AttachRegion, none of which places a card into a specific province slot as its own "entering play" position) -- "search your Dynasty deck for a Sensei Personality. Refill this Province with him, face-up" needs a new DeckSearch effect kind, plus reconciling it with ContinueEventsReveal's own already-in-progress province loop (the searched card lands in the SAME province slot the Event was just revealed and removed from, mid-reveal).</t>
-        </is>
-      </c>
-      <c r="H2061" t="inlineStr">
-        <is>
-          <t>PROVINCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2061" t="inlineStr"/>
+      <c r="H2061" t="inlineStr"/>
     </row>
     <row r="2062">
       <c r="A2062" t="inlineStr">
@@ -72713,19 +71673,11 @@
       </c>
       <c r="F2063" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2063" t="inlineStr">
-        <is>
-          <t>Needs "the rulebook Cavalry player ability", which the rules document does not define: under Emperor Edition Cavalry is the Cavalry Maneuvers segment (a unit assignment, not a player ability that targets Personalities). Until the rules lane names the ability meant (the Ivory Edition Cavalry player ability, presumably), "Personalities may not be targeted by" it cannot be given a reading. The duration, "until your second turn from now begins", is the existing ExpiresAtTurnsTaken shape (Times of Strife).</t>
-        </is>
-      </c>
-      <c r="H2063" t="inlineStr">
-        <is>
-          <t>RULES</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2063" t="inlineStr"/>
+      <c r="H2063" t="inlineStr"/>
     </row>
     <row r="2064">
       <c r="A2064" t="inlineStr">
@@ -72993,19 +71945,11 @@
       </c>
       <c r="F2071" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2071" t="inlineStr">
-        <is>
-          <t>Needs Equip to accept a target in the discard pile: "until your turn three turns from now begins, you may target Followers in your discard pile with the Equip rulebook action" changes the rulebook action for a period; ongoing Events expire (ExpiresAtTurnsTaken) but do not change Equip.</t>
-        </is>
-      </c>
-      <c r="H2071" t="inlineStr">
-        <is>
-          <t>RULEBOOK</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2071" t="inlineStr"/>
+      <c r="H2071" t="inlineStr"/>
     </row>
     <row r="2072">
       <c r="A2072" t="inlineStr">
@@ -73511,19 +72455,11 @@
       </c>
       <c r="F2086" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2086" t="inlineStr">
-        <is>
-          <t>Needs a PLAYER ability granted for a bounded time ("until your second turn from now begins, you have the ability, Limited: Put a target Ring in your hand into play. While it remains in play, it does not count towards an Enlightenment Victory"): TimingGrants.cs grants a player a timing, not an ability, and no per-player granted-ability list exists; plus a per-Ring flag that excludes it from the Enlightenment check (the check reads only the Fudo keyword) and a way to put a Ring from hand into play outside its own printed action. The duration itself is the ExpiresAtTurnsTaken shape.</t>
-        </is>
-      </c>
-      <c r="H2086" t="inlineStr">
-        <is>
-          <t>GRANT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2086" t="inlineStr"/>
+      <c r="H2086" t="inlineStr"/>
     </row>
     <row r="2087">
       <c r="A2087" t="inlineStr">
@@ -73655,19 +72591,11 @@
       </c>
       <c r="F2090" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2090" t="inlineStr">
-        <is>
-          <t>Needs "after the resolution of any Battle action, give each of your Nonhumans who performed it a +1F Frenzy token" for two turns: the performers of a resolved Battle action are not recorded, and the token is a new kind.</t>
-        </is>
-      </c>
-      <c r="H2090" t="inlineStr">
-        <is>
-          <t>TOKEN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2090" t="inlineStr"/>
+      <c r="H2090" t="inlineStr"/>
     </row>
     <row r="2091">
       <c r="A2091" t="inlineStr">
@@ -74003,19 +72931,11 @@
       </c>
       <c r="F2100" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2100" t="inlineStr">
-        <is>
-          <t>Needs the same hand-discard immunity gap as oracle-l5r-5958 (Pillowbook; see that entry), plus a per-phase counter of "actions that put cards into a player's hand" this phase (Urgency's own action-allowance counter, Seeds of Decay batch 2, is the nearest shape but counts ACTIONS taken, not a specific EFFECT category across every ability that draws/searches/returns a card to hand) -- "if a player has resolved two actions that put cards in his hand in one phase, no more cards will be put into his hand that phase" needs a new counter keyed on that effect category, incremented at every card-to-hand site (Draw, DeckSearch's ToHand, ReturnToHand, and more), not merely Urgency's one existing counter.</t>
-        </is>
-      </c>
-      <c r="H2100" t="inlineStr">
-        <is>
-          <t>HONOR</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2100" t="inlineStr"/>
+      <c r="H2100" t="inlineStr"/>
     </row>
     <row r="2101">
       <c r="A2101" t="inlineStr">
@@ -74181,19 +73101,11 @@
       </c>
       <c r="F2105" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2105" t="inlineStr">
-        <is>
-          <t>Needs two effects: destroying a Region of your choice when it is revealed (a decision in the reveal) and "negate all movement to and from battlefields" until your next turn begins (a movement lock on every card, present and future, rather than on chosen cards: MovementLocks are per card).</t>
-        </is>
-      </c>
-      <c r="H2105" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2105" t="inlineStr"/>
+      <c r="H2105" t="inlineStr"/>
     </row>
     <row r="2106">
       <c r="A2106" t="inlineStr">
@@ -74563,19 +73475,11 @@
       </c>
       <c r="F2116" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2116" t="inlineStr">
-        <is>
-          <t>Needs (a) a 'put a dead Personality on the top of its owner's deck' primitive -- ToOwnerDeck is written for cards leaving play, and nothing offers it a Zone.Dead card; (b) a shield that outlives an action, 'negate the next card effect that bows, destroys, or moves him' (NegatedEffects belong to one held action and are dropped with it); and (c) the count of dead Personalities in all players' discard piles for the Force bonus (trivial).</t>
-        </is>
-      </c>
-      <c r="H2116" t="inlineStr">
-        <is>
-          <t>ZONE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2116" t="inlineStr"/>
+      <c r="H2116" t="inlineStr"/>
     </row>
     <row r="2117">
       <c r="A2117" t="inlineStr">
@@ -74979,19 +73883,11 @@
       </c>
       <c r="F2128" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2128" t="inlineStr">
-        <is>
-          <t>Hotei's Contentment: its Proclaim clause ("if the Personality's base PH is 3 or lower, increase the Honor gain by 1") is a small, localized addition to FinishProclaim's own GainHonor call (SeedsOfDecayBatch2.cs), conditioned on this Celestial being in play for the proclaiming player. Its Open half ("discard this card and target a Personality: he may not assign to, and will not move into, an attacking army") needs a new MovementLocks.cs kind scoped to attacking-army assignment specifically (the existing MovementKinds.Assign lock is turn-scoped and not attacking-side-specific) with no stated duration (read as permanent, unlike every existing turn-scoped lock). Both pieces are small but separately unverified; left unwired this pass for lack of time to build and test the new lock kind.</t>
-        </is>
-      </c>
-      <c r="H2128" t="inlineStr">
-        <is>
-          <t>SMALL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2128" t="inlineStr"/>
+      <c r="H2128" t="inlineStr"/>
     </row>
     <row r="2129">
       <c r="A2129" t="inlineStr">
@@ -76012,7 +74908,7 @@
       </c>
       <c r="G2158" t="inlineStr">
         <is>
-          <t>Natural Aviary (Region): mechanically wirable, scan unavailable for its token. "Limited: Pay 2 Gold and target your Personality: Create a 1F Nonhuman * Falcon * Cavalry Follower and attach it to him" is a Region Limited with GoldCostRule.Fixed(2), target own-personality and Creates: new(CardType.Follower, Force: 1, Keywords: [Nonhuman, Falcon, Cavalry]) (the create-and-attach shape of Ashigaru Recruits / Makubesu). Blocked because no published CreatedOnly Proxy scan is a 1F Nonhuman Falcon Cavalry Follower (Bird of Prey oracle-l5r-9712 is a Shadowlands Undead Raptor; no Falcon Proxy is in any fetched catalogue), and the Oracle image host is blocked by the sandbox's network policy.</t>
+          <t>Natural Aviary (issue #503, P6, re-checked): its own scan is local; blocked only by its created 1F Nonhuman Falcon Cavalry Follower. Dutiful Cavalry (oracle-l5r-10003) is a near miss Mendon ruled out (no Nonhuman, no Falcon); docs/requests/created-card-scans-needed.md row A4 (falcon.jpg) is unticked. Otherwise a Region Limited paying 2 Gold with the create-and-attach shape.</t>
         </is>
       </c>
       <c r="H2158" t="inlineStr">
@@ -76088,7 +74984,7 @@
       </c>
       <c r="G2160" t="inlineStr">
         <is>
-          <t>Plains of Otosan Uchi (Region, group F): "This province holds two Dynasty cards; do not reveal the second card in the Events Phase this card enters play. You decide each time which card slot is revealed, resolved, or refilled first. Before this province is destroyed: Lose 10 Honor." Every province is modelled as exactly one card slot (ProvinceState.CardId): the Events Phase reveal loop, Purchase and Reserve recruits from a province, Refill, DestroyProvince's discard, Border Keep's and the Kharmic cycles, the private province looks, MatchView.ProvinceView and the client's province stacks all assume one card, so a second slot (a SecondCardId with its own reveal, refill, purchase and destruction paths, the controller's choice of which slot goes first, and a view/client field for it) is a structural change across the engine, the wire view and the client rather than a card-sized primitive. The 10-Honor trait ("before this province is destroyed", a cost-like loss that DestroyProvince would have to make first) is buildable once the province has both slots. Not published. Mendon (2026-09-25): a province must be able to hold two Dynasty cards; the view/client second slot is requested from Alfredo in issue #499, after which the engine side (second slot reveal, refill, purchase, destruction, the 10-Honor loss) can follow.</t>
+          <t>Plains of Otosan Uchi (issue #503, P6, re-checked): still blocked on the two-card province. Every province is one card slot (ProvinceState.CardId): the Events Phase reveal, Purchase and Reserve recruits, Refill (now also the face-up refills of Susaiken / Distant Expansion and Ietsuno's refill trigger, EmperorP6.cs), DestroyProvince, the private province sights and MatchView.ProvinceView all assume one card. Mendon (2026-09-25): a province must be able to hold two Dynasty cards; the view/client second slot is requested from Alfredo in issue #499 (not done: ProvinceView has no second card). The engine side (a second slot's reveal, refill, purchase and destruction, the owner's choice of which slot goes first, 'do not reveal the second card in the Events Phase this card enters play', and the 10-Honor loss before the province is destroyed) should follow once the view lane is agreed, so a published card does not show only half of its province.</t>
         </is>
       </c>
       <c r="H2160" t="inlineStr">
@@ -76978,7 +75874,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -76998,7 +75894,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -77018,7 +75914,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -77038,7 +75934,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -77078,7 +75974,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -77098,7 +75994,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -77118,7 +76014,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -77138,7 +76034,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -77158,7 +76054,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -77178,7 +76074,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -77198,7 +76094,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -77258,7 +76154,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -77278,7 +76174,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -77298,7 +76194,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -77318,7 +76214,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -77358,7 +76254,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -77378,7 +76274,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -77398,7 +76294,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -77418,7 +76314,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -77438,7 +76334,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -77458,7 +76354,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -77478,7 +76374,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -77498,7 +76394,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -77518,7 +76414,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wire Daigotsu Shiraume and Without Mercy (Torn Asunder) so the Spider Conquer deck is playable (issue #648)
Shiraume: entry Honor loss. Without Mercy: after-action-resolved Reaction; the resolved-action record now names what the action targeted, and the window hands priority back to the player an additional Battle action was granted to. Art pack catalogue-art-issue648-20261004-r1 (+2 scans).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GL78ciYZd42f7dqbiNuNC5
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -532,14 +532,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C6" t="n">
         <v>836</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>73.1%</t>
+          <t>73.2%</t>
         </is>
       </c>
     </row>
@@ -604,14 +604,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>76.4%</t>
+          <t>76.6%</t>
         </is>
       </c>
     </row>
@@ -712,14 +712,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1573</v>
+        <v>1575</v>
       </c>
       <c r="C16" t="n">
         <v>2196</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>71.6%</t>
+          <t>71.7%</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
         <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D22" t="n">
         <v>4</v>
@@ -896,7 +896,7 @@
         <v>12</v>
       </c>
       <c r="G22" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H22" t="n">
         <v>6</v>
@@ -911,7 +911,7 @@
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23">
@@ -1042,7 +1042,7 @@
         <v>3</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>20</v>
@@ -1054,7 +1054,7 @@
         <v>46</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H27" s="2" t="n">
         <v>56</v>
@@ -1072,7 +1072,7 @@
         <v>2</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>623</v>
+        <v>621</v>
       </c>
     </row>
   </sheetData>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G233" t="inlineStr"/>
@@ -65265,7 +65265,7 @@
       </c>
       <c r="F1886" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1886" t="inlineStr"/>

</xml_diff>

<commit_message>
Promotional-Emperor pass (#653): format, pinned inventories, inventory blockers loader, art pack metadata, decision note, handoff
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -532,14 +532,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>612</v>
+        <v>627</v>
       </c>
       <c r="C6" t="n">
         <v>836</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>73.2%</t>
+          <t>75.0%</t>
         </is>
       </c>
     </row>
@@ -550,14 +550,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C7" t="n">
         <v>136</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>85.3%</t>
+          <t>87.5%</t>
         </is>
       </c>
     </row>
@@ -568,14 +568,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C8" t="n">
         <v>136</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>53.7%</t>
+          <t>70.6%</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>65.4%</t>
+          <t>67.7%</t>
         </is>
       </c>
     </row>
@@ -604,14 +604,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>458</v>
+        <v>476</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>76.6%</t>
+          <t>79.6%</t>
         </is>
       </c>
     </row>
@@ -622,14 +622,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="C11" t="n">
         <v>152</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>63.2%</t>
+          <t>75.0%</t>
         </is>
       </c>
     </row>
@@ -640,14 +640,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>49.4%</t>
+          <t>71.6%</t>
         </is>
       </c>
     </row>
@@ -658,14 +658,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C13" t="n">
         <v>37</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>56.8%</t>
+          <t>64.9%</t>
         </is>
       </c>
     </row>
@@ -676,14 +676,14 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C14" t="n">
         <v>26</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>61.5%</t>
+          <t>80.8%</t>
         </is>
       </c>
     </row>
@@ -712,14 +712,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1575</v>
+        <v>1681</v>
       </c>
       <c r="C16" t="n">
         <v>2196</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>71.7%</t>
+          <t>76.5%</t>
         </is>
       </c>
     </row>
@@ -800,88 +800,88 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Promotional–Emperor</t>
-        </is>
+          <t>Coils of Madness</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>18</v>
+        <v>67</v>
       </c>
       <c r="D20" t="n">
         <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="F20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G20" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="H20" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="I20" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="J20" t="n">
-        <v>5</v>
-      </c>
-      <c r="K20" t="n">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2</v>
       </c>
       <c r="M20" t="n">
-        <v>134</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Coils of Madness</t>
+          <t>Torn Asunder</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E21" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F21" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="G21" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="H21" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I21" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J21" t="n">
-        <v>3</v>
-      </c>
-      <c r="L21" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Torn Asunder</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1</v>
+          <t>Gates of Chaos</t>
+        </is>
       </c>
       <c r="C22" t="n">
         <v>44</v>
@@ -890,38 +890,35 @@
         <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F22" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G22" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="H22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J22" t="n">
         <v>1</v>
       </c>
-      <c r="K22" t="n">
-        <v>1</v>
-      </c>
       <c r="M22" t="n">
-        <v>120</v>
+        <v>106</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gates of Chaos</t>
+          <t>Aftermath</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D23" t="n">
         <v>4</v>
@@ -930,78 +927,78 @@
         <v>7</v>
       </c>
       <c r="F23" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G23" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="H23" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
         <v>3</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M23" t="n">
-        <v>106</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aftermath</t>
+          <t>Promotional–Celestial</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>43</v>
+        <v>8</v>
       </c>
       <c r="D24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="n">
         <v>4</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" t="n">
         <v>7</v>
       </c>
-      <c r="F24" t="n">
-        <v>10</v>
-      </c>
-      <c r="G24" t="n">
-        <v>24</v>
-      </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J24" t="n">
         <v>3</v>
       </c>
+      <c r="K24" t="n">
+        <v>3</v>
+      </c>
       <c r="M24" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Promotional–Celestial</t>
+          <t>Promotional–Emperor</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>8</v>
-      </c>
-      <c r="D25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F25" t="n">
         <v>3</v>
       </c>
       <c r="G25" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H25" t="n">
         <v>6</v>
@@ -1010,13 +1007,13 @@
         <v>2</v>
       </c>
       <c r="J25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="26">
@@ -1042,37 +1039,37 @@
         <v>3</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L27" s="2" t="n">
         <v>2</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>621</v>
+        <v>515</v>
       </c>
     </row>
   </sheetData>
@@ -3961,7 +3958,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G84" t="inlineStr"/>
@@ -7123,7 +7120,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G177" t="inlineStr"/>
@@ -8453,7 +8450,7 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G216" t="inlineStr"/>
@@ -10205,7 +10202,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G268" t="inlineStr"/>
@@ -10276,8 +10273,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G270" t="inlineStr"/>
-      <c r="H270" t="inlineStr"/>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Fusako (issue #653, Promotional-Emperor): her own scan is local and read. "Iaijustu Limited: Target another player's Personality: Fusako challenges the target. His controller may bow him; if he is now bowed, he may refuse the duel. Destroy the duel's loser." Not wired: the challenge machinery offers refusal unconditionally (PendingDuel Stage AwaitingAccept, Dueling.cs IssueChallenge/ResolveDuelCommand), so there is no pre-challenge optional bow by the challenged player whose result (bowed) is what allows the refusal, and a new Iaijutsu Limited duel ability also needs per-ability-id entries in the shared ApplyDuelOutcome / IsIaijutsuAction / DuelPresentation switches (Sanctioned Duel's pattern). Reading to confirm when built: a target that is already bowed may refuse without the choice.</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>DUEL</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -10310,8 +10315,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G271" t="inlineStr"/>
-      <c r="H271" t="inlineStr"/>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Gaijin Sorcerer (issue #653, Promotional-Emperor): the scan prints "While your ritual is resolving, Gaijin Sorcerer counts as two Shugenja." (the catalogue's "After you announce your Ritual action..." is a later wording). Not wired: no ability carries a Ritual action keyword and every Shugenja slot (e.g. capturing-soul-remove's performing 'others', illusory-defense-province) counts each card once, so there is no weighted 'counts as two Shugenja' for a ritual's Shugenja count. RULES question to settle first: does the doubling count only toward the number of Shugenja a ritual requires, or also toward totals such as the combined Chi of the performing Shugenja (Capturing the Soul, Illusory Defense)?</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>TARGET</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -10341,7 +10354,7 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G272" t="inlineStr"/>
@@ -10812,8 +10825,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G286" t="inlineStr"/>
-      <c r="H286" t="inlineStr"/>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Gozu (issue #653, Promotional-Emperor): "Battle: Target a Terrain: Destroy it. You may discard a card. If you did, search your Fate deck for a Terrain, show it, then take an additional Battle action to play it, if legal; if not, discard it." The Terrain destruction (terrain-at-battle) and the optional discard are buildable, and Control the Field already grants an additional action scoped to Terrains in the hand; what is missing is playing a Terrain Strategy that was found by a search and is still in the Fate deck (play-from-hand is the only Strategy play path, AdditionalActionGrant.ScopeCardIds names hand cards) and discarding it when the additional action is not legal. RULES question: if the Terrain is legal but the player takes no additional action (passes), is it still discarded?</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>SEARCH</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -13257,7 +13278,7 @@
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G358" t="inlineStr"/>
@@ -15849,7 +15870,7 @@
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G434" t="inlineStr"/>
@@ -18033,7 +18054,7 @@
       </c>
       <c r="F498" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G498" t="inlineStr"/>
@@ -22351,7 +22372,7 @@
       </c>
       <c r="F625" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G625" t="inlineStr"/>
@@ -22385,7 +22406,7 @@
       </c>
       <c r="F626" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G626" t="inlineStr"/>
@@ -22453,7 +22474,7 @@
       </c>
       <c r="F628" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G628" t="inlineStr"/>
@@ -25683,7 +25704,7 @@
       </c>
       <c r="F723" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G723" t="inlineStr"/>
@@ -25717,7 +25738,7 @@
       </c>
       <c r="F724" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G724" t="inlineStr"/>
@@ -26265,7 +26286,7 @@
       </c>
       <c r="F740" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G740" t="inlineStr"/>
@@ -28055,7 +28076,7 @@
       </c>
       <c r="F793" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G793" t="inlineStr"/>
@@ -33295,14 +33316,10 @@
       </c>
       <c r="F947" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G947" t="inlineStr">
-        <is>
-          <t>Needs cost-ignoring Equip tied to a named restriction (explicitly deferred since #156).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G947" t="inlineStr"/>
       <c r="H947" t="inlineStr"/>
     </row>
     <row r="948">
@@ -34587,14 +34604,10 @@
       </c>
       <c r="F985" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G985" t="inlineStr">
-        <is>
-          <t>Needs a compound Gold-plus-card-discard cost shape (Kharmic keyword's own reminder).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G985" t="inlineStr"/>
       <c r="H985" t="inlineStr"/>
     </row>
     <row r="986">
@@ -35441,14 +35454,10 @@
       </c>
       <c r="F1010" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1010" t="inlineStr">
-        <is>
-          <t>Holding creation is built (issue #406: Charter, oracle-l5r-10806, published created-only). Needs a general Reaction trigger "after a battle resolves, if this card's army destroyed a province" (the only after-battle window is the Rings' own recruit window) and destroying this Follower as the cost.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1010" t="inlineStr"/>
       <c r="H1010" t="inlineStr"/>
     </row>
     <row r="1011">
@@ -36061,7 +36070,7 @@
       </c>
       <c r="F1028" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1028" t="inlineStr"/>
@@ -36201,7 +36210,7 @@
       </c>
       <c r="F1032" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1032" t="inlineStr"/>
@@ -36439,7 +36448,7 @@
       </c>
       <c r="F1039" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1039" t="inlineStr"/>
@@ -37085,7 +37094,7 @@
       </c>
       <c r="F1058" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1058" t="inlineStr"/>
@@ -37119,7 +37128,7 @@
       </c>
       <c r="F1059" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1059" t="inlineStr"/>
@@ -37153,7 +37162,7 @@
       </c>
       <c r="F1060" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1060" t="inlineStr"/>
@@ -37387,7 +37396,7 @@
       </c>
       <c r="F1067" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1067" t="inlineStr"/>
@@ -37489,7 +37498,7 @@
       </c>
       <c r="F1070" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1070" t="inlineStr"/>
@@ -37851,7 +37860,7 @@
       </c>
       <c r="F1081" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1081" t="inlineStr"/>
@@ -38089,7 +38098,7 @@
       </c>
       <c r="F1088" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1088" t="inlineStr"/>
@@ -38225,7 +38234,7 @@
       </c>
       <c r="F1092" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1092" t="inlineStr"/>
@@ -38259,7 +38268,7 @@
       </c>
       <c r="F1093" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1093" t="inlineStr"/>
@@ -38360,8 +38369,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1096" t="inlineStr"/>
-      <c r="H1096" t="inlineStr"/>
+      <c r="G1096" t="inlineStr">
+        <is>
+          <t>Mempo of the Amethyst Champion alters three rulebook Favor actions: "You may use Favor abilities one additional time per turn" (needs a per-player +1 use on every Favor-keyword ability, AbilityDefinition.UsesPerTurn is a fixed per-ability number), "After you announce the rulebook Favor Political Battle action: It may target any player's unit, and even if it is not attacking" (a retargeting after announcement -- favor-battle's target category 'enemy-attacking' is fixed at announcement and there is no re-selection step), and "Reaction: After you discard the Imperial Favor: Take the Imperial Favor" (no after-Favor-discard window exists; the discard is a cost paid in several places).</t>
+        </is>
+      </c>
+      <c r="H1096" t="inlineStr">
+        <is>
+          <t>RULEBOOK</t>
+        </is>
+      </c>
     </row>
     <row r="1097">
       <c r="A1097" t="inlineStr">
@@ -38697,7 +38714,7 @@
       </c>
       <c r="F1106" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1106" t="inlineStr"/>
@@ -38734,8 +38751,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1107" t="inlineStr"/>
-      <c r="H1107" t="inlineStr"/>
+      <c r="G1107" t="inlineStr">
+        <is>
+          <t>Peace Treaty (scan): "Limited: If there are more than two players, choose a player. He may choose to sign a peace treaty with you. If he chose this, then until your next Events Phase begins, neither of you may declare an attack against, or ally against, the other. If he did not choose this, you gain 3 Honor and he loses 3 Honor." The whole effect is conditional on a game of more than two players, which the engine does not support: wired it would be a Limited action that can never do anything. Question for Mendon: publish it as a deliberate two-player no-op, or leave it unpublished until multiplayer exists?</t>
+        </is>
+      </c>
+      <c r="H1107" t="inlineStr">
+        <is>
+          <t>RULES</t>
+        </is>
+      </c>
     </row>
     <row r="1108">
       <c r="A1108" t="inlineStr">
@@ -39033,7 +39058,7 @@
       </c>
       <c r="F1116" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1116" t="inlineStr"/>
@@ -39305,7 +39330,7 @@
       </c>
       <c r="F1124" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1124" t="inlineStr"/>
@@ -39339,7 +39364,7 @@
       </c>
       <c r="F1125" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1125" t="inlineStr"/>
@@ -39577,7 +39602,7 @@
       </c>
       <c r="F1132" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1132" t="inlineStr"/>
@@ -39614,8 +39639,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1133" t="inlineStr"/>
-      <c r="H1133" t="inlineStr"/>
+      <c r="G1133" t="inlineStr">
+        <is>
+          <t>The Blade of the Balash (scan): "Battle: Bow this card or, if you are a Dragon Clan player, discard it from your hand: Melee 5 Attack." The bow half is a plain wielder Attack, but the discard-from-hand half has no wielder and the text names no performer (Tsubute, the only Item played from a hand, prints "Choose your performing Ninja"). Question for Mendon: who performs the Melee 5 Attack when the Balash is discarded from hand -- an own Personality at the battlefield the player chooses, the army as a whole, or none? Wired as printed would guess one of these.</t>
+        </is>
+      </c>
+      <c r="H1133" t="inlineStr">
+        <is>
+          <t>RULES</t>
+        </is>
+      </c>
     </row>
     <row r="1134">
       <c r="A1134" t="inlineStr">
@@ -39645,7 +39678,7 @@
       </c>
       <c r="F1134" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1134" t="inlineStr"/>
@@ -39717,7 +39750,7 @@
       </c>
       <c r="F1136" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1136" t="inlineStr"/>
@@ -39754,8 +39787,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1137" t="inlineStr"/>
-      <c r="H1137" t="inlineStr"/>
+      <c r="G1137" t="inlineStr">
+        <is>
+          <t>The Isha's Yumi - exp (scan): "Battle: Bow this card or, if you are a Mantis Clan player, discard it from your hand: Ranged 6 Attack." Same open question as The Blade of the Balash: the discard-from-hand half has no wielder and prints no performing Personality, so who performs the Ranged 6 Attack (and whose Force/keywords, e.g. Conflagration-style bonuses, apply) needs a ruling before the card can be wired whole.</t>
+        </is>
+      </c>
+      <c r="H1137" t="inlineStr">
+        <is>
+          <t>RULES</t>
+        </is>
+      </c>
     </row>
     <row r="1138">
       <c r="A1138" t="inlineStr">
@@ -39785,7 +39826,7 @@
       </c>
       <c r="F1138" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1138" t="inlineStr"/>
@@ -39819,7 +39860,7 @@
       </c>
       <c r="F1139" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1139" t="inlineStr"/>
@@ -39853,7 +39894,7 @@
       </c>
       <c r="F1140" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1140" t="inlineStr"/>
@@ -39890,8 +39931,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1141" t="inlineStr"/>
-      <c r="H1141" t="inlineStr"/>
+      <c r="G1141" t="inlineStr">
+        <is>
+          <t>The Sacred Rosary of the Constrictors: "Limited: Discard all your Celestials in play. Search your Dynasty deck or discard pile for a Celestial. Put it into play. If you searched your discard pile for it, remove this card from the game." Missing primitive: a search effect that puts a Celestial into play with no province (SearchEffect.PutIntoPlay enters only a Personality; ResolveCelestial is tied to refilling the province a Celestial was revealed in and to the discard of the controller's other Celestials), plus remembering which of the two places the card came from to remove the Rosary.</t>
+        </is>
+      </c>
+      <c r="H1141" t="inlineStr">
+        <is>
+          <t>SEARCH</t>
+        </is>
+      </c>
     </row>
     <row r="1142">
       <c r="A1142" t="inlineStr">
@@ -39958,8 +40007,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1143" t="inlineStr"/>
-      <c r="H1143" t="inlineStr"/>
+      <c r="G1143" t="inlineStr">
+        <is>
+          <t>The Topaz Armor - exp: "After this card enters play: Choose two keywords; Courtier, Samurai, Archer, ... Stalwart. This Personality has the two keywords last chosen from the previous trait." The engine's deciders (DeciderChoice.cs) and entry windows choose cards, never a keyword, and a two-of-eleven keyword pick has no primitive; the phrase "the two keywords last chosen from the previous trait" is also unclear. Question for Mendon: are the two keywords kept for as long as the Armor stays attached (a re-entry after it left play choosing a fresh pair), and is the choice mandatory on entering play (a trait) rather than a Reaction the controller may decline?</t>
+        </is>
+      </c>
+      <c r="H1143" t="inlineStr">
+        <is>
+          <t>RULES</t>
+        </is>
+      </c>
     </row>
     <row r="1144">
       <c r="A1144" t="inlineStr">
@@ -40023,7 +40080,7 @@
       </c>
       <c r="F1145" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1145" t="inlineStr"/>
@@ -40464,8 +40521,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1158" t="inlineStr"/>
-      <c r="H1158" t="inlineStr"/>
+      <c r="G1158" t="inlineStr">
+        <is>
+          <t>Winter Sled: "While you control a Winter card, other players' cards' effects will not negate this Personality's movement." The Reaction half (after engaging, bow this card: Move this Personality to the battlefield if enemy units are there) is buildable, but the static is a standing 'will not be negated' on one Personality's movement spread over roughly seven independent negation sources (NegatesEffect, EnemyActionMovementAutoNegated, the delay store, Show of Restraint's and Blessings' shields, Twin Forks, Request Authorization), none of which knows whose card is negating; MovementCannotBeNegated is a per-command exemption, not per-Personality. A global per-Personality movement-negation check is needed first.</t>
+        </is>
+      </c>
+      <c r="H1158" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="1159">
       <c r="A1159" t="inlineStr">
@@ -42330,8 +42395,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1213" t="inlineStr"/>
-      <c r="H1213" t="inlineStr"/>
+      <c r="G1213" t="inlineStr">
+        <is>
+          <t>Jade Embrace (Spell). Needs the permanent removal of one chosen ability of a card; the engine has only a per-turn ability lock (DisableAbility) and a total removal.</t>
+        </is>
+      </c>
+      <c r="H1213" t="inlineStr">
+        <is>
+          <t>EFFECT</t>
+        </is>
+      </c>
     </row>
     <row r="1214">
       <c r="A1214" t="inlineStr">
@@ -42565,7 +42638,7 @@
       </c>
       <c r="F1220" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1220" t="inlineStr">
@@ -43286,8 +43359,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1241" t="inlineStr"/>
-      <c r="H1241" t="inlineStr"/>
+      <c r="G1241" t="inlineStr">
+        <is>
+          <t>Sea &amp; Sky (Spell). Needs the permanent removal of a trait or ability of a Region or Terrain; the engine has no permanent per-ability removal for those zones.</t>
+        </is>
+      </c>
+      <c r="H1241" t="inlineStr">
+        <is>
+          <t>EFFECT</t>
+        </is>
+      </c>
     </row>
     <row r="1242">
       <c r="A1242" t="inlineStr">
@@ -43490,8 +43571,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1247" t="inlineStr"/>
-      <c r="H1247" t="inlineStr"/>
+      <c r="G1247" t="inlineStr">
+        <is>
+          <t>Sleep (Spell). RULES question for Mendon: are the targeted Personalities chosen after the discarded card reveals the Focus total (a sequenced multi-target: discard first, then choose) or at announcement with the total checked at resolution? The engine cannot do the first (all targets are chosen at announcement) and the second changes what the card does.</t>
+        </is>
+      </c>
+      <c r="H1247" t="inlineStr">
+        <is>
+          <t>RULES</t>
+        </is>
+      </c>
     </row>
     <row r="1248">
       <c r="A1248" t="inlineStr">
@@ -43793,7 +43882,7 @@
       </c>
       <c r="F1256" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1256" t="inlineStr"/>
@@ -44609,7 +44698,7 @@
       </c>
       <c r="F1280" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1280" t="inlineStr"/>
@@ -45391,7 +45480,7 @@
       </c>
       <c r="F1303" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1303" t="inlineStr"/>
@@ -46819,7 +46908,7 @@
       </c>
       <c r="F1345" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1345" t="inlineStr"/>
@@ -47945,7 +48034,7 @@
       </c>
       <c r="F1378" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1378" t="inlineStr"/>
@@ -49921,7 +50010,7 @@
       </c>
       <c r="F1436" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1436" t="inlineStr"/>
@@ -50499,7 +50588,7 @@
       </c>
       <c r="F1453" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1453" t="inlineStr"/>
@@ -51587,7 +51676,7 @@
       </c>
       <c r="F1485" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1485" t="inlineStr"/>
@@ -52679,7 +52768,7 @@
       </c>
       <c r="F1517" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1517" t="inlineStr"/>
@@ -52747,7 +52836,7 @@
       </c>
       <c r="F1519" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1519" t="inlineStr"/>
@@ -53401,7 +53490,7 @@
       </c>
       <c r="F1538" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1538" t="inlineStr"/>
@@ -53571,7 +53660,7 @@
       </c>
       <c r="F1543" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1543" t="inlineStr"/>
@@ -54013,7 +54102,7 @@
       </c>
       <c r="F1556" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1556" t="inlineStr"/>
@@ -56133,7 +56222,7 @@
       </c>
       <c r="F1618" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1618" t="inlineStr"/>
@@ -56850,8 +56939,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1639" t="inlineStr"/>
-      <c r="H1639" t="inlineStr"/>
+      <c r="G1639" t="inlineStr">
+        <is>
+          <t>Profits (Strategy). Needs a payment-time optional 1-Gold reduction, a Wealth token placed on the Holding after it enters, and a Reaction Gold source that discards the card; none of the three exists as a primitive and the payment path (PaymentTokens) cannot take a discard-as-cost source.</t>
+        </is>
+      </c>
+      <c r="H1639" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
     </row>
     <row r="1640">
       <c r="A1640" t="inlineStr">
@@ -57017,7 +57114,7 @@
       </c>
       <c r="F1644" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1644" t="inlineStr"/>
@@ -57425,7 +57522,7 @@
       </c>
       <c r="F1656" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1656" t="inlineStr"/>
@@ -57561,7 +57658,7 @@
       </c>
       <c r="F1660" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1660" t="inlineStr"/>
@@ -59057,7 +59154,7 @@
       </c>
       <c r="F1704" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1704" t="inlineStr"/>
@@ -61305,7 +61402,7 @@
       </c>
       <c r="F1770" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1770" t="inlineStr"/>
@@ -61686,8 +61783,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1781" t="inlineStr"/>
-      <c r="H1781" t="inlineStr"/>
+      <c r="G1781" t="inlineStr">
+        <is>
+          <t>The Deciding Moment (Strategy). Its Open half reorders the turn (the Dynasty Phase before the Attack Phase within one turn); the phase sequence is hard wired (three transitions in SetPhase/CompleteBattleTransition) and no primitive reorders it. The Battle half (draw a card) is not wired alone, because the card is not published half-working.</t>
+        </is>
+      </c>
+      <c r="H1781" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="1782">
       <c r="A1782" t="inlineStr">
@@ -63224,8 +63329,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1826" t="inlineStr"/>
-      <c r="H1826" t="inlineStr"/>
+      <c r="G1826" t="inlineStr">
+        <is>
+          <t>Through the Breach (Strategy). Needs the permanent removal of one trait or ability of a Castle Holding (the engine has only per-turn locks and total removal), and creates a 4F/2C/0PH Oni Personality for which no published CreatedOnly proxy scan exists.</t>
+        </is>
+      </c>
+      <c r="H1826" t="inlineStr">
+        <is>
+          <t>EFFECT</t>
+        </is>
+      </c>
     </row>
     <row r="1827">
       <c r="A1827" t="inlineStr">
@@ -65129,7 +65242,7 @@
       </c>
       <c r="F1882" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1882" t="inlineStr"/>
@@ -65234,8 +65347,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1885" t="inlineStr"/>
-      <c r="H1885" t="inlineStr"/>
+      <c r="G1885" t="inlineStr">
+        <is>
+          <t>Wildfire (Strategy). Needs a Fortress tile model (a destroyed-Holding replacement that blocks movement); the engine has no such zone or tile.</t>
+        </is>
+      </c>
+      <c r="H1885" t="inlineStr">
+        <is>
+          <t>EFFECT</t>
+        </is>
+      </c>
     </row>
     <row r="1886">
       <c r="A1886" t="inlineStr">
@@ -65707,7 +65828,7 @@
       </c>
       <c r="F1899" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1899" t="inlineStr"/>
@@ -66148,8 +66269,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1912" t="inlineStr"/>
-      <c r="H1912" t="inlineStr"/>
+      <c r="G1912" t="inlineStr">
+        <is>
+          <t>Colonial Farm (Holding, issue #653): blocked only by the card it creates. "Limited, Bow: Create a 1F Ashigaru Follower and attach it to your target Personality" needs a CreatedOnly Proxy scan of a 1F Ashigaru Follower with no other keyword; the only candidates are near misses (Mounted Ashigaru oracle-l5r-10010 also has Cavalry; Humble Farmers user-scan-humble-farmers is 2F) and docs/requests/created-card-scans-needed.md row A6 (assets/requested-scans/ashigaru-1f.jpg) is unticked. The rest is buildable: ClanEntryDiscount for the Lion entry discount, a Produce 5 Holding and the bow-and-create-and-attach shape of Natural Aviary.</t>
+        </is>
+      </c>
+      <c r="H1912" t="inlineStr">
+        <is>
+          <t>SCAN</t>
+        </is>
+      </c>
     </row>
     <row r="1913">
       <c r="A1913" t="inlineStr">
@@ -66349,7 +66478,7 @@
       </c>
       <c r="F1918" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1918" t="inlineStr"/>
@@ -66420,8 +66549,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1920" t="inlineStr"/>
-      <c r="H1920" t="inlineStr"/>
+      <c r="G1920" t="inlineStr">
+        <is>
+          <t>Ever-Winter Copse (Holding, issue #653): "When another Holding produces Gold to pay for a Nonhuman, bow this card: Produce 1 Gold" is a payment source whose availability depends on which OTHER producers the payer has chosen for the same payment, and which bows its own card. The payment tokens (EmperorMechE.cs PaymentTokens/UsePaymentTokens) are computed for a payment before any source is chosen, their use never bows their card, and there is no extension point for a condition on the chosen set of sources or for a token kind that bows; adding either means editing the shared payment code, not a feature file.</t>
+        </is>
+      </c>
+      <c r="H1920" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
     </row>
     <row r="1921">
       <c r="A1921" t="inlineStr">
@@ -66553,7 +66690,7 @@
       </c>
       <c r="F1924" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1924" t="inlineStr"/>
@@ -66655,7 +66792,7 @@
       </c>
       <c r="F1927" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1927" t="inlineStr"/>
@@ -66859,7 +66996,7 @@
       </c>
       <c r="F1933" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1933" t="inlineStr"/>
@@ -67134,8 +67271,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1941" t="inlineStr"/>
-      <c r="H1941" t="inlineStr"/>
+      <c r="G1941" t="inlineStr">
+        <is>
+          <t>Hidden Weapons (Holding, issue #653): "Limited: Put a Weapon in your hand under this Holding (face-down)" and "You may Equip Weapons from under this Holding as a Battle/Limited action" need a zone of cards under a particular Holding that is hidden from the other player. The only under-card zone (Zone.Underneath) is face-up, public and kept under the Stronghold, not per card, and its view projection shows every card in it; hiding a face-down card and equipping from it with the Equip action's own pricing needs a new hidden zone and its projection.</t>
+        </is>
+      </c>
+      <c r="H1941" t="inlineStr">
+        <is>
+          <t>ZONE</t>
+        </is>
+      </c>
     </row>
     <row r="1942">
       <c r="A1942" t="inlineStr">
@@ -67475,7 +67620,7 @@
       </c>
       <c r="F1951" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1951" t="inlineStr"/>
@@ -67882,8 +68027,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1963" t="inlineStr"/>
-      <c r="H1963" t="inlineStr"/>
+      <c r="G1963" t="inlineStr">
+        <is>
+          <t>Oracle of the Void - exp (Holding, issue #653): "Limited, Bow: The next two cards in provinces you refill (this turn) may be refilled face-up" is an optional face-up refill for each of the next two refills, whichever effect causes them (a purchase, a discard, a Region). Refills happen at many call sites (Purchase, Refill, RefillProvinceSlot and the effects that discard a province card) and there is no single refill hook or per-refill decision; a watch on future refills needs one, which is shared province plumbing. The rest ("Negate this card's destruction", Limited bow draw a card) would be buildable.</t>
+        </is>
+      </c>
+      <c r="H1963" t="inlineStr">
+        <is>
+          <t>PROVINCE</t>
+        </is>
+      </c>
     </row>
     <row r="1964">
       <c r="A1964" t="inlineStr">
@@ -67947,7 +68100,7 @@
       </c>
       <c r="F1965" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1965" t="inlineStr"/>
@@ -68117,7 +68270,7 @@
       </c>
       <c r="F1970" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1970" t="inlineStr"/>
@@ -68385,7 +68538,7 @@
       </c>
       <c r="F1978" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1978" t="inlineStr"/>
@@ -68487,7 +68640,7 @@
       </c>
       <c r="F1981" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1981" t="inlineStr"/>
@@ -68555,7 +68708,7 @@
       </c>
       <c r="F1983" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1983" t="inlineStr"/>
@@ -69612,8 +69765,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2014" t="inlineStr"/>
-      <c r="H2014" t="inlineStr"/>
+      <c r="G2014" t="inlineStr">
+        <is>
+          <t>The Amethyst Court (Holding, issue #653): its second line, "Bow: Bow your target unbowed Courtier or Artisan. Produce Gold equal to his Chi", is a Gold source of its own that names a Personality as it is used (the amount is that Personality's Chi, and bowing him is part of the production). The payment tokens offer a source per candidate only for Zlkyt's destroyed Holding and Moto Rani's removed dead Personality; UsePaymentTokens switches on a closed set of token kinds and has no extension point for a source that bows a chosen Personality, so the production cannot be added from a feature file.</t>
+        </is>
+      </c>
+      <c r="H2014" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
     </row>
     <row r="2015">
       <c r="A2015" t="inlineStr">
@@ -69711,7 +69872,7 @@
       </c>
       <c r="F2017" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2017" t="inlineStr"/>
@@ -69847,7 +70008,7 @@
       </c>
       <c r="F2021" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2021" t="inlineStr"/>
@@ -69881,7 +70042,7 @@
       </c>
       <c r="F2022" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2022" t="inlineStr"/>
@@ -69983,7 +70144,7 @@
       </c>
       <c r="F2025" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2025" t="inlineStr"/>
@@ -70020,8 +70181,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2026" t="inlineStr"/>
-      <c r="H2026" t="inlineStr"/>
+      <c r="G2026" t="inlineStr">
+        <is>
+          <t>The Onyx Dueling Circle (Holding, issue #653): blocked only by the Personality it creates. "Destroy your target Shugenja. Create a 5F/2C/0PH Nonhuman - Oni - Shadowlands Personality. Destroy this Holding. Lose 4 Honor" needs a CreatedOnly Proxy scan of that 5F/2C/0PH Oni; none exists locally and docs/requests/created-card-scans-needed.md row B12 is unticked. Akuma's Power (celestial-wave-2) creates a 9F/5C Oni from a different scan, which may not stand in for it.</t>
+        </is>
+      </c>
+      <c r="H2026" t="inlineStr">
+        <is>
+          <t>SCAN</t>
+        </is>
+      </c>
     </row>
     <row r="2027">
       <c r="A2027" t="inlineStr">
@@ -70085,7 +70254,7 @@
       </c>
       <c r="F2028" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2028" t="inlineStr"/>
@@ -70187,7 +70356,7 @@
       </c>
       <c r="F2031" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2031" t="inlineStr"/>
@@ -70255,7 +70424,7 @@
       </c>
       <c r="F2033" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2033" t="inlineStr"/>
@@ -70697,7 +70866,7 @@
       </c>
       <c r="F2046" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2046" t="inlineStr"/>
@@ -71173,7 +71342,7 @@
       </c>
       <c r="F2060" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2060" t="inlineStr"/>
@@ -71309,7 +71478,7 @@
       </c>
       <c r="F2064" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2064" t="inlineStr"/>
@@ -71343,7 +71512,7 @@
       </c>
       <c r="F2065" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2065" t="inlineStr"/>
@@ -71411,7 +71580,7 @@
       </c>
       <c r="F2067" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2067" t="inlineStr"/>
@@ -71683,7 +71852,7 @@
       </c>
       <c r="F2075" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2075" t="inlineStr"/>
@@ -71785,7 +71954,7 @@
       </c>
       <c r="F2078" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2078" t="inlineStr"/>
@@ -71819,7 +71988,7 @@
       </c>
       <c r="F2079" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2079" t="inlineStr"/>
@@ -72397,7 +72566,7 @@
       </c>
       <c r="F2096" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2096" t="inlineStr"/>
@@ -72601,7 +72770,7 @@
       </c>
       <c r="F2102" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2102" t="inlineStr"/>
@@ -72669,7 +72838,7 @@
       </c>
       <c r="F2104" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2104" t="inlineStr"/>
@@ -72703,7 +72872,7 @@
       </c>
       <c r="F2105" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2105" t="inlineStr"/>
@@ -72771,7 +72940,7 @@
       </c>
       <c r="F2107" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2107" t="inlineStr"/>
@@ -72808,8 +72977,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2108" t="inlineStr"/>
-      <c r="H2108" t="inlineStr"/>
+      <c r="G2108" t="inlineStr">
+        <is>
+          <t>The Jade Championship (Event). Needs a -1F aura on Shadowlands Followers at a location (FollowerForce has no registry hook) and a mandatory trait that triggers after the resolution of an action from a Spell (no trait-after-action hook exists; AfterActionResolved offers only optional Reactions).</t>
+        </is>
+      </c>
+      <c r="H2108" t="inlineStr">
+        <is>
+          <t>TRIG-AFTER</t>
+        </is>
+      </c>
     </row>
     <row r="2109">
       <c r="A2109" t="inlineStr">
@@ -72873,7 +73050,7 @@
       </c>
       <c r="F2110" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2110" t="inlineStr"/>
@@ -72910,8 +73087,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2111" t="inlineStr"/>
-      <c r="H2111" t="inlineStr"/>
+      <c r="G2111" t="inlineStr">
+        <is>
+          <t>The Onyx Championship (Event). The granted Maho ability searches the discard pile, then the deck, then the Provinces for an Oni Personality and recruits it paying all costs; the engine's search primitive covers one source at a time and has no ordered multi-source search.</t>
+        </is>
+      </c>
+      <c r="H2111" t="inlineStr">
+        <is>
+          <t>SEARCH</t>
+        </is>
+      </c>
     </row>
     <row r="2112">
       <c r="A2112" t="inlineStr">
@@ -72941,7 +73126,7 @@
       </c>
       <c r="F2112" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2112" t="inlineStr"/>
@@ -73043,7 +73228,7 @@
       </c>
       <c r="F2115" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2115" t="inlineStr"/>
@@ -73077,7 +73262,7 @@
       </c>
       <c r="F2116" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2116" t="inlineStr"/>
@@ -73349,7 +73534,7 @@
       </c>
       <c r="F2124" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2124" t="inlineStr"/>
@@ -73893,7 +74078,7 @@
       </c>
       <c r="F2140" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2140" t="inlineStr"/>
@@ -73964,8 +74149,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2142" t="inlineStr"/>
-      <c r="H2142" t="inlineStr"/>
+      <c r="G2142" t="inlineStr">
+        <is>
+          <t>Jizo's Mercy (Celestial, issue #653): the first Battle ("Move a target attacking Personality home") is buildable, but the second, "Battle: Discard this Celestial. In this battle's resolution, before you destroy the Province, gain 4 Honor instead", has an unresolved reading. Question for Mendon: does "instead" mean the Celestial's controller gains 4 Honor INSTEAD of destroying the Province (the Province survives the battle), or only before it, so the Province is still destroyed and "instead" has no referent; and may the Defender play it (he would not be destroying the Province) or only an Attacker who wins? The engine has the resolution hooks (BeforeResolution.cs, AfterResolution.cs); the reading must be ruled first.</t>
+        </is>
+      </c>
+      <c r="H2142" t="inlineStr">
+        <is>
+          <t>RULES</t>
+        </is>
+      </c>
     </row>
     <row r="2143">
       <c r="A2143" t="inlineStr">
@@ -74029,7 +74222,7 @@
       </c>
       <c r="F2144" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2144" t="inlineStr"/>
@@ -74270,8 +74463,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2151" t="inlineStr"/>
-      <c r="H2151" t="inlineStr"/>
+      <c r="G2151" t="inlineStr">
+        <is>
+          <t>Sadahako's Artistry (Celestial, issue #653): the Honor half ("Limited: If your Family Honor is 10 or lower: Gain 1 Honor") is buildable, but the gift ("Discard this card and target a card in your hand: You offer it as a gift. Show it to another player. He may accept, putting it into his hand; if he did, you gain Honor equal to its Focus Value. If he did not, discard it and draw 3 cards") needs a ruling and a primitive. Question for Mendon: once the other player accepts, whose card is it and which discard pile does it go to when he discards or plays it (its owner's or the recipient's); may a card be put into another player's hand at all? The engine has the opponent's Either/Or decision (EitherOr.cs) but no move of a hand card into another player's hand: OwnerId means controller and ReturnCardsOutOfPlayToTheirOwners sends a card back to its owner, so the card cannot rest in the recipient's hand without a new ownership rule.</t>
+        </is>
+      </c>
+      <c r="H2151" t="inlineStr">
+        <is>
+          <t>RULES</t>
+        </is>
+      </c>
     </row>
     <row r="2152">
       <c r="A2152" t="inlineStr">
@@ -74403,7 +74604,7 @@
       </c>
       <c r="F2155" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2155" t="inlineStr"/>
@@ -74641,7 +74842,7 @@
       </c>
       <c r="F2162" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2162" t="inlineStr"/>
@@ -74709,7 +74910,7 @@
       </c>
       <c r="F2164" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2164" t="inlineStr"/>
@@ -74811,7 +75012,7 @@
       </c>
       <c r="F2167" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2167" t="inlineStr"/>
@@ -75087,7 +75288,7 @@
       </c>
       <c r="F2175" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2175" t="inlineStr"/>
@@ -75155,7 +75356,7 @@
       </c>
       <c r="F2177" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2177" t="inlineStr"/>
@@ -75464,8 +75665,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2186" t="inlineStr"/>
-      <c r="H2186" t="inlineStr"/>
+      <c r="G2186" t="inlineStr">
+        <is>
+          <t>Verdant Jungle (Region, issue #653): its Reaction, "Before an action resolves, bow this card: Negate its effects that move any Personalities into an attacking army at this Province's battlefield", negates only the movement part of an announced action by destination. The before-action Reaction window decides which Reactions apply in BeforeActionReactionApplies, a closed switch with no extension hook, and the movement a held action would make is known only per-ability (DeferredActionMovers) with no destination, so "into an attacking army at this battlefield" cannot be asked of an announced action. The first line (nonhuman Personalities enter play from this province for 1 less Gold) would be a small entry discount.</t>
+        </is>
+      </c>
+      <c r="H2186" t="inlineStr">
+        <is>
+          <t>TRIG-ANN</t>
+        </is>
+      </c>
     </row>
     <row r="2187">
       <c r="A2187" t="inlineStr">
@@ -75946,7 +76155,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -76006,7 +76215,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -76046,7 +76255,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -76086,7 +76295,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -76106,7 +76315,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -76166,7 +76375,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -76186,7 +76395,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -76226,7 +76435,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -76326,7 +76535,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -76346,7 +76555,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -76366,7 +76575,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -76406,7 +76615,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -76446,7 +76655,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Integrate the first three primitives (#672): inventory, art pack receipt, index; validate self-transfers at announcement
Field Messenger and Communion checked their transfer's attaching restrictions only at
resolution, so an illegal target was refused after a before-action Reaction window had
closed and the other player's decline became the rejected command. The bot soak stalled
on that once the deck pool changed. The check now runs as the action is announced.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PrhtAooqPUJRqFmsAknmcR
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -532,14 +532,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>641</v>
+        <v>655</v>
       </c>
       <c r="C6" t="n">
         <v>839</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>76.4%</t>
+          <t>78.1%</t>
         </is>
       </c>
     </row>
@@ -568,14 +568,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C8" t="n">
         <v>136</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>78.7%</t>
+          <t>79.4%</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>72.2%</t>
+          <t>72.9%</t>
         </is>
       </c>
     </row>
@@ -712,14 +712,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1733</v>
+        <v>1749</v>
       </c>
       <c r="C16" t="n">
         <v>2200</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>78.8%</t>
+          <t>79.5%</t>
         </is>
       </c>
     </row>
@@ -800,81 +800,81 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Coils of Madness</t>
+          <t>Torn Asunder</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E20" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F20" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="G20" t="n">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="H20" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I20" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J20" t="n">
-        <v>3</v>
-      </c>
-      <c r="L20" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>122</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Torn Asunder</t>
+          <t>Coils of Madness</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" t="n">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F21" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G21" t="n">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="H21" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I21" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2</v>
       </c>
       <c r="M21" t="n">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22">
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D22" t="n">
         <v>4</v>
@@ -893,7 +893,7 @@
         <v>7</v>
       </c>
       <c r="F22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G22" t="n">
         <v>32</v>
@@ -908,7 +908,7 @@
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23">
@@ -918,7 +918,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D23" t="n">
         <v>4</v>
@@ -942,7 +942,7 @@
         <v>3</v>
       </c>
       <c r="M23" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24">
@@ -1018,16 +1018,16 @@
         <v>3</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>15</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>112</v>
@@ -1048,7 +1048,7 @@
         <v>2</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>467</v>
+        <v>451</v>
       </c>
     </row>
   </sheetData>
@@ -6275,7 +6275,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G153" t="inlineStr"/>
@@ -8625,7 +8625,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G222" t="inlineStr"/>
@@ -10671,7 +10671,7 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G283" t="inlineStr"/>
@@ -11581,7 +11581,7 @@
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G310" t="inlineStr"/>
@@ -12189,7 +12189,7 @@
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G328" t="inlineStr"/>
@@ -18651,14 +18651,10 @@
       </c>
       <c r="F517" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G517" t="inlineStr">
-        <is>
-          <t>Needs a 'this card's Force counts twice during battle resolution' hook (no existing mechanism double-counts one specific card in a resolution total), and a personality-level 'will not attach Items' restriction (the existing 'Will only/not attach to X' restriction gates the ATTACHMENT side, not a blanket type-level refusal from the host).</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr"/>
       <c r="H517" t="inlineStr"/>
     </row>
     <row r="518">
@@ -20099,7 +20095,7 @@
       </c>
       <c r="F559" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G559" t="inlineStr"/>
@@ -20337,7 +20333,7 @@
       </c>
       <c r="F566" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G566" t="inlineStr"/>
@@ -20643,7 +20639,7 @@
       </c>
       <c r="F575" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G575" t="inlineStr"/>
@@ -23785,7 +23781,7 @@
       </c>
       <c r="F668" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G668" t="inlineStr"/>
@@ -26841,7 +26837,7 @@
       </c>
       <c r="F758" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G758" t="inlineStr"/>
@@ -27585,7 +27581,7 @@
       </c>
       <c r="F780" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G780" t="inlineStr"/>
@@ -27925,7 +27921,7 @@
       </c>
       <c r="F790" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G790" t="inlineStr"/>
@@ -30985,7 +30981,7 @@
       </c>
       <c r="F880" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G880" t="inlineStr"/>
@@ -38041,7 +38037,7 @@
       </c>
       <c r="F1088" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1088" t="inlineStr"/>
@@ -42703,7 +42699,7 @@
       </c>
       <c r="F1225" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1225" t="inlineStr"/>

</xml_diff>

<commit_message>
Wire-list wave (#674): art pack r1, inventory, decision index, handoff
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A29buqY4H1Xgn5ZxyHvSrq
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M27"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -468,7 +468,6 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -532,14 +531,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>641</v>
+        <v>728</v>
       </c>
       <c r="C6" t="n">
         <v>839</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>76.4%</t>
+          <t>86.8%</t>
         </is>
       </c>
     </row>
@@ -550,14 +549,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C7" t="n">
         <v>137</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>89.1%</t>
+          <t>92.7%</t>
         </is>
       </c>
     </row>
@@ -568,14 +567,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="C8" t="n">
         <v>136</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>78.7%</t>
+          <t>84.6%</t>
         </is>
       </c>
     </row>
@@ -586,14 +585,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>72.2%</t>
+          <t>82.7%</t>
         </is>
       </c>
     </row>
@@ -604,14 +603,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>486</v>
+        <v>545</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>81.3%</t>
+          <t>91.1%</t>
         </is>
       </c>
     </row>
@@ -622,14 +621,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="C11" t="n">
         <v>152</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>77.6%</t>
+          <t>90.1%</t>
         </is>
       </c>
     </row>
@@ -640,14 +639,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>71.6%</t>
+          <t>77.8%</t>
         </is>
       </c>
     </row>
@@ -658,14 +657,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C13" t="n">
         <v>37</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>67.6%</t>
+          <t>75.7%</t>
         </is>
       </c>
     </row>
@@ -694,14 +693,14 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C15" t="n">
         <v>10</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -712,14 +711,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1733</v>
+        <v>1935</v>
       </c>
       <c r="C16" t="n">
         <v>2200</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>78.8%</t>
+          <t>88.0%</t>
         </is>
       </c>
     </row>
@@ -788,11 +787,6 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Ring</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
           <t>TOTAL</t>
         </is>
       </c>
@@ -807,34 +801,28 @@
         <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>67</v>
-      </c>
-      <c r="D20" t="n">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="E20" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F20" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G20" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="H20" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I20" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J20" t="n">
         <v>3</v>
       </c>
       <c r="L20" t="n">
-        <v>2</v>
-      </c>
-      <c r="M20" t="n">
-        <v>122</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21">
@@ -847,102 +835,96 @@
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G21" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="H21" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
         <v>5</v>
       </c>
-      <c r="J21" t="n">
-        <v>1</v>
-      </c>
       <c r="K21" t="n">
         <v>1</v>
       </c>
-      <c r="M21" t="n">
-        <v>119</v>
+      <c r="L21" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Gates of Chaos</t>
+          <t>Aftermath</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="D22" t="n">
         <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F22" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G22" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="H22" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
-      </c>
-      <c r="M22" t="n">
-        <v>106</v>
+        <v>2</v>
+      </c>
+      <c r="L22" t="n">
+        <v>53</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aftermath</t>
+          <t>Gates of Chaos</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="D23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F23" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G23" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>3</v>
-      </c>
-      <c r="J23" t="n">
-        <v>3</v>
-      </c>
-      <c r="M23" t="n">
-        <v>98</v>
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="24">
@@ -969,7 +951,7 @@
       <c r="K24" t="n">
         <v>1</v>
       </c>
-      <c r="M24" t="n">
+      <c r="L24" t="n">
         <v>12</v>
       </c>
     </row>
@@ -991,7 +973,7 @@
       <c r="J25" t="n">
         <v>2</v>
       </c>
-      <c r="M25" t="n">
+      <c r="L25" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1004,7 +986,7 @@
       <c r="G26" t="n">
         <v>2</v>
       </c>
-      <c r="M26" t="n">
+      <c r="L26" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1018,37 +1000,34 @@
         <v>3</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>198</v>
+        <v>111</v>
       </c>
       <c r="D27" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="H27" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="E27" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="G27" s="2" t="n">
-        <v>112</v>
-      </c>
-      <c r="H27" s="2" t="n">
-        <v>34</v>
-      </c>
       <c r="I27" s="2" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>2</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M27" s="2" t="n">
-        <v>467</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -3835,7 +3814,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4001,7 +3980,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G86" t="inlineStr"/>
@@ -4171,7 +4150,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
@@ -4341,7 +4320,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G96" t="inlineStr"/>
@@ -4613,7 +4592,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G104" t="inlineStr"/>
@@ -4715,7 +4694,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G107" t="inlineStr"/>
@@ -4783,7 +4762,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G109" t="inlineStr"/>
@@ -4953,7 +4932,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G114" t="inlineStr"/>
@@ -5055,7 +5034,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
@@ -5361,7 +5340,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G126" t="inlineStr"/>
@@ -5731,7 +5710,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G137" t="inlineStr"/>
@@ -6887,7 +6866,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G171" t="inlineStr"/>
@@ -6989,7 +6968,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -7061,7 +7040,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G176" t="inlineStr"/>
@@ -7431,7 +7410,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G187" t="inlineStr"/>
@@ -7567,7 +7546,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G191" t="inlineStr"/>
@@ -7873,7 +7852,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G200" t="inlineStr"/>
@@ -7907,7 +7886,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G201" t="inlineStr"/>
@@ -7941,7 +7920,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G202" t="inlineStr"/>
@@ -8077,7 +8056,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G206" t="inlineStr"/>
@@ -8281,7 +8260,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
@@ -8319,7 +8298,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G213" t="inlineStr"/>
@@ -9633,7 +9612,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G252" t="inlineStr"/>
@@ -9803,7 +9782,7 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G257" t="inlineStr"/>
@@ -10237,7 +10216,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G270" t="inlineStr"/>
@@ -11241,7 +11220,7 @@
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G300" t="inlineStr"/>
@@ -12087,7 +12066,7 @@
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G325" t="inlineStr"/>
@@ -12321,7 +12300,7 @@
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G332" t="inlineStr"/>
@@ -12427,7 +12406,7 @@
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G335" t="inlineStr"/>
@@ -12461,7 +12440,7 @@
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G336" t="inlineStr"/>
@@ -13259,7 +13238,7 @@
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G359" t="inlineStr"/>
@@ -14143,7 +14122,7 @@
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G385" t="inlineStr"/>
@@ -14347,7 +14326,7 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G391" t="inlineStr"/>
@@ -14415,7 +14394,7 @@
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G393" t="inlineStr"/>
@@ -14759,7 +14738,7 @@
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G403" t="inlineStr"/>
@@ -14963,7 +14942,7 @@
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G409" t="inlineStr"/>
@@ -15269,7 +15248,7 @@
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G418" t="inlineStr"/>
@@ -15337,7 +15316,7 @@
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G420" t="inlineStr"/>
@@ -15885,7 +15864,7 @@
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G436" t="inlineStr"/>
@@ -16501,7 +16480,7 @@
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G454" t="inlineStr">
@@ -16641,7 +16620,7 @@
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G458" t="inlineStr">
@@ -17461,7 +17440,7 @@
       </c>
       <c r="F482" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G482" t="inlineStr"/>
@@ -17937,7 +17916,7 @@
       </c>
       <c r="F496" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G496" t="inlineStr"/>
@@ -18069,7 +18048,7 @@
       </c>
       <c r="F500" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G500" t="inlineStr"/>
@@ -19165,7 +19144,7 @@
       </c>
       <c r="F532" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G532" t="inlineStr">
@@ -19343,7 +19322,7 @@
       </c>
       <c r="F537" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G537" t="inlineStr">
@@ -19895,7 +19874,7 @@
       </c>
       <c r="F553" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G553" t="inlineStr"/>
@@ -20031,7 +20010,7 @@
       </c>
       <c r="F557" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G557" t="inlineStr"/>
@@ -20201,7 +20180,7 @@
       </c>
       <c r="F562" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G562" t="inlineStr"/>
@@ -20507,7 +20486,7 @@
       </c>
       <c r="F571" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G571" t="inlineStr"/>
@@ -21017,7 +20996,7 @@
       </c>
       <c r="F586" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G586" t="inlineStr"/>
@@ -21489,7 +21468,7 @@
       </c>
       <c r="F600" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G600" t="inlineStr"/>
@@ -22123,7 +22102,7 @@
       </c>
       <c r="F619" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G619" t="inlineStr"/>
@@ -22663,7 +22642,7 @@
       </c>
       <c r="F635" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G635" t="inlineStr"/>
@@ -22731,7 +22710,7 @@
       </c>
       <c r="F637" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G637" t="inlineStr"/>
@@ -23105,7 +23084,7 @@
       </c>
       <c r="F648" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G648" t="inlineStr"/>
@@ -23241,7 +23220,7 @@
       </c>
       <c r="F652" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G652" t="inlineStr"/>
@@ -23955,7 +23934,7 @@
       </c>
       <c r="F673" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G673" t="inlineStr"/>
@@ -23989,7 +23968,7 @@
       </c>
       <c r="F674" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G674" t="inlineStr"/>
@@ -24091,7 +24070,7 @@
       </c>
       <c r="F677" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G677" t="inlineStr"/>
@@ -24159,7 +24138,7 @@
       </c>
       <c r="F679" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G679" t="inlineStr"/>
@@ -24465,7 +24444,7 @@
       </c>
       <c r="F688" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G688" t="inlineStr"/>
@@ -24635,7 +24614,7 @@
       </c>
       <c r="F693" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G693" t="inlineStr"/>
@@ -24669,7 +24648,7 @@
       </c>
       <c r="F694" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G694" t="inlineStr"/>
@@ -25145,7 +25124,7 @@
       </c>
       <c r="F708" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G708" t="inlineStr"/>
@@ -25247,7 +25226,7 @@
       </c>
       <c r="F711" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G711" t="inlineStr"/>
@@ -25485,7 +25464,7 @@
       </c>
       <c r="F718" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G718" t="inlineStr"/>
@@ -25723,7 +25702,7 @@
       </c>
       <c r="F725" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G725" t="inlineStr"/>
@@ -26407,7 +26386,7 @@
       </c>
       <c r="F745" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G745" t="inlineStr"/>
@@ -26475,7 +26454,7 @@
       </c>
       <c r="F747" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G747" t="inlineStr"/>
@@ -27619,7 +27598,7 @@
       </c>
       <c r="F781" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G781" t="inlineStr"/>
@@ -27687,7 +27666,7 @@
       </c>
       <c r="F783" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G783" t="inlineStr"/>
@@ -27959,7 +27938,7 @@
       </c>
       <c r="F791" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G791" t="inlineStr"/>
@@ -28333,7 +28312,7 @@
       </c>
       <c r="F802" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G802" t="inlineStr"/>
@@ -28609,7 +28588,7 @@
       </c>
       <c r="F810" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G810" t="inlineStr"/>
@@ -29017,7 +28996,7 @@
       </c>
       <c r="F822" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G822" t="inlineStr"/>
@@ -29085,7 +29064,7 @@
       </c>
       <c r="F824" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G824" t="inlineStr"/>
@@ -29451,7 +29430,7 @@
       </c>
       <c r="F835" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G835" t="inlineStr"/>
@@ -29485,7 +29464,7 @@
       </c>
       <c r="F836" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G836" t="inlineStr"/>
@@ -29655,7 +29634,7 @@
       </c>
       <c r="F841" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G841" t="inlineStr"/>
@@ -29791,7 +29770,7 @@
       </c>
       <c r="F845" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G845" t="inlineStr"/>
@@ -30029,7 +30008,7 @@
       </c>
       <c r="F852" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G852" t="inlineStr"/>
@@ -30063,7 +30042,7 @@
       </c>
       <c r="F853" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G853" t="inlineStr"/>
@@ -30403,7 +30382,7 @@
       </c>
       <c r="F863" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G863" t="inlineStr"/>
@@ -30675,7 +30654,7 @@
       </c>
       <c r="F871" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G871" t="inlineStr"/>
@@ -30917,7 +30896,7 @@
       </c>
       <c r="F878" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G878" t="inlineStr"/>
@@ -31019,7 +30998,7 @@
       </c>
       <c r="F881" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G881" t="inlineStr"/>
@@ -34071,7 +34050,7 @@
       </c>
       <c r="F971" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G971" t="inlineStr">
@@ -34645,7 +34624,7 @@
       </c>
       <c r="F988" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G988" t="inlineStr">
@@ -35053,7 +35032,7 @@
       </c>
       <c r="F1000" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1000" t="inlineStr">
@@ -35321,7 +35300,7 @@
       </c>
       <c r="F1008" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1008" t="inlineStr">
@@ -35393,7 +35372,7 @@
       </c>
       <c r="F1010" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1010" t="inlineStr">
@@ -37139,7 +37118,7 @@
       </c>
       <c r="F1061" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1061" t="inlineStr"/>
@@ -37679,7 +37658,7 @@
       </c>
       <c r="F1077" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1077" t="inlineStr"/>
@@ -37871,7 +37850,7 @@
       </c>
       <c r="F1083" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1083" t="inlineStr"/>
@@ -38075,7 +38054,7 @@
       </c>
       <c r="F1089" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1089" t="inlineStr"/>
@@ -38751,7 +38730,7 @@
       </c>
       <c r="F1109" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1109" t="inlineStr"/>
@@ -39061,7 +39040,7 @@
       </c>
       <c r="F1118" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1118" t="inlineStr"/>
@@ -39571,7 +39550,7 @@
       </c>
       <c r="F1133" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1133" t="inlineStr"/>
@@ -40221,7 +40200,7 @@
       </c>
       <c r="F1152" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1152" t="inlineStr"/>
@@ -40727,7 +40706,7 @@
       </c>
       <c r="F1167" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1167" t="inlineStr"/>
@@ -40795,7 +40774,7 @@
       </c>
       <c r="F1169" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1169" t="inlineStr"/>
@@ -40931,7 +40910,7 @@
       </c>
       <c r="F1173" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1173" t="inlineStr"/>
@@ -40965,7 +40944,7 @@
       </c>
       <c r="F1174" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1174" t="inlineStr"/>
@@ -41101,7 +41080,7 @@
       </c>
       <c r="F1178" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1178" t="inlineStr"/>
@@ -41951,7 +41930,7 @@
       </c>
       <c r="F1203" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1203" t="inlineStr"/>
@@ -42121,7 +42100,7 @@
       </c>
       <c r="F1208" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1208" t="inlineStr"/>
@@ -42737,7 +42716,7 @@
       </c>
       <c r="F1226" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1226" t="inlineStr"/>
@@ -43148,8 +43127,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1238" t="inlineStr"/>
-      <c r="H1238" t="inlineStr"/>
+      <c r="G1238" t="inlineStr">
+        <is>
+          <t>Read the Essence (Spell, Torn Asunder, issue #674): "Open: Bow this card and target one face-down card in a province, or one or two such cards if this Shugenja is Void: Turn the targets face-up." Everything else exists (a bow-this-card cost; Second City's Political Open turns a face-down card face-up), but the engine names a face-down province card only by its province (the any-province command parameter, TargetPlayerId + Province, because a face-down card's id is hidden from the view), and that is ONE card. A Void Shugenja's "one or two" needs a second province in the same command (and a pair listing in QueryActions); no multi-province selection exists, and a card id may not be used (hidden information). Question for Mendon: may the Void version be two separate entries (one province each) sharing one use, or is a two-province selection UI wanted?</t>
+        </is>
+      </c>
+      <c r="H1238" t="inlineStr">
+        <is>
+          <t>HIDDEN</t>
+        </is>
+      </c>
     </row>
     <row r="1239">
       <c r="A1239" t="inlineStr">
@@ -43417,7 +43404,7 @@
       </c>
       <c r="F1246" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1246" t="inlineStr"/>
@@ -43621,7 +43608,7 @@
       </c>
       <c r="F1252" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1252" t="inlineStr"/>
@@ -43791,7 +43778,7 @@
       </c>
       <c r="F1257" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1257" t="inlineStr"/>
@@ -43995,7 +43982,7 @@
       </c>
       <c r="F1263" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1263" t="inlineStr"/>
@@ -44369,7 +44356,7 @@
       </c>
       <c r="F1274" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1274" t="inlineStr"/>
@@ -44471,7 +44458,7 @@
       </c>
       <c r="F1277" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1277" t="inlineStr"/>
@@ -45018,8 +45005,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1293" t="inlineStr"/>
-      <c r="H1293" t="inlineStr"/>
+      <c r="G1293" t="inlineStr">
+        <is>
+          <t>Witness the Untold (Spell, Torn Asunder, issue #674): "Reaction: After your Ring enters play, bow this card: Look at the top three cards of your Dynasty or Fate deck. Put them back in any order." The look and reorder exist (LookSpec, It Was a Cat's shape: either deck, three cards, reorder only), but nothing narrates a Ring entering play: every Ring is put into play by its own recruit case (RingEnteredByOwnText) and no Reaction trigger "after your Ring enters play" exists for another card to listen to (the Ring-entering gap the TRIG-AFTER category names). Needs a new reaction trigger fired from every Ring's entry, which is shared-interface work.</t>
+        </is>
+      </c>
+      <c r="H1293" t="inlineStr">
+        <is>
+          <t>TRIG-AFTER</t>
+        </is>
+      </c>
     </row>
     <row r="1294">
       <c r="A1294" t="inlineStr">
@@ -45729,7 +45724,7 @@
       </c>
       <c r="F1314" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1314" t="inlineStr"/>
@@ -45797,7 +45792,7 @@
       </c>
       <c r="F1316" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1316" t="inlineStr"/>
@@ -46205,7 +46200,7 @@
       </c>
       <c r="F1328" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1328" t="inlineStr"/>
@@ -46307,7 +46302,7 @@
       </c>
       <c r="F1331" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1331" t="inlineStr"/>
@@ -46817,7 +46812,7 @@
       </c>
       <c r="F1346" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1346" t="inlineStr"/>
@@ -47092,8 +47087,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1354" t="inlineStr"/>
-      <c r="H1354" t="inlineStr"/>
+      <c r="G1354" t="inlineStr">
+        <is>
+          <t>Benediction (Aftermath, Strategy; scan verified): "Open: Destroy your target Holding. Give a Province +3 strength." Two independent targets of different kinds, a card (your Holding) and a province (either player's, Ring of Earth's 'any-province' shape: GameCommand.Province plus TargetPlayerId). The engine has no ability that names a card and a province together: a multi-target ability is Slots (cards or players only), while the province categories ('any-province', 'enemy-province') are mutually exclusive with a card target in ValidateAbility and in the QueryActions candidate loop (one candidate per province/owner, no card). Wiring it needs a province target slot kind (TargetSlotKinds.Province with a SlotSelection province index and owner, validated in ValidateSlotCard and offered by SlotAbilityOption, plus the client picking a province inside a slot ability). That is a new decision shape for the client, not a local feature addition. Everything else is built: the effect itself is DestroyAttachment-free (DestroyUnits/Holding destroy, then GiveProvinceStrengthThisTurn(owner, index, 3)). QUESTION for Mendon: is 'Give a Province +3 strength' until end of turn (R-001 default, GiveProvinceStrengthThisTurn as Ring of Earth) and may the Province be either player's?</t>
+        </is>
+      </c>
+      <c r="H1354" t="inlineStr">
+        <is>
+          <t>TARGET</t>
+        </is>
+      </c>
     </row>
     <row r="1355">
       <c r="A1355" t="inlineStr">
@@ -47293,7 +47296,7 @@
       </c>
       <c r="F1360" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1360" t="inlineStr"/>
@@ -47735,7 +47738,7 @@
       </c>
       <c r="F1373" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1373" t="inlineStr"/>
@@ -47905,7 +47908,7 @@
       </c>
       <c r="F1378" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1378" t="inlineStr">
@@ -48011,7 +48014,7 @@
       </c>
       <c r="F1381" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1381" t="inlineStr"/>
@@ -48079,7 +48082,7 @@
       </c>
       <c r="F1383" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1383" t="inlineStr"/>
@@ -48351,7 +48354,7 @@
       </c>
       <c r="F1391" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1391" t="inlineStr"/>
@@ -48929,7 +48932,7 @@
       </c>
       <c r="F1408" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1408" t="inlineStr">
@@ -49035,7 +49038,7 @@
       </c>
       <c r="F1411" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1411" t="inlineStr"/>
@@ -49137,7 +49140,7 @@
       </c>
       <c r="F1414" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1414" t="inlineStr"/>
@@ -49851,7 +49854,7 @@
       </c>
       <c r="F1435" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1435" t="inlineStr"/>
@@ -50293,7 +50296,7 @@
       </c>
       <c r="F1448" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1448" t="inlineStr"/>
@@ -50327,7 +50330,7 @@
       </c>
       <c r="F1449" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1449" t="inlineStr"/>
@@ -50463,7 +50466,7 @@
       </c>
       <c r="F1453" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1453" t="inlineStr"/>
@@ -50905,7 +50908,7 @@
       </c>
       <c r="F1466" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1466" t="inlineStr"/>
@@ -51143,7 +51146,7 @@
       </c>
       <c r="F1473" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1473" t="inlineStr"/>
@@ -51279,7 +51282,7 @@
       </c>
       <c r="F1477" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1477" t="inlineStr"/>
@@ -51381,7 +51384,7 @@
       </c>
       <c r="F1480" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1480" t="inlineStr"/>
@@ -52651,7 +52654,7 @@
       </c>
       <c r="F1517" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1517" t="inlineStr"/>
@@ -52753,7 +52756,7 @@
       </c>
       <c r="F1520" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1520" t="inlineStr"/>
@@ -52957,7 +52960,7 @@
       </c>
       <c r="F1526" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1526" t="inlineStr"/>
@@ -53025,7 +53028,7 @@
       </c>
       <c r="F1528" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1528" t="inlineStr"/>
@@ -53093,7 +53096,7 @@
       </c>
       <c r="F1530" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1530" t="inlineStr"/>
@@ -53713,7 +53716,7 @@
       </c>
       <c r="F1548" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1548" t="inlineStr"/>
@@ -54223,7 +54226,7 @@
       </c>
       <c r="F1563" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1563" t="inlineStr">
@@ -54261,7 +54264,7 @@
       </c>
       <c r="F1564" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1564" t="inlineStr">
@@ -54333,7 +54336,7 @@
       </c>
       <c r="F1566" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1566" t="inlineStr"/>
@@ -54367,7 +54370,7 @@
       </c>
       <c r="F1567" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1567" t="inlineStr"/>
@@ -54609,7 +54612,7 @@
       </c>
       <c r="F1574" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1574" t="inlineStr"/>
@@ -54881,7 +54884,7 @@
       </c>
       <c r="F1582" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1582" t="inlineStr"/>
@@ -54915,7 +54918,7 @@
       </c>
       <c r="F1583" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1583" t="inlineStr"/>
@@ -54983,7 +54986,7 @@
       </c>
       <c r="F1585" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1585" t="inlineStr"/>
@@ -55599,7 +55602,7 @@
       </c>
       <c r="F1603" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1603" t="inlineStr"/>
@@ -55705,7 +55708,7 @@
       </c>
       <c r="F1606" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1606" t="inlineStr"/>
@@ -56079,7 +56082,7 @@
       </c>
       <c r="F1617" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1617" t="inlineStr"/>
@@ -56589,7 +56592,7 @@
       </c>
       <c r="F1632" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1632" t="inlineStr"/>
@@ -57031,7 +57034,7 @@
       </c>
       <c r="F1645" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1645" t="inlineStr"/>
@@ -57303,7 +57306,7 @@
       </c>
       <c r="F1653" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1653" t="inlineStr"/>
@@ -58221,7 +58224,7 @@
       </c>
       <c r="F1680" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1680" t="inlineStr"/>
@@ -59241,7 +59244,7 @@
       </c>
       <c r="F1710" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1710" t="inlineStr"/>
@@ -60023,7 +60026,7 @@
       </c>
       <c r="F1733" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1733" t="inlineStr"/>
@@ -60911,7 +60914,7 @@
       </c>
       <c r="F1759" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1759" t="inlineStr"/>
@@ -61285,7 +61288,7 @@
       </c>
       <c r="F1770" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1770" t="inlineStr"/>
@@ -61319,7 +61322,7 @@
       </c>
       <c r="F1771" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1771" t="inlineStr"/>
@@ -61901,7 +61904,7 @@
       </c>
       <c r="F1788" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1788" t="inlineStr"/>
@@ -61935,7 +61938,7 @@
       </c>
       <c r="F1789" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1789" t="inlineStr"/>
@@ -62275,7 +62278,7 @@
       </c>
       <c r="F1799" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1799" t="inlineStr"/>
@@ -62343,7 +62346,7 @@
       </c>
       <c r="F1801" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1801" t="inlineStr">
@@ -62517,7 +62520,7 @@
       </c>
       <c r="F1806" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1806" t="inlineStr"/>
@@ -63027,7 +63030,7 @@
       </c>
       <c r="F1821" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1821" t="inlineStr"/>
@@ -63095,7 +63098,7 @@
       </c>
       <c r="F1823" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1823" t="inlineStr"/>
@@ -63265,7 +63268,7 @@
       </c>
       <c r="F1828" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1828" t="inlineStr">
@@ -63541,7 +63544,7 @@
       </c>
       <c r="F1836" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1836" t="inlineStr"/>
@@ -64051,7 +64054,7 @@
       </c>
       <c r="F1851" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1851" t="inlineStr"/>
@@ -64425,7 +64428,7 @@
       </c>
       <c r="F1862" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1862" t="inlineStr"/>
@@ -65797,7 +65800,7 @@
       </c>
       <c r="F1902" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1902" t="inlineStr"/>
@@ -66001,7 +66004,7 @@
       </c>
       <c r="F1908" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1908" t="inlineStr"/>
@@ -66405,7 +66408,7 @@
       </c>
       <c r="F1920" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1920" t="inlineStr"/>
@@ -66583,7 +66586,7 @@
       </c>
       <c r="F1925" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1925" t="inlineStr"/>
@@ -66617,7 +66620,7 @@
       </c>
       <c r="F1926" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1926" t="inlineStr"/>
@@ -66889,7 +66892,7 @@
       </c>
       <c r="F1934" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1934" t="inlineStr"/>
@@ -67025,7 +67028,7 @@
       </c>
       <c r="F1938" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1938" t="inlineStr"/>
@@ -67127,7 +67130,7 @@
       </c>
       <c r="F1941" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1941" t="inlineStr"/>
@@ -67229,7 +67232,7 @@
       </c>
       <c r="F1944" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1944" t="inlineStr"/>
@@ -67305,7 +67308,7 @@
       </c>
       <c r="F1946" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1946" t="inlineStr"/>
@@ -67377,7 +67380,7 @@
       </c>
       <c r="F1948" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1948" t="inlineStr"/>
@@ -67887,7 +67890,7 @@
       </c>
       <c r="F1963" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1963" t="inlineStr"/>
@@ -68167,7 +68170,7 @@
       </c>
       <c r="F1971" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1971" t="inlineStr"/>
@@ -68337,7 +68340,7 @@
       </c>
       <c r="F1976" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1976" t="inlineStr"/>
@@ -68435,7 +68438,7 @@
       </c>
       <c r="F1979" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1979" t="inlineStr"/>
@@ -69565,7 +69568,7 @@
       </c>
       <c r="F2012" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2012" t="inlineStr"/>
@@ -69599,7 +69602,7 @@
       </c>
       <c r="F2013" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2013" t="inlineStr"/>
@@ -69811,7 +69814,7 @@
       </c>
       <c r="F2019" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2019" t="inlineStr"/>
@@ -69913,7 +69916,7 @@
       </c>
       <c r="F2022" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2022" t="inlineStr"/>
@@ -70839,7 +70842,7 @@
       </c>
       <c r="F2049" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2049" t="inlineStr"/>
@@ -71179,7 +71182,7 @@
       </c>
       <c r="F2059" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2059" t="inlineStr"/>
@@ -72309,7 +72312,7 @@
       </c>
       <c r="F2092" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2092" t="inlineStr"/>
@@ -72547,7 +72550,7 @@
       </c>
       <c r="F2099" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2099" t="inlineStr"/>
@@ -73209,7 +73212,7 @@
       </c>
       <c r="F2118" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2118" t="inlineStr"/>
@@ -73757,7 +73760,7 @@
       </c>
       <c r="F2134" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2134" t="inlineStr"/>
@@ -73930,8 +73933,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2139" t="inlineStr"/>
-      <c r="H2139" t="inlineStr"/>
+      <c r="G2139" t="inlineStr">
+        <is>
+          <t>Fudo's Assurances (Celestial, Coils of Madness): not wired whole. Battle/Open: Straighten a Ring is buildable, but Open: 'If you control five Fudo Rings that last entered play by their own text, destroy a Province' needs a per-Ring record of HOW it last entered play (by its own text, as the False Rings do, versus recruited, Searched or put into play by another card), and the engine records only that a Ring is in play (the Ring-search entry marks only the Enlightenment count). The only Fudo Rings are the six False Rings, none of which is wired (they exist only as training fixtures). Needs the entry-provenance record (PROVENANCE) and the False Rings wired first; a card with two printed lines is wired whole or blocked.</t>
+        </is>
+      </c>
+      <c r="H2139" t="inlineStr">
+        <is>
+          <t>PROVENANCE</t>
+        </is>
+      </c>
     </row>
     <row r="2140">
       <c r="A2140" t="inlineStr">
@@ -73995,7 +74006,7 @@
       </c>
       <c r="F2141" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2141" t="inlineStr"/>
@@ -74763,7 +74774,7 @@
       </c>
       <c r="F2163" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2163" t="inlineStr"/>
@@ -75829,7 +75840,7 @@
       </c>
       <c r="F2194" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2194" t="inlineStr">
@@ -75901,7 +75912,7 @@
       </c>
       <c r="F2196" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2196" t="inlineStr">
@@ -76258,7 +76269,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -76338,7 +76349,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -76418,7 +76429,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -76518,7 +76529,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Art pack r2 on #672's base, inventory, handoff for #674
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A29buqY4H1Xgn5ZxyHvSrq
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M27"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -468,7 +468,6 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -532,14 +531,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>655</v>
+        <v>742</v>
       </c>
       <c r="C6" t="n">
         <v>839</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>78.1%</t>
+          <t>88.4%</t>
         </is>
       </c>
     </row>
@@ -550,14 +549,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C7" t="n">
         <v>137</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>89.1%</t>
+          <t>92.7%</t>
         </is>
       </c>
     </row>
@@ -568,14 +567,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="C8" t="n">
         <v>136</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>79.4%</t>
+          <t>85.3%</t>
         </is>
       </c>
     </row>
@@ -586,14 +585,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>72.9%</t>
+          <t>83.5%</t>
         </is>
       </c>
     </row>
@@ -604,14 +603,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>486</v>
+        <v>545</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>81.3%</t>
+          <t>91.1%</t>
         </is>
       </c>
     </row>
@@ -622,14 +621,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="C11" t="n">
         <v>152</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>77.6%</t>
+          <t>90.1%</t>
         </is>
       </c>
     </row>
@@ -640,14 +639,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>71.6%</t>
+          <t>77.8%</t>
         </is>
       </c>
     </row>
@@ -658,14 +657,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C13" t="n">
         <v>37</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>67.6%</t>
+          <t>75.7%</t>
         </is>
       </c>
     </row>
@@ -694,14 +693,14 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C15" t="n">
         <v>10</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -712,14 +711,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1749</v>
+        <v>1951</v>
       </c>
       <c r="C16" t="n">
         <v>2200</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>79.5%</t>
+          <t>88.7%</t>
         </is>
       </c>
     </row>
@@ -788,11 +787,6 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Ring</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
           <t>TOTAL</t>
         </is>
       </c>
@@ -800,149 +794,137 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Torn Asunder</t>
+          <t>Coils of Madness</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>42</v>
-      </c>
-      <c r="D20" t="n">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="E20" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" t="n">
+        <v>9</v>
+      </c>
+      <c r="H20" t="n">
+        <v>2</v>
+      </c>
+      <c r="I20" t="n">
         <v>6</v>
       </c>
-      <c r="F20" t="n">
-        <v>12</v>
-      </c>
-      <c r="G20" t="n">
-        <v>39</v>
-      </c>
-      <c r="H20" t="n">
-        <v>6</v>
-      </c>
-      <c r="I20" t="n">
-        <v>5</v>
-      </c>
       <c r="J20" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" t="n">
-        <v>1</v>
-      </c>
-      <c r="M20" t="n">
-        <v>117</v>
+        <v>3</v>
+      </c>
+      <c r="L20" t="n">
+        <v>69</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Coils of Madness</t>
+          <t>Torn Asunder</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D21" t="n">
         <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G21" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="H21" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>8</v>
-      </c>
-      <c r="J21" t="n">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>2</v>
-      </c>
-      <c r="M21" t="n">
-        <v>116</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Gates of Chaos</t>
+          <t>Aftermath</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="D22" t="n">
         <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G22" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="H22" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
-      </c>
-      <c r="M22" t="n">
-        <v>101</v>
+        <v>2</v>
+      </c>
+      <c r="L22" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aftermath</t>
+          <t>Gates of Chaos</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="D23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>5</v>
+      </c>
+      <c r="F23" t="n">
         <v>4</v>
       </c>
-      <c r="E23" t="n">
-        <v>7</v>
-      </c>
-      <c r="F23" t="n">
-        <v>10</v>
-      </c>
       <c r="G23" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>3</v>
-      </c>
-      <c r="J23" t="n">
-        <v>3</v>
-      </c>
-      <c r="M23" t="n">
-        <v>95</v>
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="24">
@@ -969,7 +951,7 @@
       <c r="K24" t="n">
         <v>1</v>
       </c>
-      <c r="M24" t="n">
+      <c r="L24" t="n">
         <v>12</v>
       </c>
     </row>
@@ -991,7 +973,7 @@
       <c r="J25" t="n">
         <v>2</v>
       </c>
-      <c r="M25" t="n">
+      <c r="L25" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1004,7 +986,7 @@
       <c r="G26" t="n">
         <v>2</v>
       </c>
-      <c r="M26" t="n">
+      <c r="L26" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1018,37 +1000,34 @@
         <v>3</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>184</v>
+        <v>97</v>
       </c>
       <c r="D27" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="H27" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="E27" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="G27" s="2" t="n">
-        <v>112</v>
-      </c>
-      <c r="H27" s="2" t="n">
-        <v>34</v>
-      </c>
       <c r="I27" s="2" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>2</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M27" s="2" t="n">
-        <v>451</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -3835,7 +3814,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4001,7 +3980,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G86" t="inlineStr"/>
@@ -4171,7 +4150,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
@@ -4341,7 +4320,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G96" t="inlineStr"/>
@@ -4613,7 +4592,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G104" t="inlineStr"/>
@@ -4715,7 +4694,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G107" t="inlineStr"/>
@@ -4783,7 +4762,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G109" t="inlineStr"/>
@@ -4953,7 +4932,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G114" t="inlineStr"/>
@@ -5055,7 +5034,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
@@ -5361,7 +5340,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G126" t="inlineStr"/>
@@ -5731,7 +5710,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G137" t="inlineStr"/>
@@ -6887,7 +6866,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G171" t="inlineStr"/>
@@ -6989,7 +6968,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -7061,7 +7040,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G176" t="inlineStr"/>
@@ -7431,7 +7410,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G187" t="inlineStr"/>
@@ -7567,7 +7546,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G191" t="inlineStr"/>
@@ -7873,7 +7852,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G200" t="inlineStr"/>
@@ -7907,7 +7886,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G201" t="inlineStr"/>
@@ -7941,7 +7920,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G202" t="inlineStr"/>
@@ -8077,7 +8056,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G206" t="inlineStr"/>
@@ -8281,7 +8260,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
@@ -8319,7 +8298,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G213" t="inlineStr"/>
@@ -9633,7 +9612,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G252" t="inlineStr"/>
@@ -9803,7 +9782,7 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G257" t="inlineStr"/>
@@ -10237,7 +10216,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G270" t="inlineStr"/>
@@ -11241,7 +11220,7 @@
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G300" t="inlineStr"/>
@@ -12087,7 +12066,7 @@
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G325" t="inlineStr"/>
@@ -12321,7 +12300,7 @@
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G332" t="inlineStr"/>
@@ -12427,7 +12406,7 @@
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G335" t="inlineStr"/>
@@ -12461,7 +12440,7 @@
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G336" t="inlineStr"/>
@@ -13259,7 +13238,7 @@
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G359" t="inlineStr"/>
@@ -14143,7 +14122,7 @@
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G385" t="inlineStr"/>
@@ -14347,7 +14326,7 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G391" t="inlineStr"/>
@@ -14415,7 +14394,7 @@
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G393" t="inlineStr"/>
@@ -14759,7 +14738,7 @@
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G403" t="inlineStr"/>
@@ -14963,7 +14942,7 @@
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G409" t="inlineStr"/>
@@ -15269,7 +15248,7 @@
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G418" t="inlineStr"/>
@@ -15337,7 +15316,7 @@
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G420" t="inlineStr"/>
@@ -15885,7 +15864,7 @@
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G436" t="inlineStr"/>
@@ -16501,7 +16480,7 @@
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G454" t="inlineStr">
@@ -16641,7 +16620,7 @@
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G458" t="inlineStr">
@@ -17461,7 +17440,7 @@
       </c>
       <c r="F482" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G482" t="inlineStr"/>
@@ -17937,7 +17916,7 @@
       </c>
       <c r="F496" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G496" t="inlineStr"/>
@@ -18069,7 +18048,7 @@
       </c>
       <c r="F500" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G500" t="inlineStr"/>
@@ -19161,7 +19140,7 @@
       </c>
       <c r="F532" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G532" t="inlineStr">
@@ -19339,7 +19318,7 @@
       </c>
       <c r="F537" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G537" t="inlineStr">
@@ -19891,7 +19870,7 @@
       </c>
       <c r="F553" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G553" t="inlineStr"/>
@@ -20027,7 +20006,7 @@
       </c>
       <c r="F557" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G557" t="inlineStr"/>
@@ -20197,7 +20176,7 @@
       </c>
       <c r="F562" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G562" t="inlineStr"/>
@@ -20503,7 +20482,7 @@
       </c>
       <c r="F571" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G571" t="inlineStr"/>
@@ -21013,7 +20992,7 @@
       </c>
       <c r="F586" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G586" t="inlineStr"/>
@@ -21485,7 +21464,7 @@
       </c>
       <c r="F600" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G600" t="inlineStr"/>
@@ -22119,7 +22098,7 @@
       </c>
       <c r="F619" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G619" t="inlineStr"/>
@@ -22659,7 +22638,7 @@
       </c>
       <c r="F635" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G635" t="inlineStr"/>
@@ -22727,7 +22706,7 @@
       </c>
       <c r="F637" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G637" t="inlineStr"/>
@@ -23101,7 +23080,7 @@
       </c>
       <c r="F648" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G648" t="inlineStr"/>
@@ -23237,7 +23216,7 @@
       </c>
       <c r="F652" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G652" t="inlineStr"/>
@@ -23951,7 +23930,7 @@
       </c>
       <c r="F673" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G673" t="inlineStr"/>
@@ -23985,7 +23964,7 @@
       </c>
       <c r="F674" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G674" t="inlineStr"/>
@@ -24087,7 +24066,7 @@
       </c>
       <c r="F677" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G677" t="inlineStr"/>
@@ -24155,7 +24134,7 @@
       </c>
       <c r="F679" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G679" t="inlineStr"/>
@@ -24461,7 +24440,7 @@
       </c>
       <c r="F688" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G688" t="inlineStr"/>
@@ -24631,7 +24610,7 @@
       </c>
       <c r="F693" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G693" t="inlineStr"/>
@@ -24665,7 +24644,7 @@
       </c>
       <c r="F694" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G694" t="inlineStr"/>
@@ -25141,7 +25120,7 @@
       </c>
       <c r="F708" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G708" t="inlineStr"/>
@@ -25243,7 +25222,7 @@
       </c>
       <c r="F711" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G711" t="inlineStr"/>
@@ -25481,7 +25460,7 @@
       </c>
       <c r="F718" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G718" t="inlineStr"/>
@@ -25719,7 +25698,7 @@
       </c>
       <c r="F725" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G725" t="inlineStr"/>
@@ -26403,7 +26382,7 @@
       </c>
       <c r="F745" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G745" t="inlineStr"/>
@@ -26471,7 +26450,7 @@
       </c>
       <c r="F747" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G747" t="inlineStr"/>
@@ -27615,7 +27594,7 @@
       </c>
       <c r="F781" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G781" t="inlineStr"/>
@@ -27683,7 +27662,7 @@
       </c>
       <c r="F783" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G783" t="inlineStr"/>
@@ -27955,7 +27934,7 @@
       </c>
       <c r="F791" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G791" t="inlineStr"/>
@@ -28329,7 +28308,7 @@
       </c>
       <c r="F802" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G802" t="inlineStr"/>
@@ -28605,7 +28584,7 @@
       </c>
       <c r="F810" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G810" t="inlineStr"/>
@@ -29013,7 +28992,7 @@
       </c>
       <c r="F822" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G822" t="inlineStr"/>
@@ -29081,7 +29060,7 @@
       </c>
       <c r="F824" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G824" t="inlineStr"/>
@@ -29447,7 +29426,7 @@
       </c>
       <c r="F835" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G835" t="inlineStr"/>
@@ -29481,7 +29460,7 @@
       </c>
       <c r="F836" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G836" t="inlineStr"/>
@@ -29651,7 +29630,7 @@
       </c>
       <c r="F841" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G841" t="inlineStr"/>
@@ -29787,7 +29766,7 @@
       </c>
       <c r="F845" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G845" t="inlineStr"/>
@@ -30025,7 +30004,7 @@
       </c>
       <c r="F852" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G852" t="inlineStr"/>
@@ -30059,7 +30038,7 @@
       </c>
       <c r="F853" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G853" t="inlineStr"/>
@@ -30399,7 +30378,7 @@
       </c>
       <c r="F863" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G863" t="inlineStr"/>
@@ -30671,7 +30650,7 @@
       </c>
       <c r="F871" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G871" t="inlineStr"/>
@@ -30913,7 +30892,7 @@
       </c>
       <c r="F878" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G878" t="inlineStr"/>
@@ -31015,7 +30994,7 @@
       </c>
       <c r="F881" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G881" t="inlineStr"/>
@@ -34067,7 +34046,7 @@
       </c>
       <c r="F971" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G971" t="inlineStr">
@@ -34641,7 +34620,7 @@
       </c>
       <c r="F988" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G988" t="inlineStr">
@@ -35049,7 +35028,7 @@
       </c>
       <c r="F1000" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1000" t="inlineStr">
@@ -35317,7 +35296,7 @@
       </c>
       <c r="F1008" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1008" t="inlineStr">
@@ -35389,7 +35368,7 @@
       </c>
       <c r="F1010" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1010" t="inlineStr">
@@ -37135,7 +37114,7 @@
       </c>
       <c r="F1061" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1061" t="inlineStr"/>
@@ -37675,7 +37654,7 @@
       </c>
       <c r="F1077" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1077" t="inlineStr"/>
@@ -37867,7 +37846,7 @@
       </c>
       <c r="F1083" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1083" t="inlineStr"/>
@@ -38071,7 +38050,7 @@
       </c>
       <c r="F1089" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1089" t="inlineStr"/>
@@ -38747,7 +38726,7 @@
       </c>
       <c r="F1109" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1109" t="inlineStr"/>
@@ -39057,7 +39036,7 @@
       </c>
       <c r="F1118" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1118" t="inlineStr"/>
@@ -39567,7 +39546,7 @@
       </c>
       <c r="F1133" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1133" t="inlineStr"/>
@@ -40217,7 +40196,7 @@
       </c>
       <c r="F1152" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1152" t="inlineStr"/>
@@ -40723,7 +40702,7 @@
       </c>
       <c r="F1167" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1167" t="inlineStr"/>
@@ -40791,7 +40770,7 @@
       </c>
       <c r="F1169" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1169" t="inlineStr"/>
@@ -40927,7 +40906,7 @@
       </c>
       <c r="F1173" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1173" t="inlineStr"/>
@@ -40961,7 +40940,7 @@
       </c>
       <c r="F1174" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1174" t="inlineStr"/>
@@ -41097,7 +41076,7 @@
       </c>
       <c r="F1178" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1178" t="inlineStr"/>
@@ -41947,7 +41926,7 @@
       </c>
       <c r="F1203" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1203" t="inlineStr"/>
@@ -42117,7 +42096,7 @@
       </c>
       <c r="F1208" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1208" t="inlineStr"/>
@@ -42733,7 +42712,7 @@
       </c>
       <c r="F1226" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1226" t="inlineStr"/>
@@ -43144,8 +43123,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1238" t="inlineStr"/>
-      <c r="H1238" t="inlineStr"/>
+      <c r="G1238" t="inlineStr">
+        <is>
+          <t>Read the Essence (Spell, Torn Asunder, issue #674): "Open: Bow this card and target one face-down card in a province, or one or two such cards if this Shugenja is Void: Turn the targets face-up." Everything else exists (a bow-this-card cost; Second City's Political Open turns a face-down card face-up), but the engine names a face-down province card only by its province (the any-province command parameter, TargetPlayerId + Province, because a face-down card's id is hidden from the view), and that is ONE card. A Void Shugenja's "one or two" needs a second province in the same command (and a pair listing in QueryActions); no multi-province selection exists, and a card id may not be used (hidden information). Question for Mendon: may the Void version be two separate entries (one province each) sharing one use, or is a two-province selection UI wanted?</t>
+        </is>
+      </c>
+      <c r="H1238" t="inlineStr">
+        <is>
+          <t>HIDDEN</t>
+        </is>
+      </c>
     </row>
     <row r="1239">
       <c r="A1239" t="inlineStr">
@@ -43413,7 +43400,7 @@
       </c>
       <c r="F1246" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1246" t="inlineStr"/>
@@ -43617,7 +43604,7 @@
       </c>
       <c r="F1252" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1252" t="inlineStr"/>
@@ -43787,7 +43774,7 @@
       </c>
       <c r="F1257" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1257" t="inlineStr"/>
@@ -43991,7 +43978,7 @@
       </c>
       <c r="F1263" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1263" t="inlineStr"/>
@@ -44365,7 +44352,7 @@
       </c>
       <c r="F1274" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1274" t="inlineStr"/>
@@ -44467,7 +44454,7 @@
       </c>
       <c r="F1277" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1277" t="inlineStr"/>
@@ -45014,8 +45001,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1293" t="inlineStr"/>
-      <c r="H1293" t="inlineStr"/>
+      <c r="G1293" t="inlineStr">
+        <is>
+          <t>Witness the Untold (Spell, Torn Asunder, issue #674): "Reaction: After your Ring enters play, bow this card: Look at the top three cards of your Dynasty or Fate deck. Put them back in any order." The look and reorder exist (LookSpec, It Was a Cat's shape: either deck, three cards, reorder only), but nothing narrates a Ring entering play: every Ring is put into play by its own recruit case (RingEnteredByOwnText) and no Reaction trigger "after your Ring enters play" exists for another card to listen to (the Ring-entering gap the TRIG-AFTER category names). Needs a new reaction trigger fired from every Ring's entry, which is shared-interface work.</t>
+        </is>
+      </c>
+      <c r="H1293" t="inlineStr">
+        <is>
+          <t>TRIG-AFTER</t>
+        </is>
+      </c>
     </row>
     <row r="1294">
       <c r="A1294" t="inlineStr">
@@ -45725,7 +45720,7 @@
       </c>
       <c r="F1314" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1314" t="inlineStr"/>
@@ -45793,7 +45788,7 @@
       </c>
       <c r="F1316" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1316" t="inlineStr"/>
@@ -46201,7 +46196,7 @@
       </c>
       <c r="F1328" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1328" t="inlineStr"/>
@@ -46303,7 +46298,7 @@
       </c>
       <c r="F1331" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1331" t="inlineStr"/>
@@ -46813,7 +46808,7 @@
       </c>
       <c r="F1346" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1346" t="inlineStr"/>
@@ -47088,8 +47083,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1354" t="inlineStr"/>
-      <c r="H1354" t="inlineStr"/>
+      <c r="G1354" t="inlineStr">
+        <is>
+          <t>Benediction (Aftermath, Strategy; scan verified): "Open: Destroy your target Holding. Give a Province +3 strength." Two independent targets of different kinds, a card (your Holding) and a province (either player's, Ring of Earth's 'any-province' shape: GameCommand.Province plus TargetPlayerId). The engine has no ability that names a card and a province together: a multi-target ability is Slots (cards or players only), while the province categories ('any-province', 'enemy-province') are mutually exclusive with a card target in ValidateAbility and in the QueryActions candidate loop (one candidate per province/owner, no card). Wiring it needs a province target slot kind (TargetSlotKinds.Province with a SlotSelection province index and owner, validated in ValidateSlotCard and offered by SlotAbilityOption, plus the client picking a province inside a slot ability). That is a new decision shape for the client, not a local feature addition. Everything else is built: the effect itself is DestroyAttachment-free (DestroyUnits/Holding destroy, then GiveProvinceStrengthThisTurn(owner, index, 3)). QUESTION for Mendon: is 'Give a Province +3 strength' until end of turn (R-001 default, GiveProvinceStrengthThisTurn as Ring of Earth) and may the Province be either player's?</t>
+        </is>
+      </c>
+      <c r="H1354" t="inlineStr">
+        <is>
+          <t>TARGET</t>
+        </is>
+      </c>
     </row>
     <row r="1355">
       <c r="A1355" t="inlineStr">
@@ -47289,7 +47292,7 @@
       </c>
       <c r="F1360" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1360" t="inlineStr"/>
@@ -47731,7 +47734,7 @@
       </c>
       <c r="F1373" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1373" t="inlineStr"/>
@@ -47901,7 +47904,7 @@
       </c>
       <c r="F1378" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1378" t="inlineStr">
@@ -48007,7 +48010,7 @@
       </c>
       <c r="F1381" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1381" t="inlineStr"/>
@@ -48075,7 +48078,7 @@
       </c>
       <c r="F1383" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1383" t="inlineStr"/>
@@ -48347,7 +48350,7 @@
       </c>
       <c r="F1391" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1391" t="inlineStr"/>
@@ -48925,7 +48928,7 @@
       </c>
       <c r="F1408" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1408" t="inlineStr">
@@ -49031,7 +49034,7 @@
       </c>
       <c r="F1411" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1411" t="inlineStr"/>
@@ -49133,7 +49136,7 @@
       </c>
       <c r="F1414" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1414" t="inlineStr"/>
@@ -49847,7 +49850,7 @@
       </c>
       <c r="F1435" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1435" t="inlineStr"/>
@@ -50289,7 +50292,7 @@
       </c>
       <c r="F1448" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1448" t="inlineStr"/>
@@ -50323,7 +50326,7 @@
       </c>
       <c r="F1449" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1449" t="inlineStr"/>
@@ -50459,7 +50462,7 @@
       </c>
       <c r="F1453" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1453" t="inlineStr"/>
@@ -50901,7 +50904,7 @@
       </c>
       <c r="F1466" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1466" t="inlineStr"/>
@@ -51139,7 +51142,7 @@
       </c>
       <c r="F1473" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1473" t="inlineStr"/>
@@ -51275,7 +51278,7 @@
       </c>
       <c r="F1477" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1477" t="inlineStr"/>
@@ -51377,7 +51380,7 @@
       </c>
       <c r="F1480" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1480" t="inlineStr"/>
@@ -52647,7 +52650,7 @@
       </c>
       <c r="F1517" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1517" t="inlineStr"/>
@@ -52749,7 +52752,7 @@
       </c>
       <c r="F1520" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1520" t="inlineStr"/>
@@ -52953,7 +52956,7 @@
       </c>
       <c r="F1526" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1526" t="inlineStr"/>
@@ -53021,7 +53024,7 @@
       </c>
       <c r="F1528" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1528" t="inlineStr"/>
@@ -53089,7 +53092,7 @@
       </c>
       <c r="F1530" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1530" t="inlineStr"/>
@@ -53709,7 +53712,7 @@
       </c>
       <c r="F1548" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1548" t="inlineStr"/>
@@ -54219,7 +54222,7 @@
       </c>
       <c r="F1563" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1563" t="inlineStr">
@@ -54257,7 +54260,7 @@
       </c>
       <c r="F1564" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1564" t="inlineStr">
@@ -54329,7 +54332,7 @@
       </c>
       <c r="F1566" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1566" t="inlineStr"/>
@@ -54363,7 +54366,7 @@
       </c>
       <c r="F1567" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1567" t="inlineStr"/>
@@ -54605,7 +54608,7 @@
       </c>
       <c r="F1574" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1574" t="inlineStr"/>
@@ -54877,7 +54880,7 @@
       </c>
       <c r="F1582" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1582" t="inlineStr"/>
@@ -54911,7 +54914,7 @@
       </c>
       <c r="F1583" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1583" t="inlineStr"/>
@@ -54979,7 +54982,7 @@
       </c>
       <c r="F1585" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1585" t="inlineStr"/>
@@ -55595,7 +55598,7 @@
       </c>
       <c r="F1603" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1603" t="inlineStr"/>
@@ -55701,7 +55704,7 @@
       </c>
       <c r="F1606" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1606" t="inlineStr"/>
@@ -56075,7 +56078,7 @@
       </c>
       <c r="F1617" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1617" t="inlineStr"/>
@@ -56585,7 +56588,7 @@
       </c>
       <c r="F1632" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1632" t="inlineStr"/>
@@ -57027,7 +57030,7 @@
       </c>
       <c r="F1645" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1645" t="inlineStr"/>
@@ -57299,7 +57302,7 @@
       </c>
       <c r="F1653" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1653" t="inlineStr"/>
@@ -58217,7 +58220,7 @@
       </c>
       <c r="F1680" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1680" t="inlineStr"/>
@@ -59237,7 +59240,7 @@
       </c>
       <c r="F1710" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1710" t="inlineStr"/>
@@ -60019,7 +60022,7 @@
       </c>
       <c r="F1733" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1733" t="inlineStr"/>
@@ -60907,7 +60910,7 @@
       </c>
       <c r="F1759" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1759" t="inlineStr"/>
@@ -61281,7 +61284,7 @@
       </c>
       <c r="F1770" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1770" t="inlineStr"/>
@@ -61315,7 +61318,7 @@
       </c>
       <c r="F1771" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1771" t="inlineStr"/>
@@ -61897,7 +61900,7 @@
       </c>
       <c r="F1788" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1788" t="inlineStr"/>
@@ -61931,7 +61934,7 @@
       </c>
       <c r="F1789" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1789" t="inlineStr"/>
@@ -62271,7 +62274,7 @@
       </c>
       <c r="F1799" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1799" t="inlineStr"/>
@@ -62339,7 +62342,7 @@
       </c>
       <c r="F1801" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1801" t="inlineStr">
@@ -62513,7 +62516,7 @@
       </c>
       <c r="F1806" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1806" t="inlineStr"/>
@@ -63023,7 +63026,7 @@
       </c>
       <c r="F1821" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1821" t="inlineStr"/>
@@ -63091,7 +63094,7 @@
       </c>
       <c r="F1823" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1823" t="inlineStr"/>
@@ -63261,7 +63264,7 @@
       </c>
       <c r="F1828" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1828" t="inlineStr">
@@ -63537,7 +63540,7 @@
       </c>
       <c r="F1836" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1836" t="inlineStr"/>
@@ -64047,7 +64050,7 @@
       </c>
       <c r="F1851" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1851" t="inlineStr"/>
@@ -64421,7 +64424,7 @@
       </c>
       <c r="F1862" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1862" t="inlineStr"/>
@@ -65793,7 +65796,7 @@
       </c>
       <c r="F1902" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1902" t="inlineStr"/>
@@ -65997,7 +66000,7 @@
       </c>
       <c r="F1908" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1908" t="inlineStr"/>
@@ -66401,7 +66404,7 @@
       </c>
       <c r="F1920" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1920" t="inlineStr"/>
@@ -66579,7 +66582,7 @@
       </c>
       <c r="F1925" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1925" t="inlineStr"/>
@@ -66613,7 +66616,7 @@
       </c>
       <c r="F1926" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1926" t="inlineStr"/>
@@ -66885,7 +66888,7 @@
       </c>
       <c r="F1934" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1934" t="inlineStr"/>
@@ -67021,7 +67024,7 @@
       </c>
       <c r="F1938" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1938" t="inlineStr"/>
@@ -67123,7 +67126,7 @@
       </c>
       <c r="F1941" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1941" t="inlineStr"/>
@@ -67225,7 +67228,7 @@
       </c>
       <c r="F1944" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1944" t="inlineStr"/>
@@ -67301,7 +67304,7 @@
       </c>
       <c r="F1946" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1946" t="inlineStr"/>
@@ -67373,7 +67376,7 @@
       </c>
       <c r="F1948" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1948" t="inlineStr"/>
@@ -67883,7 +67886,7 @@
       </c>
       <c r="F1963" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1963" t="inlineStr"/>
@@ -68163,7 +68166,7 @@
       </c>
       <c r="F1971" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1971" t="inlineStr"/>
@@ -68333,7 +68336,7 @@
       </c>
       <c r="F1976" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1976" t="inlineStr"/>
@@ -68431,7 +68434,7 @@
       </c>
       <c r="F1979" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1979" t="inlineStr"/>
@@ -69561,7 +69564,7 @@
       </c>
       <c r="F2012" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2012" t="inlineStr"/>
@@ -69595,7 +69598,7 @@
       </c>
       <c r="F2013" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2013" t="inlineStr"/>
@@ -69807,7 +69810,7 @@
       </c>
       <c r="F2019" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2019" t="inlineStr"/>
@@ -69909,7 +69912,7 @@
       </c>
       <c r="F2022" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2022" t="inlineStr"/>
@@ -70835,7 +70838,7 @@
       </c>
       <c r="F2049" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2049" t="inlineStr"/>
@@ -71175,7 +71178,7 @@
       </c>
       <c r="F2059" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2059" t="inlineStr"/>
@@ -72305,7 +72308,7 @@
       </c>
       <c r="F2092" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2092" t="inlineStr"/>
@@ -72543,7 +72546,7 @@
       </c>
       <c r="F2099" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2099" t="inlineStr"/>
@@ -73205,7 +73208,7 @@
       </c>
       <c r="F2118" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2118" t="inlineStr"/>
@@ -73753,7 +73756,7 @@
       </c>
       <c r="F2134" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2134" t="inlineStr"/>
@@ -73926,8 +73929,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2139" t="inlineStr"/>
-      <c r="H2139" t="inlineStr"/>
+      <c r="G2139" t="inlineStr">
+        <is>
+          <t>Fudo's Assurances (Celestial, Coils of Madness): not wired whole. Battle/Open: Straighten a Ring is buildable, but Open: 'If you control five Fudo Rings that last entered play by their own text, destroy a Province' needs a per-Ring record of HOW it last entered play (by its own text, as the False Rings do, versus recruited, Searched or put into play by another card), and the engine records only that a Ring is in play (the Ring-search entry marks only the Enlightenment count). The only Fudo Rings are the six False Rings, none of which is wired (they exist only as training fixtures). Needs the entry-provenance record (PROVENANCE) and the False Rings wired first; a card with two printed lines is wired whole or blocked.</t>
+        </is>
+      </c>
+      <c r="H2139" t="inlineStr">
+        <is>
+          <t>PROVENANCE</t>
+        </is>
+      </c>
     </row>
     <row r="2140">
       <c r="A2140" t="inlineStr">
@@ -73991,7 +74002,7 @@
       </c>
       <c r="F2141" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2141" t="inlineStr"/>
@@ -74759,7 +74770,7 @@
       </c>
       <c r="F2163" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2163" t="inlineStr"/>
@@ -75825,7 +75836,7 @@
       </c>
       <c r="F2194" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2194" t="inlineStr">
@@ -75897,7 +75908,7 @@
       </c>
       <c r="F2196" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2196" t="inlineStr">
@@ -76254,7 +76265,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -76334,7 +76345,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -76414,7 +76425,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -76514,7 +76525,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wire 26 cards unlocked by P2, P7 and P11 (#689)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -531,14 +531,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>762</v>
+        <v>779</v>
       </c>
       <c r="C6" t="n">
         <v>851</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>89.5%</t>
+          <t>91.5%</t>
         </is>
       </c>
     </row>
@@ -549,14 +549,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C7" t="n">
         <v>141</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>93.6%</t>
+          <t>94.3%</t>
         </is>
       </c>
     </row>
@@ -585,14 +585,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>85.0%</t>
+          <t>86.5%</t>
         </is>
       </c>
     </row>
@@ -603,14 +603,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>92.0%</t>
+          <t>93.0%</t>
         </is>
       </c>
     </row>
@@ -711,14 +711,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1986</v>
+        <v>2012</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>89.6%</t>
+          <t>90.8%</t>
         </is>
       </c>
     </row>
@@ -801,13 +801,13 @@
         <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="E20" t="n">
         <v>5</v>
       </c>
       <c r="F20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
         <v>9</v>
@@ -822,7 +822,7 @@
         <v>3</v>
       </c>
       <c r="L20" t="n">
-        <v>67</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21">
@@ -835,7 +835,7 @@
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D21" t="n">
         <v>2</v>
@@ -844,10 +844,10 @@
         <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G21" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H21" t="n">
         <v>1</v>
@@ -859,7 +859,7 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22">
@@ -869,10 +869,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E22" t="n">
         <v>6</v>
@@ -881,7 +881,7 @@
         <v>4</v>
       </c>
       <c r="G22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H22" t="n">
         <v>2</v>
@@ -893,7 +893,7 @@
         <v>2</v>
       </c>
       <c r="L22" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23">
@@ -903,7 +903,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D23" t="n">
         <v>3</v>
@@ -915,7 +915,7 @@
         <v>4</v>
       </c>
       <c r="G23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
@@ -924,7 +924,7 @@
         <v>2</v>
       </c>
       <c r="L23" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24">
@@ -1000,19 +1000,19 @@
         <v>3</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>19</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H27" s="2" t="n">
         <v>14</v>
@@ -1027,7 +1027,7 @@
         <v>2</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>231</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -4391,8 +4391,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Needs P6 (after-event records and windows); P7's watch half alone does not wire it.</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4456,7 +4464,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G100" t="inlineStr"/>
@@ -4901,8 +4909,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr"/>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Needs an effective Force cap after all bonuses and a source-unit action target restriction.</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5974,7 +5990,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G145" t="inlineStr"/>
@@ -6011,8 +6027,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G146" t="inlineStr"/>
-      <c r="H146" t="inlineStr"/>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Needs P9 (conditional -1F statics for Fallen, Nonhuman and attacking-you cards) and an after-next-attack Honor loss; not wired in #689.</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -6212,7 +6236,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G152" t="inlineStr"/>
@@ -8460,7 +8484,7 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G218" t="inlineStr"/>
@@ -8771,12 +8795,12 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>Daigotsu Kikumura (Personality, issue #677): the two 1F Followers his Invest creates are the published Farmlands Conscripts (oracle-l5r-10004), and Invest 4 is Clay Kshatriya's entering-play window. "If you are a Dragon Clan player, Kikumura's Invest is 2" is a price that depends on the player: a Gold cost rule (GoldCostRule) has no player-Clan condition. The usual split into two abilities that share one use (Moto Hailung's discount) does not work in the entering-play window, where an ability with no target is listed without being validated (MatchQueries.AddReaction): both prices would be offered to every player and the wrong one refused only when used.</t>
+          <t>Not wired in #689 (draft wiring removed untested): Invest cost by Clan (a P2 ability cost term) creating two 1F Followers on Kikumura needs its own card pass, the Follower proxy check and tests.</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>LOCK</t>
         </is>
       </c>
     </row>
@@ -10986,7 +11010,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G293" t="inlineStr"/>
@@ -11427,8 +11451,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G306" t="inlineStr"/>
-      <c r="H306" t="inlineStr"/>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Needs same-army exclusions during movement and entry and unopposed Force/printed-cost accounting.</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -11967,8 +11999,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G322" t="inlineStr"/>
-      <c r="H322" t="inlineStr"/>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>Needs a controller choice when multiple attached Followers would be destroyed simultaneously; a per-card watch cannot choose which single destruction to negate.</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -13887,8 +13927,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G378" t="inlineStr"/>
-      <c r="H378" t="inlineStr"/>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>Needs same-army exclusions during movement and entry; a battlefield bar incorrectly forbids opposing armies.</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -14742,7 +14790,7 @@
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G403" t="inlineStr">
@@ -15800,7 +15848,7 @@
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G434" t="inlineStr">
@@ -17615,12 +17663,12 @@
       </c>
       <c r="G487" t="inlineStr">
         <is>
-          <t>Kitsune Yuribara (Personality, issue #677): her created card's scan is published (Yuribara's Butterflies, oracle-l5r-10808), but the Butterflies print two traits the engine does not have, so nothing may create them yet. "Other player's Battle actions must target a Butterfly Personality at this battlefield, if legal" is a forced-target rule over every Battle action the other player takes at that battlefield: target legality has bars (TargetBars.cs, TargetOfLastResort.cs) but no rule that makes one card the only legal target while it is one, for single targets, slots and Attacks alike. "After another player's Battle action targets this card: Destroy this card" is a mandatory trait on being targeted; the targeted-by-action window offers optional Reactions only. Yuribara's own Reaction (create the Butterflies after she enters play) is Kitsu Tamao's shape and needs nothing new.</t>
+          <t>Needs verified Butterfly proxy traits and alternative target selection with destruction after targeting.</t>
         </is>
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>TARGET</t>
+          <t>LOCK</t>
         </is>
       </c>
     </row>
@@ -17788,7 +17836,7 @@
       </c>
       <c r="F492" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G492" t="inlineStr"/>
@@ -19450,7 +19498,7 @@
       </c>
       <c r="F541" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G541" t="inlineStr">
@@ -21366,7 +21414,7 @@
       </c>
       <c r="F597" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G597" t="inlineStr"/>
@@ -21569,8 +21617,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G603" t="inlineStr"/>
-      <c r="H603" t="inlineStr"/>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>Needs action-source-card unit scope independent of the Personality performing a Strategy.</t>
+        </is>
+      </c>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
@@ -21736,7 +21792,7 @@
       </c>
       <c r="F608" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G608" t="inlineStr"/>
@@ -21932,7 +21988,7 @@
       </c>
       <c r="F614" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G614" t="inlineStr"/>
@@ -22101,8 +22157,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G619" t="inlineStr"/>
-      <c r="H619" t="inlineStr"/>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>Needs attack prohibition during movement and entry, not assignment alone.</t>
+        </is>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
@@ -22135,8 +22199,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G620" t="inlineStr"/>
-      <c r="H620" t="inlineStr"/>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>Needs optional remain-bowed choice, return of control when source straightens/leaves and seppuku prohibition.</t>
+        </is>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr">
@@ -22366,7 +22438,7 @@
       </c>
       <c r="F627" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G627" t="inlineStr"/>
@@ -24266,7 +24338,7 @@
       </c>
       <c r="F683" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G683" t="inlineStr"/>
@@ -26782,7 +26854,7 @@
       </c>
       <c r="F757" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G757" t="inlineStr"/>
@@ -26887,8 +26959,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G760" t="inlineStr"/>
-      <c r="H760" t="inlineStr"/>
+      <c r="G760" t="inlineStr">
+        <is>
+          <t>Not wired in #689 (a draft wiring was removed untested): the Nonhuman entry discount and "move your target Personality at any location to Shakash's location" (Home-capable) need their own card pass and tests.</t>
+        </is>
+      </c>
+      <c r="H760" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="761">
       <c r="A761" t="inlineStr">
@@ -28099,8 +28179,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G796" t="inlineStr"/>
-      <c r="H796" t="inlineStr"/>
+      <c r="G796" t="inlineStr">
+        <is>
+          <t>Not wired in #689 (draft wiring removed untested): Ring of Water entry waiver plus straightening one or two cards in units, performed from Home, need their own card pass and tests.</t>
+        </is>
+      </c>
+      <c r="H796" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="797">
       <c r="A797" t="inlineStr">
@@ -30872,7 +30960,7 @@
       </c>
       <c r="F878" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G878" t="inlineStr"/>
@@ -31084,7 +31172,11 @@
           <t>Needs an "actions must target this card if legal" forced-redirection rule (Yoritomo Naoto's own Battle ability), on top of its own Additional Action grant. The legality half now exists (ActionAcceptsTarget, issue #335 -- "if legal" is that check); the standing hook that applies it to every action is the gap.</t>
         </is>
       </c>
-      <c r="H884" t="inlineStr"/>
+      <c r="H884" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="885">
       <c r="A885" t="inlineStr">
@@ -31552,7 +31644,7 @@
       </c>
       <c r="F898" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G898" t="inlineStr"/>
@@ -34116,7 +34208,11 @@
           <t>Needs a per-card, permanent "this Personality may not attack" attachment flag (Utaku Chikako's own restriction, issue #186, is a player-and-turn-scoped flag, not directly reusable here) plus a self-destroying Limited ability. Dishonor-as-an-action is now built (Justice of the Crane) and directly reusable for its own Dishonor half.</t>
         </is>
       </c>
-      <c r="H974" t="inlineStr"/>
+      <c r="H974" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="975">
       <c r="A975" t="inlineStr">
@@ -34308,7 +34404,7 @@
       </c>
       <c r="F980" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G980" t="inlineStr">
@@ -38451,8 +38547,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1102" t="inlineStr"/>
-      <c r="H1102" t="inlineStr"/>
+      <c r="G1102" t="inlineStr">
+        <is>
+          <t>Needs Spell attachment-count limit, Shugenja grant and Focus-dependent bow-cost waiver.</t>
+        </is>
+      </c>
+      <c r="H1102" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="1103">
       <c r="A1103" t="inlineStr">
@@ -40083,8 +40187,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1150" t="inlineStr"/>
-      <c r="H1150" t="inlineStr"/>
+      <c r="G1150" t="inlineStr">
+        <is>
+          <t>Needs action-source-card unit scope independent of performer and restriction against targeting the host unit.</t>
+        </is>
+      </c>
+      <c r="H1150" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="1151">
       <c r="A1151" t="inlineStr">
@@ -40258,7 +40370,11 @@
           <t>Created copies exist (issue #398: a real copy of the target, marked as created). Still needs a second target (bow one of your unbowed Personalities, copy another), the Item removing itself from the game as a cost, a lock "will not straighten, attack, or defend until after your next turn begins" on the second target, and removing the copy after your next turn begins (a created card removed at the start of its owner's next turn is not built). Rulings needed from Mendon: who controls the copy, where it enters, and how "ignoring costs and restrictions" treats a Unique target.</t>
         </is>
       </c>
-      <c r="H1155" t="inlineStr"/>
+      <c r="H1155" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="1156">
       <c r="A1156" t="inlineStr">
@@ -41402,7 +41518,7 @@
       </c>
       <c r="F1189" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1189" t="inlineStr"/>
@@ -42260,7 +42376,7 @@
       </c>
       <c r="F1214" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1214" t="inlineStr"/>
@@ -46496,7 +46612,7 @@
       </c>
       <c r="F1338" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1338" t="inlineStr"/>
@@ -47210,7 +47326,7 @@
       </c>
       <c r="F1359" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1359" t="inlineStr"/>
@@ -52122,7 +52238,7 @@
       </c>
       <c r="F1503" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1503" t="inlineStr"/>
@@ -54726,7 +54842,7 @@
       </c>
       <c r="F1579" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1579" t="inlineStr"/>
@@ -58180,7 +58296,7 @@
       </c>
       <c r="F1680" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1680" t="inlineStr"/>
@@ -61380,7 +61496,7 @@
       </c>
       <c r="F1774" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1774" t="inlineStr"/>
@@ -64115,8 +64231,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1854" t="inlineStr"/>
-      <c r="H1854" t="inlineStr"/>
+      <c r="G1854" t="inlineStr">
+        <is>
+          <t>Needs P1 (a turn-long production adjustment on every non-Unique Holding) with the once-per-turn copy limit; not wired in #689.</t>
+        </is>
+      </c>
+      <c r="H1854" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="1855">
       <c r="A1855" t="inlineStr">
@@ -72569,8 +72693,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2101" t="inlineStr"/>
-      <c r="H2101" t="inlineStr"/>
+      <c r="G2101" t="inlineStr">
+        <is>
+          <t>Needs source-bound Event lifetime through two future owner turns and targeted-action Honor-loss filtering.</t>
+        </is>
+      </c>
+      <c r="H2101" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="2102">
       <c r="A2102" t="inlineStr">
@@ -74963,8 +75095,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2170" t="inlineStr"/>
-      <c r="H2170" t="inlineStr"/>
+      <c r="G2170" t="inlineStr">
+        <is>
+          <t>Needs attack/defend prohibition during movement and entry, not assignment alone.</t>
+        </is>
+      </c>
+      <c r="H2170" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
     </row>
     <row r="2171">
       <c r="A2171" t="inlineStr">
@@ -76943,7 +77083,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -76963,7 +77103,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -77143,7 +77283,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Art pack r1, inventory, decision index and handoff for #699
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A29buqY4H1Xgn5ZxyHvSrq
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -585,14 +585,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>86.5%</t>
+          <t>88.0%</t>
         </is>
       </c>
     </row>
@@ -603,14 +603,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>93.0%</t>
+          <t>93.1%</t>
         </is>
       </c>
     </row>
@@ -657,14 +657,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C13" t="n">
         <v>37</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>75.7%</t>
+          <t>78.4%</t>
         </is>
       </c>
     </row>
@@ -711,14 +711,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2012</v>
+        <v>2016</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>90.8%</t>
+          <t>90.9%</t>
         </is>
       </c>
     </row>
@@ -819,10 +819,10 @@
         <v>6</v>
       </c>
       <c r="J20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L20" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21">
@@ -844,7 +844,7 @@
         <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G21" t="n">
         <v>16</v>
@@ -859,7 +859,7 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22">
@@ -881,7 +881,7 @@
         <v>4</v>
       </c>
       <c r="G22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H22" t="n">
         <v>2</v>
@@ -893,7 +893,7 @@
         <v>2</v>
       </c>
       <c r="L22" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="23">
@@ -1009,10 +1009,10 @@
         <v>19</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H27" s="2" t="n">
         <v>14</v>
@@ -1021,13 +1021,13 @@
         <v>18</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>2</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -2249,8 +2249,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>The False Path (Stronghold, issue #699): "You may not win by Enlightenment" is now a one-line read of the Ring-entry primitive's Enlightenment check, but the card is a whole Stronghold: its non-Unique Monk and Fudo Personalities gain Monk and Fudo in and out of play, Fudo Personalities join for 2 less Gold, Honor Requirements of Fudo cards are ignored, no Honor is lost from owned Fudo cards, and a Limited bow search for a Fudo Ring. Granting keywords to cards out of play and the Fudo Honor waivers are separate primitives, and no stronghold scan is packaged in the rings waves.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>GRANT</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5461,8 +5469,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr"/>
-      <c r="H129" t="inlineStr"/>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Asako Usohara (Personality, Emperor Edition, issue #699): "Limited, bow: Search your Dynasty discard pile, then deck, for a Fudo Celestial. Put it into play." and "Limited: Put a Fudo Ring from your hand into play. This counts as playing it by its own text. Remove Usohara from the game." The second line is now buildable (the Ring-entry record of WlRings.cs takes an own-text entry with Usohara as source), but the first needs a search whose destination is IN PLAY for a Celestial (Zone.Celestial entry from the Dynasty discard pile or deck, honouring Unique and the Celestial's entry rules); the search catalogue's destinations are hand, province, holding and Ring-into-play only. A card with two printed lines is wired whole or blocked. Needs a search-to-Celestial-in-play destination.</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>SEARCH</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -43774,19 +43790,11 @@
       </c>
       <c r="F1255" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1255" t="inlineStr">
-        <is>
-          <t>Read the Essence (Spell, Torn Asunder, issue #674): "Open: Bow this card and target one face-down card in a province, or one or two such cards if this Shugenja is Void: Turn the targets face-up." Everything else exists (a bow-this-card cost; Second City's Political Open turns a face-down card face-up), but the engine names a face-down province card only by its province (the any-province command parameter, TargetPlayerId + Province, because a face-down card's id is hidden from the view), and that is ONE card. A Void Shugenja's "one or two" needs a second province in the same command (and a pair listing in QueryActions); no multi-province selection exists, and a card id may not be used (hidden information). Question for Mendon: may the Void version be two separate entries (one province each) sharing one use, or is a two-province selection UI wanted?</t>
-        </is>
-      </c>
-      <c r="H1255" t="inlineStr">
-        <is>
-          <t>HIDDEN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1255" t="inlineStr"/>
+      <c r="H1255" t="inlineStr"/>
     </row>
     <row r="1256">
       <c r="A1256" t="inlineStr">
@@ -45652,19 +45660,11 @@
       </c>
       <c r="F1310" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1310" t="inlineStr">
-        <is>
-          <t>Witness the Untold (Spell, Torn Asunder, issue #674): "Reaction: After your Ring enters play, bow this card: Look at the top three cards of your Dynasty or Fate deck. Put them back in any order." The look and reorder exist (LookSpec, It Was a Cat's shape: either deck, three cards, reorder only), but nothing narrates a Ring entering play: every Ring is put into play by its own recruit case (RingEnteredByOwnText) and no Reaction trigger "after your Ring enters play" exists for another card to listen to (the Ring-entering gap the TRIG-AFTER category names). Needs a new reaction trigger fired from every Ring's entry, which is shared-interface work.</t>
-        </is>
-      </c>
-      <c r="H1310" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1310" t="inlineStr"/>
+      <c r="H1310" t="inlineStr"/>
     </row>
     <row r="1311">
       <c r="A1311" t="inlineStr">
@@ -47734,19 +47734,11 @@
       </c>
       <c r="F1371" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1371" t="inlineStr">
-        <is>
-          <t>Benediction (Aftermath, Strategy; scan verified): "Open: Destroy your target Holding. Give a Province +3 strength." Two independent targets of different kinds, a card (your Holding) and a province (either player's, Ring of Earth's 'any-province' shape: GameCommand.Province plus TargetPlayerId). The engine has no ability that names a card and a province together: a multi-target ability is Slots (cards or players only), while the province categories ('any-province', 'enemy-province') are mutually exclusive with a card target in ValidateAbility and in the QueryActions candidate loop (one candidate per province/owner, no card). Wiring it needs a province target slot kind (TargetSlotKinds.Province with a SlotSelection province index and owner, validated in ValidateSlotCard and offered by SlotAbilityOption, plus the client picking a province inside a slot ability). That is a new decision shape for the client, not a local feature addition. Everything else is built: the effect itself is DestroyAttachment-free (DestroyUnits/Holding destroy, then GiveProvinceStrengthThisTurn(owner, index, 3)). QUESTION for Mendon: is 'Give a Province +3 strength' until end of turn (R-001 default, GiveProvinceStrengthThisTurn as Ring of Earth) and may the Province be either player's?</t>
-        </is>
-      </c>
-      <c r="H1371" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1371" t="inlineStr"/>
+      <c r="H1371" t="inlineStr"/>
     </row>
     <row r="1372">
       <c r="A1372" t="inlineStr">
@@ -74596,19 +74588,11 @@
       </c>
       <c r="F2156" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2156" t="inlineStr">
-        <is>
-          <t>Fudo's Assurances (Celestial, Coils of Madness): not wired whole. Battle/Open: Straighten a Ring is buildable, but Open: 'If you control five Fudo Rings that last entered play by their own text, destroy a Province' needs a per-Ring record of HOW it last entered play (by its own text, as the False Rings do, versus recruited, Searched or put into play by another card), and the engine records only that a Ring is in play (the Ring-search entry marks only the Enlightenment count). The only Fudo Rings are the six False Rings, none of which is wired (they exist only as training fixtures). Needs the entry-provenance record (PROVENANCE) and the False Rings wired first; a card with two printed lines is wired whole or blocked.</t>
-        </is>
-      </c>
-      <c r="H2156" t="inlineStr">
-        <is>
-          <t>PROVENANCE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2156" t="inlineStr"/>
+      <c r="H2156" t="inlineStr"/>
     </row>
     <row r="2157">
       <c r="A2157" t="inlineStr">
@@ -76943,7 +76927,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -77023,7 +77007,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -77103,7 +77087,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -77203,7 +77187,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -77223,7 +77207,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -77323,7 +77307,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wire wave batch 1: 15 payment and cost cards on P1/P2/P3/P12 (#732)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -531,14 +531,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>779</v>
+        <v>784</v>
       </c>
       <c r="C6" t="n">
         <v>851</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>91.5%</t>
+          <t>92.1%</t>
         </is>
       </c>
     </row>
@@ -549,14 +549,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C7" t="n">
         <v>141</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>94.3%</t>
+          <t>95.0%</t>
         </is>
       </c>
     </row>
@@ -567,14 +567,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C8" t="n">
         <v>137</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>86.1%</t>
+          <t>86.9%</t>
         </is>
       </c>
     </row>
@@ -585,14 +585,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>88.0%</t>
+          <t>88.7%</t>
         </is>
       </c>
     </row>
@@ -603,14 +603,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>93.1%</t>
+          <t>93.6%</t>
         </is>
       </c>
     </row>
@@ -621,14 +621,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C11" t="n">
         <v>152</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>90.8%</t>
+          <t>93.4%</t>
         </is>
       </c>
     </row>
@@ -711,14 +711,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2016</v>
+        <v>2031</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>90.9%</t>
+          <t>91.6%</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
         <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E20" t="n">
         <v>5</v>
@@ -812,9 +812,6 @@
       <c r="G20" t="n">
         <v>9</v>
       </c>
-      <c r="H20" t="n">
-        <v>2</v>
-      </c>
       <c r="I20" t="n">
         <v>6</v>
       </c>
@@ -822,7 +819,7 @@
         <v>2</v>
       </c>
       <c r="L20" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21">
@@ -844,10 +841,10 @@
         <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G21" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H21" t="n">
         <v>1</v>
@@ -859,7 +856,7 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22">
@@ -869,13 +866,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F22" t="n">
         <v>4</v>
@@ -893,7 +890,7 @@
         <v>2</v>
       </c>
       <c r="L22" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23">
@@ -903,7 +900,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D23" t="n">
         <v>3</v>
@@ -915,7 +912,7 @@
         <v>4</v>
       </c>
       <c r="G23" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
@@ -924,7 +921,7 @@
         <v>2</v>
       </c>
       <c r="L23" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24">
@@ -940,7 +937,7 @@
         <v>1</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
         <v>2</v>
@@ -952,7 +949,7 @@
         <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
@@ -1000,22 +997,22 @@
         <v>3</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="I27" s="2" t="n">
         <v>18</v>
@@ -1027,7 +1024,7 @@
         <v>2</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>201</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -5636,7 +5633,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G134" t="inlineStr"/>
@@ -8806,7 +8803,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -8814,11 +8811,7 @@
           <t>Not wired in #689 (draft wiring removed untested): Invest cost by Clan (a P2 ability cost term) creating two 1F Followers on Kikumura needs its own card pass, the Follower proxy check and tests.</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -9788,7 +9781,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G256" t="inlineStr"/>
@@ -20032,7 +20025,7 @@
       </c>
       <c r="F556" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G556" t="inlineStr">
@@ -22688,7 +22681,7 @@
       </c>
       <c r="F634" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G634" t="inlineStr"/>
@@ -32290,7 +32283,7 @@
       </c>
       <c r="F917" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G917" t="inlineStr">
@@ -37419,8 +37412,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1068" t="inlineStr"/>
-      <c r="H1068" t="inlineStr"/>
+      <c r="G1068" t="inlineStr">
+        <is>
+          <t>Chiyurei's Axe (Item, issue #732): its Equip discount ("Attaches to Hida Chiyurei paying 2 less Gold") is a P2 entry term and +3F is printed, but its second sentence, "Melee Attacks this Personality performs may be compared against the target's base Force", is a trait of the performer on every Melee Attack he performs. The comparison itself is built (AttackCompare.PrintedForce) but an Attack's optional comparison is a static function of the ability id (AttackCompareOptions in EmperorRulingR5.cs, read by ValidateAbility's Choice gate, the offered-ability loop's compareChoices and its label in CardAbilities.cs, and AttackComparedValue), so a performer-scoped option needs those four places to learn the performer. A shared-interface change in the central action builder, not a card-wave line; the card is not published, so no printed effect is dropped (docs/decisions/2026-10-06-690-p24-effect-primitives.md, limits).</t>
+        </is>
+      </c>
+      <c r="H1068" t="inlineStr">
+        <is>
+          <t>EFFECT</t>
+        </is>
+      </c>
     </row>
     <row r="1069">
       <c r="A1069" t="inlineStr">
@@ -40896,7 +40897,7 @@
       </c>
       <c r="F1170" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1170" t="inlineStr"/>
@@ -43518,7 +43519,7 @@
       </c>
       <c r="F1247" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1247" t="inlineStr"/>
@@ -50465,8 +50466,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1451" t="inlineStr"/>
-      <c r="H1451" t="inlineStr"/>
+      <c r="G1451" t="inlineStr">
+        <is>
+          <t>Duty Over All Things (Strategy, issue #732): the scan reads "Battle: Choose your performing discarded Yojimbo: If he would be opposed, bring him into play at the current battlefield, paying 3 less Gold if you control a Courtier or Shugenja." The performer of the action is a Yojimbo in the owner's discard pile, and the action recruits that same card into play at the battlefield. The engine has no support for a Dead or discarded Personality as an action's performer (AbilitySourceZoneAllows and the performer lists read cards in play; P21's province-source and zone pieces do not cover a discard-pile performer), and "if he would be opposed" asks whether an enemy unit stands at the battlefield the card would enter. Needs a performer-from-discard rule and a recruit of the performer by an action, with a ruling on when "would be opposed" is judged.</t>
+        </is>
+      </c>
+      <c r="H1451" t="inlineStr">
+        <is>
+          <t>ZONE</t>
+        </is>
+      </c>
     </row>
     <row r="1452">
       <c r="A1452" t="inlineStr">
@@ -64220,7 +64229,7 @@
       </c>
       <c r="F1854" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1854" t="inlineStr">
@@ -64228,11 +64237,7 @@
           <t>Needs P1 (a turn-long production adjustment on every non-Unique Holding) with the once-per-turn copy limit; not wired in #689.</t>
         </is>
       </c>
-      <c r="H1854" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+      <c r="H1854" t="inlineStr"/>
     </row>
     <row r="1855">
       <c r="A1855" t="inlineStr">
@@ -64296,7 +64301,7 @@
       </c>
       <c r="F1856" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1856" t="inlineStr"/>
@@ -64738,7 +64743,7 @@
       </c>
       <c r="F1869" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1869" t="inlineStr"/>
@@ -66888,7 +66893,7 @@
       </c>
       <c r="F1932" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1932" t="inlineStr"/>
@@ -67194,7 +67199,7 @@
       </c>
       <c r="F1941" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1941" t="inlineStr">
@@ -67202,11 +67207,7 @@
           <t>Ever-Winter Copse (Holding, issue #653): "When another Holding produces Gold to pay for a Nonhuman, bow this card: Produce 1 Gold" is a payment source whose availability depends on which OTHER producers the payer has chosen for the same payment, and which bows its own card. The payment tokens (EmperorMechE.cs PaymentTokens/UsePaymentTokens) are computed for a payment before any source is chosen, their use never bows their card, and there is no extension point for a condition on the chosen set of sources or for a token kind that bows; adding either means editing the shared payment code, not a feature file.</t>
         </is>
       </c>
-      <c r="H1941" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+      <c r="H1941" t="inlineStr"/>
     </row>
     <row r="1942">
       <c r="A1942" t="inlineStr">
@@ -70014,7 +70015,7 @@
       </c>
       <c r="F2023" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2023" t="inlineStr"/>
@@ -70422,7 +70423,7 @@
       </c>
       <c r="F2035" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2035" t="inlineStr">
@@ -70430,11 +70431,7 @@
           <t>The Amethyst Court (Holding, issue #653): its second line, "Bow: Bow your target unbowed Courtier or Artisan. Produce Gold equal to his Chi", is a Gold source of its own that names a Personality as it is used (the amount is that Personality's Chi, and bowing him is part of the production). The payment tokens offer a source per candidate only for Zlkyt's destroyed Holding and Moto Rani's removed dead Personality; UsePaymentTokens switches on a closed set of token kinds and has no extension point for a source that bows a chosen Personality, so the production cannot be added from a feature file.</t>
         </is>
       </c>
-      <c r="H2035" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+      <c r="H2035" t="inlineStr"/>
     </row>
     <row r="2036">
       <c r="A2036" t="inlineStr">
@@ -76947,7 +76944,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -77067,7 +77064,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -77267,7 +77264,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -77347,7 +77344,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wire wave batch 2: 12 recruit-gate, Proclaim and Honor cards (#733)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -513,14 +513,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C5" t="n">
         <v>51</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>94.1%</t>
+          <t>96.1%</t>
         </is>
       </c>
     </row>
@@ -531,14 +531,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>784</v>
+        <v>792</v>
       </c>
       <c r="C6" t="n">
         <v>851</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>92.1%</t>
+          <t>93.1%</t>
         </is>
       </c>
     </row>
@@ -549,14 +549,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C7" t="n">
         <v>141</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>95.0%</t>
+          <t>95.7%</t>
         </is>
       </c>
     </row>
@@ -603,14 +603,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>93.6%</t>
+          <t>94.0%</t>
         </is>
       </c>
     </row>
@@ -711,14 +711,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2031</v>
+        <v>2043</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>91.6%</t>
+          <t>92.2%</t>
         </is>
       </c>
     </row>
@@ -794,69 +794,69 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Coils of Madness</t>
+          <t>Torn Asunder</t>
         </is>
       </c>
       <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>15</v>
+      </c>
+      <c r="D20" t="n">
         <v>2</v>
       </c>
-      <c r="C20" t="n">
-        <v>27</v>
-      </c>
       <c r="E20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" t="n">
+        <v>6</v>
+      </c>
+      <c r="G20" t="n">
+        <v>15</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" t="n">
         <v>5</v>
       </c>
-      <c r="F20" t="n">
+      <c r="K20" t="n">
         <v>1</v>
       </c>
-      <c r="G20" t="n">
-        <v>9</v>
-      </c>
-      <c r="I20" t="n">
-        <v>6</v>
-      </c>
-      <c r="J20" t="n">
-        <v>2</v>
-      </c>
       <c r="L20" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Torn Asunder</t>
+          <t>Coils of Madness</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>16</v>
-      </c>
-      <c r="D21" t="n">
+        <v>21</v>
+      </c>
+      <c r="E21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>7</v>
+      </c>
+      <c r="I21" t="n">
+        <v>6</v>
+      </c>
+      <c r="J21" t="n">
         <v>2</v>
       </c>
-      <c r="E21" t="n">
-        <v>3</v>
-      </c>
-      <c r="F21" t="n">
-        <v>6</v>
-      </c>
-      <c r="G21" t="n">
-        <v>15</v>
-      </c>
-      <c r="H21" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" t="n">
-        <v>5</v>
-      </c>
-      <c r="K21" t="n">
-        <v>1</v>
-      </c>
       <c r="L21" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22">
@@ -866,10 +866,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
         <v>5</v>
@@ -890,7 +890,7 @@
         <v>2</v>
       </c>
       <c r="L22" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23">
@@ -994,13 +994,13 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>18</v>
@@ -1009,7 +1009,7 @@
         <v>15</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H27" s="2" t="n">
         <v>10</v>
@@ -1024,7 +1024,7 @@
         <v>2</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>186</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2251,11 +2251,7 @@
           <t>The False Path (Stronghold, issue #699): "You may not win by Enlightenment" is now a one-line read of the Ring-entry primitive's Enlightenment check, but the card is a whole Stronghold: its non-Unique Monk and Fudo Personalities gain Monk and Fudo in and out of play, Fudo Personalities join for 2 less Gold, Honor Requirements of Fudo cards are ignored, no Honor is lost from owned Fudo cards, and a Limited bow search for a Fudo Ring. Granting keywords to cards out of play and the Fudo Honor waivers are separate primitives, and no stronghold scan is packaged in the rings waves.</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>GRANT</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5569,7 +5565,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G132" t="inlineStr"/>
@@ -5867,7 +5863,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G141" t="inlineStr"/>
@@ -12489,7 +12485,7 @@
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G336" t="inlineStr"/>
@@ -12905,7 +12901,7 @@
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
@@ -16257,7 +16253,7 @@
       </c>
       <c r="F446" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G446" t="inlineStr">
@@ -25843,7 +25839,7 @@
       </c>
       <c r="F727" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G727" t="inlineStr"/>
@@ -28151,7 +28147,7 @@
       </c>
       <c r="F795" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G795" t="inlineStr"/>
@@ -31487,7 +31483,7 @@
       </c>
       <c r="F893" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G893" t="inlineStr"/>
@@ -31754,8 +31750,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G901" t="inlineStr"/>
-      <c r="H901" t="inlineStr"/>
+      <c r="G901" t="inlineStr">
+        <is>
+          <t>Zansho - exp (Personality, issue #733): the scan reads "Battle: Bow Zansho's target unbowed Follower. Ranged Attack with strength equal to its Force, plus 2 if the Ranged Attack targets Daigotsu Arakan." It does not say whose Follower is bowed: any unbowed Follower at the battlefield (the other player's included), only one of the controller's, or one attached to Zansho himself. The three readings are three different cards (bowing an enemy Follower as a cost is a strong effect). Needs Mendon's ruling before it is built; the gate ("will not join a Spider Clan player") and the Attack strength hook are available.</t>
+        </is>
+      </c>
+      <c r="H901" t="inlineStr">
+        <is>
+          <t>RULES</t>
+        </is>
+      </c>
     </row>
     <row r="902">
       <c r="A902" t="inlineStr">
@@ -32721,7 +32725,7 @@
       </c>
       <c r="F930" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G930" t="inlineStr">
@@ -49715,7 +49719,7 @@
       </c>
       <c r="F1429" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1429" t="inlineStr"/>
@@ -54265,7 +54269,7 @@
       </c>
       <c r="F1562" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1562" t="inlineStr"/>
@@ -55402,8 +55406,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1595" t="inlineStr"/>
-      <c r="H1595" t="inlineStr"/>
+      <c r="G1595" t="inlineStr">
+        <is>
+          <t>Merchant Patronage (Strategy, issue #733): "Political Interrupt: If the action is on another player's Holding, you choose who gains or loses any Honor from it. If you control a Courtier, you may bow him to increase the gain or loss by 1." Two gaps: an Interrupt window before ANY action targeting a Holding resolves (the before-action windows only predict movers and a few curated destroy and bow ids, P8), and a choice of who takes an Honor change made inside it (the P14 channel supports a redirect, but nothing asks the acting player at that point). Its Kharmic reminder text is the engine's.</t>
+        </is>
+      </c>
+      <c r="H1595" t="inlineStr">
+        <is>
+          <t>TRIG-ANN</t>
+        </is>
+      </c>
     </row>
     <row r="1596">
       <c r="A1596" t="inlineStr">
@@ -62694,8 +62706,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1809" t="inlineStr"/>
-      <c r="H1809" t="inlineStr"/>
+      <c r="G1809" t="inlineStr">
+        <is>
+          <t>The Heavens' Blessing (Strategy, issue #733): two Open effects. "No player can gain Honor in Action Phases (this turn)" is a P14 no-gain modifier with the action-phase-only filter, but the first, "Until the game ends, a player must pay 2 Gold to draw a card from effects of his own Strategies during an Action Phase", has no home: Draw has no source, so a draw made by a Strategy's effect cannot be told from any other, and a payment asked in the middle of an effect (declinable, with the draw lost) has no decision for it. Publishing only the second sentence would drop printed text.</t>
+        </is>
+      </c>
+      <c r="H1809" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
     </row>
     <row r="1810">
       <c r="A1810" t="inlineStr">
@@ -72684,12 +72704,12 @@
       </c>
       <c r="G2101" t="inlineStr">
         <is>
-          <t>Needs source-bound Event lifetime through two future owner turns and targeted-action Honor-loss filtering.</t>
+          <t>Marriage of the Emerald Champion (Event, issue #733): "Limited: Put this Event into play. Target your Personality. While this Event remains in play, he will not be dishonored and you will not lose Honor from other players' actions that have targeted him. After your second turn from now begins, discard this Event." The pieces exist (KeepEventInPlay with turnBeginsIn 2, a P11 dishonor bar, a P14 no-loss filter targeted-by-other), but the target is chosen when the Event is revealed and the Event then leaves its province for play, and the Event decision machinery that answers a custom choice (ResolveEventChoiceCommand's default arm) is wired only for P5's Events that stay in their province. A new kind needs one hook in that arm and a record binding the Event to its target; a shared-interface change in the Events Phase.</t>
         </is>
       </c>
       <c r="H2101" t="inlineStr">
         <is>
-          <t>LOCK</t>
+          <t>TARGET</t>
         </is>
       </c>
     </row>
@@ -76984,7 +77004,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -77064,7 +77084,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -77084,7 +77104,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -77204,7 +77224,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -77244,7 +77264,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -77264,7 +77284,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wave batch 3 (#734): 19 stat-term and Experienced cards, art pack, handoff
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -531,14 +531,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>784</v>
+        <v>795</v>
       </c>
       <c r="C6" t="n">
         <v>851</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>92.1%</t>
+          <t>93.4%</t>
         </is>
       </c>
     </row>
@@ -567,14 +567,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C8" t="n">
         <v>137</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>86.9%</t>
+          <t>89.1%</t>
         </is>
       </c>
     </row>
@@ -585,14 +585,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>88.7%</t>
+          <t>89.5%</t>
         </is>
       </c>
     </row>
@@ -603,14 +603,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>93.6%</t>
+          <t>94.0%</t>
         </is>
       </c>
     </row>
@@ -621,14 +621,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C11" t="n">
         <v>152</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>93.4%</t>
+          <t>94.1%</t>
         </is>
       </c>
     </row>
@@ -639,14 +639,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>77.8%</t>
+          <t>79.0%</t>
         </is>
       </c>
     </row>
@@ -711,14 +711,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2031</v>
+        <v>2050</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>91.6%</t>
+          <t>92.5%</t>
         </is>
       </c>
     </row>
@@ -801,10 +801,10 @@
         <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="E20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F20" t="n">
         <v>1</v>
@@ -819,7 +819,7 @@
         <v>2</v>
       </c>
       <c r="L20" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21">
@@ -832,7 +832,7 @@
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D21" t="n">
         <v>2</v>
@@ -841,10 +841,10 @@
         <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G21" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H21" t="n">
         <v>1</v>
@@ -856,7 +856,7 @@
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22">
@@ -866,22 +866,22 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D22" t="n">
         <v>2</v>
       </c>
       <c r="E22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
         <v>4</v>
       </c>
       <c r="G22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I22" t="n">
         <v>1</v>
@@ -890,7 +890,7 @@
         <v>2</v>
       </c>
       <c r="L22" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23">
@@ -900,13 +900,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D23" t="n">
         <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F23" t="n">
         <v>4</v>
@@ -918,10 +918,10 @@
         <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24">
@@ -997,25 +997,25 @@
         <v>3</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>7</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>8</v>
@@ -1024,7 +1024,7 @@
         <v>2</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>186</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -6042,12 +6042,12 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Needs P9 (conditional -1F statics for Fallen, Nonhuman and attacking-you cards) and an after-next-attack Honor loss; not wired in #689.</t>
+          <t>Bayushi Kachiko: "After the next time this turn a target Personality attacks, his controller loses 2 Honor" needs a ruling (does "attacks" mean he is declared into an attacking army, or that he makes an Attack action?) and a one-shot turn watch keyed to it. Her static -1F term is plain P9 data once the reading is chosen.</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>LOCK</t>
+          <t>WATCH</t>
         </is>
       </c>
     </row>
@@ -6555,7 +6555,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G161" t="inlineStr"/>
@@ -9679,7 +9679,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G253" t="inlineStr"/>
@@ -11053,7 +11053,7 @@
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G294" t="inlineStr"/>
@@ -13899,7 +13899,7 @@
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G377" t="inlineStr"/>
@@ -14179,7 +14179,7 @@
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G385" t="inlineStr"/>
@@ -14391,7 +14391,7 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G391" t="inlineStr"/>
@@ -17712,8 +17712,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G488" t="inlineStr"/>
-      <c r="H488" t="inlineStr"/>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>Kokujin: "if Kokujin wins, you may destroy one of your Personalities (at any location) to take control of the loser (he joins Kokujin's army)" is a choice made after the duel resolves, among one option per Personality of yours plus plain destruction. Duel outcomes in this engine apply directly; a deferred outcome decision needs the P1 after-action trait queue extended (EmperorP1.cs) or a new post-duel decision hook.</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>TRIG-AFTER</t>
+        </is>
+      </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
@@ -21321,7 +21329,7 @@
       </c>
       <c r="F594" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G594" t="inlineStr"/>
@@ -24551,7 +24559,7 @@
       </c>
       <c r="F689" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G689" t="inlineStr"/>
@@ -25231,7 +25239,7 @@
       </c>
       <c r="F709" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G709" t="inlineStr"/>
@@ -28937,7 +28945,7 @@
       </c>
       <c r="F818" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G818" t="inlineStr">
@@ -29145,7 +29153,7 @@
       </c>
       <c r="F824" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G824" t="inlineStr"/>
@@ -36793,7 +36801,7 @@
       </c>
       <c r="F1050" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1050" t="inlineStr">
@@ -38705,7 +38713,7 @@
       </c>
       <c r="F1106" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1106" t="inlineStr"/>
@@ -40133,7 +40141,7 @@
       </c>
       <c r="F1148" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1148" t="inlineStr"/>
@@ -44947,7 +44955,7 @@
       </c>
       <c r="F1289" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1289" t="inlineStr"/>
@@ -57855,7 +57863,7 @@
       </c>
       <c r="F1667" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1667" t="inlineStr"/>
@@ -65151,7 +65159,7 @@
       </c>
       <c r="F1881" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1881" t="inlineStr"/>
@@ -65804,8 +65812,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1900" t="inlineStr"/>
-      <c r="H1900" t="inlineStr"/>
+      <c r="G1900" t="inlineStr">
+        <is>
+          <t>Warded Premises: "Negate all Force bonuses from actions to cards at this battlefield" needs the engine to tell an action's Force modifier from a token, an Item, a Permanent modifier ("Permanently give him +2F") and a static term, and a ruling on whether a permanent bonus is negated for good. Its second ability (put this Terrain into play at a battlefield with no Terrain, even without a unit there) is wireable.</t>
+        </is>
+      </c>
+      <c r="H1900" t="inlineStr">
+        <is>
+          <t>EFFECT</t>
+        </is>
+      </c>
     </row>
     <row r="1901">
       <c r="A1901" t="inlineStr">
@@ -71353,7 +71369,7 @@
       </c>
       <c r="F2062" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2062" t="inlineStr"/>
@@ -73171,7 +73187,7 @@
       </c>
       <c r="F2115" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2115" t="inlineStr"/>
@@ -76964,7 +76980,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -77004,7 +77020,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -77264,7 +77280,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -77344,7 +77360,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wire wave batch 5: 14 card-restriction and immunity cards on P11/P12 (#736)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLyr6J2gRoqayc2nvJTNGy
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -531,14 +531,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="C6" t="n">
         <v>851</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>93.1%</t>
+          <t>93.5%</t>
         </is>
       </c>
     </row>
@@ -549,14 +549,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C7" t="n">
         <v>141</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>95.7%</t>
+          <t>96.5%</t>
         </is>
       </c>
     </row>
@@ -567,14 +567,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C8" t="n">
         <v>137</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>86.9%</t>
+          <t>89.1%</t>
         </is>
       </c>
     </row>
@@ -585,14 +585,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>88.7%</t>
+          <t>90.2%</t>
         </is>
       </c>
     </row>
@@ -603,14 +603,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>94.0%</t>
+          <t>94.1%</t>
         </is>
       </c>
     </row>
@@ -621,14 +621,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C11" t="n">
         <v>152</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>93.4%</t>
+          <t>94.1%</t>
         </is>
       </c>
     </row>
@@ -639,14 +639,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>77.8%</t>
+          <t>79.0%</t>
         </is>
       </c>
     </row>
@@ -657,14 +657,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C13" t="n">
         <v>37</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>78.4%</t>
+          <t>81.1%</t>
         </is>
       </c>
     </row>
@@ -711,14 +711,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2043</v>
+        <v>2057</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>92.2%</t>
+          <t>92.8%</t>
         </is>
       </c>
     </row>
@@ -801,19 +801,19 @@
         <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D20" t="n">
         <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G20" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H20" t="n">
         <v>1</v>
@@ -825,7 +825,7 @@
         <v>1</v>
       </c>
       <c r="L20" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21">
@@ -838,7 +838,7 @@
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E21" t="n">
         <v>5</v>
@@ -850,13 +850,13 @@
         <v>7</v>
       </c>
       <c r="I21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22">
@@ -872,10 +872,10 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G22" t="n">
         <v>3</v>
@@ -890,7 +890,7 @@
         <v>2</v>
       </c>
       <c r="L22" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23">
@@ -900,13 +900,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" t="n">
         <v>3</v>
-      </c>
-      <c r="E23" t="n">
-        <v>4</v>
       </c>
       <c r="F23" t="n">
         <v>4</v>
@@ -921,23 +921,20 @@
         <v>2</v>
       </c>
       <c r="L23" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Promotional–Emperor</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>1</v>
+          <t>Promotional–Celestial</t>
+        </is>
       </c>
       <c r="G24" t="n">
         <v>1</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I24" t="n">
         <v>2</v>
@@ -945,24 +942,24 @@
       <c r="J24" t="n">
         <v>2</v>
       </c>
-      <c r="K24" t="n">
-        <v>1</v>
-      </c>
       <c r="L24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Promotional–Celestial</t>
-        </is>
+          <t>Promotional–Emperor</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
       </c>
       <c r="G25" t="n">
         <v>1</v>
       </c>
       <c r="H25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
         <v>2</v>
@@ -970,6 +967,9 @@
       <c r="J25" t="n">
         <v>2</v>
       </c>
+      <c r="K25" t="n">
+        <v>1</v>
+      </c>
       <c r="L25" t="n">
         <v>8</v>
       </c>
@@ -997,34 +997,34 @@
         <v>2</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>2</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>174</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -4912,12 +4912,12 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Needs an effective Force cap after all bonuses and a source-unit action target restriction.</t>
+          <t>Asako Kaitoko - exp (Personality, issue #736): "Personalities with Fallen, Kolat, Ninja, Nonhuman, or Shadowlands opposing Kaitoko have a maximum Force of 3, and actions from cards in their units may not target Kaitoko." Two gaps: a maximum Force is a stat cap and none exists (P9 left StatCap out; PersonalityForce is additive, so a cap cannot be written without reading the Force it caps), and the target bar applies only to actors whose Personality has one of five keywords, which an ActorSpec cannot say.</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>LOCK</t>
+          <t>STAT</t>
         </is>
       </c>
     </row>
@@ -11458,7 +11458,7 @@
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>Needs same-army exclusions during movement and entry and unopposed Force/printed-cost accounting.</t>
+          <t>Hida Kaiji - exp (Personality, issue #736): "Will not attack or defend with other Personalities, and other Personalities will not attack or defend with Kaiji. Kaiji has +2F while unopposed, or +1F for each Personality opposing him with 6 or lower printed Force." The Force terms are available (a PersonalityForce hook), but the first sentence is an assignment rule over the whole army (Kaiji alone in his army, and no army that holds him holds another Personality); P11's pair restriction judges every card at the battlefield on both sides, so it would also bar him from being opposed.</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
@@ -13934,7 +13934,7 @@
       </c>
       <c r="G378" t="inlineStr">
         <is>
-          <t>Needs same-army exclusions during movement and entry; a battlefield bar incorrectly forbids opposing armies.</t>
+          <t>Isawa Ryuzo (Personality, issue #736): "Fire Open: Target two Personalities, each with more Madness tokens than printed Personal Honor. They will not attack or defend in the same army." P11's pair restriction (NoPair) stops two cards sharing a battlefield on either side, which is stricter than the printed same-army rule (they may stand opposed at one battlefield); a same-side pair restriction is needed. Entry Honor loss and the Madness-token comparison are available.</t>
         </is>
       </c>
       <c r="H378" t="inlineStr">
@@ -21619,7 +21619,7 @@
       </c>
       <c r="F603" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G603" t="inlineStr">
@@ -21627,11 +21627,7 @@
           <t>Needs action-source-card unit scope independent of the Personality performing a Strategy.</t>
         </is>
       </c>
-      <c r="H603" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+      <c r="H603" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
@@ -22159,7 +22155,7 @@
       </c>
       <c r="F619" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G619" t="inlineStr">
@@ -22167,11 +22163,7 @@
           <t>Needs attack prohibition during movement and entry, not assignment alone.</t>
         </is>
       </c>
-      <c r="H619" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+      <c r="H619" t="inlineStr"/>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
@@ -22206,12 +22198,12 @@
       </c>
       <c r="G620" t="inlineStr">
         <is>
-          <t>Needs optional remain-bowed choice, return of control when source straightens/leaves and seppuku prohibition.</t>
+          <t>P'an Ku - exp (Personality, issue #736): "Open, bow: Give a target card a Madness token" is built (the existing panku-madness shape), but "Limited, bow: P'an Ku may remain bowed. Take control of a target Personality with more Madness tokens than printed Personal Honor and remove those tokens. The target will not commit seppuku until P'an Ku straightens or leaves play. After P'an Ku does, give control of the target to his owner." needs three things together: a control change that returns when a named card straightens or leaves play (TakeControl exists; the timed return trigger does not), a seppuku bar tied to that card, and "may remain bowed" (a rule exempting him from straightening). One card, three new rules.</t>
         </is>
       </c>
       <c r="H620" t="inlineStr">
         <is>
-          <t>LOCK</t>
+          <t>CONTROL</t>
         </is>
       </c>
     </row>
@@ -25703,7 +25695,7 @@
       </c>
       <c r="F723" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G723" t="inlineStr"/>
@@ -31169,7 +31161,7 @@
       </c>
       <c r="F884" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G884" t="inlineStr">
@@ -31177,11 +31169,7 @@
           <t>Needs an "actions must target this card if legal" forced-redirection rule (Yoritomo Naoto's own Battle ability), on top of its own Additional Action grant. The legality half now exists (ActionAcceptsTarget, issue #335 -- "if legal" is that check); the standing hook that applies it to every action is the gap.</t>
         </is>
       </c>
-      <c r="H884" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+      <c r="H884" t="inlineStr"/>
     </row>
     <row r="885">
       <c r="A885" t="inlineStr">
@@ -34213,7 +34201,7 @@
       </c>
       <c r="F974" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G974" t="inlineStr">
@@ -34221,11 +34209,7 @@
           <t>Needs a per-card, permanent "this Personality may not attack" attachment flag (Utaku Chikako's own restriction, issue #186, is a player-and-turn-scoped flag, not directly reusable here) plus a self-destroying Limited ability. Dishonor-as-an-action is now built (Justice of the Crane) and directly reusable for its own Dishonor half.</t>
         </is>
       </c>
-      <c r="H974" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+      <c r="H974" t="inlineStr"/>
     </row>
     <row r="975">
       <c r="A975" t="inlineStr">
@@ -38570,12 +38554,12 @@
       </c>
       <c r="G1102" t="inlineStr">
         <is>
-          <t>Needs Spell attachment-count limit, Shugenja grant and Focus-dependent bow-cost waiver.</t>
+          <t>Koan's Jingasa (Item, issue #736): "This Personality has Shugenja, may not have more Spells than Koan cards attached, and he need not bow for his Spells with an odd Focus Value (0 is even)." The Shugenja keyword is AttachGrantsKeyword, but P11's SpellLimit counts Spell actions performed, not Spells attached (the rule here is an attachment limit counted against Koan cards), and "need not bow for his Spells" is a waiver of the bow cost of a Spell's own ability, which P24's cost waivers do not cover.</t>
         </is>
       </c>
       <c r="H1102" t="inlineStr">
         <is>
-          <t>LOCK</t>
+          <t>COST</t>
         </is>
       </c>
     </row>
@@ -38981,7 +38965,7 @@
       </c>
       <c r="F1114" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1114" t="inlineStr"/>
@@ -40205,7 +40189,7 @@
       </c>
       <c r="F1150" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1150" t="inlineStr">
@@ -40213,11 +40197,7 @@
           <t>Needs action-source-card unit scope independent of performer and restriction against targeting the host unit.</t>
         </is>
       </c>
-      <c r="H1150" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+      <c r="H1150" t="inlineStr"/>
     </row>
     <row r="1151">
       <c r="A1151" t="inlineStr">
@@ -40765,7 +40745,7 @@
       </c>
       <c r="F1166" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1166" t="inlineStr"/>
@@ -43591,7 +43571,7 @@
       </c>
       <c r="F1249" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1249" t="inlineStr"/>
@@ -44747,7 +44727,7 @@
       </c>
       <c r="F1283" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1283" t="inlineStr"/>
@@ -45906,8 +45886,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1317" t="inlineStr"/>
-      <c r="H1317" t="inlineStr"/>
+      <c r="G1317" t="inlineStr">
+        <is>
+          <t>A Cleansing Breath (Strategy, issue #736): "Battle/Open: Target your Personality at any location. He centers himself. Negate other players' cards' effects that prevent him assigning, moving or performing actions. If he is a Kensai, straighten his unit." The negations are P12 Prevention and movement/assignment immunities, but "he centers himself" has no definition anywhere in the repository (core rules, rulings or code): it names a rule the owner has not given. Needs Mendon's ruling on what centering does before the card is built; publishing it without the sentence would drop printed text.</t>
+        </is>
+      </c>
+      <c r="H1317" t="inlineStr">
+        <is>
+          <t>RULES</t>
+        </is>
+      </c>
     </row>
     <row r="1318">
       <c r="A1318" t="inlineStr">
@@ -48014,8 +48002,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1379" t="inlineStr"/>
-      <c r="H1379" t="inlineStr"/>
+      <c r="G1379" t="inlineStr">
+        <is>
+          <t>Bonds of Hospitality (Strategy, issue #736): "Limited: Target a bowed Personality: Put this card into play. While this card remains in play, negate the target's straightening, and his controller has the ability, 'Open: Pay 4 Gold: Discard a Bonds of Hospitality.'" Needs a card in play bound to its target (the Strategy sits in play tied to one Personality), a straighten bar that lasts while that card does (StraightenHolds are timed, not bound to a card), and a player-level granted ability that costs Gold and discards any copy (P4's granted abilities have a turn duration only).</t>
+        </is>
+      </c>
+      <c r="H1379" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
     </row>
     <row r="1380">
       <c r="A1380" t="inlineStr">
@@ -52693,7 +52689,7 @@
       </c>
       <c r="F1516" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1516" t="inlineStr">
@@ -68697,7 +68693,7 @@
       </c>
       <c r="F1984" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1984" t="inlineStr">
@@ -68705,11 +68701,7 @@
           <t>Oracle of the Void - exp (Holding, issue #653): "Limited, Bow: The next two cards in provinces you refill (this turn) may be refilled face-up" is an optional face-up refill for each of the next two refills, whichever effect causes them (a purchase, a discard, a Region). Refills happen at many call sites (Purchase, Refill, RefillProvinceSlot and the effects that discard a province card) and there is no single refill hook or per-refill decision; a watch on future refills needs one, which is shared province plumbing. The rest ("Negate this card's destruction", Limited bow draw a card) would be buildable.</t>
         </is>
       </c>
-      <c r="H1984" t="inlineStr">
-        <is>
-          <t>PROVINCE</t>
-        </is>
-      </c>
+      <c r="H1984" t="inlineStr"/>
     </row>
     <row r="1985">
       <c r="A1985" t="inlineStr">
@@ -73021,7 +73013,7 @@
       </c>
       <c r="F2110" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2110" t="inlineStr"/>
@@ -75093,7 +75085,7 @@
       </c>
       <c r="F2170" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2170" t="inlineStr">
@@ -75101,11 +75093,7 @@
           <t>Needs attack/defend prohibition during movement and entry, not assignment alone.</t>
         </is>
       </c>
-      <c r="H2170" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+      <c r="H2170" t="inlineStr"/>
     </row>
     <row r="2171">
       <c r="A2171" t="inlineStr">
@@ -76904,7 +76892,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -76924,7 +76912,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -76984,7 +76972,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -77084,7 +77072,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -77164,7 +77152,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -77264,7 +77252,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -77284,7 +77272,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wire wave batch 6: 15 after-event window and period watch cards on P6/P7/P8 (#737)
Fifteen of the batch's seventeen cards, in seven profiles (personality-wave-167, spell-wave-82, strategy-wave-151, holding-wave-80, event-wave-48, celestial-wave-45, region-wave-30): Akumasa, Asahina Shigemitsu - exp, Hida Tadama, Hiruma Ikeuchi, Iweko Shibatsu, Moto Taigo - exp, Susumu Kuroko, Yogo Katsuta, Reverse Fate, The Crystal Tears, Magistrate's Stipend, An End to Hostilities, Unseasonable Weather, Natsu-Togumara's Guidance and Verdant Jungle. Koan's Robes and Imperial Deployment are deferred with blocker notes.

Shared lines: FactRegistry.Trait gains an engine-aware activeIn, and the targeted-action reaction check consults a new UntargetedReaction hook when the held action names no card (P8 Interrupts).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLyr6J2gRoqayc2nvJTNGy
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -531,14 +531,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>796</v>
+        <v>804</v>
       </c>
       <c r="C6" t="n">
         <v>851</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>93.5%</t>
+          <t>94.5%</t>
         </is>
       </c>
     </row>
@@ -585,14 +585,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>90.2%</t>
+          <t>91.0%</t>
         </is>
       </c>
     </row>
@@ -603,14 +603,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>94.1%</t>
+          <t>94.3%</t>
         </is>
       </c>
     </row>
@@ -621,14 +621,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C11" t="n">
         <v>152</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>94.1%</t>
+          <t>94.7%</t>
         </is>
       </c>
     </row>
@@ -639,14 +639,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>79.0%</t>
+          <t>81.5%</t>
         </is>
       </c>
     </row>
@@ -657,14 +657,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C13" t="n">
         <v>37</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>81.1%</t>
+          <t>83.8%</t>
         </is>
       </c>
     </row>
@@ -675,14 +675,14 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C14" t="n">
         <v>26</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>96.2%</t>
         </is>
       </c>
     </row>
@@ -711,14 +711,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2057</v>
+        <v>2072</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>92.8%</t>
+          <t>93.5%</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
         <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D20" t="n">
         <v>2</v>
@@ -819,13 +819,13 @@
         <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K20" t="n">
         <v>1</v>
       </c>
       <c r="L20" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21">
@@ -838,7 +838,7 @@
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E21" t="n">
         <v>5</v>
@@ -850,13 +850,13 @@
         <v>7</v>
       </c>
       <c r="I21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J21" t="n">
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22">
@@ -866,7 +866,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D22" t="n">
         <v>1</v>
@@ -875,7 +875,7 @@
         <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G22" t="n">
         <v>3</v>
@@ -890,7 +890,7 @@
         <v>2</v>
       </c>
       <c r="L22" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23">
@@ -900,7 +900,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D23" t="n">
         <v>2</v>
@@ -912,7 +912,7 @@
         <v>4</v>
       </c>
       <c r="G23" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
@@ -921,20 +921,23 @@
         <v>2</v>
       </c>
       <c r="L23" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Promotional–Celestial</t>
-        </is>
+          <t>Promotional–Emperor</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
       </c>
       <c r="G24" t="n">
         <v>1</v>
       </c>
       <c r="H24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
         <v>2</v>
@@ -943,35 +946,29 @@
         <v>2</v>
       </c>
       <c r="L24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Promotional–Emperor</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>1</v>
+          <t>Promotional–Celestial</t>
+        </is>
       </c>
       <c r="G25" t="n">
         <v>1</v>
       </c>
       <c r="H25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I25" t="n">
         <v>2</v>
       </c>
       <c r="J25" t="n">
-        <v>2</v>
-      </c>
-      <c r="K25" t="n">
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -997,7 +994,7 @@
         <v>2</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>5</v>
@@ -1006,25 +1003,25 @@
         <v>15</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>160</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -3853,7 +3850,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G82" t="inlineStr"/>
@@ -4389,7 +4386,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -4397,11 +4394,7 @@
           <t>Needs P6 (after-event records and windows); P7's watch half alone does not wire it.</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -11733,7 +11726,7 @@
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G314" t="inlineStr"/>
@@ -12001,7 +11994,7 @@
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
@@ -12009,11 +12002,7 @@
           <t>Needs a controller choice when multiple attached Followers would be destroyed simultaneously; a per-card watch cannot choose which single destruction to negate.</t>
         </is>
       </c>
-      <c r="H322" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+      <c r="H322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -14693,7 +14682,7 @@
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G400" t="inlineStr"/>
@@ -21147,7 +21136,7 @@
       </c>
       <c r="F589" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G589" t="inlineStr"/>
@@ -25729,7 +25718,7 @@
       </c>
       <c r="F724" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G724" t="inlineStr"/>
@@ -30379,7 +30368,7 @@
       </c>
       <c r="F861" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G861" t="inlineStr"/>
@@ -38594,8 +38583,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1103" t="inlineStr"/>
-      <c r="H1103" t="inlineStr"/>
+      <c r="G1103" t="inlineStr">
+        <is>
+          <t>Koan's Robes (Item, issue #737): "This Personality has a Force bonus equal to the number of other Koan cards in this unit. This Personality need not bow for his Spells with an even Focus Value (0 is even). Negate the first destruction each turn of cards in this unit from another player's card." The destruction negation is a P7 standing watch (a unit scope is the only gap, and a Condition could stand in for it), but the other two sentences are not buildable on what is merged: a Force bonus counted from the Koan cards in the unit needs a P9 stat term that counts a keyword in the unit (batch 3 owns the stat terms and none is merged), and "need not bow for his Spells" is a waiver of the bow cost of a Spell's own ability, which no merged cost waiver covers (the same gap that deferred Koan's Jingasa in batch 5). Publishing it with only the negation would drop two printed sentences.</t>
+        </is>
+      </c>
+      <c r="H1103" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
     </row>
     <row r="1104">
       <c r="A1104" t="inlineStr">
@@ -43809,7 +43806,7 @@
       </c>
       <c r="F1256" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1256" t="inlineStr"/>
@@ -53546,8 +53543,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1541" t="inlineStr"/>
-      <c r="H1541" t="inlineStr"/>
+      <c r="G1541" t="inlineStr">
+        <is>
+          <t>Imperial Deployment (Strategy, issue #737): "Open: Choose your performing Personality: The Empress dispatches him to the Colonies. Negate other players' cards' effects that prevent him assigning. After the next time this turn an attack is declared, straighten his unit." Two gaps: no P12 immunity kind covers an effect that prevents a Personality from being assigned (Prevention covers performing actions only; the assignment bars are P11 restrictions and the Attacker's own flags), and P6 has no fact for "an attack is declared" (its facts are per-Personality assignments, not the declaration). Needs an assignment-prevention immunity and a declared-attack fact before it is built; "dispatches him to the Colonies" is flavor text with no rule.</t>
+        </is>
+      </c>
+      <c r="H1541" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
     </row>
     <row r="1542">
       <c r="A1542" t="inlineStr">
@@ -62389,7 +62394,7 @@
       </c>
       <c r="F1800" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1800" t="inlineStr">
@@ -68421,7 +68426,7 @@
       </c>
       <c r="F1976" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1976" t="inlineStr">
@@ -71671,7 +71676,7 @@
       </c>
       <c r="F2071" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2071" t="inlineStr"/>
@@ -74049,7 +74054,7 @@
       </c>
       <c r="F2140" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2140" t="inlineStr"/>
@@ -75047,7 +75052,7 @@
       </c>
       <c r="F2169" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2169" t="inlineStr">
@@ -76359,7 +76364,7 @@
       </c>
       <c r="F2207" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2207" t="inlineStr">
@@ -76367,11 +76372,7 @@
           <t>Verdant Jungle (Region, issue #653): its Reaction, "Before an action resolves, bow this card: Negate its effects that move any Personalities into an attacking army at this Province's battlefield", negates only the movement part of an announced action by destination. The before-action Reaction window decides which Reactions apply in BeforeActionReactionApplies, a closed switch with no extension hook, and the movement a held action would make is known only per-ability (DeferredActionMovers) with no destination, so "into an attacking army at this battlefield" cannot be asked of an announced action. The first line (nonhuman Personalities enter play from this province for 1 less Gold) would be a small entry discount.</t>
         </is>
       </c>
-      <c r="H2207" t="inlineStr">
-        <is>
-          <t>TRIG-ANN</t>
-        </is>
-      </c>
+      <c r="H2207" t="inlineStr"/>
     </row>
     <row r="2208">
       <c r="A2208" t="inlineStr">
@@ -76972,7 +76973,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -76992,7 +76993,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -77072,7 +77073,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -77272,7 +77273,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wave batch 7: turn-boundary, rule-flag and Events-Phase cards (#738)
Sixteen of the batch's 18 cards, wired on P4/P13/P6 and published in six wave profiles
(personality-wave-175, item-wave-75, strategy-wave-159, holding-wave-88, event-wave-56,
celestial-wave-53). The scans print no P5 clause, so the Events are ordinary; Revelations
and The Onyx Championship are deferred with blocker notes. Art pack
catalogue-art-issue738-20261008-r1 (4,535 images) extends the batch 6 pack.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLyr6J2gRoqayc2nvJTNGy
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -531,14 +531,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>804</v>
+        <v>806</v>
       </c>
       <c r="C6" t="n">
         <v>851</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>94.5%</t>
+          <t>94.7%</t>
         </is>
       </c>
     </row>
@@ -567,14 +567,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C8" t="n">
         <v>137</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>89.1%</t>
+          <t>90.5%</t>
         </is>
       </c>
     </row>
@@ -603,14 +603,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>94.3%</t>
+          <t>94.8%</t>
         </is>
       </c>
     </row>
@@ -621,14 +621,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C11" t="n">
         <v>152</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>94.7%</t>
+          <t>95.4%</t>
         </is>
       </c>
     </row>
@@ -639,14 +639,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>81.5%</t>
+          <t>90.1%</t>
         </is>
       </c>
     </row>
@@ -657,14 +657,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C13" t="n">
         <v>37</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>83.8%</t>
+          <t>86.5%</t>
         </is>
       </c>
     </row>
@@ -711,14 +711,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2072</v>
+        <v>2088</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>93.5%</t>
+          <t>94.2%</t>
         </is>
       </c>
     </row>
@@ -813,19 +813,19 @@
         <v>5</v>
       </c>
       <c r="G20" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H20" t="n">
         <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K20" t="n">
         <v>1</v>
       </c>
       <c r="L20" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21">
@@ -847,16 +847,16 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J21" t="n">
         <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22">
@@ -866,13 +866,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D22" t="n">
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
         <v>2</v>
@@ -887,10 +887,10 @@
         <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23">
@@ -906,7 +906,7 @@
         <v>2</v>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
         <v>4</v>
@@ -915,13 +915,13 @@
         <v>6</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24">
@@ -940,13 +940,13 @@
         <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J24" t="n">
         <v>2</v>
       </c>
       <c r="L24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -962,13 +962,13 @@
         <v>2</v>
       </c>
       <c r="I25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J25" t="n">
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
@@ -994,34 +994,34 @@
         <v>2</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>5</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>12</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H27" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="I27" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="I27" s="2" t="n">
-        <v>15</v>
-      </c>
       <c r="J27" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>145</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G264" t="inlineStr"/>
@@ -25174,7 +25174,7 @@
       </c>
       <c r="F708" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G708" t="inlineStr"/>
@@ -37636,7 +37636,7 @@
       </c>
       <c r="F1075" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1075" t="inlineStr"/>
@@ -38724,7 +38724,7 @@
       </c>
       <c r="F1107" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1107" t="inlineStr"/>
@@ -50290,7 +50290,7 @@
       </c>
       <c r="F1446" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1446" t="inlineStr"/>
@@ -61476,7 +61476,7 @@
       </c>
       <c r="F1773" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1773" t="inlineStr"/>
@@ -62156,7 +62156,7 @@
       </c>
       <c r="F1793" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1793" t="inlineStr"/>
@@ -66272,7 +66272,7 @@
       </c>
       <c r="F1913" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1913" t="inlineStr"/>
@@ -71472,7 +71472,7 @@
       </c>
       <c r="F2065" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2065" t="inlineStr"/>
@@ -71642,7 +71642,7 @@
       </c>
       <c r="F2070" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2070" t="inlineStr"/>
@@ -72594,7 +72594,7 @@
       </c>
       <c r="F2098" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2098" t="inlineStr"/>
@@ -72946,7 +72946,7 @@
       </c>
       <c r="F2108" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2108" t="inlineStr">
@@ -73120,7 +73120,7 @@
       </c>
       <c r="F2113" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2113" t="inlineStr"/>
@@ -73157,8 +73157,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2114" t="inlineStr"/>
-      <c r="H2114" t="inlineStr"/>
+      <c r="G2114" t="inlineStr">
+        <is>
+          <t>Revelations (Event, issue #738): "Show the top five cards of your Dynasty deck. Choose another player who may discard one of the cards. Put the rest back in any order. Refill this province face-up." The scan prints no "After you reveal" clause, so it is an ordinary Event that resolves when revealed, but its three steps are not covered by what is merged: P20's "other player chooses" belongs to a deck search (a set of picked cards), not to a look at the top of a deck; the look (DeckLook.cs) lets its own player rearrange but has no step in which another player discards one of the shown cards before the rest go back; and the Event's own province must then refill face up from the reordered deck. It needs a look disposition with an other-player discard and a reorder, which is decision-UI work for batch 8 (#739), not a card-level guess.</t>
+        </is>
+      </c>
+      <c r="H2114" t="inlineStr">
+        <is>
+          <t>SEARCH</t>
+        </is>
+      </c>
     </row>
     <row r="2115">
       <c r="A2115" t="inlineStr">
@@ -73664,7 +73672,7 @@
       </c>
       <c r="F2129" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2129" t="inlineStr">
@@ -73672,11 +73680,7 @@
           <t>The Jade Championship (Event). Needs a -1F aura on Shadowlands Followers at a location (FollowerForce has no registry hook) and a mandatory trait that triggers after the resolution of an action from a Spell (no trait-after-action hook exists; AfterActionResolved offers only optional Reactions).</t>
         </is>
       </c>
-      <c r="H2129" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+      <c r="H2129" t="inlineStr"/>
     </row>
     <row r="2130">
       <c r="A2130" t="inlineStr">
@@ -73706,7 +73710,7 @@
       </c>
       <c r="F2130" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2130" t="inlineStr"/>
@@ -73779,7 +73783,7 @@
       </c>
       <c r="G2132" t="inlineStr">
         <is>
-          <t>The Onyx Championship (Event). The granted Maho ability searches the discard pile, then the deck, then the Provinces for an Oni Personality and recruits it paying all costs; the engine's search primitive covers one source at a time and has no ordered multi-source search.</t>
+          <t>The Onyx Championship (Event, issue #738): "Choose one of your Shugenja in play. Permanently give him Shadowlands and the ability, 'Maho Limited: Bow this Shugenja and destroy your target Personality: Search your discard pile, then deck, then provinces for an Oni Personality. Bring him into play, paying all costs. Lose 3 Honor.'" The permanent keyword and ability grant are built (GrantKeyword, GrantAbility Permanent), and the ordered search of a discard pile, a deck and the provinces is P20's, but P20 lets a card found in a province enter play only ignoring its costs (SearchEffect.RecruitFromProvinceIgnoringCosts is the sole province recruit and ValidateSearchSpec refuses any other disposition for a province source), while the card prints "paying all costs" for every source. The pay-all-costs recruit from a province is not built; publishing the card with the ignoring-costs recruit would change a printed cost.</t>
         </is>
       </c>
       <c r="H2132" t="inlineStr">
@@ -74466,7 +74470,7 @@
       </c>
       <c r="F2152" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2152" t="inlineStr"/>
@@ -77013,7 +77017,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -77313,7 +77317,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Batch 8: art pack descriptor, inventory, decision doc and lint fix (#739)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLyr6J2gRoqayc2nvJTNGy
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -531,14 +530,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>806</v>
+        <v>812</v>
       </c>
       <c r="C6" t="n">
         <v>851</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>94.7%</t>
+          <t>95.4%</t>
         </is>
       </c>
     </row>
@@ -549,14 +548,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C7" t="n">
         <v>141</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>96.5%</t>
+          <t>97.2%</t>
         </is>
       </c>
     </row>
@@ -567,14 +566,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C8" t="n">
         <v>137</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>90.5%</t>
+          <t>92.0%</t>
         </is>
       </c>
     </row>
@@ -585,14 +584,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>91.0%</t>
+          <t>92.5%</t>
         </is>
       </c>
     </row>
@@ -603,14 +602,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>94.8%</t>
+          <t>95.0%</t>
         </is>
       </c>
     </row>
@@ -621,14 +620,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C11" t="n">
         <v>152</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>95.4%</t>
+          <t>97.4%</t>
         </is>
       </c>
     </row>
@@ -639,14 +638,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>90.1%</t>
+          <t>91.4%</t>
         </is>
       </c>
     </row>
@@ -675,14 +674,14 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C14" t="n">
         <v>26</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>96.2%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -711,14 +710,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2088</v>
+        <v>2105</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>94.2%</t>
+          <t>94.9%</t>
         </is>
       </c>
     </row>
@@ -782,11 +781,6 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Region</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
           <t>TOTAL</t>
         </is>
       </c>
@@ -801,31 +795,25 @@
         <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G20" t="n">
-        <v>12</v>
-      </c>
-      <c r="H20" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I20" t="n">
         <v>2</v>
       </c>
       <c r="K20" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21">
@@ -838,10 +826,10 @@
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
@@ -850,13 +838,13 @@
         <v>6</v>
       </c>
       <c r="I21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J21" t="n">
         <v>1</v>
       </c>
-      <c r="L21" t="n">
-        <v>32</v>
+      <c r="K21" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="22">
@@ -866,7 +854,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D22" t="n">
         <v>1</v>
@@ -881,7 +869,7 @@
         <v>3</v>
       </c>
       <c r="H22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I22" t="n">
         <v>1</v>
@@ -889,8 +877,8 @@
       <c r="J22" t="n">
         <v>1</v>
       </c>
-      <c r="L22" t="n">
-        <v>24</v>
+      <c r="K22" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="23">
@@ -900,7 +888,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D23" t="n">
         <v>2</v>
@@ -909,7 +897,7 @@
         <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G23" t="n">
         <v>6</v>
@@ -920,54 +908,51 @@
       <c r="I23" t="n">
         <v>1</v>
       </c>
-      <c r="L23" t="n">
-        <v>21</v>
+      <c r="K23" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Promotional–Emperor</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>1</v>
+          <t>Promotional–Celestial</t>
+        </is>
       </c>
       <c r="G24" t="n">
         <v>1</v>
       </c>
       <c r="H24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
         <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>6</v>
+        <v>1</v>
+      </c>
+      <c r="K24" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Promotional–Celestial</t>
-        </is>
+          <t>Promotional–Emperor</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
       </c>
       <c r="G25" t="n">
         <v>1</v>
       </c>
-      <c r="H25" t="n">
-        <v>2</v>
-      </c>
       <c r="I25" t="n">
         <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
-      </c>
-      <c r="L25" t="n">
+        <v>2</v>
+      </c>
+      <c r="K25" t="n">
         <v>5</v>
       </c>
     </row>
@@ -980,7 +965,7 @@
       <c r="G26" t="n">
         <v>2</v>
       </c>
-      <c r="L26" t="n">
+      <c r="K26" t="n">
         <v>2</v>
       </c>
     </row>
@@ -994,34 +979,31 @@
         <v>2</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I27" s="2" t="n">
         <v>7</v>
-      </c>
-      <c r="I27" s="2" t="n">
-        <v>8</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>5</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L27" s="2" t="n">
-        <v>129</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -5452,7 +5434,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -5460,11 +5442,7 @@
           <t>Asako Usohara (Personality, Emperor Edition, issue #699): "Limited, bow: Search your Dynasty discard pile, then deck, for a Fudo Celestial. Put it into play." and "Limited: Put a Fudo Ring from your hand into play. This counts as playing it by its own text. Remove Usohara from the game." The second line is now buildable (the Ring-entry record of WlRings.cs takes an own-text entry with Usohara as source), but the first needs a search whose destination is IN PLAY for a Celestial (Zone.Celestial entry from the Dynasty discard pile or deck, honouring Unique and the Celestial's entry rules); the search catalogue's destinations are hand, province, holding and Ring-into-play only. A card with two printed lines is wired whole or blocked. Needs a search-to-Celestial-in-play destination.</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>SEARCH</t>
-        </is>
-      </c>
+      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -12784,7 +12762,7 @@
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
@@ -14546,7 +14524,7 @@
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G396" t="inlineStr"/>
@@ -14648,7 +14626,7 @@
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G399" t="inlineStr"/>
@@ -16484,7 +16462,7 @@
       </c>
       <c r="F453" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G453" t="inlineStr">
@@ -30980,7 +30958,7 @@
       </c>
       <c r="F879" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G879" t="inlineStr"/>
@@ -32944,7 +32922,7 @@
       </c>
       <c r="F937" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G937" t="inlineStr">
@@ -37046,7 +37024,7 @@
       </c>
       <c r="F1058" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1058" t="inlineStr"/>
@@ -39298,7 +39276,7 @@
       </c>
       <c r="F1124" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1124" t="inlineStr"/>
@@ -43670,7 +43648,7 @@
       </c>
       <c r="F1252" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1252" t="inlineStr"/>
@@ -45404,7 +45382,7 @@
       </c>
       <c r="F1303" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1303" t="inlineStr"/>
@@ -56334,7 +56312,7 @@
       </c>
       <c r="F1622" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1622" t="inlineStr">
@@ -67938,7 +67916,7 @@
       </c>
       <c r="F1962" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1962" t="inlineStr">
@@ -67946,11 +67924,7 @@
           <t>Hidden Weapons (Holding, issue #653): "Limited: Put a Weapon in your hand under this Holding (face-down)" and "You may Equip Weapons from under this Holding as a Battle/Limited action" need a zone of cards under a particular Holding that is hidden from the other player. The only under-card zone (Zone.Underneath) is face-up, public and kept under the Stronghold, not per card, and its view projection shows every card in it; hiding a face-down card and equipping from it with the Equip action's own pricing needs a new hidden zone and its projection.</t>
         </is>
       </c>
-      <c r="H1962" t="inlineStr">
-        <is>
-          <t>ZONE</t>
-        </is>
-      </c>
+      <c r="H1962" t="inlineStr"/>
     </row>
     <row r="1963">
       <c r="A1963" t="inlineStr">
@@ -68222,7 +68196,7 @@
       </c>
       <c r="F1970" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1970" t="inlineStr"/>
@@ -70988,7 +70962,7 @@
       </c>
       <c r="F2051" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2051" t="inlineStr"/>
@@ -71914,7 +71888,7 @@
       </c>
       <c r="F2078" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2078" t="inlineStr"/>
@@ -75786,7 +75760,7 @@
       </c>
       <c r="F2190" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2190" t="inlineStr"/>
@@ -76957,7 +76931,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -77317,7 +77291,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Batch 4 (#735): wire 16 keyword-rule, Home and Tireless cards
Chuda Hikano, Chun, Daidoji Gensai, Doji Tatsuzo, The Shakash - exp, The Sorrow, Tsiang the Benevolent, Elephant Cavalry, Long-Range Scouts, Uji's Saboteurs, Anchored in Earth, Chikushudo's Infusion, Drawing on All Things, Scorching Lash, Suikihime's Sanction and The Inevitable Grasp of Conquest, on P10, P16, P2, P12 and P24. Isawa Tsumaro and Blood of Isawa's Tribe are deferred with blocker notes.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLyr6J2gRoqayc2nvJTNGy
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,6 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -530,14 +529,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>812</v>
+        <v>830</v>
       </c>
       <c r="C6" t="n">
         <v>851</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>95.4%</t>
+          <t>97.5%</t>
         </is>
       </c>
     </row>
@@ -548,14 +547,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C7" t="n">
         <v>141</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>97.2%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -566,14 +565,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C8" t="n">
         <v>137</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>92.0%</t>
+          <t>93.4%</t>
         </is>
       </c>
     </row>
@@ -584,14 +583,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>92.5%</t>
+          <t>98.5%</t>
         </is>
       </c>
     </row>
@@ -602,14 +601,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>568</v>
+        <v>583</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>95.0%</t>
+          <t>97.5%</t>
         </is>
       </c>
     </row>
@@ -620,14 +619,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C11" t="n">
         <v>152</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>97.4%</t>
+          <t>98.0%</t>
         </is>
       </c>
     </row>
@@ -638,14 +637,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>91.4%</t>
+          <t>92.6%</t>
         </is>
       </c>
     </row>
@@ -656,14 +655,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C13" t="n">
         <v>37</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>86.5%</t>
+          <t>91.9%</t>
         </is>
       </c>
     </row>
@@ -710,14 +709,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2105</v>
+        <v>2156</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>94.9%</t>
+          <t>97.2%</t>
         </is>
       </c>
     </row>
@@ -746,40 +745,35 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Follower</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Spell</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Spell</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Strategy</t>
+          <t>Holding</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Holding</t>
+          <t>Event</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Event</t>
+          <t>Celestial</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Celestial</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -788,7 +782,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Torn Asunder</t>
+          <t>Coils of Madness</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -798,53 +792,44 @@
         <v>12</v>
       </c>
       <c r="D20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" t="n">
         <v>1</v>
       </c>
-      <c r="E20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" t="n">
-        <v>4</v>
-      </c>
-      <c r="G20" t="n">
-        <v>11</v>
-      </c>
-      <c r="I20" t="n">
-        <v>2</v>
-      </c>
-      <c r="K20" t="n">
-        <v>32</v>
+      <c r="J20" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Coils of Madness</t>
+          <t>Torn Asunder</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>15</v>
+        <v>5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
+        <v>7</v>
+      </c>
+      <c r="H21" t="n">
         <v>1</v>
       </c>
-      <c r="G21" t="n">
-        <v>6</v>
-      </c>
-      <c r="I21" t="n">
-        <v>1</v>
-      </c>
       <c r="J21" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22">
@@ -854,53 +839,35 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="n">
         <v>1</v>
       </c>
-      <c r="E22" t="n">
-        <v>3</v>
-      </c>
-      <c r="F22" t="n">
-        <v>2</v>
-      </c>
       <c r="G22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H22" t="n">
         <v>1</v>
       </c>
-      <c r="I22" t="n">
-        <v>1</v>
-      </c>
       <c r="J22" t="n">
-        <v>1</v>
-      </c>
-      <c r="K22" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gates of Chaos</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>3</v>
-      </c>
-      <c r="D23" t="n">
+          <t>Promotional–Celestial</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="n">
         <v>2</v>
-      </c>
-      <c r="E23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G23" t="n">
-        <v>6</v>
       </c>
       <c r="H23" t="n">
         <v>1</v>
@@ -908,52 +875,52 @@
       <c r="I23" t="n">
         <v>1</v>
       </c>
-      <c r="K23" t="n">
-        <v>18</v>
+      <c r="J23" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Promotional–Celestial</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
+          <t>Promotional–Emperor</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
         <v>1</v>
       </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
       <c r="H24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" t="n">
         <v>2</v>
       </c>
-      <c r="I24" t="n">
-        <v>1</v>
-      </c>
       <c r="J24" t="n">
-        <v>1</v>
-      </c>
-      <c r="K24" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Promotional–Emperor</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
+          <t>Gates of Chaos</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
         <v>1</v>
       </c>
-      <c r="G25" t="n">
+      <c r="D25" t="n">
         <v>1</v>
       </c>
-      <c r="I25" t="n">
+      <c r="F25" t="n">
         <v>1</v>
       </c>
+      <c r="H25" t="n">
+        <v>1</v>
+      </c>
       <c r="J25" t="n">
-        <v>2</v>
-      </c>
-      <c r="K25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
@@ -962,10 +929,10 @@
           <t>War of Honor</t>
         </is>
       </c>
-      <c r="G26" t="n">
+      <c r="F26" t="n">
         <v>2</v>
       </c>
-      <c r="K26" t="n">
+      <c r="J26" t="n">
         <v>2</v>
       </c>
     </row>
@@ -979,31 +946,28 @@
         <v>2</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K27" s="2" t="n">
-        <v>112</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -3348,7 +3312,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -7236,7 +7200,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G182" t="inlineStr"/>
@@ -7440,7 +7404,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G188" t="inlineStr"/>
@@ -7576,7 +7540,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G192" t="inlineStr"/>
@@ -9612,7 +9576,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G252" t="inlineStr"/>
@@ -10054,7 +10018,7 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G265" t="inlineStr"/>
@@ -12690,7 +12654,7 @@
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
@@ -14181,12 +14145,12 @@
       </c>
       <c r="G386" t="inlineStr">
         <is>
-          <t>Isawa Tsumaro (Personality, issue #677): his created card now has a published proxy (Tsumaro's Illusion, oracle-l5r-11346, a 0F/3C/0PH Air - Illusion - Shugenja Personality). "Air Home Engage: Move your target Air Shugenja home. Create a ... Personality at the current battlefield; remove him from the game after the battle ends" is made of pieces that exist (the Engage window, the Home flag of issue #672, the move home, a creation at the battlefield until the battle ends), though they were not exercised together because he is not wired. The last sentence has no piece: "While the Illusion is there, abilities on the target's spells have Home" is a grant that lasts while one particular card stays at one battlefield. A granted Home is a keyword grant with a turn duration (TirelessHome.cs); nothing ends a grant when a named card leaves a battlefield, and the presence grants of primitive P16 were not built. Wiring him without that sentence would publish a card with a printed effect missing.</t>
+          <t>Isawa Tsumaro (Personality, issue #735): "Air Home Engage: Move your target Air Shugenja home. Create a 0F/3C/0PH Air - Illusion - Shugenja Personality at the current battlefield; remove him from the game after the battle ends. While the Illusion is there, abilities on the target's spells have Home." Three pieces are missing. (1) Home (P16) waives only the source-at-the-battlefield checks of a Battle action: an Engage action is a Reaction after the engage (IsEngageAction), whose source must be at the battlefield, so a Home Engage from home is not a merged path. (2) The created Illusion has no created-card scan: the only Illusion proxy (Minor Illusion, oracle-l5r-11341) takes the Chi and Personal Honor of a wielder and has 0 printed Chi, while this one prints 3C and the Air keyword. (3) "While the Illusion is there, abilities on the target's spells have Home" is a grant tied to a created card's presence (P10's rules read a source card's Effect, not a link from one created card to a chosen target's Spells). Publishing it without them would approximate the card, so it is left unpublished.</t>
         </is>
       </c>
       <c r="H386" t="inlineStr">
         <is>
-          <t>GRANT</t>
+          <t>TRIG-ANN</t>
         </is>
       </c>
     </row>
@@ -17460,7 +17424,7 @@
       </c>
       <c r="F482" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G482" t="inlineStr"/>
@@ -17630,7 +17594,7 @@
       </c>
       <c r="F487" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G487" t="inlineStr">
@@ -17638,11 +17602,7 @@
           <t>Needs verified Butterfly proxy traits and alternative target selection with destruction after targeting.</t>
         </is>
       </c>
-      <c r="H487" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+      <c r="H487" t="inlineStr"/>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
@@ -19292,7 +19252,7 @@
       </c>
       <c r="F536" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G536" t="inlineStr">
@@ -21658,7 +21618,7 @@
       </c>
       <c r="F605" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G605" t="inlineStr"/>
@@ -22806,7 +22766,7 @@
       </c>
       <c r="F639" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G639" t="inlineStr"/>
@@ -24064,7 +24024,7 @@
       </c>
       <c r="F676" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G676" t="inlineStr"/>
@@ -26444,7 +26404,7 @@
       </c>
       <c r="F746" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G746" t="inlineStr">
@@ -26920,7 +26880,7 @@
       </c>
       <c r="F760" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G760" t="inlineStr">
@@ -26928,11 +26888,7 @@
           <t>Not wired in #689 (a draft wiring was removed untested): the Nonhuman entry discount and "move your target Personality at any location to Shakash's location" (Home-capable) need their own card pass and tests.</t>
         </is>
       </c>
-      <c r="H760" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+      <c r="H760" t="inlineStr"/>
     </row>
     <row r="761">
       <c r="A761" t="inlineStr">
@@ -26996,7 +26952,7 @@
       </c>
       <c r="F762" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G762" t="inlineStr"/>
@@ -28140,7 +28096,7 @@
       </c>
       <c r="F796" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G796" t="inlineStr">
@@ -28148,11 +28104,7 @@
           <t>Not wired in #689 (draft wiring removed untested): Ring of Water entry waiver plus straightening one or two cards in units, performed from Home, need their own card pass and tests.</t>
         </is>
       </c>
-      <c r="H796" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+      <c r="H796" t="inlineStr"/>
     </row>
     <row r="797">
       <c r="A797" t="inlineStr">
@@ -30686,7 +30638,7 @@
       </c>
       <c r="F871" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G871" t="inlineStr"/>
@@ -33054,7 +33006,7 @@
       </c>
       <c r="F941" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G941" t="inlineStr">
@@ -33424,7 +33376,7 @@
       </c>
       <c r="F952" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G952" t="inlineStr">
@@ -34504,7 +34456,7 @@
       </c>
       <c r="F984" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G984" t="inlineStr">
@@ -36136,7 +36088,7 @@
       </c>
       <c r="F1032" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1032" t="inlineStr">
@@ -37882,7 +37834,7 @@
       </c>
       <c r="F1083" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1083" t="inlineStr"/>
@@ -41120,7 +41072,7 @@
       </c>
       <c r="F1178" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1178" t="inlineStr"/>
@@ -41358,7 +41310,7 @@
       </c>
       <c r="F1185" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1185" t="inlineStr"/>
@@ -41426,7 +41378,7 @@
       </c>
       <c r="F1187" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1187" t="inlineStr"/>
@@ -41599,8 +41551,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1192" t="inlineStr"/>
-      <c r="H1192" t="inlineStr"/>
+      <c r="G1192" t="inlineStr">
+        <is>
+          <t>Blood of Isawa's Tribe (Spell, issue #735): "After this card attaches: Choose an element keyword (Air, Earth, Fire, Void, Water) in this Shugenja's keywords or text. While this card is attached, replace all instances of that keyword on this Shugenja with another element keyword that you choose now." P10's ReplaceElementKeyword does the replacement, but the choice is the problem: it is a mandatory trait of the Spell (no "Reaction:" prefix) that needs two decisions in a row (which element, then which replacement) the moment the Spell attaches. Mandatory entry effects (ApplyMandatoryEntryEffects) are automatic and open no decision, and an optional Reaction would change the printed text from mandatory to optional. Opening a pending choice from inside the entry path (before the entry Reaction window, for an attach by Equip, Equip (Battle) or a search) is not a merged path, and "in this Shugenja's keywords or text" would also need a rule for the elements named in text. It is left unpublished rather than approximated.</t>
+        </is>
+      </c>
+      <c r="H1192" t="inlineStr">
+        <is>
+          <t>TRIG-ANN</t>
+        </is>
+      </c>
     </row>
     <row r="1193">
       <c r="A1193" t="inlineStr">
@@ -41834,7 +41794,7 @@
       </c>
       <c r="F1199" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1199" t="inlineStr"/>
@@ -42038,7 +41998,7 @@
       </c>
       <c r="F1205" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1205" t="inlineStr">
@@ -42046,11 +42006,7 @@
           <t>Constructing the Self (Spell, issue #677): its created card now has a published proxy (Minor Illusion, oracle-l5r-11341, a 0F Illusion - Nonhuman - Cavalry - Shugenja Personality whose Chi and Personal Honor are printed "*"), and the two values could be written on the created card as it is made (as The Wind's Champion's Force is, CreatedProxies677.cs). What is missing is its last sentence, "After the next time this game this Spell straightens or leaves play, remove the Illusion from the game": a standing watch that ties one created card to one Spell and fires when that Spell is straightened by anything (the Straighten Phase, an effect) or leaves play by any path. Straighten() and the leaving-play paths have no feature hook, and nothing records which Illusion a Spell made. "This Spell may remain bowed" is the engine's optional straightening (the choose-straighten effect), which exists. Question for Mendon: are the Illusion's Chi and Personal Honor fixed when it is created, or do they follow the Shugenja's as his change (the proxy prints "are equal to the Chi and Personal Honor of the caster")?</t>
         </is>
       </c>
-      <c r="H1205" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
+      <c r="H1205" t="inlineStr"/>
     </row>
     <row r="1206">
       <c r="A1206" t="inlineStr">
@@ -42284,7 +42240,7 @@
       </c>
       <c r="F1212" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1212" t="inlineStr"/>
@@ -42590,7 +42546,7 @@
       </c>
       <c r="F1221" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1221" t="inlineStr"/>
@@ -43134,7 +43090,7 @@
       </c>
       <c r="F1237" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1237" t="inlineStr"/>
@@ -43920,7 +43876,7 @@
       </c>
       <c r="F1260" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1260" t="inlineStr"/>
@@ -45934,7 +45890,7 @@
       </c>
       <c r="F1319" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1319" t="inlineStr"/>
@@ -46138,7 +46094,7 @@
       </c>
       <c r="F1325" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1325" t="inlineStr"/>
@@ -46172,7 +46128,7 @@
       </c>
       <c r="F1326" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1326" t="inlineStr"/>
@@ -49724,7 +49680,7 @@
       </c>
       <c r="F1430" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1430" t="inlineStr"/>
@@ -52736,7 +52692,7 @@
       </c>
       <c r="F1518" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1518" t="inlineStr"/>
@@ -54452,7 +54408,7 @@
       </c>
       <c r="F1568" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1568" t="inlineStr"/>
@@ -56758,7 +56714,7 @@
       </c>
       <c r="F1635" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1635" t="inlineStr"/>
@@ -57336,7 +57292,7 @@
       </c>
       <c r="F1652" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1652" t="inlineStr"/>
@@ -59614,7 +59570,7 @@
       </c>
       <c r="F1719" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1719" t="inlineStr"/>
@@ -60124,7 +60080,7 @@
       </c>
       <c r="F1734" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1734" t="inlineStr"/>
@@ -60600,7 +60556,7 @@
       </c>
       <c r="F1748" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1748" t="inlineStr"/>
@@ -61110,7 +61066,7 @@
       </c>
       <c r="F1763" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1763" t="inlineStr"/>
@@ -61590,7 +61546,7 @@
       </c>
       <c r="F1777" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1777" t="inlineStr"/>
@@ -64844,7 +64800,7 @@
       </c>
       <c r="F1872" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1872" t="inlineStr"/>
@@ -65252,7 +65208,7 @@
       </c>
       <c r="F1884" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G1884" t="inlineStr"/>
@@ -71030,7 +70986,7 @@
       </c>
       <c r="F2053" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2053" t="inlineStr">
@@ -71038,11 +70994,7 @@
           <t>The Tower of Vigilance (Holding, issue #677): its created card now has a published proxy (Tower Guard, oracle-l5r-11345, a 0F/2C/2PH Guard - Samurai Personality), and creating a Personality at the current battlefield until the battle ends is built. The card itself is a Fortification ("Fortifications attach, straightened, to the Province from which they entered play"), and no Fortification is built: a Holding has no province it is attached to, so "If you have any units at this battlefield ... create ... there" has no battlefield to read, and the Holding does not leave play with its Province.</t>
         </is>
       </c>
-      <c r="H2053" t="inlineStr">
-        <is>
-          <t>PROVINCE</t>
-        </is>
-      </c>
+      <c r="H2053" t="inlineStr"/>
     </row>
     <row r="2054">
       <c r="A2054" t="inlineStr">
@@ -72364,7 +72316,7 @@
       </c>
       <c r="F2092" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2092" t="inlineStr"/>
@@ -73581,8 +73533,16 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G2127" t="inlineStr"/>
-      <c r="H2127" t="inlineStr"/>
+      <c r="G2127" t="inlineStr">
+        <is>
+          <t>The Empire's Foe Exposed (Event, issue #740): "Limited: Target two Unique Personalities in play, exactly one of which is yours. Your Personality challenges the other Personality. Destroy the duel's loser." The scan prints no "After you reveal" clause, so it is an ordinary Event that resolves when it is revealed in the Events Phase. Every merged duel starts from an ability a player uses (IssueChallenge is reached only from the IssuesDuel branch of an ability's effects, in a battle or the Action Phase), and P18's rules, refusal and focus windows resume play with NextAction for the challenger. Starting a duel from inside an Event's reveal (a pause on two chosen Unique Personalities, then a duel whose end must resume the Events Phase's reveal loop) is not a merged path, and the Event has no ability a player could use later. Publishing it as a reveal-time duel would need that resumption built and tested, so the card is left unpublished rather than approximated.</t>
+        </is>
+      </c>
+      <c r="H2127" t="inlineStr">
+        <is>
+          <t>DUEL</t>
+        </is>
+      </c>
     </row>
     <row r="2128">
       <c r="A2128" t="inlineStr">
@@ -74682,7 +74642,7 @@
       </c>
       <c r="F2159" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2159" t="inlineStr"/>
@@ -75318,7 +75278,7 @@
       </c>
       <c r="F2177" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G2177" t="inlineStr"/>
@@ -76891,7 +76851,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -76951,7 +76911,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -76971,7 +76931,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -77111,7 +77071,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -77191,7 +77151,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -77251,7 +77211,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Refresh card inventory and audit stale blocker notes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLyr6J2gRoqayc2nvJTNGy
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -1256,7 +1256,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Foothold of the Mad (Stronghold; one of the 13 cards awaiting a ruling from Mendon): "If there is no other Foothold of the Mad player, you go first" has no engine home. The first player is fixed when the match is set up (the rulebook's higher Starting Family Honor, ties random; CustomPractice.cs chooses it for practice) and no card can alter it, and how a Stronghold trait changes that determination is unruled. The other sentences map to merged pieces (no Honor loss from cards you own is P14, Fallen joining for 2 less is P2/P3, Give a target card a Madness token is the panku-madness shape), except "-1F for each of their Madness tokens": the P9 counters (StatTerms.cs TermCounterKind) are only AttachedWithKeyword and OpposingTokens, so a count of a card's own tokens is new. Not wired.</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -1426,7 +1430,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Journey's End Keep - exp (Stronghold; one of the 13 cards awaiting a ruling from Mendon): the Gold lock ("when this Stronghold produces Gold, you may not Recruit Personalities until the phase ends or until after you have spent 5 total Gold for non-Recruit costs or payments") is buildable on merged pieces: the P1 per-phase ledger (GoldSpentThisPhaseExceptRecruit, PaymentHooks695.cs) and the P3 recruit gate (RecruitGates695.cs). Still open: (1) "'Imperial' is a Clan Alignment, and it is your Clan Alignment" (how an Imperial player's alignment interacts with Clan Allegiance, Loyal and the Clan discount is unruled; ClanEntryDiscount reads the stronghold's Clan); (2) "if no other player has an Imperial Stronghold, you begin the game with the Imperial Favor" has no setup hook; (3) the no-Clan-discount trait only matters under the optional Clan Discount rule. Not wired.</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -2174,11 +2182,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>The False Path (Stronghold, issue #699): "You may not win by Enlightenment" is now a one-line read of the Ring-entry primitive's Enlightenment check, but the card is a whole Stronghold: its non-Unique Monk and Fudo Personalities gain Monk and Fudo in and out of play, Fudo Personalities join for 2 less Gold, Honor Requirements of Fudo cards are ignored, no Honor is lost from owned Fudo cards, and a Limited bow search for a Fudo Ring. Granting keywords to cards out of play and the Fudo Honor waivers are separate primitives, and no stronghold scan is packaged in the rings waves.</t>
-        </is>
-      </c>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
@@ -3300,11 +3304,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>Needs a modifier hook into the existing Tactical Advantage rulebook action's own Force-bonus amount (a generic action-amount-modifier mechanism doesn't exist yet).</t>
-        </is>
-      </c>
+      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
@@ -3746,11 +3746,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>Needs a 'retrieve a specific card from your discard pile into hand' primitive (distinct from deck search; not built).</t>
-        </is>
-      </c>
+      <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
@@ -4320,11 +4316,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>Needs P6 (after-event records and windows); P7's watch half alone does not wire it.</t>
-        </is>
-      </c>
+      <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
@@ -5386,11 +5378,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>Asako Usohara (Personality, Emperor Edition, issue #699): "Limited, bow: Search your Dynasty discard pile, then deck, for a Fudo Celestial. Put it into play." and "Limited: Put a Fudo Ring from your hand into play. This counts as playing it by its own text. Remove Usohara from the game." The second line is now buildable (the Ring-entry record of WlRings.cs takes an own-text entry with Usohara as source), but the first needs a search whose destination is IN PLAY for a Celestial (Zone.Celestial entry from the Dynasty discard pile or deck, honouring Unique and the Celestial's entry rules); the search catalogue's destinations are hand, province, holding and Ring-into-play only. A card with two printed lines is wired whole or blocked. Needs a search-to-Celestial-in-play destination.</t>
-        </is>
-      </c>
+      <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
@@ -6984,11 +6972,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>Needs an "Absent Interrupt" mechanic (Bayushi Wateru's own printed ability, on top of Reserve).</t>
-        </is>
-      </c>
+      <c r="G176" t="inlineStr"/>
       <c r="H176" t="inlineStr"/>
     </row>
     <row r="177">
@@ -7256,7 +7240,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G184" t="inlineStr"/>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Chuda Kaito (Personality; one of the 13 cards awaiting a ruling from Mendon): "Kaito has +3GC while the effects of a Spell action he performed are resolving" needs a ruling on what +3GC modifies and when it is read. The entry Honor loss is trivial, and a bonus that applies while a particular command resolves has a precedent for Force (Usagi Seki, Wave734.cs), but no Gold Cost term reads the resolving command (CardGoldCost has no such hook). Not wired.</t>
+        </is>
+      </c>
       <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
@@ -8276,11 +8264,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G214" t="inlineStr">
-        <is>
-          <t>Needs a Follower-Equip Battle ability with no Shugenja/opposed requirement (Daigotsu Chiboshi's own "Equip a Follower to Chiboshi"; the attach primitive of issue #337 needs a hand pile for it), plus tying its own Additional Action grant to a Reserve recruitment specifically.</t>
-        </is>
-      </c>
+      <c r="G214" t="inlineStr"/>
       <c r="H214" t="inlineStr"/>
     </row>
     <row r="215">
@@ -8722,11 +8706,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G227" t="inlineStr">
-        <is>
-          <t>Not wired in #689 (draft wiring removed untested): Invest cost by Clan (a P2 ability cost term) creating two 1F Followers on Kikumura needs its own card pass, the Follower proxy check and tests.</t>
-        </is>
-      </c>
+      <c r="G227" t="inlineStr"/>
       <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
@@ -11924,11 +11904,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G322" t="inlineStr">
-        <is>
-          <t>Needs a controller choice when multiple attached Followers would be destroyed simultaneously; a per-card watch cannot choose which single destruction to negate.</t>
-        </is>
-      </c>
+      <c r="G322" t="inlineStr"/>
       <c r="H322" t="inlineStr"/>
     </row>
     <row r="323">
@@ -12366,11 +12342,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G335" t="inlineStr">
-        <is>
-          <t>Hyobuko: her 'Attaches Heart of Fudo ignoring Gold cost' needs the Heart of Fudo Item (oracle-l5r-3014), which is unwired and whose created Fudo Personality scan is still missing (docs/requests/created-card-scans-needed.md, B1); the search half alone would leave her attach trait inert.</t>
-        </is>
-      </c>
+      <c r="G335" t="inlineStr"/>
       <c r="H335" t="inlineStr"/>
     </row>
     <row r="336">
@@ -12642,11 +12614,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G343" t="inlineStr">
-        <is>
-          <t>Needs a 'will not gain [keyword]' immunity flag, and a per-performer Timing override on the shared Tactical Advantage rulebook action -- neither built.</t>
-        </is>
-      </c>
+      <c r="G343" t="inlineStr"/>
       <c r="H343" t="inlineStr"/>
     </row>
     <row r="344">
@@ -12714,11 +12682,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G345" t="inlineStr">
-        <is>
-          <t>Invest itself is built, but this variant needs 'refill the specific province this card entered from, face-up' -- a targeted, face-up province refill tied to entry-provenance (existing refills are face-down and untargeted).</t>
-        </is>
-      </c>
+      <c r="G345" t="inlineStr"/>
       <c r="H345" t="inlineStr"/>
     </row>
     <row r="346">
@@ -12820,11 +12784,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G348" t="inlineStr">
-        <is>
-          <t>The Open Cavalry-grant is directly wirable (reuses the existing generic GrantKeyword primitive); blocked only by 'will not join a Unicorn Clan player' -- a recruitment clan-exclusion rule, not built.</t>
-        </is>
-      </c>
+      <c r="G348" t="inlineStr"/>
       <c r="H348" t="inlineStr"/>
     </row>
     <row r="349">
@@ -12860,7 +12820,7 @@
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>Needs a reveal-a-hand-card-and-offer-to-another-player mechanism with an opponent's accept/reject choice, plus a Home-targeted Attack (existing Attacks only target the current battlefield).</t>
+          <t>Ikoma Satoru - exp (awaiting a ruling from Mendon): the Home-targeted Attack is no longer a gap: AttackSpec with TargetScope AnyLocation (P24, EffectPrimitivesAttack.cs) lets a Melee Attack reach a target in the other player's home (restricting it to that home is a small check). The gift step is still missing as an ability: "Show a card in your hand and choose another player: you offer him a gift; he may put the card in his hand; if he does, draw two cards, otherwise discard it and Melee Attack with strength equal to its Focus Value" needs the recipient's accept or refuse decision (EitherOr.cs supplies a decider) and a move into his hand. Naoharu's Gift does that move as Event-only code (EmperorRemainingFEvents.cs: ownership moves to the taker, OriginalOwnerId returns the card to its owner's pile when it leaves his hand), so a reusable ability form is needed and the reading carried over from that Event is for Mendon to confirm. Not wired.</t>
         </is>
       </c>
       <c r="H349" t="inlineStr"/>
@@ -14130,7 +14090,7 @@
       </c>
       <c r="G386" t="inlineStr">
         <is>
-          <t>Isawa Tsumaro (Personality, issue #735): "Air Home Engage: Move your target Air Shugenja home. Create a 0F/3C/0PH Air - Illusion - Shugenja Personality at the current battlefield; remove him from the game after the battle ends. While the Illusion is there, abilities on the target's spells have Home." Three pieces are missing. (1) Home (P16) waives only the source-at-the-battlefield checks of a Battle action: an Engage action is a Reaction after the engage (IsEngageAction), whose source must be at the battlefield, so a Home Engage from home is not a merged path. (2) The created Illusion has no created-card scan: the only Illusion proxy (Minor Illusion, oracle-l5r-11341) takes the Chi and Personal Honor of a wielder and has 0 printed Chi, while this one prints 3C and the Air keyword. (3) "While the Illusion is there, abilities on the target's spells have Home" is a grant tied to a created card's presence (P10's rules read a source card's Effect, not a link from one created card to a chosen target's Spells). Publishing it without them would approximate the card, so it is left unpublished.</t>
+          <t>Isawa Tsumaro (Personality, issue #735): "Air Home Engage: Move your target Air Shugenja home. Create a 0F/3C/0PH Air - Illusion - Shugenja Personality at the current battlefield; remove him from the game after the battle ends. While the Illusion is there, abilities on the target's spells have Home." The created card is no longer a gap: Tsumaro's Illusion (oracle-l5r-11346, 0F/3C/0PH Air - Illusion - Shugenja) is published in personality-wave-145 (issue #677). Two pieces are missing. (1) Home (P16) waives only the source-at-the-battlefield checks of a Battle action: an Engage action is a Reaction after the engage (IsEngageAction), whose source must be at the battlefield, so a Home Engage from home is not a merged path. (2) "While the Illusion is there, abilities on the target's spells have Home" is a grant tied to a created card's presence (granted Home has a turn duration only; P10's rules read a source card's Effect, not a link from one created card to a chosen target's Spells). Publishing it without them would approximate the card, so it is left unpublished.</t>
         </is>
       </c>
       <c r="H386" t="inlineStr">
@@ -14714,11 +14674,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G403" t="inlineStr">
-        <is>
-          <t>Ring of Earth is now published (ring-wave-1); 'Earth Battle' is very likely a plain printed-keyword classification too, following Moshi Ikako's own 'Fire Battle' precedent (oracle-l5r-10857, confirmed issue #194) -- not re-verified against this specific card's own scan yet. Still needs a conditional Gold-Cost waiver tied to Ring control before wiring Jikoji's own army-wide Force bonus (the waiver itself: no current Gold discount is conditional on board state, only clan-alignment-based or a fixed printed amount).</t>
-        </is>
-      </c>
+      <c r="G403" t="inlineStr"/>
       <c r="H403" t="inlineStr"/>
     </row>
     <row r="404">
@@ -15772,11 +15728,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G434" t="inlineStr">
-        <is>
-          <t>Needs conditional Gold-cost reduction (Kakita Ujirou's own "enters play for N less Gold if...").</t>
-        </is>
-      </c>
+      <c r="G434" t="inlineStr"/>
       <c r="H434" t="inlineStr"/>
     </row>
     <row r="435">
@@ -16172,11 +16124,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G446" t="inlineStr">
-        <is>
-          <t>Unchanged: the conditional zero-cost Purchase gate tied to a named Ring and the 'increase the Honor gained from your next Proclaim this turn' effect (a player-level modifier on a future gain, not a delayed effect on a card). NO LOCAL SCAN.</t>
-        </is>
-      </c>
+      <c r="G446" t="inlineStr"/>
       <c r="H446" t="inlineStr"/>
     </row>
     <row r="447">
@@ -16414,11 +16362,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G453" t="inlineStr">
-        <is>
-          <t>The deck search primitive now exists (issue #312) and its criteria can express "a non-Unique Lion Clan Shugenja" from the Dynasty deck, but the effect is "refill this province with him, face-up" (a search effect the primitive does not have yet) and the ability must be usable from a face-up province card whose own cost is discarding her and paying 2 Gold.</t>
-        </is>
-      </c>
+      <c r="G453" t="inlineStr"/>
       <c r="H453" t="inlineStr"/>
     </row>
     <row r="454">
@@ -16588,11 +16532,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G458" t="inlineStr">
-        <is>
-          <t>Needs Interrupt timing (not started); card creation is built (issue #387, the Lion Ancestor scan is published).</t>
-        </is>
-      </c>
+      <c r="G458" t="inlineStr"/>
       <c r="H458" t="inlineStr"/>
     </row>
     <row r="459">
@@ -16728,11 +16668,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G462" t="inlineStr">
-        <is>
-          <t>The look-at-the-top-N-cards primitive (issue #322) covers 'look at the top three cards of your Fate deck, show an Iaijutsu Strategy and put it into your hand, put the remaining cards back in any order' (a show disposition with criteria, exactly Bayushi Kahoku exp2's shape). Still needs the follow-up 'then discard a card' (the same after-effect step Ikoma Shizuka's Terrain half has in the deck search) and an Iaijutsu Strategy criteria check -- not wired in that PR.</t>
-        </is>
-      </c>
+      <c r="G462" t="inlineStr"/>
       <c r="H462" t="inlineStr"/>
     </row>
     <row r="463">
@@ -17582,11 +17518,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G487" t="inlineStr">
-        <is>
-          <t>Needs verified Butterfly proxy traits and alternative target selection with destruction after targeting.</t>
-        </is>
-      </c>
+      <c r="G487" t="inlineStr"/>
       <c r="H487" t="inlineStr"/>
     </row>
     <row r="488">
@@ -18334,11 +18266,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G509" t="inlineStr">
-        <is>
-          <t>Masaya: needs an Open action printed on a Personality and usable while that card is face-up in a province (not in play), with a 2-Gold reduction, plus a 'before the turn ends, put him on top of your Dynasty deck' delayed return; the engine only offers province-sourced Recruit via the Reserve keyword (RecruitReserve), a Battle-phase absent action, and has no card-sourced province Open ability.</t>
-        </is>
-      </c>
+      <c r="G509" t="inlineStr"/>
       <c r="H509" t="inlineStr"/>
     </row>
     <row r="510">
@@ -19248,11 +19176,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G536" t="inlineStr">
-        <is>
-          <t>Needs an Additional Action grant that re-triggers a second, differently-costed printed ability on the same performer -- buildable in principle by reusing the existing Additional Action primitive, but deferred this pass for scope.</t>
-        </is>
-      </c>
+      <c r="G536" t="inlineStr"/>
       <c r="H536" t="inlineStr"/>
     </row>
     <row r="537">
@@ -19320,11 +19244,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G538" t="inlineStr">
-        <is>
-          <t>Unblocked by the attach-from-a-discard-pile primitive (issue #337): "Battle, [Gold]: Equip a target non-Unique Weapon in your discard pile to Katagi" is one ability definition -- Attach: AttachSpec(Target, Own pile, Wielder Source, [Item], Keywords [Weapon], Excluded [Unique]) with Cost: GoldCostRule.AttachCost(), exactly the training-attach-weapon-discount shape at full cost (his from-hand discount does not apply to a discard-pile attach). Deferred for scope, not wired in #337.</t>
-        </is>
-      </c>
+      <c r="G538" t="inlineStr"/>
       <c r="H538" t="inlineStr"/>
     </row>
     <row r="539">
@@ -19426,11 +19346,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G541" t="inlineStr">
-        <is>
-          <t>Needs a generic 'ignore this card's own bowed status' exemption for Maneuvers assignment AND Performer selection together -- narrower exemptions exist per-ability (the 'Even if bowed' id list), but this card's own exemption is unconditional and would touch both of those shared checks broadly for a single card; deferred this pass to limit blast radius.</t>
-        </is>
-      </c>
+      <c r="G541" t="inlineStr"/>
       <c r="H541" t="inlineStr"/>
     </row>
     <row r="542">
@@ -19498,11 +19414,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G543" t="inlineStr">
-        <is>
-          <t>Needs a named-target restriction on a duel's own Target category (a self-performer duel against one specific enemy Personality by name, not any enemy) -- a small addition (mirrors AttachRequiresName's own shape) not attempted this pass.</t>
-        </is>
-      </c>
+      <c r="G543" t="inlineStr"/>
       <c r="H543" t="inlineStr"/>
     </row>
     <row r="544">
@@ -19944,11 +19856,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G556" t="inlineStr">
-        <is>
-          <t>Needs a control-transfer mechanic (explicitly deferred since Loyal, #142) -- specifically a temporary, Gold-production-only control grant over another player's Holding, without a full ownership change.</t>
-        </is>
-      </c>
+      <c r="G556" t="inlineStr"/>
       <c r="H556" t="inlineStr"/>
     </row>
     <row r="557">
@@ -21542,11 +21450,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G603" t="inlineStr">
-        <is>
-          <t>Needs action-source-card unit scope independent of the Personality performing a Strategy.</t>
-        </is>
-      </c>
+      <c r="G603" t="inlineStr"/>
       <c r="H603" t="inlineStr"/>
     </row>
     <row r="604">
@@ -22078,11 +21982,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G619" t="inlineStr">
-        <is>
-          <t>Needs attack prohibition during movement and entry, not assignment alone.</t>
-        </is>
-      </c>
+      <c r="G619" t="inlineStr"/>
       <c r="H619" t="inlineStr"/>
     </row>
     <row r="620">
@@ -22118,12 +22018,12 @@
       </c>
       <c r="G620" t="inlineStr">
         <is>
-          <t>P'an Ku - exp (Personality, issue #736): "Open, bow: Give a target card a Madness token" is built (the existing panku-madness shape), but "Limited, bow: P'an Ku may remain bowed. Take control of a target Personality with more Madness tokens than printed Personal Honor and remove those tokens. The target will not commit seppuku until P'an Ku straightens or leaves play. After P'an Ku does, give control of the target to his owner." needs three things together: a control change that returns when a named card straightens or leaves play (TakeControl exists; the timed return trigger does not), a seppuku bar tied to that card, and "may remain bowed" (a rule exempting him from straightening). One card, three new rules.</t>
+          <t>P'an Ku - exp (Personality, issue #736): "Open, bow: Give a target card a Madness token" is built (the existing panku-madness shape). "Limited, bow: P'an Ku may remain bowed. Take control of a target Personality with more Madness tokens than printed Personal Honor and remove those tokens. The target will not commit seppuku until P'an Ku straightens or leaves play. After P'an Ku does, give control of the target to his owner." Most of this is merged: the timed return of control is P24's ReturnControlWhenSourceStraightens (ControlReturnTriggers.SourceStraightens, EffectPrimitivesTokens.cs, built for this card: docs/decisions/2026-10-06-690-p24-effect-primitives.md section 8), and "may remain bowed" is the existing choose-straighten Effect (Constructing the Self uses it in batch 10). The remaining gap is the seppuku bar: no P11 restriction kind bars seppuku, and P5's SeppukuBar (EmperorP5Zones.cs) lasts one turn, so "will not commit seppuku until P'an Ku straightens or leaves play" needs a bar bound to a source card. His Effect slot must also carry choose-straighten alongside his other abilities.</t>
         </is>
       </c>
       <c r="H620" t="inlineStr">
         <is>
-          <t>CONTROL</t>
+          <t>SMALL</t>
         </is>
       </c>
     </row>
@@ -26400,11 +26300,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G746" t="inlineStr">
-        <is>
-          <t>Needs a 'destroy one of my own attached cards as a cost' cost-target category, combined with a temporary Stalwart grant and a self-Force-copy modifier -- each piece individually has precedent (DestroyAttachment, turn-duration GrantKeyword, ApplyModifier), but the three-part combination was deferred this pass for scope.</t>
-        </is>
-      </c>
+      <c r="G746" t="inlineStr"/>
       <c r="H746" t="inlineStr"/>
     </row>
     <row r="747">
@@ -26876,11 +26772,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G760" t="inlineStr">
-        <is>
-          <t>Not wired in #689 (a draft wiring was removed untested): the Nonhuman entry discount and "move your target Personality at any location to Shakash's location" (Home-capable) need their own card pass and tests.</t>
-        </is>
-      </c>
+      <c r="G760" t="inlineStr"/>
       <c r="H760" t="inlineStr"/>
     </row>
     <row r="761">
@@ -28092,11 +27984,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G796" t="inlineStr">
-        <is>
-          <t>Not wired in #689 (draft wiring removed untested): Ring of Water entry waiver plus straightening one or two cards in units, performed from Home, need their own card pass and tests.</t>
-        </is>
-      </c>
+      <c r="G796" t="inlineStr"/>
       <c r="H796" t="inlineStr"/>
     </row>
     <row r="797">
@@ -28840,11 +28728,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G818" t="inlineStr">
-        <is>
-          <t>Needs a genuine 'while another player's action is currently resolving' state flag, distinct from the simpler 'while it is not your turn' condition already used elsewhere (Tamori Yayu) -- a simplified reading would just reuse that existing pattern, but wasn't attempted here to avoid mischaracterizing the printed text.</t>
-        </is>
-      </c>
+      <c r="G818" t="inlineStr"/>
       <c r="H818" t="inlineStr"/>
     </row>
     <row r="819">
@@ -31076,11 +30960,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G884" t="inlineStr">
-        <is>
-          <t>Needs an "actions must target this card if legal" forced-redirection rule (Yoritomo Naoto's own Battle ability), on top of its own Additional Action grant. The legality half now exists (ActionAcceptsTarget, issue #335 -- "if legal" is that check); the standing hook that applies it to every action is the gap.</t>
-        </is>
-      </c>
+      <c r="G884" t="inlineStr"/>
       <c r="H884" t="inlineStr"/>
     </row>
     <row r="885">
@@ -32190,11 +32070,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G917" t="inlineStr">
-        <is>
-          <t>Needs a control-transfer mechanic (explicitly deferred since Loyal, #142).</t>
-        </is>
-      </c>
+      <c r="G917" t="inlineStr"/>
       <c r="H917" t="inlineStr"/>
     </row>
     <row r="918">
@@ -32628,11 +32504,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G930" t="inlineStr">
-        <is>
-          <t>Needs a "modify the next Honor change" pending-state mechanism.</t>
-        </is>
-      </c>
+      <c r="G930" t="inlineStr"/>
       <c r="H930" t="inlineStr"/>
     </row>
     <row r="931">
@@ -32870,11 +32742,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G937" t="inlineStr">
-        <is>
-          <t>Needs a new tracked EnteredPlayTurn field on CardInstance.</t>
-        </is>
-      </c>
+      <c r="G937" t="inlineStr"/>
       <c r="H937" t="inlineStr"/>
     </row>
     <row r="938">
@@ -33002,11 +32870,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G941" t="inlineStr">
-        <is>
-          <t>Needs "grant keyword to whole unit" (the passive Attack-strength defense half is now built -- Destrier/Singh Remnants -- and directly reusable here).</t>
-        </is>
-      </c>
+      <c r="G941" t="inlineStr"/>
       <c r="H941" t="inlineStr"/>
     </row>
     <row r="942">
@@ -33372,11 +33236,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G952" t="inlineStr">
-        <is>
-          <t>Its ordinary Equip is allowed from YOUR discard pile ("You may Equip this Follower from your discard pile"). The attach-from-a-discard-pile primitive exists (AttachAction.cs, issue #337) for an ability that TARGETS a card in a pile, but here the SOURCE card in the pile is the attachment (AttachSource.Self is hand-only) and the action is the ordinary Limited Equip command, not an ability -- not built.</t>
-        </is>
-      </c>
+      <c r="G952" t="inlineStr"/>
       <c r="H952" t="inlineStr"/>
     </row>
     <row r="953">
@@ -34116,11 +33976,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G974" t="inlineStr">
-        <is>
-          <t>Needs a per-card, permanent "this Personality may not attack" attachment flag (Utaku Chikako's own restriction, issue #186, is a player-and-turn-scoped flag, not directly reusable here) plus a self-destroying Limited ability. Dishonor-as-an-action is now built (Justice of the Crane) and directly reusable for its own Dishonor half.</t>
-        </is>
-      </c>
+      <c r="G974" t="inlineStr"/>
       <c r="H974" t="inlineStr"/>
     </row>
     <row r="975">
@@ -34316,11 +34172,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G980" t="inlineStr">
-        <is>
-          <t>Needs a persistent one-time destruction shield.</t>
-        </is>
-      </c>
+      <c r="G980" t="inlineStr"/>
       <c r="H980" t="inlineStr"/>
     </row>
     <row r="981">
@@ -34452,11 +34304,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G984" t="inlineStr">
-        <is>
-          <t>Needs an attachment Transfer mechanic plus Home-timing generalization.</t>
-        </is>
-      </c>
+      <c r="G984" t="inlineStr"/>
       <c r="H984" t="inlineStr"/>
     </row>
     <row r="985">
@@ -34524,11 +34372,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G986" t="inlineStr">
-        <is>
-          <t>Focus 4, not 1 -- outside the #192 wave's own scope. The top-of-Fate-deck discard primitive now exists (Aberrations, issue #192), but this needs a "whose deck" target choice ("any Fate deck", not just your own) plus a variable-strength Melee Attack keyed off the discarded card's Focus Value, not a Force modifier.</t>
-        </is>
-      </c>
+      <c r="G986" t="inlineStr"/>
       <c r="H986" t="inlineStr"/>
     </row>
     <row r="987">
@@ -35098,11 +34942,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1003" t="inlineStr">
-        <is>
-          <t>The Engage window and first-action claim now exist (issue #310; a Follower's 'Engage:' is a Reaction to trigger after-engaging, claim: MatchEngine.ClaimFirstOpportunity, conditional on being the Attacker). Still needs: a Follower-sourced Engage action scoped to 'this battlefield' (the Follower's own unit) and its optional 'you may target ... -3F' effect target; Reconnaissance for the acting side is settled (MatchEngine.GrantReconnaissanceAtCurrentBattlefield serves an Attacker at the enemy's province and a Defender at their own, see docs/decisions/2026-09-18-battle-timing-primitives.md decision 5).</t>
-        </is>
-      </c>
+      <c r="G1003" t="inlineStr"/>
       <c r="H1003" t="inlineStr"/>
     </row>
     <row r="1004">
@@ -35536,11 +35376,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1016" t="inlineStr">
-        <is>
-          <t>"You may Equip this Follower as a Battle action" is now a general capability (AttachSource.Self, issue #337: Fading Shadows attaches itself from hand to a performing Ninja). Shinobi Vassal differs in that the wielder is any Ninja Personality chosen as a target, and its own Battle action destroys a target enemy card without attachments and then the Follower itself -- deferred, not wired in #337.</t>
-        </is>
-      </c>
+      <c r="G1016" t="inlineStr"/>
       <c r="H1016" t="inlineStr"/>
     </row>
     <row r="1017">
@@ -35804,11 +35640,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1024" t="inlineStr">
-        <is>
-          <t>Needs a generic ability-usage-limit-reset mechanism.</t>
-        </is>
-      </c>
+      <c r="G1024" t="inlineStr"/>
       <c r="H1024" t="inlineStr"/>
     </row>
     <row r="1025">
@@ -35876,11 +35708,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1026" t="inlineStr">
-        <is>
-          <t>The Engage window now exists (issue #310); its 'Engage: Give a target enemy Personality or Follower -2F' is a Reaction to trigger after-engaging. Still needs: the same target category costly-feud uses (enemy-force), validated as 'at the current battlefield' by hand (a Reaction is not a Battle action, so the shared Battle-target check does not apply), and the Follower as source of a reaction (in play, attached).</t>
-        </is>
-      </c>
+      <c r="G1026" t="inlineStr"/>
       <c r="H1026" t="inlineStr"/>
     </row>
     <row r="1027">
@@ -36084,11 +35912,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1032" t="inlineStr">
-        <is>
-          <t>Needs a conditional-keyword-by-the-card's-own-clan mechanism (the attachment-destroy half is separately wirable).</t>
-        </is>
-      </c>
+      <c r="G1032" t="inlineStr"/>
       <c r="H1032" t="inlineStr"/>
     </row>
     <row r="1033">
@@ -36696,11 +36520,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1050" t="inlineStr">
-        <is>
-          <t>The multi-target slots exist (issue #336: one or two target enemy cards, a Min 1 / Max 2 slot); still needs the printed Fallen/maximum-Personal-Honor static and the bow cost; not yet wired.</t>
-        </is>
-      </c>
+      <c r="G1050" t="inlineStr"/>
       <c r="H1050" t="inlineStr"/>
     </row>
     <row r="1051">
@@ -37422,11 +37242,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1071" t="inlineStr">
-        <is>
-          <t>Coin Pouch: needs a payment-time Reaction in which this Item bows to add one Gold to a Holding bowing to produce Gold (a source tied to a specific Holding rather than a standalone Gold source), plus a static +2 Gold Cost on its wielder and an Item that enters play bowed.</t>
-        </is>
-      </c>
+      <c r="G1071" t="inlineStr"/>
       <c r="H1071" t="inlineStr"/>
     </row>
     <row r="1072">
@@ -38466,12 +38282,12 @@
       </c>
       <c r="G1102" t="inlineStr">
         <is>
-          <t>Koan's Jingasa (Item, issue #736): "This Personality has Shugenja, may not have more Spells than Koan cards attached, and he need not bow for his Spells with an odd Focus Value (0 is even)." The Shugenja keyword is AttachGrantsKeyword, but P11's SpellLimit counts Spell actions performed, not Spells attached (the rule here is an attachment limit counted against Koan cards), and "need not bow for his Spells" is a waiver of the bow cost of a Spell's own ability, which P24's cost waivers do not cover.</t>
+          <t>Koan's Jingasa (Item, issue #736): "This Personality has Shugenja, may not have more Spells than Koan cards attached, and he need not bow for his Spells with an odd Focus Value (0 is even)." The Shugenja keyword is AttachGrantsKeyword, and the bow waiver is merged: P24's EngineHooks.CostWaivers with SpellFocusParityWaives (EffectPrimitivesCosts.cs) is written for this card and Koan's Robes, and a wave registers the callback with the Item's Effect. What is still missing is the attachment limit: P11's SpellLimit counts Spell actions performed, not Spells attached, and NoAttach bars by type or keyword without counting, so "may not have more Spells than Koan cards attached" (a count of Koan cards on the host against his attached Spells) needs a new attach rule.</t>
         </is>
       </c>
       <c r="H1102" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>SMALL</t>
         </is>
       </c>
     </row>
@@ -38508,12 +38324,12 @@
       </c>
       <c r="G1103" t="inlineStr">
         <is>
-          <t>Koan's Robes (Item, issue #737): "This Personality has a Force bonus equal to the number of other Koan cards in this unit. This Personality need not bow for his Spells with an even Focus Value (0 is even). Negate the first destruction each turn of cards in this unit from another player's card." The destruction negation is a P7 standing watch (a unit scope is the only gap, and a Condition could stand in for it), but the other two sentences are not buildable on what is merged: a Force bonus counted from the Koan cards in the unit needs a P9 stat term that counts a keyword in the unit (batch 3 owns the stat terms and none is merged), and "need not bow for his Spells" is a waiver of the bow cost of a Spell's own ability, which no merged cost waiver covers (the same gap that deferred Koan's Jingasa in batch 5). Publishing it with only the negation would drop two printed sentences.</t>
+          <t>Koan's Robes (Item, issue #737): "This Personality has a Force bonus equal to the number of other Koan cards in this unit. This Personality need not bow for his Spells with an even Focus Value (0 is even). Negate the first destruction each turn of cards in this unit from another player's card." Part is merged: "need not bow for his Spells with an even Focus Value" is P24's EngineHooks.CostWaivers with SpellFocusParityWaives (odd: false; EffectPrimitivesCosts.cs, written for this card and Koan's Jingasa), and the destruction negation is a P7 standing watch whose scope is the gap (a StandingWatch covers the card, its controller's cards that fit a keyword, or its attached Followers; there is no cards-in-this-unit scope, and a Condition could stand in for it). Still missing: the Force bonus equal to the number of other Koan cards in this unit. Batch 3 merged its stat terms (StatTerms.cs), but the counters are only AttachedWithKeyword (the host's own attachments) and OpposingTokens; none counts a keyword across a unit (host, Followers and the other attachments). Publishing it without that sentence would drop printed text.</t>
         </is>
       </c>
       <c r="H1103" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>STAT</t>
         </is>
       </c>
     </row>
@@ -39122,7 +38938,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1121" t="inlineStr"/>
+      <c r="G1121" t="inlineStr">
+        <is>
+          <t>Ningen's 'Treatise on the Nezumi' (Item): multiplayer-only, and excluded from the wirable-card wave plan (#742, docs/decisions/2026-10-07-wirable-card-wave-plan.md) by Mendon. Its ability makes two players invite each other to ally and assign into each other's armies, and the engine has no allies and only two players; the Multiplayer keyword itself has no rules effect (core rules). Not wired; revisit only if multiplayer is built.</t>
+        </is>
+      </c>
       <c r="H1121" t="inlineStr"/>
     </row>
     <row r="1122">
@@ -40112,11 +39932,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1150" t="inlineStr">
-        <is>
-          <t>Needs action-source-card unit scope independent of performer and restriction against targeting the host unit.</t>
-        </is>
-      </c>
+      <c r="G1150" t="inlineStr"/>
       <c r="H1150" t="inlineStr"/>
     </row>
     <row r="1151">
@@ -40288,7 +40104,7 @@
       </c>
       <c r="G1155" t="inlineStr">
         <is>
-          <t>Created copies exist (issue #398: a real copy of the target, marked as created). Still needs a second target (bow one of your unbowed Personalities, copy another), the Item removing itself from the game as a cost, a lock "will not straighten, attack, or defend until after your next turn begins" on the second target, and removing the copy after your next turn begins (a created card removed at the start of its owner's next turn is not built). Rulings needed from Mendon: who controls the copy, where it enters, and how "ignoring costs and restrictions" treats a Unique target.</t>
+          <t>The Egg of P'an Ku - exp (awaiting a ruling from Mendon): the build pieces are merged. P22's CopyOfTarget with CreatedRemoval.NextTurnBegins removes the copy after the creator's next turn begins, and "will not straighten, attack, or defend until after your next turn begins" is a straighten hold plus P11 NoAttack/NoDefend with P4's owner-turn duration (docs/decisions/2026-10-06-690-p22-created-copies-grants.md lists this card); the second target is an ordinary slot. What is still open is Mendon's ruling: who controls the copy, where it enters, and how "ignoring costs and restrictions" treats a Unique target. Not wired; no missing engine primitive is known, but the pieces have not been exercised together.</t>
         </is>
       </c>
       <c r="H1155" t="inlineStr">
@@ -41136,11 +40952,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1180" t="inlineStr">
-        <is>
-          <t>Wyrmbone Katana: its second Battle ability 'Move this Personality to the current battlefield if he assigned there' needs a ruling: whether 'assigned there' means he was assigned to the battlefield earlier this phase and has since moved away (IvoryAssignedBattlefields) or is already at it, as the Charge Into Danger / Keep of the Dead reading has it, which would leave the move a no-op. The first ability is not wired alone.</t>
-        </is>
-      </c>
+      <c r="G1180" t="inlineStr"/>
       <c r="H1180" t="inlineStr"/>
     </row>
     <row r="1181">
@@ -41994,11 +41806,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1205" t="inlineStr">
-        <is>
-          <t>Constructing the Self (Spell, issue #677): its created card now has a published proxy (Minor Illusion, oracle-l5r-11341, a 0F Illusion - Nonhuman - Cavalry - Shugenja Personality whose Chi and Personal Honor are printed "*"), and the two values could be written on the created card as it is made (as The Wind's Champion's Force is, CreatedProxies677.cs). What is missing is its last sentence, "After the next time this game this Spell straightens or leaves play, remove the Illusion from the game": a standing watch that ties one created card to one Spell and fires when that Spell is straightened by anything (the Straighten Phase, an effect) or leaves play by any path. Straighten() and the leaving-play paths have no feature hook, and nothing records which Illusion a Spell made. "This Spell may remain bowed" is the engine's optional straightening (the choose-straighten effect), which exists. Question for Mendon: are the Illusion's Chi and Personal Honor fixed when it is created, or do they follow the Shugenja's as his change (the proxy prints "are equal to the Chi and Personal Honor of the caster")?</t>
-        </is>
-      </c>
+      <c r="G1205" t="inlineStr"/>
       <c r="H1205" t="inlineStr"/>
     </row>
     <row r="1206">
@@ -43222,11 +43030,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1241" t="inlineStr">
-        <is>
-          <t>Needs a keyword-conditional cost EXEMPTION (bow the performer unless it has a given keyword) -- distinct from every existing keyword-conditional EFFECT.</t>
-        </is>
-      </c>
+      <c r="G1241" t="inlineStr"/>
       <c r="H1241" t="inlineStr"/>
     </row>
     <row r="1242">
@@ -47586,7 +47390,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1369" t="inlineStr"/>
+      <c r="G1369" t="inlineStr">
+        <is>
+          <t>Begone, Fool! (Strategy): multiplayer-only, and excluded from the wirable-card wave plan (#742, docs/decisions/2026-10-07-wirable-card-wave-plan.md) by Mendon. It targets an allying Personality, and the engine has no allies and only two players. Not published as a two-player no-op; revisit only if multiplayer is built.</t>
+        </is>
+      </c>
       <c r="H1369" t="inlineStr"/>
     </row>
     <row r="1370">
@@ -47928,12 +47736,12 @@
       </c>
       <c r="G1379" t="inlineStr">
         <is>
-          <t>Bonds of Hospitality (Strategy, issue #736): "Limited: Target a bowed Personality: Put this card into play. While this card remains in play, negate the target's straightening, and his controller has the ability, 'Open: Pay 4 Gold: Discard a Bonds of Hospitality.'" Needs a card in play bound to its target (the Strategy sits in play tied to one Personality), a straighten bar that lasts while that card does (StraightenHolds are timed, not bound to a card), and a player-level granted ability that costs Gold and discards any copy (P4's granted abilities have a turn duration only).</t>
+          <t>Bonds of Hospitality (Strategy, issue #736): "Limited: Target a bowed Personality: Put this card into play. While this card remains in play, negate the target's straightening, and his controller has the ability, 'Open: Pay 4 Gold: Discard a Bonds of Hospitality.'" Wirable now on merged pieces; the gaps first noted are closed. A straighten bar that lasts while a card is in play is StraightenHold.WhileInPlay (StraightenHolds.cs names this card). The player-level ability is P4's GrantPlayerAbility(..., whileInPlay: the card's id) (docs/decisions/2026-10-06-690-p4-turn-boundary.md lists this card), and a PlayerAbility that costs Gold and discards a card by title is the Fortress of Lidless Eyes shape (fortress-lidless-destroy). A Strategy that stays in play exists (the Kata, Economic Repercussions, The Bite of Winter). The pieces have not been exercised together for this card, so build and test them as a unit.</t>
         </is>
       </c>
       <c r="H1379" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>WIRE</t>
         </is>
       </c>
     </row>
@@ -48478,11 +48286,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1395" t="inlineStr">
-        <is>
-          <t>The multi-target slots exist (issue #336: one or two target opposed Personalities); still needs the count of different Clan alignments at the battlefield; not yet wired.</t>
-        </is>
-      </c>
+      <c r="G1395" t="inlineStr"/>
       <c r="H1395" t="inlineStr"/>
     </row>
     <row r="1396">
@@ -49502,11 +49306,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1425" t="inlineStr">
-        <is>
-          <t>Not blocked since issue #336: one to three of your target defending Personalities, +2F -- a Min 1 / Max 3 slot; not yet wired.</t>
-        </is>
-      </c>
+      <c r="G1425" t="inlineStr"/>
       <c r="H1425" t="inlineStr"/>
     </row>
     <row r="1426">
@@ -52474,7 +52274,7 @@
       </c>
       <c r="G1512" t="inlineStr">
         <is>
-          <t>Green Nightshade Blend: needs a new multi-select token-transfer decision (choose direction and any subset of tokens) with its own client contract; MoveToken exists, but no chooser for several tokens or a direction.</t>
+          <t>REJECTED BY MENDON (2026-10-05) for complexity: Green Nightshade Blend (transfer any tokens between two Personalities, then destroy each that now holds a Fire, Poison and Sake token) is not to be wired.</t>
         </is>
       </c>
       <c r="H1512" t="inlineStr">
@@ -52616,11 +52416,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1516" t="inlineStr">
-        <is>
-          <t>Needs a movement-negation passive for a Terrain (the Terrain-play and additional-Battle-action halves are separately wirable).</t>
-        </is>
-      </c>
+      <c r="G1516" t="inlineStr"/>
       <c r="H1516" t="inlineStr"/>
     </row>
     <row r="1517">
@@ -53472,7 +53268,7 @@
       </c>
       <c r="G1541" t="inlineStr">
         <is>
-          <t>Imperial Deployment (Strategy, issue #737): "Open: Choose your performing Personality: The Empress dispatches him to the Colonies. Negate other players' cards' effects that prevent him assigning. After the next time this turn an attack is declared, straighten his unit." Two gaps: no P12 immunity kind covers an effect that prevents a Personality from being assigned (Prevention covers performing actions only; the assignment bars are P11 restrictions and the Attacker's own flags), and P6 has no fact for "an attack is declared" (its facts are per-Personality assignments, not the declaration). Needs an assignment-prevention immunity and a declared-attack fact before it is built; "dispatches him to the Colonies" is flavor text with no rule.</t>
+          <t>Imperial Deployment (Strategy, issue #737): "Open: Choose your performing Personality: The Empress dispatches him to the Colonies. Negate other players' cards' effects that prevent him assigning. After the next time this turn an attack is declared, straighten his unit." Two gaps, the first narrower than first noted. (1) P12's Prevention immunity reads movement locks, which also refuse assigning (MovementLocked and MovementKinds.Assign, MovementLocks.cs; docs/decisions/2026-10-06-p12-immunities.md), so a lock made by another player's card with a known source player is covered. Locks with no source player (Too Close to Home, The Perfect Moment) and P11's stored NoAttack/NoDefend restrictions (no source player) are not, so whether that is enough is a reading. (2) "After the next time this turn an attack is declared, straighten his unit": P6's nearest fact is AssignedToAttack, per Personality (AfterFacts.cs), not the declaration of an attack, and there is no one-shot next-time-this-turn watch on a fact; the reading (declaration or first assignment) needs Mendon. "Dispatches him to the Colonies" is flavor text with no rule.</t>
         </is>
       </c>
       <c r="H1541" t="inlineStr">
@@ -53852,11 +53648,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1552" t="inlineStr">
-        <is>
-          <t>Inexorable (Embers of War): "Reaction: After another player announces a Reaction during the Combat Segment: Its effects will not negate other effects." Re-checked after issue #503. The trigger is now reachable (group P3 built announce windows that ask more than one watcher per announcement, EmperorP3Priority.cs, and the window could be opened for the OTHER player's hand Strategy when the announced action is a Reaction in a Combat Segment), but the effect is not: "its effects will not negate other effects" needs one engine-wide notion of 'a negation made by this action's effects' that can be switched off for one resolving action. Negations live in a dozen unrelated places -- MatchState.NegatedEffects (per card and kind), the whole-action flags (DeferredActionNegated, PendingAttack.Negated, AnnouncedActionNegated, RemANegatesHeldAction, HeldProclaim.Negated, the P3 Event negation), standing card fields that negate later effects (StraightenHolds, MovementLocks, TargetShield, ForceModifiersNegatedTurn, Stalwart-style per-turn stamps), the R4 Honor marks (RemC.NegateLossesActionKey, HonorReducedActionKey, P3 NegatedHonorGains), Fujita's Follower shields and the delay store's negated entries -- and no action records which of them it set. A snapshot-and-revert of a hand-picked list would silently miss the rest, so the card would be partial. Needs: a single NegationLedger that every negation writes through (kind, target, source action key), so an action marked 'non-negating' (Inexorable) has its entries dropped as it resolves; then Inexorable is an announce-window Reaction of the other player that marks the announced Reaction's key.</t>
-        </is>
-      </c>
+      <c r="G1552" t="inlineStr"/>
       <c r="H1552" t="inlineStr"/>
     </row>
     <row r="1553">
@@ -53958,11 +53750,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1555" t="inlineStr">
-        <is>
-          <t>Its Follower may come from your hand OR a discard pile, paying 1 less Gold. The attach-from-a-discard-pile primitive (issue #337) covers the discard half (AttachCost(-1, 0)); a hand-or-discard pile choice (AttachPile has discard values only) is the piece left.</t>
-        </is>
-      </c>
+      <c r="G1555" t="inlineStr"/>
       <c r="H1555" t="inlineStr"/>
     </row>
     <row r="1556">
@@ -54812,11 +54600,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1580" t="inlineStr">
-        <is>
-          <t>Needs a self-replacing Terrain variant plus an ongoing army-wide Force passive tied to being in play as Terrain (same two gaps as oracle-l5r-10941).</t>
-        </is>
-      </c>
+      <c r="G1580" t="inlineStr"/>
       <c r="H1580" t="inlineStr"/>
     </row>
     <row r="1581">
@@ -54850,11 +54634,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1581" t="inlineStr">
-        <is>
-          <t>Needs a unit-Force-total comparison Target (same gap as oracle-l5r-2900/4118).</t>
-        </is>
-      </c>
+      <c r="G1581" t="inlineStr"/>
       <c r="H1581" t="inlineStr"/>
     </row>
     <row r="1582">
@@ -55024,11 +54804,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1586" t="inlineStr">
-        <is>
-          <t>Lying in Ambush: needs a per-action record of Personalities created (a new fact in ActionEffectTracking fed from CreatedCardEntry), a shared-record change beyond a one-line term; also open: whether Political/Iaijutsu Limited actions count and what happens when one action creates several Personalities.</t>
-        </is>
-      </c>
+      <c r="G1586" t="inlineStr"/>
       <c r="H1586" t="inlineStr"/>
     </row>
     <row r="1587">
@@ -55818,11 +55594,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1609" t="inlineStr">
-        <is>
-          <t>Near Miss: its second Reaction ('When paying for an attachment: Produce 2 Gold') needs a Strategy in hand to act as an alternate Gold source; payment sources are limited to cards in Home/Stronghold/Battlefield (GoldQuotes), and no hand-card Gold source is modelled. The first Reaction alone is not wired, since half the card would be silently dropped.</t>
-        </is>
-      </c>
+      <c r="G1609" t="inlineStr"/>
       <c r="H1609" t="inlineStr"/>
     </row>
     <row r="1610">
@@ -56264,11 +56036,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1622" t="inlineStr">
-        <is>
-          <t>Needs a dual-target selection with a relational constraint ("not sharing a Clan alignment"). The multi-target shape (issue #336) makes the two targets independent slots, each judged on its own; a constraint BETWEEN the two chosen targets is still not expressible.</t>
-        </is>
-      </c>
+      <c r="G1622" t="inlineStr"/>
       <c r="H1622" t="inlineStr"/>
     </row>
     <row r="1623">
@@ -57052,7 +56820,7 @@
       </c>
       <c r="G1645" t="inlineStr">
         <is>
-          <t>Needs a "count copies of this same card played this battle" mechanism (novel; the additional-Battle-action half is separately wirable).</t>
+          <t>Pierce the Tapestery (awaiting a ruling from Mendon on the seven-copy deck rule and the per-battle count): the mechanisms are merged. "Up to seven copies" is CardDefinition.DeckCopyLimit (issue #337, DeckWorkshop CopyLimit), "two or more other Pierce the Tapestry played this battle" is a P7 period counter (AddPeriodCount / PeriodCountOf with Period.Battle, PeriodWatches.cs; this card is its design example), and "an additional Battle action to play a Pierce the Tapestry" is P17's additional-action scope (AdditionalActionScope.cs). Not wired.</t>
         </is>
       </c>
       <c r="H1645" t="inlineStr"/>
@@ -57526,7 +57294,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1659" t="inlineStr"/>
+      <c r="G1659" t="inlineStr">
+        <is>
+          <t>Prideful Allies (Strategy): multiplayer-only, and excluded from the wirable-card wave plan (#742, docs/decisions/2026-10-07-wirable-card-wave-plan.md) by Mendon. It targets an allying unit, and the engine has no allies and only two players. Not published as a two-player no-op; revisit only if multiplayer is built.</t>
+        </is>
+      </c>
       <c r="H1659" t="inlineStr"/>
     </row>
     <row r="1660">
@@ -61232,11 +61004,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1768" t="inlineStr">
-        <is>
-          <t>The multi-target slots exist (issue #336: one to three Personalities controlled by other players) and the command keeps the order they were chosen in, which is what its -1F, -2F, -3F assignment reads; not yet wired.</t>
-        </is>
-      </c>
+      <c r="G1768" t="inlineStr"/>
       <c r="H1768" t="inlineStr"/>
     </row>
     <row r="1769">
@@ -62324,11 +62092,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1800" t="inlineStr">
-        <is>
-          <t>Refreshed: the "delayed post-destruction straighten" is a delayed effect of a card that is no longer in play, which the store negates by rule (a card that left play has nothing to be affected); it needs a straighten of another card triggered by this card's destruction, plus the self-replacing Terrain variant (unchanged). NO LOCAL SCAN.</t>
-        </is>
-      </c>
+      <c r="G1800" t="inlineStr"/>
       <c r="H1800" t="inlineStr"/>
     </row>
     <row r="1801">
@@ -62948,11 +62712,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1818" t="inlineStr">
-        <is>
-          <t>Needs a "Political" Reaction timing (not built; the plain Ranged 1 Attack half is separately wirable).</t>
-        </is>
-      </c>
+      <c r="G1818" t="inlineStr"/>
       <c r="H1818" t="inlineStr"/>
     </row>
     <row r="1819">
@@ -63870,11 +63630,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1845" t="inlineStr">
-        <is>
-          <t>Needs a unit-Force-total comparison Target (same gap as oracle-l5r-2900).</t>
-        </is>
-      </c>
+      <c r="G1845" t="inlineStr"/>
       <c r="H1845" t="inlineStr"/>
     </row>
     <row r="1846">
@@ -64180,11 +63936,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1854" t="inlineStr">
-        <is>
-          <t>Needs P1 (a turn-long production adjustment on every non-Unique Holding) with the once-per-turn copy limit; not wired in #689.</t>
-        </is>
-      </c>
+      <c r="G1854" t="inlineStr"/>
       <c r="H1854" t="inlineStr"/>
     </row>
     <row r="1855">
@@ -64626,7 +64378,11 @@
           <t>Unwired</t>
         </is>
       </c>
-      <c r="G1867" t="inlineStr"/>
+      <c r="G1867" t="inlineStr">
+        <is>
+          <t>Unbearable Weight (Strategy; one of the 13 cards awaiting a ruling from Mendon): "If this destroyed the target, his controller puts this Strategy in his hand" puts a played Strategy into the other player's hand; whose card it is afterwards and which discard pile it goes to when he plays it is unruled. Naoharu's Gift (EmperorRemainingFEvents.cs, naoharu-take) is a precedent for a card resting in another player's hand (ownership moves, OriginalOwnerId returns it to its owner's pile when it leaves), but it is Event-only code. Also unruled: "a Fate deck" (any player's, or the performer's own). Discarding the top card of a Fate deck and using its Focus Value are merged (aberrations-boost, fires-of-turmoil). Not wired.</t>
+        </is>
+      </c>
       <c r="H1867" t="inlineStr"/>
     </row>
     <row r="1868">
@@ -65714,11 +65470,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1899" t="inlineStr">
-        <is>
-          <t>Wanted for Questioning (issue #503, P6, re-checked against its scan): 'Battle: Choose your performing unbowed Magistrate and target an enemy Personality: Your Magistrate takes him into custody. If he is dishonorable, destroy his attachments. Move him home.' 'Custody' is still undefined: docs/rules/EMPEROR_EDITION_CORE_RULES.md has no entry for it (grep finds none) and the engine has no custody state. Rules-lane question for Mendon: is 'takes him into custody' flavour (then the card is buildable at once: an unbowed-Magistrate performer at the battle, an enemy-personality target, destroy his attachments if dishonorable, MoveHome), or a mechanic (what it does, how long it lasts, how it ends)?</t>
-        </is>
-      </c>
+      <c r="G1899" t="inlineStr"/>
       <c r="H1899" t="inlineStr"/>
     </row>
     <row r="1900">
@@ -65754,7 +65506,7 @@
       </c>
       <c r="G1900" t="inlineStr">
         <is>
-          <t>Warded Premises: "Negate all Force bonuses from actions to cards at this battlefield" needs the engine to tell an action's Force modifier from a token, an Item, a Permanent modifier ("Permanently give him +2F") and a static term, and a ruling on whether a permanent bonus is negated for good. Its second ability (put this Terrain into play at a battlefield with no Terrain, even without a unit there) is wireable.</t>
+          <t>Warded Premises (Strategy): "Before this battle's resolution: Negate all Force bonuses from actions to cards at this battlefield." Part of the first gap is closed: Creating Order's NegateActionForceModifiers and ActionForceModifierNegated (ForgottenLegacyBatch3.cs) already tell a Force modifier given by an action (a Modifier whose Effect is an action ability) from a trait's standing modifier, and leave tokens alone, and the Terrain's before-resolution timing exists (BeforeResolution.cs). What remains: a bonuses-only variant applied to every card at a battlefield (the existing helper negates penalties too and covers one card for the rest of the turn), and a ruling from Mendon on whether a Permanent bonus ("Permanently give him +2F") is negated for good or only suspended and whether Item and token bonuses count. Its second ability (put this Terrain into play at a battlefield with no Terrain, even without a unit there) is wireable.</t>
         </is>
       </c>
       <c r="H1900" t="inlineStr">
@@ -67158,11 +66910,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1941" t="inlineStr">
-        <is>
-          <t>Ever-Winter Copse (Holding, issue #653): "When another Holding produces Gold to pay for a Nonhuman, bow this card: Produce 1 Gold" is a payment source whose availability depends on which OTHER producers the payer has chosen for the same payment, and which bows its own card. The payment tokens (EmperorMechE.cs PaymentTokens/UsePaymentTokens) are computed for a payment before any source is chosen, their use never bows their card, and there is no extension point for a condition on the chosen set of sources or for a token kind that bows; adding either means editing the shared payment code, not a feature file.</t>
-        </is>
-      </c>
+      <c r="G1941" t="inlineStr"/>
       <c r="H1941" t="inlineStr"/>
     </row>
     <row r="1942">
@@ -67876,11 +67624,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1962" t="inlineStr">
-        <is>
-          <t>Hidden Weapons (Holding, issue #653): "Limited: Put a Weapon in your hand under this Holding (face-down)" and "You may Equip Weapons from under this Holding as a Battle/Limited action" need a zone of cards under a particular Holding that is hidden from the other player. The only under-card zone (Zone.Underneath) is face-up, public and kept under the Stronghold, not per card, and its view projection shows every card in it; hiding a face-down card and equipping from it with the Equip action's own pricing needs a new hidden zone and its projection.</t>
-        </is>
-      </c>
+      <c r="G1962" t="inlineStr"/>
       <c r="H1962" t="inlineStr"/>
     </row>
     <row r="1963">
@@ -67948,11 +67692,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1964" t="inlineStr">
-        <is>
-          <t>Humble Farm (issue #503, P6, re-checked): its own scan is local; blocked only by its created plain 2F Ashigaru Follower. No local Proxy fits (Fledgling Ashigaru is 0F, Mounted Ashigaru 1F Cavalry with no local scan, Ronin Follower 2F Ronin, Infantry Follower 2F with no keyword); docs/requests/created-card-scans-needed.md row B3 (ashigaru-2f.jpg) is unticked. Otherwise GoldProduction 2 plus Ashigaru Recruits' Battle/Open create-and-attach with a Sacrifice cost.</t>
-        </is>
-      </c>
+      <c r="G1964" t="inlineStr"/>
       <c r="H1964" t="inlineStr"/>
     </row>
     <row r="1965">
@@ -68360,11 +68100,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1976" t="inlineStr">
-        <is>
-          <t>Magistrate's Stipend: its Reaction needs a new announce trigger for non-Iaijutsu actions with a Magistrate performer and a new '+1C until the action ends' stat modifier cleared at action end, neither of which exists; also unruled whether a Reaction counts as an announced non-Iaijutsu action and whether it has any per-use limit.</t>
-        </is>
-      </c>
+      <c r="G1976" t="inlineStr"/>
       <c r="H1976" t="inlineStr"/>
     </row>
     <row r="1977">
@@ -68632,11 +68368,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1984" t="inlineStr">
-        <is>
-          <t>Oracle of the Void - exp (Holding, issue #653): "Limited, Bow: The next two cards in provinces you refill (this turn) may be refilled face-up" is an optional face-up refill for each of the next two refills, whichever effect causes them (a purchase, a discard, a Region). Refills happen at many call sites (Purchase, Refill, RefillProvinceSlot and the effects that discard a province card) and there is no single refill hook or per-refill decision; a watch on future refills needs one, which is shared province plumbing. The rest ("Negate this card's destruction", Limited bow draw a card) would be buildable.</t>
-        </is>
-      </c>
+      <c r="G1984" t="inlineStr"/>
       <c r="H1984" t="inlineStr"/>
     </row>
     <row r="1985">
@@ -69518,7 +69250,7 @@
       </c>
       <c r="G2010" t="inlineStr">
         <is>
-          <t>Shrine to the Heavens: a Celestial-reveal choice must precede ResolveCelestial's discard of the player's other Celestials, but ResolveCelestial returns void and has no pending-choice path (a shared-interface change). Open readings: whether 'one of your Celestials in play' may be the newly revealed one, what happens with a third Celestial, and whether two Celestials persist if the Shrine leaves play; ControlsCelestialEffect and similar code assume at most one.</t>
+          <t>Shrine to the Heavens (awaiting a ruling from Mendon): the old gap, a Celestial-reveal choice before the discard of the other Celestials, is closed: P6 (AfterFacts.cs, CelestialEntryRegistry) opens a choice when a Celestial enters play, with SparesFromDiscard so a chosen Celestial is not discarded and the discard of the others waits for the answer (this card is its design example). Still open: whether "one of your Celestials in play" may be the newly revealed one, what happens with a third Celestial, and whether two Celestials persist if the Shrine leaves play; ControlsCelestialEffect and similar code assume at most one Celestial. Not wired.</t>
         </is>
       </c>
       <c r="H2010" t="inlineStr"/>
@@ -70374,11 +70106,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G2035" t="inlineStr">
-        <is>
-          <t>The Amethyst Court (Holding, issue #653): its second line, "Bow: Bow your target unbowed Courtier or Artisan. Produce Gold equal to his Chi", is a Gold source of its own that names a Personality as it is used (the amount is that Personality's Chi, and bowing him is part of the production). The payment tokens offer a source per candidate only for Zlkyt's destroyed Holding and Moto Rani's removed dead Personality; UsePaymentTokens switches on a closed set of token kinds and has no extension point for a source that bows a chosen Personality, so the production cannot be added from a feature file.</t>
-        </is>
-      </c>
+      <c r="G2035" t="inlineStr"/>
       <c r="H2035" t="inlineStr"/>
     </row>
     <row r="2036">
@@ -70990,11 +70718,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G2053" t="inlineStr">
-        <is>
-          <t>The Tower of Vigilance (Holding, issue #677): its created card now has a published proxy (Tower Guard, oracle-l5r-11345, a 0F/2C/2PH Guard - Samurai Personality), and creating a Personality at the current battlefield until the battle ends is built. The card itself is a Fortification ("Fortifications attach, straightened, to the Province from which they entered play"), and no Fortification is built: a Holding has no province it is attached to, so "If you have any units at this battlefield ... create ... there" has no battlefield to read, and the Holding does not leave play with its Province.</t>
-        </is>
-      </c>
+      <c r="G2053" t="inlineStr"/>
       <c r="H2053" t="inlineStr"/>
     </row>
     <row r="2054">
@@ -72628,12 +72352,12 @@
       </c>
       <c r="G2101" t="inlineStr">
         <is>
-          <t>Marriage of the Emerald Champion (Event, issue #733): "Limited: Put this Event into play. Target your Personality. While this Event remains in play, he will not be dishonored and you will not lose Honor from other players' actions that have targeted him. After your second turn from now begins, discard this Event." The pieces exist (KeepEventInPlay with turnBeginsIn 2, a P11 dishonor bar, a P14 no-loss filter targeted-by-other), but the target is chosen when the Event is revealed and the Event then leaves its province for play, and the Event decision machinery that answers a custom choice (ResolveEventChoiceCommand's default arm) is wired only for P5's Events that stay in their province. A new kind needs one hook in that arm and a record binding the Event to its target; a shared-interface change in the Events Phase.</t>
+          <t>Marriage of the Emerald Champion (Event, issue #733): "Limited: Put this Event into play. Target your Personality. While this Event remains in play, he will not be dishonored and you will not lose Honor from other players' actions that have targeted him. After your second turn from now begins, discard this Event." Wirable now on merged pieces: KeepEventInPlay with turnBeginsIn 2, a P11 dishonor bar and a P14 targeted-by-other filter. The binding the first note thought missing exists: an Event that chooses its target at reveal and stays in play is built for Delayed Arrival (a PendingEventChoice answered in ResolveEventChoiceCommand, the target kept in EventTargets, FinishRevealedEvent with keep and turnBeginsIn), and later waves add their Event answers with one hook line in that method's default arm (ResolveWave738EventChoice, ResolveP5EventChoice). This card needs the same one hook and its own record, not a new shared mechanism. The pieces have not been exercised together.</t>
         </is>
       </c>
       <c r="H2101" t="inlineStr">
         <is>
-          <t>TARGET</t>
+          <t>WIRE</t>
         </is>
       </c>
     </row>
@@ -72670,7 +72394,7 @@
       </c>
       <c r="G2102" t="inlineStr">
         <is>
-          <t>Minor Blackmail: needs a ruling on whether 'an action that he performed' means only the performer slot or his own card's abilities, and whether 'his unit is assigned' includes defender assignment (also a game-long watch that survives his leaving play or changing controller).</t>
+          <t>Minor Blackmail (awaiting a ruling from Mendon): the reveal-time window ("after you reveal cards in your Provinces at the start of your turn, if this Event is face-up") is P5's province-reveal Events, and P6 has an AssignedToAttack fact, but that fact covers an attacker's assignment only (no defender-assignment fact), and nothing is a game-long watch on "an action that he performed" that survives him leaving play or changing controller. Rulings needed: whether "an action that he performed" means only the performer slot or his own card's abilities, and whether "his unit is assigned" includes defender assignment. Not wired.</t>
         </is>
       </c>
       <c r="H2102" t="inlineStr"/>
@@ -72876,11 +72600,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G2108" t="inlineStr">
-        <is>
-          <t>Open Recruitment: needs a generic 'after a Personality turns face-up in one of your provinces' trigger; face-up flips are scattered across the start-of-turn reveal and effect-driven sites, none of which publishes an event, and the order of the Event's reveal against the other provinces' reveals is unruled. Also, Keyword 'Unaligned' ignores alignment granted by an 'X Clan' keyword.</t>
-        </is>
-      </c>
+      <c r="G2108" t="inlineStr"/>
       <c r="H2108" t="inlineStr"/>
     </row>
     <row r="2109">
@@ -73086,7 +72806,7 @@
       </c>
       <c r="G2114" t="inlineStr">
         <is>
-          <t>Revelations (Event, issue #738): "Show the top five cards of your Dynasty deck. Choose another player who may discard one of the cards. Put the rest back in any order. Refill this province face-up." The scan prints no "After you reveal" clause, so it is an ordinary Event that resolves when revealed, but its three steps are not covered by what is merged: P20's "other player chooses" belongs to a deck search (a set of picked cards), not to a look at the top of a deck; the look (DeckLook.cs) lets its own player rearrange but has no step in which another player discards one of the shown cards before the rest go back; and the Event's own province must then refill face up from the reordered deck. It needs a look disposition with an other-player discard and a reorder, which is decision-UI work for batch 8 (#739), not a card-level guess.</t>
+          <t>Revelations (Event, issue #738): "Show the top five cards of your Dynasty deck. Choose another player who may discard one of the cards. Put the rest back in any order. Refill this province face-up." The scan prints no "After you reveal" clause, so it is an ordinary Event that resolves when revealed. Its three steps are still not composed from what is merged: P25's shown choice (PendingShownChoice, used by Dark Audience) lets another player pick among shown cards but hangs off a search, the look (DeckLook.cs) lets its own player rearrange but has no step in which another player discards one of the shown cards before the rest go back, and the Event's own province must then refill face up (RefillSourceProvinceFaceUp is a search disposition). Batch 8 (#739) merged without this card, so no decision work is pending elsewhere; it needs a look disposition with an other-player discard and a reorder.</t>
         </is>
       </c>
       <c r="H2114" t="inlineStr">
@@ -73610,11 +73330,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G2129" t="inlineStr">
-        <is>
-          <t>The Jade Championship (Event). Needs a -1F aura on Shadowlands Followers at a location (FollowerForce has no registry hook) and a mandatory trait that triggers after the resolution of an action from a Spell (no trait-after-action hook exists; AfterActionResolved offers only optional Reactions).</t>
-        </is>
-      </c>
+      <c r="G2129" t="inlineStr"/>
       <c r="H2129" t="inlineStr"/>
     </row>
     <row r="2130">
@@ -74304,7 +74020,7 @@
       </c>
       <c r="G2149" t="inlineStr">
         <is>
-          <t>Benten's Blessing: needs the same missing Celestial entry window to choose zero to two face-up Personalities (ResolveCelestial offers no entry choice), and an unresolved reading of which out-of-play zones count as face-up and whether the +1PH persists when a chosen card changes zone.</t>
+          <t>Benten's Blessing (awaiting a ruling from Mendon): the entry window is merged (P6 CelestialEntryRegistry, used by Natsu-Togumara's Guidance), but it asks for one card per choice, so "zero to two face-up Personalities" needs two queued choices or a multi-pick. The Reaction half (an action that would target your Personality targets your performing Personality instead, discarding the Celestial) is a redirection of the kind built in docs/decisions/2026-09-19-redirection-and-protective-reactions.md, which names this card. Unresolved reading: which out-of-play zones count as face-up, and whether the +1PH persists when a chosen card changes zone. Not wired.</t>
         </is>
       </c>
       <c r="H2149" t="inlineStr"/>
@@ -74994,11 +74710,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G2169" t="inlineStr">
-        <is>
-          <t>Natsu-Togumara's Guidance: its entry half ('After this card enters play: You may choose a Personality') cannot be offered because a Celestial enters play through MatchEngine.ResolveCelestial, which opens no entry-reaction window and no mid-reveal decision; the will-not-bow chain (AfterResolution.ResolutionWillNotBow) would also need a stored chosen Personality.</t>
-        </is>
-      </c>
+      <c r="G2169" t="inlineStr"/>
       <c r="H2169" t="inlineStr"/>
     </row>
     <row r="2170">
@@ -75032,11 +74744,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G2170" t="inlineStr">
-        <is>
-          <t>Needs attack/defend prohibition during movement and entry, not assignment alone.</t>
-        </is>
-      </c>
+      <c r="G2170" t="inlineStr"/>
       <c r="H2170" t="inlineStr"/>
     </row>
     <row r="2171">
@@ -75106,7 +74814,7 @@
       </c>
       <c r="G2172" t="inlineStr">
         <is>
-          <t>Sadahako's Artistry (Celestial, issue #653): the Honor half ("Limited: If your Family Honor is 10 or lower: Gain 1 Honor") is buildable, but the gift ("Discard this card and target a card in your hand: You offer it as a gift. Show it to another player. He may accept, putting it into his hand; if he did, you gain Honor equal to its Focus Value. If he did not, discard it and draw 3 cards") needs a ruling and a primitive. Question for Mendon: once the other player accepts, whose card is it and which discard pile does it go to when he discards or plays it (its owner's or the recipient's); may a card be put into another player's hand at all? The engine has the opponent's Either/Or decision (EitherOr.cs) but no move of a hand card into another player's hand: OwnerId means controller and ReturnCardsOutOfPlayToTheirOwners sends a card back to its owner, so the card cannot rest in the recipient's hand without a new ownership rule.</t>
+          <t>Sadahako's Artistry (Celestial, issue #653): the Honor half ("Limited: If your Family Honor is 10 or lower: Gain 1 Honor") is buildable, but the gift ("Discard this card and target a card in your hand: You offer it as a gift. Show it to another player. He may accept, putting it into his hand; if he did, you gain Honor equal to its Focus Value. If he did not, discard it and draw 3 cards") is not yet an ability. The ownership question has a precedent: Naoharu's Gift (EmperorRemainingFEvents.cs, naoharu-take) moves a hand card into the other player's hand, sets OwnerId to the taker and records OriginalOwnerId so ReturnCardsOutOfPlayToTheirOwners sends it to its owner's pile when it leaves his hand. That is Event-only code, so an ability needs a reusable gift step with the recipient's accept or refuse decision (EitherOr.cs supplies a decider). Question for Mendon: confirm that Naoharu's Gift reading (the card stays the giver's for discard-pile purposes) carries over to this Celestial.</t>
         </is>
       </c>
       <c r="H2172" t="inlineStr">
@@ -75860,11 +75568,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G2194" t="inlineStr">
-        <is>
-          <t>Plains of Otosan Uchi (issue #503, P6, re-checked): still blocked on the two-card province. Every province is one card slot (ProvinceState.CardId): the Events Phase reveal, Purchase and Reserve recruits, Refill (now also the face-up refills of Susaiken / Distant Expansion and Ietsuno's refill trigger, EmperorP6.cs), DestroyProvince, the private province sights and MatchView.ProvinceView all assume one card. Mendon (2026-09-25): a province must be able to hold two Dynasty cards; the view/client second slot is requested from Alfredo in issue #499 (not done: ProvinceView has no second card). The engine side (a second slot's reveal, refill, purchase and destruction, the owner's choice of which slot goes first, 'do not reveal the second card in the Events Phase this card enters play', and the 10-Honor loss before the province is destroyed) should follow once the view lane is agreed, so a published card does not show only half of its province.</t>
-        </is>
-      </c>
+      <c r="G2194" t="inlineStr"/>
       <c r="H2194" t="inlineStr"/>
     </row>
     <row r="2195">
@@ -76306,11 +76010,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G2207" t="inlineStr">
-        <is>
-          <t>Verdant Jungle (Region, issue #653): its Reaction, "Before an action resolves, bow this card: Negate its effects that move any Personalities into an attacking army at this Province's battlefield", negates only the movement part of an announced action by destination. The before-action Reaction window decides which Reactions apply in BeforeActionReactionApplies, a closed switch with no extension hook, and the movement a held action would make is known only per-ability (DeferredActionMovers) with no destination, so "into an attacking army at this battlefield" cannot be asked of an announced action. The first line (nonhuman Personalities enter play from this province for 1 less Gold) would be a small entry discount.</t>
-        </is>
-      </c>
+      <c r="G2207" t="inlineStr"/>
       <c r="H2207" t="inlineStr"/>
     </row>
     <row r="2208">
@@ -76446,11 +76146,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G2211" t="inlineStr">
-        <is>
-          <t>Needs an Interrupt timing (not built) for its own printed action ('Interrupt: Reduce all Honor gains and losses from an action by 2'). Its own recruitment condition ('if your maximum hand size is 10 or more') is no longer blocked -- MaxHandSize (issue #223) already exposes this per player.</t>
-        </is>
-      </c>
+      <c r="G2211" t="inlineStr"/>
       <c r="H2211" t="inlineStr"/>
     </row>
     <row r="2212">
@@ -76518,11 +76214,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G2213" t="inlineStr">
-        <is>
-          <t>The Engage window now exists (issue #310) for its own printed 'Engage, bow: A target Personality at any location will not move this turn' (a Ring, in play, bow cost). Still needs: a 'will not move this turn' restriction (no such durable movement block exists) and its target at any location; its recruitment condition is otherwise wirable.</t>
-        </is>
-      </c>
+      <c r="G2213" t="inlineStr"/>
       <c r="H2213" t="inlineStr"/>
     </row>
     <row r="2214">
@@ -76752,7 +76444,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -76772,7 +76464,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -76832,7 +76524,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -76912,7 +76604,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -77012,7 +76704,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -77032,7 +76724,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -77092,7 +76784,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wire Foothold of the Mad (#766)
Mendon's ruling: counts as 39 Honor for going first, then 0 before the first turn,
silently; Madness tokens are -1F tokens while it is a Stronghold in play. Also wires its
Honor-loss immunity, Fallen discount and two Limited bow abilities; art pack r1.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -511,14 +511,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C5" t="n">
         <v>51</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>96.1%</t>
+          <t>98.0%</t>
         </is>
       </c>
     </row>
@@ -709,14 +709,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2175</v>
+        <v>2176</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>98.1%</t>
+          <t>98.2%</t>
         </is>
       </c>
     </row>
@@ -785,9 +785,6 @@
           <t>Coils of Madness</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>1</v>
-      </c>
       <c r="C20" t="n">
         <v>6</v>
       </c>
@@ -801,7 +798,7 @@
         <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21">
@@ -928,7 +925,7 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" s="2" t="n">
         <v>10</v>
@@ -952,7 +949,7 @@
         <v>3</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1253,7 +1250,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Unwired</t>
+          <t>Wired</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>

</xml_diff>

<commit_message>
Force cap primitive and Asako Kaitoko - exp (#768)
A live maximum-Force rule that lowers and never raises, lapses with its source and is
negated by Force-penalty negations and immunities; Kaitoko wired on it with the
keyword-conditioned target bar. Art pack r1.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -529,14 +529,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="C6" t="n">
         <v>851</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>98.8%</t>
+          <t>98.9%</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2176</v>
+        <v>2177</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
@@ -782,17 +782,23 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Coils of Madness</t>
-        </is>
+          <t>Torn Asunder</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
       </c>
       <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
         <v>6</v>
-      </c>
-      <c r="D20" t="n">
-        <v>3</v>
-      </c>
-      <c r="F20" t="n">
-        <v>2</v>
       </c>
       <c r="H20" t="n">
         <v>1</v>
@@ -804,29 +810,23 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Torn Asunder</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1</v>
+          <t>Coils of Madness</t>
+        </is>
       </c>
       <c r="C21" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" t="n">
         <v>2</v>
-      </c>
-      <c r="D21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" t="n">
-        <v>6</v>
       </c>
       <c r="H21" t="n">
         <v>1</v>
       </c>
       <c r="J21" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22">
@@ -928,7 +928,7 @@
         <v>1</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>6</v>
@@ -949,7 +949,7 @@
         <v>3</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -4816,19 +4816,11 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>Asako Kaitoko - exp (Personality, issue #736): "Personalities with Fallen, Kolat, Ninja, Nonhuman, or Shadowlands opposing Kaitoko have a maximum Force of 3, and actions from cards in their units may not target Kaitoko." Two gaps: a maximum Force is a stat cap and none exists (P9 left StatCap out; PersonalityForce is additive, so a cap cannot be written without reading the Force it caps), and the target bar applies only to actors whose Personality has one of five keywords, which an ActorSpec cannot say.</t>
-        </is>
-      </c>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t>STAT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -76777,7 +76769,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wire Journey's End Keep - exp and the Imperial Clan (#771)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TLyr6J2gRoqayc2nvJTNGy
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -465,7 +465,6 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,14 +510,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C5" t="n">
         <v>51</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>98.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -601,14 +600,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="C10" t="n">
         <v>598</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>97.8%</t>
+          <t>98.0%</t>
         </is>
       </c>
     </row>
@@ -637,14 +636,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C12" t="n">
         <v>81</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>93.8%</t>
+          <t>95.1%</t>
         </is>
       </c>
     </row>
@@ -709,14 +708,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2176</v>
+        <v>2179</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>98.2%</t>
+          <t>98.3%</t>
         </is>
       </c>
     </row>
@@ -735,45 +734,40 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Stronghold</t>
+          <t>Personality</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Personality</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Spell</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Spell</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Strategy</t>
+          <t>Holding</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Holding</t>
+          <t>Event</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Event</t>
+          <t>Celestial</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>Celestial</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -785,19 +779,19 @@
           <t>Coils of Madness</t>
         </is>
       </c>
+      <c r="B20" t="n">
+        <v>6</v>
+      </c>
       <c r="C20" t="n">
-        <v>6</v>
-      </c>
-      <c r="D20" t="n">
         <v>3</v>
       </c>
-      <c r="F20" t="n">
+      <c r="E20" t="n">
         <v>2</v>
       </c>
-      <c r="H20" t="n">
+      <c r="G20" t="n">
         <v>1</v>
       </c>
-      <c r="J20" t="n">
+      <c r="I20" t="n">
         <v>12</v>
       </c>
     </row>
@@ -808,25 +802,22 @@
         </is>
       </c>
       <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="n">
         <v>1</v>
-      </c>
-      <c r="C21" t="n">
-        <v>2</v>
       </c>
       <c r="D21" t="n">
         <v>1</v>
       </c>
       <c r="E21" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" t="n">
         <v>1</v>
       </c>
-      <c r="F21" t="n">
-        <v>6</v>
-      </c>
-      <c r="H21" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" t="n">
-        <v>12</v>
+      <c r="I21" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="22">
@@ -835,19 +826,19 @@
           <t>Promotional–Celestial</t>
         </is>
       </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
       <c r="F22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" t="n">
         <v>1</v>
-      </c>
-      <c r="G22" t="n">
-        <v>2</v>
       </c>
       <c r="H22" t="n">
         <v>1</v>
       </c>
       <c r="I22" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" t="n">
         <v>5</v>
       </c>
     </row>
@@ -857,19 +848,19 @@
           <t>Promotional–Emperor</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="C23" t="n">
         <v>1</v>
       </c>
-      <c r="F23" t="n">
+      <c r="E23" t="n">
         <v>1</v>
       </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
       <c r="H23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>2</v>
-      </c>
-      <c r="J23" t="n">
         <v>5</v>
       </c>
     </row>
@@ -879,17 +870,14 @@
           <t>Aftermath</t>
         </is>
       </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
       <c r="C24" t="n">
-        <v>2</v>
-      </c>
-      <c r="D24" t="n">
         <v>1</v>
       </c>
-      <c r="H24" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" t="n">
-        <v>4</v>
+      <c r="I24" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -898,10 +886,10 @@
           <t>War of Honor</t>
         </is>
       </c>
-      <c r="F25" t="n">
+      <c r="E25" t="n">
         <v>2</v>
       </c>
-      <c r="J25" t="n">
+      <c r="I25" t="n">
         <v>2</v>
       </c>
     </row>
@@ -911,10 +899,10 @@
           <t>Gates of Chaos</t>
         </is>
       </c>
-      <c r="F26" t="n">
+      <c r="E26" t="n">
         <v>1</v>
       </c>
-      <c r="J26" t="n">
+      <c r="I26" t="n">
         <v>1</v>
       </c>
     </row>
@@ -925,31 +913,28 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C27" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="D27" s="2" t="n">
-        <v>6</v>
-      </c>
       <c r="E27" s="2" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J27" s="2" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1420,14 +1405,10 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Journey's End Keep - exp (Stronghold; one of the 13 cards awaiting a ruling from Mendon): the Gold lock ("when this Stronghold produces Gold, you may not Recruit Personalities until the phase ends or until after you have spent 5 total Gold for non-Recruit costs or payments") is buildable on merged pieces: the P1 per-phase ledger (GoldSpentThisPhaseExceptRecruit, PaymentHooks695.cs) and the P3 recruit gate (RecruitGates695.cs). Still open: (1) "'Imperial' is a Clan Alignment, and it is your Clan Alignment" (how an Imperial player's alignment interacts with Clan Allegiance, Loyal and the Clan discount is unruled; ClanEntryDiscount reads the stronghold's Clan); (2) "if no other player has an Imperial Stronghold, you begin the game with the Imperial Favor" has no setup hook; (3) the no-Clan-discount trait only matters under the optional Clan Discount rule. Not wired.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -22011,12 +21992,12 @@
       </c>
       <c r="G620" t="inlineStr">
         <is>
-          <t>P'an Ku - exp (Personality, issue #736): "Open, bow: Give a target card a Madness token" is built (the existing panku-madness shape). "Limited, bow: P'an Ku may remain bowed. Take control of a target Personality with more Madness tokens than printed Personal Honor and remove those tokens. The target will not commit seppuku until P'an Ku straightens or leaves play. After P'an Ku does, give control of the target to his owner." Most of this is merged: the timed return of control is P24's ReturnControlWhenSourceStraightens (ControlReturnTriggers.SourceStraightens, EffectPrimitivesTokens.cs, built for this card: docs/decisions/2026-10-06-690-p24-effect-primitives.md section 8), and "may remain bowed" is the existing choose-straighten Effect (Constructing the Self uses it in batch 10). The remaining gap is the seppuku bar: no P11 restriction kind bars seppuku, and P5's SeppukuBar (EmperorP5Zones.cs) lasts one turn, so "will not commit seppuku until P'an Ku straightens or leaves play" needs a bar bound to a source card. His Effect slot must also carry choose-straighten alongside his other abilities.</t>
+          <t>P'an Ku - exp (Personality, issue #736): "Open, bow: Give a target card a Madness token" is built (the existing panku-madness shape), but "Limited, bow: P'an Ku may remain bowed. Take control of a target Personality with more Madness tokens than printed Personal Honor and remove those tokens. The target will not commit seppuku until P'an Ku straightens or leaves play. After P'an Ku does, give control of the target to his owner." needs three things together: a control change that returns when a named card straightens or leaves play (TakeControl exists; the timed return trigger does not), a seppuku bar tied to that card, and "may remain bowed" (a rule exempting him from straightening). One card, three new rules.</t>
         </is>
       </c>
       <c r="H620" t="inlineStr">
         <is>
-          <t>SMALL</t>
+          <t>CONTROL</t>
         </is>
       </c>
     </row>
@@ -38275,12 +38256,12 @@
       </c>
       <c r="G1102" t="inlineStr">
         <is>
-          <t>Koan's Jingasa (Item, issue #736): "This Personality has Shugenja, may not have more Spells than Koan cards attached, and he need not bow for his Spells with an odd Focus Value (0 is even)." The Shugenja keyword is AttachGrantsKeyword, and the bow waiver is merged: P24's EngineHooks.CostWaivers with SpellFocusParityWaives (EffectPrimitivesCosts.cs) is written for this card and Koan's Robes, and a wave registers the callback with the Item's Effect. What is still missing is the attachment limit: P11's SpellLimit counts Spell actions performed, not Spells attached, and NoAttach bars by type or keyword without counting, so "may not have more Spells than Koan cards attached" (a count of Koan cards on the host against his attached Spells) needs a new attach rule.</t>
+          <t>Koan's Jingasa (Item, issue #736): "This Personality has Shugenja, may not have more Spells than Koan cards attached, and he need not bow for his Spells with an odd Focus Value (0 is even)." The Shugenja keyword is AttachGrantsKeyword, but P11's SpellLimit counts Spell actions performed, not Spells attached (the rule here is an attachment limit counted against Koan cards), and "need not bow for his Spells" is a waiver of the bow cost of a Spell's own ability, which P24's cost waivers do not cover.</t>
         </is>
       </c>
       <c r="H1102" t="inlineStr">
         <is>
-          <t>SMALL</t>
+          <t>COST</t>
         </is>
       </c>
     </row>
@@ -47724,19 +47705,11 @@
       </c>
       <c r="F1379" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1379" t="inlineStr">
-        <is>
-          <t>Bonds of Hospitality (Strategy, issue #736): "Limited: Target a bowed Personality: Put this card into play. While this card remains in play, negate the target's straightening, and his controller has the ability, 'Open: Pay 4 Gold: Discard a Bonds of Hospitality.'" Wirable now on merged pieces; the gaps first noted are closed. A straighten bar that lasts while a card is in play is StraightenHold.WhileInPlay (StraightenHolds.cs names this card). The player-level ability is P4's GrantPlayerAbility(..., whileInPlay: the card's id) (docs/decisions/2026-10-06-690-p4-turn-boundary.md lists this card), and a PlayerAbility that costs Gold and discards a card by title is the Fortress of Lidless Eyes shape (fortress-lidless-destroy). A Strategy that stays in play exists (the Kata, Economic Repercussions, The Bite of Winter). The pieces have not been exercised together for this card, so build and test them as a unit.</t>
-        </is>
-      </c>
-      <c r="H1379" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1379" t="inlineStr"/>
+      <c r="H1379" t="inlineStr"/>
     </row>
     <row r="1380">
       <c r="A1380" t="inlineStr">
@@ -72340,19 +72313,11 @@
       </c>
       <c r="F2101" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2101" t="inlineStr">
-        <is>
-          <t>Marriage of the Emerald Champion (Event, issue #733): "Limited: Put this Event into play. Target your Personality. While this Event remains in play, he will not be dishonored and you will not lose Honor from other players' actions that have targeted him. After your second turn from now begins, discard this Event." Wirable now on merged pieces: KeepEventInPlay with turnBeginsIn 2, a P11 dishonor bar and a P14 targeted-by-other filter. The binding the first note thought missing exists: an Event that chooses its target at reveal and stays in play is built for Delayed Arrival (a PendingEventChoice answered in ResolveEventChoiceCommand, the target kept in EventTargets, FinishRevealedEvent with keep and turnBeginsIn), and later waves add their Event answers with one hook line in that method's default arm (ResolveWave738EventChoice, ResolveP5EventChoice). This card needs the same one hook and its own record, not a new shared mechanism. The pieces have not been exercised together.</t>
-        </is>
-      </c>
-      <c r="H2101" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2101" t="inlineStr"/>
+      <c r="H2101" t="inlineStr"/>
     </row>
     <row r="2102">
       <c r="A2102" t="inlineStr">
@@ -76437,7 +76402,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -76457,7 +76422,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -76517,7 +76482,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -76697,7 +76662,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wire Bayushi Kachiko on Mendon's reading of attacks (#778)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -528,14 +528,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="C6" t="n">
         <v>851</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>98.9%</t>
+          <t>99.1%</t>
         </is>
       </c>
     </row>
@@ -708,14 +708,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2180</v>
+        <v>2181</v>
       </c>
       <c r="C16" t="n">
         <v>2217</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>98.3%</t>
+          <t>98.4%</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C20" t="n">
         <v>3</v>
@@ -792,7 +792,7 @@
         <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C27" s="2" t="n">
         <v>6</v>
@@ -934,7 +934,7 @@
         <v>3</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -5907,19 +5907,11 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G146" t="inlineStr">
-        <is>
-          <t>Bayushi Kachiko: "After the next time this turn a target Personality attacks, his controller loses 2 Honor" needs a ruling (does "attacks" mean he is declared into an attacking army, or that he makes an Attack action?) and a one-shot turn watch keyed to it. Her static -1F term is plain P9 data once the reading is chosen.</t>
-        </is>
-      </c>
-      <c r="H146" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -76554,7 +76546,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wire Kalani's Landing: Gold Cost reduction on a card in play after any announced action (#816)
Mendon's ruling (R-041): the Reaction targets a card in play with a non-zero Gold Cost
after either player's announced action and gives it -2 Gold Cost until end of turn, once
per turn. Also wires its no-Gold-for-attachments production and "after each phase begins:
straighten" (new EngineHooks.PhaseBegins channel). The Gold Cost modifier already existed;
this adds its target rule and the announce window for either player's action.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -511,14 +511,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C5" t="n">
         <v>53</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>96.2%</t>
+          <t>98.1%</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2181</v>
+        <v>2182</v>
       </c>
       <c r="C16" t="n">
         <v>2224</v>
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
         <v>3</v>
@@ -845,7 +845,7 @@
         <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C28" s="2" t="n">
         <v>8</v>
@@ -965,7 +965,7 @@
         <v>3</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1470,19 +1470,11 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Kalani's Landing (Mantis Stronghold, Emperor Edition #408, issue #812): production 4, strength 7, starting Honor 2. "This card will not produce Gold when paying for an attachment" and "After each phase begins: Straighten this card" look expressible (payment kinds distinguish attachments, PaymentKind.Equip; Stronghold phase-start straightening has precedent, though neither was checked closely). The blocker is the Reaction: "After an action is announced, target a card (in play): Give it -2 Gold Cost." It needs an after-announcement Reaction for any action (TRIG-ANN), a persistent Gold Cost modifier on a card in play (no such modifier exists for cards in play), and the text states no duration or what a Gold Cost on a card in play affects, which needs a ruling from Mendon. Oracle lists it as banned (September 21st, 2013).</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>RULES</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2333,7 +2325,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>The Governor's Estate (Stronghold, Emperor Edition, unnumbered, issue #812): production 4, strength 7, starting Honor 8. "Your face-down Dynasty cards in play are Holdings with the trait, ':bow:: Produce 2 Gold.'" and "Twice per turn, after your Dynasty Phase begins, you may pay 2 Gold to turn a card in your Province face-down (if needed) and put it into play bowed" need face-down cards IN PLAY, which the engine has no representation for (cards are put into play face-up; Hidden Weapons' face-down cards sit under a Holding, not in play), plus a granted Holding trait on them. Its Limited Honor gain with no attack and its Tireless Battle (discard a card for +2F or -2F) are expressible. Not listed as banned: Oracle labels it Legacy only.</t>
+          <t>The Governor's Estate (Stronghold, Emperor Edition, unnumbered, issue #812): production 4, strength 7, starting Honor 8. "Your face-down Dynasty cards in play are Holdings with the trait, ':bow:: Produce 2 Gold.'" and "Twice per turn, after your Dynasty Phase begins, you may pay 2 Gold to turn a card in your Province face-down (if needed) and put it into play bowed" need face-down cards IN PLAY, which the engine has no representation for (cards are put into play face-up; Hidden Weapons' face-down cards sit under a Holding, not in play), plus a granted Holding trait on them. Its Limited Honor gain with no attack and its Tireless Battle (discard a card for +2F or -2F) are expressible. Playable by R-040; Oracle labels it Legacy only and lists no ban.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -48285,7 +48277,7 @@
       </c>
       <c r="G1395" t="inlineStr">
         <is>
-          <t>Caught Unawares (Strategy, issue #812). Open: "If you control no Personalities, target one or two Personalities: Bow them. Negate their straightening (this turn). If it is not your turn, draw a card." Battle: "Target an enemy card with no unbowed attachments: Bow it." Bow and negate-straighten effects exist (Bow Before My Will, Quagmire), but this needs a "you control no Personalities" condition, a one-or-two target count, a straighten negation lasting THIS TURN (the existing ones are "next straightening"), a draw conditional on whose turn it is, and a target filter for "no unbowed attachments" (the existing filter is no attachments at all). Read against the engine, not built. Oracle lists it as banned (September 21st, 2013).</t>
+          <t>Caught Unawares (Strategy, issue #812). Open: "If you control no Personalities, target one or two Personalities: Bow them. Negate their straightening (this turn). If it is not your turn, draw a card." Battle: "Target an enemy card with no unbowed attachments: Bow it." Bow and negate-straighten effects exist (Bow Before My Will, Quagmire), but this needs a "you control no Personalities" condition, a one-or-two target count, a straighten negation lasting THIS TURN (the existing ones are "next straightening"), a draw conditional on whose turn it is, and a target filter for "no unbowed attachments" (the existing filter is no attachments at all). Read against the engine, not built. Playable by R-040; Oracle's tournament ban (September 21st, 2013) is a data note only and is never shown in game.</t>
         </is>
       </c>
       <c r="H1395" t="inlineStr">
@@ -56349,7 +56341,7 @@
       </c>
       <c r="G1631" t="inlineStr">
         <is>
-          <t>One Koku (Strategy, issue #812): "Reaction: When paying a Gold cost: Produce one Gold." No engine gap found. Near Miss (PromoPaymentSources.cs, issue #667) is the precedent for a Strategy IN HAND offered as a payment token and discarded when chosen, and Seaside Bazaar's "When paying a Gold Cost: Produce 1 Gold" (EmperorMechE.cs, AnyGoldCostWhen) is the unrestricted trigger. The designer note ("worth one koku") has no rules effect. Imported from the Emperor Edition printing (#326); Oracle lists it as banned from Emperor Edition tournaments (12/24/12) and Mendon has not ruled on playing banned cards.</t>
+          <t>One Koku (Strategy, issue #812): "Reaction: When paying a Gold cost: Produce one Gold." No engine gap found. Near Miss (PromoPaymentSources.cs, issue #667) is the precedent for a Strategy IN HAND offered as a payment token and discarded when chosen, and Seaside Bazaar's "When paying a Gold Cost: Produce 1 Gold" (EmperorMechE.cs, AnyGoldCostWhen) is the unrestricted trigger. The designer note ("worth one koku") has no rules effect. Imported from the Emperor Edition printing (#326); Playable by Mendon's ruling R-040; Oracle's tournament ban (12/24/12) is a data note only and is never shown in game.</t>
         </is>
       </c>
       <c r="H1631" t="inlineStr">
@@ -62345,7 +62337,7 @@
       </c>
       <c r="G1807" t="inlineStr">
         <is>
-          <t>The Duty of the Crab (Strategy, issue #812). Its Focus Effect ("delay the effects of losing this duel until after the next Dynasty Phase begins") is an existing shape: add its Focus Effect to DelayFocusEffects (EmperorRulingR2Cards.cs, which The Honor of the Lion and five more Strategies use). The Battle half ("If you control any units at the current battlefield, choose your performing Crab Clan Personality who is face-up in your provinces or discarded (not dead): Bring him into play there, paying all costs") is a recruit at a battlefield from a province or the discard pile; the Reserve recruit and the dead-pile gap (ZONE) are the nearest primitives, and whether one action can offer both a province and the discard pile as sources has NOT been checked. Oracle lists it as banned (September 21st, 2013).</t>
+          <t>The Duty of the Crab (Strategy, issue #812). Its Focus Effect ("delay the effects of losing this duel until after the next Dynasty Phase begins") is an existing shape: add its Focus Effect to DelayFocusEffects (EmperorRulingR2Cards.cs, which The Honor of the Lion and five more Strategies use). The Battle half ("If you control any units at the current battlefield, choose your performing Crab Clan Personality who is face-up in your provinces or discarded (not dead): Bring him into play there, paying all costs") is a recruit at a battlefield from a province or the discard pile; the Reserve recruit and the dead-pile gap (ZONE) are the nearest primitives, and whether one action can offer both a province and the discard pile as sources has NOT been checked. Playable by R-040; Oracle's tournament ban (September 21st, 2013) is a data note only and is never shown in game.</t>
         </is>
       </c>
       <c r="H1807" t="inlineStr">
@@ -71251,7 +71243,7 @@
       </c>
       <c r="G2068" t="inlineStr">
         <is>
-          <t>Well-Tended Farm (Holding, issue #812): ":bow:: Produce 1 Gold. Limited, :bow:: Gain 1 Honor." No engine gap found. A Holding with a printed bow-for-Gold production and a Limited bow ability that gains Honor is the shape the Holding waves already use (package_holding_wave_2.py, _50.py, _51.py). Wire it as a Holding wave entry from Emperor Edition #56. Oracle lists it as banned from Emperor Edition tournaments (12/24/12); Mendon has not ruled on playing banned cards.</t>
+          <t>Well-Tended Farm (Holding, issue #812): ":bow:: Produce 1 Gold. Limited, :bow:: Gain 1 Honor." No engine gap found. A Holding with a printed bow-for-Gold production and a Limited bow ability that gains Honor is the shape the Holding waves already use (package_holding_wave_2.py, _50.py, _51.py). Wire it as a Holding wave entry from Emperor Edition #56. Playable by Mendon's ruling R-040; Oracle's tournament ban (12/24/12) is a data note only and is never shown in game.</t>
         </is>
       </c>
       <c r="H2068" t="inlineStr">
@@ -71803,7 +71795,7 @@
       </c>
       <c r="G2084" t="inlineStr">
         <is>
-          <t>Cross-Clan Wedding (Event, issue #812). Province-reveal Events exist (ProvinceRevealEvents.cs, primitive P5) and taking control of a Personality exists (TakeControlOfPersonality, EmperorRemainingC.cs), so the engine has the trigger and the transfer. Missing: the other player's OWN choice of which of their Personalities to give back (the "other player chooses" primitive exists only for deck searches, SearchExtensions.cs), the "If he now controls the Personality" condition, and a check of the Unique/Singular rules for both transfers (docs/decisions/2026-09-12-unique-singular-control-transfer.md). The Emperor-era Event scans may print only the effect without the "After you reveal cards in your Provinces" lead-in (EmperorRemainingFEvents.cs), so compare the Emperor Edition #15 scan before wiring. Oracle lists it as banned (12/24/12).</t>
+          <t>Cross-Clan Wedding (Event, issue #812). Province-reveal Events exist (ProvinceRevealEvents.cs, primitive P5) and taking control of a Personality exists (TakeControlOfPersonality, EmperorRemainingC.cs), so the engine has the trigger and the transfer. Missing: the other player's OWN choice of which of their Personalities to give back (the "other player chooses" primitive exists only for deck searches, SearchExtensions.cs), the "If he now controls the Personality" condition, and a check of the Unique/Singular rules for both transfers (docs/decisions/2026-09-12-unique-singular-control-transfer.md). The Emperor-era Event scans may print only the effect without the "After you reveal cards in your Provinces" lead-in (EmperorRemainingFEvents.cs), so compare the Emperor Edition #15 scan before wiring. Playable by R-040; Oracle's tournament ban (12/24/12) is a data note only and is never shown in game.</t>
         </is>
       </c>
       <c r="H2084" t="inlineStr">
@@ -77151,7 +77143,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wire Kokujin, P'an Ku - exp, Zansho - exp, Chiyurei's Axe, Koan's Jingasa and Koan's Robes (#827)
Rulings R-049..R-053. New primitives: Kokujin's sacrifice decision after a won duel, P'an Ku's
remain-bowed control link with a seppuku bar, WatchScope.Unit, the Koan Spell limit. Ningen's Treatise
is left out (allies). The bot answers the three new decisions. Inventory 2190 -> 2196 wired; the art pack
for the six scans is built locally (not published).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQdg2Z7Kwb92sRNhB7ZuaZ
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -464,7 +464,6 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -528,14 +527,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>848</v>
+        <v>851</v>
       </c>
       <c r="C6" t="n">
         <v>851</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>99.6%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -564,14 +563,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C8" t="n">
         <v>137</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>95.6%</t>
+          <t>97.8%</t>
         </is>
       </c>
     </row>
@@ -708,14 +707,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2190</v>
+        <v>2196</v>
       </c>
       <c r="C16" t="n">
         <v>2225</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>98.4%</t>
+          <t>98.7%</t>
         </is>
       </c>
     </row>
@@ -734,40 +733,35 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Personality</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Spell</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Spell</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Strategy</t>
+          <t>Holding</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Holding</t>
+          <t>Event</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Event</t>
+          <t>Celestial</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Celestial</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -776,55 +770,52 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Coils of Madness</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>3</v>
+          <t>Torn Asunder</t>
+        </is>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
-      </c>
-      <c r="E20" t="n">
-        <v>2</v>
-      </c>
-      <c r="G20" t="n">
         <v>1</v>
       </c>
-      <c r="I20" t="n">
-        <v>9</v>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Torn Asunder</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
+          <t>Emperor Edition</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
         <v>1</v>
       </c>
-      <c r="D21" t="n">
+      <c r="F21" t="n">
         <v>1</v>
       </c>
-      <c r="E21" t="n">
+      <c r="H21" t="n">
         <v>5</v>
-      </c>
-      <c r="G21" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Emperor Edition</t>
-        </is>
+          <t>Promotional–Celestial</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
         <v>1</v>
@@ -832,30 +823,27 @@
       <c r="G22" t="n">
         <v>1</v>
       </c>
-      <c r="I22" t="n">
+      <c r="H22" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Promotional–Celestial</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
+          <t>Coils of Madness</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
         <v>1</v>
       </c>
+      <c r="D23" t="n">
+        <v>2</v>
+      </c>
       <c r="F23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G23" t="n">
         <v>1</v>
       </c>
       <c r="H23" t="n">
-        <v>1</v>
-      </c>
-      <c r="I23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
@@ -864,19 +852,19 @@
           <t>Promotional–Emperor</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="B24" t="n">
         <v>1</v>
       </c>
-      <c r="E24" t="n">
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="n">
         <v>1</v>
       </c>
       <c r="G24" t="n">
         <v>1</v>
       </c>
       <c r="H24" t="n">
-        <v>1</v>
-      </c>
-      <c r="I24" t="n">
         <v>4</v>
       </c>
     </row>
@@ -886,10 +874,10 @@
           <t>War of Honor</t>
         </is>
       </c>
-      <c r="E25" t="n">
+      <c r="D25" t="n">
         <v>2</v>
       </c>
-      <c r="I25" t="n">
+      <c r="H25" t="n">
         <v>2</v>
       </c>
     </row>
@@ -899,10 +887,10 @@
           <t>Aftermath</t>
         </is>
       </c>
-      <c r="C26" t="n">
+      <c r="B26" t="n">
         <v>1</v>
       </c>
-      <c r="I26" t="n">
+      <c r="H26" t="n">
         <v>1</v>
       </c>
     </row>
@@ -912,10 +900,10 @@
           <t>Gates of Chaos</t>
         </is>
       </c>
-      <c r="E27" t="n">
+      <c r="D27" t="n">
         <v>1</v>
       </c>
-      <c r="I27" t="n">
+      <c r="H27" t="n">
         <v>1</v>
       </c>
     </row>
@@ -929,25 +917,22 @@
         <v>3</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I28" s="2" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -17556,19 +17541,11 @@
       </c>
       <c r="F490" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G490" t="inlineStr">
-        <is>
-          <t>Kokujin: "if Kokujin wins, you may destroy one of your Personalities (at any location) to take control of the loser (he joins Kokujin's army)" is a choice made after the duel resolves, among one option per Personality of yours plus plain destruction. Duel outcomes in this engine apply directly; a deferred outcome decision needs the P1 after-action trait queue extended (EmperorP1.cs) or a new post-duel decision hook.</t>
-        </is>
-      </c>
-      <c r="H490" t="inlineStr">
-        <is>
-          <t>TRIG-AFTER</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr"/>
+      <c r="H490" t="inlineStr"/>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
@@ -22020,19 +21997,11 @@
       </c>
       <c r="F622" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G622" t="inlineStr">
-        <is>
-          <t>P'an Ku - exp (Personality, issue #736): "Open, bow: Give a target card a Madness token" is built (the existing panku-madness shape), but "Limited, bow: P'an Ku may remain bowed. Take control of a target Personality with more Madness tokens than printed Personal Honor and remove those tokens. The target will not commit seppuku until P'an Ku straightens or leaves play. After P'an Ku does, give control of the target to his owner." needs three things together: a control change that returns when a named card straightens or leaves play (TakeControl exists; the timed return trigger does not), a seppuku bar tied to that card, and "may remain bowed" (a rule exempting him from straightening). One card, three new rules.</t>
-        </is>
-      </c>
-      <c r="H622" t="inlineStr">
-        <is>
-          <t>CONTROL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr"/>
+      <c r="H622" t="inlineStr"/>
     </row>
     <row r="623">
       <c r="A623" t="inlineStr">
@@ -31534,19 +31503,11 @@
       </c>
       <c r="F903" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G903" t="inlineStr">
-        <is>
-          <t>Zansho - exp (Personality, issue #733): the scan reads "Battle: Bow Zansho's target unbowed Follower. Ranged Attack with strength equal to its Force, plus 2 if the Ranged Attack targets Daigotsu Arakan." It does not say whose Follower is bowed: any unbowed Follower at the battlefield (the other player's included), only one of the controller's, or one attached to Zansho himself. The three readings are three different cards (bowing an enemy Follower as a cost is a strong effect). Needs Mendon's ruling before it is built; the gate ("will not join a Spider Clan player") and the Attack strength hook are available.</t>
-        </is>
-      </c>
-      <c r="H903" t="inlineStr">
-        <is>
-          <t>RULES</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G903" t="inlineStr"/>
+      <c r="H903" t="inlineStr"/>
     </row>
     <row r="904">
       <c r="A904" t="inlineStr">
@@ -37136,19 +37097,11 @@
       </c>
       <c r="F1070" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1070" t="inlineStr">
-        <is>
-          <t>Chiyurei's Axe (Item, issue #732): its Equip discount ("Attaches to Hida Chiyurei paying 2 less Gold") is a P2 entry term and +3F is printed, but its second sentence, "Melee Attacks this Personality performs may be compared against the target's base Force", is a trait of the performer on every Melee Attack he performs. The comparison itself is built (AttackCompare.PrintedForce) but an Attack's optional comparison is a static function of the ability id (AttackCompareOptions in EmperorRulingR5.cs, read by ValidateAbility's Choice gate, the offered-ability loop's compareChoices and its label in CardAbilities.cs, and AttackComparedValue), so a performer-scoped option needs those four places to learn the performer. A shared-interface change in the central action builder, not a card-wave line; the card is not published, so no printed effect is dropped (docs/decisions/2026-10-06-690-p24-effect-primitives.md, limits).</t>
-        </is>
-      </c>
-      <c r="H1070" t="inlineStr">
-        <is>
-          <t>EFFECT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1070" t="inlineStr"/>
+      <c r="H1070" t="inlineStr"/>
     </row>
     <row r="1071">
       <c r="A1071" t="inlineStr">
@@ -38284,19 +38237,11 @@
       </c>
       <c r="F1104" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1104" t="inlineStr">
-        <is>
-          <t>Koan's Jingasa (Item, issue #736): "This Personality has Shugenja, may not have more Spells than Koan cards attached, and he need not bow for his Spells with an odd Focus Value (0 is even)." The Shugenja keyword is AttachGrantsKeyword, but P11's SpellLimit counts Spell actions performed, not Spells attached (the rule here is an attachment limit counted against Koan cards), and "need not bow for his Spells" is a waiver of the bow cost of a Spell's own ability, which P24's cost waivers do not cover.</t>
-        </is>
-      </c>
-      <c r="H1104" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1104" t="inlineStr"/>
+      <c r="H1104" t="inlineStr"/>
     </row>
     <row r="1105">
       <c r="A1105" t="inlineStr">
@@ -38326,19 +38271,11 @@
       </c>
       <c r="F1105" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1105" t="inlineStr">
-        <is>
-          <t>Koan's Robes (Item, issue #737): "This Personality has a Force bonus equal to the number of other Koan cards in this unit. This Personality need not bow for his Spells with an even Focus Value (0 is even). Negate the first destruction each turn of cards in this unit from another player's card." Part is merged: "need not bow for his Spells with an even Focus Value" is P24's EngineHooks.CostWaivers with SpellFocusParityWaives (odd: false; EffectPrimitivesCosts.cs, written for this card and Koan's Jingasa), and the destruction negation is a P7 standing watch whose scope is the gap (a StandingWatch covers the card, its controller's cards that fit a keyword, or its attached Followers; there is no cards-in-this-unit scope, and a Condition could stand in for it). Still missing: the Force bonus equal to the number of other Koan cards in this unit. Batch 3 merged its stat terms (StatTerms.cs), but the counters are only AttachedWithKeyword (the host's own attachments) and OpposingTokens; none counts a keyword across a unit (host, Followers and the other attachments). Publishing it without that sentence would drop printed text.</t>
-        </is>
-      </c>
-      <c r="H1105" t="inlineStr">
-        <is>
-          <t>STAT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1105" t="inlineStr"/>
+      <c r="H1105" t="inlineStr"/>
     </row>
     <row r="1106">
       <c r="A1106" t="inlineStr">
@@ -76747,7 +76684,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -76867,7 +76804,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -76927,7 +76864,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -77007,7 +76944,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -77107,7 +77044,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -77207,7 +77144,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wire Well-Tended Farm, One Koku, Shrine to the Heavens, Stone of Remembrance, Cross-Clan Wedding, Minor Blackmail, The Onyx Championship, Caught Unawares, The Duty of the Crab, Benten's Blessing and Jizo's Mercy (#829)
Eleven cards on Mendon's 2026-10-11 rulings (R-054 to R-062), in four waves
(holding/event/strategy/celestial-wave-829) with Wave829.cs: the first users of
the P5 province-reveal Events, a Sleep-style multi-select for Benten's Blessing,
the Stone's card-tear animation and zero-count deck minimum, the five Caught
Unawares primitives, and bot rules for the new decisions. Art pack
catalogue-art-issue829-20261011-r1 (4655 images) built; inventory 2196 -> 2207.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQdg2Z7Kwb92sRNhB7ZuaZ
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -462,8 +462,6 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -599,14 +597,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="C10" t="n">
         <v>601</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>97.5%</t>
+          <t>98.0%</t>
         </is>
       </c>
     </row>
@@ -617,14 +615,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C11" t="n">
         <v>154</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>98.1%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -635,14 +633,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C12" t="n">
         <v>82</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>93.9%</t>
+          <t>97.6%</t>
         </is>
       </c>
     </row>
@@ -653,14 +651,14 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C13" t="n">
         <v>37</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>94.6%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -707,14 +705,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2196</v>
+        <v>2207</v>
       </c>
       <c r="C16" t="n">
         <v>2225</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>98.7%</t>
+          <t>99.2%</t>
         </is>
       </c>
     </row>
@@ -748,20 +746,10 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Holding</t>
+          <t>Event</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Celestial</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -779,160 +767,120 @@
       <c r="D20" t="n">
         <v>5</v>
       </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
       <c r="F20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Emperor Edition</t>
-        </is>
+          <t>Coils of Madness</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E21" t="n">
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Promotional–Celestial</t>
-        </is>
+          <t>Promotional–Emperor</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
       </c>
       <c r="D22" t="n">
         <v>1</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>2</v>
-      </c>
-      <c r="F22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Coils of Madness</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>1</v>
+          <t>War of Honor</t>
+        </is>
       </c>
       <c r="D23" t="n">
         <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
-      </c>
-      <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Promotional–Emperor</t>
+          <t>Aftermath</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>1</v>
       </c>
-      <c r="D24" t="n">
-        <v>1</v>
-      </c>
       <c r="F24" t="n">
         <v>1</v>
       </c>
-      <c r="G24" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" t="n">
-        <v>4</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>War of Honor</t>
+          <t>Gates of Chaos</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2</v>
-      </c>
-      <c r="H25" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Aftermath</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
+          <t>Promotional–Celestial</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
         <v>1</v>
       </c>
-      <c r="H26" t="n">
+      <c r="F26" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Gates of Chaos</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H27" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="E28" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F28" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G28" s="2" t="n">
+      <c r="D27" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E27" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H28" s="2" t="n">
-        <v>29</v>
+      <c r="F27" s="2" t="n">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -48151,19 +48099,11 @@
       </c>
       <c r="F1395" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1395" t="inlineStr">
-        <is>
-          <t>Caught Unawares (Strategy, issue #812). Open: "If you control no Personalities, target one or two Personalities: Bow them. Negate their straightening (this turn). If it is not your turn, draw a card." Battle: "Target an enemy card with no unbowed attachments: Bow it." Bow and negate-straighten effects exist (Bow Before My Will, Quagmire), but this needs a "you control no Personalities" condition, a one-or-two target count, a straighten negation lasting THIS TURN (the existing ones are "next straightening"), a draw conditional on whose turn it is, and a target filter for "no unbowed attachments" (the existing filter is no attachments at all). Read against the engine, not built. Playable by R-040; Oracle's tournament ban (September 21st, 2013) is a data note only and is never shown in game.</t>
-        </is>
-      </c>
-      <c r="H1395" t="inlineStr">
-        <is>
-          <t>SMALL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1395" t="inlineStr"/>
+      <c r="H1395" t="inlineStr"/>
     </row>
     <row r="1396">
       <c r="A1396" t="inlineStr">
@@ -56215,19 +56155,11 @@
       </c>
       <c r="F1631" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1631" t="inlineStr">
-        <is>
-          <t>One Koku (Strategy, issue #812): "Reaction: When paying a Gold cost: Produce one Gold." No engine gap found. Near Miss (PromoPaymentSources.cs, issue #667) is the precedent for a Strategy IN HAND offered as a payment token and discarded when chosen, and Seaside Bazaar's "When paying a Gold Cost: Produce 1 Gold" (EmperorMechE.cs, AnyGoldCostWhen) is the unrestricted trigger. The designer note ("worth one koku") has no rules effect. Imported from the Emperor Edition printing (#326); Playable by Mendon's ruling R-040; Oracle's tournament ban (12/24/12) is a data note only and is never shown in game.</t>
-        </is>
-      </c>
-      <c r="H1631" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1631" t="inlineStr"/>
+      <c r="H1631" t="inlineStr"/>
     </row>
     <row r="1632">
       <c r="A1632" t="inlineStr">
@@ -62211,19 +62143,11 @@
       </c>
       <c r="F1807" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1807" t="inlineStr">
-        <is>
-          <t>The Duty of the Crab (Strategy, issue #812). Its Focus Effect ("delay the effects of losing this duel until after the next Dynasty Phase begins") is an existing shape: add its Focus Effect to DelayFocusEffects (EmperorRulingR2Cards.cs, which The Honor of the Lion and five more Strategies use). The Battle half ("If you control any units at the current battlefield, choose your performing Crab Clan Personality who is face-up in your provinces or discarded (not dead): Bring him into play there, paying all costs") is a recruit at a battlefield from a province or the discard pile; the Reserve recruit and the dead-pile gap (ZONE) are the nearest primitives, and whether one action can offer both a province and the discard pile as sources has NOT been checked. Playable by R-040; Oracle's tournament ban (September 21st, 2013) is a data note only and is never shown in game.</t>
-        </is>
-      </c>
-      <c r="H1807" t="inlineStr">
-        <is>
-          <t>SMALL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1807" t="inlineStr"/>
+      <c r="H1807" t="inlineStr"/>
     </row>
     <row r="1808">
       <c r="A1808" t="inlineStr">
@@ -69337,14 +69261,10 @@
       </c>
       <c r="F2016" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2016" t="inlineStr">
-        <is>
-          <t>Shrine to the Heavens (awaiting a ruling from Mendon): the old gap, a Celestial-reveal choice before the discard of the other Celestials, is closed: P6 (AfterFacts.cs, CelestialEntryRegistry) opens a choice when a Celestial enters play, with SparesFromDiscard so a chosen Celestial is not discarded and the discard of the others waits for the answer (this card is its design example). Still open: whether "one of your Celestials in play" may be the newly revealed one, what happens with a third Celestial, and whether two Celestials persist if the Shrine leaves play; ControlsCelestialEffect and similar code assume at most one Celestial. Not wired.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2016" t="inlineStr"/>
       <c r="H2016" t="inlineStr"/>
     </row>
     <row r="2017">
@@ -69715,14 +69635,10 @@
       </c>
       <c r="F2027" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2027" t="inlineStr">
-        <is>
-          <t>Stone of Remembrance: needs a Dynasty-deck-minimum exemption (a new field on DeckCardInfo, a shared interface), and has unresolved readings: whether 'tear it in half' is flavor (R-025 ruled that for 'custody'), and whether it may react to any action that targets any of your cards.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2027" t="inlineStr"/>
       <c r="H2027" t="inlineStr"/>
     </row>
     <row r="2028">
@@ -71147,19 +71063,11 @@
       </c>
       <c r="F2069" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2069" t="inlineStr">
-        <is>
-          <t>Well-Tended Farm (Holding, issue #812): ":bow:: Produce 1 Gold. Limited, :bow:: Gain 1 Honor." No engine gap found. A Holding with a printed bow-for-Gold production and a Limited bow ability that gains Honor is the shape the Holding waves already use (package_holding_wave_2.py, _50.py, _51.py). Wire it as a Holding wave entry from Emperor Edition #56. Playable by Mendon's ruling R-040; Oracle's tournament ban (12/24/12) is a data note only and is never shown in game.</t>
-        </is>
-      </c>
-      <c r="H2069" t="inlineStr">
-        <is>
-          <t>WIRE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2069" t="inlineStr"/>
+      <c r="H2069" t="inlineStr"/>
     </row>
     <row r="2070">
       <c r="A2070" t="inlineStr">
@@ -71699,19 +71607,11 @@
       </c>
       <c r="F2085" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2085" t="inlineStr">
-        <is>
-          <t>Cross-Clan Wedding (Event, issue #812). Province-reveal Events exist (ProvinceRevealEvents.cs, primitive P5) and taking control of a Personality exists (TakeControlOfPersonality, EmperorRemainingC.cs), so the engine has the trigger and the transfer. Missing: the other player's OWN choice of which of their Personalities to give back (the "other player chooses" primitive exists only for deck searches, SearchExtensions.cs), the "If he now controls the Personality" condition, and a check of the Unique/Singular rules for both transfers (docs/decisions/2026-09-12-unique-singular-control-transfer.md). The Emperor-era Event scans may print only the effect without the "After you reveal cards in your Provinces" lead-in (EmperorRemainingFEvents.cs), so compare the Emperor Edition #15 scan before wiring. Playable by R-040; Oracle's tournament ban (12/24/12) is a data note only and is never shown in game.</t>
-        </is>
-      </c>
-      <c r="H2085" t="inlineStr">
-        <is>
-          <t>SMALL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2085" t="inlineStr"/>
+      <c r="H2085" t="inlineStr"/>
     </row>
     <row r="2086">
       <c r="A2086" t="inlineStr">
@@ -72557,14 +72457,10 @@
       </c>
       <c r="F2110" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2110" t="inlineStr">
-        <is>
-          <t>Minor Blackmail (awaiting a ruling from Mendon): the reveal-time window ("after you reveal cards in your Provinces at the start of your turn, if this Event is face-up") is P5's province-reveal Events, and P6 has an AssignedToAttack fact, but that fact covers an attacker's assignment only (no defender-assignment fact), and nothing is a game-long watch on "an action that he performed" that survives him leaving play or changing controller. Rulings needed: whether "an action that he performed" means only the performer slot or his own card's abilities, and whether "his unit is assigned" includes defender assignment. Not wired.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2110" t="inlineStr"/>
       <c r="H2110" t="inlineStr"/>
     </row>
     <row r="2111">
@@ -73597,19 +73493,11 @@
       </c>
       <c r="F2140" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2140" t="inlineStr">
-        <is>
-          <t>The Onyx Championship (Event, issue #738): "Choose one of your Shugenja in play. Permanently give him Shadowlands and the ability, 'Maho Limited: Bow this Shugenja and destroy your target Personality: Search your discard pile, then deck, then provinces for an Oni Personality. Bring him into play, paying all costs. Lose 3 Honor.'" The permanent keyword and ability grant are built (GrantKeyword, GrantAbility Permanent), and the ordered search of a discard pile, a deck and the provinces is P20's, but P20 lets a card found in a province enter play only ignoring its costs (SearchEffect.RecruitFromProvinceIgnoringCosts is the sole province recruit and ValidateSearchSpec refuses any other disposition for a province source), while the card prints "paying all costs" for every source. The pay-all-costs recruit from a province is not built; publishing the card with the ignoring-costs recruit would change a printed cost.</t>
-        </is>
-      </c>
-      <c r="H2140" t="inlineStr">
-        <is>
-          <t>SEARCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2140" t="inlineStr"/>
+      <c r="H2140" t="inlineStr"/>
     </row>
     <row r="2141">
       <c r="A2141" t="inlineStr">
@@ -74183,14 +74071,10 @@
       </c>
       <c r="F2157" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2157" t="inlineStr">
-        <is>
-          <t>Benten's Blessing (awaiting a ruling from Mendon): the entry window is merged (P6 CelestialEntryRegistry, used by Natsu-Togumara's Guidance), but it asks for one card per choice, so "zero to two face-up Personalities" needs two queued choices or a multi-pick. The Reaction half (an action that would target your Personality targets your performing Personality instead, discarding the Celestial) is a redirection of the kind built in docs/decisions/2026-09-19-redirection-and-protective-reactions.md, which names this card. Unresolved reading: which out-of-play zones count as face-up, and whether the +1PH persists when a chosen card changes zone. Not wired.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2157" t="inlineStr"/>
       <c r="H2157" t="inlineStr"/>
     </row>
     <row r="2158">
@@ -74663,19 +74547,11 @@
       </c>
       <c r="F2171" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2171" t="inlineStr">
-        <is>
-          <t>Jizo's Mercy (Celestial, issue #653): the first Battle ("Move a target attacking Personality home") is buildable, but the second, "Battle: Discard this Celestial. In this battle's resolution, before you destroy the Province, gain 4 Honor instead", has an unresolved reading. Question for Mendon: does "instead" mean the Celestial's controller gains 4 Honor INSTEAD of destroying the Province (the Province survives the battle), or only before it, so the Province is still destroyed and "instead" has no referent; and may the Defender play it (he would not be destroying the Province) or only an Attacker who wins? The engine has the resolution hooks (BeforeResolution.cs, AfterResolution.cs); the reading must be ruled first.</t>
-        </is>
-      </c>
-      <c r="H2171" t="inlineStr">
-        <is>
-          <t>RULES</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2171" t="inlineStr"/>
+      <c r="H2171" t="inlineStr"/>
     </row>
     <row r="2172">
       <c r="A2172" t="inlineStr">
@@ -76604,7 +76480,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -76624,7 +76500,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -77044,7 +76920,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -77104,7 +76980,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Record rules questions from the single-action audit in the card inventory (#833)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vn5ze8TWKcKMzNTke2svyH
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -22114,7 +22114,11 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G627" t="inlineStr"/>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>RULING NEEDED (issue #833 audit): Rata's "Rata sacrifices his victim's corpse" is not modeled; only "Draw a card" runs. What does sacrificing the corpse do?</t>
+        </is>
+      </c>
       <c r="H627" t="inlineStr"/>
     </row>
     <row r="628">
@@ -35624,7 +35628,11 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1028" t="inlineStr"/>
+      <c r="G1028" t="inlineStr">
+        <is>
+          <t>RULING NEEDED (issue #833 audit): The Bestial Ones' Engage has no location condition in its text and the engine offers it from a Follower whose Personality is at home. Intended?</t>
+        </is>
+      </c>
       <c r="H1028" t="inlineStr"/>
     </row>
     <row r="1029">
@@ -42888,7 +42896,11 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1242" t="inlineStr"/>
+      <c r="G1242" t="inlineStr">
+        <is>
+          <t>RULING NEEDED (issue #833 audit): Mastering the Elements is "Once per game", but CopyKataTargetingTests asserts the Reaction is available again after the card re-enters play. Is once per game absolute, or once per time in play?</t>
+        </is>
+      </c>
       <c r="H1242" t="inlineStr"/>
     </row>
     <row r="1243">
@@ -59834,7 +59846,11 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1739" t="inlineStr"/>
+      <c r="G1739" t="inlineStr">
+        <is>
+          <t>RULING NEEDED (issue #833 audit): "Permanently give your Samurai Shadowlands and Undead" -- the engine gives it only to the performing Samurai (IvoryMovementTests asserts that reading). Is it the performer, or every Samurai you control?</t>
+        </is>
+      </c>
       <c r="H1739" t="inlineStr"/>
     </row>
     <row r="1740">
@@ -75366,7 +75382,11 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G2195" t="inlineStr"/>
+      <c r="G2195" t="inlineStr">
+        <is>
+          <t>RULING NEEDED (issue #833 audit): Fallow Lands' Reaction is gated by the engine to its own province under attack with its controller the Defender and present there; the printed text states none of that. Which gates are intended?</t>
+        </is>
+      </c>
       <c r="H2195" t="inlineStr"/>
     </row>
     <row r="2196">

</xml_diff>

<commit_message>
Apply rules rulings from the #833 audit: Bestial Ones is battlefield-specific, Mastering the Elements loses its copy on leaving play (#838)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vn5ze8TWKcKMzNTke2svyH
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -22114,11 +22114,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G627" t="inlineStr">
-        <is>
-          <t>RULING NEEDED (issue #833 audit): Rata's "Rata sacrifices his victim's corpse" is not modeled; only "Draw a card" runs. What does sacrificing the corpse do?</t>
-        </is>
-      </c>
+      <c r="G627" t="inlineStr"/>
       <c r="H627" t="inlineStr"/>
     </row>
     <row r="628">
@@ -35628,11 +35624,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1028" t="inlineStr">
-        <is>
-          <t>RULING NEEDED (issue #833 audit): The Bestial Ones' Engage has no location condition in its text and the engine offers it from a Follower whose Personality is at home. Intended?</t>
-        </is>
-      </c>
+      <c r="G1028" t="inlineStr"/>
       <c r="H1028" t="inlineStr"/>
     </row>
     <row r="1029">
@@ -42896,11 +42888,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1242" t="inlineStr">
-        <is>
-          <t>RULING NEEDED (issue #833 audit): Mastering the Elements is "Once per game", but CopyKataTargetingTests asserts the Reaction is available again after the card re-enters play. Is once per game absolute, or once per time in play?</t>
-        </is>
-      </c>
+      <c r="G1242" t="inlineStr"/>
       <c r="H1242" t="inlineStr"/>
     </row>
     <row r="1243">
@@ -59846,11 +59834,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G1739" t="inlineStr">
-        <is>
-          <t>RULING NEEDED (issue #833 audit): "Permanently give your Samurai Shadowlands and Undead" -- the engine gives it only to the performing Samurai (IvoryMovementTests asserts that reading). Is it the performer, or every Samurai you control?</t>
-        </is>
-      </c>
+      <c r="G1739" t="inlineStr"/>
       <c r="H1739" t="inlineStr"/>
     </row>
     <row r="1740">
@@ -75382,11 +75366,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G2195" t="inlineStr">
-        <is>
-          <t>RULING NEEDED (issue #833 audit): Fallow Lands' Reaction is gated by the engine to its own province under attack with its controller the Defender and present there; the printed text states none of that. Which gates are intended?</t>
-        </is>
-      </c>
+      <c r="G2195" t="inlineStr"/>
       <c r="H2195" t="inlineStr"/>
     </row>
     <row r="2196">

</xml_diff>

<commit_message>
Rulings, decision record, blocker removal, name correction and pinned inventories for the twelve ruled cards (#835)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GLVY8srUKbYJTyoNmoGWDm
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -453,15 +453,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -561,14 +559,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C8" t="n">
         <v>137</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>97.8%</t>
+          <t>98.5%</t>
         </is>
       </c>
     </row>
@@ -579,14 +577,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C9" t="n">
         <v>133</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>99.2%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -597,14 +595,14 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>589</v>
+        <v>597</v>
       </c>
       <c r="C10" t="n">
         <v>601</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>98.0%</t>
+          <t>99.3%</t>
         </is>
       </c>
     </row>
@@ -633,14 +631,14 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C12" t="n">
         <v>82</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>97.6%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -705,14 +703,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2207</v>
+        <v>2219</v>
       </c>
       <c r="C16" t="n">
         <v>2225</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>99.2%</t>
+          <t>99.7%</t>
         </is>
       </c>
     </row>
@@ -736,20 +734,10 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Spell</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Strategy</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -758,45 +746,36 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Torn Asunder</t>
-        </is>
+          <t>Promotional–Emperor</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
       </c>
       <c r="C20" t="n">
         <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>5</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Coils of Madness</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1</v>
+          <t>War of Honor</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
       </c>
       <c r="D21" t="n">
         <v>2</v>
       </c>
-      <c r="E21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" t="n">
-        <v>4</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Promotional–Emperor</t>
+          <t>Aftermath</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -805,82 +784,34 @@
       <c r="D22" t="n">
         <v>1</v>
       </c>
-      <c r="F22" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>War of Honor</t>
-        </is>
+          <t>Promotional–Celestial</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
       </c>
       <c r="D23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F23" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Aftermath</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Gates of Chaos</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Promotional–Celestial</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>18</v>
+      <c r="C24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -39999,19 +39930,11 @@
       </c>
       <c r="F1157" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1157" t="inlineStr">
-        <is>
-          <t>The Egg of P'an Ku - exp (awaiting a ruling from Mendon): the build pieces are merged. P22's CopyOfTarget with CreatedRemoval.NextTurnBegins removes the copy after the creator's next turn begins, and "will not straighten, attack, or defend until after your next turn begins" is a straighten hold plus P11 NoAttack/NoDefend with P4's owner-turn duration (docs/decisions/2026-10-06-690-p22-created-copies-grants.md lists this card); the second target is an ordinary slot. What is still open is Mendon's ruling: who controls the copy, where it enters, and how "ignoring costs and restrictions" treats a Unique target. Not wired; no missing engine primitive is known, but the pieces have not been exercised together.</t>
-        </is>
-      </c>
-      <c r="H1157" t="inlineStr">
-        <is>
-          <t>LOCK</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1157" t="inlineStr"/>
+      <c r="H1157" t="inlineStr"/>
     </row>
     <row r="1158">
       <c r="A1158" t="inlineStr">
@@ -41253,19 +41176,11 @@
       </c>
       <c r="F1194" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1194" t="inlineStr">
-        <is>
-          <t>Blood of Isawa's Tribe (Spell, issue #735): "After this card attaches: Choose an element keyword (Air, Earth, Fire, Void, Water) in this Shugenja's keywords or text. While this card is attached, replace all instances of that keyword on this Shugenja with another element keyword that you choose now." P10's ReplaceElementKeyword does the replacement, but the choice is the problem: it is a mandatory trait of the Spell (no "Reaction:" prefix) that needs two decisions in a row (which element, then which replacement) the moment the Spell attaches. Mandatory entry effects (ApplyMandatoryEntryEffects) are automatic and open no decision, and an optional Reaction would change the printed text from mandatory to optional. Opening a pending choice from inside the entry path (before the entry Reaction window, for an attach by Equip, Equip (Battle) or a search) is not a merged path, and "in this Shugenja's keywords or text" would also need a rule for the elements named in text. It is left unpublished rather than approximated.</t>
-        </is>
-      </c>
-      <c r="H1194" t="inlineStr">
-        <is>
-          <t>TRIG-ANN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1194" t="inlineStr"/>
+      <c r="H1194" t="inlineStr"/>
     </row>
     <row r="1195">
       <c r="A1195" t="inlineStr">
@@ -45515,19 +45430,11 @@
       </c>
       <c r="F1319" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1319" t="inlineStr">
-        <is>
-          <t>A Cleansing Breath (Strategy, issue #736): "Battle/Open: Target your Personality at any location. He centers himself. Negate other players' cards' effects that prevent him assigning, moving or performing actions. If he is a Kensai, straighten his unit." The negations are P12 Prevention and movement/assignment immunities, but "he centers himself" has no definition anywhere in the repository (core rules, rulings or code): it names a rule the owner has not given. Needs Mendon's ruling on what centering does before the card is built; publishing it without the sentence would drop printed text.</t>
-        </is>
-      </c>
-      <c r="H1319" t="inlineStr">
-        <is>
-          <t>RULES</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1319" t="inlineStr"/>
+      <c r="H1319" t="inlineStr"/>
     </row>
     <row r="1320">
       <c r="A1320" t="inlineStr">
@@ -50117,19 +50024,11 @@
       </c>
       <c r="F1454" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1454" t="inlineStr">
-        <is>
-          <t>Duty Over All Things (Strategy, issue #732): the scan reads "Battle: Choose your performing discarded Yojimbo: If he would be opposed, bring him into play at the current battlefield, paying 3 less Gold if you control a Courtier or Shugenja." The performer of the action is a Yojimbo in the owner's discard pile, and the action recruits that same card into play at the battlefield. The engine has no support for a Dead or discarded Personality as an action's performer (AbilitySourceZoneAllows and the performer lists read cards in play; P21's province-source and zone pieces do not cover a discard-pile performer), and "if he would be opposed" asks whether an enemy unit stands at the battlefield the card would enter. Needs a performer-from-discard rule and a recruit of the performer by an action, with a ruling on when "would be opposed" is judged.</t>
-        </is>
-      </c>
-      <c r="H1454" t="inlineStr">
-        <is>
-          <t>ZONE</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1454" t="inlineStr"/>
+      <c r="H1454" t="inlineStr"/>
     </row>
     <row r="1455">
       <c r="A1455" t="inlineStr">
@@ -53193,19 +53092,11 @@
       </c>
       <c r="F1544" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1544" t="inlineStr">
-        <is>
-          <t>Imperial Deployment (Strategy, issue #737): "Open: Choose your performing Personality: The Empress dispatches him to the Colonies. Negate other players' cards' effects that prevent him assigning. After the next time this turn an attack is declared, straighten his unit." Two gaps, the first narrower than first noted. (1) P12's Prevention immunity reads movement locks, which also refuse assigning (MovementLocked and MovementKinds.Assign, MovementLocks.cs; docs/decisions/2026-10-06-p12-immunities.md), so a lock made by another player's card with a known source player is covered. Locks with no source player (Too Close to Home, The Perfect Moment) and P11's stored NoAttack/NoDefend restrictions (no source player) are not, so whether that is enough is a reading. (2) "After the next time this turn an attack is declared, straighten his unit": P6's nearest fact is AssignedToAttack, per Personality (AfterFacts.cs), not the declaration of an attack, and there is no one-shot next-time-this-turn watch on a fact; the reading (declaration or first assignment) needs Mendon. "Dispatches him to the Colonies" is flavor text with no rule.</t>
-        </is>
-      </c>
-      <c r="H1544" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1544" t="inlineStr"/>
+      <c r="H1544" t="inlineStr"/>
     </row>
     <row r="1545">
       <c r="A1545" t="inlineStr">
@@ -55037,19 +54928,11 @@
       </c>
       <c r="F1598" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1598" t="inlineStr">
-        <is>
-          <t>Merchant Patronage (Strategy, issue #733): "Political Interrupt: If the action is on another player's Holding, you choose who gains or loses any Honor from it. If you control a Courtier, you may bow him to increase the gain or loss by 1." Two gaps: an Interrupt window before ANY action targeting a Holding resolves (the before-action windows only predict movers and a few curated destroy and bow ids, P8), and a choice of who takes an Honor change made inside it (the P14 channel supports a redirect, but nothing asks the acting player at that point). Its Kharmic reminder text is the engine's.</t>
-        </is>
-      </c>
-      <c r="H1598" t="inlineStr">
-        <is>
-          <t>TRIG-ANN</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1598" t="inlineStr"/>
+      <c r="H1598" t="inlineStr"/>
     </row>
     <row r="1599">
       <c r="A1599" t="inlineStr">
@@ -56759,7 +56642,7 @@
       </c>
       <c r="B1649" t="inlineStr">
         <is>
-          <t>Pierce the Tapestery</t>
+          <t>Pierce the Tapestry</t>
         </is>
       </c>
       <c r="C1649" t="inlineStr">
@@ -56779,14 +56662,10 @@
       </c>
       <c r="F1649" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1649" t="inlineStr">
-        <is>
-          <t>Pierce the Tapestery (awaiting a ruling from Mendon on the seven-copy deck rule and the per-battle count): the mechanisms are merged. "Up to seven copies" is CardDefinition.DeckCopyLimit (issue #337, DeckWorkshop CopyLimit), "two or more other Pierce the Tapestry played this battle" is a P7 period counter (AddPeriodCount / PeriodCountOf with Period.Battle, PeriodWatches.cs; this card is its design example), and "an additional Battle action to play a Pierce the Tapestry" is P17's additional-action scope (AdditionalActionScope.cs). Not wired.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1649" t="inlineStr"/>
       <c r="H1649" t="inlineStr"/>
     </row>
     <row r="1650">
@@ -62397,19 +62276,11 @@
       </c>
       <c r="F1814" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1814" t="inlineStr">
-        <is>
-          <t>The Heavens' Blessing (Strategy, issue #733): two Open effects. "No player can gain Honor in Action Phases (this turn)" is a P14 no-gain modifier with the action-phase-only filter, but the first, "Until the game ends, a player must pay 2 Gold to draw a card from effects of his own Strategies during an Action Phase", has no home: Draw has no source, so a draw made by a Strategy's effect cannot be told from any other, and a payment asked in the middle of an effect (declinable, with the draw lost) has no decision for it. Publishing only the second sentence would drop printed text.</t>
-        </is>
-      </c>
-      <c r="H1814" t="inlineStr">
-        <is>
-          <t>COST</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1814" t="inlineStr"/>
+      <c r="H1814" t="inlineStr"/>
     </row>
     <row r="1815">
       <c r="A1815" t="inlineStr">
@@ -64377,14 +64248,10 @@
       </c>
       <c r="F1872" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1872" t="inlineStr">
-        <is>
-          <t>Unbearable Weight (Strategy; one of the 13 cards awaiting a ruling from Mendon): "If this destroyed the target, his controller puts this Strategy in his hand" puts a played Strategy into the other player's hand; whose card it is afterwards and which discard pile it goes to when he plays it is unruled. Naoharu's Gift (EmperorRemainingFEvents.cs, naoharu-take) is a precedent for a card resting in another player's hand (ownership moves, OriginalOwnerId returns it to its owner's pile when it leaves), but it is Event-only code. Also unruled: "a Fate deck" (any player's, or the performer's own). Discarding the top card of a Fate deck and using its Focus Value are merged (aberrations-boost, fires-of-turmoil). Not wired.</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1872" t="inlineStr"/>
       <c r="H1872" t="inlineStr"/>
     </row>
     <row r="1873">
@@ -65503,19 +65370,11 @@
       </c>
       <c r="F1905" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G1905" t="inlineStr">
-        <is>
-          <t>Warded Premises (Strategy): "Before this battle's resolution: Negate all Force bonuses from actions to cards at this battlefield." Part of the first gap is closed: Creating Order's NegateActionForceModifiers and ActionForceModifierNegated (ForgottenLegacyBatch3.cs) already tell a Force modifier given by an action (a Modifier whose Effect is an action ability) from a trait's standing modifier, and leave tokens alone, and the Terrain's before-resolution timing exists (BeforeResolution.cs). What remains: a bonuses-only variant applied to every card at a battlefield (the existing helper negates penalties too and covers one card for the rest of the turn), and a ruling from Mendon on whether a Permanent bonus ("Permanently give him +2F") is negated for good or only suspended and whether Item and token bonuses count. Its second ability (put this Terrain into play at a battlefield with no Terrain, even without a unit there) is wireable.</t>
-        </is>
-      </c>
-      <c r="H1905" t="inlineStr">
-        <is>
-          <t>EFFECT</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G1905" t="inlineStr"/>
+      <c r="H1905" t="inlineStr"/>
     </row>
     <row r="1906">
       <c r="A1906" t="inlineStr">
@@ -72881,19 +72740,11 @@
       </c>
       <c r="F2122" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2122" t="inlineStr">
-        <is>
-          <t>Revelations (Event, issue #738): "Show the top five cards of your Dynasty deck. Choose another player who may discard one of the cards. Put the rest back in any order. Refill this province face-up." The scan prints no "After you reveal" clause, so it is an ordinary Event that resolves when revealed. Its three steps are still not composed from what is merged: P25's shown choice (PendingShownChoice, used by Dark Audience) lets another player pick among shown cards but hangs off a search, the look (DeckLook.cs) lets its own player rearrange but has no step in which another player discards one of the shown cards before the rest go back, and the Event's own province must then refill face up (RefillSourceProvinceFaceUp is a search disposition). Batch 8 (#739) merged without this card, so no decision work is pending elsewhere; it needs a look disposition with an other-player discard and a reorder.</t>
-        </is>
-      </c>
-      <c r="H2122" t="inlineStr">
-        <is>
-          <t>SEARCH</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2122" t="inlineStr"/>
+      <c r="H2122" t="inlineStr"/>
     </row>
     <row r="2123">
       <c r="A2123" t="inlineStr">
@@ -73331,19 +73182,11 @@
       </c>
       <c r="F2135" t="inlineStr">
         <is>
-          <t>Unwired</t>
-        </is>
-      </c>
-      <c r="G2135" t="inlineStr">
-        <is>
-          <t>The Empire's Foe Exposed (Event, issue #740): "Limited: Target two Unique Personalities in play, exactly one of which is yours. Your Personality challenges the other Personality. Destroy the duel's loser." The scan prints no "After you reveal" clause, so it is an ordinary Event that resolves when it is revealed in the Events Phase. Every merged duel starts from an ability a player uses (IssueChallenge is reached only from the IssuesDuel branch of an ability's effects, in a battle or the Action Phase), and P18's rules, refusal and focus windows resume play with NextAction for the challenger. Starting a duel from inside an Event's reveal (a pause on two chosen Unique Personalities, then a duel whose end must resume the Events Phase's reveal loop) is not a merged path, and the Event has no ability a player could use later. Publishing it as a reveal-time duel would need that resumption built and tested, so the card is left unpublished rather than approximated.</t>
-        </is>
-      </c>
-      <c r="H2135" t="inlineStr">
-        <is>
-          <t>DUEL</t>
-        </is>
-      </c>
+          <t>Wired</t>
+        </is>
+      </c>
+      <c r="G2135" t="inlineStr"/>
+      <c r="H2135" t="inlineStr"/>
     </row>
     <row r="2136">
       <c r="A2136" t="inlineStr">
@@ -76640,7 +76483,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -76660,7 +76503,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -76680,7 +76523,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -76760,7 +76603,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -76820,7 +76663,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -76940,7 +76783,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -76960,7 +76803,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -77000,7 +76843,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -77040,7 +76883,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Record Tamori Kazushige and Togashi Korimi as partially wired (#856)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GLVY8srUKbYJTyoNmoGWDm
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -25815,7 +25815,11 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G738" t="inlineStr"/>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>Tamori Kazushige: only his +2F while defending is wired. His printed "Open: If it is another player's turn, target one of his Personalities: Before this phase ends, straighten him. Before this turn ends, if the Personality did not assign to attack this turn, gain 2 Honor." has no ability (Bayushi Misaki's action is the same shape and is wired). Found by the printed-action sweep after #848.</t>
+        </is>
+      </c>
       <c r="H738" t="inlineStr"/>
     </row>
     <row r="739">
@@ -26929,7 +26933,11 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G771" t="inlineStr"/>
+      <c r="G771" t="inlineStr">
+        <is>
+          <t>Togashi Korimi: only his +2F while defending is wired. His printed "Interrupt, Bow this card: After you Recruit Korimi, draw a card." has no ability. Found by the printed-action sweep after #848.</t>
+        </is>
+      </c>
       <c r="H771" t="inlineStr"/>
     </row>
     <row r="772">

</xml_diff>

<commit_message>
Wire Tamori Kazushige's Open and Togashi Korimi's entering-play draw (#859)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GLVY8srUKbYJTyoNmoGWDm
</commit_message>
<xml_diff>
--- a/docs/CARD_INVENTORY.xlsx
+++ b/docs/CARD_INVENTORY.xlsx
@@ -25815,11 +25815,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G738" t="inlineStr">
-        <is>
-          <t>Tamori Kazushige: only his +2F while defending is wired. His printed "Open: If it is another player's turn, target one of his Personalities: Before this phase ends, straighten him. Before this turn ends, if the Personality did not assign to attack this turn, gain 2 Honor." has no ability (Bayushi Misaki's action is the same shape and is wired). Found by the printed-action sweep after #848.</t>
-        </is>
-      </c>
+      <c r="G738" t="inlineStr"/>
       <c r="H738" t="inlineStr"/>
     </row>
     <row r="739">
@@ -26933,11 +26929,7 @@
           <t>Wired</t>
         </is>
       </c>
-      <c r="G771" t="inlineStr">
-        <is>
-          <t>Togashi Korimi: only his +2F while defending is wired. His printed "Interrupt, Bow this card: After you Recruit Korimi, draw a card." has no ability. Found by the printed-action sweep after #848.</t>
-        </is>
-      </c>
+      <c r="G771" t="inlineStr"/>
       <c r="H771" t="inlineStr"/>
     </row>
     <row r="772">

</xml_diff>